<commit_message>
Document execution and evidence for all test cases
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R7923b74bafb044a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd6b8a7e63d4a4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2318af0963d643d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rdeae70d6a6f64485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ffd30ebb36349e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd0c75cd158cf4db1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4888fb3296aa4901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra5fa0a5cf6fc4af5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -50,13 +50,49 @@
       <x:color rgb="FF875700"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF243247"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23395B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23395B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1D6"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -85,7 +121,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -119,6 +155,60 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2139,6 +2229,10 @@
     <x:col min="7" max="7" width="70" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="63" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="39" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="79" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="43" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="77" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="28" customHeight="1">
@@ -2156,7 +2250,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>历史人工样本已删除；重新验收须使用当前版本和新样本留存新的证据。</x:v>
+        <x:v>H/I 列为历史验收状态与证据；J–M 列说明当前执行入口和覆盖，本轮结果须另留证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2206,6 +2300,18 @@
       <x:c r="I5" s="8" t="str">
         <x:v>证据</x:v>
       </x:c>
+      <x:c r="J5" s="26" t="str">
+        <x:v>单用例执行命令</x:v>
+      </x:c>
+      <x:c r="K5" s="26" t="str">
+        <x:v>实际绑定测试</x:v>
+      </x:c>
+      <x:c r="L5" s="26" t="str">
+        <x:v>自动化覆盖</x:v>
+      </x:c>
+      <x:c r="M5" s="26" t="str">
+        <x:v>本轮证据要求</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -2235,6 +2341,18 @@
       <x:c r="I6" s="9" t="str">
         <x:v>docs/feasibility.md；2026-10-02</x:v>
       </x:c>
+      <x:c r="J6" s="9" t="str">
+        <x:v>npm run test:case -- TC-001</x:v>
+      </x:c>
+      <x:c r="K6" s="9" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L6" s="9" t="str">
+        <x:v>人工入口；仅有历史证据</x:v>
+      </x:c>
+      <x:c r="M6" s="9" t="str">
+        <x:v>脱敏字段映射与计数、工具版本、日期；历史证据为 docs/feasibility.md，当前验收须另存新证据。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="10" t="str">
@@ -2264,6 +2382,18 @@
       <x:c r="I7" s="10" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A1</x:v>
       </x:c>
+      <x:c r="J7" s="27" t="str">
+        <x:v>npm run test:case -- TC-002</x:v>
+      </x:c>
+      <x:c r="K7" s="27" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L7" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M7" s="27" t="str">
+        <x:v>保存命令、退出码和 Playwright 脱敏日志；记录提交及 macOS 环境。</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="9" t="str">
@@ -2293,6 +2423,18 @@
       <x:c r="I8" s="9" t="str">
         <x:v>tests/auth.test.ts；docs/validation.md A1</x:v>
       </x:c>
+      <x:c r="J8" s="9" t="str">
+        <x:v>npm run test:case -- TC-003</x:v>
+      </x:c>
+      <x:c r="K8" s="9" t="str">
+        <x:v>tests/auth.test.ts：首次管理员、重启后的登录和失败尝试限速</x:v>
+      </x:c>
+      <x:c r="L8" s="9" t="str">
+        <x:v>单函数绑定；按源码断言</x:v>
+      </x:c>
+      <x:c r="M8" s="9" t="str">
+        <x:v>保存该 Vitest 测试的命令、退出码和脱敏日志。</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="60" customHeight="1">
       <x:c r="A9" s="10" t="str">
@@ -2322,6 +2464,18 @@
       <x:c r="I9" s="10" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
       </x:c>
+      <x:c r="J9" s="27" t="str">
+        <x:v>npm run test:case -- TC-004</x:v>
+      </x:c>
+      <x:c r="K9" s="27" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L9" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M9" s="27" t="str">
+        <x:v>保存共享 Playwright 函数的命令与退出码；说明本编号没有独立测试函数。</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="9" t="str">
@@ -2351,6 +2505,18 @@
       <x:c r="I10" s="9" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
       </x:c>
+      <x:c r="J10" s="9" t="str">
+        <x:v>npm run test:case -- TC-005</x:v>
+      </x:c>
+      <x:c r="K10" s="9" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L10" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M10" s="9" t="str">
+        <x:v>保存共享 Playwright 函数的命令与退出码；标注三项 IPC 结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
       <x:c r="A11" s="10" t="str">
@@ -2380,6 +2546,18 @@
       <x:c r="I11" s="10" t="str">
         <x:v>docs/validation.md A3；样本已删除</x:v>
       </x:c>
+      <x:c r="J11" s="27" t="str">
+        <x:v>npm run test:case -- TC-006</x:v>
+      </x:c>
+      <x:c r="K11" s="27" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L11" s="27" t="str">
+        <x:v>人工入口；仅有历史证据</x:v>
+      </x:c>
+      <x:c r="M11" s="27" t="str">
+        <x:v>版本、样本数、脱敏摘要和差异为零的核对记录；2026-10-02 的 A3 样本已删除，不能复用作本轮证据。</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="60" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -2409,6 +2587,18 @@
       <x:c r="I12" s="9" t="str">
         <x:v>tests/collector.test.ts</x:v>
       </x:c>
+      <x:c r="J12" s="9" t="str">
+        <x:v>npm run test:case -- TC-007</x:v>
+      </x:c>
+      <x:c r="K12" s="9" t="str">
+        <x:v>tests/collector.test.ts：模型切换与 Claude 子代理记录按实际模型归档</x:v>
+      </x:c>
+      <x:c r="L12" s="9" t="str">
+        <x:v>单函数绑定；按源码断言</x:v>
+      </x:c>
+      <x:c r="M12" s="9" t="str">
+        <x:v>保存该 Vitest 函数的命令、退出码与四行脱敏结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" s="10" t="str">
@@ -2438,6 +2628,18 @@
       <x:c r="I13" s="10" t="str">
         <x:v>docs/validation.md A4；样本已删除</x:v>
       </x:c>
+      <x:c r="J13" s="27" t="str">
+        <x:v>npm run test:case -- TC-008</x:v>
+      </x:c>
+      <x:c r="K13" s="27" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L13" s="27" t="str">
+        <x:v>人工入口；仅有历史证据</x:v>
+      </x:c>
+      <x:c r="M13" s="27" t="str">
+        <x:v>脱敏逐条摘要和差异为零的核对记录；历史 A4 样本已删除，当前验收须新取样。</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="9" t="str">
@@ -2467,6 +2669,18 @@
       <x:c r="I14" s="9" t="str">
         <x:v>tests/collector.test.ts</x:v>
       </x:c>
+      <x:c r="J14" s="9" t="str">
+        <x:v>npm run test:case -- TC-009</x:v>
+      </x:c>
+      <x:c r="K14" s="9" t="str">
+        <x:v>tests/collector.test.ts：两个采集器按请求去重，重扫和增量扫描不重复计数</x:v>
+      </x:c>
+      <x:c r="L14" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M14" s="9" t="str">
+        <x:v>保存共享 Vitest 函数的命令、退出码和 1 条 Claude 事实结果。</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
       <x:c r="A15" s="10" t="str">
@@ -2496,6 +2710,19 @@
       <x:c r="I15" s="10" t="str">
         <x:v>tests/collector.test.ts；tests/e2e/app.spec.ts；A5</x:v>
       </x:c>
+      <x:c r="J15" s="27" t="str">
+        <x:v>npm run test:case -- TC-010</x:v>
+      </x:c>
+      <x:c r="K15" s="27" t="str">
+        <x:v>tests/collector.test.ts：两个采集器按请求去重，重扫和增量扫描不重复计数
+tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L15" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M15" s="27" t="str">
+        <x:v>保留同一 TC 命令的两段测试日志及退出码；说明两个绑定函数均通过。</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="9" t="str">
@@ -2525,6 +2752,18 @@
       <x:c r="I16" s="9" t="str">
         <x:v>tests/collector.test.ts；docs/validation.md A5</x:v>
       </x:c>
+      <x:c r="J16" s="9" t="str">
+        <x:v>npm run test:case -- TC-011</x:v>
+      </x:c>
+      <x:c r="K16" s="9" t="str">
+        <x:v>tests/collector.test.ts：未写完的末行等待补齐，截断重写后不重复统计</x:v>
+      </x:c>
+      <x:c r="L16" s="9" t="str">
+        <x:v>单函数绑定；按源码断言</x:v>
+      </x:c>
+      <x:c r="M16" s="9" t="str">
+        <x:v>保存该 Vitest 函数命令、退出码和事实数序列。</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
       <x:c r="A17" s="10" t="str">
@@ -2554,6 +2793,18 @@
       <x:c r="I17" s="10" t="str">
         <x:v>tests/collector.test.ts；docs/feasibility.md</x:v>
       </x:c>
+      <x:c r="J17" s="27" t="str">
+        <x:v>npm run test:case -- TC-012</x:v>
+      </x:c>
+      <x:c r="K17" s="27" t="str">
+        <x:v>tests/collector.test.ts：两个采集器按请求去重，重扫和增量扫描不重复计数</x:v>
+      </x:c>
+      <x:c r="L17" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M17" s="27" t="str">
+        <x:v>保存共享 Vitest 函数命令和关键字段断言；无专属函数。</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="9" t="str">
@@ -2583,6 +2834,18 @@
       <x:c r="I18" s="9" t="str">
         <x:v>tests/collector.test.ts；docs/feasibility.md</x:v>
       </x:c>
+      <x:c r="J18" s="9" t="str">
+        <x:v>npm run test:case -- TC-013</x:v>
+      </x:c>
+      <x:c r="K18" s="9" t="str">
+        <x:v>tests/collector.test.ts：两个采集器按请求去重，重扫和增量扫描不重复计数</x:v>
+      </x:c>
+      <x:c r="L18" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M18" s="9" t="str">
+        <x:v>保存共享 Vitest 函数命令和分类/总量断言；无专属函数。</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
       <x:c r="A19" s="10" t="str">
@@ -2612,6 +2875,18 @@
       <x:c r="I19" s="10" t="str">
         <x:v>tests/telemetry.test.ts</x:v>
       </x:c>
+      <x:c r="J19" s="27" t="str">
+        <x:v>npm run test:case -- TC-014</x:v>
+      </x:c>
+      <x:c r="K19" s="27" t="str">
+        <x:v>tests/telemetry.test.ts：本机遥测只接受密钥，Codex 去重，Claude 累计点计算增量，报表避免双来源相加</x:v>
+      </x:c>
+      <x:c r="L19" s="27" t="str">
+        <x:v>共享测试；非独立断言；回环地址未单独断言</x:v>
+      </x:c>
+      <x:c r="M19" s="27" t="str">
+        <x:v>保存共享 Vitest 函数日志与 HTTP 状态；现有测试未单独断言绑定地址为 127.0.0.1。</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
       <x:c r="A20" s="9" t="str">
@@ -2641,6 +2916,18 @@
       <x:c r="I20" s="9" t="str">
         <x:v>tests/telemetry.test.ts</x:v>
       </x:c>
+      <x:c r="J20" s="9" t="str">
+        <x:v>npm run test:case -- TC-015</x:v>
+      </x:c>
+      <x:c r="K20" s="9" t="str">
+        <x:v>tests/telemetry.test.ts：遥测配置提示现有用户设置而不修改文件</x:v>
+      </x:c>
+      <x:c r="L20" s="9" t="str">
+        <x:v>单函数绑定；按源码断言；原配置未字节比对</x:v>
+      </x:c>
+      <x:c r="M20" s="9" t="str">
+        <x:v>保存该 Vitest 函数日志；当前测试未逐字节断言原配置内容未变化。</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
       <x:c r="A21" s="10" t="str">
@@ -2670,6 +2957,18 @@
       <x:c r="I21" s="10" t="str">
         <x:v>tests/telemetry.test.ts</x:v>
       </x:c>
+      <x:c r="J21" s="27" t="str">
+        <x:v>npm run test:case -- TC-016</x:v>
+      </x:c>
+      <x:c r="K21" s="27" t="str">
+        <x:v>tests/telemetry.test.ts：本机遥测只接受密钥，Codex 去重，Claude 累计点计算增量，报表避免双来源相加</x:v>
+      </x:c>
+      <x:c r="L21" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M21" s="27" t="str">
+        <x:v>保存共享 Vitest 函数命令、退出码和 12/8/20/27 断言。</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
       <x:c r="A22" s="9" t="str">
@@ -2699,6 +2998,19 @@
       <x:c r="I22" s="9" t="str">
         <x:v>tests/collector.test.ts；tests/e2e/source-status.spec.ts；A6</x:v>
       </x:c>
+      <x:c r="J22" s="9" t="str">
+        <x:v>npm run test:case -- TC-017</x:v>
+      </x:c>
+      <x:c r="K22" s="9" t="str">
+        <x:v>tests/e2e/source-status.spec.ts：工具目录缺失、无权限和空目录有清晰状态
+tests/collector.test.ts：空目录、错误字段及不可读文件显示可辨认的状态</x:v>
+      </x:c>
+      <x:c r="L22" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M22" s="9" t="str">
+        <x:v>保存同一 TC 命令的 Playwright 与 Vitest 日志和退出码；错误单元函数也被 TC-018 共用。</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="10" t="str">
@@ -2728,6 +3040,18 @@
       <x:c r="I23" s="10" t="str">
         <x:v>tests/collector.test.ts；docs/validation.md A6</x:v>
       </x:c>
+      <x:c r="J23" s="27" t="str">
+        <x:v>npm run test:case -- TC-018</x:v>
+      </x:c>
+      <x:c r="K23" s="27" t="str">
+        <x:v>tests/collector.test.ts：空目录、错误字段及不可读文件显示可辨认的状态</x:v>
+      </x:c>
+      <x:c r="L23" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M23" s="27" t="str">
+        <x:v>保存共享 Vitest 函数命令、退出码和错误状态字段。</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="60" customHeight="1">
       <x:c r="A24" s="9" t="str">
@@ -2757,6 +3081,18 @@
       <x:c r="I24" s="9" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A7</x:v>
       </x:c>
+      <x:c r="J24" s="9" t="str">
+        <x:v>npm run test:case -- TC-019</x:v>
+      </x:c>
+      <x:c r="K24" s="9" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L24" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M24" s="9" t="str">
+        <x:v>保存共享 Playwright 函数命令、退出码和 12/14 权限对比。</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="10" t="str">
@@ -2786,6 +3122,18 @@
       <x:c r="I25" s="10" t="str">
         <x:v>tests/report.test.ts；docs/validation.md A8</x:v>
       </x:c>
+      <x:c r="J25" s="27" t="str">
+        <x:v>npm run test:case -- TC-020</x:v>
+      </x:c>
+      <x:c r="K25" s="27" t="str">
+        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属</x:v>
+      </x:c>
+      <x:c r="L25" s="27" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M25" s="27" t="str">
+        <x:v>保存共享 Vitest 函数命令、退出码和周期值。</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="60" customHeight="1">
       <x:c r="A26" s="9" t="str">
@@ -2815,6 +3163,19 @@
       <x:c r="I26" s="9" t="str">
         <x:v>tests/report.test.ts；tests/e2e/app.spec.ts；A8</x:v>
       </x:c>
+      <x:c r="J26" s="9" t="str">
+        <x:v>npm run test:case -- TC-021</x:v>
+      </x:c>
+      <x:c r="K26" s="9" t="str">
+        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属
+tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L26" s="9" t="str">
+        <x:v>共享测试；非独立断言；第二页未测试</x:v>
+      </x:c>
+      <x:c r="M26" s="9" t="str">
+        <x:v>保存两段共享测试日志；现有自动化没有构造超过 50 条以检查第二页分页。</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
       <x:c r="A27" s="10" t="str">
@@ -2844,6 +3205,18 @@
       <x:c r="I27" s="10" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A9</x:v>
       </x:c>
+      <x:c r="J27" s="27" t="str">
+        <x:v>npm run test:case -- TC-022</x:v>
+      </x:c>
+      <x:c r="K27" s="27" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L27" s="27" t="str">
+        <x:v>共享测试；非独立断言；CSV 列结构未测试</x:v>
+      </x:c>
+      <x:c r="M27" s="27" t="str">
+        <x:v>保存共享 Playwright 日志和脱敏 CSV 数值；当前测试没有检查表头 8/9 列错位，见 TC-029。</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
       <x:c r="A28" s="9" t="str">
@@ -2873,6 +3246,18 @@
       <x:c r="I28" s="9" t="str">
         <x:v>tests/report.test.ts</x:v>
       </x:c>
+      <x:c r="J28" s="9" t="str">
+        <x:v>npm run test:case -- TC-023</x:v>
+      </x:c>
+      <x:c r="K28" s="9" t="str">
+        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属</x:v>
+      </x:c>
+      <x:c r="L28" s="9" t="str">
+        <x:v>共享测试；非独立断言</x:v>
+      </x:c>
+      <x:c r="M28" s="9" t="str">
+        <x:v>保存共享 Vitest 函数日志及脱敏 CSV 字段断言。</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
       <x:c r="A29" s="10" t="str">
@@ -2902,6 +3287,18 @@
       <x:c r="I29" s="10" t="str">
         <x:v>tests/backup.test.ts</x:v>
       </x:c>
+      <x:c r="J29" s="27" t="str">
+        <x:v>npm run test:case -- TC-024</x:v>
+      </x:c>
+      <x:c r="K29" s="27" t="str">
+        <x:v>tests/backup.test.ts：数据库备份完整性校验并保留账户与用量</x:v>
+      </x:c>
+      <x:c r="L29" s="27" t="str">
+        <x:v>单函数绑定；按源码断言</x:v>
+      </x:c>
+      <x:c r="M29" s="27" t="str">
+        <x:v>保存该 Vitest 函数命令、退出码和备份校验断言；不保留数据库文件。</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
       <x:c r="A30" s="9" t="str">
@@ -2931,6 +3328,18 @@
       <x:c r="I30" s="9" t="str">
         <x:v>tests/e2e/restore.spec.ts</x:v>
       </x:c>
+      <x:c r="J30" s="9" t="str">
+        <x:v>npm run test:case -- TC-025</x:v>
+      </x:c>
+      <x:c r="K30" s="9" t="str">
+        <x:v>tests/e2e/restore.spec.ts：管理员备份、恢复后账户回到备份状态</x:v>
+      </x:c>
+      <x:c r="L30" s="9" t="str">
+        <x:v>单函数绑定；按源码断言</x:v>
+      </x:c>
+      <x:c r="M30" s="9" t="str">
+        <x:v>保存 Playwright 日志和脱敏账户状态；不提交 snapshot.sqlite 或数据库副本。</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
       <x:c r="A31" s="10" t="str">
@@ -2960,6 +3369,18 @@
       <x:c r="I31" s="10" t="str">
         <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
       </x:c>
+      <x:c r="J31" s="27" t="str">
+        <x:v>npm run test:case -- TC-026</x:v>
+      </x:c>
+      <x:c r="K31" s="27" t="str">
+        <x:v>tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+      </x:c>
+      <x:c r="L31" s="27" t="str">
+        <x:v>共享测试；非独立断言；磁盘隐私未测试</x:v>
+      </x:c>
+      <x:c r="M31" s="27" t="str">
+        <x:v>保存共享 Playwright 日志；现有测试未断言磁盘/导出中不存在正文或密钥。</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
       <x:c r="A32" s="9" t="str">
@@ -2989,6 +3410,18 @@
       <x:c r="I32" s="9" t="str">
         <x:v>docs/validation.md A10；2026-10-02</x:v>
       </x:c>
+      <x:c r="J32" s="9" t="str">
+        <x:v>npm run test:case -- TC-027</x:v>
+      </x:c>
+      <x:c r="K32" s="9" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L32" s="9" t="str">
+        <x:v>人工入口；仅有历史证据</x:v>
+      </x:c>
+      <x:c r="M32" s="9" t="str">
+        <x:v>DMG 校验输出、包哈希/版本、当前 Mac 信息、复制后应用的脱敏流程记录；历史 A10 不能替代本轮。</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="60" customHeight="1">
       <x:c r="A33" s="10" t="str">
@@ -3018,6 +3451,18 @@
       <x:c r="I33" s="10" t="str">
         <x:v>尚无签名、公证及其他目标设备证据</x:v>
       </x:c>
+      <x:c r="J33" s="27" t="str">
+        <x:v>npm run test:case -- TC-028</x:v>
+      </x:c>
+      <x:c r="K33" s="27" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L33" s="30" t="str">
+        <x:v>人工入口；待验证</x:v>
+      </x:c>
+      <x:c r="M33" s="27" t="str">
+        <x:v>证书身份脱敏信息、签名验证、公证状态、目标 Mac 版本/架构和脱敏流程记录。</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
       <x:c r="A34" s="9" t="str">
@@ -3046,6 +3491,18 @@
       </x:c>
       <x:c r="I34" s="9" t="str">
         <x:v>src/main/report.ts 当前表头 8 列、数据行 9 列</x:v>
+      </x:c>
+      <x:c r="J34" s="9" t="str">
+        <x:v>npm run test:case -- TC-029</x:v>
+      </x:c>
+      <x:c r="K34" s="9" t="str">
+        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+      </x:c>
+      <x:c r="L34" s="30" t="str">
+        <x:v>已知缺陷；禁止通过</x:v>
+      </x:c>
+      <x:c r="M34" s="9" t="str">
+        <x:v>脱敏 CSV 表头/行列数对比与解析结果；修复前仅可记录 fail，不得记录 pass。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Document M5 feature requirements and change history
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ffd30ebb36349e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd0c75cd158cf4db1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4888fb3296aa4901"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra5fa0a5cf6fc4af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R0c1fa1c217164d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rddde2b5fa22645cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R8c4ec72069f645ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd03d2509fa004398"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,6 +109,26 @@
         <x:fgColor rgb="FFFFF1D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -121,7 +141,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -210,6 +230,21 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1146,6 +1181,489 @@
         <x:v>待验证</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>REQ-019</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>信任此设备自动登录</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="D35" s="35" t="str">
+        <x:v>受信设备令牌与启动恢复</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>TC-030</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>信任设备恢复登录</x:v>
+      </x:c>
+      <x:c r="G35" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="62" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>REQ-020</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>撤销受信设备</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>受信设备撤销与失效检查</x:v>
+      </x:c>
+      <x:c r="E36" s="14" t="str">
+        <x:v>TC-031</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>信任撤销与账户失效</x:v>
+      </x:c>
+      <x:c r="G36" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="62" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="B37" s="35" t="str">
+        <x:v>独立本地更新与汇总服务</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="D37" s="35" t="str">
+        <x:v>独立服务版本发布与聚合接口</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>TC-032</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>独立服务回环绑定</x:v>
+      </x:c>
+      <x:c r="G37" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="62" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>独立本地更新与汇总服务</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>独立服务版本发布与聚合接口</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="str">
+        <x:v>TC-033</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>版本清单和安装包</x:v>
+      </x:c>
+      <x:c r="G38" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="62" customHeight="1">
+      <x:c r="A39" s="35" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="B39" s="35" t="str">
+        <x:v>版本检查和安装包下载</x:v>
+      </x:c>
+      <x:c r="C39" s="35" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="D39" s="35" t="str">
+        <x:v>更新检查下载与完整性验证</x:v>
+      </x:c>
+      <x:c r="E39" s="35" t="str">
+        <x:v>TC-034</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>更新版本判断与下载校验</x:v>
+      </x:c>
+      <x:c r="G39" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="62" customHeight="1">
+      <x:c r="A40" s="14" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="B40" s="14" t="str">
+        <x:v>版本检查和安装包下载</x:v>
+      </x:c>
+      <x:c r="C40" s="14" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="D40" s="14" t="str">
+        <x:v>更新检查下载与完整性验证</x:v>
+      </x:c>
+      <x:c r="E40" s="14" t="str">
+        <x:v>TC-035</x:v>
+      </x:c>
+      <x:c r="F40" s="14" t="str">
+        <x:v>更新服务故障恢复</x:v>
+      </x:c>
+      <x:c r="G40" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="62" customHeight="1">
+      <x:c r="A41" s="35" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="B41" s="35" t="str">
+        <x:v>未签名 macOS 更新交接</x:v>
+      </x:c>
+      <x:c r="C41" s="35" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="D41" s="35" t="str">
+        <x:v>未签名安装包打开与回退</x:v>
+      </x:c>
+      <x:c r="E41" s="35" t="str">
+        <x:v>TC-036</x:v>
+      </x:c>
+      <x:c r="F41" s="35" t="str">
+        <x:v>未签名安装包交接</x:v>
+      </x:c>
+      <x:c r="G41" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="62" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>REQ-024</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>扫描频率与上传触发</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>DEV-026</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>十分钟调度与扫描完成事件</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="str">
+        <x:v>TC-037</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>启动定时手动扫描与上传</x:v>
+      </x:c>
+      <x:c r="G42" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="62" customHeight="1">
+      <x:c r="A43" s="35" t="str">
+        <x:v>REQ-025</x:v>
+      </x:c>
+      <x:c r="B43" s="35" t="str">
+        <x:v>最小化聚合用量上报</x:v>
+      </x:c>
+      <x:c r="C43" s="35" t="str">
+        <x:v>DEV-027</x:v>
+      </x:c>
+      <x:c r="D43" s="35" t="str">
+        <x:v>聚合投影和字段白名单</x:v>
+      </x:c>
+      <x:c r="E43" s="35" t="str">
+        <x:v>TC-038</x:v>
+      </x:c>
+      <x:c r="F43" s="35" t="str">
+        <x:v>聚合载荷隐私和数值</x:v>
+      </x:c>
+      <x:c r="G43" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="62" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>聚合幂等、重试和状态</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>DEV-028</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>待传队列和客户端幂等</x:v>
+      </x:c>
+      <x:c r="E44" s="14" t="str">
+        <x:v>TC-039</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>重复快照幂等</x:v>
+      </x:c>
+      <x:c r="G44" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="62" customHeight="1">
+      <x:c r="A45" s="35" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="B45" s="35" t="str">
+        <x:v>聚合幂等、重试和状态</x:v>
+      </x:c>
+      <x:c r="C45" s="35" t="str">
+        <x:v>DEV-028</x:v>
+      </x:c>
+      <x:c r="D45" s="35" t="str">
+        <x:v>待传队列和客户端幂等</x:v>
+      </x:c>
+      <x:c r="E45" s="35" t="str">
+        <x:v>TC-040</x:v>
+      </x:c>
+      <x:c r="F45" s="35" t="str">
+        <x:v>离线重试与状态</x:v>
+      </x:c>
+      <x:c r="G45" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="62" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>REQ-027</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>Token 紧凑显示与精确值</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>DEV-029</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>统一 Token 格式化</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>TC-041</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>1024 单位与原值</x:v>
+      </x:c>
+      <x:c r="G46" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="62" customHeight="1">
+      <x:c r="A47" s="35" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="B47" s="35" t="str">
+        <x:v>用量概览与趋势分析</x:v>
+      </x:c>
+      <x:c r="C47" s="35" t="str">
+        <x:v>DEV-030</x:v>
+      </x:c>
+      <x:c r="D47" s="35" t="str">
+        <x:v>概览指标与比较</x:v>
+      </x:c>
+      <x:c r="E47" s="35" t="str">
+        <x:v>TC-042</x:v>
+      </x:c>
+      <x:c r="F47" s="35" t="str">
+        <x:v>概览指标与区间比较</x:v>
+      </x:c>
+      <x:c r="G47" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="62" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>用量概览与趋势分析</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>DEV-031</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>趋势下钻和模型排行</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>TC-043</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>趋势筛选与下钻</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="62" customHeight="1">
+      <x:c r="A49" s="35" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="B49" s="35" t="str">
+        <x:v>模型排行与来源覆盖状态</x:v>
+      </x:c>
+      <x:c r="C49" s="35" t="str">
+        <x:v>DEV-031</x:v>
+      </x:c>
+      <x:c r="D49" s="35" t="str">
+        <x:v>趋势下钻和模型排行</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="str">
+        <x:v>TC-044</x:v>
+      </x:c>
+      <x:c r="F49" s="35" t="str">
+        <x:v>模型排行与明细</x:v>
+      </x:c>
+      <x:c r="G49" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="62" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>模型排行与来源覆盖状态</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>DEV-032</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>来源健康视图</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>TC-045</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>未覆盖与真实零区分</x:v>
+      </x:c>
+      <x:c r="G50" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="62" customHeight="1">
+      <x:c r="A51" s="35" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="B51" s="35" t="str">
+        <x:v>模型排行与来源覆盖状态</x:v>
+      </x:c>
+      <x:c r="C51" s="35" t="str">
+        <x:v>DEV-032</x:v>
+      </x:c>
+      <x:c r="D51" s="35" t="str">
+        <x:v>来源健康视图</x:v>
+      </x:c>
+      <x:c r="E51" s="35" t="str">
+        <x:v>TC-046</x:v>
+      </x:c>
+      <x:c r="F51" s="35" t="str">
+        <x:v>来源状态概览</x:v>
+      </x:c>
+      <x:c r="G51" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="62" customHeight="1">
+      <x:c r="A52" s="14" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="B52" s="14" t="str">
+        <x:v>独立本地更新与汇总服务</x:v>
+      </x:c>
+      <x:c r="C52" s="14" t="str">
+        <x:v>DEV-023</x:v>
+      </x:c>
+      <x:c r="D52" s="14" t="str">
+        <x:v>聚合接口鉴权与 upsert</x:v>
+      </x:c>
+      <x:c r="E52" s="14" t="str">
+        <x:v>TC-047</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
+        <x:v>聚合接口授权</x:v>
+      </x:c>
+      <x:c r="G52" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="62" customHeight="1">
+      <x:c r="A53" s="35" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="B53" s="35" t="str">
+        <x:v>趋势图自适应和周月日期</x:v>
+      </x:c>
+      <x:c r="C53" s="35" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="D53" s="35" t="str">
+        <x:v>响应式趋势图与时间标签</x:v>
+      </x:c>
+      <x:c r="E53" s="35" t="str">
+        <x:v>TC-048</x:v>
+      </x:c>
+      <x:c r="F53" s="35" t="str">
+        <x:v>趋势图窗口缩放布局</x:v>
+      </x:c>
+      <x:c r="G53" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="62" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>趋势图自适应和周月日期</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>响应式趋势图与时间标签</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>TC-049</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>周月横轴日期格式</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="62" customHeight="1">
+      <x:c r="A55" s="35" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="B55" s="35" t="str">
+        <x:v>聚合幂等、重试和状态</x:v>
+      </x:c>
+      <x:c r="C55" s="35" t="str">
+        <x:v>DEV-023</x:v>
+      </x:c>
+      <x:c r="D55" s="35" t="str">
+        <x:v>聚合接口鉴权与 upsert</x:v>
+      </x:c>
+      <x:c r="E55" s="35" t="str">
+        <x:v>TC-039</x:v>
+      </x:c>
+      <x:c r="F55" s="35" t="str">
+        <x:v>重复快照幂等</x:v>
+      </x:c>
+      <x:c r="G55" s="35" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1182,7 +1700,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>验收条件写可观察结果；“已实现（本机）”只适用于当前已验证环境。</x:v>
+        <x:v>REQ-001–018 为原版；REQ-019–030 是 M5 计划，尚未实现。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1694,6 +2212,318 @@
       </x:c>
       <x:c r="H23" s="10" t="str">
         <x:v>docs/design.md §7；docs/validation.md 末段</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="62" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>REQ-019</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>信任此设备自动登录</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>登录页默认不勾选；主动勾选并成功登录后，在同一 macOS 账户重启应用可自动进入原用户；不保存明文密码，普通登录退出进程后仍失效。</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="G24" s="14" t="str">
+        <x:v>TC-030</x:v>
+      </x:c>
+      <x:c r="H24" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="62" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:v>REQ-020</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="str">
+        <x:v>撤销受信设备</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="str">
+        <x:v>受信状态无固定到期时间；保持自动登录直到手动退出登录，退出立即撤销本设备信任；管理员禁用账户或密码重置也撤销该账户信任凭证；失效/损坏令牌可清理并回到登录页。</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F25" s="35" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="G25" s="35" t="str">
+        <x:v>TC-031</x:v>
+      </x:c>
+      <x:c r="H25" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="62" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>独立本地更新与汇总服务</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>提供独立进程，默认仅绑定 127.0.0.1；明确版本清单、安装包和聚合接收接口；非回环访问拒绝，管理/上报接口需授权；服务故障不影响本机报表。</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>DEV-022、DEV-023</x:v>
+      </x:c>
+      <x:c r="G26" s="14" t="str">
+        <x:v>TC-032、TC-033、TC-047</x:v>
+      </x:c>
+      <x:c r="H26" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="62" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="str">
+        <x:v>版本检查和安装包下载</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="str">
+        <x:v>应用请求本地服务版本清单，仅在版本更新且平台匹配时提示；下载到受控临时目录，校验长度和 SHA-256 后才可交给系统打开；无服务、损坏或低版本给出可恢复状态。</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F27" s="35" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="G27" s="35" t="str">
+        <x:v>TC-034、TC-035</x:v>
+      </x:c>
+      <x:c r="H27" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="62" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>未签名 macOS 更新交接</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>当前未签名应用发现更新后下载并打开安装包，由用户完成安装；不得调用静默替换或承诺自动安装；取消打开或安装失败保留旧版可运行。</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="G28" s="14" t="str">
+        <x:v>TC-036</x:v>
+      </x:c>
+      <x:c r="H28" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="62" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>REQ-024</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="str">
+        <x:v>扫描频率与上传触发</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="str">
+        <x:v>应用启动、每 10 分钟及手动触发完整扫描；每次扫描完成后触发一次聚合快照上报；并发扫描串行化，失败扫描不得上报伪完整快照。</x:v>
+      </x:c>
+      <x:c r="D29" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F29" s="35" t="str">
+        <x:v>DEV-026</x:v>
+      </x:c>
+      <x:c r="G29" s="35" t="str">
+        <x:v>TC-037</x:v>
+      </x:c>
+      <x:c r="H29" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="62" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>REQ-025</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>最小化聚合用量上报</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>上报仅含设备/用户归属标识、UTC 统计区间、提供方、模型、Token 分类/总量、记录数与覆盖状态；不含会话正文、提示词、源码、密钥、原始路径或原始事件。</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>DEV-027</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str">
+        <x:v>TC-038</x:v>
+      </x:c>
+      <x:c r="H30" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="62" customHeight="1">
+      <x:c r="A31" s="35" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="B31" s="35" t="str">
+        <x:v>聚合幂等、重试和状态</x:v>
+      </x:c>
+      <x:c r="C31" s="35" t="str">
+        <x:v>同一设备、归属用户、统计区间及数据修订只计入一次；重复上报更新快照而不累加；服务不可用时保留待传队列，有限退避重试，并显示最近成功/失败与积压。</x:v>
+      </x:c>
+      <x:c r="D31" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E31" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F31" s="35" t="str">
+        <x:v>DEV-028、DEV-023</x:v>
+      </x:c>
+      <x:c r="G31" s="35" t="str">
+        <x:v>TC-039、TC-040</x:v>
+      </x:c>
+      <x:c r="H31" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="62" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>REQ-027</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>Token 紧凑显示与精确值</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>显示按自定义 K→M→P 逐级 1024 进位：1024 Token=1K，1024K=1M，1024M=1P，不引入 G/T；边界和舍入一致；明细/悬浮说明与 CSV 保留原始整数。</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>DEV-029</x:v>
+      </x:c>
+      <x:c r="G32" s="14" t="str">
+        <x:v>TC-041</x:v>
+      </x:c>
+      <x:c r="H32" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="62" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="B33" s="35" t="str">
+        <x:v>用量概览与趋势分析</x:v>
+      </x:c>
+      <x:c r="C33" s="35" t="str">
+        <x:v>概览展示总 Token、请求数、相对上一等长区间变化；日期/工具/用户筛选联动趋势与明细，点击数据点可下钻；比较区间不足显示未知。</x:v>
+      </x:c>
+      <x:c r="D33" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E33" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F33" s="35" t="str">
+        <x:v>DEV-030、DEV-031</x:v>
+      </x:c>
+      <x:c r="G33" s="35" t="str">
+        <x:v>TC-042、TC-043</x:v>
+      </x:c>
+      <x:c r="H33" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="62" customHeight="1">
+      <x:c r="A34" s="14" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="B34" s="14" t="str">
+        <x:v>模型排行与来源覆盖状态</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
+        <x:v>模型排行按 Token 降序且可进入明细；概览可见来源最后成功时间、正常/异常/未知/未覆盖，真实零用量与未覆盖分开显示。</x:v>
+      </x:c>
+      <x:c r="D34" s="14" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E34" s="14" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F34" s="14" t="str">
+        <x:v>DEV-031、DEV-032</x:v>
+      </x:c>
+      <x:c r="G34" s="14" t="str">
+        <x:v>TC-044、TC-045、TC-046</x:v>
+      </x:c>
+      <x:c r="H34" s="14" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>趋势图自适应和周月日期</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str">
+        <x:v>用量趋势图随应用窗口宽度重排，柱顶数值与横轴标签不重叠；周粒度按所选时区的 ISO 周周一显示 YYYY-MM-DD，月粒度显示 YYYY-MM。</x:v>
+      </x:c>
+      <x:c r="D35" s="35" t="str">
+        <x:v>M5（计划）</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>待实现</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="G35" s="35" t="str">
+        <x:v>TC-048、TC-049</x:v>
+      </x:c>
+      <x:c r="H35" s="35" t="str">
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2206,6 +3036,328 @@
       </x:c>
       <x:c r="G24" s="9" t="str">
         <x:v>当前表头 8 列，数据行 9 列；补总 Token 列头和结构断言</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="62" customHeight="1">
+      <x:c r="A25" s="35" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="B25" s="35" t="str">
+        <x:v>受信设备令牌与启动恢复</x:v>
+      </x:c>
+      <x:c r="C25" s="35" t="str">
+        <x:v>REQ-019</x:v>
+      </x:c>
+      <x:c r="D25" s="35" t="str">
+        <x:v>TC-030</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str">
+        <x:v>src/main/auth.ts；src/renderer/index.tsx；系统安全存储</x:v>
+      </x:c>
+      <x:c r="F25" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G25" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="62" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>受信设备撤销与失效检查</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>REQ-020</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>TC-031</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>src/main/auth.ts；src/renderer/settings.tsx</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G26" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="62" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="B27" s="35" t="str">
+        <x:v>独立服务版本发布与聚合接口</x:v>
+      </x:c>
+      <x:c r="C27" s="35" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="D27" s="35" t="str">
+        <x:v>TC-032、TC-033</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str">
+        <x:v>server/</x:v>
+      </x:c>
+      <x:c r="F27" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G27" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="62" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>DEV-023</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>聚合接口鉴权与 upsert</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>REQ-021、REQ-026</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>TC-039、TC-047</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>server/；SQLite</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G28" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="62" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="B29" s="35" t="str">
+        <x:v>更新检查下载与完整性验证</x:v>
+      </x:c>
+      <x:c r="C29" s="35" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="D29" s="35" t="str">
+        <x:v>TC-034、TC-035</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str">
+        <x:v>src/main/update.ts；src/preload</x:v>
+      </x:c>
+      <x:c r="F29" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G29" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="62" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>未签名安装包打开与回退</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>TC-036</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>src/main/update.ts</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="62" customHeight="1">
+      <x:c r="A31" s="35" t="str">
+        <x:v>DEV-026</x:v>
+      </x:c>
+      <x:c r="B31" s="35" t="str">
+        <x:v>十分钟调度与扫描完成事件</x:v>
+      </x:c>
+      <x:c r="C31" s="35" t="str">
+        <x:v>REQ-024</x:v>
+      </x:c>
+      <x:c r="D31" s="35" t="str">
+        <x:v>TC-037</x:v>
+      </x:c>
+      <x:c r="E31" s="35" t="str">
+        <x:v>src/collectors/scanner.ts</x:v>
+      </x:c>
+      <x:c r="F31" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G31" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="62" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>DEV-027</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>聚合投影和字段白名单</x:v>
+      </x:c>
+      <x:c r="C32" s="14" t="str">
+        <x:v>REQ-025</x:v>
+      </x:c>
+      <x:c r="D32" s="14" t="str">
+        <x:v>TC-038</x:v>
+      </x:c>
+      <x:c r="E32" s="14" t="str">
+        <x:v>src/main/report.ts；src/main/upload.ts</x:v>
+      </x:c>
+      <x:c r="F32" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G32" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="62" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>DEV-028</x:v>
+      </x:c>
+      <x:c r="B33" s="35" t="str">
+        <x:v>待传队列和客户端幂等</x:v>
+      </x:c>
+      <x:c r="C33" s="35" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="D33" s="35" t="str">
+        <x:v>TC-039、TC-040</x:v>
+      </x:c>
+      <x:c r="E33" s="35" t="str">
+        <x:v>src/main/upload.ts；SQLite 迁移</x:v>
+      </x:c>
+      <x:c r="F33" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G33" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="62" customHeight="1">
+      <x:c r="A34" s="14" t="str">
+        <x:v>DEV-029</x:v>
+      </x:c>
+      <x:c r="B34" s="14" t="str">
+        <x:v>统一 Token 格式化</x:v>
+      </x:c>
+      <x:c r="C34" s="14" t="str">
+        <x:v>REQ-027</x:v>
+      </x:c>
+      <x:c r="D34" s="14" t="str">
+        <x:v>TC-041</x:v>
+      </x:c>
+      <x:c r="E34" s="14" t="str">
+        <x:v>src/renderer/format.ts</x:v>
+      </x:c>
+      <x:c r="F34" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G34" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>DEV-030</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>概览指标与比较</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="D35" s="35" t="str">
+        <x:v>TC-042</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>src/renderer/index.tsx</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G35" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="62" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>DEV-031</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>趋势下钻和模型排行</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>REQ-028、REQ-029</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>TC-043、TC-044</x:v>
+      </x:c>
+      <x:c r="E36" s="14" t="str">
+        <x:v>src/renderer/report.tsx</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G36" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="62" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>DEV-032</x:v>
+      </x:c>
+      <x:c r="B37" s="35" t="str">
+        <x:v>来源健康视图</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="D37" s="35" t="str">
+        <x:v>TC-045、TC-046</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>src/renderer/index.tsx</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G37" s="35" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="62" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>响应式趋势图与时间标签</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>TC-048、TC-049</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="str">
+        <x:v>src/renderer/report.tsx；src/renderer/styles.css</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G38" s="14" t="str">
+        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2250,7 +3402,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>H/I 列为历史验收状态与证据；J–M 列说明当前执行入口和覆盖，本轮结果须另留证据。</x:v>
+        <x:v>TC-001–029 有现行入口；TC-030–049 待注册/实现，不能标记为通过。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3505,6 +4657,826 @@
         <x:v>脱敏 CSV 表头/行列数对比与解析结果；修复前仅可记录 fail，不得记录 pass。</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="70" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>TC-030</x:v>
+      </x:c>
+      <x:c r="B35" s="35" t="str">
+        <x:v>REQ-019</x:v>
+      </x:c>
+      <x:c r="C35" s="35" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="D35" s="35" t="str">
+        <x:v>信任设备恢复登录</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F35" s="35" t="str">
+        <x:v>临时账户首次登录勾选信任，关闭并重启应用。</x:v>
+      </x:c>
+      <x:c r="G35" s="35" t="str">
+        <x:v>自动登录同一用户且磁盘无明文密码。</x:v>
+      </x:c>
+      <x:c r="H35" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I35" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J35" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-030</x:v>
+      </x:c>
+      <x:c r="K35" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L35" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M35" s="35" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="70" customHeight="1">
+      <x:c r="A36" s="14" t="str">
+        <x:v>TC-031</x:v>
+      </x:c>
+      <x:c r="B36" s="14" t="str">
+        <x:v>REQ-020</x:v>
+      </x:c>
+      <x:c r="C36" s="14" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="D36" s="14" t="str">
+        <x:v>信任撤销与账户失效</x:v>
+      </x:c>
+      <x:c r="E36" s="14" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F36" s="14" t="str">
+        <x:v>信任后分别退出/撤销、禁用、重置密码并重启。</x:v>
+      </x:c>
+      <x:c r="G36" s="14" t="str">
+        <x:v>所有旧令牌失效，回到登录页；损坏令牌可恢复。</x:v>
+      </x:c>
+      <x:c r="H36" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I36" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J36" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-031</x:v>
+      </x:c>
+      <x:c r="K36" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L36" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M36" s="14" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="70" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>TC-032</x:v>
+      </x:c>
+      <x:c r="B37" s="35" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="C37" s="35" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="D37" s="35" t="str">
+        <x:v>独立服务回环绑定</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F37" s="35" t="str">
+        <x:v>独立启动服务，从回环和非回环地址请求清单。</x:v>
+      </x:c>
+      <x:c r="G37" s="35" t="str">
+        <x:v>回环可访问，非回环不能连接；停服不影响本机报表。</x:v>
+      </x:c>
+      <x:c r="H37" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I37" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J37" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-032</x:v>
+      </x:c>
+      <x:c r="K37" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L37" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M37" s="35" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="70" customHeight="1">
+      <x:c r="A38" s="14" t="str">
+        <x:v>TC-033</x:v>
+      </x:c>
+      <x:c r="B38" s="14" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="C38" s="14" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="D38" s="14" t="str">
+        <x:v>版本清单和安装包</x:v>
+      </x:c>
+      <x:c r="E38" s="14" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F38" s="14" t="str">
+        <x:v>发布测试版本及安装包，请求清单和下载流。</x:v>
+      </x:c>
+      <x:c r="G38" s="14" t="str">
+        <x:v>版本、平台、长度、摘要及文件内容匹配。</x:v>
+      </x:c>
+      <x:c r="H38" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I38" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J38" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-033</x:v>
+      </x:c>
+      <x:c r="K38" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L38" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M38" s="14" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="70" customHeight="1">
+      <x:c r="A39" s="35" t="str">
+        <x:v>TC-034</x:v>
+      </x:c>
+      <x:c r="B39" s="35" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="C39" s="35" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="D39" s="35" t="str">
+        <x:v>更新版本判断与下载校验</x:v>
+      </x:c>
+      <x:c r="E39" s="35" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F39" s="35" t="str">
+        <x:v>模拟新/同/旧版本和正确/错误 SHA-256。</x:v>
+      </x:c>
+      <x:c r="G39" s="35" t="str">
+        <x:v>仅新且匹配版本提示；错误摘要不得打开文件。</x:v>
+      </x:c>
+      <x:c r="H39" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I39" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J39" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-034</x:v>
+      </x:c>
+      <x:c r="K39" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L39" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M39" s="35" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="70" customHeight="1">
+      <x:c r="A40" s="14" t="str">
+        <x:v>TC-035</x:v>
+      </x:c>
+      <x:c r="B40" s="14" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="C40" s="14" t="str">
+        <x:v>DEV-024</x:v>
+      </x:c>
+      <x:c r="D40" s="14" t="str">
+        <x:v>更新服务故障恢复</x:v>
+      </x:c>
+      <x:c r="E40" s="14" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F40" s="14" t="str">
+        <x:v>模拟停服、超时、中断和空间不足后重试。</x:v>
+      </x:c>
+      <x:c r="G40" s="14" t="str">
+        <x:v>显示可恢复错误，本机报表可用，无损坏包残留。</x:v>
+      </x:c>
+      <x:c r="H40" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I40" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J40" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-035</x:v>
+      </x:c>
+      <x:c r="K40" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L40" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M40" s="14" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="70" customHeight="1">
+      <x:c r="A41" s="35" t="str">
+        <x:v>TC-036</x:v>
+      </x:c>
+      <x:c r="B41" s="35" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="C41" s="35" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="D41" s="35" t="str">
+        <x:v>未签名安装包交接</x:v>
+      </x:c>
+      <x:c r="E41" s="35" t="str">
+        <x:v>macOS 人工</x:v>
+      </x:c>
+      <x:c r="F41" s="35" t="str">
+        <x:v>未签名包通过校验后下载，选择打开/取消。</x:v>
+      </x:c>
+      <x:c r="G41" s="35" t="str">
+        <x:v>只打开安装包供用户安装；取消后旧版和数据仍可用。</x:v>
+      </x:c>
+      <x:c r="H41" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I41" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J41" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-036</x:v>
+      </x:c>
+      <x:c r="K41" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L41" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M41" s="35" t="str">
+        <x:v>实现后保存 macOS 人工 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="70" customHeight="1">
+      <x:c r="A42" s="14" t="str">
+        <x:v>TC-037</x:v>
+      </x:c>
+      <x:c r="B42" s="14" t="str">
+        <x:v>REQ-024</x:v>
+      </x:c>
+      <x:c r="C42" s="14" t="str">
+        <x:v>DEV-026</x:v>
+      </x:c>
+      <x:c r="D42" s="14" t="str">
+        <x:v>启动定时手动扫描与上传</x:v>
+      </x:c>
+      <x:c r="E42" s="14" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F42" s="14" t="str">
+        <x:v>假时钟推进 10 分钟，启动与手动扫描，加入并发/失败。</x:v>
+      </x:c>
+      <x:c r="G42" s="14" t="str">
+        <x:v>每次完整扫描后上报一次；并发串行，失败不报伪完整快照。</x:v>
+      </x:c>
+      <x:c r="H42" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I42" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J42" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-037</x:v>
+      </x:c>
+      <x:c r="K42" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L42" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M42" s="14" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="70" customHeight="1">
+      <x:c r="A43" s="35" t="str">
+        <x:v>TC-038</x:v>
+      </x:c>
+      <x:c r="B43" s="35" t="str">
+        <x:v>REQ-025</x:v>
+      </x:c>
+      <x:c r="C43" s="35" t="str">
+        <x:v>DEV-027</x:v>
+      </x:c>
+      <x:c r="D43" s="35" t="str">
+        <x:v>聚合载荷隐私和数值</x:v>
+      </x:c>
+      <x:c r="E43" s="35" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F43" s="35" t="str">
+        <x:v>构造含敏感正文/路径的记录，截获上传体。</x:v>
+      </x:c>
+      <x:c r="G43" s="35" t="str">
+        <x:v>仅允许字段存在，Token 与本机聚合一致。</x:v>
+      </x:c>
+      <x:c r="H43" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I43" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J43" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-038</x:v>
+      </x:c>
+      <x:c r="K43" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L43" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M43" s="35" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="70" customHeight="1">
+      <x:c r="A44" s="14" t="str">
+        <x:v>TC-039</x:v>
+      </x:c>
+      <x:c r="B44" s="14" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="C44" s="14" t="str">
+        <x:v>DEV-028</x:v>
+      </x:c>
+      <x:c r="D44" s="14" t="str">
+        <x:v>重复快照幂等</x:v>
+      </x:c>
+      <x:c r="E44" s="14" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F44" s="14" t="str">
+        <x:v>重复发送同键快照、修订快照并重启客户端。</x:v>
+      </x:c>
+      <x:c r="G44" s="14" t="str">
+        <x:v>服务端 upsert 后总量不累加重复项，修订值替换旧值。</x:v>
+      </x:c>
+      <x:c r="H44" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I44" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J44" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-039</x:v>
+      </x:c>
+      <x:c r="K44" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L44" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M44" s="14" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="70" customHeight="1">
+      <x:c r="A45" s="35" t="str">
+        <x:v>TC-040</x:v>
+      </x:c>
+      <x:c r="B45" s="35" t="str">
+        <x:v>REQ-026</x:v>
+      </x:c>
+      <x:c r="C45" s="35" t="str">
+        <x:v>DEV-028</x:v>
+      </x:c>
+      <x:c r="D45" s="35" t="str">
+        <x:v>离线重试与状态</x:v>
+      </x:c>
+      <x:c r="E45" s="35" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F45" s="35" t="str">
+        <x:v>停服完成扫描，检查积压并恢复服务。</x:v>
+      </x:c>
+      <x:c r="G45" s="35" t="str">
+        <x:v>有限退避补传，最近错误/成功及积压数量可见。</x:v>
+      </x:c>
+      <x:c r="H45" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I45" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J45" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-040</x:v>
+      </x:c>
+      <x:c r="K45" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L45" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M45" s="35" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="70" customHeight="1">
+      <x:c r="A46" s="14" t="str">
+        <x:v>TC-041</x:v>
+      </x:c>
+      <x:c r="B46" s="14" t="str">
+        <x:v>REQ-027</x:v>
+      </x:c>
+      <x:c r="C46" s="14" t="str">
+        <x:v>DEV-029</x:v>
+      </x:c>
+      <x:c r="D46" s="14" t="str">
+        <x:v>1024 单位与原值</x:v>
+      </x:c>
+      <x:c r="E46" s="14" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="str">
+        <x:v>检查 1023、1024、1024²、1024³ 边界、负值/未知及 CSV。</x:v>
+      </x:c>
+      <x:c r="G46" s="14" t="str">
+        <x:v>只按 K→M→P 逐级 1024 进位，不出现 G/T；原始 Token 整数未改。</x:v>
+      </x:c>
+      <x:c r="H46" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I46" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J46" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-041</x:v>
+      </x:c>
+      <x:c r="K46" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L46" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M46" s="14" t="str">
+        <x:v>实现后保存 单元 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="70" customHeight="1">
+      <x:c r="A47" s="35" t="str">
+        <x:v>TC-042</x:v>
+      </x:c>
+      <x:c r="B47" s="35" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="C47" s="35" t="str">
+        <x:v>DEV-030</x:v>
+      </x:c>
+      <x:c r="D47" s="35" t="str">
+        <x:v>概览指标与区间比较</x:v>
+      </x:c>
+      <x:c r="E47" s="35" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F47" s="35" t="str">
+        <x:v>两段脱敏数据切换用户、工具和日期。</x:v>
+      </x:c>
+      <x:c r="G47" s="35" t="str">
+        <x:v>总量与请求数同明细，比较基期缺失显示未知。</x:v>
+      </x:c>
+      <x:c r="H47" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I47" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J47" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-042</x:v>
+      </x:c>
+      <x:c r="K47" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L47" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M47" s="35" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="70" customHeight="1">
+      <x:c r="A48" s="14" t="str">
+        <x:v>TC-043</x:v>
+      </x:c>
+      <x:c r="B48" s="14" t="str">
+        <x:v>REQ-028</x:v>
+      </x:c>
+      <x:c r="C48" s="14" t="str">
+        <x:v>DEV-031</x:v>
+      </x:c>
+      <x:c r="D48" s="14" t="str">
+        <x:v>趋势筛选与下钻</x:v>
+      </x:c>
+      <x:c r="E48" s="14" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="str">
+        <x:v>切换日/周/月筛选并点击数据点。</x:v>
+      </x:c>
+      <x:c r="G48" s="14" t="str">
+        <x:v>趋势汇总与明细一致，下钻继承筛选和时区。</x:v>
+      </x:c>
+      <x:c r="H48" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I48" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J48" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-043</x:v>
+      </x:c>
+      <x:c r="K48" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L48" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M48" s="14" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="70" customHeight="1">
+      <x:c r="A49" s="35" t="str">
+        <x:v>TC-044</x:v>
+      </x:c>
+      <x:c r="B49" s="35" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="C49" s="35" t="str">
+        <x:v>DEV-031</x:v>
+      </x:c>
+      <x:c r="D49" s="35" t="str">
+        <x:v>模型排行与明细</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F49" s="35" t="str">
+        <x:v>构造多模型同值及未知模型，切换筛选后点排行。</x:v>
+      </x:c>
+      <x:c r="G49" s="35" t="str">
+        <x:v>按 Token 降序、同值稳定排序，点击明细数值一致。</x:v>
+      </x:c>
+      <x:c r="H49" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I49" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J49" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-044</x:v>
+      </x:c>
+      <x:c r="K49" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L49" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M49" s="35" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="70" customHeight="1">
+      <x:c r="A50" s="14" t="str">
+        <x:v>TC-045</x:v>
+      </x:c>
+      <x:c r="B50" s="14" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="C50" s="14" t="str">
+        <x:v>DEV-032</x:v>
+      </x:c>
+      <x:c r="D50" s="14" t="str">
+        <x:v>未覆盖与真实零区分</x:v>
+      </x:c>
+      <x:c r="E50" s="14" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F50" s="14" t="str">
+        <x:v>分别模拟已扫描无记录、未检测、权限失败。</x:v>
+      </x:c>
+      <x:c r="G50" s="14" t="str">
+        <x:v>零、未覆盖和错误状态独立且最后成功时间正确。</x:v>
+      </x:c>
+      <x:c r="H50" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I50" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J50" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-045</x:v>
+      </x:c>
+      <x:c r="K50" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L50" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M50" s="14" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="70" customHeight="1">
+      <x:c r="A51" s="35" t="str">
+        <x:v>TC-046</x:v>
+      </x:c>
+      <x:c r="B51" s="35" t="str">
+        <x:v>REQ-029</x:v>
+      </x:c>
+      <x:c r="C51" s="35" t="str">
+        <x:v>DEV-032</x:v>
+      </x:c>
+      <x:c r="D51" s="35" t="str">
+        <x:v>来源状态概览</x:v>
+      </x:c>
+      <x:c r="E51" s="35" t="str">
+        <x:v>端到端</x:v>
+      </x:c>
+      <x:c r="F51" s="35" t="str">
+        <x:v>模拟正常、等待、权限不足、格式不支持。</x:v>
+      </x:c>
+      <x:c r="G51" s="35" t="str">
+        <x:v>来源卡片显示状态、覆盖时间及可操作诊断。</x:v>
+      </x:c>
+      <x:c r="H51" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I51" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J51" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-046</x:v>
+      </x:c>
+      <x:c r="K51" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L51" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M51" s="35" t="str">
+        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="70" customHeight="1">
+      <x:c r="A52" s="14" t="str">
+        <x:v>TC-047</x:v>
+      </x:c>
+      <x:c r="B52" s="14" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="C52" s="14" t="str">
+        <x:v>DEV-023</x:v>
+      </x:c>
+      <x:c r="D52" s="14" t="str">
+        <x:v>聚合接口授权</x:v>
+      </x:c>
+      <x:c r="E52" s="14" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F52" s="14" t="str">
+        <x:v>携带错误/缺失凭证请求上传接口。</x:v>
+      </x:c>
+      <x:c r="G52" s="14" t="str">
+        <x:v>拒绝请求且不写入数据；有效凭证仅有最小权限。</x:v>
+      </x:c>
+      <x:c r="H52" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I52" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J52" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-047</x:v>
+      </x:c>
+      <x:c r="K52" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L52" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M52" s="14" t="str">
+        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="70" customHeight="1">
+      <x:c r="A53" s="35" t="str">
+        <x:v>TC-048</x:v>
+      </x:c>
+      <x:c r="B53" s="35" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="C53" s="35" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="D53" s="35" t="str">
+        <x:v>趋势图窗口缩放布局</x:v>
+      </x:c>
+      <x:c r="E53" s="35" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F53" s="35" t="str">
+        <x:v>在多组窄/宽窗口尺寸下绘制长日期和大数值柱图，调整窗口尺寸。</x:v>
+      </x:c>
+      <x:c r="G53" s="35" t="str">
+        <x:v>图形随容器宽度重排，柱顶数值与横轴标签不相交、不被裁切。</x:v>
+      </x:c>
+      <x:c r="H53" s="35" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I53" s="35" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J53" s="35" t="str">
+        <x:v>待注册：npm run test:case -- TC-048</x:v>
+      </x:c>
+      <x:c r="K53" s="35" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L53" s="35" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M53" s="35" t="str">
+        <x:v>实现后保存 Electron 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="70" customHeight="1">
+      <x:c r="A54" s="14" t="str">
+        <x:v>TC-049</x:v>
+      </x:c>
+      <x:c r="B54" s="14" t="str">
+        <x:v>REQ-030</x:v>
+      </x:c>
+      <x:c r="C54" s="14" t="str">
+        <x:v>DEV-033</x:v>
+      </x:c>
+      <x:c r="D54" s="14" t="str">
+        <x:v>周月横轴日期格式</x:v>
+      </x:c>
+      <x:c r="E54" s="14" t="str">
+        <x:v>单元+端到端</x:v>
+      </x:c>
+      <x:c r="F54" s="14" t="str">
+        <x:v>构造 ISO 跨年周及跨月样本，切换周/月并点击柱。</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="str">
+        <x:v>周标签是该周周一 YYYY-MM-DD，月标签 YYYY-MM；点击分桶和报表区间一致。</x:v>
+      </x:c>
+      <x:c r="H54" s="14" t="str">
+        <x:v>待验证</x:v>
+      </x:c>
+      <x:c r="I54" s="14" t="str">
+        <x:v>尚未实现；待留脱敏执行证据</x:v>
+      </x:c>
+      <x:c r="J54" s="14" t="str">
+        <x:v>待注册：npm run test:case -- TC-049</x:v>
+      </x:c>
+      <x:c r="K54" s="14" t="str">
+        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+      </x:c>
+      <x:c r="L54" s="14" t="str">
+        <x:v>未自动化；不可执行</x:v>
+      </x:c>
+      <x:c r="M54" s="14" t="str">
+        <x:v>实现后保存 单元+端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Allow configurable update server addresses in docs
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R0c1fa1c217164d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rddde2b5fa22645cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R8c4ec72069f645ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd03d2509fa004398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R80a7a7fc69844bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7b29771011534867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce351779b18546ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R08edb4b33a544803"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1244,7 +1244,7 @@
         <x:v>TC-032</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
-        <x:v>独立服务回环绑定</x:v>
+        <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
         <x:v>待验证（计划）</x:v>
@@ -2274,7 +2274,7 @@
         <x:v>独立本地更新与汇总服务</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>提供独立进程，默认仅绑定 127.0.0.1；明确版本清单、安装包和聚合接收接口；非回环访问拒绝，管理/上报接口需授权；服务故障不影响本机报表。</x:v>
+        <x:v>服务独立运行；监听主机/端口及 App 连接地址均可配置，默认 127.0.0.1；提供版本清单、安装包和聚合接口；非回环配置仍须鉴权并保护传输；服务故障不影响本机报表。</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>M5（计划）</x:v>
@@ -3104,7 +3104,7 @@
         <x:v>待启动</x:v>
       </x:c>
       <x:c r="G27" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>M5 计划；监听地址与 App 连接地址可配置、默认 127.0.0.1；需注册对应 TC 并实测</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
@@ -4750,16 +4750,16 @@
         <x:v>DEV-022</x:v>
       </x:c>
       <x:c r="D37" s="35" t="str">
-        <x:v>独立服务回环绑定</x:v>
+        <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="E37" s="35" t="str">
         <x:v>集成</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
-        <x:v>独立启动服务，从回环和非回环地址请求清单。</x:v>
+        <x:v>独立启停服务；验证默认监听/连接地址，显式配置其他地址，再测试地址不匹配。</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>回环可访问，非回环不能连接；停服不影响本机报表。</x:v>
+        <x:v>默认双方使用 127.0.0.1；配置匹配时可连，错误地址有可恢复状态；停服不影响本机报表。</x:v>
       </x:c>
       <x:c r="H37" s="35" t="str">
         <x:v>待验证</x:v>
@@ -4777,7 +4777,7 @@
         <x:v>未自动化；不可执行</x:v>
       </x:c>
       <x:c r="M37" s="35" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>保存监听配置、App 连接地址、成功/失败连接及停服后的报表证据；不要求仅回环可连。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
@@ -5371,10 +5371,10 @@
         <x:v>集成</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>携带错误/缺失凭证请求上传接口。</x:v>
+        <x:v>在默认及非回环配置下，以缺失/错误/正确凭证请求清单、包和上报接口，并尝试跨用户覆盖。</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>拒绝请求且不写入数据；有效凭证仅有最小权限。</x:v>
+        <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
         <x:v>待验证</x:v>

</xml_diff>

<commit_message>
Document M5 implementation and acceptance evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R80a7a7fc69844bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7b29771011534867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce351779b18546ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R08edb4b33a544803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R84c121e875b440ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Reaa419cada8f412f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc767b26c801f445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R1a2b00ba4eae4db0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1178,7 +1178,7 @@
         <x:v>CSV 表头与数据列对齐</x:v>
       </x:c>
       <x:c r="G34" s="12" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
@@ -1201,7 +1201,7 @@
         <x:v>信任设备恢复登录</x:v>
       </x:c>
       <x:c r="G35" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -1224,7 +1224,7 @@
         <x:v>信任撤销与账户失效</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
@@ -1247,7 +1247,7 @@
         <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
@@ -1270,7 +1270,7 @@
         <x:v>版本清单和安装包</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="62" customHeight="1">
@@ -1293,7 +1293,7 @@
         <x:v>更新版本判断与下载校验</x:v>
       </x:c>
       <x:c r="G39" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1316,7 +1316,7 @@
         <x:v>更新服务故障恢复</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1339,7 +1339,7 @@
         <x:v>未签名安装包交接</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -1362,7 +1362,7 @@
         <x:v>启动定时手动扫描与上传</x:v>
       </x:c>
       <x:c r="G42" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="62" customHeight="1">
@@ -1385,7 +1385,7 @@
         <x:v>聚合载荷隐私和数值</x:v>
       </x:c>
       <x:c r="G43" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="62" customHeight="1">
@@ -1408,7 +1408,7 @@
         <x:v>重复快照幂等</x:v>
       </x:c>
       <x:c r="G44" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="62" customHeight="1">
@@ -1431,7 +1431,7 @@
         <x:v>离线重试与状态</x:v>
       </x:c>
       <x:c r="G45" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="62" customHeight="1">
@@ -1454,7 +1454,7 @@
         <x:v>1024 单位与原值</x:v>
       </x:c>
       <x:c r="G46" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="62" customHeight="1">
@@ -1477,7 +1477,7 @@
         <x:v>概览指标与区间比较</x:v>
       </x:c>
       <x:c r="G47" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="62" customHeight="1">
@@ -1500,7 +1500,7 @@
         <x:v>趋势筛选与下钻</x:v>
       </x:c>
       <x:c r="G48" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="62" customHeight="1">
@@ -1523,7 +1523,7 @@
         <x:v>模型排行与明细</x:v>
       </x:c>
       <x:c r="G49" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="62" customHeight="1">
@@ -1546,7 +1546,7 @@
         <x:v>未覆盖与真实零区分</x:v>
       </x:c>
       <x:c r="G50" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="62" customHeight="1">
@@ -1569,7 +1569,7 @@
         <x:v>来源状态概览</x:v>
       </x:c>
       <x:c r="G51" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="62" customHeight="1">
@@ -1592,7 +1592,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -1615,7 +1615,7 @@
         <x:v>趋势图窗口缩放布局</x:v>
       </x:c>
       <x:c r="G53" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="62" customHeight="1">
@@ -1638,7 +1638,7 @@
         <x:v>周月横轴日期格式</x:v>
       </x:c>
       <x:c r="G54" s="14" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="62" customHeight="1">
@@ -1661,7 +1661,7 @@
         <x:v>重复快照幂等</x:v>
       </x:c>
       <x:c r="G55" s="35" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1700,7 +1700,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–018 为原版；REQ-019–030 是 M5 计划，尚未实现。</x:v>
+        <x:v>REQ-001–030；M5 已有代码与自动测试，完整验收状态见需求列和逐项验收文档。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2098,7 +2098,7 @@
         <x:v>M3</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>部分实现（列头待修）</x:v>
+        <x:v>已验证（自动）</x:v>
       </x:c>
       <x:c r="F19" s="10" t="str">
         <x:v>DEV-014、DEV-019</x:v>
@@ -2228,7 +2228,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E24" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
         <x:v>DEV-020</x:v>
@@ -2254,7 +2254,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E25" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
         <x:v>DEV-021</x:v>
@@ -2280,7 +2280,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>DEV-022、DEV-023</x:v>
@@ -2306,7 +2306,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>DEV-024</x:v>
@@ -2332,7 +2332,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -2358,7 +2358,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E29" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
         <x:v>DEV-026</x:v>
@@ -2384,7 +2384,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
         <x:v>DEV-027</x:v>
@@ -2410,7 +2410,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E31" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
         <x:v>DEV-028、DEV-023</x:v>
@@ -2436,7 +2436,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
         <x:v>DEV-029</x:v>
@@ -2462,7 +2462,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E33" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
         <x:v>DEV-030、DEV-031</x:v>
@@ -2488,7 +2488,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
         <x:v>DEV-031、DEV-032</x:v>
@@ -2514,7 +2514,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E35" s="35" t="str">
-        <x:v>待实现</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
         <x:v>DEV-033</x:v>
@@ -3029,13 +3029,13 @@
         <x:v>TC-029</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>src/main/report.ts；tests/report.test.ts</x:v>
+        <x:v>src/main/report.ts；tests/next-report.test.ts</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已完成（自动）</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>当前表头 8 列，数据行 9 列；补总 Token 列头和结构断言</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="62" customHeight="1">
@@ -3052,13 +3052,13 @@
         <x:v>TC-030</x:v>
       </x:c>
       <x:c r="E25" s="35" t="str">
-        <x:v>src/main/auth.ts；src/renderer/index.tsx；系统安全存储</x:v>
+        <x:v>src/main/auth.ts；src/main/trusted-device.ts；tests/next-auth.test.ts；tests/e2e/trust.spec.ts</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G25" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="62" customHeight="1">
@@ -3075,13 +3075,13 @@
         <x:v>TC-031</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>src/main/auth.ts；src/renderer/settings.tsx</x:v>
+        <x:v>src/main/auth.ts；src/main/trusted-device.ts；tests/next-auth.test.ts</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -3098,13 +3098,13 @@
         <x:v>TC-032、TC-033</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>server/</x:v>
+        <x:v>src/server/server.ts；src/server/cli.ts；src/main/server-connection.ts；tests/next-server.test.ts</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G27" s="35" t="str">
-        <x:v>M5 计划；监听地址与 App 连接地址可配置、默认 127.0.0.1；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
@@ -3121,13 +3121,13 @@
         <x:v>TC-039、TC-047</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>server/；SQLite</x:v>
+        <x:v>src/server/server.ts；tests/next-server.test.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -3144,13 +3144,13 @@
         <x:v>TC-034、TC-035</x:v>
       </x:c>
       <x:c r="E29" s="35" t="str">
-        <x:v>src/main/update.ts；src/preload</x:v>
+        <x:v>src/main/update-client.ts；src/main/server-connection.ts；tests/next-update.test.ts</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G29" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -3167,13 +3167,13 @@
         <x:v>TC-036</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>src/main/update.ts</x:v>
+        <x:v>src/main/update-client.ts；tests/next-update.test.ts</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -3190,13 +3190,13 @@
         <x:v>TC-037</x:v>
       </x:c>
       <x:c r="E31" s="35" t="str">
-        <x:v>src/collectors/scanner.ts</x:v>
+        <x:v>src/collectors/scanner.ts；src/main/index.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G31" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -3213,13 +3213,13 @@
         <x:v>TC-038</x:v>
       </x:c>
       <x:c r="E32" s="14" t="str">
-        <x:v>src/main/report.ts；src/main/upload.ts</x:v>
+        <x:v>src/main/usage-sync.ts；tests/next-sync.test.ts；tests/e2e/upload.spec.ts</x:v>
       </x:c>
       <x:c r="F32" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G32" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="62" customHeight="1">
@@ -3236,13 +3236,13 @@
         <x:v>TC-039、TC-040</x:v>
       </x:c>
       <x:c r="E33" s="35" t="str">
-        <x:v>src/main/upload.ts；SQLite 迁移</x:v>
+        <x:v>src/main/usage-sync.ts；src/server/server.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G33" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -3259,13 +3259,13 @@
         <x:v>TC-041</x:v>
       </x:c>
       <x:c r="E34" s="14" t="str">
-        <x:v>src/renderer/format.ts</x:v>
+        <x:v>src/renderer/format.ts；tests/next-report.test.ts</x:v>
       </x:c>
       <x:c r="F34" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G34" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="62" customHeight="1">
@@ -3282,13 +3282,13 @@
         <x:v>TC-042</x:v>
       </x:c>
       <x:c r="E35" s="35" t="str">
-        <x:v>src/renderer/index.tsx</x:v>
+        <x:v>src/renderer/overview.tsx；src/renderer/index.tsx；tests/next-report.test.ts</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G35" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
@@ -3305,13 +3305,13 @@
         <x:v>TC-043、TC-044</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
-        <x:v>src/renderer/report.tsx</x:v>
+        <x:v>src/renderer/report.tsx；tests/next-report.test.ts</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G36" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="62" customHeight="1">
@@ -3328,13 +3328,13 @@
         <x:v>TC-045、TC-046</x:v>
       </x:c>
       <x:c r="E37" s="35" t="str">
-        <x:v>src/renderer/index.tsx</x:v>
+        <x:v>src/renderer/overview.tsx；tests/next-report.test.ts</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
@@ -3351,13 +3351,13 @@
         <x:v>TC-048、TC-049</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>src/renderer/report.tsx；src/renderer/styles.css</x:v>
+        <x:v>src/renderer/report.tsx；src/renderer/style.css；tests/e2e/trend.spec.ts</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G38" s="14" t="str">
-        <x:v>M5 计划；需注册对应 TC 并实测</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3402,7 +3402,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–029 有现行入口；TC-030–049 待注册/实现，不能标记为通过。</x:v>
+        <x:v>TC-001–049 均有入口；TC-029 已自动化，TC-030–049 的覆盖边界见 docs/test-case-acceptance.md。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4639,22 +4639,22 @@
         <x:v>每行 9 列，列名与数值语义一一对应。</x:v>
       </x:c>
       <x:c r="H34" s="12" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动）</x:v>
       </x:c>
       <x:c r="I34" s="9" t="str">
-        <x:v>src/main/report.ts 当前表头 8 列、数据行 9 列</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
         <x:v>npm run test:case -- TC-029</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
-        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-029 CSV 表头和数据列对齐')</x:v>
       </x:c>
       <x:c r="L34" s="30" t="str">
-        <x:v>已知缺陷；禁止通过</x:v>
+        <x:v>固定一行 9 列与总 Token/记录数；复杂 CSV 转义另见 TC-023</x:v>
       </x:c>
       <x:c r="M34" s="9" t="str">
-        <x:v>脱敏 CSV 表头/行列数对比与解析结果；修复前仅可记录 fail，不得记录 pass。</x:v>
+        <x:v>记录 TC-029 命令、退出码、提交、环境和脱敏日志；覆盖与限制：固定一行 9 列与总 Token/记录数；复杂 CSV 转义另见 TC-023。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="70" customHeight="1">
@@ -4671,7 +4671,7 @@
         <x:v>信任设备恢复登录</x:v>
       </x:c>
       <x:c r="E35" s="35" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元+Electron</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
         <x:v>临时账户首次登录勾选信任，关闭并重启应用。</x:v>
@@ -4680,22 +4680,23 @@
         <x:v>自动登录同一用户且磁盘无明文密码。</x:v>
       </x:c>
       <x:c r="H35" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I35" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J35" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-030</x:v>
+        <x:v>npm run test:case -- TC-030</x:v>
       </x:c>
       <x:c r="K35" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-auth.test.ts：test('TC-030 勾选信任后重启恢复且未勾选不恢复')
+tests/e2e/trust.spec.ts：test('TC-030 应用重启自动登录并在退出后撤销')</x:v>
       </x:c>
       <x:c r="L35" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>单元与 Electron 重启/退出；未测另一 macOS 账户</x:v>
       </x:c>
       <x:c r="M35" s="35" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-030 命令、退出码、提交、环境和脱敏日志；覆盖与限制：单元与 Electron 重启/退出；未测另一 macOS 账户。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="70" customHeight="1">
@@ -4712,7 +4713,7 @@
         <x:v>信任撤销与账户失效</x:v>
       </x:c>
       <x:c r="E36" s="14" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F36" s="14" t="str">
         <x:v>信任后分别退出/撤销、禁用、重置密码并重启。</x:v>
@@ -4721,22 +4722,22 @@
         <x:v>所有旧令牌失效，回到登录页；损坏令牌可恢复。</x:v>
       </x:c>
       <x:c r="H36" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I36" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J36" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-031</x:v>
+        <x:v>npm run test:case -- TC-031</x:v>
       </x:c>
       <x:c r="K36" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-auth.test.ts：test('TC-031 退出停用重置密码撤销受信凭证')</x:v>
       </x:c>
       <x:c r="L36" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>无固定过期、撤销/停用/重置密码；未测全部管理界面操作</x:v>
       </x:c>
       <x:c r="M36" s="14" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-031 命令、退出码、提交、环境和脱敏日志；覆盖与限制：无固定过期、撤销/停用/重置密码；未测全部管理界面操作。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="70" customHeight="1">
@@ -4753,7 +4754,7 @@
         <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="E37" s="35" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
         <x:v>独立启停服务；验证默认监听/连接地址，显式配置其他地址，再测试地址不匹配。</x:v>
@@ -4762,22 +4763,22 @@
         <x:v>默认双方使用 127.0.0.1；配置匹配时可连，错误地址有可恢复状态；停服不影响本机报表。</x:v>
       </x:c>
       <x:c r="H37" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I37" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J37" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-032</x:v>
+        <x:v>npm run test:case -- TC-032</x:v>
       </x:c>
       <x:c r="K37" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-032 服务默认地址可配置且停服不影响本机数据库')</x:v>
       </x:c>
       <x:c r="L37" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配</x:v>
       </x:c>
       <x:c r="M37" s="35" t="str">
-        <x:v>保存监听配置、App 连接地址、成功/失败连接及停服后的报表证据；不要求仅回环可连。</x:v>
+        <x:v>记录 TC-032 命令、退出码、提交、环境和脱敏日志；覆盖与限制：默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
@@ -4794,7 +4795,7 @@
         <x:v>版本清单和安装包</x:v>
       </x:c>
       <x:c r="E38" s="14" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F38" s="14" t="str">
         <x:v>发布测试版本及安装包，请求清单和下载流。</x:v>
@@ -4803,22 +4804,22 @@
         <x:v>版本、平台、长度、摘要及文件内容匹配。</x:v>
       </x:c>
       <x:c r="H38" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I38" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J38" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-033</x:v>
+        <x:v>npm run test:case -- TC-033</x:v>
       </x:c>
       <x:c r="K38" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-033 更新清单与包哈希一致且拒绝路径穿越')</x:v>
       </x:c>
       <x:c r="L38" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>合成包清单/哈希/路径穿越；未测真实发布 DMG</x:v>
       </x:c>
       <x:c r="M38" s="14" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-033 命令、退出码、提交、环境和脱敏日志；覆盖与限制：合成包清单/哈希/路径穿越；未测真实发布 DMG。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="70" customHeight="1">
@@ -4835,7 +4836,7 @@
         <x:v>更新版本判断与下载校验</x:v>
       </x:c>
       <x:c r="E39" s="35" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F39" s="35" t="str">
         <x:v>模拟新/同/旧版本和正确/错误 SHA-256。</x:v>
@@ -4844,22 +4845,22 @@
         <x:v>仅新且匹配版本提示；错误摘要不得打开文件。</x:v>
       </x:c>
       <x:c r="H39" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I39" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J39" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-034</x:v>
+        <x:v>npm run test:case -- TC-034</x:v>
       </x:c>
       <x:c r="K39" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-034 只提示较新且架构匹配的版本并校验包摘要')</x:v>
       </x:c>
       <x:c r="L39" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>版本、架构、坏摘要；合成包路径</x:v>
       </x:c>
       <x:c r="M39" s="35" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-034 命令、退出码、提交、环境和脱敏日志；覆盖与限制：版本、架构、坏摘要；合成包路径。</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="70" customHeight="1">
@@ -4876,7 +4877,7 @@
         <x:v>更新服务故障恢复</x:v>
       </x:c>
       <x:c r="E40" s="14" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
         <x:v>模拟停服、超时、中断和空间不足后重试。</x:v>
@@ -4885,22 +4886,22 @@
         <x:v>显示可恢复错误，本机报表可用，无损坏包残留。</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J40" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-035</x:v>
+        <x:v>npm run test:case -- TC-035</x:v>
       </x:c>
       <x:c r="K40" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-035 停服和下载失败可重试且不留临时包')</x:v>
       </x:c>
       <x:c r="L40" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>停服/重试/临时文件；未测超时、磁盘不足</x:v>
       </x:c>
       <x:c r="M40" s="14" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-035 命令、退出码、提交、环境和脱敏日志；覆盖与限制：停服/重试/临时文件；未测超时、磁盘不足。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="70" customHeight="1">
@@ -4917,7 +4918,7 @@
         <x:v>未签名安装包交接</x:v>
       </x:c>
       <x:c r="E41" s="35" t="str">
-        <x:v>macOS 人工</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
         <x:v>未签名包通过校验后下载，选择打开/取消。</x:v>
@@ -4926,22 +4927,22 @@
         <x:v>只打开安装包供用户安装；取消后旧版和数据仍可用。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-036</x:v>
+        <x:v>npm run test:case -- TC-036</x:v>
       </x:c>
       <x:c r="K41" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>注入打开回调和旧文件；未测真实 Mac 打开/取消安装</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>实现后保存 macOS 人工 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-036 命令、退出码、提交、环境和脱敏日志；覆盖与限制：注入打开回调和旧文件；未测真实 Mac 打开/取消安装。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">
@@ -4958,7 +4959,7 @@
         <x:v>启动定时手动扫描与上传</x:v>
       </x:c>
       <x:c r="E42" s="14" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F42" s="14" t="str">
         <x:v>假时钟推进 10 分钟，启动与手动扫描，加入并发/失败。</x:v>
@@ -4967,22 +4968,22 @@
         <x:v>每次完整扫描后上报一次；并发串行，失败不报伪完整快照。</x:v>
       </x:c>
       <x:c r="H42" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I42" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J42" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-037</x:v>
+        <x:v>npm run test:case -- TC-037</x:v>
       </x:c>
       <x:c r="K42" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-sync.test.ts：test('TC-037 启动及十分钟定时扫描并串行执行')</x:v>
       </x:c>
       <x:c r="L42" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>假时钟三种扫描触发；mock 扫描，未单测并发/失败上传</x:v>
       </x:c>
       <x:c r="M42" s="14" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-037 命令、退出码、提交、环境和脱敏日志；覆盖与限制：假时钟三种扫描触发；mock 扫描，未单测并发/失败上传。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="70" customHeight="1">
@@ -4999,7 +5000,7 @@
         <x:v>聚合载荷隐私和数值</x:v>
       </x:c>
       <x:c r="E43" s="35" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元+Electron</x:v>
       </x:c>
       <x:c r="F43" s="35" t="str">
         <x:v>构造含敏感正文/路径的记录，截获上传体。</x:v>
@@ -5008,22 +5009,23 @@
         <x:v>仅允许字段存在，Token 与本机聚合一致。</x:v>
       </x:c>
       <x:c r="H43" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I43" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J43" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-038</x:v>
+        <x:v>npm run test:case -- TC-038</x:v>
       </x:c>
       <x:c r="K43" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-sync.test.ts：test('TC-038 聚合上报只含授权用量字段不含正文路径密钥')
+tests/e2e/upload.spec.ts：test('TC-038 应用扫描后自动上报到独立本机服务')</x:v>
       </x:c>
       <x:c r="L43" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>单元隐私与 Electron 扫描上报；未覆盖全部敏感样本</x:v>
       </x:c>
       <x:c r="M43" s="35" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-038 命令、退出码、提交、环境和脱敏日志；覆盖与限制：单元隐私与 Electron 扫描上报；未覆盖全部敏感样本。</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="70" customHeight="1">
@@ -5040,7 +5042,7 @@
         <x:v>重复快照幂等</x:v>
       </x:c>
       <x:c r="E44" s="14" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F44" s="14" t="str">
         <x:v>重复发送同键快照、修订快照并重启客户端。</x:v>
@@ -5049,22 +5051,22 @@
         <x:v>服务端 upsert 后总量不累加重复项，修订值替换旧值。</x:v>
       </x:c>
       <x:c r="H44" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J44" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-039</x:v>
+        <x:v>npm run test:case -- TC-039</x:v>
       </x:c>
       <x:c r="K44" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-sync.test.ts：test('TC-039 重复上报幂等且修订快照替换旧值')</x:v>
       </x:c>
       <x:c r="L44" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>重复快照和修订替换；未测多设备并发</x:v>
       </x:c>
       <x:c r="M44" s="14" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-039 命令、退出码、提交、环境和脱敏日志；覆盖与限制：重复快照和修订替换；未测多设备并发。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="70" customHeight="1">
@@ -5081,7 +5083,7 @@
         <x:v>离线重试与状态</x:v>
       </x:c>
       <x:c r="E45" s="35" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F45" s="35" t="str">
         <x:v>停服完成扫描，检查积压并恢复服务。</x:v>
@@ -5090,22 +5092,22 @@
         <x:v>有限退避补传，最近错误/成功及积压数量可见。</x:v>
       </x:c>
       <x:c r="H45" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I45" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J45" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-040</x:v>
+        <x:v>npm run test:case -- TC-040</x:v>
       </x:c>
       <x:c r="K45" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-sync.test.ts：test('TC-040 停服后待传快照持久化并恢复补传')</x:v>
       </x:c>
       <x:c r="L45" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>持久待传和恢复补传；未长时间运行验证退避</x:v>
       </x:c>
       <x:c r="M45" s="35" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-040 命令、退出码、提交、环境和脱敏日志；覆盖与限制：持久待传和恢复补传；未长时间运行验证退避。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="70" customHeight="1">
@@ -5131,22 +5133,22 @@
         <x:v>只按 K→M→P 逐级 1024 进位，不出现 G/T；原始 Token 整数未改。</x:v>
       </x:c>
       <x:c r="H46" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I46" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J46" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-041</x:v>
+        <x:v>npm run test:case -- TC-041</x:v>
       </x:c>
       <x:c r="K46" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-041 K M P 1024 进位且原值保留在 CSV')</x:v>
       </x:c>
       <x:c r="L46" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>K/M/P 边界及 CSV 原值；未测超安全整数</x:v>
       </x:c>
       <x:c r="M46" s="14" t="str">
-        <x:v>实现后保存 单元 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-041 命令、退出码、提交、环境和脱敏日志；覆盖与限制：K/M/P 边界及 CSV 原值；未测超安全整数。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="70" customHeight="1">
@@ -5163,7 +5165,7 @@
         <x:v>概览指标与区间比较</x:v>
       </x:c>
       <x:c r="E47" s="35" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F47" s="35" t="str">
         <x:v>两段脱敏数据切换用户、工具和日期。</x:v>
@@ -5172,22 +5174,22 @@
         <x:v>总量与请求数同明细，比较基期缺失显示未知。</x:v>
       </x:c>
       <x:c r="H47" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I47" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J47" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-042</x:v>
+        <x:v>npm run test:case -- TC-042</x:v>
       </x:c>
       <x:c r="K47" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-042 概览等长区间比较与未知基期')</x:v>
       </x:c>
       <x:c r="L47" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>等长区间与文案；未测全部界面筛选</x:v>
       </x:c>
       <x:c r="M47" s="35" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-042 命令、退出码、提交、环境和脱敏日志；覆盖与限制：等长区间与文案；未测全部界面筛选。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="70" customHeight="1">
@@ -5204,7 +5206,7 @@
         <x:v>趋势筛选与下钻</x:v>
       </x:c>
       <x:c r="E48" s="14" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F48" s="14" t="str">
         <x:v>切换日/周/月筛选并点击数据点。</x:v>
@@ -5213,22 +5215,22 @@
         <x:v>趋势汇总与明细一致，下钻继承筛选和时区。</x:v>
       </x:c>
       <x:c r="H48" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I48" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J48" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-043</x:v>
+        <x:v>npm run test:case -- TC-043</x:v>
       </x:c>
       <x:c r="K48" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-043 日周月趋势点击下钻保持同一时间桶')</x:v>
       </x:c>
       <x:c r="L48" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>日周月点/明细求和；未测全部时区</x:v>
       </x:c>
       <x:c r="M48" s="14" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-043 命令、退出码、提交、环境和脱敏日志；覆盖与限制：日周月点/明细求和；未测全部时区。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="70" customHeight="1">
@@ -5245,7 +5247,7 @@
         <x:v>模型排行与明细</x:v>
       </x:c>
       <x:c r="E49" s="35" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F49" s="35" t="str">
         <x:v>构造多模型同值及未知模型，切换筛选后点排行。</x:v>
@@ -5254,22 +5256,22 @@
         <x:v>按 Token 降序、同值稳定排序，点击明细数值一致。</x:v>
       </x:c>
       <x:c r="H49" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I49" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J49" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-044</x:v>
+        <x:v>npm run test:case -- TC-044</x:v>
       </x:c>
       <x:c r="K49" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-044 模型排行总量降序且同值稳定')</x:v>
       </x:c>
       <x:c r="L49" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>排序/同值/明细；未测未知模型和界面点击</x:v>
       </x:c>
       <x:c r="M49" s="35" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-044 命令、退出码、提交、环境和脱敏日志；覆盖与限制：排序/同值/明细；未测未知模型和界面点击。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="70" customHeight="1">
@@ -5286,7 +5288,7 @@
         <x:v>未覆盖与真实零区分</x:v>
       </x:c>
       <x:c r="E50" s="14" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F50" s="14" t="str">
         <x:v>分别模拟已扫描无记录、未检测、权限失败。</x:v>
@@ -5295,22 +5297,22 @@
         <x:v>零、未覆盖和错误状态独立且最后成功时间正确。</x:v>
       </x:c>
       <x:c r="H50" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J50" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-045</x:v>
+        <x:v>npm run test:case -- TC-045</x:v>
       </x:c>
       <x:c r="K50" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-045 已覆盖零与未覆盖错误状态分开显示')</x:v>
       </x:c>
       <x:c r="L50" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>零/错误状态；未测全部界面缺失/权限状态</x:v>
       </x:c>
       <x:c r="M50" s="14" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-045 命令、退出码、提交、环境和脱敏日志；覆盖与限制：零/错误状态；未测全部界面缺失/权限状态。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="70" customHeight="1">
@@ -5327,7 +5329,7 @@
         <x:v>来源状态概览</x:v>
       </x:c>
       <x:c r="E51" s="35" t="str">
-        <x:v>端到端</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F51" s="35" t="str">
         <x:v>模拟正常、等待、权限不足、格式不支持。</x:v>
@@ -5336,22 +5338,22 @@
         <x:v>来源卡片显示状态、覆盖时间及可操作诊断。</x:v>
       </x:c>
       <x:c r="H51" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I51" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J51" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-046</x:v>
+        <x:v>npm run test:case -- TC-046</x:v>
       </x:c>
       <x:c r="K51" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-report.test.ts：test('TC-046 来源状态和最近扫描时间一致')</x:v>
       </x:c>
       <x:c r="L51" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>事实数/扫描时间/缺目录；未测全部状态卡片</x:v>
       </x:c>
       <x:c r="M51" s="35" t="str">
-        <x:v>实现后保存 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-046 命令、退出码、提交、环境和脱敏日志；覆盖与限制：事实数/扫描时间/缺目录；未测全部状态卡片。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="70" customHeight="1">
@@ -5368,7 +5370,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="E52" s="14" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
         <x:v>在默认及非回环配置下，以缺失/错误/正确凭证请求清单、包和上报接口，并尝试跨用户覆盖。</x:v>
@@ -5377,22 +5379,22 @@
         <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J52" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-047</x:v>
+        <x:v>npm run test:case -- TC-047</x:v>
       </x:c>
       <x:c r="K52" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')</x:v>
       </x:c>
       <x:c r="L52" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>凭证/字段/Origin/HTTPS 地址；未在非回环 HTTPS 连接上验鉴权及跨用户授权</x:v>
       </x:c>
       <x:c r="M52" s="14" t="str">
-        <x:v>实现后保存 集成 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-047 命令、退出码、提交、环境和脱敏日志；覆盖与限制：凭证/字段/Origin/HTTPS 地址；未在非回环 HTTPS 连接上验鉴权及跨用户授权。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="70" customHeight="1">
@@ -5418,22 +5420,22 @@
         <x:v>图形随容器宽度重排，柱顶数值与横轴标签不相交、不被裁切。</x:v>
       </x:c>
       <x:c r="H53" s="35" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I53" s="35" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J53" s="35" t="str">
-        <x:v>待注册：npm run test:case -- TC-048</x:v>
+        <x:v>npm run test:case -- TC-048</x:v>
       </x:c>
       <x:c r="K53" s="35" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/e2e/trend.spec.ts：test('TC-048 趋势图宽窄窗口自适应且数值日期不重叠')</x:v>
       </x:c>
       <x:c r="L53" s="35" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>1180/860 两种窗口与边界框；未测更窄或字体裁切</x:v>
       </x:c>
       <x:c r="M53" s="35" t="str">
-        <x:v>实现后保存 Electron 端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-048 命令、退出码、提交、环境和脱敏日志；覆盖与限制：1180/860 两种窗口与边界框；未测更窄或字体裁切。</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="70" customHeight="1">
@@ -5450,7 +5452,7 @@
         <x:v>周月横轴日期格式</x:v>
       </x:c>
       <x:c r="E54" s="14" t="str">
-        <x:v>单元+端到端</x:v>
+        <x:v>Electron 端到端</x:v>
       </x:c>
       <x:c r="F54" s="14" t="str">
         <x:v>构造 ISO 跨年周及跨月样本，切换周/月并点击柱。</x:v>
@@ -5459,22 +5461,22 @@
         <x:v>周标签是该周周一 YYYY-MM-DD，月标签 YYYY-MM；点击分桶和报表区间一致。</x:v>
       </x:c>
       <x:c r="H54" s="14" t="str">
-        <x:v>待验证</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I54" s="14" t="str">
-        <x:v>尚未实现；待留脱敏执行证据</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J54" s="14" t="str">
-        <x:v>待注册：npm run test:case -- TC-049</x:v>
+        <x:v>npm run test:case -- TC-049</x:v>
       </x:c>
       <x:c r="K54" s="14" t="str">
-        <x:v>scripts/test-cases.mjs 尚无该编号</x:v>
+        <x:v>tests/e2e/trend.spec.ts：test('TC-049 周横轴显示周一日期月横轴显示年月且下钻一致')</x:v>
       </x:c>
       <x:c r="L54" s="14" t="str">
-        <x:v>未自动化；不可执行</x:v>
+        <x:v>跨年周/月标签及点击；未测其他时区/长期跨度</x:v>
       </x:c>
       <x:c r="M54" s="14" t="str">
-        <x:v>实现后保存 单元+端到端 运行日志、提交、环境和脱敏断言；不得用计划代替通过。</x:v>
+        <x:v>记录 TC-049 命令、退出码、提交、环境和脱敏日志；覆盖与限制：跨年周/月标签及点击；未测其他时区/长期跨度。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: plan M6 product scope and traceable acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R84c121e875b440ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Reaa419cada8f412f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc767b26c801f445b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R1a2b00ba4eae4db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3eb70382dfd64eda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R623952fe022a4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7e34ee02e4ee4f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R522c444409674d2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="15">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -129,6 +129,16 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -141,7 +151,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="38">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -244,6 +254,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1664,6 +1680,535 @@
         <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
+    <x:row r="56" ht="66" customHeight="1">
+      <x:c r="A56" s="36" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="B56" s="36" t="str">
+        <x:v>会话工作目录识别项目与本机隐私</x:v>
+      </x:c>
+      <x:c r="C56" s="36" t="str">
+        <x:v>DEV-034</x:v>
+      </x:c>
+      <x:c r="D56" s="36" t="str">
+        <x:v>解析 Codex/Claude 会话工作目录</x:v>
+      </x:c>
+      <x:c r="E56" s="36" t="str">
+        <x:v>TC-050</x:v>
+      </x:c>
+      <x:c r="F56" s="36" t="str">
+        <x:v>Codex 工作目录识别</x:v>
+      </x:c>
+      <x:c r="G56" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="66" customHeight="1">
+      <x:c r="A57" s="37" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="B57" s="37" t="str">
+        <x:v>会话工作目录识别项目与本机隐私</x:v>
+      </x:c>
+      <x:c r="C57" s="37" t="str">
+        <x:v>DEV-034</x:v>
+      </x:c>
+      <x:c r="D57" s="37" t="str">
+        <x:v>解析 Codex/Claude 会话工作目录</x:v>
+      </x:c>
+      <x:c r="E57" s="37" t="str">
+        <x:v>TC-051</x:v>
+      </x:c>
+      <x:c r="F57" s="37" t="str">
+        <x:v>Claude 工作目录识别</x:v>
+      </x:c>
+      <x:c r="G57" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="66" customHeight="1">
+      <x:c r="A58" s="36" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="B58" s="36" t="str">
+        <x:v>会话工作目录识别项目与本机隐私</x:v>
+      </x:c>
+      <x:c r="C58" s="36" t="str">
+        <x:v>DEV-035</x:v>
+      </x:c>
+      <x:c r="D58" s="36" t="str">
+        <x:v>项目标识、本机路径存储与迁移</x:v>
+      </x:c>
+      <x:c r="E58" s="36" t="str">
+        <x:v>TC-052</x:v>
+      </x:c>
+      <x:c r="F58" s="36" t="str">
+        <x:v>同名项目与路径本机边界</x:v>
+      </x:c>
+      <x:c r="G58" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="66" customHeight="1">
+      <x:c r="A59" s="37" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="B59" s="37" t="str">
+        <x:v>项目与模型分析视图</x:v>
+      </x:c>
+      <x:c r="C59" s="37" t="str">
+        <x:v>DEV-036</x:v>
+      </x:c>
+      <x:c r="D59" s="37" t="str">
+        <x:v>项目×模型授权聚合与导出</x:v>
+      </x:c>
+      <x:c r="E59" s="37" t="str">
+        <x:v>TC-053</x:v>
+      </x:c>
+      <x:c r="F59" s="37" t="str">
+        <x:v>项目模型聚合及权限</x:v>
+      </x:c>
+      <x:c r="G59" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="66" customHeight="1">
+      <x:c r="A60" s="36" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="B60" s="36" t="str">
+        <x:v>项目与模型分析视图</x:v>
+      </x:c>
+      <x:c r="C60" s="36" t="str">
+        <x:v>DEV-037</x:v>
+      </x:c>
+      <x:c r="D60" s="36" t="str">
+        <x:v>项目与模型分析界面</x:v>
+      </x:c>
+      <x:c r="E60" s="36" t="str">
+        <x:v>TC-054</x:v>
+      </x:c>
+      <x:c r="F60" s="36" t="str">
+        <x:v>分析视图筛选与下钻</x:v>
+      </x:c>
+      <x:c r="G60" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="66" customHeight="1">
+      <x:c r="A61" s="37" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="B61" s="37" t="str">
+        <x:v>项目与模型分析视图</x:v>
+      </x:c>
+      <x:c r="C61" s="37" t="str">
+        <x:v>DEV-036</x:v>
+      </x:c>
+      <x:c r="D61" s="37" t="str">
+        <x:v>项目×模型授权聚合与导出</x:v>
+      </x:c>
+      <x:c r="E61" s="37" t="str">
+        <x:v>TC-055</x:v>
+      </x:c>
+      <x:c r="F61" s="37" t="str">
+        <x:v>项目模型 CSV 一致性</x:v>
+      </x:c>
+      <x:c r="G61" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="66" customHeight="1">
+      <x:c r="A62" s="36" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="B62" s="36" t="str">
+        <x:v>固定侧栏与响应式导航</x:v>
+      </x:c>
+      <x:c r="C62" s="36" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="D62" s="36" t="str">
+        <x:v>固定侧栏、滚动区和面包屑</x:v>
+      </x:c>
+      <x:c r="E62" s="36" t="str">
+        <x:v>TC-056</x:v>
+      </x:c>
+      <x:c r="F62" s="36" t="str">
+        <x:v>侧栏固定右侧独立滚动</x:v>
+      </x:c>
+      <x:c r="G62" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="66" customHeight="1">
+      <x:c r="A63" s="37" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="B63" s="37" t="str">
+        <x:v>固定侧栏与响应式导航</x:v>
+      </x:c>
+      <x:c r="C63" s="37" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="D63" s="37" t="str">
+        <x:v>固定侧栏、滚动区和面包屑</x:v>
+      </x:c>
+      <x:c r="E63" s="37" t="str">
+        <x:v>TC-057</x:v>
+      </x:c>
+      <x:c r="F63" s="37" t="str">
+        <x:v>窗口自适应与面包屑</x:v>
+      </x:c>
+      <x:c r="G63" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="66" customHeight="1">
+      <x:c r="A64" s="36" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="B64" s="36" t="str">
+        <x:v>可发现的检查更新入口与状态</x:v>
+      </x:c>
+      <x:c r="C64" s="36" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="D64" s="36" t="str">
+        <x:v>更新入口迁移和状态机界面</x:v>
+      </x:c>
+      <x:c r="E64" s="36" t="str">
+        <x:v>TC-058</x:v>
+      </x:c>
+      <x:c r="F64" s="36" t="str">
+        <x:v>更新入口可发现</x:v>
+      </x:c>
+      <x:c r="G64" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="66" customHeight="1">
+      <x:c r="A65" s="37" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="B65" s="37" t="str">
+        <x:v>可发现的检查更新入口与状态</x:v>
+      </x:c>
+      <x:c r="C65" s="37" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="D65" s="37" t="str">
+        <x:v>更新入口迁移和状态机界面</x:v>
+      </x:c>
+      <x:c r="E65" s="37" t="str">
+        <x:v>TC-059</x:v>
+      </x:c>
+      <x:c r="F65" s="37" t="str">
+        <x:v>更新状态与失败恢复</x:v>
+      </x:c>
+      <x:c r="G65" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="66" customHeight="1">
+      <x:c r="A66" s="36" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="B66" s="36" t="str">
+        <x:v>集中系统设置与 macOS 文件权限引导</x:v>
+      </x:c>
+      <x:c r="C66" s="36" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D66" s="36" t="str">
+        <x:v>集中设置与文件权限指引</x:v>
+      </x:c>
+      <x:c r="E66" s="36" t="str">
+        <x:v>TC-060</x:v>
+      </x:c>
+      <x:c r="F66" s="36" t="str">
+        <x:v>集中设置权限</x:v>
+      </x:c>
+      <x:c r="G66" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="66" customHeight="1">
+      <x:c r="A67" s="37" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="B67" s="37" t="str">
+        <x:v>集中系统设置与 macOS 文件权限引导</x:v>
+      </x:c>
+      <x:c r="C67" s="37" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D67" s="37" t="str">
+        <x:v>集中设置与文件权限指引</x:v>
+      </x:c>
+      <x:c r="E67" s="37" t="str">
+        <x:v>TC-061</x:v>
+      </x:c>
+      <x:c r="F67" s="37" t="str">
+        <x:v>权限缺失指引与重试</x:v>
+      </x:c>
+      <x:c r="G67" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="66" customHeight="1">
+      <x:c r="A68" s="36" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="B68" s="36" t="str">
+        <x:v>采集诊断定位漏采</x:v>
+      </x:c>
+      <x:c r="C68" s="36" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="D68" s="36" t="str">
+        <x:v>采集诊断与脱敏摘要</x:v>
+      </x:c>
+      <x:c r="E68" s="36" t="str">
+        <x:v>TC-062</x:v>
+      </x:c>
+      <x:c r="F68" s="36" t="str">
+        <x:v>漏采链路定位</x:v>
+      </x:c>
+      <x:c r="G68" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="66" customHeight="1">
+      <x:c r="A69" s="37" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="B69" s="37" t="str">
+        <x:v>采集诊断定位漏采</x:v>
+      </x:c>
+      <x:c r="C69" s="37" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="D69" s="37" t="str">
+        <x:v>采集诊断与脱敏摘要</x:v>
+      </x:c>
+      <x:c r="E69" s="37" t="str">
+        <x:v>TC-063</x:v>
+      </x:c>
+      <x:c r="F69" s="37" t="str">
+        <x:v>诊断脱敏与权限</x:v>
+      </x:c>
+      <x:c r="G69" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="66" customHeight="1">
+      <x:c r="A70" s="36" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="B70" s="36" t="str">
+        <x:v>用户问题反馈上报</x:v>
+      </x:c>
+      <x:c r="C70" s="36" t="str">
+        <x:v>DEV-042</x:v>
+      </x:c>
+      <x:c r="D70" s="36" t="str">
+        <x:v>反馈表单、预览和本机待传</x:v>
+      </x:c>
+      <x:c r="E70" s="36" t="str">
+        <x:v>TC-064</x:v>
+      </x:c>
+      <x:c r="F70" s="36" t="str">
+        <x:v>反馈预览与提交</x:v>
+      </x:c>
+      <x:c r="G70" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="66" customHeight="1">
+      <x:c r="A71" s="37" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="B71" s="37" t="str">
+        <x:v>用户问题反馈上报</x:v>
+      </x:c>
+      <x:c r="C71" s="37" t="str">
+        <x:v>DEV-043</x:v>
+      </x:c>
+      <x:c r="D71" s="37" t="str">
+        <x:v>服务端反馈接收、鉴权与幂等</x:v>
+      </x:c>
+      <x:c r="E71" s="37" t="str">
+        <x:v>TC-065</x:v>
+      </x:c>
+      <x:c r="F71" s="37" t="str">
+        <x:v>反馈鉴权与失败重试</x:v>
+      </x:c>
+      <x:c r="G71" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="66" customHeight="1">
+      <x:c r="A72" s="36" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="B72" s="36" t="str">
+        <x:v>管理员反馈与运行状态视图</x:v>
+      </x:c>
+      <x:c r="C72" s="36" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="D72" s="36" t="str">
+        <x:v>管理员反馈/账号/采集概览</x:v>
+      </x:c>
+      <x:c r="E72" s="36" t="str">
+        <x:v>TC-066</x:v>
+      </x:c>
+      <x:c r="F72" s="36" t="str">
+        <x:v>管理员反馈列表权限</x:v>
+      </x:c>
+      <x:c r="G72" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="66" customHeight="1">
+      <x:c r="A73" s="37" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="B73" s="37" t="str">
+        <x:v>管理员反馈与运行状态视图</x:v>
+      </x:c>
+      <x:c r="C73" s="37" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="D73" s="37" t="str">
+        <x:v>管理员反馈/账号/采集概览</x:v>
+      </x:c>
+      <x:c r="E73" s="37" t="str">
+        <x:v>TC-067</x:v>
+      </x:c>
+      <x:c r="F73" s="37" t="str">
+        <x:v>管理员账号采集状态</x:v>
+      </x:c>
+      <x:c r="G73" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="66" customHeight="1">
+      <x:c r="A74" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="B74" s="36" t="str">
+        <x:v>固定 admin 超管与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C74" s="36" t="str">
+        <x:v>DEV-045</x:v>
+      </x:c>
+      <x:c r="D74" s="36" t="str">
+        <x:v>固定 admin 派生角色与旧库兼容</x:v>
+      </x:c>
+      <x:c r="E74" s="36" t="str">
+        <x:v>TC-068</x:v>
+      </x:c>
+      <x:c r="F74" s="36" t="str">
+        <x:v>固定 admin 初始化</x:v>
+      </x:c>
+      <x:c r="G74" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="66" customHeight="1">
+      <x:c r="A75" s="37" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="B75" s="37" t="str">
+        <x:v>固定 admin 超管与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C75" s="37" t="str">
+        <x:v>DEV-046</x:v>
+      </x:c>
+      <x:c r="D75" s="37" t="str">
+        <x:v>超管账号操作与跨角色授权</x:v>
+      </x:c>
+      <x:c r="E75" s="37" t="str">
+        <x:v>TC-069</x:v>
+      </x:c>
+      <x:c r="F75" s="37" t="str">
+        <x:v>派生三级角色与管理边界</x:v>
+      </x:c>
+      <x:c r="G75" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="66" customHeight="1">
+      <x:c r="A76" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="B76" s="36" t="str">
+        <x:v>固定 admin 超管与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C76" s="36" t="str">
+        <x:v>DEV-045</x:v>
+      </x:c>
+      <x:c r="D76" s="36" t="str">
+        <x:v>固定 admin 派生角色与旧库兼容</x:v>
+      </x:c>
+      <x:c r="E76" s="36" t="str">
+        <x:v>TC-070</x:v>
+      </x:c>
+      <x:c r="F76" s="36" t="str">
+        <x:v>旧库 admin 迁移及冲突</x:v>
+      </x:c>
+      <x:c r="G76" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="66" customHeight="1">
+      <x:c r="A77" s="37" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="B77" s="37" t="str">
+        <x:v>固定 admin 超管与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C77" s="37" t="str">
+        <x:v>DEV-046</x:v>
+      </x:c>
+      <x:c r="D77" s="37" t="str">
+        <x:v>超管账号操作与跨角色授权</x:v>
+      </x:c>
+      <x:c r="E77" s="37" t="str">
+        <x:v>TC-071</x:v>
+      </x:c>
+      <x:c r="F77" s="37" t="str">
+        <x:v>超管创建角色与审计边界</x:v>
+      </x:c>
+      <x:c r="G77" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="66" customHeight="1">
+      <x:c r="A78" s="36" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="B78" s="36" t="str">
+        <x:v>集中系统设置与 macOS 文件权限引导</x:v>
+      </x:c>
+      <x:c r="C78" s="36" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D78" s="36" t="str">
+        <x:v>集中设置与文件权限指引</x:v>
+      </x:c>
+      <x:c r="E78" s="36" t="str">
+        <x:v>TC-072</x:v>
+      </x:c>
+      <x:c r="F78" s="36" t="str">
+        <x:v>目标 Mac 文件授权手工验收</x:v>
+      </x:c>
+      <x:c r="G78" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1700,7 +2245,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–030；M5 已有代码与自动测试，完整验收状态见需求列和逐项验收文档。</x:v>
+        <x:v>REQ-001–039；M6 REQ-031–039 为规划项，候选功能未分配本轮编号。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2524,6 +3069,240 @@
       </x:c>
       <x:c r="H35" s="35" t="str">
         <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="66" customHeight="1">
+      <x:c r="A36" s="36" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="B36" s="36" t="str">
+        <x:v>会话工作目录识别项目与本机隐私</x:v>
+      </x:c>
+      <x:c r="C36" s="36" t="str">
+        <x:v>从 Codex/Claude 会话工作目录自动建议稳定项目归属，展示项目名；缺失或无效目录为“未知项目”，同名不同路径不得误合并；原始完整路径仅本机存储，不进入聚合上报、反馈或诊断外发。</x:v>
+      </x:c>
+      <x:c r="D36" s="36" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E36" s="36" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F36" s="36" t="str">
+        <x:v>DEV-034、DEV-035</x:v>
+      </x:c>
+      <x:c r="G36" s="36" t="str">
+        <x:v>TC-050、TC-051、TC-052</x:v>
+      </x:c>
+      <x:c r="H36" s="36" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="66" customHeight="1">
+      <x:c r="A37" s="37" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="B37" s="37" t="str">
+        <x:v>项目与模型分析视图</x:v>
+      </x:c>
+      <x:c r="C37" s="37" t="str">
+        <x:v>按授权用户、项目、模型、提供方和时间区间查看 Token 分类、总量、请求数、趋势与排行；项目×模型筛选下钻与 CSV 同口径，未知项目可见，不重复计数。</x:v>
+      </x:c>
+      <x:c r="D37" s="37" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E37" s="37" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F37" s="37" t="str">
+        <x:v>DEV-036、DEV-037</x:v>
+      </x:c>
+      <x:c r="G37" s="37" t="str">
+        <x:v>TC-053、TC-054、TC-055</x:v>
+      </x:c>
+      <x:c r="H37" s="37" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="66" customHeight="1">
+      <x:c r="A38" s="36" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="B38" s="36" t="str">
+        <x:v>固定侧栏与响应式导航</x:v>
+      </x:c>
+      <x:c r="C38" s="36" t="str">
+        <x:v>应用侧栏固定，右侧内容独立滚动；窗口宽度变化时内容不遮挡、可操作；页面面包屑与当前导航和下钻路径一致。</x:v>
+      </x:c>
+      <x:c r="D38" s="36" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E38" s="36" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F38" s="36" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="G38" s="36" t="str">
+        <x:v>TC-056、TC-057</x:v>
+      </x:c>
+      <x:c r="H38" s="36" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="66" customHeight="1">
+      <x:c r="A39" s="37" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="B39" s="37" t="str">
+        <x:v>可发现的检查更新入口与状态</x:v>
+      </x:c>
+      <x:c r="C39" s="37" t="str">
+        <x:v>把已有“检查更新”移至明显导航或设置位置，展示检查中、最新版本、发现版本、下载、校验、打开安装包及可恢复失败状态；不自动替换未签名应用。</x:v>
+      </x:c>
+      <x:c r="D39" s="37" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E39" s="37" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F39" s="37" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="G39" s="37" t="str">
+        <x:v>TC-058、TC-059</x:v>
+      </x:c>
+      <x:c r="H39" s="37" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="66" customHeight="1">
+      <x:c r="A40" s="36" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="B40" s="36" t="str">
+        <x:v>集中系统设置与 macOS 文件权限引导</x:v>
+      </x:c>
+      <x:c r="C40" s="36" t="str">
+        <x:v>集中展示服务器、采集、更新与本机权限设置；按角色保护修改入口；来源无权限时说明所需 macOS 操作和重试路径，不自动提权或读取其他账户文件。</x:v>
+      </x:c>
+      <x:c r="D40" s="36" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E40" s="36" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F40" s="36" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="G40" s="36" t="str">
+        <x:v>TC-060、TC-061、TC-072</x:v>
+      </x:c>
+      <x:c r="H40" s="36" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="66" customHeight="1">
+      <x:c r="A41" s="37" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="B41" s="37" t="str">
+        <x:v>采集诊断定位漏采</x:v>
+      </x:c>
+      <x:c r="C41" s="37" t="str">
+        <x:v>按来源列出检测、解析、游标、覆盖区间、最近成功/失败和未归属原因，能定位漏采环节；未知与真实零分离；诊断信息脱敏，原始路径只在本机可见。</x:v>
+      </x:c>
+      <x:c r="D41" s="37" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E41" s="37" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F41" s="37" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="G41" s="37" t="str">
+        <x:v>TC-062、TC-063</x:v>
+      </x:c>
+      <x:c r="H41" s="37" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="66" customHeight="1">
+      <x:c r="A42" s="36" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="B42" s="36" t="str">
+        <x:v>用户问题反馈上报</x:v>
+      </x:c>
+      <x:c r="C42" s="36" t="str">
+        <x:v>用户显式提交反馈到配置的服务端，提交前可预览白名单字段；不包含提示词、源码、密钥或完整项目路径；失败可重试且不重复生成反馈。</x:v>
+      </x:c>
+      <x:c r="D42" s="36" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E42" s="36" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F42" s="36" t="str">
+        <x:v>DEV-042、DEV-043</x:v>
+      </x:c>
+      <x:c r="G42" s="36" t="str">
+        <x:v>TC-064、TC-065</x:v>
+      </x:c>
+      <x:c r="H42" s="36" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="66" customHeight="1">
+      <x:c r="A43" s="37" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="B43" s="37" t="str">
+        <x:v>管理员反馈与运行状态视图</x:v>
+      </x:c>
+      <x:c r="C43" s="37" t="str">
+        <x:v>管理员及超管可查看授权范围内的反馈、账号启停/角色状态和采集健康状态；普通用户不能跨用户读取或调用管理 IPC；查看不等于处理闭环。</x:v>
+      </x:c>
+      <x:c r="D43" s="37" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E43" s="37" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F43" s="37" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="G43" s="37" t="str">
+        <x:v>TC-066、TC-067</x:v>
+      </x:c>
+      <x:c r="H43" s="37" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="66" customHeight="1">
+      <x:c r="A44" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="B44" s="36" t="str">
+        <x:v>固定 admin 超管与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C44" s="36" t="str">
+        <x:v>全新安装首建固定用户名 admin；库内仍存 admin/viewer，仅用户名 admin 且库角色 admin 对外呈现 superadmin；旧库该账号自动成为超管，其他管理员保留原权限；旧库无 admin 时现有管理员可创建之；非超管不得停用或重置该账号，冲突不得静默升权。</x:v>
+      </x:c>
+      <x:c r="D44" s="36" t="str">
+        <x:v>M6（规划）</x:v>
+      </x:c>
+      <x:c r="E44" s="36" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="F44" s="36" t="str">
+        <x:v>DEV-045、DEV-046</x:v>
+      </x:c>
+      <x:c r="G44" s="36" t="str">
+        <x:v>TC-068、TC-069、TC-070、TC-071</x:v>
+      </x:c>
+      <x:c r="H44" s="36" t="str">
+        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3358,6 +4137,305 @@
       </x:c>
       <x:c r="G38" s="14" t="str">
         <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="66" customHeight="1">
+      <x:c r="A39" s="37" t="str">
+        <x:v>DEV-034</x:v>
+      </x:c>
+      <x:c r="B39" s="37" t="str">
+        <x:v>解析 Codex/Claude 会话工作目录</x:v>
+      </x:c>
+      <x:c r="C39" s="37" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="D39" s="37" t="str">
+        <x:v>TC-050、TC-051</x:v>
+      </x:c>
+      <x:c r="E39" s="37" t="str">
+        <x:v>src/collectors/codex.ts；src/collectors/claude.ts；tests/m6-project.test.ts</x:v>
+      </x:c>
+      <x:c r="F39" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G39" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="66" customHeight="1">
+      <x:c r="A40" s="36" t="str">
+        <x:v>DEV-035</x:v>
+      </x:c>
+      <x:c r="B40" s="36" t="str">
+        <x:v>项目标识、本机路径存储与迁移</x:v>
+      </x:c>
+      <x:c r="C40" s="36" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="D40" s="36" t="str">
+        <x:v>TC-052</x:v>
+      </x:c>
+      <x:c r="E40" s="36" t="str">
+        <x:v>src/main/database.ts；src/main/usage-sync.ts；tests/m6-project.test.ts</x:v>
+      </x:c>
+      <x:c r="F40" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G40" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="66" customHeight="1">
+      <x:c r="A41" s="37" t="str">
+        <x:v>DEV-036</x:v>
+      </x:c>
+      <x:c r="B41" s="37" t="str">
+        <x:v>项目×模型授权聚合与导出</x:v>
+      </x:c>
+      <x:c r="C41" s="37" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="D41" s="37" t="str">
+        <x:v>TC-053、TC-055</x:v>
+      </x:c>
+      <x:c r="E41" s="37" t="str">
+        <x:v>src/main/report.ts；src/shared/types.ts；tests/m6-report.test.ts</x:v>
+      </x:c>
+      <x:c r="F41" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G41" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="66" customHeight="1">
+      <x:c r="A42" s="36" t="str">
+        <x:v>DEV-037</x:v>
+      </x:c>
+      <x:c r="B42" s="36" t="str">
+        <x:v>项目与模型分析界面</x:v>
+      </x:c>
+      <x:c r="C42" s="36" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="D42" s="36" t="str">
+        <x:v>TC-054</x:v>
+      </x:c>
+      <x:c r="E42" s="36" t="str">
+        <x:v>src/renderer/report.tsx；tests/e2e/m6-analysis.spec.ts</x:v>
+      </x:c>
+      <x:c r="F42" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G42" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="66" customHeight="1">
+      <x:c r="A43" s="37" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="B43" s="37" t="str">
+        <x:v>固定侧栏、滚动区和面包屑</x:v>
+      </x:c>
+      <x:c r="C43" s="37" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="D43" s="37" t="str">
+        <x:v>TC-056、TC-057</x:v>
+      </x:c>
+      <x:c r="E43" s="37" t="str">
+        <x:v>src/renderer/index.tsx；src/renderer/style.css；tests/e2e/m6-shell.spec.ts</x:v>
+      </x:c>
+      <x:c r="F43" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G43" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="66" customHeight="1">
+      <x:c r="A44" s="36" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="B44" s="36" t="str">
+        <x:v>更新入口迁移和状态机界面</x:v>
+      </x:c>
+      <x:c r="C44" s="36" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="D44" s="36" t="str">
+        <x:v>TC-058、TC-059</x:v>
+      </x:c>
+      <x:c r="E44" s="36" t="str">
+        <x:v>src/renderer/index.tsx；src/main/update-client.ts；tests/e2e/m6-update.spec.ts</x:v>
+      </x:c>
+      <x:c r="F44" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G44" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="66" customHeight="1">
+      <x:c r="A45" s="37" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="B45" s="37" t="str">
+        <x:v>集中设置与文件权限指引</x:v>
+      </x:c>
+      <x:c r="C45" s="37" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="D45" s="37" t="str">
+        <x:v>TC-060、TC-061、TC-072</x:v>
+      </x:c>
+      <x:c r="E45" s="37" t="str">
+        <x:v>src/renderer/index.tsx；src/main/index.ts；tests/e2e/m6-settings.spec.ts</x:v>
+      </x:c>
+      <x:c r="F45" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G45" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="66" customHeight="1">
+      <x:c r="A46" s="36" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="B46" s="36" t="str">
+        <x:v>采集诊断与脱敏摘要</x:v>
+      </x:c>
+      <x:c r="C46" s="36" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="D46" s="36" t="str">
+        <x:v>TC-062、TC-063</x:v>
+      </x:c>
+      <x:c r="E46" s="36" t="str">
+        <x:v>src/collectors/scanner.ts；src/main/index.ts；tests/m6-diagnostics.test.ts</x:v>
+      </x:c>
+      <x:c r="F46" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G46" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="66" customHeight="1">
+      <x:c r="A47" s="37" t="str">
+        <x:v>DEV-042</x:v>
+      </x:c>
+      <x:c r="B47" s="37" t="str">
+        <x:v>反馈表单、预览和本机待传</x:v>
+      </x:c>
+      <x:c r="C47" s="37" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="D47" s="37" t="str">
+        <x:v>TC-064</x:v>
+      </x:c>
+      <x:c r="E47" s="37" t="str">
+        <x:v>src/renderer/index.tsx；src/main/feedback.ts；tests/m6-feedback.test.ts</x:v>
+      </x:c>
+      <x:c r="F47" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G47" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="66" customHeight="1">
+      <x:c r="A48" s="36" t="str">
+        <x:v>DEV-043</x:v>
+      </x:c>
+      <x:c r="B48" s="36" t="str">
+        <x:v>服务端反馈接收、鉴权与幂等</x:v>
+      </x:c>
+      <x:c r="C48" s="36" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="D48" s="36" t="str">
+        <x:v>TC-065</x:v>
+      </x:c>
+      <x:c r="E48" s="36" t="str">
+        <x:v>src/server/server.ts；tests/m6-feedback.test.ts</x:v>
+      </x:c>
+      <x:c r="F48" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G48" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="66" customHeight="1">
+      <x:c r="A49" s="37" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="B49" s="37" t="str">
+        <x:v>管理员反馈/账号/采集概览</x:v>
+      </x:c>
+      <x:c r="C49" s="37" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="D49" s="37" t="str">
+        <x:v>TC-066、TC-067</x:v>
+      </x:c>
+      <x:c r="E49" s="37" t="str">
+        <x:v>src/main/index.ts；src/renderer/index.tsx；tests/e2e/m6-admin.spec.ts</x:v>
+      </x:c>
+      <x:c r="F49" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G49" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="66" customHeight="1">
+      <x:c r="A50" s="36" t="str">
+        <x:v>DEV-045</x:v>
+      </x:c>
+      <x:c r="B50" s="36" t="str">
+        <x:v>固定 admin 派生角色与旧库兼容</x:v>
+      </x:c>
+      <x:c r="C50" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="D50" s="36" t="str">
+        <x:v>TC-068、TC-070</x:v>
+      </x:c>
+      <x:c r="E50" s="36" t="str">
+        <x:v>src/main/auth.ts；src/main/database.ts；tests/m6-roles.test.ts</x:v>
+      </x:c>
+      <x:c r="F50" s="36" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G50" s="36" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="66" customHeight="1">
+      <x:c r="A51" s="37" t="str">
+        <x:v>DEV-046</x:v>
+      </x:c>
+      <x:c r="B51" s="37" t="str">
+        <x:v>超管账号操作与跨角色授权</x:v>
+      </x:c>
+      <x:c r="C51" s="37" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="D51" s="37" t="str">
+        <x:v>TC-069、TC-071</x:v>
+      </x:c>
+      <x:c r="E51" s="37" t="str">
+        <x:v>src/main/auth.ts；src/main/index.ts；src/renderer/index.tsx；tests/m6-roles.test.ts</x:v>
+      </x:c>
+      <x:c r="F51" s="37" t="str">
+        <x:v>待启动</x:v>
+      </x:c>
+      <x:c r="G51" s="37" t="str">
+        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3402,7 +4480,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–049 均有入口；TC-029 已自动化，TC-030–049 的覆盖边界见 docs/test-case-acceptance.md。</x:v>
+        <x:v>TC-001–049 已有入口；TC-050–072 仅规划，scripts/test-cases.mjs 尚未注册，不得写成可执行或通过。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -5479,6 +6557,949 @@
         <x:v>记录 TC-049 命令、退出码、提交、环境和脱敏日志；覆盖与限制：跨年周/月标签及点击；未测其他时区/长期跨度。</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="82" customHeight="1">
+      <x:c r="A55" s="37" t="str">
+        <x:v>TC-050</x:v>
+      </x:c>
+      <x:c r="B55" s="37" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="C55" s="37" t="str">
+        <x:v>DEV-034</x:v>
+      </x:c>
+      <x:c r="D55" s="37" t="str">
+        <x:v>Codex 工作目录识别</x:v>
+      </x:c>
+      <x:c r="E55" s="37" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F55" s="37" t="str">
+        <x:v>临时 Codex 会话含工作目录、模型切换与无目录对照。</x:v>
+      </x:c>
+      <x:c r="G55" s="37" t="str">
+        <x:v>项目稳定归属；无目录保持未知，不读取工作目录内容。</x:v>
+      </x:c>
+      <x:c r="H55" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I55" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J55" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-050</x:v>
+      </x:c>
+      <x:c r="K55" s="37" t="str">
+        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-050 Codex 工作目录归属')</x:v>
+      </x:c>
+      <x:c r="L55" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M55" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc050-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="82" customHeight="1">
+      <x:c r="A56" s="36" t="str">
+        <x:v>TC-051</x:v>
+      </x:c>
+      <x:c r="B56" s="36" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="C56" s="36" t="str">
+        <x:v>DEV-034</x:v>
+      </x:c>
+      <x:c r="D56" s="36" t="str">
+        <x:v>Claude 工作目录识别</x:v>
+      </x:c>
+      <x:c r="E56" s="36" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F56" s="36" t="str">
+        <x:v>临时 Claude 会话及子代理记录包含/缺失 cwd。</x:v>
+      </x:c>
+      <x:c r="G56" s="36" t="str">
+        <x:v>同会话归属一致；缺失为未知，子代理不误归其他项目。</x:v>
+      </x:c>
+      <x:c r="H56" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I56" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J56" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-051</x:v>
+      </x:c>
+      <x:c r="K56" s="36" t="str">
+        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-051 Claude 工作目录归属')</x:v>
+      </x:c>
+      <x:c r="L56" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M56" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc051-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="82" customHeight="1">
+      <x:c r="A57" s="37" t="str">
+        <x:v>TC-052</x:v>
+      </x:c>
+      <x:c r="B57" s="37" t="str">
+        <x:v>REQ-031</x:v>
+      </x:c>
+      <x:c r="C57" s="37" t="str">
+        <x:v>DEV-035</x:v>
+      </x:c>
+      <x:c r="D57" s="37" t="str">
+        <x:v>同名项目与路径本机边界</x:v>
+      </x:c>
+      <x:c r="E57" s="37" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F57" s="37" t="str">
+        <x:v>两条不同绝对路径同 basename，扫描后抓取上报/反馈/诊断外发。</x:v>
+      </x:c>
+      <x:c r="G57" s="37" t="str">
+        <x:v>内部项目标识区分；显示名可区分；外发无完整路径、项目 ID 或别名；旧事实无 cwd 保持未知。</x:v>
+      </x:c>
+      <x:c r="H57" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I57" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J57" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-052</x:v>
+      </x:c>
+      <x:c r="K57" s="37" t="str">
+        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-052 同名项目不合并且完整路径不外传')</x:v>
+      </x:c>
+      <x:c r="L57" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M57" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc052-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="82" customHeight="1">
+      <x:c r="A58" s="36" t="str">
+        <x:v>TC-053</x:v>
+      </x:c>
+      <x:c r="B58" s="36" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="C58" s="36" t="str">
+        <x:v>DEV-036</x:v>
+      </x:c>
+      <x:c r="D58" s="36" t="str">
+        <x:v>项目模型聚合及权限</x:v>
+      </x:c>
+      <x:c r="E58" s="36" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F58" s="36" t="str">
+        <x:v>临时库多用户、项目、模型、时区和未知项目。</x:v>
+      </x:c>
+      <x:c r="G58" s="36" t="str">
+        <x:v>聚合等于授权事实求和，普通用户不越权，未知项目单列。</x:v>
+      </x:c>
+      <x:c r="H58" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I58" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J58" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-053</x:v>
+      </x:c>
+      <x:c r="K58" s="36" t="str">
+        <x:v>计划绑定 tests/m6-report.test.ts：test('TC-053 项目模型聚合权限与时区')</x:v>
+      </x:c>
+      <x:c r="L58" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M58" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc053-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="82" customHeight="1">
+      <x:c r="A59" s="37" t="str">
+        <x:v>TC-054</x:v>
+      </x:c>
+      <x:c r="B59" s="37" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="C59" s="37" t="str">
+        <x:v>DEV-037</x:v>
+      </x:c>
+      <x:c r="D59" s="37" t="str">
+        <x:v>分析视图筛选与下钻</x:v>
+      </x:c>
+      <x:c r="E59" s="37" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F59" s="37" t="str">
+        <x:v>临时用户数据启动 Electron，构造跨项目多模型记录。</x:v>
+      </x:c>
+      <x:c r="G59" s="37" t="str">
+        <x:v>项目/模型排行、趋势和下钻同筛选，切换不会混入其他项目。</x:v>
+      </x:c>
+      <x:c r="H59" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I59" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J59" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-054</x:v>
+      </x:c>
+      <x:c r="K59" s="37" t="str">
+        <x:v>计划绑定 tests/e2e/m6-analysis.spec.ts：test('TC-054 项目模型分析筛选下钻')</x:v>
+      </x:c>
+      <x:c r="L59" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M59" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc054-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="82" customHeight="1">
+      <x:c r="A60" s="36" t="str">
+        <x:v>TC-055</x:v>
+      </x:c>
+      <x:c r="B60" s="36" t="str">
+        <x:v>REQ-032</x:v>
+      </x:c>
+      <x:c r="C60" s="36" t="str">
+        <x:v>DEV-036</x:v>
+      </x:c>
+      <x:c r="D60" s="36" t="str">
+        <x:v>项目模型 CSV 一致性</x:v>
+      </x:c>
+      <x:c r="E60" s="36" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F60" s="36" t="str">
+        <x:v>同一筛选查询报表与 CSV，含未知项目和跨年周。</x:v>
+      </x:c>
+      <x:c r="G60" s="36" t="str">
+        <x:v>页面、明细、CSV 总量/分类一致；文本防公式注入；路径不导出。</x:v>
+      </x:c>
+      <x:c r="H60" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I60" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J60" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-055</x:v>
+      </x:c>
+      <x:c r="K60" s="36" t="str">
+        <x:v>计划绑定 tests/m6-report.test.ts：test('TC-055 项目模型页面与 CSV 对账')</x:v>
+      </x:c>
+      <x:c r="L60" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M60" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc055-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="82" customHeight="1">
+      <x:c r="A61" s="37" t="str">
+        <x:v>TC-056</x:v>
+      </x:c>
+      <x:c r="B61" s="37" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="C61" s="37" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="D61" s="37" t="str">
+        <x:v>侧栏固定右侧独立滚动</x:v>
+      </x:c>
+      <x:c r="E61" s="37" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F61" s="37" t="str">
+        <x:v>临时账户登录，长报表滚动右侧容器。</x:v>
+      </x:c>
+      <x:c r="G61" s="37" t="str">
+        <x:v>侧栏位置不变、右侧独立滚动，焦点和操作可见。</x:v>
+      </x:c>
+      <x:c r="H61" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I61" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J61" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-056</x:v>
+      </x:c>
+      <x:c r="K61" s="37" t="str">
+        <x:v>计划绑定 tests/e2e/m6-shell.spec.ts：test('TC-056 固定侧栏和右侧滚动')</x:v>
+      </x:c>
+      <x:c r="L61" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M61" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc056-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="82" customHeight="1">
+      <x:c r="A62" s="36" t="str">
+        <x:v>TC-057</x:v>
+      </x:c>
+      <x:c r="B62" s="36" t="str">
+        <x:v>REQ-033</x:v>
+      </x:c>
+      <x:c r="C62" s="36" t="str">
+        <x:v>DEV-038</x:v>
+      </x:c>
+      <x:c r="D62" s="36" t="str">
+        <x:v>窗口自适应与面包屑</x:v>
+      </x:c>
+      <x:c r="E62" s="36" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F62" s="36" t="str">
+        <x:v>宽/窄窗口切换设置、报表与下钻。</x:v>
+      </x:c>
+      <x:c r="G62" s="36" t="str">
+        <x:v>无遮挡和横向丢失；面包屑反映层级并可回退。</x:v>
+      </x:c>
+      <x:c r="H62" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I62" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J62" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-057</x:v>
+      </x:c>
+      <x:c r="K62" s="36" t="str">
+        <x:v>计划绑定 tests/e2e/m6-shell.spec.ts：test('TC-057 响应式布局和面包屑')</x:v>
+      </x:c>
+      <x:c r="L62" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M62" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc057-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="82" customHeight="1">
+      <x:c r="A63" s="37" t="str">
+        <x:v>TC-058</x:v>
+      </x:c>
+      <x:c r="B63" s="37" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="C63" s="37" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="D63" s="37" t="str">
+        <x:v>更新入口可发现</x:v>
+      </x:c>
+      <x:c r="E63" s="37" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F63" s="37" t="str">
+        <x:v>登录后不向下滚概览，查导航或设置中的更新入口。</x:v>
+      </x:c>
+      <x:c r="G63" s="37" t="str">
+        <x:v>入口在显著位置且普通授权用户可找到；不重复藏在概览下方。</x:v>
+      </x:c>
+      <x:c r="H63" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I63" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J63" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-058</x:v>
+      </x:c>
+      <x:c r="K63" s="37" t="str">
+        <x:v>计划绑定 tests/e2e/m6-update.spec.ts：test('TC-058 显著更新入口')</x:v>
+      </x:c>
+      <x:c r="L63" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M63" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc058-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="82" customHeight="1">
+      <x:c r="A64" s="36" t="str">
+        <x:v>TC-059</x:v>
+      </x:c>
+      <x:c r="B64" s="36" t="str">
+        <x:v>REQ-034</x:v>
+      </x:c>
+      <x:c r="C64" s="36" t="str">
+        <x:v>DEV-039</x:v>
+      </x:c>
+      <x:c r="D64" s="36" t="str">
+        <x:v>更新状态与失败恢复</x:v>
+      </x:c>
+      <x:c r="E64" s="36" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F64" s="36" t="str">
+        <x:v>模拟同版、新版、下载中断、摘要错误和重试。</x:v>
+      </x:c>
+      <x:c r="G64" s="36" t="str">
+        <x:v>每阶段状态准确，错误可恢复；坏包不打开，旧版可用。</x:v>
+      </x:c>
+      <x:c r="H64" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I64" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J64" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-059</x:v>
+      </x:c>
+      <x:c r="K64" s="36" t="str">
+        <x:v>计划绑定 tests/e2e/m6-update.spec.ts：test('TC-059 更新状态成功失败恢复')</x:v>
+      </x:c>
+      <x:c r="L64" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M64" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc059-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="82" customHeight="1">
+      <x:c r="A65" s="37" t="str">
+        <x:v>TC-060</x:v>
+      </x:c>
+      <x:c r="B65" s="37" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="C65" s="37" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D65" s="37" t="str">
+        <x:v>集中设置权限</x:v>
+      </x:c>
+      <x:c r="E65" s="37" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F65" s="37" t="str">
+        <x:v>临时 superadmin/admin/viewer 登录并访问设置。</x:v>
+      </x:c>
+      <x:c r="G65" s="37" t="str">
+        <x:v>采集/更新/服务器/权限集中；受限角色不能调用管理修改 IPC。</x:v>
+      </x:c>
+      <x:c r="H65" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I65" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J65" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-060</x:v>
+      </x:c>
+      <x:c r="K65" s="37" t="str">
+        <x:v>计划绑定 tests/e2e/m6-settings.spec.ts：test('TC-060 设置分组与角色保护')</x:v>
+      </x:c>
+      <x:c r="L65" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M65" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc060-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="82" customHeight="1">
+      <x:c r="A66" s="36" t="str">
+        <x:v>TC-061</x:v>
+      </x:c>
+      <x:c r="B66" s="36" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="C66" s="36" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D66" s="36" t="str">
+        <x:v>权限缺失指引与重试</x:v>
+      </x:c>
+      <x:c r="E66" s="36" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F66" s="36" t="str">
+        <x:v>临时目录模拟无权限与恢复可读。</x:v>
+      </x:c>
+      <x:c r="G66" s="36" t="str">
+        <x:v>显示具体来源、macOS 手动授权和重试路径；恢复后状态更新，不自动提权。</x:v>
+      </x:c>
+      <x:c r="H66" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I66" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J66" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-061</x:v>
+      </x:c>
+      <x:c r="K66" s="36" t="str">
+        <x:v>计划绑定 tests/e2e/m6-settings.spec.ts：test('TC-061 macOS 文件权限指引模拟')</x:v>
+      </x:c>
+      <x:c r="L66" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M66" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc061-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="82" customHeight="1">
+      <x:c r="A67" s="37" t="str">
+        <x:v>TC-062</x:v>
+      </x:c>
+      <x:c r="B67" s="37" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="C67" s="37" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="D67" s="37" t="str">
+        <x:v>漏采链路定位</x:v>
+      </x:c>
+      <x:c r="E67" s="37" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F67" s="37" t="str">
+        <x:v>临时库构造目录缺失、解析失败、游标停滞、未归属与重复。</x:v>
+      </x:c>
+      <x:c r="G67" s="37" t="str">
+        <x:v>诊断指出对应环节和最后成功时间，不把未知当零。</x:v>
+      </x:c>
+      <x:c r="H67" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I67" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J67" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-062</x:v>
+      </x:c>
+      <x:c r="K67" s="37" t="str">
+        <x:v>计划绑定 tests/m6-diagnostics.test.ts：test('TC-062 检测解析游标漏采定位')</x:v>
+      </x:c>
+      <x:c r="L67" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M67" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc062-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="82" customHeight="1">
+      <x:c r="A68" s="36" t="str">
+        <x:v>TC-063</x:v>
+      </x:c>
+      <x:c r="B68" s="36" t="str">
+        <x:v>REQ-036</x:v>
+      </x:c>
+      <x:c r="C68" s="36" t="str">
+        <x:v>DEV-041</x:v>
+      </x:c>
+      <x:c r="D68" s="36" t="str">
+        <x:v>诊断脱敏与权限</x:v>
+      </x:c>
+      <x:c r="E68" s="36" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F68" s="36" t="str">
+        <x:v>合成路径、正文、密钥样式字段；按角色请求诊断摘要。</x:v>
+      </x:c>
+      <x:c r="G68" s="36" t="str">
+        <x:v>外发与日志无敏感字段；普通用户仅看授权来源。</x:v>
+      </x:c>
+      <x:c r="H68" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I68" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J68" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-063</x:v>
+      </x:c>
+      <x:c r="K68" s="36" t="str">
+        <x:v>计划绑定 tests/m6-diagnostics.test.ts：test('TC-063 诊断脱敏和角色范围')</x:v>
+      </x:c>
+      <x:c r="L68" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M68" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc063-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="82" customHeight="1">
+      <x:c r="A69" s="37" t="str">
+        <x:v>TC-064</x:v>
+      </x:c>
+      <x:c r="B69" s="37" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="C69" s="37" t="str">
+        <x:v>DEV-042</x:v>
+      </x:c>
+      <x:c r="D69" s="37" t="str">
+        <x:v>反馈预览与提交</x:v>
+      </x:c>
+      <x:c r="E69" s="37" t="str">
+        <x:v>单元+Electron</x:v>
+      </x:c>
+      <x:c r="F69" s="37" t="str">
+        <x:v>临时用户数据和本机测试服务，输入含敏感样式文本。</x:v>
+      </x:c>
+      <x:c r="G69" s="37" t="str">
+        <x:v>用户确认后才发白名单数据；原始路径、正文、密钥不发送。</x:v>
+      </x:c>
+      <x:c r="H69" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I69" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J69" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-064</x:v>
+      </x:c>
+      <x:c r="K69" s="37" t="str">
+        <x:v>计划绑定 tests/m6-feedback.test.ts：test('TC-064 反馈预览白名单提交')</x:v>
+      </x:c>
+      <x:c r="L69" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M69" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc064-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="82" customHeight="1">
+      <x:c r="A70" s="36" t="str">
+        <x:v>TC-065</x:v>
+      </x:c>
+      <x:c r="B70" s="36" t="str">
+        <x:v>REQ-037</x:v>
+      </x:c>
+      <x:c r="C70" s="36" t="str">
+        <x:v>DEV-043</x:v>
+      </x:c>
+      <x:c r="D70" s="36" t="str">
+        <x:v>反馈鉴权与失败重试</x:v>
+      </x:c>
+      <x:c r="E70" s="36" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F70" s="36" t="str">
+        <x:v>临时服务目录/随机端口；模拟无凭证、停服和重复提交。</x:v>
+      </x:c>
+      <x:c r="G70" s="36" t="str">
+        <x:v>无权拒绝；重试不重复入库；失败与成功状态可见。</x:v>
+      </x:c>
+      <x:c r="H70" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I70" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J70" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-065</x:v>
+      </x:c>
+      <x:c r="K70" s="36" t="str">
+        <x:v>计划绑定 tests/m6-feedback.test.ts：test('TC-065 反馈鉴权幂等重试')</x:v>
+      </x:c>
+      <x:c r="L70" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M70" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc065-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="82" customHeight="1">
+      <x:c r="A71" s="37" t="str">
+        <x:v>TC-066</x:v>
+      </x:c>
+      <x:c r="B71" s="37" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="C71" s="37" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="D71" s="37" t="str">
+        <x:v>管理员反馈列表权限</x:v>
+      </x:c>
+      <x:c r="E71" s="37" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F71" s="37" t="str">
+        <x:v>临时库有多用户反馈，以三种角色登录。</x:v>
+      </x:c>
+      <x:c r="G71" s="37" t="str">
+        <x:v>superadmin/admin 可按授权范围查看；viewer 无管理入口/IPC。</x:v>
+      </x:c>
+      <x:c r="H71" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I71" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J71" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-066</x:v>
+      </x:c>
+      <x:c r="K71" s="37" t="str">
+        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-066 管理员反馈可见性')</x:v>
+      </x:c>
+      <x:c r="L71" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M71" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc066-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="82" customHeight="1">
+      <x:c r="A72" s="36" t="str">
+        <x:v>TC-067</x:v>
+      </x:c>
+      <x:c r="B72" s="36" t="str">
+        <x:v>REQ-038</x:v>
+      </x:c>
+      <x:c r="C72" s="36" t="str">
+        <x:v>DEV-044</x:v>
+      </x:c>
+      <x:c r="D72" s="36" t="str">
+        <x:v>管理员账号采集状态</x:v>
+      </x:c>
+      <x:c r="E72" s="36" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F72" s="36" t="str">
+        <x:v>临时库有启停用户及正常/异常来源。</x:v>
+      </x:c>
+      <x:c r="G72" s="36" t="str">
+        <x:v>管理员可见账号角色/启停及来源最近成功和错误；数据不越权。</x:v>
+      </x:c>
+      <x:c r="H72" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I72" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J72" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-067</x:v>
+      </x:c>
+      <x:c r="K72" s="36" t="str">
+        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-067 管理员账号来源状态')</x:v>
+      </x:c>
+      <x:c r="L72" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M72" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc067-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="82" customHeight="1">
+      <x:c r="A73" s="37" t="str">
+        <x:v>TC-068</x:v>
+      </x:c>
+      <x:c r="B73" s="37" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="C73" s="37" t="str">
+        <x:v>DEV-045</x:v>
+      </x:c>
+      <x:c r="D73" s="37" t="str">
+        <x:v>固定 admin 初始化</x:v>
+      </x:c>
+      <x:c r="E73" s="37" t="str">
+        <x:v>单元+Electron</x:v>
+      </x:c>
+      <x:c r="F73" s="37" t="str">
+        <x:v>空临时库启动并初始化，检查数据库存值与对外角色。</x:v>
+      </x:c>
+      <x:c r="G73" s="37" t="str">
+        <x:v>首建用户名固定 admin；库内 role=admin、对外 superadmin；重复初始化拒绝。</x:v>
+      </x:c>
+      <x:c r="H73" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I73" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J73" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-068</x:v>
+      </x:c>
+      <x:c r="K73" s="37" t="str">
+        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-068 固定 admin 超管初始化')</x:v>
+      </x:c>
+      <x:c r="L73" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M73" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc068-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="82" customHeight="1">
+      <x:c r="A74" s="36" t="str">
+        <x:v>TC-069</x:v>
+      </x:c>
+      <x:c r="B74" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="C74" s="36" t="str">
+        <x:v>DEV-046</x:v>
+      </x:c>
+      <x:c r="D74" s="36" t="str">
+        <x:v>派生三级角色与管理边界</x:v>
+      </x:c>
+      <x:c r="E74" s="36" t="str">
+        <x:v>单元</x:v>
+      </x:c>
+      <x:c r="F74" s="36" t="str">
+        <x:v>临时库建立 admin(库 admin)、普通管理员与 viewer。</x:v>
+      </x:c>
+      <x:c r="G74" s="36" t="str">
+        <x:v>仅固定 admin 对外 superadmin；其他管理员保持创建 admin/viewer 等原权限但不能停用/重置固定 admin；viewer 无管理权限。</x:v>
+      </x:c>
+      <x:c r="H74" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I74" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J74" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-069</x:v>
+      </x:c>
+      <x:c r="K74" s="36" t="str">
+        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-069 派生超管和原管理员授权')</x:v>
+      </x:c>
+      <x:c r="L74" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M74" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc069-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="82" customHeight="1">
+      <x:c r="A75" s="37" t="str">
+        <x:v>TC-070</x:v>
+      </x:c>
+      <x:c r="B75" s="37" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="C75" s="37" t="str">
+        <x:v>DEV-045</x:v>
+      </x:c>
+      <x:c r="D75" s="37" t="str">
+        <x:v>旧库 admin 迁移及冲突</x:v>
+      </x:c>
+      <x:c r="E75" s="37" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F75" s="37" t="str">
+        <x:v>复制人工旧库：已有 admin 管理员、无 admin、admin 为 viewer、迁移失败。</x:v>
+      </x:c>
+      <x:c r="G75" s="37" t="str">
+        <x:v>已有 admin 管理员自动对外 superadmin；无 admin 时原管理员可创建之；其他账号/哈希/归属不变；viewer 冲突不自动升权且可回退。</x:v>
+      </x:c>
+      <x:c r="H75" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I75" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J75" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-070</x:v>
+      </x:c>
+      <x:c r="K75" s="37" t="str">
+        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-070 旧库固定账号兼容')</x:v>
+      </x:c>
+      <x:c r="L75" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M75" s="37" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc070-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="82" customHeight="1">
+      <x:c r="A76" s="36" t="str">
+        <x:v>TC-071</x:v>
+      </x:c>
+      <x:c r="B76" s="36" t="str">
+        <x:v>REQ-039</x:v>
+      </x:c>
+      <x:c r="C76" s="36" t="str">
+        <x:v>DEV-046</x:v>
+      </x:c>
+      <x:c r="D76" s="36" t="str">
+        <x:v>超管创建角色与审计边界</x:v>
+      </x:c>
+      <x:c r="E76" s="36" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F76" s="36" t="str">
+        <x:v>固定 admin 登录创建普通管理员/viewer，并用其他角色访问超管专属操作。</x:v>
+      </x:c>
+      <x:c r="G76" s="36" t="str">
+        <x:v>超管可创建两类账号；普通管理员保留原创建权限但不能停用/重置固定 admin；若提供审计查看则仅超管可见。</x:v>
+      </x:c>
+      <x:c r="H76" s="36" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I76" s="36" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J76" s="36" t="str">
+        <x:v>待注册：npm run test:case -- TC-071</x:v>
+      </x:c>
+      <x:c r="K76" s="36" t="str">
+        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-071 超管创建账户和审计边界')</x:v>
+      </x:c>
+      <x:c r="L76" s="36" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M76" s="36" t="str">
+        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc071-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="82" customHeight="1">
+      <x:c r="A77" s="37" t="str">
+        <x:v>TC-072</x:v>
+      </x:c>
+      <x:c r="B77" s="37" t="str">
+        <x:v>REQ-035</x:v>
+      </x:c>
+      <x:c r="C77" s="37" t="str">
+        <x:v>DEV-040</x:v>
+      </x:c>
+      <x:c r="D77" s="37" t="str">
+        <x:v>目标 Mac 文件授权手工验收</x:v>
+      </x:c>
+      <x:c r="E77" s="37" t="str">
+        <x:v>人工</x:v>
+      </x:c>
+      <x:c r="F77" s="37" t="str">
+        <x:v>独立测试用户数据、目标 Mac、可控测试目录；先拒绝再手动授予文件权限。</x:v>
+      </x:c>
+      <x:c r="G77" s="37" t="str">
+        <x:v>指引与系统设置路径可执行，重新扫描恢复；无权限时不越权且显示未知。</x:v>
+      </x:c>
+      <x:c r="H77" s="37" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+      <x:c r="I77" s="37" t="str">
+        <x:v>尚无测试运行结果</x:v>
+      </x:c>
+      <x:c r="J77" s="37" t="str">
+        <x:v>待注册：npm run test:case -- TC-072</x:v>
+      </x:c>
+      <x:c r="K77" s="37" t="str">
+        <x:v>计划绑定 scripts/test-cases.mjs 人工清单</x:v>
+      </x:c>
+      <x:c r="L77" s="37" t="str">
+        <x:v>未注册；不可执行</x:v>
+      </x:c>
+      <x:c r="M77" s="37" t="str">
+        <x:v>使用独立临时用户数据目录 token-test-db-tc072；真实 Mac 授权操作后留脱敏证据，未执行不得 pass。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record M6 implementation and final acceptance evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3eb70382dfd64eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R623952fe022a4f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7e34ee02e4ee4f59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R522c444409674d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd52ae2341b6a4dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R56d2bfbf2b014c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re70ea8cadffe4e18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5d60f5d01b2646b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1700,7 +1700,7 @@
         <x:v>Codex 工作目录识别</x:v>
       </x:c>
       <x:c r="G56" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="66" customHeight="1">
@@ -1723,7 +1723,7 @@
         <x:v>Claude 工作目录识别</x:v>
       </x:c>
       <x:c r="G57" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="66" customHeight="1">
@@ -1746,7 +1746,7 @@
         <x:v>同名项目与路径本机边界</x:v>
       </x:c>
       <x:c r="G58" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="66" customHeight="1">
@@ -1769,7 +1769,7 @@
         <x:v>项目模型聚合及权限</x:v>
       </x:c>
       <x:c r="G59" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="66" customHeight="1">
@@ -1792,7 +1792,7 @@
         <x:v>分析视图筛选与下钻</x:v>
       </x:c>
       <x:c r="G60" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="66" customHeight="1">
@@ -1815,7 +1815,7 @@
         <x:v>项目模型 CSV 一致性</x:v>
       </x:c>
       <x:c r="G61" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="66" customHeight="1">
@@ -1838,7 +1838,7 @@
         <x:v>侧栏固定右侧独立滚动</x:v>
       </x:c>
       <x:c r="G62" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="66" customHeight="1">
@@ -1861,7 +1861,7 @@
         <x:v>窗口自适应与面包屑</x:v>
       </x:c>
       <x:c r="G63" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="66" customHeight="1">
@@ -1884,7 +1884,7 @@
         <x:v>更新入口可发现</x:v>
       </x:c>
       <x:c r="G64" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="66" customHeight="1">
@@ -1907,7 +1907,7 @@
         <x:v>更新状态与失败恢复</x:v>
       </x:c>
       <x:c r="G65" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="66" customHeight="1">
@@ -1930,7 +1930,7 @@
         <x:v>集中设置权限</x:v>
       </x:c>
       <x:c r="G66" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="66" customHeight="1">
@@ -1953,7 +1953,7 @@
         <x:v>权限缺失指引与重试</x:v>
       </x:c>
       <x:c r="G67" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="66" customHeight="1">
@@ -1976,7 +1976,7 @@
         <x:v>漏采链路定位</x:v>
       </x:c>
       <x:c r="G68" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="66" customHeight="1">
@@ -1999,7 +1999,7 @@
         <x:v>诊断脱敏与权限</x:v>
       </x:c>
       <x:c r="G69" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="66" customHeight="1">
@@ -2022,7 +2022,7 @@
         <x:v>反馈预览与提交</x:v>
       </x:c>
       <x:c r="G70" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="66" customHeight="1">
@@ -2045,7 +2045,7 @@
         <x:v>反馈鉴权与失败重试</x:v>
       </x:c>
       <x:c r="G71" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="66" customHeight="1">
@@ -2068,7 +2068,7 @@
         <x:v>管理员反馈列表权限</x:v>
       </x:c>
       <x:c r="G72" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="66" customHeight="1">
@@ -2091,7 +2091,7 @@
         <x:v>管理员账号采集状态</x:v>
       </x:c>
       <x:c r="G73" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="66" customHeight="1">
@@ -2114,7 +2114,7 @@
         <x:v>固定 admin 初始化</x:v>
       </x:c>
       <x:c r="G74" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="66" customHeight="1">
@@ -2137,7 +2137,7 @@
         <x:v>派生三级角色与管理边界</x:v>
       </x:c>
       <x:c r="G75" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="66" customHeight="1">
@@ -2160,7 +2160,7 @@
         <x:v>旧库 admin 迁移及冲突</x:v>
       </x:c>
       <x:c r="G76" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="66" customHeight="1">
@@ -2183,7 +2183,7 @@
         <x:v>超管创建角色与审计边界</x:v>
       </x:c>
       <x:c r="G77" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="66" customHeight="1">
@@ -2206,7 +2206,7 @@
         <x:v>目标 Mac 文件授权手工验收</x:v>
       </x:c>
       <x:c r="G78" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>待验证（人工）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2245,7 +2245,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；M6 REQ-031–039 为规划项，候选功能未分配本轮编号。</x:v>
+        <x:v>REQ-001–039；M6 REQ-031–039 代码已落地，TC-050–071 自动结果通过，TC-072 目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3082,10 +3082,10 @@
         <x:v>从 Codex/Claude 会话工作目录自动建议稳定项目归属，展示项目名；缺失或无效目录为“未知项目”，同名不同路径不得误合并；原始完整路径仅本机存储，不进入聚合上报、反馈或诊断外发。</x:v>
       </x:c>
       <x:c r="D36" s="36" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E36" s="36" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F36" s="36" t="str">
         <x:v>DEV-034、DEV-035</x:v>
@@ -3094,7 +3094,7 @@
         <x:v>TC-050、TC-051、TC-052</x:v>
       </x:c>
       <x:c r="H36" s="36" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="66" customHeight="1">
@@ -3108,10 +3108,10 @@
         <x:v>按授权用户、项目、模型、提供方和时间区间查看 Token 分类、总量、请求数、趋势与排行；项目×模型筛选下钻与 CSV 同口径，未知项目可见，不重复计数。</x:v>
       </x:c>
       <x:c r="D37" s="37" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E37" s="37" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F37" s="37" t="str">
         <x:v>DEV-036、DEV-037</x:v>
@@ -3120,7 +3120,7 @@
         <x:v>TC-053、TC-054、TC-055</x:v>
       </x:c>
       <x:c r="H37" s="37" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="66" customHeight="1">
@@ -3134,10 +3134,10 @@
         <x:v>应用侧栏固定，右侧内容独立滚动；窗口宽度变化时内容不遮挡、可操作；页面面包屑与当前导航和下钻路径一致。</x:v>
       </x:c>
       <x:c r="D38" s="36" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E38" s="36" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F38" s="36" t="str">
         <x:v>DEV-038</x:v>
@@ -3146,7 +3146,7 @@
         <x:v>TC-056、TC-057</x:v>
       </x:c>
       <x:c r="H38" s="36" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="66" customHeight="1">
@@ -3160,10 +3160,10 @@
         <x:v>把已有“检查更新”移至明显导航或设置位置，展示检查中、最新版本、发现版本、下载、校验、打开安装包及可恢复失败状态；不自动替换未签名应用。</x:v>
       </x:c>
       <x:c r="D39" s="37" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E39" s="37" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F39" s="37" t="str">
         <x:v>DEV-039</x:v>
@@ -3172,7 +3172,7 @@
         <x:v>TC-058、TC-059</x:v>
       </x:c>
       <x:c r="H39" s="37" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="66" customHeight="1">
@@ -3186,10 +3186,10 @@
         <x:v>集中展示服务器、采集、更新与本机权限设置；按角色保护修改入口；来源无权限时说明所需 macOS 操作和重试路径，不自动提权或读取其他账户文件。</x:v>
       </x:c>
       <x:c r="D40" s="36" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E40" s="36" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（TC-072 目标 Mac 待验）</x:v>
       </x:c>
       <x:c r="F40" s="36" t="str">
         <x:v>DEV-040</x:v>
@@ -3198,7 +3198,7 @@
         <x:v>TC-060、TC-061、TC-072</x:v>
       </x:c>
       <x:c r="H40" s="36" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -3212,10 +3212,10 @@
         <x:v>按来源列出检测、解析、游标、覆盖区间、最近成功/失败和未归属原因，能定位漏采环节；未知与真实零分离；诊断信息脱敏，原始路径只在本机可见。</x:v>
       </x:c>
       <x:c r="D41" s="37" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E41" s="37" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F41" s="37" t="str">
         <x:v>DEV-041</x:v>
@@ -3224,7 +3224,7 @@
         <x:v>TC-062、TC-063</x:v>
       </x:c>
       <x:c r="H41" s="37" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="66" customHeight="1">
@@ -3238,10 +3238,10 @@
         <x:v>用户显式提交反馈到配置的服务端，提交前可预览白名单字段；不包含提示词、源码、密钥或完整项目路径；失败可重试且不重复生成反馈。</x:v>
       </x:c>
       <x:c r="D42" s="36" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E42" s="36" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F42" s="36" t="str">
         <x:v>DEV-042、DEV-043</x:v>
@@ -3250,7 +3250,7 @@
         <x:v>TC-064、TC-065</x:v>
       </x:c>
       <x:c r="H42" s="36" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="66" customHeight="1">
@@ -3264,10 +3264,10 @@
         <x:v>管理员及超管可查看授权范围内的反馈、账号启停/角色状态和采集健康状态；普通用户不能跨用户读取或调用管理 IPC；查看不等于处理闭环。</x:v>
       </x:c>
       <x:c r="D43" s="37" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E43" s="37" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F43" s="37" t="str">
         <x:v>DEV-044</x:v>
@@ -3276,7 +3276,7 @@
         <x:v>TC-066、TC-067</x:v>
       </x:c>
       <x:c r="H43" s="37" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="66" customHeight="1">
@@ -3290,10 +3290,10 @@
         <x:v>全新安装首建固定用户名 admin；库内仍存 admin/viewer，仅用户名 admin 且库角色 admin 对外呈现 superadmin；旧库该账号自动成为超管，其他管理员保留原权限；旧库无 admin 时现有管理员可创建之；非超管不得停用或重置该账号，冲突不得静默升权。</x:v>
       </x:c>
       <x:c r="D44" s="36" t="str">
-        <x:v>M6（规划）</x:v>
+        <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E44" s="36" t="str">
-        <x:v>待开发</x:v>
+        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="F44" s="36" t="str">
         <x:v>DEV-045、DEV-046</x:v>
@@ -3302,7 +3302,7 @@
         <x:v>TC-068、TC-069、TC-070、TC-071</x:v>
       </x:c>
       <x:c r="H44" s="36" t="str">
-        <x:v>docs/design.md §14–19；docs/development-plan.md §8</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4153,13 +4153,13 @@
         <x:v>TC-050、TC-051</x:v>
       </x:c>
       <x:c r="E39" s="37" t="str">
-        <x:v>src/collectors/codex.ts；src/collectors/claude.ts；tests/m6-project.test.ts</x:v>
+        <x:v>src/collectors/codex.ts、claude.ts、project.ts；tests/m6-project.test.ts</x:v>
       </x:c>
       <x:c r="F39" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G39" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="66" customHeight="1">
@@ -4176,13 +4176,13 @@
         <x:v>TC-052</x:v>
       </x:c>
       <x:c r="E40" s="36" t="str">
-        <x:v>src/main/database.ts；src/main/usage-sync.ts；tests/m6-project.test.ts</x:v>
+        <x:v>src/collectors/project.ts、scanner.ts；src/main/database.ts；tests/m6-project.test.ts</x:v>
       </x:c>
       <x:c r="F40" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G40" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -4202,10 +4202,10 @@
         <x:v>src/main/report.ts；src/shared/types.ts；tests/m6-report.test.ts</x:v>
       </x:c>
       <x:c r="F41" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G41" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="66" customHeight="1">
@@ -4225,10 +4225,10 @@
         <x:v>src/renderer/report.tsx；tests/e2e/m6-analysis.spec.ts</x:v>
       </x:c>
       <x:c r="F42" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G42" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="66" customHeight="1">
@@ -4245,13 +4245,13 @@
         <x:v>TC-056、TC-057</x:v>
       </x:c>
       <x:c r="E43" s="37" t="str">
-        <x:v>src/renderer/index.tsx；src/renderer/style.css；tests/e2e/m6-shell.spec.ts</x:v>
+        <x:v>src/renderer/index.tsx、style.css；tests/e2e/m6-shell.spec.ts</x:v>
       </x:c>
       <x:c r="F43" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G43" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="66" customHeight="1">
@@ -4268,13 +4268,13 @@
         <x:v>TC-058、TC-059</x:v>
       </x:c>
       <x:c r="E44" s="36" t="str">
-        <x:v>src/renderer/index.tsx；src/main/update-client.ts；tests/e2e/m6-update.spec.ts</x:v>
+        <x:v>src/renderer/settings.tsx、index.tsx；tests/e2e/m6-update.spec.ts</x:v>
       </x:c>
       <x:c r="F44" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G44" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="66" customHeight="1">
@@ -4291,13 +4291,13 @@
         <x:v>TC-060、TC-061、TC-072</x:v>
       </x:c>
       <x:c r="E45" s="37" t="str">
-        <x:v>src/renderer/index.tsx；src/main/index.ts；tests/e2e/m6-settings.spec.ts</x:v>
+        <x:v>src/renderer/settings.tsx；src/main/index.ts；tests/e2e/m6-settings.spec.ts</x:v>
       </x:c>
       <x:c r="F45" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（TC-072 人工待验）</x:v>
       </x:c>
       <x:c r="G45" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="66" customHeight="1">
@@ -4314,13 +4314,13 @@
         <x:v>TC-062、TC-063</x:v>
       </x:c>
       <x:c r="E46" s="36" t="str">
-        <x:v>src/collectors/scanner.ts；src/main/index.ts；tests/m6-diagnostics.test.ts</x:v>
+        <x:v>src/collectors/scanner.ts；src/renderer/diagnostics.tsx；tests/m6-diagnostics.test.ts</x:v>
       </x:c>
       <x:c r="F46" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G46" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="66" customHeight="1">
@@ -4337,13 +4337,13 @@
         <x:v>TC-064</x:v>
       </x:c>
       <x:c r="E47" s="37" t="str">
-        <x:v>src/renderer/index.tsx；src/main/feedback.ts；tests/m6-feedback.test.ts</x:v>
+        <x:v>src/main/feedback.ts；src/renderer/feedback.tsx；tests/m6-feedback.test.ts</x:v>
       </x:c>
       <x:c r="F47" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G47" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="66" customHeight="1">
@@ -4363,10 +4363,10 @@
         <x:v>src/server/server.ts；tests/m6-feedback.test.ts</x:v>
       </x:c>
       <x:c r="F48" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G48" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="66" customHeight="1">
@@ -4386,10 +4386,10 @@
         <x:v>src/main/index.ts；src/renderer/index.tsx；tests/e2e/m6-admin.spec.ts</x:v>
       </x:c>
       <x:c r="F49" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G49" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="66" customHeight="1">
@@ -4406,13 +4406,13 @@
         <x:v>TC-068、TC-070</x:v>
       </x:c>
       <x:c r="E50" s="36" t="str">
-        <x:v>src/main/auth.ts；src/main/database.ts；tests/m6-roles.test.ts</x:v>
+        <x:v>src/main/auth.ts、database.ts；tests/m6-roles.test.ts</x:v>
       </x:c>
       <x:c r="F50" s="36" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G50" s="36" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="66" customHeight="1">
@@ -4429,13 +4429,13 @@
         <x:v>TC-069、TC-071</x:v>
       </x:c>
       <x:c r="E51" s="37" t="str">
-        <x:v>src/main/auth.ts；src/main/index.ts；src/renderer/index.tsx；tests/m6-roles.test.ts</x:v>
+        <x:v>src/main/auth.ts、index.ts；src/renderer/index.tsx；tests/m6-roles.test.ts</x:v>
       </x:c>
       <x:c r="F51" s="37" t="str">
-        <x:v>待启动</x:v>
+        <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G51" s="37" t="str">
-        <x:v>M6 文档方案；代码与测试尚未实现</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4480,7 +4480,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–049 已有入口；TC-050–072 仅规划，scripts/test-cases.mjs 尚未注册，不得写成可执行或通过。</x:v>
+        <x:v>TC-001–072 已注册；TC-050–071 于 6223c30 逐编号自动通过，TC-072 仅人工清单、尚未验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6580,22 +6580,22 @@
         <x:v>项目稳定归属；无目录保持未知，不读取工作目录内容。</x:v>
       </x:c>
       <x:c r="H55" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I55" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:36 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-050.log</x:v>
       </x:c>
       <x:c r="J55" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-050</x:v>
+        <x:v>npm run test:case -- TC-050</x:v>
       </x:c>
       <x:c r="K55" s="37" t="str">
-        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-050 Codex 工作目录归属')</x:v>
+        <x:v>tests/m6-project.test.ts：test('TC-050 Codex cwd 归属与缺失项目保持未知')</x:v>
       </x:c>
       <x:c r="L55" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>合成 Codex cwd 归属及缺失为未知；真实版本格式变化未覆盖。</x:v>
       </x:c>
       <x:c r="M55" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc050-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-050 创建 token-test-db-tc050-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="82" customHeight="1">
@@ -6621,22 +6621,22 @@
         <x:v>同会话归属一致；缺失为未知，子代理不误归其他项目。</x:v>
       </x:c>
       <x:c r="H56" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I56" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:37 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-051.log</x:v>
       </x:c>
       <x:c r="J56" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-051</x:v>
+        <x:v>npm run test:case -- TC-051</x:v>
       </x:c>
       <x:c r="K56" s="36" t="str">
-        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-051 Claude 工作目录归属')</x:v>
+        <x:v>tests/m6-project.test.ts：test('TC-051 Claude cwd 和子代理文件独立归属')</x:v>
       </x:c>
       <x:c r="L56" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>合成 Claude 主/子代理分开归属及缺失为未知；其他真实子代理格式未覆盖。</x:v>
       </x:c>
       <x:c r="M56" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc051-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-051 创建 token-test-db-tc051-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="82" customHeight="1">
@@ -6662,22 +6662,22 @@
         <x:v>内部项目标识区分；显示名可区分；外发无完整路径、项目 ID 或别名；旧事实无 cwd 保持未知。</x:v>
       </x:c>
       <x:c r="H57" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I57" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:38 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-052.log</x:v>
       </x:c>
       <x:c r="J57" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-052</x:v>
+        <x:v>npm run test:case -- TC-052</x:v>
       </x:c>
       <x:c r="K57" s="37" t="str">
-        <x:v>计划绑定 tests/m6-project.test.ts：test('TC-052 同名项目不合并且完整路径不外传')</x:v>
+        <x:v>tests/m6-project.test.ts：test('TC-052 同名路径不合并且外发摘要无项目标识')</x:v>
       </x:c>
       <x:c r="L57" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>同名不同路径分开；诊断摘要无路径/项目键，其他外发通道另见 TC-064。</x:v>
       </x:c>
       <x:c r="M57" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc052-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-052 创建 token-test-db-tc052-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="82" customHeight="1">
@@ -6703,22 +6703,22 @@
         <x:v>聚合等于授权事实求和，普通用户不越权，未知项目单列。</x:v>
       </x:c>
       <x:c r="H58" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I58" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:39 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-053.log</x:v>
       </x:c>
       <x:c r="J58" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-053</x:v>
+        <x:v>npm run test:case -- TC-053</x:v>
       </x:c>
       <x:c r="K58" s="36" t="str">
-        <x:v>计划绑定 tests/m6-report.test.ts：test('TC-053 项目模型聚合权限与时区')</x:v>
+        <x:v>tests/m6-report.test.ts：test('TC-053 项目模型聚合沿用授权范围和未知项目')</x:v>
       </x:c>
       <x:c r="L58" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>多用户授权、项目/模型/未知聚合；只覆盖 UTC 示例。</x:v>
       </x:c>
       <x:c r="M58" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc053-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-053 创建 token-test-db-tc053-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="82" customHeight="1">
@@ -6744,22 +6744,22 @@
         <x:v>项目/模型排行、趋势和下钻同筛选，切换不会混入其他项目。</x:v>
       </x:c>
       <x:c r="H59" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I59" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:41 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-054.log</x:v>
       </x:c>
       <x:c r="J59" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-054</x:v>
+        <x:v>npm run test:case -- TC-054</x:v>
       </x:c>
       <x:c r="K59" s="37" t="str">
-        <x:v>计划绑定 tests/e2e/m6-analysis.spec.ts：test('TC-054 项目模型分析筛选下钻')</x:v>
+        <x:v>tests/e2e/m6-analysis.spec.ts：test('TC-054 项目模型筛选及趋势下钻保持同一用量范围')</x:v>
       </x:c>
       <x:c r="L59" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>Electron 项目筛选、42→12 Token 与一次日下钻；其他粒度组合待测。</x:v>
       </x:c>
       <x:c r="M59" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc054-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-054 创建 token-test-db-tc054-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="82" customHeight="1">
@@ -6785,22 +6785,22 @@
         <x:v>页面、明细、CSV 总量/分类一致；文本防公式注入；路径不导出。</x:v>
       </x:c>
       <x:c r="H60" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I60" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:47 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-055.log</x:v>
       </x:c>
       <x:c r="J60" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-055</x:v>
+        <x:v>npm run test:case -- TC-055</x:v>
       </x:c>
       <x:c r="K60" s="36" t="str">
-        <x:v>计划绑定 tests/m6-report.test.ts：test('TC-055 项目模型页面与 CSV 对账')</x:v>
+        <x:v>tests/m6-report.test.ts：test('TC-055 项目筛选 CSV 与页面同口径且文本安全')</x:v>
       </x:c>
       <x:c r="L60" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>项目 CSV 与页面/明细 10 Token 对账、公式文本转义；大数据量待测。</x:v>
       </x:c>
       <x:c r="M60" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc055-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-055 创建 token-test-db-tc055-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="82" customHeight="1">
@@ -6826,22 +6826,22 @@
         <x:v>侧栏位置不变、右侧独立滚动，焦点和操作可见。</x:v>
       </x:c>
       <x:c r="H61" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I61" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:48 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-056.log</x:v>
       </x:c>
       <x:c r="J61" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-056</x:v>
+        <x:v>npm run test:case -- TC-056</x:v>
       </x:c>
       <x:c r="K61" s="37" t="str">
-        <x:v>计划绑定 tests/e2e/m6-shell.spec.ts：test('TC-056 固定侧栏和右侧滚动')</x:v>
+        <x:v>tests/e2e/m6-shell.spec.ts：test('TC-056 长报表右侧滚动时左侧导航保持固定')</x:v>
       </x:c>
       <x:c r="L61" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>长页右侧滚动时侧栏位置不变；键盘焦点与更多尺寸待测。</x:v>
       </x:c>
       <x:c r="M61" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc056-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-056 创建 token-test-db-tc056-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="82" customHeight="1">
@@ -6867,22 +6867,22 @@
         <x:v>无遮挡和横向丢失；面包屑反映层级并可回退。</x:v>
       </x:c>
       <x:c r="H62" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I62" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:56:54 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-057.log</x:v>
       </x:c>
       <x:c r="J62" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-057</x:v>
+        <x:v>npm run test:case -- TC-057</x:v>
       </x:c>
       <x:c r="K62" s="36" t="str">
-        <x:v>计划绑定 tests/e2e/m6-shell.spec.ts：test('TC-057 响应式布局和面包屑')</x:v>
+        <x:v>tests/e2e/m6-shell.spec.ts：test('TC-057 窄窗口路径可见且下钻可从面包屑返回')</x:v>
       </x:c>
       <x:c r="L62" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>760×700 窗口面包屑回退且无横向溢出；更窄尺寸待测。</x:v>
       </x:c>
       <x:c r="M62" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc057-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-057 创建 token-test-db-tc057-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="82" customHeight="1">
@@ -6908,22 +6908,22 @@
         <x:v>入口在显著位置且普通授权用户可找到；不重复藏在概览下方。</x:v>
       </x:c>
       <x:c r="H63" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I63" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:00 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-058.log</x:v>
       </x:c>
       <x:c r="J63" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-058</x:v>
+        <x:v>npm run test:case -- TC-058</x:v>
       </x:c>
       <x:c r="K63" s="37" t="str">
-        <x:v>计划绑定 tests/e2e/m6-update.spec.ts：test('TC-058 显著更新入口')</x:v>
+        <x:v>tests/e2e/m6-update.spec.ts：test('TC-058 登录后可直接发现检查更新入口')</x:v>
       </x:c>
       <x:c r="L63" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>登录后系统设置可发现检查更新；真实用户发现率未测。</x:v>
       </x:c>
       <x:c r="M63" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc058-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-058 创建 token-test-db-tc058-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="82" customHeight="1">
@@ -6949,22 +6949,22 @@
         <x:v>每阶段状态准确，错误可恢复；坏包不打开，旧版可用。</x:v>
       </x:c>
       <x:c r="H64" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I64" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:06 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-059.log</x:v>
       </x:c>
       <x:c r="J64" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-059</x:v>
+        <x:v>npm run test:case -- TC-059</x:v>
       </x:c>
       <x:c r="K64" s="36" t="str">
-        <x:v>计划绑定 tests/e2e/m6-update.spec.ts：test('TC-059 更新状态成功失败恢复')</x:v>
+        <x:v>tests/e2e/m6-update.spec.ts：test('TC-059 新版坏包提示错误且重试后可重新检查')</x:v>
       </x:c>
       <x:c r="L64" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>合成坏摘要拒绝、重查旧版显示最新；真实 DMG 安装未测。</x:v>
       </x:c>
       <x:c r="M64" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc059-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-059 创建 token-test-db-tc059-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="82" customHeight="1">
@@ -6990,22 +6990,22 @@
         <x:v>采集/更新/服务器/权限集中；受限角色不能调用管理修改 IPC。</x:v>
       </x:c>
       <x:c r="H65" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I65" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:12 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-060.log</x:v>
       </x:c>
       <x:c r="J65" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-060</x:v>
+        <x:v>npm run test:case -- TC-060</x:v>
       </x:c>
       <x:c r="K65" s="37" t="str">
-        <x:v>计划绑定 tests/e2e/m6-settings.spec.ts：test('TC-060 设置分组与角色保护')</x:v>
+        <x:v>tests/e2e/m6-settings.spec.ts：test('TC-060 设置分组完整且普通用户修改接口被拒绝')</x:v>
       </x:c>
       <x:c r="L65" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>设置分组与 viewer 修改 IPC 拒绝；普通管理员组合待测。</x:v>
       </x:c>
       <x:c r="M65" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc060-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-060 创建 token-test-db-tc060-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="82" customHeight="1">
@@ -7031,22 +7031,22 @@
         <x:v>显示具体来源、macOS 手动授权和重试路径；恢复后状态更新，不自动提权。</x:v>
       </x:c>
       <x:c r="H66" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I66" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:18 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-061.log</x:v>
       </x:c>
       <x:c r="J66" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-061</x:v>
+        <x:v>npm run test:case -- TC-061</x:v>
       </x:c>
       <x:c r="K66" s="36" t="str">
-        <x:v>计划绑定 tests/e2e/m6-settings.spec.ts：test('TC-061 macOS 文件权限指引模拟')</x:v>
+        <x:v>tests/e2e/m6-settings.spec.ts：test('TC-061 缺少目录时诊断引导权限设置和重新扫描')</x:v>
       </x:c>
       <x:c r="L66" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>缺目录显示权限指引及重扫入口；真实 Mac 授权见 TC-072。</x:v>
       </x:c>
       <x:c r="M66" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc061-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-061 创建 token-test-db-tc061-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="82" customHeight="1">
@@ -7072,22 +7072,22 @@
         <x:v>诊断指出对应环节和最后成功时间，不把未知当零。</x:v>
       </x:c>
       <x:c r="H67" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I67" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:24 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-062.log</x:v>
       </x:c>
       <x:c r="J67" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-062</x:v>
+        <x:v>npm run test:case -- TC-062</x:v>
       </x:c>
       <x:c r="K67" s="37" t="str">
-        <x:v>计划绑定 tests/m6-diagnostics.test.ts：test('TC-062 检测解析游标漏采定位')</x:v>
+        <x:v>tests/m6-diagnostics.test.ts：test('TC-062 缺目录解析错待写完记录及未归属有独立诊断')</x:v>
       </x:c>
       <x:c r="L67" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>缺目录、错误记录、待写尾行、未归属及最后成功；长期游标停滞未测。</x:v>
       </x:c>
       <x:c r="M67" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc062-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-062 创建 token-test-db-tc062-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="82" customHeight="1">
@@ -7113,22 +7113,22 @@
         <x:v>外发与日志无敏感字段；普通用户仅看授权来源。</x:v>
       </x:c>
       <x:c r="H68" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I68" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:25 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-063.log</x:v>
       </x:c>
       <x:c r="J68" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-063</x:v>
+        <x:v>npm run test:case -- TC-063</x:v>
       </x:c>
       <x:c r="K68" s="36" t="str">
-        <x:v>计划绑定 tests/m6-diagnostics.test.ts：test('TC-063 诊断脱敏和角色范围')</x:v>
+        <x:v>tests/m6-diagnostics.test.ts：test('TC-063 诊断摘要不包含原始路径正文与项目标识')</x:v>
       </x:c>
       <x:c r="L68" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>诊断摘要无合成路径/项目键；全部日志与外发渠道系统审计待补。</x:v>
       </x:c>
       <x:c r="M68" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc063-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-063 创建 token-test-db-tc063-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="82" customHeight="1">
@@ -7154,22 +7154,22 @@
         <x:v>用户确认后才发白名单数据；原始路径、正文、密钥不发送。</x:v>
       </x:c>
       <x:c r="H69" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I69" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:27 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-064.log</x:v>
       </x:c>
       <x:c r="J69" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-064</x:v>
+        <x:v>npm run test:case -- TC-064</x:v>
       </x:c>
       <x:c r="K69" s="37" t="str">
-        <x:v>计划绑定 tests/m6-feedback.test.ts：test('TC-064 反馈预览白名单提交')</x:v>
+        <x:v>tests/m6-feedback.test.ts：test('TC-064 反馈仅显式提交且阻止路径密钥进入服务')</x:v>
       </x:c>
       <x:c r="L69" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>反馈显式提交、路径/密钥样式拒绝、预生成编号入库；UI 用户名/编号预览另见 TC-066。</x:v>
       </x:c>
       <x:c r="M69" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc064-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-064 创建 token-test-db-tc064-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="82" customHeight="1">
@@ -7195,22 +7195,22 @@
         <x:v>无权拒绝；重试不重复入库；失败与成功状态可见。</x:v>
       </x:c>
       <x:c r="H70" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I70" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:28 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-065.log</x:v>
       </x:c>
       <x:c r="J70" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-065</x:v>
+        <x:v>npm run test:case -- TC-065</x:v>
       </x:c>
       <x:c r="K70" s="36" t="str">
-        <x:v>计划绑定 tests/m6-feedback.test.ts：test('TC-065 反馈鉴权幂等重试')</x:v>
+        <x:v>tests/m6-feedback.test.ts：test('TC-065 反馈离线持久化重试幂等且管理读取需独立密钥')</x:v>
       </x:c>
       <x:c r="L70" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>离线排队、恢复后幂等、独立管理密钥；长期退避未测。</x:v>
       </x:c>
       <x:c r="M70" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc065-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-065 创建 token-test-db-tc065-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="82" customHeight="1">
@@ -7236,22 +7236,22 @@
         <x:v>superadmin/admin 可按授权范围查看；viewer 无管理入口/IPC。</x:v>
       </x:c>
       <x:c r="H71" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I71" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:29 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-066.log</x:v>
       </x:c>
       <x:c r="J71" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-066</x:v>
+        <x:v>npm run test:case -- TC-066</x:v>
       </x:c>
       <x:c r="K71" s="37" t="str">
-        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-066 管理员反馈可见性')</x:v>
+        <x:v>tests/e2e/m6-admin.spec.ts：test('TC-066 管理员可看反馈列表而普通用户接口拒绝')</x:v>
       </x:c>
       <x:c r="L71" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>超管预览真实用户名/编号且提交一致、反馈列表可见，viewer 管理 IPC 拒绝；普通管理员视图待单测。</x:v>
       </x:c>
       <x:c r="M71" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc066-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-066 创建 token-test-db-tc066-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="82" customHeight="1">
@@ -7277,22 +7277,22 @@
         <x:v>管理员可见账号角色/启停及来源最近成功和错误；数据不越权。</x:v>
       </x:c>
       <x:c r="H72" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I72" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:35 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-067.log</x:v>
       </x:c>
       <x:c r="J72" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-067</x:v>
+        <x:v>npm run test:case -- TC-067</x:v>
       </x:c>
       <x:c r="K72" s="36" t="str">
-        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-067 管理员账号来源状态')</x:v>
+        <x:v>tests/e2e/m6-admin.spec.ts：test('TC-067 账号启停归属和采集状态随操作更新')</x:v>
       </x:c>
       <x:c r="L72" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>一名 viewer 的来源绑定、采集状态及停启；多来源异常待测。</x:v>
       </x:c>
       <x:c r="M72" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc067-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-067 创建 token-test-db-tc067-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="82" customHeight="1">
@@ -7318,22 +7318,22 @@
         <x:v>首建用户名固定 admin；库内 role=admin、对外 superadmin；重复初始化拒绝。</x:v>
       </x:c>
       <x:c r="H73" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I73" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:41 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-068.log</x:v>
       </x:c>
       <x:c r="J73" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-068</x:v>
+        <x:v>npm run test:case -- TC-068</x:v>
       </x:c>
       <x:c r="K73" s="37" t="str">
-        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-068 固定 admin 超管初始化')</x:v>
+        <x:v>tests/m6-roles.test.ts：test('TC-068 首建固定 admin 且库内角色兼容旧约束')</x:v>
       </x:c>
       <x:c r="L73" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>固定 admin 首建、库 role=admin/对外 superadmin、重复首建拒绝。</x:v>
       </x:c>
       <x:c r="M73" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc068-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-068 创建 token-test-db-tc068-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="82" customHeight="1">
@@ -7359,22 +7359,22 @@
         <x:v>仅固定 admin 对外 superadmin；其他管理员保持创建 admin/viewer 等原权限但不能停用/重置固定 admin；viewer 无管理权限。</x:v>
       </x:c>
       <x:c r="H74" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I74" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:42 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-069.log</x:v>
       </x:c>
       <x:c r="J74" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-069</x:v>
+        <x:v>npm run test:case -- TC-069</x:v>
       </x:c>
       <x:c r="K74" s="36" t="str">
-        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-069 派生超管和原管理员授权')</x:v>
+        <x:v>tests/m6-roles.test.ts：test('TC-069 普通管理员保留建户权限但不能改动固定 admin')</x:v>
       </x:c>
       <x:c r="L74" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>普通管理员保留建户权，不能停用/重置固定 admin；其他 IPC 待测。</x:v>
       </x:c>
       <x:c r="M74" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc069-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-069 创建 token-test-db-tc069-* / token.sqlite；合成 Codex/Claude 目录同属该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="82" customHeight="1">
@@ -7400,22 +7400,22 @@
         <x:v>已有 admin 管理员自动对外 superadmin；无 admin 时原管理员可创建之；其他账号/哈希/归属不变；viewer 冲突不自动升权且可回退。</x:v>
       </x:c>
       <x:c r="H75" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I75" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:43 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-070.log</x:v>
       </x:c>
       <x:c r="J75" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-070</x:v>
+        <x:v>npm run test:case -- TC-070</x:v>
       </x:c>
       <x:c r="K75" s="37" t="str">
-        <x:v>计划绑定 tests/m6-roles.test.ts：test('TC-070 旧库固定账号兼容')</x:v>
+        <x:v>tests/m6-roles.test.ts：test('TC-070 旧库 admin 冲突显式处理且保留账号 ID 和哈希')</x:v>
       </x:c>
       <x:c r="L75" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>旧库已有/无 admin 与 viewer 占用冲突、失败改名和哈希保留；生产库演练未做。</x:v>
       </x:c>
       <x:c r="M75" s="37" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc070-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-070 创建 token-test-db-tc070-*、tc070-existing-admin-*、tc070-missing-admin-* 各自独立 token.sqlite；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="82" customHeight="1">
@@ -7441,22 +7441,22 @@
         <x:v>超管可创建两类账号；普通管理员保留原创建权限但不能停用/重置固定 admin；若提供审计查看则仅超管可见。</x:v>
       </x:c>
       <x:c r="H76" s="36" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I76" s="36" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:45 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-071.log</x:v>
       </x:c>
       <x:c r="J76" s="36" t="str">
-        <x:v>待注册：npm run test:case -- TC-071</x:v>
+        <x:v>npm run test:case -- TC-071</x:v>
       </x:c>
       <x:c r="K76" s="36" t="str">
-        <x:v>计划绑定 tests/e2e/m6-admin.spec.ts：test('TC-071 超管创建账户和审计边界')</x:v>
+        <x:v>tests/e2e/m6-admin.spec.ts：test('TC-071 固定 admin 创建管理员与普通用户且角色边界生效')</x:v>
       </x:c>
       <x:c r="L76" s="36" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>超管界面建 admin/viewer，普通管理员不能停用/重置固定账号。</x:v>
       </x:c>
       <x:c r="M76" s="36" t="str">
-        <x:v>计划由 tests/support/test-workspace.ts 创建专用 token-test-db-tc071-* / token.sqlite；Electron 用 --token-user-data 指向该目录，服务用目录内随机端口；不读生产数据库，结束清理。</x:v>
+        <x:v>tests/support/test-workspace.ts 为 TC-071 创建 token-test-db-tc071-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="82" customHeight="1">
@@ -7482,22 +7482,22 @@
         <x:v>指引与系统设置路径可执行，重新扫描恢复；无权限时不越权且显示未知。</x:v>
       </x:c>
       <x:c r="H77" s="37" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>待验证（人工）</x:v>
       </x:c>
       <x:c r="I77" s="37" t="str">
-        <x:v>尚无测试运行结果</x:v>
+        <x:v>已注册人工清单；截至 2026-10-02 尚无目标 Mac 拒绝、授予、撤销文件访问权限的脱敏证据；不得登记 pass。</x:v>
       </x:c>
       <x:c r="J77" s="37" t="str">
-        <x:v>待注册：npm run test:case -- TC-072</x:v>
+        <x:v>npm run test:case -- TC-072</x:v>
       </x:c>
       <x:c r="K77" s="37" t="str">
-        <x:v>计划绑定 scripts/test-cases.mjs 人工清单</x:v>
+        <x:v>scripts/test-cases.mjs：TC-072 人工清单（非自动断言）</x:v>
       </x:c>
       <x:c r="L77" s="37" t="str">
-        <x:v>未注册；不可执行</x:v>
+        <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。</x:v>
       </x:c>
       <x:c r="M77" s="37" t="str">
-        <x:v>使用独立临时用户数据目录 token-test-db-tc072；真实 Mac 授权操作后留脱敏证据，未执行不得 pass。</x:v>
+        <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record v0.3.0 TC-027 local DMG acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd52ae2341b6a4dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R56d2bfbf2b014c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re70ea8cadffe4e18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5d60f5d01b2646b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R69f124c574b64410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbdaa21d74fc64e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc1456aef16b84873"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf31bb7ac2a4e4930"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2730,7 +2730,7 @@
         <x:v>TC-027</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
-        <x:v>docs/validation.md A10</x:v>
+        <x:v>历史：docs/validation.md A10；v0.3.0：同文 TC-027 新批次，本机未签名 DMG 人工 pass（2026-10-02）</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -3768,7 +3768,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
-        <x:v>2026-10-02 当前 Mac 未签名包</x:v>
+        <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5638,7 +5638,7 @@
         <x:v>已验证（人工）</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>docs/validation.md A10；2026-10-02</x:v>
+        <x:v>历史：docs/validation.md A10；2026-10-02。v0.3.0：2026-10-02 本机人工 pass；test-results/manual/TC-027.json、evidence/TC-027.md（本机 Git 忽略）；docs/validation.md 新批次</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
         <x:v>npm run test:case -- TC-027</x:v>
@@ -5647,10 +5647,10 @@
         <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
       </x:c>
       <x:c r="L32" s="9" t="str">
-        <x:v>人工入口；仅有历史证据</x:v>
+        <x:v>人工入口；v0.3.0 复制版 Playwright 主流程 1/1，加独立应用副本界面复核；原 A10 历史保留</x:v>
       </x:c>
       <x:c r="M32" s="9" t="str">
-        <x:v>DMG 校验输出、包哈希/版本、当前 Mac 信息、复制后应用的脱敏流程记录；历史 A10 不能替代本轮。</x:v>
+        <x:v>macOS 15.7.4 x86_64；代码 6223c30；Token-0.3.0.dmg SHA-256 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；hdiutil VALID、ditto 复制、启动/扫描/报表通过。截图 evidence/TC-027-report.png；Finder 拖拽、真实更新替换、签名公证、异机未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="60" customHeight="1">

</xml_diff>

<commit_message>
docs: record local 0.2 to 0.3 upgrade evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R69f124c574b64410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbdaa21d74fc64e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc1456aef16b84873"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf31bb7ac2a4e4930"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R982d9789a8ce477b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R5a839ee41c274d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R5ab9dd2080874cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re4908076999f4ee3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1355,7 +1355,7 @@
         <x:v>未签名安装包交接</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>部分验证（本机链路通过；取消/失败待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2877,7 +2877,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
+        <x:v>代码已落地；本机隔离升级链路部分验证</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -2886,7 +2886,7 @@
         <x:v>TC-036</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；新增：44a96e8 本机 0.2.0→0.3.0 交接/替换通过，取消/失败回退等未验；docs/validation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -3946,13 +3946,13 @@
         <x:v>TC-036</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>src/main/update-client.ts；tests/next-update.test.ts</x:v>
+        <x:v>src/main/update-client.ts；tests/next-update.test.ts；scripts/verify-local-upgrade.mjs</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>已编码（自动覆盖；边界待验）</x:v>
+        <x:v>已编码；本机隔离升级链路部分验证</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+        <x:v>历史自动测试 96e99be；新增 44a96e8 本机升级脚本重复通过，开发工作树 test-results/manual/evidence/TC-036-upgrade.log；边界见 docs/validation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -5996,7 +5996,7 @@
         <x:v>未签名安装包交接</x:v>
       </x:c>
       <x:c r="E41" s="35" t="str">
-        <x:v>单元</x:v>
+        <x:v>单元＋本机隔离链路</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
         <x:v>未签名包通过校验后下载，选择打开/取消。</x:v>
@@ -6005,22 +6005,22 @@
         <x:v>只打开安装包供用户安装；取消后旧版和数据仍可用。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>部分验证（本机交接/替换通过；取消/失败待验）</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>历史：96e99be 逐项自动日志（本机 Git 忽略）。新增：44a96e8，2026-10-02，本机脚本重复通过；开发工作树 test-results/manual/evidence/TC-036-upgrade.log；摘要见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
-        <x:v>npm run test:case -- TC-036</x:v>
+        <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
       </x:c>
       <x:c r="K41" s="35" t="str">
-        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>注入打开回调和旧文件；未测真实 Mac 打开/取消安装</x:v>
+        <x:v>历史单元仅注入打开回调。新增本机：DMG 验证、下载打开、同路径 ditto 替换、受信登录和合成 1280 Token 通过；未测取消、失败回退、Finder 安装、生产数据或异机。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>记录 TC-036 命令、退出码、提交、环境和脱敏日志；覆盖与限制：注入打开回调和旧文件；未测真实 Mac 打开/取消安装。</x:v>
+        <x:v>旧/新 DMG SHA-256 分别为 49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；本机日志见 I 列；签名公证与目标 Mac 另验。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">

</xml_diff>

<commit_message>
docs: record TC-036 cancellation and open failure evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R982d9789a8ce477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R5a839ee41c274d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R5ab9dd2080874cea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re4908076999f4ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1933ade2c5d442ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbb19d2612a5542ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R34e39fe781214fb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd19ce7166eb34a65"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1355,7 +1355,7 @@
         <x:v>未签名安装包交接</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>部分验证（本机链路通过；取消/失败待验）</x:v>
+        <x:v>部分验证（本机取消通过；Finder 回退待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2886,7 +2886,7 @@
         <x:v>TC-036</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；新增：44a96e8 本机 0.2.0→0.3.0 交接/替换通过，取消/失败回退等未验；docs/validation.md</x:v>
+        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -3952,7 +3952,7 @@
         <x:v>已编码；本机隔离升级链路部分验证</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>历史自动测试 96e99be；新增 44a96e8 本机升级脚本重复通过，开发工作树 test-results/manual/evidence/TC-036-upgrade.log；边界见 docs/validation.md</x:v>
+        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -6005,10 +6005,10 @@
         <x:v>只打开安装包供用户安装；取消后旧版和数据仍可用。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>部分验证（本机交接/替换通过；取消/失败待验）</x:v>
+        <x:v>部分验证（本机交接/替换/取消通过；真实安装回退待验）</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>历史：96e99be 逐项自动日志（本机 Git 忽略）。新增：44a96e8，2026-10-02，本机脚本重复通过；开发工作树 test-results/manual/evidence/TC-036-upgrade.log；摘要见 docs/validation.md</x:v>
+        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过。新增：2026-10-03 b224dde，TC-036 单元 1/1、本机升级脚本重复通过；开发工作树 test-results/manual/evidence/TC-036-cancel.log（Git 忽略），摘要见 docs/validation.md</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
         <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
@@ -6017,10 +6017,10 @@
         <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>历史单元仅注入打开回调。新增本机：DMG 验证、下载打开、同路径 ditto 替换、受信登录和合成 1280 Token 通过；未测取消、失败回退、Finder 安装、生产数据或异机。</x:v>
+        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变。Finder 真实失败回退、手动安装未测。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>旧/新 DMG SHA-256 分别为 49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；本机日志见 I 列；签名公证与目标 Mac 另验。</x:v>
+        <x:v>旧/新 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；2026-10-03 日志见 I 列；生产库迁移、签名公证及目标 Mac 另验。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">

</xml_diff>

<commit_message>
docs: plan Codex fallback reconciliation regression
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1933ade2c5d442ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbb19d2612a5542ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R34e39fe781214fb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd19ce7166eb34a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re76a05f507984427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc0c55bda31ad4d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa45f30864814c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re8b67ca806c94a67"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -139,6 +139,26 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -151,7 +171,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -260,6 +280,18 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2209,6 +2241,29 @@
         <x:v>待验证（人工）</x:v>
       </x:c>
     </x:row>
+    <x:row r="79" ht="76" customHeight="1">
+      <x:c r="A79" s="41" t="str">
+        <x:v>REQ-006</x:v>
+      </x:c>
+      <x:c r="B79" s="41" t="str">
+        <x:v>增量扫描与幂等恢复</x:v>
+      </x:c>
+      <x:c r="C79" s="41" t="str">
+        <x:v>DEV-047</x:v>
+      </x:c>
+      <x:c r="D79" s="41" t="str">
+        <x:v>修复 Codex fallback 跨扫描归并与旧库双事实</x:v>
+      </x:c>
+      <x:c r="E79" s="41" t="str">
+        <x:v>TC-073</x:v>
+      </x:c>
+      <x:c r="F79" s="41" t="str">
+        <x:v>Codex fallback 跨扫描归并</x:v>
+      </x:c>
+      <x:c r="G79" s="41" t="str">
+        <x:v>待验证（计划）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2245,7 +2300,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；M6 REQ-031–039 代码已落地，TC-050–071 自动结果通过，TC-072 目标 Mac 人工待验。</x:v>
+        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已规划 DEV-047 / TC-073，尚未修复。M6 REQ-031–039 本机代码已落地。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2421,7 +2476,7 @@
         <x:v>docs/feasibility.md §Claude Code；A4</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="54" customHeight="1">
+    <x:row r="11" ht="82" customHeight="1">
       <x:c r="A11" s="10" t="str">
         <x:v>REQ-006</x:v>
       </x:c>
@@ -2429,22 +2484,22 @@
         <x:v>增量扫描与幂等恢复</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>历史导入后持续扫描；重扫、重启、未写完末行、文件截断或轮转不造成重复计数。</x:v>
+        <x:v>历史导入后持续扫描；重扫、重启、未写完末行、文件截断或轮转不造成重复计数。Codex 同会话 fallback 后到正式记录时只计正式；旧库双事实可安全修复。</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>M2</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>已实现（本机）</x:v>
+        <x:v>部分实现（跨扫描替换缺陷待修）</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>DEV-006</x:v>
+        <x:v>DEV-006、DEV-047</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>TC-010、TC-011</x:v>
+        <x:v>TC-010、TC-011、TC-073</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>docs/design.md §4.3；A5</x:v>
+        <x:v>历史：docs/design.md §4.3；A5。新增缺口与方案：docs/design.md §4.4；DEV-047 / TC-073 尚未实施或验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -3339,7 +3394,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-02 仓库为准；变更后同步更新关系与验证证据。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 为待开发的 Codex fallback 跨扫描修复，其他任务按各行证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4436,6 +4491,29 @@
       </x:c>
       <x:c r="G51" s="37" t="str">
         <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="82" customHeight="1">
+      <x:c r="A52" s="40" t="str">
+        <x:v>DEV-047</x:v>
+      </x:c>
+      <x:c r="B52" s="40" t="str">
+        <x:v>修复 Codex fallback 跨扫描归并与旧库双事实</x:v>
+      </x:c>
+      <x:c r="C52" s="40" t="str">
+        <x:v>REQ-006</x:v>
+      </x:c>
+      <x:c r="D52" s="40" t="str">
+        <x:v>TC-073</x:v>
+      </x:c>
+      <x:c r="E52" s="40" t="str">
+        <x:v>src/collectors/codex.ts、scanner.ts；src/main/database.ts；计划 tests/collector-fallback.test.ts</x:v>
+      </x:c>
+      <x:c r="F52" s="40" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="G52" s="40" t="str">
+        <x:v>2026-10-03 文档计划；先复现跨扫描重复，再实现同会话正式事实优先和旧库幂等修复；不丢其他会话/来源/项目；见 docs/development-plan.md §9</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4480,7 +4558,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–072 已注册；TC-050–071 于 6223c30 逐编号自动通过，TC-072 仅人工清单、尚未验证。</x:v>
+        <x:v>TC-001–072 已注册；TC-050–071 于 6223c30 自动通过、TC-072 人工待验；TC-073 仅规划，尚未注册或验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7500,6 +7578,47 @@
         <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
       </x:c>
     </x:row>
+    <x:row r="78" ht="112" customHeight="1">
+      <x:c r="A78" s="40" t="str">
+        <x:v>TC-073</x:v>
+      </x:c>
+      <x:c r="B78" s="40" t="str">
+        <x:v>REQ-006</x:v>
+      </x:c>
+      <x:c r="C78" s="40" t="str">
+        <x:v>DEV-047</x:v>
+      </x:c>
+      <x:c r="D78" s="40" t="str">
+        <x:v>Codex fallback 跨扫描归并</x:v>
+      </x:c>
+      <x:c r="E78" s="40" t="str">
+        <x:v>单元/集成（计划）</x:v>
+      </x:c>
+      <x:c r="F78" s="40" t="str">
+        <x:v>独立临时库：先仅 event_msg:token_count 并首扫，再追加 token_usage_record 增量扫描；另造旧库双事实、其他会话/来源/项目对照。</x:v>
+      </x:c>
+      <x:c r="G78" s="40" t="str">
+        <x:v>同会话只保留正式总量；旧库启动修复不丢其他事实/归属/项目；重扫、重启、重复修复后事实数和报表总量稳定。</x:v>
+      </x:c>
+      <x:c r="H78" s="40" t="str">
+        <x:v>待验证（未注册）</x:v>
+      </x:c>
+      <x:c r="I78" s="40" t="str">
+        <x:v>2026-10-03 仅文档计划；尚无 TC-073 脚本、运行或通过证据；历史 TC-010/A5 不替代本项。</x:v>
+      </x:c>
+      <x:c r="J78" s="40" t="str">
+        <x:v>待注册：npm run test:case -- TC-073</x:v>
+      </x:c>
+      <x:c r="K78" s="40" t="str">
+        <x:v>计划绑定 tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描归并及旧库修复')</x:v>
+      </x:c>
+      <x:c r="L78" s="40" t="str">
+        <x:v>未注册、未执行；预计逐阶段核对事实键/数量、明细/汇总/导出总量及项目归属。</x:v>
+      </x:c>
+      <x:c r="M78" s="40" t="str">
+        <x:v>各子场景使用 tests/support/test-workspace.ts 的独立 token-test-db-tc073-* / token.sqlite 和合成 JSONL；不读生产库，结束清理；保存命令、提交、环境、退出码与脱敏事实对账。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record TC-073 implementation and regression evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re76a05f507984427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc0c55bda31ad4d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa45f30864814c9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re8b67ca806c94a67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd30e40f2e73a41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R01c1f0575eef429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R84590a1c73194f3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R241ab693910f4c8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2261,7 +2261,7 @@
         <x:v>Codex fallback 跨扫描归并</x:v>
       </x:c>
       <x:c r="G79" s="41" t="str">
-        <x:v>待验证（计划）</x:v>
+        <x:v>已验证（自动；打包待验）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2300,7 +2300,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已规划 DEV-047 / TC-073，尚未修复。M6 REQ-031–039 本机代码已落地。</x:v>
+        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已在 aa6d91b 修复并经 TC-073 合成数据验证；现有 0.3.0 DMG 待重建。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2490,7 +2490,7 @@
         <x:v>M2</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>部分实现（跨扫描替换缺陷待修）</x:v>
+        <x:v>代码已修复（合成回归通过；DMG 待重建）</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>DEV-006、DEV-047</x:v>
@@ -2499,7 +2499,7 @@
         <x:v>TC-010、TC-011、TC-073</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>历史：docs/design.md §4.3；A5。新增缺口与方案：docs/design.md §4.4；DEV-047 / TC-073 尚未实施或验证。</x:v>
+        <x:v>历史：docs/design.md §4.3/A5；规划：§4.4。当前：代码 aa6d91b、DEV-047 / TC-073 独立回归通过，见 docs/validation.md；现有 0.3.0 DMG 未含修复。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -3394,7 +3394,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 为待开发的 Codex fallback 跨扫描修复，其他任务按各行证据判定。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并自动验收，现有 0.3.0 DMG 未重建。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4507,13 +4507,13 @@
         <x:v>TC-073</x:v>
       </x:c>
       <x:c r="E52" s="40" t="str">
-        <x:v>src/collectors/codex.ts、scanner.ts；src/main/database.ts；计划 tests/collector-fallback.test.ts</x:v>
+        <x:v>src/collectors/scanner.ts；scripts/test-cases.mjs；tests/collector-fallback.test.ts（database.ts 未改）</x:v>
       </x:c>
       <x:c r="F52" s="40" t="str">
-        <x:v>待开发</x:v>
+        <x:v>已编码（自动验证；DMG 待重建）</x:v>
       </x:c>
       <x:c r="G52" s="40" t="str">
-        <x:v>2026-10-03 文档计划；先复现跨扫描重复，再实现同会话正式事实优先和旧库幂等修复；不丢其他会话/来源/项目；见 docs/development-plan.md §9</x:v>
+        <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；开发工作树 test-results/acceptance/TC-073.log；实际范围见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4558,7 +4558,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–072 已注册；TC-050–071 于 6223c30 自动通过、TC-072 人工待验；TC-073 仅规划，尚未注册或验证。</x:v>
+        <x:v>TC-001–073 已注册；TC-073 于 aa6d91b 以合成临时库单编号通过，TC-072 仍为目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7578,7 +7578,7 @@
         <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="112" customHeight="1">
+    <x:row r="78" ht="132" customHeight="1">
       <x:c r="A78" s="40" t="str">
         <x:v>TC-073</x:v>
       </x:c>
@@ -7592,7 +7592,7 @@
         <x:v>Codex fallback 跨扫描归并</x:v>
       </x:c>
       <x:c r="E78" s="40" t="str">
-        <x:v>单元/集成（计划）</x:v>
+        <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F78" s="40" t="str">
         <x:v>独立临时库：先仅 event_msg:token_count 并首扫，再追加 token_usage_record 增量扫描；另造旧库双事实、其他会话/来源/项目对照。</x:v>
@@ -7601,22 +7601,22 @@
         <x:v>同会话只保留正式总量；旧库启动修复不丢其他事实/归属/项目；重扫、重启、重复修复后事实数和报表总量稳定。</x:v>
       </x:c>
       <x:c r="H78" s="40" t="str">
-        <x:v>待验证（未注册）</x:v>
+        <x:v>已验证（自动；合成样本）</x:v>
       </x:c>
       <x:c r="I78" s="40" t="str">
-        <x:v>2026-10-03 仅文档计划；尚无 TC-073 脚本、运行或通过证据；历史 TC-010/A5 不替代本项。</x:v>
+        <x:v>2026-10-03 00:50 CST；aa6d91b；macOS 15.7.4 x86_64 / Node v24.15.0；TC-073 1/1、TC-010 单元+Electron，退出码 0。开发工作树 test-results/acceptance/TC-073.log 与 TC-010-fallback-regression.log（Git 忽略）；docs/validation.md。</x:v>
       </x:c>
       <x:c r="J78" s="40" t="str">
-        <x:v>待注册：npm run test:case -- TC-073</x:v>
+        <x:v>npm run test:case -- TC-073</x:v>
       </x:c>
       <x:c r="K78" s="40" t="str">
-        <x:v>计划绑定 tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描归并及旧库修复')</x:v>
+        <x:v>tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描替换与旧库修复保持幂等')；scripts/test-cases.mjs 已注册</x:v>
       </x:c>
       <x:c r="L78" s="40" t="str">
-        <x:v>未注册、未执行；预计逐阶段核对事实键/数量、明细/汇总/导出总量及项目归属。</x:v>
+        <x:v>首扫 fallback 12、次扫正式 12 且旧事实删除；明细/汇总/CSV 只计正式；跨文件后到 fallback 不重增；旧库仅清同会话 fallback/项目关联，其他会话、Claude、身份和项目保留；游标/旧库清理失败回滚，重扫重启稳定。真实生产库/未知格式及打包应用未验。</x:v>
       </x:c>
       <x:c r="M78" s="40" t="str">
-        <x:v>各子场景使用 tests/support/test-workspace.ts 的独立 token-test-db-tc073-* / token.sqlite 和合成 JSONL；不读生产库，结束清理；保存命令、提交、环境、退出码与脱敏事实对账。</x:v>
+        <x:v>tests/support/test-workspace.ts 的 tc073-incremental、tc073-legacy 两个独立临时 token.sqlite/合成 JSONL；结束清理。开发会话先见双 12 Token 失败再修复；本机日志见 I 列，文档会话单编号复跑通过。旧 Token-0.3.0.dmg 不含 aa6d91b；修复后包另验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.1 candidate upgrade evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd30e40f2e73a41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R01c1f0575eef429b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R84590a1c73194f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R241ab693910f4c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R978c4cb3c4d94c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R76fa959e773141ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd0a67d790ee34dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra4094e2e1f914f85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2261,7 +2261,7 @@
         <x:v>Codex fallback 跨扫描归并</x:v>
       </x:c>
       <x:c r="G79" s="41" t="str">
-        <x:v>已验证（自动；打包待验）</x:v>
+        <x:v>已验证（自动及本机候选包；生产安装待验）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2300,7 +2300,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已在 aa6d91b 修复并经 TC-073 合成数据验证；现有 0.3.0 DMG 待重建。</x:v>
+        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已在 aa6d91b 修复，TC-073 合成回归及 0.3.1 本机候选包同库升级通过；生产库/真实安装待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2476,7 +2476,7 @@
         <x:v>docs/feasibility.md §Claude Code；A4</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="82" customHeight="1">
+    <x:row r="11" ht="96" customHeight="1">
       <x:c r="A11" s="10" t="str">
         <x:v>REQ-006</x:v>
       </x:c>
@@ -2490,7 +2490,7 @@
         <x:v>M2</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>代码已修复（合成回归通过；DMG 待重建）</x:v>
+        <x:v>代码已修复（合成回归及 0.3.1 本机候选包同库升级通过）</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>DEV-006、DEV-047</x:v>
@@ -2499,7 +2499,7 @@
         <x:v>TC-010、TC-011、TC-073</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>历史：docs/design.md §4.3/A5；规划：§4.4。当前：代码 aa6d91b、DEV-047 / TC-073 独立回归通过，见 docs/validation.md；现有 0.3.0 DMG 未含修复。</x:v>
+        <x:v>历史：docs/design.md §4.3/A5；规划：§4.4；代码 aa6d91b、DEV-047 / TC-073 合成回归通过。2026-10-03：867a03a 制成 0.3.1 未签名候选包，同一隔离测试库从旧 0.3.0 的 2560 Token 升级后回到 1280；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库及真实安装待验，见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -3394,7 +3394,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并自动验收，现有 0.3.0 DMG 未重建。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并自动验收，867a03a 的 0.3.1 本机候选包同库升级通过；生产库/真实安装待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4493,7 +4493,7 @@
         <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="82" customHeight="1">
+    <x:row r="52" ht="108" customHeight="1">
       <x:c r="A52" s="40" t="str">
         <x:v>DEV-047</x:v>
       </x:c>
@@ -4510,10 +4510,10 @@
         <x:v>src/collectors/scanner.ts；scripts/test-cases.mjs；tests/collector-fallback.test.ts（database.ts 未改）</x:v>
       </x:c>
       <x:c r="F52" s="40" t="str">
-        <x:v>已编码（自动验证；DMG 待重建）</x:v>
+        <x:v>已编码（自动及 0.3.1 本机候选包验证）</x:v>
       </x:c>
       <x:c r="G52" s="40" t="str">
-        <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；开发工作树 test-results/acceptance/TC-073.log；实际范围见 docs/validation.md。</x:v>
+        <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b，0.3.1 制品 867a03a。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；2026-10-03 同一隔离库 0.3.0→0.3.1 复现 2560→修复 1280，文档会话独立复跑退出码 0；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库/实际安装待验，见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4558,7 +4558,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–073 已注册；TC-073 于 aa6d91b 以合成临时库单编号通过，TC-072 仍为目标 Mac 人工待验。</x:v>
+        <x:v>TC-001–073 已注册；TC-073 自动合成回归及 0.3.1 本机候选包隔离同库升级通过；TC-072 仍为目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6060,7 +6060,7 @@
         <x:v>记录 TC-035 命令、退出码、提交、环境和脱敏日志；覆盖与限制：停服/重试/临时文件；未测超时、磁盘不足。</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="70" customHeight="1">
+    <x:row r="41" ht="118" customHeight="1">
       <x:c r="A41" s="35" t="str">
         <x:v>TC-036</x:v>
       </x:c>
@@ -6086,7 +6086,7 @@
         <x:v>部分验证（本机交接/替换/取消通过；真实安装回退待验）</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过。新增：2026-10-03 b224dde，TC-036 单元 1/1、本机升级脚本重复通过；开发工作树 test-results/manual/evidence/TC-036-cancel.log（Git 忽略），摘要见 docs/validation.md</x:v>
+        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
         <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
@@ -6095,10 +6095,10 @@
         <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变。Finder 真实失败回退、手动安装未测。</x:v>
+        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>旧/新 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；2026-10-03 日志见 I 列；生产库迁移、签名公证及目标 Mac 另验。</x:v>
+        <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">
@@ -7578,7 +7578,7 @@
         <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" ht="132" customHeight="1">
+    <x:row r="78" ht="152" customHeight="1">
       <x:c r="A78" s="40" t="str">
         <x:v>TC-073</x:v>
       </x:c>
@@ -7601,10 +7601,10 @@
         <x:v>同会话只保留正式总量；旧库启动修复不丢其他事实/归属/项目；重扫、重启、重复修复后事实数和报表总量稳定。</x:v>
       </x:c>
       <x:c r="H78" s="40" t="str">
-        <x:v>已验证（自动；合成样本）</x:v>
+        <x:v>已验证（自动及 0.3.1 本机候选包；合成数据）</x:v>
       </x:c>
       <x:c r="I78" s="40" t="str">
-        <x:v>2026-10-03 00:50 CST；aa6d91b；macOS 15.7.4 x86_64 / Node v24.15.0；TC-073 1/1、TC-010 单元+Electron，退出码 0。开发工作树 test-results/acceptance/TC-073.log 与 TC-010-fallback-regression.log（Git 忽略）；docs/validation.md。</x:v>
+        <x:v>2026-10-03：aa6d91b TC-073 1/1、TC-010 单元+Electron，退出码 0；开发工作树 test-results/acceptance/TC-073.log。867a03a：0.3.1 未签名 x64 DMG SHA-256 7e56933298505f5d08def3811b891e187b6cefb264bfab3538e5accdb6235a7c，hdiutil VALID；文档会话独立复跑 --fallback-repair 退出码 0；开发工作树 test-results/manual/evidence/TC-073-package-upgrade.log（Git 忽略）；docs/validation.md。</x:v>
       </x:c>
       <x:c r="J78" s="40" t="str">
         <x:v>npm run test:case -- TC-073</x:v>
@@ -7613,10 +7613,10 @@
         <x:v>tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描替换与旧库修复保持幂等')；scripts/test-cases.mjs 已注册</x:v>
       </x:c>
       <x:c r="L78" s="40" t="str">
-        <x:v>首扫 fallback 12、次扫正式 12 且旧事实删除；明细/汇总/CSV 只计正式；跨文件后到 fallback 不重增；旧库仅清同会话 fallback/项目关联，其他会话、Claude、身份和项目保留；游标/旧库清理失败回滚，重扫重启稳定。真实生产库/未知格式及打包应用未验。</x:v>
+        <x:v>单元：首扫 fallback 12、次扫正式 12 且旧事实删除；明细/汇总/CSV 只计正式；跨文件后到 fallback 不重增；旧库仅清同会话 fallback/项目关联，其他会话、Claude、身份和项目保留；游标/旧库清理失败回滚，重扫重启稳定。0.3.1 本机候选包：同一隔离库旧版 1280→2560，新版回到 1280 且受信登录保留。真实生产库、未知格式及实际安装未验。</x:v>
       </x:c>
       <x:c r="M78" s="40" t="str">
-        <x:v>tests/support/test-workspace.ts 的 tc073-incremental、tc073-legacy 两个独立临时 token.sqlite/合成 JSONL；结束清理。开发会话先见双 12 Token 失败再修复；本机日志见 I 列，文档会话单编号复跑通过。旧 Token-0.3.0.dmg 不含 aa6d91b；修复后包另验。</x:v>
+        <x:v>单元使用 tc073-incremental、tc073-legacy 独立临时 token.sqlite/合成 JSONL。打包升级使用独立临时用户数据和安装目录；先在旧 0.3.0 包复现重复计数，下载并校验 0.3.1，取消分支保留旧版，再同库替换修复。文档会话独立复跑；本机服务目录已发布同哈希包，但生产账户 App 连接/安装、生产库及 Finder /Applications 未验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record TC-021 pagination acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R978c4cb3c4d94c36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R76fa959e773141ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd0a67d790ee34dc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra4094e2e1f914f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1284caa47d45417f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra9f9626beb0f4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb91c2a357bd54129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bcac8ba7d724436"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1042,7 +1042,7 @@
         <x:v>筛选与分页明细</x:v>
       </x:c>
       <x:c r="G26" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动；独立翻页）</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="38" customHeight="1">
@@ -2658,7 +2658,7 @@
         <x:v>docs/design.md §5；A8</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="54" customHeight="1">
+    <x:row r="18" ht="86" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>REQ-013</x:v>
       </x:c>
@@ -2681,7 +2681,7 @@
         <x:v>TC-021</x:v>
       </x:c>
       <x:c r="H18" s="9" t="str">
-        <x:v>docs/design.md §2、§5；A8</x:v>
+        <x:v>历史：docs/design.md §2、§5；A8。2026-10-03：代码 f7fcdee 为 TC-021 增加独立单元与 Electron 翻页验证；123 条合成事实的 50/50/23 分页、报表合计及普通用户授权范围通过；61 条合成 Codex 界面记录可翻第二页、切换模型回首页。见 docs/validation.md；产品行为未改。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -3711,7 +3711,7 @@
         <x:v>日、ISO 周、月、年与时区</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="54" customHeight="1">
+    <x:row r="18" ht="88" customHeight="1">
       <x:c r="A18" s="9" t="str">
         <x:v>DEV-013</x:v>
       </x:c>
@@ -3731,7 +3731,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="G18" s="9" t="str">
-        <x:v>同一事实集驱动汇总与明细</x:v>
+        <x:v>原实现由同一事实集驱动汇总与明细。2026-10-03 测试提交 f7fcdee 补强 TC-021：tests/report-pagination.test.ts 与 tests/e2e/report-pagination.spec.ts；单编号四个绑定通过，开发会话报告门禁 73 入口/42 单元/18 Electron 通过；合成数据边界见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -5443,7 +5443,7 @@
         <x:v>保存共享 Vitest 函数命令、退出码和周期值。</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="60" customHeight="1">
+    <x:row r="26" ht="138" customHeight="1">
       <x:c r="A26" s="9" t="str">
         <x:v>TC-021</x:v>
       </x:c>
@@ -5466,23 +5466,22 @@
         <x:v>汇总和授权明细一致，可定位对应记录。</x:v>
       </x:c>
       <x:c r="H26" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动；独立翻页）</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>tests/report.test.ts；tests/e2e/app.spec.ts；A8</x:v>
+        <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
         <x:v>npm run test:case -- TC-021</x:v>
       </x:c>
       <x:c r="K26" s="9" t="str">
-        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属
-tests/e2e/app.spec.ts：管理员创建、用户管理与普通用户权限</x:v>
+        <x:v>tests/report.test.ts：test('报表按本地时区与 ISO 周汇总，并限制普通用户归属')；tests/e2e/app.spec.ts：test('管理员创建、用户管理与普通用户权限')；tests/report-pagination.test.ts：test('TC-021 明细翻页不漏记录且筛选和用户权限贯穿每页')；tests/e2e/report-pagination.spec.ts：test('TC-021 报表明细可翻到第二页且切换模型重置页码')。四项均在 scripts/test-cases.mjs 绑定。</x:v>
       </x:c>
       <x:c r="L26" s="9" t="str">
-        <x:v>共享测试；非独立断言；第二页未测试</x:v>
+        <x:v>共享旧测试继续运行。独立单元：123 条事实分页 50/50/23、ID 不重复、总 Token 与报表一致；普通用户仅见 61 条、第二页 11 条，用户/提供方/模型/项目/日期筛选贯穿分页。独立 Electron：61 条合成 Codex 记录首屏 50、第二页 11，切换第二模型后回首页并显示 10。未用生产库或新版安装包；TC-047 跨用户服务授权未验。</x:v>
       </x:c>
       <x:c r="M26" s="9" t="str">
-        <x:v>保存两段共享测试日志；现有自动化没有构造超过 50 条以检查第二页分页。</x:v>
+        <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">

</xml_diff>

<commit_message>
docs: plan scoped usage upload authorization
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1284caa47d45417f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra9f9626beb0f4b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb91c2a357bd54129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bcac8ba7d724436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rdc7ce8ad09cf41c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6534cd0e38184c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rae28844e69314275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bc0f5f9889c4b7b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -159,6 +159,16 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -171,7 +181,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -292,6 +302,12 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1640,7 +1656,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>部分验证（跨用户覆盖缺陷已复现）</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2262,6 +2278,29 @@
       </x:c>
       <x:c r="G79" s="41" t="str">
         <x:v>已验证（自动及本机候选包；生产安装待验）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="82" customHeight="1">
+      <x:c r="A80" s="43" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="B80" s="43" t="str">
+        <x:v>独立本地更新与汇总服务</x:v>
+      </x:c>
+      <x:c r="C80" s="43" t="str">
+        <x:v>DEV-048</x:v>
+      </x:c>
+      <x:c r="D80" s="43" t="str">
+        <x:v>修复聚合上报的设备和用户归属授权</x:v>
+      </x:c>
+      <x:c r="E80" s="43" t="str">
+        <x:v>TC-074</x:v>
+      </x:c>
+      <x:c r="F80" s="43" t="str">
+        <x:v>聚合上报设备与用户归属授权回归</x:v>
+      </x:c>
+      <x:c r="G80" s="43" t="str">
+        <x:v>待验证（未注册；缺陷已复现）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2866,7 +2905,7 @@
         <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="62" customHeight="1">
+    <x:row r="26" ht="120" customHeight="1">
       <x:c r="A26" s="14" t="str">
         <x:v>REQ-021</x:v>
       </x:c>
@@ -2874,22 +2913,22 @@
         <x:v>独立本地更新与汇总服务</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>服务独立运行；监听主机/端口及 App 连接地址均可配置，默认 127.0.0.1；提供版本清单、安装包和聚合接口；非回环配置仍须鉴权并保护传输；服务故障不影响本机报表。</x:v>
+        <x:v>服务独立运行；监听主机/端口及 App 连接地址均可配置，默认 127.0.0.1；提供版本清单、安装包和聚合接口；非回环配置仍须鉴权并保护传输；服务故障不影响本机报表。聚合写入还须把可信请求身份与设备及允许的应用用户范围绑定；不得仅凭全局 bearer 或请求体自报 deviceId/ownerUserId 覆盖其他用户快照。拒绝越权时原聚合、修订和覆盖状态不变。</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
+        <x:v>部分实现（聚合归属授权缺口待修）</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
-        <x:v>DEV-022、DEV-023</x:v>
+        <x:v>DEV-022、DEV-023、DEV-048</x:v>
       </x:c>
       <x:c r="G26" s="14" t="str">
-        <x:v>TC-032、TC-033、TC-047</x:v>
+        <x:v>TC-032、TC-033、TC-047、TC-074</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+        <x:v>历史：docs/design.md §9–13；docs/development-plan.md §7；TC-047 已验证全局 bearer/字段/Origin/HTTPS 配置的部分断言。2026-10-03：开发会话隔离服务复现同一 bearer 可把同设备 owner A 的 12 Token 用 owner B 的 99 Token、较高修订覆盖；代码审查见 src/server/server.ts。DEV-048 / TC-074 待实施，SOP-002 选定管理密钥登记与独立设备令牌；见 docs/design.md §12.1–12.2、docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -3394,7 +3433,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并自动验收，867a03a 的 0.3.1 本机候选包同库升级通过；生产库/真实安装待验。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现，0.3.1 本机候选包同库升级通过；DEV-048 聚合归属授权修复待开发，相关证据见各行。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3941,7 +3980,7 @@
         <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="62" customHeight="1">
+    <x:row r="28" ht="100" customHeight="1">
       <x:c r="A28" s="14" t="str">
         <x:v>DEV-023</x:v>
       </x:c>
@@ -3958,10 +3997,10 @@
         <x:v>src/server/server.ts；tests/next-server.test.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>已编码（自动覆盖；边界待验）</x:v>
+        <x:v>已编码（部分自动覆盖；归属授权缺口）</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+        <x:v>历史：96e99be 的 TC-047 验证全局 bearer、字段白名单、Origin 与 HTTPS 配置；同一 bearer 跨用户覆盖未测。2026-10-03 隔离复现表明 src/server/server.ts 仅检查全局 bearer，较高修订按 device_id/provider 替换聚合；修复规划另见 DEV-048 / TC-074，当前不可标为完整授权通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4514,6 +4553,29 @@
       </x:c>
       <x:c r="G52" s="40" t="str">
         <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b，0.3.1 制品 867a03a。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；2026-10-03 同一隔离库 0.3.0→0.3.1 复现 2560→修复 1280，文档会话独立复跑退出码 0；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库/实际安装待验，见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="108" customHeight="1">
+      <x:c r="A53" s="42" t="str">
+        <x:v>DEV-048</x:v>
+      </x:c>
+      <x:c r="B53" s="42" t="str">
+        <x:v>修复聚合上报的设备和用户归属授权</x:v>
+      </x:c>
+      <x:c r="C53" s="42" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="D53" s="42" t="str">
+        <x:v>TC-074</x:v>
+      </x:c>
+      <x:c r="E53" s="42" t="str">
+        <x:v>计划 src/server/server.ts、src/main/server-connection.ts、src/main/usage-sync.ts、tests/server-ownership.test.ts；见 docs/design.md §12.2</x:v>
+      </x:c>
+      <x:c r="F53" s="42" t="str">
+        <x:v>待开发</x:v>
+      </x:c>
+      <x:c r="G53" s="42" t="str">
+        <x:v>2026-10-03 SOP-002 设计：保留全局 bearer 供原接口，管理密钥登记设备/允许 owner 并签发随机上报令牌；服务仅存令牌哈希并先授权后查修订/写库，客户端 safeStorage 加密保存。越权保持旧聚合、修订、覆盖；合法修订/幂等保留。旧数据与队列不自动清空，换服务重新登记，撤销不自动绕过；当前未编码或通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4558,7 +4620,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–073 已注册；TC-073 自动合成回归及 0.3.1 本机候选包隔离同库升级通过；TC-072 仍为目标 Mac 人工待验。</x:v>
+        <x:v>TC-001–073 已注册；TC-074 是聚合归属授权待开发独立回归，尚未注册/验证；TC-072 仍为目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -5443,7 +5505,7 @@
         <x:v>保存共享 Vitest 函数命令、退出码和周期值。</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="138" customHeight="1">
+    <x:row r="26" ht="158" customHeight="1">
       <x:c r="A26" s="9" t="str">
         <x:v>TC-021</x:v>
       </x:c>
@@ -5469,7 +5531,7 @@
         <x:v>已验证（自动；独立翻页）</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。</x:v>
+        <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。 后续：961c96c 补启动失败清理；8234dcc 补样本写入/数据库关闭异常清理。开发会话在 8234dcc 上报告类型检查、TC-021 单编号及完整门禁通过（73 入口/42 单元/18 Electron）；文档会话独立复跑四个绑定退出码 0；见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
         <x:v>npm run test:case -- TC-021</x:v>
@@ -5481,7 +5543,7 @@
         <x:v>共享旧测试继续运行。独立单元：123 条事实分页 50/50/23、ID 不重复、总 Token 与报表一致；普通用户仅见 61 条、第二页 11 条，用户/提供方/模型/项目/日期筛选贯穿分页。独立 Electron：61 条合成 Codex 记录首屏 50、第二页 11，切换第二模型后回首页并显示 10。未用生产库或新版安装包；TC-047 跨用户服务授权未验。</x:v>
       </x:c>
       <x:c r="M26" s="9" t="str">
-        <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。</x:v>
+        <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。 8234dcc 使测试异常时的一次性目录清理更完整；产品行为、断言和绑定未变。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -6511,7 +6573,7 @@
         <x:v>记录 TC-046 命令、退出码、提交、环境和脱敏日志；覆盖与限制：事实数/扫描时间/缺目录；未测全部状态卡片。</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="70" customHeight="1">
+    <x:row r="52" ht="146" customHeight="1">
       <x:c r="A52" s="14" t="str">
         <x:v>TC-047</x:v>
       </x:c>
@@ -6534,10 +6596,10 @@
         <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>部分验证（自动；跨用户覆盖缺陷已复现）</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>历史：96e99be 单编号自动断言通过，覆盖错误凭证、字段白名单、Origin 和 HTTPS 地址限制；开发日志被 Git 忽略。2026-10-03：开发会话用隔离 /tmp 服务和人工快照复现：同一 bearer 对同设备先报 owner A/revision 1/12 Token 得 200，再报 owner B/revision 2/99 Token 仍得 200（accepted=true, duplicate=false），旧聚合被替换；文档会话核对 src/server/server.ts。跨用户预期失败，见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J52" s="14" t="str">
         <x:v>npm run test:case -- TC-047</x:v>
@@ -6546,10 +6608,10 @@
         <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')</x:v>
       </x:c>
       <x:c r="L52" s="14" t="str">
-        <x:v>凭证/字段/Origin/HTTPS 地址；未在非回环 HTTPS 连接上验鉴权及跨用户授权</x:v>
+        <x:v>现有 tests/next-server.test.ts 只断言全局 bearer、字段、Origin 和 HTTPS 配置，不检验可信身份与 deviceId/ownerUserId 的绑定；跨用户修订覆盖在当前代码可发生。非回环 HTTPS 上的真实鉴权亦未验证。新增独立回归 TC-074 待注册/待通过，不能借 TC-047 自动通过宣称全项已验。</x:v>
       </x:c>
       <x:c r="M52" s="14" t="str">
-        <x:v>记录 TC-047 命令、退出码、提交、环境和脱敏日志；覆盖与限制：凭证/字段/Origin/HTTPS 地址；未在非回环 HTTPS 连接上验鉴权及跨用户授权。</x:v>
+        <x:v>保留 96e99be 及既有日志历史。隔离复现使用一次性 /tmp 服务数据库、两个人工 owner UUID 和同设备较高修订，无真实用户数据或密钥入库；结果见 I 列。修复后须复跑 TC-047 与 TC-074，并对账拒绝前后聚合、device_revisions、source_coverage；当前没有修复后证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="70" customHeight="1">
@@ -7616,6 +7678,47 @@
       </x:c>
       <x:c r="M78" s="40" t="str">
         <x:v>单元使用 tc073-incremental、tc073-legacy 独立临时 token.sqlite/合成 JSONL。打包升级使用独立临时用户数据和安装目录；先在旧 0.3.0 包复现重复计数，下载并校验 0.3.1，取消分支保留旧版，再同库替换修复。文档会话独立复跑；本机服务目录已发布同哈希包，但生产账户 App 连接/安装、生产库及 Finder /Applications 未验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="146" customHeight="1">
+      <x:c r="A79" s="42" t="str">
+        <x:v>TC-074</x:v>
+      </x:c>
+      <x:c r="B79" s="42" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="C79" s="42" t="str">
+        <x:v>DEV-048</x:v>
+      </x:c>
+      <x:c r="D79" s="42" t="str">
+        <x:v>聚合上报设备与用户归属授权回归</x:v>
+      </x:c>
+      <x:c r="E79" s="42" t="str">
+        <x:v>单元/集成（计划）</x:v>
+      </x:c>
+      <x:c r="F79" s="42" t="str">
+        <x:v>独立临时服务库：管理凭据登记设备 A/owner A 并签发上报令牌；先用全局 bearer 单独尝试上报，再以设备令牌报 revision 1、12 Token；持同令牌尝试同设备 revision 2、owner B 的 99 Token 和跨设备冒用；再验证有权修订、重传、撤销及显式管理员多用户范围。</x:v>
+      </x:c>
+      <x:c r="G79" s="42" t="str">
+        <x:v>全局 bearer 单独上报返回 401；设备令牌越权返回 403，owner A 的 12 Token、设备修订和来源覆盖不变；只有服务端登记范围允许的设备/用户组合可写。合法较高修订正常替换，同修订重传幂等；撤销后拒绝，管理员多用户快照须显式授权并逐用户隔离。</x:v>
+      </x:c>
+      <x:c r="H79" s="42" t="str">
+        <x:v>待验证（未注册；现代码缺陷已复现）</x:v>
+      </x:c>
+      <x:c r="I79" s="42" t="str">
+        <x:v>2026-10-03 SOP-001 仅规划；开发会话隔离复现旧代码跨用户 200 覆盖，见 docs/validation.md。尚无 TC-074 注册、执行或通过证据。</x:v>
+      </x:c>
+      <x:c r="J79" s="42" t="str">
+        <x:v>待注册：npm run test:case -- TC-074</x:v>
+      </x:c>
+      <x:c r="K79" s="42" t="str">
+        <x:v>计划 tests/server-ownership.test.ts：test('TC-074 聚合上报拒绝跨设备跨用户覆盖并保留原快照')；修复后在 scripts/test-cases.mjs 注册独立入口</x:v>
+      </x:c>
+      <x:c r="L79" s="42" t="str">
+        <x:v>预计断言管理登记/令牌签发、全局 bearer 单独上报拒绝、越权 403 及 aggregates、device_revisions、source_coverage 不变；覆盖合法修订/重传、撤销、管理员范围、旧数据/队列保留和服务切换。方案见 docs/design.md §12.2，未执行。</x:v>
+      </x:c>
+      <x:c r="M79" s="42" t="str">
+        <x:v>tests/support/test-workspace.ts 一次性独立 token.sqlite/服务目录、人工 UUID 和无正文快照；随机端口，结束清理。保留提交、命令、环境、退出码和脱敏前后计数；不得使用生产服务密钥或数据库。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.3 device auth verification
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rdc7ce8ad09cf41c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6534cd0e38184c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rae28844e69314275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bc0f5f9889c4b7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R38d7380ac9b346c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2bc5dea754834adb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R15573a89af8a408e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rfac8e0aad2154783"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1656,7 +1656,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>部分验证（跨用户覆盖缺陷已复现）</x:v>
+        <x:v>已验证（自动；可信证书与异机待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2300,7 +2300,7 @@
         <x:v>聚合上报设备与用户归属授权回归</x:v>
       </x:c>
       <x:c r="G80" s="43" t="str">
-        <x:v>待验证（未注册；缺陷已复现）</x:v>
+        <x:v>已验证（自动及 0.3.3 本机候选包；生产部署待验）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2339,7 +2339,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；REQ-006 的 Codex fallback 跨扫描缺陷已在 aa6d91b 修复，TC-073 合成回归及 0.3.1 本机候选包同库升级通过；生产库/真实安装待验。</x:v>
+        <x:v>REQ-001–039；REQ-021 的 DEV-048 已在 3d60b5e 完成设备/owner 授权与服务切换竞态回归，0.3.3 本机候选包已核验；生产部署与目标 Mac 待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2919,7 +2919,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>部分实现（聚合归属授权缺口待修）</x:v>
+        <x:v>代码已落地（本机合成授权与竞态自动覆盖；部署边界待验）</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>DEV-022、DEV-023、DEV-048</x:v>
@@ -2928,7 +2928,8 @@
         <x:v>TC-032、TC-033、TC-047、TC-074</x:v>
       </x:c>
       <x:c r="H26" s="14" t="str">
-        <x:v>历史：docs/design.md §9–13；docs/development-plan.md §7；TC-047 已验证全局 bearer/字段/Origin/HTTPS 配置的部分断言。2026-10-03：开发会话隔离服务复现同一 bearer 可把同设备 owner A 的 12 Token 用 owner B 的 99 Token、较高修订覆盖；代码审查见 src/server/server.ts。DEV-048 / TC-074 待实施，SOP-002 选定管理密钥登记与独立设备令牌；见 docs/design.md §12.1–12.2、docs/validation.md。</x:v>
+        <x:v>历史：docs/design.md §9–13；docs/development-plan.md §7；TC-047 已验证全局 bearer/字段/Origin/HTTPS 配置的部分断言。2026-10-03：开发会话隔离服务复现同一 bearer 可把同设备 owner A 的 12 Token 用 owner B 的 99 Token、较高修订覆盖；代码审查见 src/server/server.ts。DEV-048 / TC-074 待实施，SOP-002 选定管理密钥登记与独立设备令牌；见 docs/design.md §12.1–12.2、docs/validation.md。
+2026-10-03 后续：ca0f37f 实现设备令牌与写库前归属授权，533992e 仅补 TC-047 测试清理；3d60b5e 修复在途登记的服务切换竞态。TC-074 四项绑定、TC-047 两项在 0.3.3 独立复跑通过；门禁与 0.3.3 未签名本机候选包、隔离升级见 docs/validation.md。旧跨用户覆盖为修复前历史；生产账户/库、可信证书异机、签名公证、目标 Mac 待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -3433,7 +3434,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现，0.3.1 本机候选包同库升级通过；DEV-048 聚合归属授权修复待开发，相关证据见各行。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并有 0.3.1 本机候选包同库升级证据；DEV-048 已在 ca0f37f、3d60b5e 实现并有 TC-074 与 0.3.3 本机候选包证据。生产部署边界见各行。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3997,10 +3998,11 @@
         <x:v>src/server/server.ts；tests/next-server.test.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>已编码（部分自动覆盖；归属授权缺口）</x:v>
+        <x:v>已编码（授权回归自动通过；部署边界待验）</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>历史：96e99be 的 TC-047 验证全局 bearer、字段白名单、Origin 与 HTTPS 配置；同一 bearer 跨用户覆盖未测。2026-10-03 隔离复现表明 src/server/server.ts 仅检查全局 bearer，较高修订按 device_id/provider 替换聚合；修复规划另见 DEV-048 / TC-074，当前不可标为完整授权通过。</x:v>
+        <x:v>历史：96e99be 的 TC-047 验证全局 bearer、字段白名单、Origin 与 HTTPS 配置；同一 bearer 跨用户覆盖未测。2026-10-03 隔离复现表明 src/server/server.ts 仅检查全局 bearer，较高修订按 device_id/provider 替换聚合；修复规划另见 DEV-048 / TC-074，当前不可标为完整授权通过。
+后续：ca0f37f 以设备令牌替代全局 bearer 上报，服务按登记的设备/owner 范围在写库前授权；TC-047/TC-074 在隔离库通过。3d60b5e 修复客户端连接切换竞态；修复前 200 覆盖记录仅为历史。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4569,13 +4571,13 @@
         <x:v>TC-074</x:v>
       </x:c>
       <x:c r="E53" s="42" t="str">
-        <x:v>计划 src/server/server.ts、src/main/server-connection.ts、src/main/usage-sync.ts、tests/server-ownership.test.ts；见 docs/design.md §12.2</x:v>
+        <x:v>src/server/server.ts；src/main/server-connection.ts、usage-sync.ts；scripts/test-cases.mjs；tests/server-ownership.test.ts、next-sync.test.ts、next-server.test.ts；docs/design.md §12.2–12.4</x:v>
       </x:c>
       <x:c r="F53" s="42" t="str">
-        <x:v>待开发</x:v>
+        <x:v>已编码（自动及 0.3.3 本机候选包验证；生产部署待验）</x:v>
       </x:c>
       <x:c r="G53" s="42" t="str">
-        <x:v>2026-10-03 SOP-002 设计：保留全局 bearer 供原接口，管理密钥登记设备/允许 owner 并签发随机上报令牌；服务仅存令牌哈希并先授权后查修订/写库，客户端 safeStorage 加密保存。越权保持旧聚合、修订、覆盖；合法修订/幂等保留。旧数据与队列不自动清空，换服务重新登记，撤销不自动绕过；当前未编码或通过。</x:v>
+        <x:v>2026-10-03：ca0f37f 完成管理密钥登记/撤销、设备令牌哈希、设备/owner 写库前授权、客户端加密凭据与待传恢复；TC-074 初版三项。533992e 只清理 TC-047 TLS 测试资源。3d60b5e 以配置代次防止切换服务器时旧登记响应落盘或上传，TC-074 增为四项；文档会话独立复跑四项通过。开发会话报告门禁 74 编号、47 单元、18 Electron 和目录包 18/18；0.3.3 DMG 摘要与本机服务目录、隔离升级独立核验。生产账户/库、可信证书异机、签名公证、目标 Mac 待验；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4620,7 +4622,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–073 已注册；TC-074 是聚合归属授权待开发独立回归，尚未注册/验证；TC-072 仍为目标 Mac 人工待验。</x:v>
+        <x:v>TC-001–074 均已注册；TC-074 在 3d60b5e 有四项隔离自动绑定并通过，TC-072 仍为目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6229,7 +6231,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I43" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。</x:v>
       </x:c>
       <x:c r="J43" s="35" t="str">
         <x:v>npm run test:case -- TC-038</x:v>
@@ -6271,7 +6274,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I44" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。</x:v>
       </x:c>
       <x:c r="J44" s="14" t="str">
         <x:v>npm run test:case -- TC-039</x:v>
@@ -6312,7 +6316,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I45" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。</x:v>
       </x:c>
       <x:c r="J45" s="35" t="str">
         <x:v>npm run test:case -- TC-040</x:v>
@@ -6596,22 +6601,23 @@
         <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
-        <x:v>部分验证（自动；跨用户覆盖缺陷已复现）</x:v>
+        <x:v>已验证（自动；可信证书与异机连接待验）</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
-        <x:v>历史：96e99be 单编号自动断言通过，覆盖错误凭证、字段白名单、Origin 和 HTTPS 地址限制；开发日志被 Git 忽略。2026-10-03：开发会话用隔离 /tmp 服务和人工快照复现：同一 bearer 对同设备先报 owner A/revision 1/12 Token 得 200，再报 owner B/revision 2/99 Token 仍得 200（accepted=true, duplicate=false），旧聚合被替换；文档会话核对 src/server/server.ts。跨用户预期失败，见 docs/validation.md。</x:v>
+        <x:v>历史：96e99be 单编号自动断言通过，覆盖错误凭证、字段白名单、Origin 和 HTTPS 地址限制；开发日志被 Git 忽略。2026-10-03：开发会话用隔离 /tmp 服务和人工快照复现：同一 bearer 对同设备先报 owner A/revision 1/12 Token 得 200，再报 owner B/revision 2/99 Token 仍得 200（accepted=true, duplicate=false），旧聚合被替换；文档会话核对 src/server/server.ts。跨用户预期失败，见 docs/validation.md。
+2026-10-03：ca0f37f 加入本机自签 TLS 非回环鉴权，533992e 仅补测试资源清理；文档会话在 3d60b5e 独立复跑两项绑定退出码 0。跨设备/owner 写库前校验由 TC-074 覆盖；修复前 200 覆盖仅为历史。</x:v>
       </x:c>
       <x:c r="J52" s="14" t="str">
         <x:v>npm run test:case -- TC-047</x:v>
       </x:c>
       <x:c r="K52" s="14" t="str">
-        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')；test('TC-047 非回环 HTTPS 监听仍执行清单与上报鉴权')；scripts/test-cases.mjs 已注册两项</x:v>
       </x:c>
       <x:c r="L52" s="14" t="str">
-        <x:v>现有 tests/next-server.test.ts 只断言全局 bearer、字段、Origin 和 HTTPS 配置，不检验可信身份与 deviceId/ownerUserId 的绑定；跨用户修订覆盖在当前代码可发生。非回环 HTTPS 上的真实鉴权亦未验证。新增独立回归 TC-074 待注册/待通过，不能借 TC-047 自动通过宣称全项已验。</x:v>
+        <x:v>默认地址的清单/包/管理/上报鉴权及本机 0.0.0.0 自签 TLS 下的鉴权已测；测试客户端关闭证书验证，可信证书、异机连接和实际生产部署未测。跨设备/owner 授权及服务切换由 TC-074 测。</x:v>
       </x:c>
       <x:c r="M52" s="14" t="str">
-        <x:v>保留 96e99be 及既有日志历史。隔离复现使用一次性 /tmp 服务数据库、两个人工 owner UUID 和同设备较高修订，无真实用户数据或密钥入库；结果见 I 列。修复后须复跑 TC-047 与 TC-074，并对账拒绝前后聚合、device_revisions、source_coverage；当前没有修复后证据。</x:v>
+        <x:v>文档会话在 3d60b5e 独立复跑 TC-047 两项退出码 0；一次性服务目录、自签证书和人工快照，结束清理。旧越权复现作为历史；当前拒绝前后三表状态由 TC-074 对账。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="70" customHeight="1">
@@ -7132,7 +7138,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I65" s="37" t="str">
-        <x:v>提交 6223c30；2026-10-02 14:57:12 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-060.log</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:12 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-060.log
+2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。</x:v>
       </x:c>
       <x:c r="J65" s="37" t="str">
         <x:v>npm run test:case -- TC-060</x:v>
@@ -7694,31 +7701,33 @@
         <x:v>聚合上报设备与用户归属授权回归</x:v>
       </x:c>
       <x:c r="E79" s="42" t="str">
-        <x:v>单元/集成（计划）</x:v>
+        <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F79" s="42" t="str">
-        <x:v>独立临时服务库：管理凭据登记设备 A/owner A 并签发上报令牌；先用全局 bearer 单独尝试上报，再以设备令牌报 revision 1、12 Token；持同令牌尝试同设备 revision 2、owner B 的 99 Token 和跨设备冒用；再验证有权修订、重传、撤销及显式管理员多用户范围。</x:v>
+        <x:v>独立临时服务库：管理凭据登记设备 A/owner A 并签发上报令牌；先用全局 bearer 单独尝试上报，再以设备令牌报 revision 1、12 Token；持同令牌尝试同设备 revision 2、owner B 的 99 Token 和跨设备冒用；再验证有权修订、重传、撤销及显式管理员多用户范围。
+0.3.3 追加：让设备登记响应悬而未决时切换服务 URL，及同 URL 重新保存配置，再返回旧令牌。</x:v>
       </x:c>
       <x:c r="G79" s="42" t="str">
-        <x:v>全局 bearer 单独上报返回 401；设备令牌越权返回 403，owner A 的 12 Token、设备修订和来源覆盖不变；只有服务端登记范围允许的设备/用户组合可写。合法较高修订正常替换，同修订重传幂等；撤销后拒绝，管理员多用户快照须显式授权并逐用户隔离。</x:v>
+        <x:v>全局 bearer 单独上报返回 401；设备令牌越权返回 403，owner A 的 12 Token、设备修订和来源覆盖不变；只有服务端登记范围允许的设备/用户组合可写。合法较高修订正常替换，同修订重传幂等；撤销后拒绝，管理员多用户快照须显式授权并逐用户隔离。
+切换期间的旧登记请求报可重试错误，旧令牌不写本机凭据文件，也不用于新连接上报。</x:v>
       </x:c>
       <x:c r="H79" s="42" t="str">
-        <x:v>待验证（未注册；现代码缺陷已复现）</x:v>
+        <x:v>已验证（自动及 0.3.3 本机候选包；合成数据）</x:v>
       </x:c>
       <x:c r="I79" s="42" t="str">
-        <x:v>2026-10-03 SOP-001 仅规划；开发会话隔离复现旧代码跨用户 200 覆盖，见 docs/validation.md。尚无 TC-074 注册、执行或通过证据。</x:v>
+        <x:v>历史：SOP-001 修复前隔离复现旧代码跨用户 200 覆盖。ca0f37f 登记三项绑定，533992e 只补 TC-047 清理；3d60b5e 增加竞态第四项。文档会话在 3d60b5e 独立复跑 TC-074 四项退出码 0，TC-047 两项通过；开发会话报告门禁 74 编号、47 单元、18 Electron、目录包 18/18。0.3.3 未签名 x64 DMG SHA-256 0030246d50b5fed9a1980c8839e6c7ad97afd229d0718ad71116294a39d6ec85，隔离 0.3.2→0.3.3 升级与本机发布目录独立核验；详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J79" s="42" t="str">
-        <x:v>待注册：npm run test:case -- TC-074</x:v>
+        <x:v>npm run test:case -- TC-074</x:v>
       </x:c>
       <x:c r="K79" s="42" t="str">
-        <x:v>计划 tests/server-ownership.test.ts：test('TC-074 聚合上报拒绝跨设备跨用户覆盖并保留原快照')；修复后在 scripts/test-cases.mjs 注册独立入口</x:v>
+        <x:v>tests/server-ownership.test.ts：test('TC-074 聚合上报拒绝跨设备跨用户覆盖并保留原快照')；test('TC-074 客户端加密保存设备令牌且撤销后须显式重新登记')；test('TC-074 切换服务器时不向新地址发送旧设备令牌')；tests/next-sync.test.ts：test('TC-074 管理员重新配置后可立即重试待传快照')；scripts/test-cases.mjs 已注册四项</x:v>
       </x:c>
       <x:c r="L79" s="42" t="str">
-        <x:v>预计断言管理登记/令牌签发、全局 bearer 单独上报拒绝、越权 403 及 aggregates、device_revisions、source_coverage 不变；覆盖合法修订/重传、撤销、管理员范围、旧数据/队列保留和服务切换。方案见 docs/design.md §12.2，未执行。</x:v>
+        <x:v>隔离服务断言全局 bearer 401、设备/owner 越权 403 且 aggregates、device_revisions、source_coverage 不变；合法修订/重传、管理员范围、撤销、旧聚合保留。客户端注入加密接口检查密文、权限、撤销、重配待传及切换竞态。真实 Electron safeStorage、生产账户/库、可信证书异机连接、同 URL 服务实例无配置保存时替换未测。</x:v>
       </x:c>
       <x:c r="M79" s="42" t="str">
-        <x:v>tests/support/test-workspace.ts 一次性独立 token.sqlite/服务目录、人工 UUID 和无正文快照；随机端口，结束清理。保留提交、命令、环境、退出码和脱敏前后计数；不得使用生产服务密钥或数据库。</x:v>
+        <x:v>tests/support/test-workspace.ts 的独立临时 token.sqlite/服务目录、人工 UUID 和无正文快照；竞态使用 tc074-switch-race 临时目录并在结束时清理。文档会话复跑命令退出码 0，0.3.3 DMG 摘要、hdiutil、本机服务目录及隔离升级另行核验；不使用生产密钥或数据库。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.4 startup performance verification
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R38d7380ac9b346c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2bc5dea754834adb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R15573a89af8a408e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rfac8e0aad2154783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra396d6407ab041db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R25d9ba21f54b460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcbe9b9fe55ff4011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R834a6c26b7534cf6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2268,16 +2268,16 @@
         <x:v>DEV-047</x:v>
       </x:c>
       <x:c r="D79" s="41" t="str">
-        <x:v>修复 Codex fallback 跨扫描归并与旧库双事实</x:v>
+        <x:v>修复 Codex fallback 跨扫描归并、旧库双事实与大会话启动性能</x:v>
       </x:c>
       <x:c r="E79" s="41" t="str">
         <x:v>TC-073</x:v>
       </x:c>
       <x:c r="F79" s="41" t="str">
-        <x:v>Codex fallback 跨扫描归并</x:v>
+        <x:v>Codex fallback 跨扫描归并与大会话启动性能</x:v>
       </x:c>
       <x:c r="G79" s="41" t="str">
-        <x:v>已验证（自动及本机候选包；生产安装待验）</x:v>
+        <x:v>已验证（两项自动及 0.3.4 本机候选/生产库副本；真实安装待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="82" customHeight="1">
@@ -2339,7 +2339,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；REQ-021 的 DEV-048 已在 3d60b5e 完成设备/owner 授权与服务切换竞态回归，0.3.3 本机候选包已核验；生产部署与目标 Mac 待验。</x:v>
+        <x:v>REQ-001–039；REQ-006 / DEV-047 的 fallback 归并和大会话启动性能回归已在 0.3.4 本机候选验证；生产库仅用临时副本启动，真实安装/目标 Mac 待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2523,13 +2523,14 @@
         <x:v>增量扫描与幂等恢复</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>历史导入后持续扫描；重扫、重启、未写完末行、文件截断或轮转不造成重复计数。Codex 同会话 fallback 后到正式记录时只计正式；旧库双事实可安全修复。</x:v>
+        <x:v>历史导入后持续扫描；重扫、重启、未写完末行、文件截断或轮转不造成重复计数。Codex 同会话 fallback 后到正式记录时只计正式；旧库双事实可安全修复。
+旧库启动修复不得在没有 fallback 的大会话上对每条正式事实重复相关扫描；保持可验证的启动可用性，且事实/账户/来源/游标不因修复丢失。</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
         <x:v>M2</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>代码已修复（合成回归及 0.3.1 本机候选包同库升级通过）</x:v>
+        <x:v>代码已修复（归并与大会话合成回归、0.3.4 本机候选及生产库副本启动通过；真实安装待验）</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>DEV-006、DEV-047</x:v>
@@ -2538,7 +2539,8 @@
         <x:v>TC-010、TC-011、TC-073</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>历史：docs/design.md §4.3/A5；规划：§4.4；代码 aa6d91b、DEV-047 / TC-073 合成回归通过。2026-10-03：867a03a 制成 0.3.1 未签名候选包，同一隔离测试库从旧 0.3.0 的 2560 Token 升级后回到 1280；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库及真实安装待验，见 docs/validation.md。</x:v>
+        <x:v>历史：docs/design.md §4.3/A5；规划：§4.4；代码 aa6d91b、DEV-047 / TC-073 合成回归通过。2026-10-03：867a03a 制成 0.3.1 未签名候选包，同一隔离测试库从旧 0.3.0 的 2560 Token 升级后回到 1280；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库及真实安装待验，见 docs/validation.md。
+2026-10-03 后续：7abd640 先查存在 fallback 的会话再核对正式事实；TC-073 增加 6000 条无 fallback 规模回归，单编号两项通过。0.3.4 打包 App 在生产库只读临时副本上启动，完整性与账户/事实/来源/游标数量保持；0.3.3→0.3.4 隔离升级、DMG 与本机发布目录核验见 docs/validation.md。原库未修改；真实生产账户安装、目标 Mac 和签名公证待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -3434,7 +3436,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 已在 aa6d91b 实现并有 0.3.1 本机候选包同库升级证据；DEV-048 已在 ca0f37f、3d60b5e 实现并有 TC-074 与 0.3.3 本机候选包证据。生产部署边界见各行。</x:v>
+        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 在 aa6d91b 修复 fallback 归并、7abd640 修复大会话启动性能，0.3.4 有自动与隔离生产库副本证据；DEV-048 的 0.3.3 设备授权证据保留。真实安装与目标环境待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4539,7 +4541,7 @@
         <x:v>DEV-047</x:v>
       </x:c>
       <x:c r="B52" s="40" t="str">
-        <x:v>修复 Codex fallback 跨扫描归并与旧库双事实</x:v>
+        <x:v>修复 Codex fallback 跨扫描归并、旧库双事实与大会话启动性能</x:v>
       </x:c>
       <x:c r="C52" s="40" t="str">
         <x:v>REQ-006</x:v>
@@ -4548,13 +4550,14 @@
         <x:v>TC-073</x:v>
       </x:c>
       <x:c r="E52" s="40" t="str">
-        <x:v>src/collectors/scanner.ts；scripts/test-cases.mjs；tests/collector-fallback.test.ts（database.ts 未改）</x:v>
+        <x:v>src/collectors/scanner.ts；scripts/test-cases.mjs、verify-production-copy.mjs；tests/collector-fallback.test.ts（database.ts 未改）</x:v>
       </x:c>
       <x:c r="F52" s="40" t="str">
-        <x:v>已编码（自动及 0.3.1 本机候选包验证）</x:v>
+        <x:v>已编码（两项自动回归及 0.3.4 本机候选/生产库副本验证；真实安装待验）</x:v>
       </x:c>
       <x:c r="G52" s="40" t="str">
-        <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b，0.3.1 制品 867a03a。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；2026-10-03 同一隔离库 0.3.0→0.3.1 复现 2560→修复 1280，文档会话独立复跑退出码 0；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库/实际安装待验，见 docs/validation.md。</x:v>
+        <x:v>规划见 docs/development-plan.md §9；代码 aa6d91b，0.3.1 制品 867a03a。TC-073 单编号 1/1、TC-010 单元+Electron、73 编号入口通过；2026-10-03 同一隔离库 0.3.0→0.3.1 复现 2560→修复 1280，文档会话独立复跑退出码 0；本机更新服务目录已发布同哈希包。旧 0.3.0 DMG 不含修复；生产库/实际安装待验，见 docs/validation.md。
+7abd640：旧库启动修复先枚举有 fallback 的会话，避免无 fallback 大会话重复相关扫描；TC-073 第二项在独立临时库以 6000 条事实检查启动低于 5 秒且数量保持。文档会话独立复跑 TC-073 两项、74 编号检查、生产库临时副本打包启动、0.3.3→0.3.4 隔离升级，均退出码 0；DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，本机发布目录同哈希。开发会话报告门禁 48 单元/18 Electron、目录包 18/18；真实生产账户安装、目标 Mac、签名公证待验，见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="108" customHeight="1">
@@ -4622,7 +4625,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–074 均已注册；TC-074 在 3d60b5e 有四项隔离自动绑定并通过，TC-072 仍为目标 Mac 人工待验。</x:v>
+        <x:v>TC-001–074 均已注册；TC-073 在 7abd640 有归并和 6000 条大会话两项绑定并通过；TC-074 四项设备授权绑定保留，TC-072 目标 Mac 人工待验。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7657,34 +7660,39 @@
         <x:v>DEV-047</x:v>
       </x:c>
       <x:c r="D78" s="40" t="str">
-        <x:v>Codex fallback 跨扫描归并</x:v>
+        <x:v>Codex fallback 跨扫描归并与大会话启动性能</x:v>
       </x:c>
       <x:c r="E78" s="40" t="str">
         <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F78" s="40" t="str">
-        <x:v>独立临时库：先仅 event_msg:token_count 并首扫，再追加 token_usage_record 增量扫描；另造旧库双事实、其他会话/来源/项目对照。</x:v>
+        <x:v>独立临时库：先仅 event_msg:token_count 并首扫，再追加 token_usage_record 增量扫描；另造旧库双事实、其他会话/来源/项目对照。
+0.3.4 补充独立 tc073-large-session 临时库：6000 条同会话正式事实、无 fallback，重开库后构造 UsageScanner；另在生产库的只读临时副本启动打包 App。</x:v>
       </x:c>
       <x:c r="G78" s="40" t="str">
-        <x:v>同会话只保留正式总量；旧库启动修复不丢其他事实/归属/项目；重扫、重启、重复修复后事实数和报表总量稳定。</x:v>
+        <x:v>同会话只保留正式总量；旧库启动修复不丢其他事实/归属/项目；重扫、重启、重复修复后事实数和报表总量稳定。
+6000 条合成事实的扫描器构造低于 5 秒，事实数仍为 6000；副本 App 启动后数据库完整，账户/事实/来源身份/游标数量保持，原生产库不写入。</x:v>
       </x:c>
       <x:c r="H78" s="40" t="str">
-        <x:v>已验证（自动及 0.3.1 本机候选包；合成数据）</x:v>
+        <x:v>已验证（两项自动及 0.3.4 本机候选/生产库副本；真实安装待验）</x:v>
       </x:c>
       <x:c r="I78" s="40" t="str">
-        <x:v>2026-10-03：aa6d91b TC-073 1/1、TC-010 单元+Electron，退出码 0；开发工作树 test-results/acceptance/TC-073.log。867a03a：0.3.1 未签名 x64 DMG SHA-256 7e56933298505f5d08def3811b891e187b6cefb264bfab3538e5accdb6235a7c，hdiutil VALID；文档会话独立复跑 --fallback-repair 退出码 0；开发工作树 test-results/manual/evidence/TC-073-package-upgrade.log（Git 忽略）；docs/validation.md。</x:v>
+        <x:v>2026-10-03：aa6d91b TC-073 1/1、TC-010 单元+Electron，退出码 0；开发工作树 test-results/acceptance/TC-073.log。867a03a：0.3.1 未签名 x64 DMG SHA-256 7e56933298505f5d08def3811b891e187b6cefb264bfab3538e5accdb6235a7c，hdiutil VALID；文档会话独立复跑 --fallback-repair 退出码 0；开发工作树 test-results/manual/evidence/TC-073-package-upgrade.log（Git 忽略）；docs/validation.md。
+7abd640：TC-073 增加大会话规模函数，文档会话独立复跑两项均通过、退出码 0；另独立执行 test:production-copy 与 0.3.3→0.3.4 隔离升级退出码 0，DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588、hdiutil VALID，本机发布目录同哈希。开发会话报告门禁 74 编号、48 单元、18 Electron、目录包 18/18；详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J78" s="40" t="str">
         <x:v>npm run test:case -- TC-073</x:v>
       </x:c>
       <x:c r="K78" s="40" t="str">
-        <x:v>tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描替换与旧库修复保持幂等')；scripts/test-cases.mjs 已注册</x:v>
+        <x:v>tests/collector-fallback.test.ts：test('TC-073 Codex fallback 跨扫描替换与旧库修复保持幂等')；test('TC-073 大会话无 fallback 时启动修复保持线性耗时')；scripts/test-cases.mjs 已注册两项</x:v>
       </x:c>
       <x:c r="L78" s="40" t="str">
-        <x:v>单元：首扫 fallback 12、次扫正式 12 且旧事实删除；明细/汇总/CSV 只计正式；跨文件后到 fallback 不重增；旧库仅清同会话 fallback/项目关联，其他会话、Claude、身份和项目保留；游标/旧库清理失败回滚，重扫重启稳定。0.3.1 本机候选包：同一隔离库旧版 1280→2560，新版回到 1280 且受信登录保留。真实生产库、未知格式及实际安装未验。</x:v>
+        <x:v>单元：首扫 fallback 12、次扫正式 12 且旧事实删除；明细/汇总/CSV 只计正式；跨文件后到 fallback 不重增；旧库仅清同会话 fallback/项目关联，其他会话、Claude、身份和项目保留；游标/旧库清理失败回滚，重扫重启稳定。0.3.1 本机候选包：同一隔离库旧版 1280→2560，新版回到 1280 且受信登录保留。真实生产库、未知格式及实际安装未验。
+规模函数只验证本机 6000 条、无 fallback 场景在 5 秒内且数量不变，不证明所有环境严格线性。生产库副本检查只验证打包启动、隔离路径、完整性和四类数量；不扫描真实来源，不等于生产账户真实安装或逐项报表验收。</x:v>
       </x:c>
       <x:c r="M78" s="40" t="str">
-        <x:v>单元使用 tc073-incremental、tc073-legacy 独立临时 token.sqlite/合成 JSONL。打包升级使用独立临时用户数据和安装目录；先在旧 0.3.0 包复现重复计数，下载并校验 0.3.1，取消分支保留旧版，再同库替换修复。文档会话独立复跑；本机服务目录已发布同哈希包，但生产账户 App 连接/安装、生产库及 Finder /Applications 未验。</x:v>
+        <x:v>单元使用 tc073-incremental、tc073-legacy 独立临时 token.sqlite/合成 JSONL。打包升级使用独立临时用户数据和安装目录；先在旧 0.3.0 包复现重复计数，下载并校验 0.3.1，取消分支保留旧版，再同库替换修复。文档会话独立复跑；本机服务目录已发布同哈希包，但生产账户 App 连接/安装、生产库及 Finder /Applications 未验。
+tc073-large-session 独立临时 token.sqlite，结束清理；test:production-copy 用 SQLite 备份把授权读取的数据库复制到系统临时目录，空来源目录启动 0.3.4 打包 App，检查后清理。不要把原生产数据库、凭据、会话正文或副本提交仓库。</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="146" customHeight="1">

</xml_diff>

<commit_message>
docs: record 0.3.4 local TC-027 acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra396d6407ab041db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R25d9ba21f54b460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcbe9b9fe55ff4011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R834a6c26b7534cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1d47d0134d0047f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R593e9976ff3d4041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rbec55ca45d4b494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rbd3a2db0be124651"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1196,7 +1196,7 @@
         <x:v>未签名 DMG 本机验收</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>已验证（人工）</x:v>
+        <x:v>已验证（人工；0.3.4 本机隔离子范围，Finder/生产安装待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="38" customHeight="1">
@@ -2817,7 +2817,7 @@
         <x:v>M4</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>已验证（本机）</x:v>
+        <x:v>已验证（0.3.4 本机隔离挂载/复制与主流程；Finder、生产安装待验）</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
         <x:v>DEV-017</x:v>
@@ -2826,7 +2826,8 @@
         <x:v>TC-027</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
-        <x:v>历史：docs/validation.md A10；v0.3.0：同文 TC-027 新批次，本机未签名 DMG 人工 pass（2026-10-02）</x:v>
+        <x:v>历史：docs/validation.md A10；v0.3.0：同文 TC-027 新批次，本机未签名 DMG 人工 pass（2026-10-02）
+2026-10-03：代码 7abd640 的 0.3.4 未签名 DMG 在 macOS 15.7.4 x86_64 以独立临时库/人工 Codex JSONL 挂载、ditto 复制、启动，受信登录、扫描和 1280 Token 报表通过；TC-027 人工 pass 登记时间 2026-10-02T20:46:08.228Z，证据见 docs/validation.md。Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -3862,10 +3863,11 @@
         <x:v>scripts/package-dmg.mjs；package.json；release/</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>已完成</x:v>
+        <x:v>已完成（0.3.4 本机隔离子范围人工通过；Finder、生产安装待验）</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
-        <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md</x:v>
+        <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md
+0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5779,10 +5781,11 @@
         <x:v>当前 Mac 能启动、登录和采集。</x:v>
       </x:c>
       <x:c r="H32" s="9" t="str">
-        <x:v>已验证（人工）</x:v>
+        <x:v>已验证（人工；0.3.4 本机隔离挂载/复制和主流程子范围）</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>历史：docs/validation.md A10；2026-10-02。v0.3.0：2026-10-02 本机人工 pass；test-results/manual/TC-027.json、evidence/TC-027.md（本机 Git 忽略）；docs/validation.md 新批次</x:v>
+        <x:v>历史：docs/validation.md A10；2026-10-02。v0.3.0：2026-10-02 本机人工 pass；test-results/manual/TC-027.json、evidence/TC-027.md（本机 Git 忽略）；docs/validation.md 新批次
+0.3.4：2026-10-03 当前 macOS 15.7.4 x86_64，代码 7abd640；开发会话重跑 0.3.3→0.3.4 隔离升级与 hdiutil，退出码 0。test-results/manual/TC-027.json 当前为 pass（2026-10-02T20:46:08.228Z），证据指向 Git 忽略的 evidence/TC-027-0.3.4.md，脱敏日志 TC-027-0.3.4-upgrade.log。文档会话核对文件并此前独立复跑同命令；0.3.0 旧结果备份为 evidence/TC-027-0.3.0-result.json。详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
         <x:v>npm run test:case -- TC-027</x:v>
@@ -5791,10 +5794,12 @@
         <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
       </x:c>
       <x:c r="L32" s="9" t="str">
-        <x:v>人工入口；v0.3.0 复制版 Playwright 主流程 1/1，加独立应用副本界面复核；原 A10 历史保留</x:v>
+        <x:v>人工入口；v0.3.0 复制版 Playwright 主流程 1/1，加独立应用副本界面复核；原 A10 历史保留
+0.3.4 本机子范围：脚本用人工 Codex JSONL/独立临时库挂载 DMG、ditto 复制、运行打包 App，检查受信登录、扫描、1280 Token 报表及取消/替换后的状态。人工 pass 只对应当前 Mac；Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 未验。</x:v>
       </x:c>
       <x:c r="M32" s="9" t="str">
-        <x:v>macOS 15.7.4 x86_64；代码 6223c30；Token-0.3.0.dmg SHA-256 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；hdiutil VALID、ditto 复制、启动/扫描/报表通过。截图 evidence/TC-027-report.png；Finder 拖拽、真实更新替换、签名公证、异机未验。</x:v>
+        <x:v>macOS 15.7.4 x86_64；代码 6223c30；Token-0.3.0.dmg SHA-256 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；hdiutil VALID、ditto 复制、启动/扫描/报表通过。截图 evidence/TC-027-report.png；Finder 拖拽、真实更新替换、签名公证、异机未验。
+0.3.4 包 SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；test:upgrade:local 0.3.3→0.3.4 退出码 0，取消保留旧版与 1280 Token，替换后新版保留受信登录和 1280 Token。TC-027 pass 证据为 evidence/TC-027-0.3.4.md；隔离目录已清理。不得以此代替 Finder、真实生产安装、目标 Mac 或签名公证。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="60" customHeight="1">

</xml_diff>

<commit_message>
docs: plan trusted CA TLS regression coverage
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1d47d0134d0047f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R593e9976ff3d4041"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rbec55ca45d4b494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rbd3a2db0be124651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2e972b2d8e424884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf3e51357aa924100"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re16d7fcdcadf4018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R32567d99abd3421d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1311,7 +1311,7 @@
         <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>部分验证（现有自签自动通过；可信 CA 严格 TLS 待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
@@ -1656,7 +1656,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>已验证（自动；可信证书与异机待验）</x:v>
+        <x:v>部分验证（现有鉴权自动通过；可信 CA 严格 TLS 待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2916,13 +2916,14 @@
         <x:v>独立本地更新与汇总服务</x:v>
       </x:c>
       <x:c r="C26" s="14" t="str">
-        <x:v>服务独立运行；监听主机/端口及 App 连接地址均可配置，默认 127.0.0.1；提供版本清单、安装包和聚合接口；非回环配置仍须鉴权并保护传输；服务故障不影响本机报表。聚合写入还须把可信请求身份与设备及允许的应用用户范围绑定；不得仅凭全局 bearer 或请求体自报 deviceId/ownerUserId 覆盖其他用户快照。拒绝越权时原聚合、修订和覆盖状态不变。</x:v>
+        <x:v>服务独立运行；监听主机/端口及 App 连接地址均可配置，默认 127.0.0.1；提供版本清单、安装包和聚合接口；非回环配置仍须鉴权并保护传输；服务故障不影响本机报表。聚合写入还须把可信请求身份与设备及允许的应用用户范围绑定；不得仅凭全局 bearer 或请求体自报 deviceId/ownerUserId 覆盖其他用户快照。拒绝越权时原聚合、修订和覆盖状态不变。
+非回环 HTTPS 的连接地址应在可信证书链且证书 SAN 匹配时可连接；不受信证书或主机名不匹配应拒绝连接，不以关闭证书校验规避。</x:v>
       </x:c>
       <x:c r="D26" s="14" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>代码已落地（本机合成授权与竞态自动覆盖；部署边界待验）</x:v>
+        <x:v>代码已落地（设备/owner 授权自动覆盖；可信 CA 严格 TLS 补证与异机部署待验）</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>DEV-022、DEV-023、DEV-048</x:v>
@@ -2932,7 +2933,8 @@
       </x:c>
       <x:c r="H26" s="14" t="str">
         <x:v>历史：docs/design.md §9–13；docs/development-plan.md §7；TC-047 已验证全局 bearer/字段/Origin/HTTPS 配置的部分断言。2026-10-03：开发会话隔离服务复现同一 bearer 可把同设备 owner A 的 12 Token 用 owner B 的 99 Token、较高修订覆盖；代码审查见 src/server/server.ts。DEV-048 / TC-074 待实施，SOP-002 选定管理密钥登记与独立设备令牌；见 docs/design.md §12.1–12.2、docs/validation.md。
-2026-10-03 后续：ca0f37f 实现设备令牌与写库前归属授权，533992e 仅补 TC-047 测试清理；3d60b5e 修复在途登记的服务切换竞态。TC-074 四项绑定、TC-047 两项在 0.3.3 独立复跑通过；门禁与 0.3.3 未签名本机候选包、隔离升级见 docs/validation.md。旧跨用户覆盖为修复前历史；生产账户/库、可信证书异机、签名公证、目标 Mac 待验。</x:v>
+2026-10-03 后续：ca0f37f 实现设备令牌与写库前归属授权，533992e 仅补 TC-047 测试清理；3d60b5e 修复在途登记的服务切换竞态。TC-074 四项绑定、TC-047 两项在 0.3.3 独立复跑通过；门禁与 0.3.3 未签名本机候选包、隔离升级见 docs/validation.md。旧跨用户覆盖为修复前历史；生产账户/库、可信证书异机、签名公证、目标 Mac 待验。
+2026-10-03 补证规划：沿用 DEV-022/023 与 TC-032/047；既有本机自签测试关闭证书校验，其历史通过不证明可信 CA 或主机名。计划用一次性 CA、含本机连接地址 SAN 的服务端证书，在严格 TLS 客户端测试健康检查、拒绝不受信 CA/错误主机名，并重验受保护接口鉴权；新增函数尚未注册或通过，不涉及系统信任或异机连接。见 docs/design.md §11、docs/development-plan.md §7。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -3979,10 +3981,11 @@
         <x:v>src/server/server.ts；src/server/cli.ts；src/main/server-connection.ts；tests/next-server.test.ts</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
-        <x:v>已编码（自动覆盖；边界待验）</x:v>
+        <x:v>已编码（现有自签自动覆盖；可信 CA 严格 TLS 补证待验）</x:v>
       </x:c>
       <x:c r="G27" s="35" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md
+2026-10-03：TC-032 计划在一次性目录生成 CA 与含本机连接地址 SAN 的证书，指定测试 CA 严格校验健康端点，并分别拒绝不受信证书和主机名不匹配；拟在 tests/next-server.test.ts 增加独立绑定。当前无新增代码/通过证据，不改系统信任、不用生产证书或异机。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="100" customHeight="1">
@@ -4002,11 +4005,12 @@
         <x:v>src/server/server.ts；tests/next-server.test.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>已编码（授权回归自动通过；部署边界待验）</x:v>
+        <x:v>已编码（现有授权回归通过；可信 CA 严格 TLS 补证与部署待验）</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
         <x:v>历史：96e99be 的 TC-047 验证全局 bearer、字段白名单、Origin 与 HTTPS 配置；同一 bearer 跨用户覆盖未测。2026-10-03 隔离复现表明 src/server/server.ts 仅检查全局 bearer，较高修订按 device_id/provider 替换聚合；修复规划另见 DEV-048 / TC-074，当前不可标为完整授权通过。
-后续：ca0f37f 以设备令牌替代全局 bearer 上报，服务按登记的设备/owner 范围在写库前授权；TC-047/TC-074 在隔离库通过。3d60b5e 修复客户端连接切换竞态；修复前 200 覆盖记录仅为历史。</x:v>
+后续：ca0f37f 以设备令牌替代全局 bearer 上报，服务按登记的设备/owner 范围在写库前授权；TC-047/TC-074 在隔离库通过。3d60b5e 修复客户端连接切换竞态；修复前 200 覆盖记录仅为历史。
+2026-10-03：TC-047 拟复用严格 TLS 测试 CA 客户端，在本机非回环 HTTPS 核对清单、包、管理、上报接口的缺失/错误/合法凭据；新增独立绑定尚未提交或验证。现有关闭证书校验的历史结果保留，真实部署证书及异机连接待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -5984,28 +5988,34 @@
         <x:v>单元</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
-        <x:v>独立启停服务；验证默认监听/连接地址，显式配置其他地址，再测试地址不匹配。</x:v>
+        <x:v>独立启停服务；验证默认监听/连接地址，显式配置其他地址，再测试地址不匹配。
+补证计划：一次性 CA、证书 SAN 包含本机测试连接地址；指定该 CA 严格 TLS 请求非回环健康端点，再分别换不受信 CA 与错误主机名。</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>默认双方使用 127.0.0.1；配置匹配时可连，错误地址有可恢复状态；停服不影响本机报表。</x:v>
+        <x:v>默认双方使用 127.0.0.1；配置匹配时可连，错误地址有可恢复状态；停服不影响本机报表。
+可信 CA 且地址匹配时 HTTPS 健康检查成功；不受信证书、主机名不匹配均连接失败，不关闭证书校验。</x:v>
       </x:c>
       <x:c r="H37" s="35" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>部分验证（现有自签自动通过；可信 CA 严格 TLS 补证待注册/待验）</x:v>
       </x:c>
       <x:c r="I37" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03 补证规划：旧自签客户端关闭证书校验，仅历史结果有效；严格 CA/主机名及两类失败分支尚无新增测试函数、注册或通过日志。单编号命令保持 npm run test:case -- TC-032；实现后按同编号复跑并记录提交、环境和退出码。</x:v>
       </x:c>
       <x:c r="J37" s="35" t="str">
         <x:v>npm run test:case -- TC-032</x:v>
       </x:c>
       <x:c r="K37" s="35" t="str">
-        <x:v>tests/next-server.test.ts：test('TC-032 服务默认地址可配置且停服不影响本机数据库')</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-032 服务默认地址可配置且停服不影响本机数据库')
+计划新增 tests/next-server.test.ts 中 TC-032 严格 CA/主机名独立函数，并在 scripts/test-cases.mjs 追加绑定；当前未注册。</x:v>
       </x:c>
       <x:c r="L37" s="35" t="str">
-        <x:v>默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配</x:v>
+        <x:v>默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配
+待验证：指定测试 CA 的证书链、SAN 主机名匹配、拒绝不受信 CA/不匹配主机名。即使本机通过也不代表异机连接或生产证书部署。</x:v>
       </x:c>
       <x:c r="M37" s="35" t="str">
-        <x:v>记录 TC-032 命令、退出码、提交、环境和脱敏日志；覆盖与限制：默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配。</x:v>
+        <x:v>记录 TC-032 命令、退出码、提交、环境和脱敏日志；覆盖与限制：默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配。
+一次性证书目录与合成服务库；不改 macOS 系统信任、不用生产证书。测试完成清理证书、监听与服务目录，保存脱敏错误类别；当前无新执行证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
@@ -6603,29 +6613,35 @@
         <x:v>单元</x:v>
       </x:c>
       <x:c r="F52" s="14" t="str">
-        <x:v>在默认及非回环配置下，以缺失/错误/正确凭证请求清单、包和上报接口，并尝试跨用户覆盖。</x:v>
+        <x:v>在默认及非回环配置下，以缺失/错误/正确凭证请求清单、包和上报接口，并尝试跨用户覆盖。
+补证计划：在指定测试 CA 且严格校验证书/主机名的本机 HTTPS 客户端上，请求清单、包、管理和上报接口的缺失/错误/合法凭据。</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。</x:v>
+        <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。
+严格 TLS 校验成功后仍按凭据范围鉴权；缺失/错误凭据不返回受保护制品、不写库，合法凭据仅访问授权设备/用户。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
-        <x:v>已验证（自动；可信证书与异机连接待验）</x:v>
+        <x:v>部分验证（现有鉴权自动通过；可信 CA 严格 TLS 补证待注册/待验）</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
         <x:v>历史：96e99be 单编号自动断言通过，覆盖错误凭证、字段白名单、Origin 和 HTTPS 地址限制；开发日志被 Git 忽略。2026-10-03：开发会话用隔离 /tmp 服务和人工快照复现：同一 bearer 对同设备先报 owner A/revision 1/12 Token 得 200，再报 owner B/revision 2/99 Token 仍得 200（accepted=true, duplicate=false），旧聚合被替换；文档会话核对 src/server/server.ts。跨用户预期失败，见 docs/validation.md。
-2026-10-03：ca0f37f 加入本机自签 TLS 非回环鉴权，533992e 仅补测试资源清理；文档会话在 3d60b5e 独立复跑两项绑定退出码 0。跨设备/owner 写库前校验由 TC-074 覆盖；修复前 200 覆盖仅为历史。</x:v>
+2026-10-03：ca0f37f 加入本机自签 TLS 非回环鉴权，533992e 仅补测试资源清理；文档会话在 3d60b5e 独立复跑两项绑定退出码 0。跨设备/owner 写库前校验由 TC-074 覆盖；修复前 200 覆盖仅为历史。
+2026-10-03 补证规划：现有两项绑定的非回环自签客户端关闭证书校验；拟在同一 TC-047 命令追加严格 CA 客户端鉴权函数，尚无新增代码、绑定或通过日志。不得把历史单编号通过写为严格 TLS 已通过。</x:v>
       </x:c>
       <x:c r="J52" s="14" t="str">
         <x:v>npm run test:case -- TC-047</x:v>
       </x:c>
       <x:c r="K52" s="14" t="str">
-        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')；test('TC-047 非回环 HTTPS 监听仍执行清单与上报鉴权')；scripts/test-cases.mjs 已注册两项</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')；test('TC-047 非回环 HTTPS 监听仍执行清单与上报鉴权')；scripts/test-cases.mjs 已注册两项
+计划新增 tests/next-server.test.ts 中 TC-047 严格 TLS 鉴权独立函数并在 scripts/test-cases.mjs 追加绑定；当前未注册。</x:v>
       </x:c>
       <x:c r="L52" s="14" t="str">
-        <x:v>默认地址的清单/包/管理/上报鉴权及本机 0.0.0.0 自签 TLS 下的鉴权已测；测试客户端关闭证书验证，可信证书、异机连接和实际生产部署未测。跨设备/owner 授权及服务切换由 TC-074 测。</x:v>
+        <x:v>默认地址的清单/包/管理/上报鉴权及本机 0.0.0.0 自签 TLS 下的鉴权已测；测试客户端关闭证书验证，可信证书、异机连接和实际生产部署未测。跨设备/owner 授权及服务切换由 TC-074 测。
+待验证：指定测试 CA 严格校验证书与主机名的本机非回环连接上，清单、包、管理和上报仍执行授权；生产证书与异机连接不在本次补证。</x:v>
       </x:c>
       <x:c r="M52" s="14" t="str">
-        <x:v>文档会话在 3d60b5e 独立复跑 TC-047 两项退出码 0；一次性服务目录、自签证书和人工快照，结束清理。旧越权复现作为历史；当前拒绝前后三表状态由 TC-074 对账。</x:v>
+        <x:v>文档会话在 3d60b5e 独立复跑 TC-047 两项退出码 0；一次性服务目录、自签证书和人工快照，结束清理。旧越权复现作为历史；当前拒绝前后三表状态由 TC-074 对账。
+与 TC-032 共用测试 CA 生成方式，服务库、设备/用户及包均为合成；结束清理临时证书和服务目录。实施后记录响应、拒绝前后脱敏数据库计数、提交与退出码；目前无新证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="70" customHeight="1">

</xml_diff>

<commit_message>
docs: record trusted CA TLS regression evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2e972b2d8e424884"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf3e51357aa924100"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re16d7fcdcadf4018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R32567d99abd3421d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra86a4d325ad745a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcf7779330c19458d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R949e3be3a5fd464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf52e1e8932e242bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1311,7 +1311,7 @@
         <x:v>服务地址配置与连接</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
-        <x:v>部分验证（现有自签自动通过；可信 CA 严格 TLS 待验）</x:v>
+        <x:v>已验证（临时 CA 严格 TLS 本机自动通过；生产证书/异机待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="62" customHeight="1">
@@ -1656,7 +1656,7 @@
         <x:v>聚合接口授权</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
-        <x:v>部分验证（现有鉴权自动通过；可信 CA 严格 TLS 待验）</x:v>
+        <x:v>已验证（临时 CA 严格 TLS 本机自动通过；生产证书/异机待验）</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="62" customHeight="1">
@@ -2923,7 +2923,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E26" s="14" t="str">
-        <x:v>代码已落地（设备/owner 授权自动覆盖；可信 CA 严格 TLS 补证与异机部署待验）</x:v>
+        <x:v>代码已落地（设备/owner 授权及临时 CA 严格 TLS 本机自动覆盖；生产证书与异机部署待验）</x:v>
       </x:c>
       <x:c r="F26" s="14" t="str">
         <x:v>DEV-022、DEV-023、DEV-048</x:v>
@@ -2934,7 +2934,8 @@
       <x:c r="H26" s="14" t="str">
         <x:v>历史：docs/design.md §9–13；docs/development-plan.md §7；TC-047 已验证全局 bearer/字段/Origin/HTTPS 配置的部分断言。2026-10-03：开发会话隔离服务复现同一 bearer 可把同设备 owner A 的 12 Token 用 owner B 的 99 Token、较高修订覆盖；代码审查见 src/server/server.ts。DEV-048 / TC-074 待实施，SOP-002 选定管理密钥登记与独立设备令牌；见 docs/design.md §12.1–12.2、docs/validation.md。
 2026-10-03 后续：ca0f37f 实现设备令牌与写库前归属授权，533992e 仅补 TC-047 测试清理；3d60b5e 修复在途登记的服务切换竞态。TC-074 四项绑定、TC-047 两项在 0.3.3 独立复跑通过；门禁与 0.3.3 未签名本机候选包、隔离升级见 docs/validation.md。旧跨用户覆盖为修复前历史；生产账户/库、可信证书异机、签名公证、目标 Mac 待验。
-2026-10-03 补证规划：沿用 DEV-022/023 与 TC-032/047；既有本机自签测试关闭证书校验，其历史通过不证明可信 CA 或主机名。计划用一次性 CA、含本机连接地址 SAN 的服务端证书，在严格 TLS 客户端测试健康检查、拒绝不受信 CA/错误主机名，并重验受保护接口鉴权；新增函数尚未注册或通过，不涉及系统信任或异机连接。见 docs/design.md §11、docs/development-plan.md §7。</x:v>
+2026-10-03 补证规划：沿用 DEV-022/023 与 TC-032/047；既有本机自签测试关闭证书校验，其历史通过不证明可信 CA 或主机名。计划用一次性 CA、含本机连接地址 SAN 的服务端证书，在严格 TLS 客户端测试健康检查、拒绝不受信 CA/错误主机名，并重验受保护接口鉴权；新增函数尚未注册或通过，不涉及系统信任或异机连接。见 docs/design.md §11、docs/development-plan.md §7。
+2026-10-03 实施：测试提交 57fd884 为 TC-032/TC-047 各新增严格 TLS 函数并注册；文档会话独立复跑分别 2/2、3/3，74 个编号入口检查通过。一次性 CA 与本机非回环 IPv4 SAN 证明本机严格证书链/主机名校验及接口鉴权，不代表生产证书、系统信任或另一台 Mac 连接；0.3.4 DMG 未改。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="62" customHeight="1">
@@ -3981,11 +3982,12 @@
         <x:v>src/server/server.ts；src/server/cli.ts；src/main/server-connection.ts；tests/next-server.test.ts</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
-        <x:v>已编码（现有自签自动覆盖；可信 CA 严格 TLS 补证待验）</x:v>
+        <x:v>已编码（临时 CA 严格 TLS 本机自动通过；生产证书与异机待验）</x:v>
       </x:c>
       <x:c r="G27" s="35" t="str">
         <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md
-2026-10-03：TC-032 计划在一次性目录生成 CA 与含本机连接地址 SAN 的证书，指定测试 CA 严格校验健康端点，并分别拒绝不受信证书和主机名不匹配；拟在 tests/next-server.test.ts 增加独立绑定。当前无新增代码/通过证据，不改系统信任、不用生产证书或异机。</x:v>
+2026-10-03：TC-032 计划在一次性目录生成 CA 与含本机连接地址 SAN 的证书，指定测试 CA 严格校验健康端点，并分别拒绝不受信证书和主机名不匹配；拟在 tests/next-server.test.ts 增加独立绑定。当前无新增代码/通过证据，不改系统信任、不用生产证书或异机。
+实施：57fd884 在 tests/next-server.test.ts 追加 TC-032 严格 CA/主机名测试并于 scripts/test-cases.mjs 注册。文档会话独立复跑 TC-032 2/2、编号检查 74 项通过；本机非回环 IPv4 SAN 和真实 ServerConnection 子进程连通，无 CA/错误主机名拒绝。未改系统信任，生产证书与异机仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="100" customHeight="1">
@@ -4005,12 +4007,13 @@
         <x:v>src/server/server.ts；tests/next-server.test.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
-        <x:v>已编码（现有授权回归通过；可信 CA 严格 TLS 补证与部署待验）</x:v>
+        <x:v>已编码（设备/owner 授权及临时 CA 严格 TLS 本机自动通过；生产部署待验）</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
         <x:v>历史：96e99be 的 TC-047 验证全局 bearer、字段白名单、Origin 与 HTTPS 配置；同一 bearer 跨用户覆盖未测。2026-10-03 隔离复现表明 src/server/server.ts 仅检查全局 bearer，较高修订按 device_id/provider 替换聚合；修复规划另见 DEV-048 / TC-074，当前不可标为完整授权通过。
 后续：ca0f37f 以设备令牌替代全局 bearer 上报，服务按登记的设备/owner 范围在写库前授权；TC-047/TC-074 在隔离库通过。3d60b5e 修复客户端连接切换竞态；修复前 200 覆盖记录仅为历史。
-2026-10-03：TC-047 拟复用严格 TLS 测试 CA 客户端，在本机非回环 HTTPS 核对清单、包、管理、上报接口的缺失/错误/合法凭据；新增独立绑定尚未提交或验证。现有关闭证书校验的历史结果保留，真实部署证书及异机连接待验。</x:v>
+2026-10-03：TC-047 拟复用严格 TLS 测试 CA 客户端，在本机非回环 HTTPS 核对清单、包、管理、上报接口的缺失/错误/合法凭据；新增独立绑定尚未提交或验证。现有关闭证书校验的历史结果保留，真实部署证书及异机连接待验。
+实施：57fd884 在 tests/next-server.test.ts 追加 TC-047 严格 TLS 鉴权测试并于 scripts/test-cases.mjs 注册。文档会话独立复跑 TC-047 3/3：清单/包错误或缺失凭据拒绝，合法凭据可取；管理登记仅接受管理员密钥；设备令牌可上传，越权 owner 403 且原聚合不变。仅本机临时 CA 与合成库，生产证书/异机待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -5989,33 +5992,30 @@
       </x:c>
       <x:c r="F37" s="35" t="str">
         <x:v>独立启停服务；验证默认监听/连接地址，显式配置其他地址，再测试地址不匹配。
-补证计划：一次性 CA、证书 SAN 包含本机测试连接地址；指定该 CA 严格 TLS 请求非回环健康端点，再分别换不受信 CA 与错误主机名。</x:v>
+补证实施：一次性 CA、证书 SAN 包含本机测试连接地址；指定该 CA 严格 TLS 请求非回环健康端点，再分别换不受信 CA 与错误主机名。</x:v>
       </x:c>
       <x:c r="G37" s="35" t="str">
         <x:v>默认双方使用 127.0.0.1；配置匹配时可连，错误地址有可恢复状态；停服不影响本机报表。
 可信 CA 且地址匹配时 HTTPS 健康检查成功；不受信证书、主机名不匹配均连接失败，不关闭证书校验。</x:v>
       </x:c>
       <x:c r="H37" s="35" t="str">
-        <x:v>部分验证（现有自签自动通过；可信 CA 严格 TLS 补证待注册/待验）</x:v>
+        <x:v>已验证（自动；临时 CA 严格 TLS 本机通过，生产证书/异机待验）</x:v>
       </x:c>
       <x:c r="I37" s="35" t="str">
         <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
-2026-10-03 补证规划：旧自签客户端关闭证书校验，仅历史结果有效；严格 CA/主机名及两类失败分支尚无新增测试函数、注册或通过日志。单编号命令保持 npm run test:case -- TC-032；实现后按同编号复跑并记录提交、环境和退出码。</x:v>
+2026-10-03：57fd884 注册第二项绑定；文档会话独立运行 npm run test:case -- TC-032，2/2 通过、退出码 0；npm run test:cases:check，74 个编号通过。详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J37" s="35" t="str">
         <x:v>npm run test:case -- TC-032</x:v>
       </x:c>
       <x:c r="K37" s="35" t="str">
-        <x:v>tests/next-server.test.ts：test('TC-032 服务默认地址可配置且停服不影响本机数据库')
-计划新增 tests/next-server.test.ts 中 TC-032 严格 CA/主机名独立函数，并在 scripts/test-cases.mjs 追加绑定；当前未注册。</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-032 服务默认地址可配置且停服不影响本机数据库')；test('TC-032 临时 CA 严格验证非回环服务与证书失败路径')；scripts/test-cases.mjs 已注册两项</x:v>
       </x:c>
       <x:c r="L37" s="35" t="str">
-        <x:v>默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配
-待验证：指定测试 CA 的证书链、SAN 主机名匹配、拒绝不受信 CA/不匹配主机名。即使本机通过也不代表异机连接或生产证书部署。</x:v>
+        <x:v>原函数覆盖默认回环/localhost、无 TLS 非回环拒绝、自签证书下 0.0.0.0 HTTPS 监听（历史客户端关闭证书校验）。新增函数用指定临时 CA 且 rejectUnauthorized: true 验证本机非回环 IPv4 SAN 健康检查 200，无 CA 与主机名不匹配均拒绝；真实 ServerConnection 子进程经 NODE_EXTRA_CA_CERTS 连通。生产证书、系统信任与异机连接未测。</x:v>
       </x:c>
       <x:c r="M37" s="35" t="str">
-        <x:v>记录 TC-032 命令、退出码、提交、环境和脱敏日志；覆盖与限制：默认回环/localhost、无 TLS 非回环拒绝；自签证书下 0.0.0.0 HTTPS 监听成功；未测异机连接、证书信任与地址不匹配。
-一次性证书目录与合成服务库；不改 macOS 系统信任、不用生产证书。测试完成清理证书、监听与服务目录，保存脱敏错误类别；当前无新执行证据。</x:v>
+        <x:v>57fd884：文档会话独立复跑 TC-032 2/2、退出码 0；一次性 OpenSSL CA、SAN 证书和合成服务库，测试结束清理证书、监听与服务目录。只证明本机严格 TLS 连接与失败路径，不代表生产证书部署或另一台 Mac 可连；未修改 macOS 系统信任。</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="70" customHeight="1">
@@ -6614,34 +6614,31 @@
       </x:c>
       <x:c r="F52" s="14" t="str">
         <x:v>在默认及非回环配置下，以缺失/错误/正确凭证请求清单、包和上报接口，并尝试跨用户覆盖。
-补证计划：在指定测试 CA 且严格校验证书/主机名的本机 HTTPS 客户端上，请求清单、包、管理和上报接口的缺失/错误/合法凭据。</x:v>
+补证实施：在指定测试 CA 且严格校验证书/主机名的本机 HTTPS 客户端上，请求清单、包、管理和上报接口的缺失/错误/合法凭据。</x:v>
       </x:c>
       <x:c r="G52" s="14" t="str">
         <x:v>未授权请求不返回受保护制品或写库；合法凭证只访问授权范围；非回环连接使用受保护传输。
 严格 TLS 校验成功后仍按凭据范围鉴权；缺失/错误凭据不返回受保护制品、不写库，合法凭据仅访问授权设备/用户。</x:v>
       </x:c>
       <x:c r="H52" s="14" t="str">
-        <x:v>部分验证（现有鉴权自动通过；可信 CA 严格 TLS 补证待注册/待验）</x:v>
+        <x:v>已验证（自动；临时 CA 严格 TLS 本机通过，生产证书/异机待验）</x:v>
       </x:c>
       <x:c r="I52" s="14" t="str">
         <x:v>历史：96e99be 单编号自动断言通过，覆盖错误凭证、字段白名单、Origin 和 HTTPS 地址限制；开发日志被 Git 忽略。2026-10-03：开发会话用隔离 /tmp 服务和人工快照复现：同一 bearer 对同设备先报 owner A/revision 1/12 Token 得 200，再报 owner B/revision 2/99 Token 仍得 200（accepted=true, duplicate=false），旧聚合被替换；文档会话核对 src/server/server.ts。跨用户预期失败，见 docs/validation.md。
 2026-10-03：ca0f37f 加入本机自签 TLS 非回环鉴权，533992e 仅补测试资源清理；文档会话在 3d60b5e 独立复跑两项绑定退出码 0。跨设备/owner 写库前校验由 TC-074 覆盖；修复前 200 覆盖仅为历史。
-2026-10-03 补证规划：现有两项绑定的非回环自签客户端关闭证书校验；拟在同一 TC-047 命令追加严格 CA 客户端鉴权函数，尚无新增代码、绑定或通过日志。不得把历史单编号通过写为严格 TLS 已通过。</x:v>
+2026-10-03：57fd884 注册第三项绑定；文档会话独立运行 npm run test:case -- TC-047，3/3 通过、退出码 0；npm run test:cases:check，74 个编号通过。详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J52" s="14" t="str">
         <x:v>npm run test:case -- TC-047</x:v>
       </x:c>
       <x:c r="K52" s="14" t="str">
-        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')；test('TC-047 非回环 HTTPS 监听仍执行清单与上报鉴权')；scripts/test-cases.mjs 已注册两项
-计划新增 tests/next-server.test.ts 中 TC-047 严格 TLS 鉴权独立函数并在 scripts/test-cases.mjs 追加绑定；当前未注册。</x:v>
+        <x:v>tests/next-server.test.ts：test('TC-047 上报接口鉴权和字段白名单')；test('TC-047 非回环 HTTPS 监听仍执行清单与上报鉴权')；test('TC-047 严格 TLS 下保护接口维持鉴权')；scripts/test-cases.mjs 已注册三项</x:v>
       </x:c>
       <x:c r="L52" s="14" t="str">
-        <x:v>默认地址的清单/包/管理/上报鉴权及本机 0.0.0.0 自签 TLS 下的鉴权已测；测试客户端关闭证书验证，可信证书、异机连接和实际生产部署未测。跨设备/owner 授权及服务切换由 TC-074 测。
-待验证：指定测试 CA 严格校验证书与主机名的本机非回环连接上，清单、包、管理和上报仍执行授权；生产证书与异机连接不在本次补证。</x:v>
+        <x:v>原两项覆盖默认地址与本机非回环自签 TLS 鉴权（历史客户端关闭证书校验）。新增函数在指定临时 CA、正确 SAN、rejectUnauthorized: true 的连接上检查清单/包缺失或错误 bearer 拒绝、合法 bearer 可取；管理员登记错误密钥 403、合法 200，全局 bearer 上报 401、设备令牌上报 200，错误 owner 403 且聚合不变。生产证书、异机及真实部署未测。</x:v>
       </x:c>
       <x:c r="M52" s="14" t="str">
-        <x:v>文档会话在 3d60b5e 独立复跑 TC-047 两项退出码 0；一次性服务目录、自签证书和人工快照，结束清理。旧越权复现作为历史；当前拒绝前后三表状态由 TC-074 对账。
-与 TC-032 共用测试 CA 生成方式，服务库、设备/用户及包均为合成；结束清理临时证书和服务目录。实施后记录响应、拒绝前后脱敏数据库计数、提交与退出码；目前无新证据。</x:v>
+        <x:v>57fd884：文档会话独立复跑 TC-047 3/3、退出码 0；一次性 OpenSSL CA、SAN 证书、人工凭据/快照及隔离服务库，结束清理。只证明本机严格 TLS 下的接口鉴权；生产证书与另一台 Mac 连接待验，0.3.4 DMG 未改。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="70" customHeight="1">

</xml_diff>

<commit_message>
docs: plan signed release preflight and TC-075
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra86a4d325ad745a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcf7779330c19458d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R949e3be3a5fd464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf52e1e8932e242bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R9d006df8ce9c42bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R4361da22077c4ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rdc8da68f41e844cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rff1dfc8ffb104d1c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -169,6 +169,16 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -181,7 +191,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="44">
+  <x:cellXfs count="50">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -309,6 +319,20 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2303,6 +2327,29 @@
         <x:v>已验证（自动及 0.3.3 本机候选包；生产部署待验）</x:v>
       </x:c>
     </x:row>
+    <x:row r="81" ht="82" customHeight="1">
+      <x:c r="A81" s="49" t="str">
+        <x:v>REQ-018</x:v>
+      </x:c>
+      <x:c r="B81" s="49" t="str">
+        <x:v>外部分发验证</x:v>
+      </x:c>
+      <x:c r="C81" s="49" t="str">
+        <x:v>DEV-018</x:v>
+      </x:c>
+      <x:c r="D81" s="49" t="str">
+        <x:v>完成公开分发流程</x:v>
+      </x:c>
+      <x:c r="E81" s="49" t="str">
+        <x:v>TC-075</x:v>
+      </x:c>
+      <x:c r="F81" s="49" t="str">
+        <x:v>签名发布脚本预检与命令构造</x:v>
+      </x:c>
+      <x:c r="G81" s="49" t="str">
+        <x:v>待注册、待验证（自动；脚本尚未实现）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2838,7 +2885,7 @@
         <x:v>外部分发验证</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
-        <x:v>面向其他 Mac 分发前完成 Apple 签名、公证，并在目标设备验证安装、启动和核心流程。</x:v>
+        <x:v>面向其他 Mac 分发前，独立签名发布入口须在构建前拒绝缺失或错误的 Developer ID 身份与公证凭据；完整凭据下生成已签名、公证并核验的 DMG，记录制品完整性；目标设备安装、启动、登录和采集通过。现有未签名本机打包入口保持独立。</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
         <x:v>发布</x:v>
@@ -2850,10 +2897,10 @@
         <x:v>DEV-018</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>TC-028</x:v>
+        <x:v>TC-028、TC-075</x:v>
       </x:c>
       <x:c r="H23" s="10" t="str">
-        <x:v>docs/design.md §7；docs/validation.md 末段</x:v>
+        <x:v>docs/design.md §7；docs/development-plan.md 外部分发计划；docs/test-case-acceptance.md TC-028/TC-075；docs/validation.md。2026-10-03：签名脚本与自动预检均未实现，缺有效签名身份及另一台目标 Mac；不得把未签名 0.3.4 DMG 或将来的 TC-075 模拟通过写成外部分发通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
@@ -3884,16 +3931,16 @@
         <x:v>REQ-018</x:v>
       </x:c>
       <x:c r="D23" s="10" t="str">
-        <x:v>TC-028</x:v>
+        <x:v>TC-028、TC-075</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>签名/公证配置；目标 Mac 验收记录</x:v>
+        <x:v>package.json 的 pack:signed；独立签名脚本；scripts/test-cases.mjs 与测试函数；发布环境脱敏核验记录；目标 Mac 验收记录。现有 scripts/package-dmg.mjs 未签名通道保留。</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>待启动</x:v>
+        <x:v>待开发（TC-075 预检回归待注册；真实签名、公证与目标 Mac 待验）</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>需证书、构建环境与目标设备</x:v>
+        <x:v>2026-10-03 SOP-001/002 计划：构建前检查 Developer ID Application 身份和完整公证凭据，缺项安全失败；electron-builder v26 使用 forceCodeSigning:true、mac.notarize:true，之后逐项核对 codesign、spctl、stapler、hdiutil 与 DMG SHA-256。先实现/运行模拟 TC-075 与门禁，再在具备有效证书凭据的环境构建并执行 TC-028 目标 Mac 人工验收。凭据和私钥不得入库/日志，pack:dmg 仍为本机未签名通道。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -4634,7 +4681,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–074 均已注册；TC-073 在 7abd640 有归并和 6000 条大会话两项绑定并通过；TC-074 四项设备授权绑定保留，TC-072 目标 Mac 人工待验。</x:v>
+        <x:v>TC-001–075 已分配；TC-001–074 已注册，TC-075 签名脚本预检待注册/待验证。TC-028 真实签名、公证及目标 Mac 人工验收仍待验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -5835,7 +5882,7 @@
         <x:v>待验证</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
-        <x:v>尚无签名、公证及其他目标设备证据</x:v>
+        <x:v>尚无签名、公证及其他目标设备证据；2026-10-03 已规划 pack:signed 与 TC-075 模拟预检，均尚无代码/结果；真实签名、公证、票据及目标 Mac 仍无证据。</x:v>
       </x:c>
       <x:c r="J33" s="27" t="str">
         <x:v>npm run test:case -- TC-028</x:v>
@@ -5847,7 +5894,7 @@
         <x:v>人工入口；待验证</x:v>
       </x:c>
       <x:c r="M33" s="27" t="str">
-        <x:v>证书身份脱敏信息、签名验证、公证状态、目标 Mac 版本/架构和脱敏流程记录。</x:v>
+        <x:v>证书身份脱敏信息、签名验证、公证状态、目标 Mac 版本/架构和脱敏流程记录。 TC-075 的模拟身份与命令构造通过不能替代本项真实发布验收；证据须对应同一签名候选的 App/DMG，并含目标机安装、启动、登录和采集。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
@@ -7756,6 +7803,47 @@
         <x:v>tests/support/test-workspace.ts 的独立临时 token.sqlite/服务目录、人工 UUID 和无正文快照；竞态使用 tc074-switch-race 临时目录并在结束时清理。文档会话复跑命令退出码 0，0.3.3 DMG 摘要、hdiutil、本机服务目录及隔离升级另行核验；不使用生产密钥或数据库。</x:v>
       </x:c>
     </x:row>
+    <x:row r="80" ht="180" customHeight="1">
+      <x:c r="A80" s="46" t="str">
+        <x:v>TC-075</x:v>
+      </x:c>
+      <x:c r="B80" s="46" t="str">
+        <x:v>REQ-018</x:v>
+      </x:c>
+      <x:c r="C80" s="46" t="str">
+        <x:v>DEV-018</x:v>
+      </x:c>
+      <x:c r="D80" s="46" t="str">
+        <x:v>签名发布脚本预检与命令构造</x:v>
+      </x:c>
+      <x:c r="E80" s="46" t="str">
+        <x:v>单元/脚本</x:v>
+      </x:c>
+      <x:c r="F80" s="46" t="str">
+        <x:v>用假 Developer ID 身份、三种公证凭据组的占位值和注入式执行器，分别模拟身份缺失/类型错误、凭据全缺/部分缺失/冲突、完整凭据以及构建后各核验步骤失败；不调用真实 Apple 服务。</x:v>
+      </x:c>
+      <x:c r="G80" s="46" t="str">
+        <x:v>异常输入须在构建前失败且执行器零调用；完整输入生成 forceCodeSigning:true、mac.notarize:true 的 v26 构建命令，并安排 codesign、spctl、stapler、hdiutil、DMG SHA-256 校验；任一步失败不得发布或复用旧未签名包，pack:dmg 仍独立可用。</x:v>
+      </x:c>
+      <x:c r="H80" s="46" t="str">
+        <x:v>待注册、待验证（自动；签名脚本尚未实现）</x:v>
+      </x:c>
+      <x:c r="I80" s="46" t="str">
+        <x:v>2026-10-03 SOP-001/002 仅完成实施前计划；尚无 pack:signed、测试函数、scripts/test-cases.mjs 绑定或执行日志。不得把 planned 命令、既有未签名 DMG 或 TC-028 人工清单记为本项通过。</x:v>
+      </x:c>
+      <x:c r="J80" s="46" t="str">
+        <x:v>npm run test:case -- TC-075</x:v>
+      </x:c>
+      <x:c r="K80" s="46" t="str">
+        <x:v>拟新增以 TC-075 开头的独立脚本测试函数，并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L80" s="46" t="str">
+        <x:v>模拟预检、错误处理和命令构造；不读取真实钥匙串/私钥、不向 Apple 提交公证，不生成已签名 DMG。自动通过不证明证书有效、票据/Gatekeeper 结果或另一台 Mac 安装。</x:v>
+      </x:c>
+      <x:c r="M80" s="46" t="str">
+        <x:v>实施后保存提交、macOS/Node、单编号命令和退出码、脱敏断言与失败分支；在隔离测试目录使用假凭据，日志不得含私钥/口令。真实签名、公证和目标 Mac 结果由 TC-028 单独记录。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record signed release script test evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R9d006df8ce9c42bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R4361da22077c4ae5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rdc8da68f41e844cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rff1dfc8ffb104d1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R212741314ee54a4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R03d097e75444458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9d309dd7744b4320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R87cc198de15041f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2347,7 +2347,7 @@
         <x:v>签名发布脚本预检与命令构造</x:v>
       </x:c>
       <x:c r="G81" s="49" t="str">
-        <x:v>待注册、待验证（自动；脚本尚未实现）</x:v>
+        <x:v>部分验证（自动预检/命令构造 1/1；构建后失败注入与真实发布待验）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2891,7 +2891,7 @@
         <x:v>发布</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>待完成</x:v>
+        <x:v>部分实现（签名发布脚本与 TC-075 自动子范围已落地；真实外部分发待验）</x:v>
       </x:c>
       <x:c r="F23" s="10" t="str">
         <x:v>DEV-018</x:v>
@@ -2900,7 +2900,8 @@
         <x:v>TC-028、TC-075</x:v>
       </x:c>
       <x:c r="H23" s="10" t="str">
-        <x:v>docs/design.md §7；docs/development-plan.md 外部分发计划；docs/test-case-acceptance.md TC-028/TC-075；docs/validation.md。2026-10-03：签名脚本与自动预检均未实现，缺有效签名身份及另一台目标 Mac；不得把未签名 0.3.4 DMG 或将来的 TC-075 模拟通过写成外部分发通过。</x:v>
+        <x:v>docs/design.md §7；docs/development-plan.md 外部分发计划；docs/test-case-acceptance.md TC-028/TC-075；docs/validation.md。2026-10-03：签名脚本与自动预检均未实现，缺有效签名身份及另一台目标 Mac；不得把未签名 0.3.4 DMG 或将来的 TC-075 模拟通过写成外部分发通过。
+2026-10-03 后续：dc37b8b 实现 pack:signed、预检与同候选制品核验脚本，TC-075 一项自动绑定；文档会话独立复跑 1/1、75 编号检查，缺凭据构建前退出码 1 且无 signed 制品。DEV-018 仅部分落地；没有真实签名/公证、票据或目标 Mac 证据，TC-028 仍待验证。见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
@@ -3934,13 +3935,14 @@
         <x:v>TC-028、TC-075</x:v>
       </x:c>
       <x:c r="E23" s="10" t="str">
-        <x:v>package.json 的 pack:signed；独立签名脚本；scripts/test-cases.mjs 与测试函数；发布环境脱敏核验记录；目标 Mac 验收记录。现有 scripts/package-dmg.mjs 未签名通道保留。</x:v>
+        <x:v>package.json 的 pack:signed；scripts/package-signed-dmg.mjs；build/entitlements.mac.plist；tests/signed-release.test.ts、scripts/test-cases.mjs；后续真实签名/公证 evidence JSON 与目标 Mac 验收记录。scripts/package-dmg.mjs 未签名通道保留。</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>待开发（TC-075 预检回归待注册；真实签名、公证与目标 Mac 待验）</x:v>
+        <x:v>部分已编码（签名脚本与 TC-075 自动子范围通过；真实签名、公证和目标 Mac 待验）</x:v>
       </x:c>
       <x:c r="G23" s="10" t="str">
-        <x:v>2026-10-03 SOP-001/002 计划：构建前检查 Developer ID Application 身份和完整公证凭据，缺项安全失败；electron-builder v26 使用 forceCodeSigning:true、mac.notarize:true，之后逐项核对 codesign、spctl、stapler、hdiutil 与 DMG SHA-256。先实现/运行模拟 TC-075 与门禁，再在具备有效证书凭据的环境构建并执行 TC-028 目标 Mac 人工验收。凭据和私钥不得入库/日志，pack:dmg 仍为本机未签名通道。</x:v>
+        <x:v>2026-10-03 SOP-001/002 计划：构建前检查 Developer ID Application 身份和完整公证凭据，缺项安全失败；electron-builder v26 使用 forceCodeSigning:true、mac.notarize:true，之后逐项核对 codesign、spctl、stapler、hdiutil 与 DMG SHA-256。先实现/运行模拟 TC-075 与门禁，再在具备有效证书凭据的环境构建并执行 TC-028 目标 Mac 人工验收。凭据和私钥不得入库/日志，pack:dmg 仍为本机未签名通道。
+后续 dc37b8b：electron-builder 26.15.3 以 mac.forceCodeSigning、mac.notarize、mac.hardenedRuntime、JIT entitlement 在一次性 release/token-signed-* 目录构建；逐项 codesign/spctl/stapler/hdiutil、DMG 大小/SHA-256 后才原子移到 release/signed 并写不含密钥的 release-evidence.json。TC-075 1/1、75 入口由文档会话独立复跑；无公证凭据时构建前拒绝且无 signed 制品。完整门禁 75 入口/51 单元/18 Electron 为开发会话报告；真正签名、公证、异机 TC-028 未执行。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -4681,7 +4683,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–075 已分配；TC-001–074 已注册，TC-075 签名脚本预检待注册/待验证。TC-028 真实签名、公证及目标 Mac 人工验收仍待验证。</x:v>
+        <x:v>TC-001–075 均已注册；TC-075 在 dc37b8b 有一项签名脚本自动绑定，预检/命令构造子范围通过，构建后失败注入待补；TC-028 真实签名、公证与目标 Mac 人工验收待验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -5882,19 +5884,19 @@
         <x:v>待验证</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
-        <x:v>尚无签名、公证及其他目标设备证据；2026-10-03 已规划 pack:signed 与 TC-075 模拟预检，均尚无代码/结果；真实签名、公证、票据及目标 Mac 仍无证据。</x:v>
+        <x:v>历史：实施前无签名、公证和目标 Mac 证据。2026-10-03 dc37b8b 已新增 pack:signed，但当前 Mac 无有效签名身份/公证凭据；文档会话运行 TC-028 人工清单，退出码 2，未登记 pass。尚无真实签名、公证票据、Gatekeeper 或另一台 Mac 的安装/启动/登录/采集结果；TC-075 自动通过不能替代本项。</x:v>
       </x:c>
       <x:c r="J33" s="27" t="str">
         <x:v>npm run test:case -- TC-028</x:v>
       </x:c>
       <x:c r="K33" s="27" t="str">
-        <x:v>scripts/test-cases.mjs 人工清单；无自动断言</x:v>
+        <x:v>scripts/test-cases.mjs：TC-028 人工清单；已更新为先运行 pack:signed、核对 release/signed 证据，再在另一台目标 Mac 安装与验证；无自动通过断言。</x:v>
       </x:c>
       <x:c r="L33" s="30" t="str">
         <x:v>人工入口；待验证</x:v>
       </x:c>
       <x:c r="M33" s="27" t="str">
-        <x:v>证书身份脱敏信息、签名验证、公证状态、目标 Mac 版本/架构和脱敏流程记录。 TC-075 的模拟身份与命令构造通过不能替代本项真实发布验收；证据须对应同一签名候选的 App/DMG，并含目标机安装、启动、登录和采集。</x:v>
+        <x:v>运行 npm run test:case -- TC-028 仅输出人工清单、退出码 2；实际验收需同一签名候选的 App/DMG、脱敏 Developer ID 身份、公证和票据/Gatekeeper 核验、包大小/SHA-256、目标 Mac 版本/架构与安装、启动、登录、采集记录。当前无 pass 证据，不得借用 TC-075 1/1 或 0.3.4 未签名包。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
@@ -7826,22 +7828,22 @@
         <x:v>异常输入须在构建前失败且执行器零调用；完整输入生成 forceCodeSigning:true、mac.notarize:true 的 v26 构建命令，并安排 codesign、spctl、stapler、hdiutil、DMG SHA-256 校验；任一步失败不得发布或复用旧未签名包，pack:dmg 仍独立可用。</x:v>
       </x:c>
       <x:c r="H80" s="46" t="str">
-        <x:v>待注册、待验证（自动；签名脚本尚未实现）</x:v>
+        <x:v>部分验证（自动 1/1；构建后核验失败注入及真实签名待验）</x:v>
       </x:c>
       <x:c r="I80" s="46" t="str">
-        <x:v>2026-10-03 SOP-001/002 仅完成实施前计划；尚无 pack:signed、测试函数、scripts/test-cases.mjs 绑定或执行日志。不得把 planned 命令、既有未签名 DMG 或 TC-028 人工清单记为本项通过。</x:v>
+        <x:v>2026-10-03 dc37b8b：文档会话独立运行 npm run test:case -- TC-075，1/1 通过、退出码 0；npm run test:cases:check 为 75 个入口、退出码 0。清除 Apple/CSC 环境变量独立运行 pack:signed，构建前退出码 1，无 release/signed 制品。开发会话报告完整门禁 75 编号、51 单元、18 Electron 通过；文档会话未独立归档完整门禁输出。见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J80" s="46" t="str">
         <x:v>npm run test:case -- TC-075</x:v>
       </x:c>
       <x:c r="K80" s="46" t="str">
-        <x:v>拟新增以 TC-075 开头的独立脚本测试函数，并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/signed-release.test.ts：test('TC-075 签名发布预检与命令构造')；scripts/test-cases.mjs 已注册一项。</x:v>
       </x:c>
       <x:c r="L80" s="46" t="str">
-        <x:v>模拟预检、错误处理和命令构造；不读取真实钥匙串/私钥、不向 Apple 提交公证，不生成已签名 DMG。自动通过不证明证书有效、票据/Gatekeeper 结果或另一台 Mac 安装。</x:v>
+        <x:v>自动函数覆盖 macOS/凭据/Developer ID 身份预检、三种凭据方式及冲突、合成 p12 本地路径与 base64 解析、forceCodeSigning/notarize/hardenedRuntime/JIT entitlement 参数、codesign/spctl/stapler/hdiutil 命令顺序、无凭据实际子进程构建前失败且不新增发布目录。未用真实钥匙串或有效 Apple 证书；未注入每个构建后核验失败、验证真实公证、DMG 原子发布或本轮 pack:dmg 回归。</x:v>
       </x:c>
       <x:c r="M80" s="46" t="str">
-        <x:v>实施后保存提交、macOS/Node、单编号命令和退出码、脱敏断言与失败分支；在隔离测试目录使用假凭据，日志不得含私钥/口令。真实签名、公证和目标 Mac 结果由 TC-028 单独记录。</x:v>
+        <x:v>文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 上独立复跑单编号 1/1 与 75 入口检查；无凭据 pack:signed 退出码 1 是预期拒绝，不算签名包。测试 p12 为 OpenSSL 一次性合成并清理，日志不含私钥/口令；真实 Apple 签名、公证、票据/Gatekeeper 与另一台 Mac 由 TC-028 单独留证。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record TC-075 failure cleanup evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R212741314ee54a4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R03d097e75444458e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9d309dd7744b4320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R87cc198de15041f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R97bae134a11d4065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd2b84efae0fc4b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R171d4d9ebe1749c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Redbd1c83007c42ea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2347,7 +2347,7 @@
         <x:v>签名发布脚本预检与命令构造</x:v>
       </x:c>
       <x:c r="G81" s="49" t="str">
-        <x:v>部分验证（自动预检/命令构造 1/1；构建后失败注入与真实发布待验）</x:v>
+        <x:v>已验证（自动；模拟预检、命令构造与五处核验失败清理）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2901,7 +2901,8 @@
       </x:c>
       <x:c r="H23" s="10" t="str">
         <x:v>docs/design.md §7；docs/development-plan.md 外部分发计划；docs/test-case-acceptance.md TC-028/TC-075；docs/validation.md。2026-10-03：签名脚本与自动预检均未实现，缺有效签名身份及另一台目标 Mac；不得把未签名 0.3.4 DMG 或将来的 TC-075 模拟通过写成外部分发通过。
-2026-10-03 后续：dc37b8b 实现 pack:signed、预检与同候选制品核验脚本，TC-075 一项自动绑定；文档会话独立复跑 1/1、75 编号检查，缺凭据构建前退出码 1 且无 signed 制品。DEV-018 仅部分落地；没有真实签名/公证、票据或目标 Mac 证据，TC-028 仍待验证。见 docs/validation.md。</x:v>
+2026-10-03 后续：dc37b8b 实现 pack:signed、预检与同候选制品核验脚本，TC-075 一项自动绑定；文档会话独立复跑 1/1、75 编号检查，缺凭据构建前退出码 1 且无 signed 制品。DEV-018 仅部分落地；没有真实签名/公证、票据或目标 Mac 证据，TC-028 仍待验证。见 docs/validation.md。
+2026-10-03 继续：2f43b00 为 TC-075 补四项核验命令与 Developer ID 身份核对共五个模拟失败分支；文档会话独立复跑同一函数 1/1、75 入口和类型检查通过。模拟失败只证明停止发布与清理，真实签名、公证及异机 TC-028 未执行；REQ-018 仍为部分实现。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
@@ -3942,7 +3943,8 @@
       </x:c>
       <x:c r="G23" s="10" t="str">
         <x:v>2026-10-03 SOP-001/002 计划：构建前检查 Developer ID Application 身份和完整公证凭据，缺项安全失败；electron-builder v26 使用 forceCodeSigning:true、mac.notarize:true，之后逐项核对 codesign、spctl、stapler、hdiutil 与 DMG SHA-256。先实现/运行模拟 TC-075 与门禁，再在具备有效证书凭据的环境构建并执行 TC-028 目标 Mac 人工验收。凭据和私钥不得入库/日志，pack:dmg 仍为本机未签名通道。
-后续 dc37b8b：electron-builder 26.15.3 以 mac.forceCodeSigning、mac.notarize、mac.hardenedRuntime、JIT entitlement 在一次性 release/token-signed-* 目录构建；逐项 codesign/spctl/stapler/hdiutil、DMG 大小/SHA-256 后才原子移到 release/signed 并写不含密钥的 release-evidence.json。TC-075 1/1、75 入口由文档会话独立复跑；无公证凭据时构建前拒绝且无 signed 制品。完整门禁 75 入口/51 单元/18 Electron 为开发会话报告；真正签名、公证、异机 TC-028 未执行。</x:v>
+后续 dc37b8b：electron-builder 26.15.3 以 mac.forceCodeSigning、mac.notarize、mac.hardenedRuntime、JIT entitlement 在一次性 release/token-signed-* 目录构建；逐项 codesign/spctl/stapler/hdiutil、DMG 大小/SHA-256 后才原子移到 release/signed 并写不含密钥的 release-evidence.json。TC-075 1/1、75 入口由文档会话独立复跑；无公证凭据时构建前拒绝且无 signed 制品。完整门禁 75 入口/51 单元/18 Electron 为开发会话报告；真正签名、公证、异机 TC-028 未执行。
+继续 2f43b00：真实发布主流程复用可注入 verifySignedCandidate / withTemporaryReleaseDirectory；TC-075 对 codesign、spctl、stapler、hdiutil 和 Developer ID Authority 五处逐项模拟失败，均断言停止、删除临时目录、无 signed 候选。文档会话单编号 1/1、75 入口检查和类型检查退出码 0；开发会话报告门禁 75 编号/51 单元/18 Electron。真实成功构建、公证及异机 TC-028 仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -4683,7 +4685,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–075 均已注册；TC-075 在 dc37b8b 有一项签名脚本自动绑定，预检/命令构造子范围通过，构建后失败注入待补；TC-028 真实签名、公证与目标 Mac 人工验收待验证。</x:v>
+        <x:v>TC-001–075 均已注册；TC-075 在 2f43b00 的一项自动绑定覆盖预检、命令构造及五处模拟核验失败/清理并通过。TC-028 真实签名、公证与目标 Mac 人工验收仍待验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7828,10 +7830,11 @@
         <x:v>异常输入须在构建前失败且执行器零调用；完整输入生成 forceCodeSigning:true、mac.notarize:true 的 v26 构建命令，并安排 codesign、spctl、stapler、hdiutil、DMG SHA-256 校验；任一步失败不得发布或复用旧未签名包，pack:dmg 仍独立可用。</x:v>
       </x:c>
       <x:c r="H80" s="46" t="str">
-        <x:v>部分验证（自动 1/1；构建后核验失败注入及真实签名待验）</x:v>
+        <x:v>已验证（自动；模拟预检、命令构造与五处核验失败清理）</x:v>
       </x:c>
       <x:c r="I80" s="46" t="str">
-        <x:v>2026-10-03 dc37b8b：文档会话独立运行 npm run test:case -- TC-075，1/1 通过、退出码 0；npm run test:cases:check 为 75 个入口、退出码 0。清除 Apple/CSC 环境变量独立运行 pack:signed，构建前退出码 1，无 release/signed 制品。开发会话报告完整门禁 75 编号、51 单元、18 Electron 通过；文档会话未独立归档完整门禁输出。见 docs/validation.md。</x:v>
+        <x:v>2026-10-03 dc37b8b：文档会话独立运行 npm run test:case -- TC-075，1/1 通过、退出码 0；npm run test:cases:check 为 75 个入口、退出码 0。清除 Apple/CSC 环境变量独立运行 pack:signed，构建前退出码 1，无 release/signed 制品。开发会话报告完整门禁 75 编号、51 单元、18 Electron 通过；文档会话未独立归档完整门禁输出。见 docs/validation.md。
+2026-10-03 继续 2f43b00：同一 TC-075 函数新增四项核验命令及 Developer ID Authority 身份核对五处逐项失败注入。文档会话独立复跑单编号 1/1、75 入口检查、类型检查均退出码 0；开发会话报告完整门禁 75 编号、51 单元、18 Electron 通过。没有真实签名、公证或目标 Mac 证据；详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J80" s="46" t="str">
         <x:v>npm run test:case -- TC-075</x:v>
@@ -7840,10 +7843,11 @@
         <x:v>tests/signed-release.test.ts：test('TC-075 签名发布预检与命令构造')；scripts/test-cases.mjs 已注册一项。</x:v>
       </x:c>
       <x:c r="L80" s="46" t="str">
-        <x:v>自动函数覆盖 macOS/凭据/Developer ID 身份预检、三种凭据方式及冲突、合成 p12 本地路径与 base64 解析、forceCodeSigning/notarize/hardenedRuntime/JIT entitlement 参数、codesign/spctl/stapler/hdiutil 命令顺序、无凭据实际子进程构建前失败且不新增发布目录。未用真实钥匙串或有效 Apple 证书；未注入每个构建后核验失败、验证真实公证、DMG 原子发布或本轮 pack:dmg 回归。</x:v>
+        <x:v>自动函数覆盖 macOS/凭据/Developer ID 身份预检、三种凭据方式及冲突、合成 p12 本地路径与 base64、forceCodeSigning/notarize/hardenedRuntime/JIT entitlement 参数、核验命令顺序、无凭据实际子进程构建前失败。2f43b00 增加 codesign、spctl、stapler、hdiutil 和 Developer ID Authority 五处模拟失败：每次停止发布、清理临时目录、无 signed 目录。未用真实钥匙串/有效 Apple 证书，未执行真实签名公证、成功 DMG 原子发布或本轮 pack:dmg 重跑；这些属 TC-028/发布验收边界。</x:v>
       </x:c>
       <x:c r="M80" s="46" t="str">
-        <x:v>文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 上独立复跑单编号 1/1 与 75 入口检查；无凭据 pack:signed 退出码 1 是预期拒绝，不算签名包。测试 p12 为 OpenSSL 一次性合成并清理，日志不含私钥/口令；真实 Apple 签名、公证、票据/Gatekeeper 与另一台 Mac 由 TC-028 单独留证。</x:v>
+        <x:v>文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 上独立复跑单编号 1/1 与 75 入口检查；无凭据 pack:signed 退出码 1 是预期拒绝，不算签名包。测试 p12 为 OpenSSL 一次性合成并清理，日志不含私钥/口令；真实 Apple 签名、公证、票据/Gatekeeper 与另一台 Mac 由 TC-028 单独留证。
+2f43b00：文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 独立复跑 TC-075 1/1、75 个编号入口和类型检查，均退出码 0。五个失败分支均用注入执行器与合成 DMG，临时 token-tc075-failed-build-* 目录结束清理；只证明模拟控制流，不生成签名制品。真实签名、公证、票据/Gatekeeper 和另一台 Mac 仍由 TC-028 留证。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: plan in-app automatic macOS updates
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R97bae134a11d4065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd2b84efae0fc4b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R171d4d9ebe1749c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Redbd1c83007c42ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R75c12ea0991d4bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R3f794961ff7946b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd621854a018646a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R1f362f11f7134801"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="25">
+  <x:fills count="26">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -179,6 +179,11 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -191,7 +196,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -332,6 +337,13 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1381,7 +1393,7 @@
         <x:v>更新版本判断与下载校验</x:v>
       </x:c>
       <x:c r="G39" s="35" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>历史自动子范围已验证；新安装前拒绝待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1404,7 +1416,7 @@
         <x:v>更新服务故障恢复</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>历史自动子范围已验证；新增故障状态待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1412,22 +1424,22 @@
         <x:v>REQ-023</x:v>
       </x:c>
       <x:c r="B41" s="35" t="str">
-        <x:v>未签名 macOS 更新交接</x:v>
+        <x:v>应用内自动安装升级</x:v>
       </x:c>
       <x:c r="C41" s="35" t="str">
         <x:v>DEV-025</x:v>
       </x:c>
       <x:c r="D41" s="35" t="str">
-        <x:v>未签名安装包打开与回退</x:v>
+        <x:v>受约束自动安装辅助进程与失败回滚</x:v>
       </x:c>
       <x:c r="E41" s="35" t="str">
         <x:v>TC-036</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
-        <x:v>未签名安装包交接</x:v>
+        <x:v>自动安装控制与回退</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>部分验证（本机取消通过；Finder 回退待验）</x:v>
+        <x:v>旧手动交接部分验证；新自动安装待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2348,6 +2360,29 @@
       </x:c>
       <x:c r="G81" s="49" t="str">
         <x:v>已验证（自动；模拟预检、命令构造与五处核验失败清理）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="100" customHeight="1">
+      <x:c r="A82" s="52" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="B82" s="52" t="str">
+        <x:v>应用内自动安装升级</x:v>
+      </x:c>
+      <x:c r="C82" s="52" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="D82" s="52" t="str">
+        <x:v>受约束自动安装辅助进程与失败回滚</x:v>
+      </x:c>
+      <x:c r="E82" s="52" t="str">
+        <x:v>TC-076</x:v>
+      </x:c>
+      <x:c r="F82" s="52" t="str">
+        <x:v>实际打包 App 隔离自动升级</x:v>
+      </x:c>
+      <x:c r="G82" s="52" t="str">
+        <x:v>待注册、待验证（实际制品自动升级）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2995,13 +3030,13 @@
         <x:v>版本检查和安装包下载</x:v>
       </x:c>
       <x:c r="C27" s="35" t="str">
-        <x:v>应用请求本地服务版本清单，仅在版本更新且平台匹配时提示；下载到受控临时目录，校验长度和 SHA-256 后才可交给系统打开；无服务、损坏或低版本给出可恢复状态。</x:v>
+        <x:v>应用请求已配置服务的版本清单，仅较新且平台/架构匹配时提示；下载到受控临时目录，在安装前校验大小和 SHA-256。停服、超时、中断、空间不足、错误摘要和用户取消须展示阶段与可重试状态，坏包绝不交给安装辅助进程，旧版与本机报表仍可用。</x:v>
       </x:c>
       <x:c r="D27" s="35" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
+        <x:v>既有检查/下载代码已落地；自动安装前错误口径与新增断言待实现/待验证</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>DEV-024</x:v>
@@ -3010,7 +3045,7 @@
         <x:v>TC-034、TC-035</x:v>
       </x:c>
       <x:c r="H27" s="35" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
@@ -3018,25 +3053,25 @@
         <x:v>REQ-023</x:v>
       </x:c>
       <x:c r="B28" s="14" t="str">
-        <x:v>未签名 macOS 更新交接</x:v>
+        <x:v>应用内自动安装升级</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>当前未签名应用发现更新后下载并打开安装包，由用户完成安装；不得调用静默替换或承诺自动安装；取消打开或安装失败保留旧版可运行。</x:v>
+        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。取消或挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>代码已落地；本机隔离升级链路部分验证</x:v>
+        <x:v>旧下载打开流程已编码且仅有历史部分验证；新自动安装目标待实现/待验证</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>TC-036</x:v>
+        <x:v>TC-036、TC-076</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md</x:v>
+        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4081,13 +4116,13 @@
         <x:v>TC-034、TC-035</x:v>
       </x:c>
       <x:c r="E29" s="35" t="str">
-        <x:v>src/main/update-client.ts；src/main/server-connection.ts；tests/next-update.test.ts</x:v>
+        <x:v>src/main/update-client.ts；src/main/server-connection.ts；更新状态 IPC/界面；tests/next-update.test.ts；scripts/test-cases.mjs 的 TC-034/035 绑定</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
-        <x:v>已编码（自动覆盖；边界待验）</x:v>
+        <x:v>既有检查/下载已编码；自动安装前故障状态与新增断言待实现/待验证</x:v>
       </x:c>
       <x:c r="G29" s="35" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -4095,22 +4130,22 @@
         <x:v>DEV-025</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>未签名安装包打开与回退</x:v>
+        <x:v>受约束自动安装辅助进程与失败回滚</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
         <x:v>REQ-023</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>TC-036</x:v>
+        <x:v>TC-036、TC-076</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>src/main/update-client.ts；tests/next-update.test.ts；scripts/verify-local-upgrade.mjs</x:v>
+        <x:v>src/main/update-client.ts；待实现独立更新辅助进程、安装状态 IPC/界面；tests/next-update.test.ts；待注册 TC-076 实际打包 App 隔离升级；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>已编码；本机隔离升级链路部分验证</x:v>
+        <x:v>旧下载打开/隔离脚本替换仅历史部分验证；新自动安装与 TC-076 待开发/待验证</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md</x:v>
+        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -4685,7 +4720,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–075 均已注册；TC-075 在 2f43b00 的一项自动绑定覆盖预检、命令构造及五处模拟核验失败/清理并通过。TC-028 真实签名、公证与目标 Mac 人工验收仍待验证。</x:v>
+        <x:v>TC-001–076 已分配；TC-001–075 已注册，TC-076 实际打包 App 自动升级待注册/待验证。TC-034–036 新自动安装目标待验证；TC-028 真实签名、公证及目标 Mac 人工验收仍待验证。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6127,16 +6162,16 @@
         <x:v>单元</x:v>
       </x:c>
       <x:c r="F39" s="35" t="str">
-        <x:v>模拟新/同/旧版本和正确/错误 SHA-256。</x:v>
+        <x:v>模拟新/同/旧版本、架构不符、错误大小与 SHA-256，检查只有完整校验的包可交给安装辅助进程。</x:v>
       </x:c>
       <x:c r="G39" s="35" t="str">
-        <x:v>仅新且匹配版本提示；错误摘要不得打开文件。</x:v>
+        <x:v>只提示匹配的新版本；大小或摘要错误绝不启动安装，临时包清理。</x:v>
       </x:c>
       <x:c r="H39" s="35" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>历史自动子范围已验证；新增安装前拒绝断言待验证</x:v>
       </x:c>
       <x:c r="I39" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：旧通过只覆盖当时的版本/架构/摘要与打开路径，不证明辅助进程从未收到坏包；新增断言待实现。</x:v>
       </x:c>
       <x:c r="J39" s="35" t="str">
         <x:v>npm run test:case -- TC-034</x:v>
@@ -6145,7 +6180,7 @@
         <x:v>tests/next-update.test.ts：test('TC-034 只提示较新且架构匹配的版本并校验包摘要')</x:v>
       </x:c>
       <x:c r="L39" s="35" t="str">
-        <x:v>版本、架构、坏摘要；合成包路径</x:v>
+        <x:v>版本、架构、坏摘要；合成包路径；新增目标须断言坏包不触发自动安装。</x:v>
       </x:c>
       <x:c r="M39" s="35" t="str">
         <x:v>记录 TC-034 命令、退出码、提交、环境和脱敏日志；覆盖与限制：版本、架构、坏摘要；合成包路径。</x:v>
@@ -6168,16 +6203,16 @@
         <x:v>单元</x:v>
       </x:c>
       <x:c r="F40" s="14" t="str">
-        <x:v>模拟停服、超时、中断和空间不足后重试。</x:v>
+        <x:v>模拟停服、超时、中断、磁盘空间不足与取消，核对下载/校验阶段错误、清理和重试。</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>显示可恢复错误，本机报表可用，无损坏包残留。</x:v>
+        <x:v>错误阶段可见且可重试；无损坏临时包，旧版和本机报表继续可用。</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>历史自动子范围已验证；新增故障状态待验证</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：原停服/重试通过仍有效于旧范围；超时、空间不足、取消和安装前状态/旧版可用性待新增断言。</x:v>
       </x:c>
       <x:c r="J40" s="14" t="str">
         <x:v>npm run test:case -- TC-035</x:v>
@@ -6186,7 +6221,7 @@
         <x:v>tests/next-update.test.ts：test('TC-035 停服和下载失败可重试且不留临时包')</x:v>
       </x:c>
       <x:c r="L40" s="14" t="str">
-        <x:v>停服/重试/临时文件；未测超时、磁盘不足</x:v>
+        <x:v>停服/重试/临时文件；未测超时、磁盘不足；新增目标须覆盖安装前失败和取消，不得留下坏包。</x:v>
       </x:c>
       <x:c r="M40" s="14" t="str">
         <x:v>记录 TC-035 命令、退出码、提交、环境和脱敏日志；覆盖与限制：停服/重试/临时文件；未测超时、磁盘不足。</x:v>
@@ -6203,34 +6238,34 @@
         <x:v>DEV-025</x:v>
       </x:c>
       <x:c r="D41" s="35" t="str">
-        <x:v>未签名安装包交接</x:v>
+        <x:v>自动安装控制与回退</x:v>
       </x:c>
       <x:c r="E41" s="35" t="str">
-        <x:v>单元＋本机隔离链路</x:v>
+        <x:v>单元/辅助进程故障注入</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
-        <x:v>未签名包通过校验后下载，选择打开/取消。</x:v>
+        <x:v>注入已校验包的辅助进程启动、旧进程退出、挂载、替换、重启和健康确认成功/失败；测试取消及不可写安装位置。</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>只打开安装包供用户安装；取消后旧版和数据仍可用。</x:v>
+        <x:v>成功路径自动退出旧版、安装替换并启动新版；失败回滚旧版、保留用户数据、清理挂载/临时文件；权限不足不静默绕过，成功无需 Finder 拖拽。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>部分验证（本机交接/替换/取消通过；真实安装回退待验）</x:v>
+        <x:v>旧手动交接部分验证；新自动安装目标待验证</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。</x:v>
+        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
         <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
       </x:c>
       <x:c r="K41" s="35" t="str">
-        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs；计划将 TC-036 独立绑定改为自动安装控制/回滚断言，当前绑定仅是历史旧行为。</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。</x:v>
+        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。；新目标的自动替换、重启、权限/回滚未验证；真实制品见待注册 TC-076。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。</x:v>
+        <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。；2026-10-03 起旧 Finder 手动安装不再是自动成功路径目标；原缺口与证据作为历史保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">
@@ -7850,6 +7885,47 @@
 2f43b00：文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 独立复跑 TC-075 1/1、75 个编号入口和类型检查，均退出码 0。五个失败分支均用注入执行器与合成 DMG，临时 token-tc075-failed-build-* 目录结束清理；只证明模拟控制流，不生成签名制品。真实签名、公证、票据/Gatekeeper 和另一台 Mac 仍由 TC-028 留证。</x:v>
       </x:c>
     </x:row>
+    <x:row r="81" ht="200" customHeight="1">
+      <x:c r="A81" s="52" t="str">
+        <x:v>TC-076</x:v>
+      </x:c>
+      <x:c r="B81" s="52" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="C81" s="52" t="str">
+        <x:v>DEV-025</x:v>
+      </x:c>
+      <x:c r="D81" s="52" t="str">
+        <x:v>实际打包 App 隔离自动升级</x:v>
+      </x:c>
+      <x:c r="E81" s="52" t="str">
+        <x:v>打包应用/本机隔离</x:v>
+      </x:c>
+      <x:c r="F81" s="52" t="str">
+        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。分别注入取消、磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。</x:v>
+      </x:c>
+      <x:c r="G81" s="52" t="str">
+        <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。</x:v>
+      </x:c>
+      <x:c r="H81" s="52" t="str">
+        <x:v>待注册、待验证（新自动升级制品目标）</x:v>
+      </x:c>
+      <x:c r="I81" s="52" t="str">
+        <x:v>2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。</x:v>
+      </x:c>
+      <x:c r="J81" s="52" t="str">
+        <x:v>npm run test:case -- TC-076（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K81" s="52" t="str">
+        <x:v>拟新增以 TC-076 开头的独立打包应用测试函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L81" s="52" t="str">
+        <x:v>使用隔离可写安装位置、临时用户数据/SQLite、人工合成无正文 Codex/Claude 用量；检查旧进程退出、新版安装/重启和健康、只读 DMG 两条目标选择，故障回滚及清理。真实生产库、系统 /Applications 授权和另一台 Mac 需独立边界说明。</x:v>
+      </x:c>
+      <x:c r="M81" s="52" t="str">
+        <x:v>实施后保存旧/新 DMG SHA-256、macOS/架构、固定代码提交、单编号命令及退出码、脱敏启动/安装/回滚日志；不读取真实会话或生产数据库。真实签名/公证和其他目标 Mac 归 TC-028。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: trace product polish and 0.3.5 evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R75c12ea0991d4bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R3f794961ff7946b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd621854a018646a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R1f362f11f7134801"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ad500fb40c54648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R925e1fb276eb47b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R916b6bed4c6e402d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf05099fe074d40bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -184,6 +184,26 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -196,7 +216,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="53">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -344,6 +364,34 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -979,7 +1027,7 @@
         <x:v>遥测幂等和重叠优先级</x:v>
       </x:c>
       <x:c r="G21" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>旧 UTC 日去重历史自动通过；跨用户误排除待 REQ-048 修复</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
@@ -1393,7 +1441,7 @@
         <x:v>更新版本判断与下载校验</x:v>
       </x:c>
       <x:c r="G39" s="35" t="str">
-        <x:v>历史自动子范围已验证；新安装前拒绝待验证</x:v>
+        <x:v>0.3.5 自动子范围通过；边界待验</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1416,7 +1464,7 @@
         <x:v>更新服务故障恢复</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>历史自动子范围已验证；新增故障状态待验证</x:v>
+        <x:v>0.3.5 自动子范围通过；边界待验</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1439,7 +1487,7 @@
         <x:v>自动安装控制与回退</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>旧手动交接部分验证；新自动安装待验证</x:v>
+        <x:v>0.3.5 单元控制/回滚通过；真实制品边界待验</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -1962,13 +2010,13 @@
         <x:v>更新入口迁移和状态机界面</x:v>
       </x:c>
       <x:c r="E64" s="36" t="str">
-        <x:v>TC-058</x:v>
+        <x:v>TC-059</x:v>
       </x:c>
       <x:c r="F64" s="36" t="str">
         <x:v>更新入口可发现</x:v>
       </x:c>
       <x:c r="G64" s="36" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>0.3.5 自动 E2E 子范围通过；真实安装待验</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="66" customHeight="1">
@@ -2382,7 +2430,398 @@
         <x:v>实际打包 App 隔离自动升级</x:v>
       </x:c>
       <x:c r="G82" s="52" t="str">
-        <x:v>待注册、待验证（实际制品自动升级）</x:v>
+        <x:v>已注册；合成旧版自动成功链路部分验证</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="85" customHeight="1">
+      <x:c r="A83" s="55" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="B83" s="55" t="str">
+        <x:v>所选范围的可证覆盖与可比区间</x:v>
+      </x:c>
+      <x:c r="C83" s="55" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="D83" s="55" t="str">
+        <x:v>构建按筛选范围的覆盖判定与可比性门禁</x:v>
+      </x:c>
+      <x:c r="E83" s="55" t="str">
+        <x:v>TC-077</x:v>
+      </x:c>
+      <x:c r="F83" s="55" t="str">
+        <x:v>所选范围覆盖真值表</x:v>
+      </x:c>
+      <x:c r="G83" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="85" customHeight="1">
+      <x:c r="A84" s="58" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="B84" s="58" t="str">
+        <x:v>所选范围的可证覆盖与可比区间</x:v>
+      </x:c>
+      <x:c r="C84" s="58" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="D84" s="58" t="str">
+        <x:v>构建按筛选范围的覆盖判定与可比性门禁</x:v>
+      </x:c>
+      <x:c r="E84" s="58" t="str">
+        <x:v>TC-078</x:v>
+      </x:c>
+      <x:c r="F84" s="58" t="str">
+        <x:v>区间比较可比性门禁</x:v>
+      </x:c>
+      <x:c r="G84" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="85" customHeight="1">
+      <x:c r="A85" s="55" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="B85" s="55" t="str">
+        <x:v>筛选异步加载与 CSV 同一查询</x:v>
+      </x:c>
+      <x:c r="C85" s="55" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="D85" s="55" t="str">
+        <x:v>统一异步查询键与页面 CSV 快照</x:v>
+      </x:c>
+      <x:c r="E85" s="55" t="str">
+        <x:v>TC-079</x:v>
+      </x:c>
+      <x:c r="F85" s="55" t="str">
+        <x:v>异步筛选与 CSV 快照一致</x:v>
+      </x:c>
+      <x:c r="G85" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="85" customHeight="1">
+      <x:c r="A86" s="58" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="B86" s="58" t="str">
+        <x:v>多维下钻上下文与模型身份</x:v>
+      </x:c>
+      <x:c r="C86" s="58" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="D86" s="58" t="str">
+        <x:v>实现概览多维下钻与提供方模型键</x:v>
+      </x:c>
+      <x:c r="E86" s="58" t="str">
+        <x:v>TC-080</x:v>
+      </x:c>
+      <x:c r="F86" s="58" t="str">
+        <x:v>趋势下钻保留 7/30/90 天上下文</x:v>
+      </x:c>
+      <x:c r="G86" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="85" customHeight="1">
+      <x:c r="A87" s="55" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="B87" s="55" t="str">
+        <x:v>多维下钻上下文与模型身份</x:v>
+      </x:c>
+      <x:c r="C87" s="55" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="D87" s="55" t="str">
+        <x:v>实现概览多维下钻与提供方模型键</x:v>
+      </x:c>
+      <x:c r="E87" s="55" t="str">
+        <x:v>TC-081</x:v>
+      </x:c>
+      <x:c r="F87" s="55" t="str">
+        <x:v>跨提供方同名模型排行隔离</x:v>
+      </x:c>
+      <x:c r="G87" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="85" customHeight="1">
+      <x:c r="A88" s="58" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="B88" s="58" t="str">
+        <x:v>可跳过的首次使用四步引导</x:v>
+      </x:c>
+      <x:c r="C88" s="58" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D88" s="58" t="str">
+        <x:v>实现角色感知的可跳过首次引导</x:v>
+      </x:c>
+      <x:c r="E88" s="58" t="str">
+        <x:v>TC-082</x:v>
+      </x:c>
+      <x:c r="F88" s="58" t="str">
+        <x:v>管理员四步引导与跳过恢复</x:v>
+      </x:c>
+      <x:c r="G88" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="85" customHeight="1">
+      <x:c r="A89" s="55" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="B89" s="55" t="str">
+        <x:v>可跳过的首次使用四步引导</x:v>
+      </x:c>
+      <x:c r="C89" s="55" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D89" s="55" t="str">
+        <x:v>实现角色感知的可跳过首次引导</x:v>
+      </x:c>
+      <x:c r="E89" s="55" t="str">
+        <x:v>TC-083</x:v>
+      </x:c>
+      <x:c r="F89" s="55" t="str">
+        <x:v>普通用户引导角色边界</x:v>
+      </x:c>
+      <x:c r="G89" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="85" customHeight="1">
+      <x:c r="A90" s="58" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="B90" s="58" t="str">
+        <x:v>可操作空状态与扫描反馈</x:v>
+      </x:c>
+      <x:c r="C90" s="58" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="D90" s="58" t="str">
+        <x:v>实现分型空状态、诊断行动与扫描进展</x:v>
+      </x:c>
+      <x:c r="E90" s="58" t="str">
+        <x:v>TC-084</x:v>
+      </x:c>
+      <x:c r="F90" s="58" t="str">
+        <x:v>六类空状态与可操作下一步</x:v>
+      </x:c>
+      <x:c r="G90" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="85" customHeight="1">
+      <x:c r="A91" s="55" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="B91" s="55" t="str">
+        <x:v>可操作空状态与扫描反馈</x:v>
+      </x:c>
+      <x:c r="C91" s="55" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="D91" s="55" t="str">
+        <x:v>实现分型空状态、诊断行动与扫描进展</x:v>
+      </x:c>
+      <x:c r="E91" s="55" t="str">
+        <x:v>TC-085</x:v>
+      </x:c>
+      <x:c r="F91" s="55" t="str">
+        <x:v>长扫描进展与诊断重试</x:v>
+      </x:c>
+      <x:c r="G91" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="85" customHeight="1">
+      <x:c r="A92" s="58" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="B92" s="58" t="str">
+        <x:v>来源重新绑定预览确认与最小审计</x:v>
+      </x:c>
+      <x:c r="C92" s="58" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="D92" s="58" t="str">
+        <x:v>实现来源重绑预览事务与最小审计</x:v>
+      </x:c>
+      <x:c r="E92" s="58" t="str">
+        <x:v>TC-086</x:v>
+      </x:c>
+      <x:c r="F92" s="58" t="str">
+        <x:v>来源重绑预览与确认范围</x:v>
+      </x:c>
+      <x:c r="G92" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="85" customHeight="1">
+      <x:c r="A93" s="55" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="B93" s="55" t="str">
+        <x:v>来源重新绑定预览确认与最小审计</x:v>
+      </x:c>
+      <x:c r="C93" s="55" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="D93" s="55" t="str">
+        <x:v>实现来源重绑预览事务与最小审计</x:v>
+      </x:c>
+      <x:c r="E93" s="55" t="str">
+        <x:v>TC-087</x:v>
+      </x:c>
+      <x:c r="F93" s="55" t="str">
+        <x:v>来源重绑失败回滚与最小审计</x:v>
+      </x:c>
+      <x:c r="G93" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="85" customHeight="1">
+      <x:c r="A94" s="58" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="B94" s="58" t="str">
+        <x:v>本机采集与可选服务上报分离</x:v>
+      </x:c>
+      <x:c r="C94" s="58" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="D94" s="58" t="str">
+        <x:v>分离本机采集与服务上报状态</x:v>
+      </x:c>
+      <x:c r="E94" s="58" t="str">
+        <x:v>TC-088</x:v>
+      </x:c>
+      <x:c r="F94" s="58" t="str">
+        <x:v>本机采集与可选服务状态分离</x:v>
+      </x:c>
+      <x:c r="G94" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="85" customHeight="1">
+      <x:c r="A95" s="55" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="B95" s="55" t="str">
+        <x:v>窄窗口与无障碍精确值</x:v>
+      </x:c>
+      <x:c r="C95" s="55" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D95" s="55" t="str">
+        <x:v>补齐键盘 VoiceOver 精确值及文案走查</x:v>
+      </x:c>
+      <x:c r="E95" s="55" t="str">
+        <x:v>TC-089</x:v>
+      </x:c>
+      <x:c r="F95" s="55" t="str">
+        <x:v>窄窗口键盘与 VoiceOver 主路径</x:v>
+      </x:c>
+      <x:c r="G95" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="85" customHeight="1">
+      <x:c r="A96" s="58" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="B96" s="58" t="str">
+        <x:v>窄窗口与无障碍精确值</x:v>
+      </x:c>
+      <x:c r="C96" s="58" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D96" s="58" t="str">
+        <x:v>补齐键盘 VoiceOver 精确值及文案走查</x:v>
+      </x:c>
+      <x:c r="E96" s="58" t="str">
+        <x:v>TC-090</x:v>
+      </x:c>
+      <x:c r="F96" s="58" t="str">
+        <x:v>精确 Token 与覆盖状态非悬浮可读</x:v>
+      </x:c>
+      <x:c r="G96" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="85" customHeight="1">
+      <x:c r="A97" s="55" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="B97" s="55" t="str">
+        <x:v>窄窗口与无障碍精确值</x:v>
+      </x:c>
+      <x:c r="C97" s="55" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D97" s="55" t="str">
+        <x:v>补齐键盘 VoiceOver 精确值及文案走查</x:v>
+      </x:c>
+      <x:c r="E97" s="55" t="str">
+        <x:v>TC-091</x:v>
+      </x:c>
+      <x:c r="F97" s="55" t="str">
+        <x:v>关键文案与动作逐状态走查</x:v>
+      </x:c>
+      <x:c r="G97" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="90" customHeight="1">
+      <x:c r="A98" s="61" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="B98" s="61" t="str">
+        <x:v>本地与遥测按身份去重及冲突可见</x:v>
+      </x:c>
+      <x:c r="C98" s="61" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="D98" s="61" t="str">
+        <x:v>修复本地/遥测重叠选择的身份粒度</x:v>
+      </x:c>
+      <x:c r="E98" s="61" t="str">
+        <x:v>TC-092</x:v>
+      </x:c>
+      <x:c r="F98" s="61" t="str">
+        <x:v>同会话重复与跨用户独立保留</x:v>
+      </x:c>
+      <x:c r="G98" s="61" t="str">
+        <x:v>待注册、待验证（缺陷已复现）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="90" customHeight="1">
+      <x:c r="A99" s="64" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="B99" s="64" t="str">
+        <x:v>本地与遥测按身份去重及冲突可见</x:v>
+      </x:c>
+      <x:c r="C99" s="64" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="D99" s="64" t="str">
+        <x:v>修复本地/遥测重叠选择的身份粒度</x:v>
+      </x:c>
+      <x:c r="E99" s="64" t="str">
+        <x:v>TC-093</x:v>
+      </x:c>
+      <x:c r="F99" s="64" t="str">
+        <x:v>无法关联冲突与三处报表权限一致</x:v>
+      </x:c>
+      <x:c r="G99" s="64" t="str">
+        <x:v>待注册、待验证；TC-093 明确已确认小计、待核对来源/条数和总量不可确认的页面/CSV 同口径</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2685,13 +3124,13 @@
         <x:v>遥测去重与来源重叠</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>重复遥测批次不增加总量；累计指标计算增量；同提供方同 UTC 日有本地记录时报表优先本地记录。</x:v>
+        <x:v>重复遥测批次不增加总量、累计指标按增量计算。本地与遥测只有可确认属于同一会话/事件的重复事实才按主来源去重；不同用户或不同会话的独立事实保留；无法可靠关联的重叠标冲突，不静默相加或整日排除。旧“同提供方同 UTC 日有任意本地事实即排除全部遥测”的规则是修复前历史，详见 REQ-048。</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>M2</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>已实现（本机）</x:v>
+        <x:v>旧 UTC 日优先逻辑已编码；跨用户/不同会话误排除待 REQ-048 修复</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
         <x:v>DEV-009</x:v>
@@ -2700,7 +3139,8 @@
         <x:v>TC-016</x:v>
       </x:c>
       <x:c r="H14" s="9" t="str">
-        <x:v>README.md §可选官方遥测；docs/design.md §4.3</x:v>
+        <x:v>README.md §可选官方遥测；docs/design.md §4.3
+2026-10-03 隔离 SQLite 复现：同日 Codex 本地 owner A 12 Token 与遥测 owner B 99 Token 输入，src/main/report.ts selectFacts 的 provider+UTC 日 NOT EXISTS 只返回 A。现有 TC-016 历史通过不能证明不同用户独立。新规则由 REQ-048/DEV-057/TC-092–093 承接。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -3036,7 +3476,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>既有检查/下载代码已落地；自动安装前错误口径与新增断言待实现/待验证</x:v>
+        <x:v>已编码（0.3.5 检查/下载与坏摘要拒绝自动通过；超时/空间不足等新增边界待验）</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>DEV-024</x:v>
@@ -3045,7 +3485,8 @@
         <x:v>TC-034、TC-035</x:v>
       </x:c>
       <x:c r="H27" s="35" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。</x:v>
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
+2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
@@ -3062,7 +3503,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>旧下载打开流程已编码且仅有历史部分验证；新自动安装目标待实现/待验证</x:v>
+        <x:v>0.3.5 自动安装代码已落地；合成旧版隔离成功链路/单元回滚通过，真实历史旧版一键过渡与环境边界待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3071,7 +3512,8 @@
         <x:v>TC-036、TC-076</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。</x:v>
+        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
+2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -3368,7 +3810,7 @@
         <x:v>集中系统设置与 macOS 文件权限引导</x:v>
       </x:c>
       <x:c r="C40" s="36" t="str">
-        <x:v>集中展示服务器、采集、更新与本机权限设置；按角色保护修改入口；来源无权限时说明所需 macOS 操作和重试路径，不自动提权或读取其他账户文件。</x:v>
+        <x:v>集中展示服务器、采集、更新与本机权限设置；按角色保护修改入口；来源无权限时说明所需 macOS 操作和重试路径，不自动提权或读取其他账户文件。 目标 Mac 须以独立测试账户实测拒绝、授予、撤销及每步重扫，未获授权时保持未知并不越权。</x:v>
       </x:c>
       <x:c r="D40" s="36" t="str">
         <x:v>M6（本机实现）</x:v>
@@ -3383,7 +3825,7 @@
         <x:v>TC-060、TC-061、TC-072</x:v>
       </x:c>
       <x:c r="H40" s="36" t="str">
-        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 明确目标 Mac 拒绝→授予→撤销→重扫闭环；原自动模拟结果不代替真实系统证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -3488,6 +3930,240 @@
       </x:c>
       <x:c r="H44" s="36" t="str">
         <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="150" customHeight="1">
+      <x:c r="A45" s="55" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="B45" s="55" t="str">
+        <x:v>所选范围的可证覆盖与可比区间</x:v>
+      </x:c>
+      <x:c r="C45" s="55" t="str">
+        <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。</x:v>
+      </x:c>
+      <x:c r="D45" s="55" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E45" s="55" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F45" s="55" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="G45" s="55" t="str">
+        <x:v>TC-077、TC-078</x:v>
+      </x:c>
+      <x:c r="H45" s="55" t="str">
+        <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="150" customHeight="1">
+      <x:c r="A46" s="58" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="B46" s="58" t="str">
+        <x:v>筛选异步加载与 CSV 同一查询</x:v>
+      </x:c>
+      <x:c r="C46" s="58" t="str">
+        <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。</x:v>
+      </x:c>
+      <x:c r="D46" s="58" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E46" s="58" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F46" s="58" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="G46" s="58" t="str">
+        <x:v>TC-079</x:v>
+      </x:c>
+      <x:c r="H46" s="58" t="str">
+        <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="150" customHeight="1">
+      <x:c r="A47" s="55" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="B47" s="55" t="str">
+        <x:v>多维下钻上下文与模型身份</x:v>
+      </x:c>
+      <x:c r="C47" s="55" t="str">
+        <x:v>概览趋势和模型排行可下钻到授权明细；继承近 7/30/90 天、工具、模型、用户、时区和时间桶，返回面包屑保留筛选与可见焦点。同名模型按提供方+模型键区分，不能串数。</x:v>
+      </x:c>
+      <x:c r="D47" s="55" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E47" s="55" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F47" s="55" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="G47" s="55" t="str">
+        <x:v>TC-080、TC-081</x:v>
+      </x:c>
+      <x:c r="H47" s="55" t="str">
+        <x:v>承接 REQ-013/028/029/033；同名模型跨提供方使用稳定复合身份。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="150" customHeight="1">
+      <x:c r="A48" s="58" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="B48" s="58" t="str">
+        <x:v>可跳过的首次使用四步引导</x:v>
+      </x:c>
+      <x:c r="C48" s="58" t="str">
+        <x:v>首次使用按检测→扫描→归属→第一笔用量四步引导，可跳过并从入口重新打开；每步只显示真实完成状态。管理员可执行来源归属，普通用户只看授权用量及请求管理员操作指引；不自动重绑或读取额外文件。</x:v>
+      </x:c>
+      <x:c r="D48" s="58" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E48" s="58" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F48" s="58" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="G48" s="58" t="str">
+        <x:v>TC-082、TC-083</x:v>
+      </x:c>
+      <x:c r="H48" s="58" t="str">
+        <x:v>独立新能力；与现有首次建账及角色授权兼容。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="150" customHeight="1">
+      <x:c r="A49" s="55" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="B49" s="55" t="str">
+        <x:v>可操作空状态与扫描反馈</x:v>
+      </x:c>
+      <x:c r="C49" s="55" t="str">
+        <x:v>真零、未扫描、权限不足、格式不支持、筛选无匹配和部分覆盖分别说明原因与下一步；诊断原因指向相应授权/重扫/调整筛选动作。长扫描持续显示阶段与最近进展，不伪造百分比，失败可重试。</x:v>
+      </x:c>
+      <x:c r="D49" s="55" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E49" s="55" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F49" s="55" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="G49" s="55" t="str">
+        <x:v>TC-084、TC-085</x:v>
+      </x:c>
+      <x:c r="H49" s="55" t="str">
+        <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="150" customHeight="1">
+      <x:c r="A50" s="58" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="B50" s="58" t="str">
+        <x:v>来源重新绑定预览确认与最小审计</x:v>
+      </x:c>
+      <x:c r="C50" s="58" t="str">
+        <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、来源稳定键、前后用户 ID、数量和结果码，不含路径/正文。</x:v>
+      </x:c>
+      <x:c r="D50" s="58" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E50" s="58" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F50" s="58" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="G50" s="58" t="str">
+        <x:v>TC-086、TC-087</x:v>
+      </x:c>
+      <x:c r="H50" s="58" t="str">
+        <x:v>承接 REQ-011；归属与报表权限应在同一提交边界生效。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="150" customHeight="1">
+      <x:c r="A51" s="55" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="B51" s="55" t="str">
+        <x:v>本机采集与可选服务上报分离</x:v>
+      </x:c>
+      <x:c r="C51" s="55" t="str">
+        <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。</x:v>
+      </x:c>
+      <x:c r="D51" s="55" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E51" s="55" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F51" s="55" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="G51" s="55" t="str">
+        <x:v>TC-088</x:v>
+      </x:c>
+      <x:c r="H51" s="55" t="str">
+        <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="150" customHeight="1">
+      <x:c r="A52" s="58" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="B52" s="58" t="str">
+        <x:v>窄窗口与无障碍精确值</x:v>
+      </x:c>
+      <x:c r="C52" s="58" t="str">
+        <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。</x:v>
+      </x:c>
+      <x:c r="D52" s="58" t="str">
+        <x:v>下一轮产品打磨（计划）</x:v>
+      </x:c>
+      <x:c r="E52" s="58" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F52" s="58" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="G52" s="58" t="str">
+        <x:v>TC-089、TC-090、TC-091</x:v>
+      </x:c>
+      <x:c r="H52" s="58" t="str">
+        <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="170" customHeight="1">
+      <x:c r="A53" s="61" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="B53" s="61" t="str">
+        <x:v>本地与遥测按身份去重及冲突可见</x:v>
+      </x:c>
+      <x:c r="C53" s="61" t="str">
+        <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。</x:v>
+      </x:c>
+      <x:c r="D53" s="61" t="str">
+        <x:v>缺陷修复（已复现）</x:v>
+      </x:c>
+      <x:c r="E53" s="61" t="str">
+        <x:v>待修复/待验证</x:v>
+      </x:c>
+      <x:c r="F53" s="61" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="G53" s="61" t="str">
+        <x:v>TC-092、TC-093</x:v>
+      </x:c>
+      <x:c r="H53" s="61" t="str">
+        <x:v>2026-10-03 在一次性 SQLite 内按 src/main/report.ts selectFacts SQL 构造本地 owner A 12 Token、遥测 owner B 99 Token（同日 Codex），实际查询只返回 A；无真实数据。修复前 REQ-009/TC-016 的 UTC 日优先为历史证据。设计 docs/design.md §4.3、§20；开发计划 §13。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3769,7 +4445,8 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="G14" s="9" t="str">
-        <x:v>重复批次、累计指标、同日重叠</x:v>
+        <x:v>重复批次、累计指标、同日重叠
+2026-10-03 旧按 provider+UTC 日整日排除的实现有跨用户误删复现；修复由 DEV-057 承接，DEV-009/TC-016 结果留作历史。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -4119,10 +4796,11 @@
         <x:v>src/main/update-client.ts；src/main/server-connection.ts；更新状态 IPC/界面；tests/next-update.test.ts；scripts/test-cases.mjs 的 TC-034/035 绑定</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
-        <x:v>既有检查/下载已编码；自动安装前故障状态与新增断言待实现/待验证</x:v>
+        <x:v>0.3.5 已编码；TC-034/035/059 自动子范围通过，安装前异常边界待补</x:v>
       </x:c>
       <x:c r="G29" s="35" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。
+86a4b5b：客户端下载后校验大小/SHA-256 再交自动安装器，坏包不会触发 helper；文档会话 TC-034/035/059 与 76 入口检查退出码 0。超时/磁盘不足与真实用户错误恢复仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -4139,13 +4817,14 @@
         <x:v>TC-036、TC-076</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>src/main/update-client.ts；待实现独立更新辅助进程、安装状态 IPC/界面；tests/next-update.test.ts；待注册 TC-076 实际打包 App 隔离升级；scripts/test-cases.mjs</x:v>
+        <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>旧下载打开/隔离脚本替换仅历史部分验证；新自动安装与 TC-076 待开发/待验证</x:v>
+        <x:v>0.3.5 已编码；单元回滚与合成旧版隔离自动成功通过；真实历史旧版/只读 DMG 及目标环境部分待验</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。</x:v>
+        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
+86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -4490,7 +5169,7 @@
         <x:v>已编码（TC-072 人工待验）</x:v>
       </x:c>
       <x:c r="G45" s="37" t="str">
-        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 真实目标 Mac 文件权限拒绝、授予、撤销及重扫继续待验，所需系统版本/截图/日志须脱敏。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="66" customHeight="1">
@@ -4676,6 +5355,215 @@
       </x:c>
       <x:c r="G53" s="42" t="str">
         <x:v>2026-10-03：ca0f37f 完成管理密钥登记/撤销、设备令牌哈希、设备/owner 写库前授权、客户端加密凭据与待传恢复；TC-074 初版三项。533992e 只清理 TC-047 TLS 测试资源。3d60b5e 以配置代次防止切换服务器时旧登记响应落盘或上传，TC-074 增为四项；文档会话独立复跑四项通过。开发会话报告门禁 74 编号、47 单元、18 Electron 和目录包 18/18；0.3.3 DMG 摘要与本机服务目录、隔离升级独立核验。生产账户/库、可信证书异机、签名公证、目标 Mac 待验；详见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="155" customHeight="1">
+      <x:c r="A54" s="55" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="B54" s="55" t="str">
+        <x:v>构建按筛选范围的覆盖判定与可比性门禁</x:v>
+      </x:c>
+      <x:c r="C54" s="55" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="D54" s="55" t="str">
+        <x:v>TC-077、TC-078</x:v>
+      </x:c>
+      <x:c r="E54" s="55" t="str">
+        <x:v>src/collectors/scanner.ts；src/main/report.ts；src/renderer/overview.tsx；独立合成覆盖区间测试</x:v>
+      </x:c>
+      <x:c r="F54" s="55" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G54" s="55" t="str">
+        <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="155" customHeight="1">
+      <x:c r="A55" s="58" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="B55" s="58" t="str">
+        <x:v>统一异步查询键与页面 CSV 快照</x:v>
+      </x:c>
+      <x:c r="C55" s="58" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="D55" s="58" t="str">
+        <x:v>TC-079</x:v>
+      </x:c>
+      <x:c r="E55" s="58" t="str">
+        <x:v>src/renderer/report.tsx、overview.tsx；src/main/report.ts；CSV IPC；Electron 竞态测试</x:v>
+      </x:c>
+      <x:c r="F55" s="58" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G55" s="58" t="str">
+        <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="155" customHeight="1">
+      <x:c r="A56" s="55" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="B56" s="55" t="str">
+        <x:v>实现概览多维下钻与提供方模型键</x:v>
+      </x:c>
+      <x:c r="C56" s="55" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="D56" s="55" t="str">
+        <x:v>TC-080、TC-081</x:v>
+      </x:c>
+      <x:c r="E56" s="55" t="str">
+        <x:v>src/renderer/overview.tsx、report.tsx、index.tsx；src/main/report.ts；Electron 下钻测试</x:v>
+      </x:c>
+      <x:c r="F56" s="55" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G56" s="55" t="str">
+        <x:v>下钻传递 7/30/90 天、工具/模型/用户/时区/时间桶；面包屑返回保留筛选与焦点，同名模型依提供方+模型分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="155" customHeight="1">
+      <x:c r="A57" s="58" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="B57" s="58" t="str">
+        <x:v>实现角色感知的可跳过首次引导</x:v>
+      </x:c>
+      <x:c r="C57" s="58" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="D57" s="58" t="str">
+        <x:v>TC-082、TC-083</x:v>
+      </x:c>
+      <x:c r="E57" s="58" t="str">
+        <x:v>src/renderer/；src/main/index.ts；独立用户数据与角色 Electron 测试</x:v>
+      </x:c>
+      <x:c r="F57" s="58" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G57" s="58" t="str">
+        <x:v>四步只读真实状态；跳过可重开；viewer 不出现管理员绑定动作，任何状态写入受主进程角色校验。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="155" customHeight="1">
+      <x:c r="A58" s="55" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="B58" s="55" t="str">
+        <x:v>实现分型空状态、诊断行动与扫描进展</x:v>
+      </x:c>
+      <x:c r="C58" s="55" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="D58" s="55" t="str">
+        <x:v>TC-084、TC-085</x:v>
+      </x:c>
+      <x:c r="E58" s="55" t="str">
+        <x:v>src/collectors/scanner.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；状态测试</x:v>
+      </x:c>
+      <x:c r="F58" s="55" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G58" s="55" t="str">
+        <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="155" customHeight="1">
+      <x:c r="A59" s="58" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="B59" s="58" t="str">
+        <x:v>实现来源重绑预览事务与最小审计</x:v>
+      </x:c>
+      <x:c r="C59" s="58" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="D59" s="58" t="str">
+        <x:v>TC-086、TC-087</x:v>
+      </x:c>
+      <x:c r="E59" s="58" t="str">
+        <x:v>src/main/database.ts、index.ts；src/renderer/index.tsx；受控 IPC；事务与 Electron 测试</x:v>
+      </x:c>
+      <x:c r="F59" s="58" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G59" s="58" t="str">
+        <x:v>预览受影响事实数/可见范围，确认后主进程复验权限和版本；事务提交归属及最小审计，失败不改变归属；审计不保存路径/正文。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+需求复核补充：成功绑定与最小审计同事务；业务拒绝可另记结果，DB 不可写时绑定不变且不得声称审计已持久化。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="155" customHeight="1">
+      <x:c r="A60" s="55" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="B60" s="55" t="str">
+        <x:v>分离本机采集与服务上报状态</x:v>
+      </x:c>
+      <x:c r="C60" s="55" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="D60" s="55" t="str">
+        <x:v>TC-088</x:v>
+      </x:c>
+      <x:c r="E60" s="55" t="str">
+        <x:v>src/main/usage-sync.ts、server-connection.ts；src/renderer/overview.tsx、settings.tsx；离线测试</x:v>
+      </x:c>
+      <x:c r="F60" s="55" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G60" s="55" t="str">
+        <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="155" customHeight="1">
+      <x:c r="A61" s="58" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="B61" s="58" t="str">
+        <x:v>补齐键盘 VoiceOver 精确值及文案走查</x:v>
+      </x:c>
+      <x:c r="C61" s="58" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="D61" s="58" t="str">
+        <x:v>TC-089、TC-090、TC-091</x:v>
+      </x:c>
+      <x:c r="E61" s="58" t="str">
+        <x:v>src/renderer/、style.css；Electron 键盘/布局测试；目标 Mac VoiceOver 人工证据</x:v>
+      </x:c>
+      <x:c r="F61" s="58" t="str">
+        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G61" s="58" t="str">
+        <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="165" customHeight="1">
+      <x:c r="A62" s="61" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="B62" s="61" t="str">
+        <x:v>修复本地/遥测重叠选择的身份粒度</x:v>
+      </x:c>
+      <x:c r="C62" s="61" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="D62" s="61" t="str">
+        <x:v>TC-092、TC-093</x:v>
+      </x:c>
+      <x:c r="E62" s="61" t="str">
+        <x:v>src/main/report.ts；usage_facts/source_identities 关联键；src/main/database.ts（如需可追溯冲突状态）；tests/report-overlap.test.ts；scripts/test-cases.mjs</x:v>
+      </x:c>
+      <x:c r="F62" s="61" t="str">
+        <x:v>待开发；故障已在隔离 SQLite 复现</x:v>
+      </x:c>
+      <x:c r="G62" s="61" t="str">
+        <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4720,7 +5608,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–076 已分配；TC-001–075 已注册，TC-076 实际打包 App 自动升级待注册/待验证。TC-034–036 新自动安装目标待验证；TC-028 真实签名、公证及目标 Mac 人工验收仍待验证。</x:v>
+        <x:v>TC-001–093 已分配；TC-001–076 已注册，TC-077–093 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6168,10 +7056,11 @@
         <x:v>只提示匹配的新版本；大小或摘要错误绝不启动安装，临时包清理。</x:v>
       </x:c>
       <x:c r="H39" s="35" t="str">
-        <x:v>历史自动子范围已验证；新增安装前拒绝断言待验证</x:v>
+        <x:v>0.3.5 自动子范围通过；大小/空间等边界待验</x:v>
       </x:c>
       <x:c r="I39" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：旧通过只覆盖当时的版本/架构/摘要与打开路径，不证明辅助进程从未收到坏包；新增断言待实现。</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：旧通过只覆盖当时的版本/架构/摘要与打开路径，不证明辅助进程从未收到坏包；新增断言待实现。
+86a4b5b：文档会话单编号 TC-034 1/1 退出码 0，坏 SHA-256 无安装回调；版本/架构/摘要为合成包断言。</x:v>
       </x:c>
       <x:c r="J39" s="35" t="str">
         <x:v>npm run test:case -- TC-034</x:v>
@@ -6209,10 +7098,11 @@
         <x:v>错误阶段可见且可重试；无损坏临时包，旧版和本机报表继续可用。</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>历史自动子范围已验证；新增故障状态待验证</x:v>
+        <x:v>0.3.5 自动子范围通过；超时/空间不足待验</x:v>
       </x:c>
       <x:c r="I40" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：原停服/重试通过仍有效于旧范围；超时、空间不足、取消和安装前状态/旧版可用性待新增断言。</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：原停服/重试通过仍有效于旧范围；超时、空间不足、取消和安装前状态/旧版可用性待新增断言。
+86a4b5b：文档会话单编号 TC-035 1/1 退出码 0，停服下载失败后重试；未注入超时或磁盘空间不足。</x:v>
       </x:c>
       <x:c r="J40" s="14" t="str">
         <x:v>npm run test:case -- TC-035</x:v>
@@ -6250,19 +7140,21 @@
         <x:v>成功路径自动退出旧版、安装替换并启动新版；失败回滚旧版、保留用户数据、清理挂载/临时文件；权限不足不静默绕过，成功无需 Finder 拖拽。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>旧手动交接部分验证；新自动安装目标待验证</x:v>
+        <x:v>0.3.5 自动控制与回滚单元通过；真实历史旧版/制品故障边界待验</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。</x:v>
+        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。
+86a4b5b：文档会话单编号 TC-036 两项 2/2 退出码 0：下载校验后交自动安装器及启动失败不退出旧版；合成 Bundle/命令覆盖 /Applications/~/Applications 选择、成功、挂载/复制/替换/重启/健康超时及篡改失败回滚。真实旧二进制、只读 DMG 实测及系统权限未由单元证明。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
         <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
       </x:c>
       <x:c r="K41" s="35" t="str">
-        <x:v>tests/next-update.test.ts：test('TC-036 校验后只打开安装包而不替换现有应用')；scripts/verify-local-upgrade.mjs；计划将 TC-036 独立绑定改为自动安装控制/回滚断言，当前绑定仅是历史旧行为。</x:v>
+        <x:v>tests/next-update.test.ts：test('TC-036 校验后只交给自动安装器且启动失败时旧版不退出')；tests/update-install.test.ts：test('TC-036 自动安装目标选择、退出后替换和失败回滚')；两项均在 scripts/test-cases.mjs 绑定。历史 tests/next-update.test.ts 的只打开包断言仅对应旧提交。</x:v>
       </x:c>
       <x:c r="L41" s="35" t="str">
-        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。；新目标的自动替换、重启、权限/回滚未验证；真实制品见待注册 TC-076。</x:v>
+        <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。；新目标的自动替换、重启、权限/回滚未验证；真实制品见待注册 TC-076。
+0.3.5 合成测试覆盖 helper 控制流和路径选择；不等于真实只读 DMG、不可写系统安装或历史 0.3.0/0.3.4 UI 一键升级。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
         <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。；2026-10-03 起旧 Finder 手动安装不再是自动成功路径目标；原缺口与证据作为历史保留。</x:v>
@@ -7201,10 +8093,11 @@
         <x:v>每阶段状态准确，错误可恢复；坏包不打开，旧版可用。</x:v>
       </x:c>
       <x:c r="H64" s="36" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>0.3.5 自动 E2E 子范围通过；真实安装状态边界待验</x:v>
       </x:c>
       <x:c r="I64" s="36" t="str">
-        <x:v>提交 6223c30；2026-10-02 14:57:06 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-059.log</x:v>
+        <x:v>提交 6223c30；2026-10-02 14:57:06 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-059.log
+86a4b5b：文档会话单编号 TC-059 1/1 退出码 0；合成坏摘要显示错误，改清单后可重新检查；不执行真实 DMG 安装。</x:v>
       </x:c>
       <x:c r="J64" s="36" t="str">
         <x:v>npm run test:case -- TC-059</x:v>
@@ -7213,7 +8106,8 @@
         <x:v>tests/e2e/m6-update.spec.ts：test('TC-059 新版坏包提示错误且重试后可重新检查')</x:v>
       </x:c>
       <x:c r="L64" s="36" t="str">
-        <x:v>合成坏摘要拒绝、重查旧版显示最新；真实 DMG 安装未测。</x:v>
+        <x:v>合成坏摘要拒绝、重查旧版显示最新；真实 DMG 安装未测。
+0.3.5 按钮文案改为“下载并更新”；坏包/重新检查 E2E 通过，真实 helper 安装进度与系统权限未覆盖。</x:v>
       </x:c>
       <x:c r="M64" s="36" t="str">
         <x:v>tests/support/test-workspace.ts 为 TC-059 创建 token-test-db-tc059-* / token.sqlite；Electron --token-user-data 指向该目录；结束清理，不读生产库。</x:v>
@@ -7729,16 +8623,16 @@
         <x:v>人工</x:v>
       </x:c>
       <x:c r="F77" s="37" t="str">
-        <x:v>独立测试用户数据、目标 Mac、可控测试目录；先拒绝再手动授予文件权限。</x:v>
+        <x:v>目标 Mac 的独立测试账户和用户数据、可控测试目录：先拒绝文件访问并扫描，再在系统设置授予后重扫，最后撤销并再次重扫。</x:v>
       </x:c>
       <x:c r="G77" s="37" t="str">
-        <x:v>指引与系统设置路径可执行，重新扫描恢复；无权限时不越权且显示未知。</x:v>
+        <x:v>拒绝时来源未知且不越权；授予后恢复可观察用量；撤销后重新显示权限不足/未知，不保留伪零；指引与系统设置路径可执行。</x:v>
       </x:c>
       <x:c r="H77" s="37" t="str">
         <x:v>待验证（人工）</x:v>
       </x:c>
       <x:c r="I77" s="37" t="str">
-        <x:v>已注册人工清单；截至 2026-10-02 尚无目标 Mac 拒绝、授予、撤销文件访问权限的脱敏证据；不得登记 pass。</x:v>
+        <x:v>已注册人工清单；截至 2026-10-02 尚无目标 Mac 拒绝、授予、撤销文件访问权限的脱敏证据；不得登记 pass。 2026-10-03 验收口径补充撤销后的重扫与回到未知；当前仍无目标 Mac 证据。</x:v>
       </x:c>
       <x:c r="J77" s="37" t="str">
         <x:v>npm run test:case -- TC-072</x:v>
@@ -7747,7 +8641,7 @@
         <x:v>scripts/test-cases.mjs：TC-072 人工清单（非自动断言）</x:v>
       </x:c>
       <x:c r="L77" s="37" t="str">
-        <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。</x:v>
+        <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。；新增目标还须实测撤销后的状态/重扫。</x:v>
       </x:c>
       <x:c r="M77" s="37" t="str">
         <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
@@ -7908,22 +8802,721 @@
         <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>待注册、待验证（新自动升级制品目标）</x:v>
+        <x:v>已注册；部分验证（0.3.5 合成旧版打包 App 自动成功链路通过）</x:v>
       </x:c>
       <x:c r="I81" s="52" t="str">
-        <x:v>2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。</x:v>
+        <x:v>2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
+86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="str">
-        <x:v>npm run test:case -- TC-076（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-076（已注册；文档会话 2026-10-03 退出码 0）</x:v>
       </x:c>
       <x:c r="K81" s="52" t="str">
-        <x:v>拟新增以 TC-076 开头的独立打包应用测试函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；脚本在隔离目录用当前包复制并改版本元数据模拟前一补丁版本，再运行旧/新 App 自动升级成功链路。</x:v>
       </x:c>
       <x:c r="L81" s="52" t="str">
-        <x:v>使用隔离可写安装位置、临时用户数据/SQLite、人工合成无正文 Codex/Claude 用量；检查旧进程退出、新版安装/重启和健康、只读 DMG 两条目标选择，故障回滚及清理。真实生产库、系统 /Applications 授权和另一台 Mac 需独立边界说明。</x:v>
+        <x:v>0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
-        <x:v>实施后保存旧/新 DMG SHA-256、macOS/架构、固定代码提交、单编号命令及退出码、脱敏启动/安装/回滚日志；不读取真实会话或生产数据库。真实签名/公证和其他目标 Mac 归 TC-028。</x:v>
+        <x:v>实施后保存旧/新 DMG SHA-256、macOS/架构、固定代码提交、单编号命令及退出码、脱敏启动/安装/回滚日志；不读取真实会话或生产数据库。真实签名/公证和其他目标 Mac 归 TC-028。
+文档会话独立复跑 TC-076 1/1、TC-036 2/2、TC-034/035/059 各 1/1 和 76 入口检查，均退出码 0；开发会话报告 test:gate 52 单元/18 E2E。0.3.5 未签名 DMG 只在当前 Mac 核验；真实签名公证、目标 Mac 属 TC-028。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="185" customHeight="1">
+      <x:c r="A82" s="55" t="str">
+        <x:v>TC-077</x:v>
+      </x:c>
+      <x:c r="B82" s="55" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="C82" s="55" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="D82" s="55" t="str">
+        <x:v>所选范围覆盖真值表</x:v>
+      </x:c>
+      <x:c r="E82" s="55" t="str">
+        <x:v>单元/集成</x:v>
+      </x:c>
+      <x:c r="F82" s="55" t="str">
+        <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。</x:v>
+      </x:c>
+      <x:c r="G82" s="55" t="str">
+        <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。</x:v>
+      </x:c>
+      <x:c r="H82" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I82" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J82" s="55" t="str">
+        <x:v>npm run test:case -- TC-077（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K82" s="55" t="str">
+        <x:v>拟新增以 TC-077 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L82" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M82" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="185" customHeight="1">
+      <x:c r="A83" s="58" t="str">
+        <x:v>TC-078</x:v>
+      </x:c>
+      <x:c r="B83" s="58" t="str">
+        <x:v>REQ-040</x:v>
+      </x:c>
+      <x:c r="C83" s="58" t="str">
+        <x:v>DEV-049</x:v>
+      </x:c>
+      <x:c r="D83" s="58" t="str">
+        <x:v>区间比较可比性门禁</x:v>
+      </x:c>
+      <x:c r="E83" s="58" t="str">
+        <x:v>单元/界面</x:v>
+      </x:c>
+      <x:c r="F83" s="58" t="str">
+        <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。</x:v>
+      </x:c>
+      <x:c r="G83" s="58" t="str">
+        <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。</x:v>
+      </x:c>
+      <x:c r="H83" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I83" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J83" s="58" t="str">
+        <x:v>npm run test:case -- TC-078（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K83" s="58" t="str">
+        <x:v>拟新增以 TC-078 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L83" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M83" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="185" customHeight="1">
+      <x:c r="A84" s="55" t="str">
+        <x:v>TC-079</x:v>
+      </x:c>
+      <x:c r="B84" s="55" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="C84" s="55" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="D84" s="55" t="str">
+        <x:v>异步筛选与 CSV 快照一致</x:v>
+      </x:c>
+      <x:c r="E84" s="55" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F84" s="55" t="str">
+        <x:v>独立库快速切换 A/B 筛选并延迟 A 返回；B 查询完成后再扫描入库，分别在 B 加载、完成及新扫描后导出。</x:v>
+      </x:c>
+      <x:c r="G84" s="55" t="str">
+        <x:v>旧响应不覆盖 B；加载时导出禁用或等待 B；页面和 CSV 的授权查询键、数据库 revision/快照身份及逐事实集合一致；新扫描不能造成旧页面/新 CSV 错配。</x:v>
+      </x:c>
+      <x:c r="H84" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I84" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J84" s="55" t="str">
+        <x:v>npm run test:case -- TC-079（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K84" s="55" t="str">
+        <x:v>拟新增以 TC-079 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L84" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M84" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="185" customHeight="1">
+      <x:c r="A85" s="58" t="str">
+        <x:v>TC-080</x:v>
+      </x:c>
+      <x:c r="B85" s="58" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="C85" s="58" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="D85" s="58" t="str">
+        <x:v>趋势下钻保留 7/30/90 天上下文</x:v>
+      </x:c>
+      <x:c r="E85" s="58" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F85" s="58" t="str">
+        <x:v>选择 7、30、90 天及工具/用户/时区，点击概览趋势桶、翻页后经面包屑返回。</x:v>
+      </x:c>
+      <x:c r="G85" s="58" t="str">
+        <x:v>明细继承全部筛选和桶区间；面包屑返回保留状态，键盘焦点可见。</x:v>
+      </x:c>
+      <x:c r="H85" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I85" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J85" s="58" t="str">
+        <x:v>npm run test:case -- TC-080（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K85" s="58" t="str">
+        <x:v>拟新增以 TC-080 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L85" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M85" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="185" customHeight="1">
+      <x:c r="A86" s="55" t="str">
+        <x:v>TC-081</x:v>
+      </x:c>
+      <x:c r="B86" s="55" t="str">
+        <x:v>REQ-042</x:v>
+      </x:c>
+      <x:c r="C86" s="55" t="str">
+        <x:v>DEV-051</x:v>
+      </x:c>
+      <x:c r="D86" s="55" t="str">
+        <x:v>跨提供方同名模型排行隔离</x:v>
+      </x:c>
+      <x:c r="E86" s="55" t="str">
+        <x:v>单元/Electron</x:v>
+      </x:c>
+      <x:c r="F86" s="55" t="str">
+        <x:v>Codex 和 Claude 构造相同模型名、不同用量，分别选全部/单工具并点击模型排行。</x:v>
+      </x:c>
+      <x:c r="G86" s="55" t="str">
+        <x:v>排行与下钻以提供方+模型分组，事实和合计不混用。</x:v>
+      </x:c>
+      <x:c r="H86" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I86" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J86" s="55" t="str">
+        <x:v>npm run test:case -- TC-081（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K86" s="55" t="str">
+        <x:v>拟新增以 TC-081 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L86" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M86" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="185" customHeight="1">
+      <x:c r="A87" s="58" t="str">
+        <x:v>TC-082</x:v>
+      </x:c>
+      <x:c r="B87" s="58" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="C87" s="58" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D87" s="58" t="str">
+        <x:v>管理员四步引导与跳过恢复</x:v>
+      </x:c>
+      <x:c r="E87" s="58" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F87" s="58" t="str">
+        <x:v>新管理员临时用户数据，依次检测、扫描、归属、首笔用量；中途跳过并重新打开。</x:v>
+      </x:c>
+      <x:c r="G87" s="58" t="str">
+        <x:v>四步状态与真实数据一致，跳过不产生归属/采集副作用，重开可继续。</x:v>
+      </x:c>
+      <x:c r="H87" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I87" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J87" s="58" t="str">
+        <x:v>npm run test:case -- TC-082（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K87" s="58" t="str">
+        <x:v>拟新增以 TC-082 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L87" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M87" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="185" customHeight="1">
+      <x:c r="A88" s="55" t="str">
+        <x:v>TC-083</x:v>
+      </x:c>
+      <x:c r="B88" s="55" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="C88" s="55" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D88" s="55" t="str">
+        <x:v>普通用户引导角色边界</x:v>
+      </x:c>
+      <x:c r="E88" s="55" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F88" s="55" t="str">
+        <x:v>临时管理员/普通用户及授权/未授权来源；普通用户查看引导并尝试归属动作。</x:v>
+      </x:c>
+      <x:c r="G88" s="55" t="str">
+        <x:v>普通用户仅见授权结果和请求管理员指引，不能从 UI/IPC 绑定来源；跳过和首笔用量状态正确。</x:v>
+      </x:c>
+      <x:c r="H88" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I88" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J88" s="55" t="str">
+        <x:v>npm run test:case -- TC-083（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K88" s="55" t="str">
+        <x:v>拟新增以 TC-083 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L88" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M88" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="185" customHeight="1">
+      <x:c r="A89" s="58" t="str">
+        <x:v>TC-084</x:v>
+      </x:c>
+      <x:c r="B89" s="58" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="C89" s="58" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="D89" s="58" t="str">
+        <x:v>六类空状态与可操作下一步</x:v>
+      </x:c>
+      <x:c r="E89" s="58" t="str">
+        <x:v>单元/Electron</x:v>
+      </x:c>
+      <x:c r="F89" s="58" t="str">
+        <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。</x:v>
+      </x:c>
+      <x:c r="G89" s="58" t="str">
+        <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。</x:v>
+      </x:c>
+      <x:c r="H89" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I89" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J89" s="58" t="str">
+        <x:v>npm run test:case -- TC-084（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K89" s="58" t="str">
+        <x:v>拟新增以 TC-084 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L89" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M89" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="185" customHeight="1">
+      <x:c r="A90" s="55" t="str">
+        <x:v>TC-085</x:v>
+      </x:c>
+      <x:c r="B90" s="55" t="str">
+        <x:v>REQ-044</x:v>
+      </x:c>
+      <x:c r="C90" s="55" t="str">
+        <x:v>DEV-053</x:v>
+      </x:c>
+      <x:c r="D90" s="55" t="str">
+        <x:v>长扫描进展与诊断重试</x:v>
+      </x:c>
+      <x:c r="E90" s="55" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F90" s="55" t="str">
+        <x:v>慢速合成扫描、阶段停顿、解析错误及随后修复重试。</x:v>
+      </x:c>
+      <x:c r="G90" s="55" t="str">
+        <x:v>期间持续反馈真实阶段/最近进展，无假百分比或无响应；原因→下一步→重试后状态更新。</x:v>
+      </x:c>
+      <x:c r="H90" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I90" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J90" s="55" t="str">
+        <x:v>npm run test:case -- TC-085（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K90" s="55" t="str">
+        <x:v>拟新增以 TC-085 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L90" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M90" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="185" customHeight="1">
+      <x:c r="A91" s="58" t="str">
+        <x:v>TC-086</x:v>
+      </x:c>
+      <x:c r="B91" s="58" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="C91" s="58" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="D91" s="58" t="str">
+        <x:v>来源重绑预览与确认范围</x:v>
+      </x:c>
+      <x:c r="E91" s="58" t="str">
+        <x:v>集成/Electron</x:v>
+      </x:c>
+      <x:c r="F91" s="58" t="str">
+        <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。</x:v>
+      </x:c>
+      <x:c r="G91" s="58" t="str">
+        <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。</x:v>
+      </x:c>
+      <x:c r="H91" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I91" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J91" s="58" t="str">
+        <x:v>npm run test:case -- TC-086（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K91" s="58" t="str">
+        <x:v>拟新增以 TC-086 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L91" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M91" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="185" customHeight="1">
+      <x:c r="A92" s="55" t="str">
+        <x:v>TC-087</x:v>
+      </x:c>
+      <x:c r="B92" s="55" t="str">
+        <x:v>REQ-045</x:v>
+      </x:c>
+      <x:c r="C92" s="55" t="str">
+        <x:v>DEV-054</x:v>
+      </x:c>
+      <x:c r="D92" s="55" t="str">
+        <x:v>来源重绑失败回滚与最小审计</x:v>
+      </x:c>
+      <x:c r="E92" s="55" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F92" s="55" t="str">
+        <x:v>在业务规则拒绝、事务写入失败及数据库不可写处分别注入异常，检查归属/报表；成功路径检查审计字段。</x:v>
+      </x:c>
+      <x:c r="G92" s="55" t="str">
+        <x:v>成功绑定与最小审计同事务；各失败均保持旧归属/统计。业务拒绝可单记最小结果；数据库不可写时不要求持久审计，但不得误报成功或更改归属；审计无路径/正文。</x:v>
+      </x:c>
+      <x:c r="H92" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I92" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J92" s="55" t="str">
+        <x:v>npm run test:case -- TC-087（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K92" s="55" t="str">
+        <x:v>拟新增以 TC-087 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L92" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M92" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="185" customHeight="1">
+      <x:c r="A93" s="58" t="str">
+        <x:v>TC-088</x:v>
+      </x:c>
+      <x:c r="B93" s="58" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="C93" s="58" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="D93" s="58" t="str">
+        <x:v>本机采集与可选服务状态分离</x:v>
+      </x:c>
+      <x:c r="E93" s="58" t="str">
+        <x:v>集成/Electron</x:v>
+      </x:c>
+      <x:c r="F93" s="58" t="str">
+        <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。</x:v>
+      </x:c>
+      <x:c r="G93" s="58" t="str">
+        <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。</x:v>
+      </x:c>
+      <x:c r="H93" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I93" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J93" s="58" t="str">
+        <x:v>npm run test:case -- TC-088（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K93" s="58" t="str">
+        <x:v>拟新增以 TC-088 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L93" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M93" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="185" customHeight="1">
+      <x:c r="A94" s="55" t="str">
+        <x:v>TC-089</x:v>
+      </x:c>
+      <x:c r="B94" s="55" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="C94" s="55" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D94" s="55" t="str">
+        <x:v>窄窗口键盘与 VoiceOver 主路径</x:v>
+      </x:c>
+      <x:c r="E94" s="55" t="str">
+        <x:v>Electron/目标 Mac 人工</x:v>
+      </x:c>
+      <x:c r="F94" s="55" t="str">
+        <x:v>覆盖窄宽窗口、Tab/Shift+Tab、Enter/Escape、面包屑与主要控件；目标 Mac 用 VoiceOver 逐项朗读。</x:v>
+      </x:c>
+      <x:c r="G94" s="55" t="str">
+        <x:v>无控件遮挡，焦点可见、顺序与动作合理；名称/角色/状态可读，人工证据不由自动布局测试替代。</x:v>
+      </x:c>
+      <x:c r="H94" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I94" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J94" s="55" t="str">
+        <x:v>npm run test:case -- TC-089（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K94" s="55" t="str">
+        <x:v>拟新增以 TC-089 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L94" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M94" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="185" customHeight="1">
+      <x:c r="A95" s="58" t="str">
+        <x:v>TC-090</x:v>
+      </x:c>
+      <x:c r="B95" s="58" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="C95" s="58" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D95" s="58" t="str">
+        <x:v>精确 Token 与覆盖状态非悬浮可读</x:v>
+      </x:c>
+      <x:c r="E95" s="58" t="str">
+        <x:v>Electron 端到端</x:v>
+      </x:c>
+      <x:c r="F95" s="58" t="str">
+        <x:v>无 hover、仅键盘/朗读方式查看概览、趋势、模型排行及明细。</x:v>
+      </x:c>
+      <x:c r="G95" s="58" t="str">
+        <x:v>精确原值与覆盖状态有可见文本或可聚焦可读入口，不仅藏在 title/tooltip。</x:v>
+      </x:c>
+      <x:c r="H95" s="58" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I95" s="58" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J95" s="58" t="str">
+        <x:v>npm run test:case -- TC-090（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K95" s="58" t="str">
+        <x:v>拟新增以 TC-090 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L95" s="58" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M95" s="58" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="185" customHeight="1">
+      <x:c r="A96" s="55" t="str">
+        <x:v>TC-091</x:v>
+      </x:c>
+      <x:c r="B96" s="55" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="C96" s="55" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D96" s="55" t="str">
+        <x:v>关键文案与动作逐状态走查</x:v>
+      </x:c>
+      <x:c r="E96" s="55" t="str">
+        <x:v>Electron/人工</x:v>
+      </x:c>
+      <x:c r="F96" s="55" t="str">
+        <x:v>逐项触发首次引导、六类空状态、诊断重试与自动升级失败状态，核对文案及对应按钮。</x:v>
+      </x:c>
+      <x:c r="G96" s="55" t="str">
+        <x:v>每条文案与实际状态、权限和可执行下一步一致；不把未配置服务、未知覆盖、更新失败写为采集为零或成功。</x:v>
+      </x:c>
+      <x:c r="H96" s="55" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I96" s="55" t="str">
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+      </x:c>
+      <x:c r="J96" s="55" t="str">
+        <x:v>npm run test:case -- TC-091（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K96" s="55" t="str">
+        <x:v>拟新增以 TC-091 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L96" s="55" t="str">
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+      </x:c>
+      <x:c r="M96" s="55" t="str">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="185" customHeight="1">
+      <x:c r="A97" s="61" t="str">
+        <x:v>TC-092</x:v>
+      </x:c>
+      <x:c r="B97" s="61" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="C97" s="61" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="D97" s="61" t="str">
+        <x:v>同会话重复与跨用户独立保留</x:v>
+      </x:c>
+      <x:c r="E97" s="61" t="str">
+        <x:v>单元/集成</x:v>
+      </x:c>
+      <x:c r="F97" s="61" t="str">
+        <x:v>独立临时库构造同提供方同 UTC 日本地用户 A 12 Token、遥测用户 B 99 Token；另造有共同稳定事件 ID 的重复、仅同会话但无共同事件 ID 的候选，以及同用户不同会话。</x:v>
+      </x:c>
+      <x:c r="G97" s="61" t="str">
+        <x:v>A/B 独立事实各按权限保留；可证同事件只计主来源；仅同会话的候选标冲突且不当成已证重复；同日存在本地事实不能整批屏蔽遥测。</x:v>
+      </x:c>
+      <x:c r="H97" s="61" t="str">
+        <x:v>待注册、待验证（已复现缺陷）</x:v>
+      </x:c>
+      <x:c r="I97" s="61" t="str">
+        <x:v>2026-10-03 仅在一次性 SQLite 以现有 selectFacts SQL 复现 owner B 的 99 Token 被误排除；尚无修复代码、独立函数或通过证据。</x:v>
+      </x:c>
+      <x:c r="J97" s="61" t="str">
+        <x:v>npm run test:case -- TC-092（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K97" s="61" t="str">
+        <x:v>拟新增 tests/report-overlap.test.ts 中以 TC-092 开头的独立函数并在 scripts/test-cases.mjs 注册。</x:v>
+      </x:c>
+      <x:c r="L97" s="61" t="str">
+        <x:v>专用临时数据库和无正文合成记录；不得使用生产库。需核对不同用户授权及 Codex/Claude 各自来源身份。</x:v>
+      </x:c>
+      <x:c r="M97" s="61" t="str">
+        <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="185" customHeight="1">
+      <x:c r="A98" s="64" t="str">
+        <x:v>TC-093</x:v>
+      </x:c>
+      <x:c r="B98" s="64" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="C98" s="64" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="D98" s="64" t="str">
+        <x:v>无法关联冲突与三处报表权限一致</x:v>
+      </x:c>
+      <x:c r="E98" s="64" t="str">
+        <x:v>单元/集成</x:v>
+      </x:c>
+      <x:c r="F98" s="64" t="str">
+        <x:v>独立库构造无法确认关联的本地/遥测重叠、多用户筛选、时区边界和 CSV；核对授权汇总、分页明细、导出各状态及数值。</x:v>
+      </x:c>
+      <x:c r="G98" s="64" t="str">
+        <x:v>仅可确认独立事实进入“已确认小计”；授权范围内待核对来源/条数可见，整体显示“总量不可确认”。页面/CSV 不把小计称为总 Token，不静默相加冲突候选；汇总、明细、CSV 同一调和结果，普通用户不见其他用户事实及原始账户/会话 ID。</x:v>
+      </x:c>
+      <x:c r="H98" s="64" t="str">
+        <x:v>待注册、待验证（已复现缺陷）</x:v>
+      </x:c>
+      <x:c r="I98" s="64" t="str">
+        <x:v>2026-10-03 仅在一次性 SQLite 以现有 selectFacts SQL 复现 owner B 的 99 Token 被误排除；尚无修复代码、独立函数或通过证据。</x:v>
+      </x:c>
+      <x:c r="J98" s="64" t="str">
+        <x:v>npm run test:case -- TC-093（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K98" s="64" t="str">
+        <x:v>拟新增 tests/report-overlap.test.ts 中以 TC-093 开头的独立函数并在 scripts/test-cases.mjs 注册。</x:v>
+      </x:c>
+      <x:c r="L98" s="64" t="str">
+        <x:v>专用临时数据库与无正文合成记录；当前本地/遥测没有通用事件 ID，同会话不能证明逐事件重复。不得使用生产库，不得用未知代替已证零，也不得把已确认小计称为完整总量。</x:v>
+      </x:c>
+      <x:c r="M98" s="64" t="str">
+        <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: trace overlap in usage sync snapshots
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ad500fb40c54648"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R925e1fb276eb47b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R916b6bed4c6e402d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf05099fe074d40bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1c15980ab660497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc97db9d1d50c49fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R25a6e9b02d2c49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re7cb970c24414f1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +57,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="30">
+  <x:fills count="31">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -204,6 +204,11 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -216,7 +221,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -392,6 +397,13 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2824,6 +2836,29 @@
         <x:v>待注册、待验证；TC-093 明确已确认小计、待核对来源/条数和总量不可确认的页面/CSV 同口径</x:v>
       </x:c>
     </x:row>
+    <x:row r="100" ht="95" customHeight="1">
+      <x:c r="A100" s="67" t="str">
+        <x:v>REQ-048</x:v>
+      </x:c>
+      <x:c r="B100" s="67" t="str">
+        <x:v>本地与遥测按身份去重及冲突可见</x:v>
+      </x:c>
+      <x:c r="C100" s="67" t="str">
+        <x:v>DEV-057</x:v>
+      </x:c>
+      <x:c r="D100" s="67" t="str">
+        <x:v>修复本地/遥测重叠选择的身份粒度</x:v>
+      </x:c>
+      <x:c r="E100" s="67" t="str">
+        <x:v>TC-094</x:v>
+      </x:c>
+      <x:c r="F100" s="67" t="str">
+        <x:v>服务上报与本地冲突计量同口径</x:v>
+      </x:c>
+      <x:c r="G100" s="67" t="str">
+        <x:v>待注册、待验证；版本 2 快照/旧聚合清除/旧协议拒绝/权限与隐私</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4096,7 +4131,8 @@
         <x:v>本机采集与可选服务上报分离</x:v>
       </x:c>
       <x:c r="C51" s="55" t="str">
-        <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。</x:v>
+        <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。
+若某范围因用量冲突或上报协议不兼容而暂停同步，显示“待核对/未同步”及原因，不归入网络离线、零用量或扫描失败。</x:v>
       </x:c>
       <x:c r="D51" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4148,7 +4184,8 @@
         <x:v>本地与遥测按身份去重及冲突可见</x:v>
       </x:c>
       <x:c r="C53" s="61" t="str">
-        <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。</x:v>
+        <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。
+聚合上报与本机报表、明细、CSV 共用有版本的调和规则及授权范围；版本 2 快照显式表达已确认小计、总量不可确认、待核对来源/条数，不能把小计作为完整 totalTokens 上传。旧服务不兼容时保留待传并明确提示；旧 outbox 重算或阻断，旧聚合在新快照中清除。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4160,10 +4197,11 @@
         <x:v>DEV-057</x:v>
       </x:c>
       <x:c r="G53" s="61" t="str">
-        <x:v>TC-092、TC-093</x:v>
+        <x:v>TC-092、TC-093、TC-094</x:v>
       </x:c>
       <x:c r="H53" s="61" t="str">
-        <x:v>2026-10-03 在一次性 SQLite 内按 src/main/report.ts selectFacts SQL 构造本地 owner A 12 Token、遥测 owner B 99 Token（同日 Codex），实际查询只返回 A；无真实数据。修复前 REQ-009/TC-016 的 UTC 日优先为历史证据。设计 docs/design.md §4.3、§20；开发计划 §13。</x:v>
+        <x:v>2026-10-03 在一次性 SQLite 内按 src/main/report.ts selectFacts SQL 构造本地 owner A 12 Token、遥测 owner B 99 Token（同日 Codex），实际查询只返回 A；无真实数据。修复前 REQ-009/TC-016 的 UTC 日优先为历史证据。设计 docs/design.md §4.3、§20；开发计划 §13。
+2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 有独立同日排除 SQL，src/server/server.ts 的 UsageSnapshot/字段白名单无冲突状态；上报路径尚未动态复现。TC-094 单独验收版本 2 快照、旧协议、旧待传与权限/隐私。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5517,7 +5555,8 @@
         <x:v>待开发；关联新 TC 待注册/待验证</x:v>
       </x:c>
       <x:c r="G60" s="55" t="str">
-        <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="155" customHeight="1">
@@ -5554,16 +5593,18 @@
         <x:v>REQ-048</x:v>
       </x:c>
       <x:c r="D62" s="61" t="str">
-        <x:v>TC-092、TC-093</x:v>
+        <x:v>TC-092、TC-093、TC-094</x:v>
       </x:c>
       <x:c r="E62" s="61" t="str">
-        <x:v>src/main/report.ts；usage_facts/source_identities 关联键；src/main/database.ts（如需可追溯冲突状态）；tests/report-overlap.test.ts；scripts/test-cases.mjs</x:v>
+        <x:v>src/main/report.ts；usage_facts/source_identities 关联键；src/main/database.ts（如需可追溯冲突状态）；tests/report-overlap.test.ts；scripts/test-cases.mjs
+src/main/usage-sync.ts；src/server/server.ts（版本 2 快照校验/存储/查询）；tests/usage-sync-overlap.test.ts；服务隔离集成测试</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
         <x:v>待开发；故障已在隔离 SQLite 复现</x:v>
       </x:c>
       <x:c r="G62" s="61" t="str">
-        <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。</x:v>
+        <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
+上报与报表共用有版本调和结果；版本 2 快照按 owner/提供方/日期/模型声明已确认小计、总量状态与待核对来源/条数，不在旧 totalTokens 冒充完整总量。服务端清除该范围旧完整聚合并存储冲突状态，旧服务拒绝时待传+明示原因，旧 outbox 重算或阻断，恢复后重传且 revision 幂等。仅白名单聚合数据、设备令牌 owner 授权；TC-094 独立验证并回归 TC-088。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5608,7 +5649,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–093 已分配；TC-001–076 已注册，TC-077–093 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
+        <x:v>TC-001–094 已分配；TC-001–076 已注册，TC-077–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -9290,10 +9331,12 @@
         <x:v>集成/Electron</x:v>
       </x:c>
       <x:c r="F93" s="58" t="str">
-        <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。</x:v>
+        <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。
+追加用量冲突与旧上报协议不兼容两类状态，观察本地报表和服务状态。</x:v>
       </x:c>
       <x:c r="G93" s="58" t="str">
-        <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。</x:v>
+        <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。
+本地统计仍可用；冲突/协议不兼容显示“待核对/未同步”及原因，不误写网络离线、零用量或扫描失败；与 TC-094 的服务快照结果一致。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9517,6 +9560,47 @@
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="195" customHeight="1">
+      <x:c r="A99" s="67" t="str">
+        <x:v>TC-094</x:v>
+      </x:c>
+      <x:c r="B99" s="67" t="str">
+        <x:v>REQ-048；关联 REQ-046</x:v>
+      </x:c>
+      <x:c r="C99" s="67" t="str">
+        <x:v>DEV-057；关联 DEV-055</x:v>
+      </x:c>
+      <x:c r="D99" s="67" t="str">
+        <x:v>服务上报与本地冲突计量同口径</x:v>
+      </x:c>
+      <x:c r="E99" s="67" t="str">
+        <x:v>集成</x:v>
+      </x:c>
+      <x:c r="F99" s="67" t="str">
+        <x:v>隔离客户端和服务库构造同日跨 owner 本地/遥测、同 owner 疑似重叠；检查扫描后的版本 2 快照、服务端存储/查询、旧完整聚合清除、旧 outbox、旧协议拒绝/恢复重传、设备令牌范围与 TC-088 状态。</x:v>
+      </x:c>
+      <x:c r="G99" s="67" t="str">
+        <x:v>上报与页面/明细/CSV 共用调和版本和授权事实集；跨 owner 独立保留，冲突只传白名单已确认小计、待核对来源/条数及总量不可确认，旧 totalTokens 不冒充完整总量；旧服务安全拒绝并保留待传，旧 outbox 重算或阻断，恢复后 revision 幂等重传。旧完整聚合被清除，越权 403 不改状态，无原始账户、会话 ID、路径或正文；待核对/未同步不混成网络离线/零/扫描失败。</x:v>
+      </x:c>
+      <x:c r="H99" s="67" t="str">
+        <x:v>待注册、待验证（静态代码核对）</x:v>
+      </x:c>
+      <x:c r="I99" s="67" t="str">
+        <x:v>2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 另有 provider+UTC 日 NOT EXISTS；src/server/server.ts 的 UsageSnapshot/白名单无冲突状态。尚未动态复现、无新协议或通过证据。</x:v>
+      </x:c>
+      <x:c r="J99" s="67" t="str">
+        <x:v>npm run test:case -- TC-094（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K99" s="67" t="str">
+        <x:v>拟新增 tests/usage-sync-overlap.test.ts 中以 TC-094 开头的独立函数、服务隔离集成用例，在 scripts/test-cases.mjs 注册。</x:v>
+      </x:c>
+      <x:c r="L99" s="67" t="str">
+        <x:v>专用临时客户端/服务数据库，无正文合成事实与假设备令牌；不得使用生产库或密钥。版本 2 协议需兼容/迁移设计，旧服务不能静默接收小计。</x:v>
+      </x:c>
+      <x:c r="M99" s="67" t="str">
+        <x:v>实施后保存固定提交、环境、单编号命令/退出码、版本 2 快照白名单/权限/冲突/旧协议/旧 outbox/恢复重传的脱敏证据；关联复跑 TC-038–040、TC-047、TC-074、TC-088。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record query snapshot acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1c15980ab660497f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc97db9d1d50c49fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R25a6e9b02d2c49b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re7cb970c24414f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R09f33937e0fb4620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6d764a3f85ae4178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rbab51ac6aa0f4eb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bfd693c7fee4bd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2511,7 +2511,7 @@
         <x:v>异步筛选与 CSV 快照一致</x:v>
       </x:c>
       <x:c r="G85" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>78b3a3b 已注册；TC-079 单元 1/1 + Electron 1/1 通过；仅 REQ-041 同事实集合查询/导出子范围</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="85" customHeight="1">
@@ -4004,10 +4004,10 @@
         <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。</x:v>
       </x:c>
       <x:c r="D46" s="58" t="str">
-        <x:v>下一轮产品打磨（计划）</x:v>
+        <x:v>下一轮产品打磨（第一批 B 阶段实现）</x:v>
       </x:c>
       <x:c r="E46" s="58" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>已实现；同事实集合查询/导出子范围验证通过（78b3a3b，本机隔离样本）</x:v>
       </x:c>
       <x:c r="F46" s="58" t="str">
         <x:v>DEV-050</x:v>
@@ -4016,7 +4016,8 @@
         <x:v>TC-079</x:v>
       </x:c>
       <x:c r="H46" s="58" t="str">
-        <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="150" customHeight="1">
@@ -5432,14 +5433,15 @@
         <x:v>TC-079</x:v>
       </x:c>
       <x:c r="E55" s="58" t="str">
-        <x:v>src/renderer/report.tsx、overview.tsx；src/main/report.ts；CSV IPC；Electron 竞态测试</x:v>
+        <x:v>src/main/report.ts、index.ts；src/preload/index.ts；src/renderer/report.tsx；src/shared/types.ts；tests/report-snapshot.test.ts、tests/e2e/report-snapshot.spec.ts；scripts/test-cases.mjs、run-test-case.mjs</x:v>
       </x:c>
       <x:c r="F55" s="58" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>已实现；TC-079 单元/Electron 各 1/1 通过（78b3a3b）</x:v>
       </x:c>
       <x:c r="G55" s="58" t="str">
         <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。</x:v>
+需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。
+78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="155" customHeight="1">
@@ -5649,7 +5651,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–094 已分配；TC-001–076 已注册，TC-077–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
+        <x:v>TC-001–094 已分配；TC-001–076 与 TC-079 已注册，TC-077–078、TC-080–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -8959,31 +8961,34 @@
         <x:v>异步筛选与 CSV 快照一致</x:v>
       </x:c>
       <x:c r="E84" s="55" t="str">
-        <x:v>Electron 端到端</x:v>
+        <x:v>单元 + Electron 端到端</x:v>
       </x:c>
       <x:c r="F84" s="55" t="str">
-        <x:v>独立库快速切换 A/B 筛选并延迟 A 返回；B 查询完成后再扫描入库，分别在 B 加载、完成及新扫描后导出。</x:v>
+        <x:v>独立库快速切换 A/B 筛选并延迟 A 返回；B 查询完成后再扫描入库，分别在 B 加载、完成及新扫描后导出。
+已注册单元以专用临时 SQLite 在查询后插入同筛选事实并重算快照；Electron 以延迟 IPC 模拟 A→B 快速切换与过期导出。</x:v>
       </x:c>
       <x:c r="G84" s="55" t="str">
-        <x:v>旧响应不覆盖 B；加载时导出禁用或等待 B；页面和 CSV 的授权查询键、数据库 revision/快照身份及逐事实集合一致；新扫描不能造成旧页面/新 CSV 错配。</x:v>
+        <x:v>旧响应不覆盖 B；加载时导出禁用或等待 B；页面和 CSV 的授权查询键、数据库 revision/快照身份及逐事实集合一致；新扫描不能造成旧页面/新 CSV 错配。
+授权查询和选中事实的 SHA-256 快照 ID；事实变化后旧 ID 拒绝并提示刷新，刷新后 12→111 Token；不同筛选/角色的旧 ID 拒绝。Electron 最终只显示 B，加载中禁用导出，IPC 携带 B 筛选及 B ID。</x:v>
       </x:c>
       <x:c r="H84" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；单元 1/1 + Electron 1/1 通过（78b3a3b，本机隔离样本）</x:v>
       </x:c>
       <x:c r="I84" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
-        <x:v>npm run test:case -- TC-079（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
       </x:c>
       <x:c r="K84" s="55" t="str">
-        <x:v>拟新增以 TC-079 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。</x:v>
       </x:c>
       <x:c r="L84" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>测试为本机隔离临时库/合成事实及 Electron 模拟 IPC；snapshotId 基于查询和选中事实，不是全库 revision。TC-079 不覆盖 REQ-040 历史覆盖、其他打磨需求或打包安装。CSV 原 10 列由 TC-029、公式转义由 TC-023 回归。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="185" customHeight="1">

</xml_diff>

<commit_message>
docs: record overview drilldown and CSV contract
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R09f33937e0fb4620"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6d764a3f85ae4178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rbab51ac6aa0f4eb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R8bfd693c7fee4bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R283918ddae7e4c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R12c85520fda84525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra9242dcfaee149f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rcaef6dfdff674626"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2534,7 +2534,7 @@
         <x:v>趋势下钻保留 7/30/90 天上下文</x:v>
       </x:c>
       <x:c r="G86" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>d18bb47 已注册；TC-080 Electron 1/1 子范围通过；扫描延迟/DST/全键盘待验</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="85" customHeight="1">
@@ -2557,7 +2557,7 @@
         <x:v>跨提供方同名模型排行隔离</x:v>
       </x:c>
       <x:c r="G87" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>d18bb47 已注册；TC-081 Electron 1/1 子范围通过；真实来源/全键盘待验</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="85" customHeight="1">
@@ -3290,7 +3290,8 @@
         <x:v>CSV 导出一致性与安全</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>CSV 使用页面相同筛选和口径，合计一致；表头与数据列一一对应；文本字段防表格公式注入，不导出会话正文。</x:v>
+        <x:v>CSV 使用页面相同筛选和口径，合计一致；表头与数据列一一对应；文本字段防表格公式注入，不导出会话正文。
+CSV 版本契约：无冲突授权查询沿用当前 v1 十列及顺序；含未解决冲突时显式导出 v2 十四列，前十列表头不变，末四列为计量状态、已确认小计 Token、待核对来源、待核对条数。v2 冲突行原数值列留空，不把小计填为总 Token；v2 由 REQ-048/TC-093 待实现。</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
         <x:v>M3</x:v>
@@ -3305,7 +3306,8 @@
         <x:v>TC-022、TC-023、TC-029</x:v>
       </x:c>
       <x:c r="H19" s="10" t="str">
-        <x:v>docs/design.md §5、§6；A9；src/main/report.ts</x:v>
+        <x:v>docs/design.md §5、§6；A9；src/main/report.ts
+当前 d18bb47 的 tests/next-report.test.ts TC-029 与 src/main/report.ts 为 10 列；工作簿旧“9 列”仅为历史描述。本轮不改已通过的 v1 导出或 TC-029 证据；v2 尚未实现。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -4031,10 +4033,10 @@
         <x:v>概览趋势和模型排行可下钻到授权明细；继承近 7/30/90 天、工具、模型、用户、时区和时间桶，返回面包屑保留筛选与可见焦点。同名模型按提供方+模型键区分，不能串数。</x:v>
       </x:c>
       <x:c r="D47" s="55" t="str">
-        <x:v>下一轮产品打磨（计划）</x:v>
+        <x:v>下一轮产品打磨（第一批 C 阶段实现）</x:v>
       </x:c>
       <x:c r="E47" s="55" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>已编码；TC-080/081 隔离 Electron 子范围通过，扫描延迟/全键盘/目标环境待验</x:v>
       </x:c>
       <x:c r="F47" s="55" t="str">
         <x:v>DEV-051</x:v>
@@ -4043,7 +4045,8 @@
         <x:v>TC-080、TC-081</x:v>
       </x:c>
       <x:c r="H47" s="55" t="str">
-        <x:v>承接 REQ-013/028/029/033；同名模型跨提供方使用稳定复合身份。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-013/028/029/033；同名模型跨提供方使用稳定复合身份。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 d18bb47：概览 7/30/90 天按所选 IANA 时区日历、管理员用户/工具/时区筛选、趋势桶与提供方+模型排行下钻、面包屑保留基础筛选及已测来源回焦。今日进行中、各来源分别显示采集时间；比较因同截止证据不足标不可比较；切换筛选显示加载。文档会话独立复跑 TC-080 1/1、TC-081 1/1、TC-054 1/1、TC-021 三绑定及 test:gate（79 入口、53 单元、21 Electron），均退出码 0。用例只造 UTC 当前日期，未造夏令时、扫描延迟量化或完整键盘/VoiceOver。</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="150" customHeight="1">
@@ -4186,7 +4189,8 @@
       </x:c>
       <x:c r="C53" s="61" t="str">
         <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。
-聚合上报与本机报表、明细、CSV 共用有版本的调和规则及授权范围；版本 2 快照显式表达已确认小计、总量不可确认、待核对来源/条数，不能把小计作为完整 totalTokens 上传。旧服务不兼容时保留待传并明确提示；旧 outbox 重算或阻断，旧聚合在新快照中清除。</x:v>
+聚合上报与本机报表、明细、CSV 共用有版本的调和规则及授权范围；版本 2 快照显式表达已确认小计、总量不可确认、待核对来源/条数，不能把小计作为完整 totalTokens 上传。旧服务不兼容时保留待传并明确提示；旧 outbox 重算或阻断，旧聚合在新快照中清除。
+CSV 冲突契约：v2 沿用时间桶+提供方+模型+项目键一组一行，逐组只填该组已确认小计，不在多个冲突行重复全查询小计；冲突行旧数值列空，末四列状态/小计/白名单来源/条数，整份文件显式标 v2。无冲突仍用 v1 十列。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -5458,13 +5462,14 @@
         <x:v>TC-080、TC-081</x:v>
       </x:c>
       <x:c r="E56" s="55" t="str">
-        <x:v>src/renderer/overview.tsx、report.tsx、index.tsx；src/main/report.ts；Electron 下钻测试</x:v>
+        <x:v>src/renderer/overview.tsx、report.tsx、index.tsx、report-navigation.ts；src/main/report.ts、src/shared/types.ts；tests/e2e/overview-drilldown.spec.ts；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F56" s="55" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>已实现；TC-080/081 各 1/1 Electron 子范围通过（d18bb47）</x:v>
       </x:c>
       <x:c r="G56" s="55" t="str">
-        <x:v>下钻传递 7/30/90 天、工具/模型/用户/时区/时间桶；面包屑返回保留筛选与焦点，同名模型依提供方+模型分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>下钻传递 7/30/90 天、工具/模型/用户/时区/时间桶；面包屑返回保留筛选与焦点，同名模型依提供方+模型分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+d18bb47：概览状态保留天数/工具/管理员用户/时区，下钻带完整查询和桶或 provider+model；面包屑清明细条件留基础筛选，回概览恢复来源按钮焦点。TC-080/081/054 各 1/1、TC-021 三绑定、test:gate 79 入口/53 单元/21 Electron 由文档会话独立复跑均退出码 0；扫描延迟、DST 和全键盘/VoiceOver 边界仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="155" customHeight="1">
@@ -5606,7 +5611,8 @@
       </x:c>
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
-上报与报表共用有版本调和结果；版本 2 快照按 owner/提供方/日期/模型声明已确认小计、总量状态与待核对来源/条数，不在旧 totalTokens 冒充完整总量。服务端清除该范围旧完整聚合并存储冲突状态，旧服务拒绝时待传+明示原因，旧 outbox 重算或阻断，恢复后重传且 revision 幂等。仅白名单聚合数据、设备令牌 owner 授权；TC-094 独立验证并回归 TC-088。</x:v>
+上报与报表共用有版本调和结果；版本 2 快照按 owner/提供方/日期/模型声明已确认小计、总量状态与待核对来源/条数，不在旧 totalTokens 冒充完整总量。服务端清除该范围旧完整聚合并存储冲突状态，旧服务拒绝时待传+明示原因，旧 outbox 重算或阻断，恢复后重传且 revision 幂等。仅白名单聚合数据、设备令牌 owner 授权；TC-094 独立验证并回归 TC-088。
+CSV 版本迁移：无冲突 v1 十列不变；含冲突显式 v2 十四列并改导出标签/文件名，前十列同顺序、冲突数值列空、末四列只给逐组小计与状态/来源/条数；旧消费者按表头或文件名识别版本。TC-029 仍验 v1，TC-093 验两个冲突组小计不重复，TC-023/079 扩到两版。现有本地/OTel 无共同事件 ID，TC-092 当前只验不误删/标冲突；同事件正向去重待双方真实具备并证明共同稳定 ID 后再验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5651,7 +5657,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–094 已分配；TC-001–076 与 TC-079 已注册，TC-077–078、TC-080–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
+        <x:v>TC-001–094 已分配；TC-001–076 与 TC-079–081 已注册，TC-077–078、TC-082–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6887,13 +6893,14 @@
         <x:v>导出至少一行数据；用 CSV 解析器逐列核对表头、总 Token 和用量记录数。</x:v>
       </x:c>
       <x:c r="G34" s="9" t="str">
-        <x:v>每行 9 列，列名与数值语义一一对应。</x:v>
+        <x:v>当前 v1 表头与数据行各 10 列，原列顺序不变；第 9 列总 Token 为精确整数，第 10 列用量记录数；旧 9 列为历史阶段。含冲突 v2 十四列由 TC-093 待验。</x:v>
       </x:c>
       <x:c r="H34" s="12" t="str">
         <x:v>已验证（自动）</x:v>
       </x:c>
       <x:c r="I34" s="9" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03 在 d18bb47 只读核对 tests/next-report.test.ts 实际断言 header/row 各 10 列、总 Token 12、记录数 1；旧 96e99be 的 9 列描述仅阶段历史。</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
         <x:v>npm run test:case -- TC-029</x:v>
@@ -6902,10 +6909,11 @@
         <x:v>tests/next-report.test.ts：test('TC-029 CSV 表头和数据列对齐')</x:v>
       </x:c>
       <x:c r="L34" s="30" t="str">
-        <x:v>固定一行 9 列与总 Token/记录数；复杂 CSV 转义另见 TC-023</x:v>
+        <x:v>当前固定一行 10 列与总 Token/记录数，适用于无冲突 v1；复杂 CSV 转义见 TC-023，含冲突 v2 十四列由 TC-093 另验。</x:v>
       </x:c>
       <x:c r="M34" s="9" t="str">
-        <x:v>记录 TC-029 命令、退出码、提交、环境和脱敏日志；覆盖与限制：固定一行 9 列与总 Token/记录数；复杂 CSV 转义另见 TC-023。</x:v>
+        <x:v>记录 TC-029 命令、退出码、提交、环境和脱敏日志；覆盖与限制：固定一行 9 列与总 Token/记录数；复杂 CSV 转义另见 TC-023。
+当前 d18bb47 源码/断言为 v1 十列，不能用于证明未实现的 v2 或冲突状态。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="70" customHeight="1">
@@ -8985,7 +8993,8 @@
         <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。</x:v>
       </x:c>
       <x:c r="L84" s="55" t="str">
-        <x:v>测试为本机隔离临时库/合成事实及 Electron 模拟 IPC；snapshotId 基于查询和选中事实，不是全库 revision。TC-079 不覆盖 REQ-040 历史覆盖、其他打磨需求或打包安装。CSV 原 10 列由 TC-029、公式转义由 TC-023 回归。</x:v>
+        <x:v>测试为本机隔离临时库/合成事实及 Electron 模拟 IPC；snapshotId 基于查询和选中事实，不是全库 revision。TC-079 不覆盖 REQ-040 历史覆盖、其他打磨需求或打包安装。CSV 原 10 列由 TC-029、公式转义由 TC-023 回归。
+DEV-057 后须回归 v1/v2 两版同授权查询快照；当前 TC-079 仅测 v1。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
         <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。</x:v>
@@ -9014,22 +9023,23 @@
         <x:v>明细继承全部筛选和桶区间；面包屑返回保留状态，键盘焦点可见。</x:v>
       </x:c>
       <x:c r="H85" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；隔离 Electron 子范围 1/1 通过（d18bb47）</x:v>
       </x:c>
       <x:c r="I85" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在固定代码 d18bb47 独立运行 npm run test:case -- TC-080，Electron 1/1 退出码 0；受影响 TC-054 1/1、TC-021 三绑定及完整 test:gate（79 入口、53 unit、21 E2E）均退出码 0。</x:v>
       </x:c>
       <x:c r="J85" s="58" t="str">
-        <x:v>npm run test:case -- TC-080（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-080（已注册；文档会话 2026-10-03 退出码 0）</x:v>
       </x:c>
       <x:c r="K85" s="58" t="str">
-        <x:v>拟新增以 TC-080 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：e2e 绑定 tests/e2e/overview-drilldown.spec.ts：TC-080 概览趋势继承时间工具并在面包屑返回后保留筛选与焦点。</x:v>
       </x:c>
       <x:c r="L85" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>UTC 当前日期隔离合成事实覆盖 90/30/7、管理员 viewer、工具/时区、趋势桶、第二页、面包屑筛选与趋势按钮回焦；未造 DST、扫描延迟量化、所有键盘/VoiceOver 路径。</x:v>
       </x:c>
       <x:c r="M85" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>固定代码 d18bb47；macOS 本机隔离合成工作区；单编号 1/1、相关 TC-054 1/1、TC-021 三绑定、test:gate 79 入口/53 unit/21 E2E 均退出码 0。真实生产数据、目标 Mac、完整无障碍边界未验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="185" customHeight="1">
@@ -9046,7 +9056,7 @@
         <x:v>跨提供方同名模型排行隔离</x:v>
       </x:c>
       <x:c r="E86" s="55" t="str">
-        <x:v>单元/Electron</x:v>
+        <x:v>Electron 端到端</x:v>
       </x:c>
       <x:c r="F86" s="55" t="str">
         <x:v>Codex 和 Claude 构造相同模型名、不同用量，分别选全部/单工具并点击模型排行。</x:v>
@@ -9055,22 +9065,23 @@
         <x:v>排行与下钻以提供方+模型分组，事实和合计不混用。</x:v>
       </x:c>
       <x:c r="H86" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；隔离 Electron 子范围 1/1 通过（d18bb47）</x:v>
       </x:c>
       <x:c r="I86" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在固定代码 d18bb47 独立运行 npm run test:case -- TC-081，Electron 1/1 退出码 0；受影响 TC-054 1/1、TC-021 三绑定及完整 test:gate（79 入口、53 unit、21 E2E）均退出码 0。</x:v>
       </x:c>
       <x:c r="J86" s="55" t="str">
-        <x:v>npm run test:case -- TC-081（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-081（已注册；文档会话 2026-10-03 退出码 0）</x:v>
       </x:c>
       <x:c r="K86" s="55" t="str">
-        <x:v>拟新增以 TC-081 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：e2e 绑定 tests/e2e/overview-drilldown.spec.ts：TC-081 同名模型按提供方下钻且筛选选项不混合。</x:v>
       </x:c>
       <x:c r="L86" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>隔离同名模型样本验证 Codex/Claude 选项分离、Claude 下钻 30 Token、排行按钮回焦；未验证真实来源格式、所有键盘/VoiceOver 路径或目标 Mac。</x:v>
       </x:c>
       <x:c r="M86" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>固定代码 d18bb47；macOS 本机隔离合成工作区；单编号 1/1、相关 TC-054 1/1、TC-021 三绑定、test:gate 79 入口/53 unit/21 E2E 均退出码 0。真实生产数据、目标 Mac、完整无障碍边界未验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="185" customHeight="1">
@@ -9543,10 +9554,12 @@
         <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F98" s="64" t="str">
-        <x:v>独立库构造无法确认关联的本地/遥测重叠、多用户筛选、时区边界和 CSV；核对授权汇总、分页明细、导出各状态及数值。</x:v>
+        <x:v>独立库构造无法确认关联的本地/遥测重叠、多用户筛选、时区边界和 CSV；核对授权汇总、分页明细、导出各状态及数值。
+CSV v2 再造两个不同时间桶/提供方/模型/项目组的冲突，各组有不同已确认小计。</x:v>
       </x:c>
       <x:c r="G98" s="64" t="str">
-        <x:v>仅可确认独立事实进入“已确认小计”；授权范围内待核对来源/条数可见，整体显示“总量不可确认”。页面/CSV 不把小计称为总 Token，不静默相加冲突候选；汇总、明细、CSV 同一调和结果，普通用户不见其他用户事实及原始账户/会话 ID。</x:v>
+        <x:v>仅可确认独立事实进入“已确认小计”；授权范围内待核对来源/条数可见，整体显示“总量不可确认”。页面/CSV 不把小计称为总 Token，不静默相加冲突候选；汇总、明细、CSV 同一调和结果，普通用户不见其他用户事实及原始账户/会话 ID。
+无冲突 v1 严格十列；冲突 v2 显式十四列，前十列顺序不变，冲突行第 5–10 列空而非零，末四列逐组状态/小计/来源/条数；两组小计求和等于页面查询级小计，不重复写全查询小计。</x:v>
       </x:c>
       <x:c r="H98" s="64" t="str">
         <x:v>待注册、待验证（已复现缺陷）</x:v>
@@ -9561,7 +9574,8 @@
         <x:v>拟新增 tests/report-overlap.test.ts 中以 TC-093 开头的独立函数并在 scripts/test-cases.mjs 注册。</x:v>
       </x:c>
       <x:c r="L98" s="64" t="str">
-        <x:v>专用临时数据库与无正文合成记录；当前本地/遥测没有通用事件 ID，同会话不能证明逐事件重复。不得使用生产库，不得用未知代替已证零，也不得把已确认小计称为完整总量。</x:v>
+        <x:v>专用临时数据库与无正文合成记录；当前本地/遥测没有通用事件 ID，同会话不能证明逐事件重复。不得使用生产库，不得用未知代替已证零，也不得把已确认小计称为完整总量。
+v2 仍待开发；TC-029 的既有自动通过只覆盖 v1 十列。TC-023 公式转义与 TC-079 同快照约束需扩到 v2。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>

</xml_diff>

<commit_message>
docs: define legacy sync trust boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R283918ddae7e4c39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R12c85520fda84525"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra9242dcfaee149f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rcaef6dfdff674626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R59222fd1add9449e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcd801bdc3f564a11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7bb1e57f98f04c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R4197a2e431dc4d77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2856,7 +2856,7 @@
         <x:v>服务上报与本地冲突计量同口径</x:v>
       </x:c>
       <x:c r="G100" s="67" t="str">
-        <x:v>待注册、待验证；版本 2 快照/旧聚合清除/旧协议拒绝/权限与隐私</x:v>
+        <x:v>待注册、待验证；另验历史 v1 迁移 legacy/unverified、旧客户端追加、授权 v2 重算、同设备 v1 回滚拒绝与 owner 范围</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4190,7 +4190,8 @@
       <x:c r="C53" s="61" t="str">
         <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。
 聚合上报与本机报表、明细、CSV 共用有版本的调和规则及授权范围；版本 2 快照显式表达已确认小计、总量不可确认、待核对来源/条数，不能把小计作为完整 totalTokens 上传。旧服务不兼容时保留待传并明确提示；旧 outbox 重算或阻断，旧聚合在新快照中清除。
-CSV 冲突契约：v2 沿用时间桶+提供方+模型+项目键一组一行，逐组只填该组已确认小计，不在多个冲突行重复全查询小计；冲突行旧数值列空，末四列状态/小计/白名单来源/条数，整份文件显式标 v2。无冲突仍用 v1 十列。</x:v>
+CSV 冲突契约：v2 沿用时间桶+提供方+模型+项目键一组一行，逐组只填该组已确认小计，不在多个冲突行重复全查询小计；冲突行旧数值列空，末四列状态/小计/白名单来源/条数，整份文件显式标 v2。无冲突仍用 v1 十列。
+服务 v2 旧值：迁移历史 v1 聚合/覆盖先标 legacy/unverified，旧客户端继续上报也不得标 confirmed；同设备成功接收 v2 后拒绝任何 v1（包括更高 revision），且旧聚合/覆盖/状态/修订不变。只有授权 v2 当前事实重算后按证据变为 confirmed 或 uncertain。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4206,7 +4207,8 @@
       </x:c>
       <x:c r="H53" s="61" t="str">
         <x:v>2026-10-03 在一次性 SQLite 内按 src/main/report.ts selectFacts SQL 构造本地 owner A 12 Token、遥测 owner B 99 Token（同日 Codex），实际查询只返回 A；无真实数据。修复前 REQ-009/TC-016 的 UTC 日优先为历史证据。设计 docs/design.md §4.3、§20；开发计划 §13。
-2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 有独立同日排除 SQL，src/server/server.ts 的 UsageSnapshot/字段白名单无冲突状态；上报路径尚未动态复现。TC-094 单独验收版本 2 快照、旧协议、旧待传与权限/隐私。</x:v>
+2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 有独立同日排除 SQL，src/server/server.ts 的 UsageSnapshot/字段白名单无冲突状态；上报路径尚未动态复现。TC-094 单独验收版本 2 快照、旧协议、旧待传与权限/隐私。
+2026-10-03 旧 v1 服务聚合由已知同日误排除规则生成，不得自动视为完整；TC-094 增加历史库迁移与 v1 回滚验收。当前仅设计，尚无实现/通过证据。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5612,7 +5614,8 @@
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
 上报与报表共用有版本调和结果；版本 2 快照按 owner/提供方/日期/模型声明已确认小计、总量状态与待核对来源/条数，不在旧 totalTokens 冒充完整总量。服务端清除该范围旧完整聚合并存储冲突状态，旧服务拒绝时待传+明示原因，旧 outbox 重算或阻断，恢复后重传且 revision 幂等。仅白名单聚合数据、设备令牌 owner 授权；TC-094 独立验证并回归 TC-088。
-CSV 版本迁移：无冲突 v1 十列不变；含冲突显式 v2 十四列并改导出标签/文件名，前十列同顺序、冲突数值列空、末四列只给逐组小计与状态/来源/条数；旧消费者按表头或文件名识别版本。TC-029 仍验 v1，TC-093 验两个冲突组小计不重复，TC-023/079 扩到两版。现有本地/OTel 无共同事件 ID，TC-092 当前只验不误删/标冲突；同事件正向去重待双方真实具备并证明共同稳定 ID 后再验。</x:v>
+CSV 版本迁移：无冲突 v1 十列不变；含冲突显式 v2 十四列并改导出标签/文件名，前十列同顺序、冲突数值列空、末四列只给逐组小计与状态/来源/条数；旧消费者按表头或文件名识别版本。TC-029 仍验 v1，TC-093 验两个冲突组小计不重复，TC-023/079 扩到两版。现有本地/OTel 无共同事件 ID，TC-092 当前只验不误删/标冲突；同事件正向去重待双方真实具备并证明共同稳定 ID 后再验。
+升级服务先为旧 aggregates/source_coverage 标 legacy/unverified 并保留原值；同设备未收 v2 前若仍收 v1，也只能维持未核实。首次授权 v2 原子替换后，可证范围才 confirmed，冲突范围 uncertain；此后任何 v1（含更高 revision）须拒绝且聚合、覆盖、状态和 device_revisions 均不变。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9598,10 +9601,12 @@
         <x:v>集成</x:v>
       </x:c>
       <x:c r="F99" s="67" t="str">
-        <x:v>隔离客户端和服务库构造同日跨 owner 本地/遥测、同 owner 疑似重叠；检查扫描后的版本 2 快照、服务端存储/查询、旧完整聚合清除、旧 outbox、旧协议拒绝/恢复重传、设备令牌范围与 TC-088 状态。</x:v>
+        <x:v>隔离客户端和服务库构造同日跨 owner 本地/遥测、同 owner 疑似重叠；检查扫描后的版本 2 快照、服务端存储/查询、旧完整聚合清除、旧 outbox、旧协议拒绝/恢复重传、设备令牌范围与 TC-088 状态。
+预置有跨 owner 误排除风险的 v1 历史 aggregates/coverage，升级服务后依次发送旧客户端 v1 追加、授权 v2 重算、同设备更高 revision 的 v1 回滚，并另测越权 owner。</x:v>
       </x:c>
       <x:c r="G99" s="67" t="str">
-        <x:v>上报与页面/明细/CSV 共用调和版本和授权事实集；跨 owner 独立保留，冲突只传白名单已确认小计、待核对来源/条数及总量不可确认，旧 totalTokens 不冒充完整总量；旧服务安全拒绝并保留待传，旧 outbox 重算或阻断，恢复后 revision 幂等重传。旧完整聚合被清除，越权 403 不改状态，无原始账户、会话 ID、路径或正文；待核对/未同步不混成网络离线/零/扫描失败。</x:v>
+        <x:v>上报与页面/明细/CSV 共用调和版本和授权事实集；跨 owner 独立保留，冲突只传白名单已确认小计、待核对来源/条数及总量不可确认，旧 totalTokens 不冒充完整总量；旧服务安全拒绝并保留待传，旧 outbox 重算或阻断，恢复后 revision 幂等重传。旧完整聚合被清除，越权 403 不改状态，无原始账户、会话 ID、路径或正文；待核对/未同步不混成网络离线/零/扫描失败。
+迁移及旧客户端追加均显示 legacy/unverified，不把旧数值当完整；v2 原子替换后仅可证范围 confirmed、冲突 uncertain；收过 v2 的设备拒绝所有 v1，拒绝前后 aggregates/coverage/状态/revision 完全相同，跨 owner 授权仍拒绝。</x:v>
       </x:c>
       <x:c r="H99" s="67" t="str">
         <x:v>待注册、待验证（静态代码核对）</x:v>
@@ -9616,7 +9621,8 @@
         <x:v>拟新增 tests/usage-sync-overlap.test.ts 中以 TC-094 开头的独立函数、服务隔离集成用例，在 scripts/test-cases.mjs 注册。</x:v>
       </x:c>
       <x:c r="L99" s="67" t="str">
-        <x:v>专用临时客户端/服务数据库，无正文合成事实与假设备令牌；不得使用生产库或密钥。版本 2 协议需兼容/迁移设计，旧服务不能静默接收小计。</x:v>
+        <x:v>专用临时客户端/服务数据库，无正文合成事实与假设备令牌；不得使用生产库或密钥。版本 2 协议需兼容/迁移设计，旧服务不能静默接收小计。
+当前 v1 数据已知可能跨 owner 误排除；TC-094 必须用历史库实测降级边界，不能仅测新 v2 干净库，也不能从旧 200/ready 推断完整。当前尚未注册或执行。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>实施后保存固定提交、环境、单编号命令/退出码、版本 2 快照白名单/权限/冲突/旧协议/旧 outbox/恢复重传的脱敏证据；关联复跑 TC-038–040、TC-047、TC-074、TC-088。</x:v>

</xml_diff>

<commit_message>
docs: scope viewer coverage and diagnostics by owner
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R59222fd1add9449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcd801bdc3f564a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7bb1e57f98f04c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R4197a2e431dc4d77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra2f5478c90d54e7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R98d6df3bc08e43fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf90ac158c32d4d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R2a97fc786c6f4601"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2833,7 +2833,7 @@
         <x:v>无法关联冲突与三处报表权限一致</x:v>
       </x:c>
       <x:c r="G99" s="64" t="str">
-        <x:v>待注册、待验证；TC-093 明确已确认小计、待核对来源/条数和总量不可确认的页面/CSV 同口径</x:v>
+        <x:v>待注册、待验证；TC-093 验冲突计量及 viewer 状态/报表覆盖/诊断 IPC、概览与诊断 UI、可选反馈附件的双 owner 隔离和未知语义</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="95" customHeight="1">
@@ -4191,7 +4191,9 @@
         <x:v>先按授权 owner 筛选。可由共同稳定事件身份等证据证明的本地/遥测重复只计主来源；同日不同用户或明确不同会话的独立事实保留。现有两路没有通用事件 ID，仅同会话不足以证明逐事件重复或完整覆盖；疑似重叠保留原始明细并标冲突。只将可确认独立事实计入“已确认小计”，另列授权范围内待核对事实的来源/条数并显示“总量不可确认”；页面和 CSV 不把小计称为总 Token，不静默相加或整日排除。普通用户不可见其他用户事实、原始账户或会话 ID。
 聚合上报与本机报表、明细、CSV 共用有版本的调和规则及授权范围；版本 2 快照显式表达已确认小计、总量不可确认、待核对来源/条数，不能把小计作为完整 totalTokens 上传。旧服务不兼容时保留待传并明确提示；旧 outbox 重算或阻断，旧聚合在新快照中清除。
 CSV 冲突契约：v2 沿用时间桶+提供方+模型+项目键一组一行，逐组只填该组已确认小计，不在多个冲突行重复全查询小计；冲突行旧数值列空，末四列状态/小计/白名单来源/条数，整份文件显式标 v2。无冲突仍用 v1 十列。
-服务 v2 旧值：迁移历史 v1 聚合/覆盖先标 legacy/unverified，旧客户端继续上报也不得标 confirmed；同设备成功接收 v2 后拒绝任何 v1（包括更高 revision），且旧聚合/覆盖/状态/修订不变。只有授权 v2 当前事实重算后按证据变为 confirmed 或 uncertain。</x:v>
+服务 v2 旧值：迁移历史 v1 聚合/覆盖先标 legacy/unverified，旧客户端继续上报也不得标 confirmed；同设备成功接收 v2 后拒绝任何 v1（包括更高 revision），且旧聚合/覆盖/状态/修订不变。只有授权 v2 当前事实重算后按证据变为 confirmed 或 uncertain。
+viewer 来源状态隔离：报表 coverage、sources:statuses 和概览/报表来源信息只能含当前登录用户及授权查询范围可证明归属的记录数、扫描/遥测时间、状态和诊断细节；不能返回其他 owner 的全局元数据。来源级证据无法归属时显示未知/未覆盖及空值，不得伪装成真零；管理员全局范围须明确。
+同一授权边界覆盖 sources:diagnostics 与 feedback:submit 可选诊断附件；按 provider 筛选不能代表按 owner 隔离。viewer 可得通用修复建议和本人可证状态，跨 owner 位置、原因、各类计数与时间须过滤或未知；勾选附件不扩大读取权限。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4208,7 +4210,9 @@
       <x:c r="H53" s="61" t="str">
         <x:v>2026-10-03 在一次性 SQLite 内按 src/main/report.ts selectFacts SQL 构造本地 owner A 12 Token、遥测 owner B 99 Token（同日 Codex），实际查询只返回 A；无真实数据。修复前 REQ-009/TC-016 的 UTC 日优先为历史证据。设计 docs/design.md §4.3、§20；开发计划 §13。
 2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 有独立同日排除 SQL，src/server/server.ts 的 UsageSnapshot/字段白名单无冲突状态；上报路径尚未动态复现。TC-094 单独验收版本 2 快照、旧协议、旧待传与权限/隐私。
-2026-10-03 旧 v1 服务聚合由已知同日误排除规则生成，不得自动视为完整；TC-094 增加历史库迁移与 v1 回滚验收。当前仅设计，尚无实现/通过证据。</x:v>
+2026-10-03 旧 v1 服务聚合由已知同日误排除规则生成，不得自动视为完整；TC-094 增加历史库迁移与 v1 回滚验收。当前仅设计，尚无实现/通过证据。
+2026-10-03 静态审查发现 sources:statuses 与报表 coverage 返回全局 scanner.statuses()，概览/报表显示全局计数与采集时间；TC-093 增双 owner IPC/UI 验收。尚未动态复现、修复或通过。
+同日补充静态发现：诊断 IPC/可选反馈附件按 provider 保留整条全局诊断，TC-093 扩至两入口；尚无动态验证。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5606,7 +5610,9 @@
       </x:c>
       <x:c r="E62" s="61" t="str">
         <x:v>src/main/report.ts；usage_facts/source_identities 关联键；src/main/database.ts（如需可追溯冲突状态）；tests/report-overlap.test.ts；scripts/test-cases.mjs
-src/main/usage-sync.ts；src/server/server.ts（版本 2 快照校验/存储/查询）；tests/usage-sync-overlap.test.ts；服务隔离集成测试</x:v>
+src/main/usage-sync.ts；src/server/server.ts（版本 2 快照校验/存储/查询）；tests/usage-sync-overlap.test.ts；服务隔离集成测试
+viewer 元数据路径：src/main/index.ts 的 sources:statuses、src/main/report.ts 的 coverage、src/renderer/overview.tsx 与 report.tsx；src/shared/types.ts 的 SourceStatus；对应 IPC/UI 测试。
+另查 src/main/index.ts 的 sources:diagnostics 与 feedback:submit、src/renderer/diagnostics.tsx、src/shared/types.ts 的 CollectionDiagnostic。</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
         <x:v>待开发；故障已在隔离 SQLite 复现</x:v>
@@ -5615,7 +5621,9 @@
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
 上报与报表共用有版本调和结果；版本 2 快照按 owner/提供方/日期/模型声明已确认小计、总量状态与待核对来源/条数，不在旧 totalTokens 冒充完整总量。服务端清除该范围旧完整聚合并存储冲突状态，旧服务拒绝时待传+明示原因，旧 outbox 重算或阻断，恢复后重传且 revision 幂等。仅白名单聚合数据、设备令牌 owner 授权；TC-094 独立验证并回归 TC-088。
 CSV 版本迁移：无冲突 v1 十列不变；含冲突显式 v2 十四列并改导出标签/文件名，前十列同顺序、冲突数值列空、末四列只给逐组小计与状态/来源/条数；旧消费者按表头或文件名识别版本。TC-029 仍验 v1，TC-093 验两个冲突组小计不重复，TC-023/079 扩到两版。现有本地/OTel 无共同事件 ID，TC-092 当前只验不误删/标冲突；同事件正向去重待双方真实具备并证明共同稳定 ID 后再验。
-升级服务先为旧 aggregates/source_coverage 标 legacy/unverified 并保留原值；同设备未收 v2 前若仍收 v1，也只能维持未核实。首次授权 v2 原子替换后，可证范围才 confirmed，冲突范围 uncertain；此后任何 v1（含更高 revision）须拒绝且聚合、覆盖、状态和 device_revisions 均不变。</x:v>
+升级服务先为旧 aggregates/source_coverage 标 legacy/unverified 并保留原值；同设备未收 v2 前若仍收 v1，也只能维持未核实。首次授权 v2 原子替换后，可证范围才 confirmed，冲突范围 uncertain；此后任何 v1（含更高 revision）须拒绝且聚合、覆盖、状态和 device_revisions 均不变。
+在主进程按登录态/授权查询范围构造 viewer 来源状态；不能仅前端隐藏全局 fileCount/factCount/telemetryFactCount、lastTelemetry/lastScan、detail 或由全局状态推导真零。无法证明 owner 归属则未知/空值；对齐来源状态 IPC、报表 coverage 与概览/报表 UI，管理员全局视图标明范围。TC-093 双 owner IPC/UI 回归，关联 TC-021/045/046/077/078。当前仅静态审查。
+诊断 IPC 和可选反馈附件必须复用按 owner 授权后的视图；通用 suggestion 可留，跨 owner location/reason、文件/事实/未归属/异常计数、lastScan/lastSuccess 不能经 IPC、UI 或反馈载荷泄露。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9558,11 +9566,15 @@
       </x:c>
       <x:c r="F98" s="64" t="str">
         <x:v>独立库构造无法确认关联的本地/遥测重叠、多用户筛选、时区边界和 CSV；核对授权汇总、分页明细、导出各状态及数值。
-CSV v2 再造两个不同时间桶/提供方/模型/项目组的冲突，各组有不同已确认小计。</x:v>
+CSV v2 再造两个不同时间桶/提供方/模型/项目组的冲突，各组有不同已确认小计。
+再造 owner A/B 来源事实、不同记录数及采集/遥测时间；以 viewer A 登录直调 sources:statuses 与报表 coverage，核对概览来源卡、最近采集时间、报表覆盖条；比较管理员授权全局视图并直调 viewer sources:scan。
+同样直调 viewer A 的 sources:diagnostics、核诊断页；在隔离反馈服务/测试桩中勾选 attachDiagnostics，检查最终提交载荷是否含 B 独有标记。</x:v>
       </x:c>
       <x:c r="G98" s="64" t="str">
         <x:v>仅可确认独立事实进入“已确认小计”；授权范围内待核对来源/条数可见，整体显示“总量不可确认”。页面/CSV 不把小计称为总 Token，不静默相加冲突候选；汇总、明细、CSV 同一调和结果，普通用户不见其他用户事实及原始账户/会话 ID。
-无冲突 v1 严格十列；冲突 v2 显式十四列，前十列顺序不变，冲突行第 5–10 列空而非零，末四列逐组状态/小计/来源/条数；两组小计求和等于页面查询级小计，不重复写全查询小计。</x:v>
+无冲突 v1 严格十列；冲突 v2 显式十四列，前十列顺序不变，冲突行第 5–10 列空而非零，末四列逐组状态/小计/来源/条数；两组小计求和等于页面查询级小计，不重复写全查询小计。
+viewer A 的 IPC 和 UI 均不得出现 B 独有的文件/事实/遥测计数、采集/遥测时间、诊断细节或由 B 状态推断的真零；来源级证据无法证明属 A 时返回未知/空值而非 0。管理员全局范围明确，viewer 直调 sources:scan 拒绝。
+只按 provider 相同不得泄露 B 的文件/事实/未归属/异常计数、位置/原因、扫描/成功时间；通用指引和 A 可证字段可保留，无法归属字段未知/省略，反馈附件不增加权限。</x:v>
       </x:c>
       <x:c r="H98" s="64" t="str">
         <x:v>待注册、待验证（已复现缺陷）</x:v>
@@ -9578,7 +9590,9 @@
       </x:c>
       <x:c r="L98" s="64" t="str">
         <x:v>专用临时数据库与无正文合成记录；当前本地/遥测没有通用事件 ID，同会话不能证明逐事件重复。不得使用生产库，不得用未知代替已证零，也不得把已确认小计称为完整总量。
-v2 仍待开发；TC-029 的既有自动通过只覆盖 v1 十列。TC-023 公式转义与 TC-079 同快照约束需扩到 v2。</x:v>
+v2 仍待开发；TC-029 的既有自动通过只覆盖 v1 十列。TC-023 公式转义与 TC-079 同快照约束需扩到 v2。
+静态审查发现全局状态暴露路径；尚未动态复现或验收。验收必须在主进程 IPC 层断言，不以 UI 隐藏代替。
+反馈载荷用隔离接收器或桩验收，不提交真实反馈；不能只看诊断 UI，必须核主进程 IPC/附件。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>

</xml_diff>

<commit_message>
docs: define admin filtered coverage evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra2f5478c90d54e7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R98d6df3bc08e43fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf90ac158c32d4d09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R2a97fc786c6f4601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rfeb9c85e587c4284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R3c595ae9a08c4430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R17a172f9be244a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra26cbfe14e5c4111"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2465,7 +2465,7 @@
         <x:v>所选范围覆盖真值表</x:v>
       </x:c>
       <x:c r="G83" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；管理员双 owner+未归属，API/UI 按所选范围判未知/部分/真零；全局诊断单独标识</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="85" customHeight="1">
@@ -2488,7 +2488,7 @@
         <x:v>区间比较可比性门禁</x:v>
       </x:c>
       <x:c r="G84" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；管理员筛选范围两期同截止且完整才比较，全局 ready/其他 owner 时间不得补证</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -3977,7 +3977,8 @@
         <x:v>所选范围的可证覆盖与可比区间</x:v>
       </x:c>
       <x:c r="C45" s="55" t="str">
-        <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。</x:v>
+        <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。
+管理员选具体用户或“未归属”后，来源卡、报表 coverage、真零与比较只按该用户+所选工具/IANA 时区/区间的可证覆盖判定。全局 ready/计数/最近扫描时间只能另标“全局”诊断，不能补全选中范围；全局 ready 而所选用户空且缺证据时为未知/部分，不是已确认零。</x:v>
       </x:c>
       <x:c r="D45" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -3992,7 +3993,8 @@
         <x:v>TC-077、TC-078</x:v>
       </x:c>
       <x:c r="H45" s="55" t="str">
-        <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -5420,13 +5422,15 @@
         <x:v>TC-077、TC-078</x:v>
       </x:c>
       <x:c r="E54" s="55" t="str">
-        <x:v>src/collectors/scanner.ts；src/main/report.ts；src/renderer/overview.tsx；独立合成覆盖区间测试</x:v>
+        <x:v>src/collectors/scanner.ts；src/main/report.ts；src/renderer/overview.tsx；独立合成覆盖区间测试
+另核 src/renderer/report.tsx 的 coverage 与 src/main/index.ts 的授权报表 IPC；全局诊断若保留需显式标范围。</x:v>
       </x:c>
       <x:c r="F54" s="55" t="str">
         <x:v>待开发；关联新 TC 待注册/待验证</x:v>
       </x:c>
       <x:c r="G54" s="55" t="str">
-        <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -8901,10 +8905,12 @@
         <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F82" s="55" t="str">
-        <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。</x:v>
+        <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。
+构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
-        <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。</x:v>
+        <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
+B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -8919,7 +8925,8 @@
         <x:v>拟新增以 TC-077 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L82" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
@@ -8942,10 +8949,12 @@
         <x:v>单元/界面</x:v>
       </x:c>
       <x:c r="F83" s="58" t="str">
-        <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。</x:v>
+        <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。
+管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。</x:v>
       </x:c>
       <x:c r="G83" s="58" t="str">
-        <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。</x:v>
+        <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。
+全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -8960,7 +8969,8 @@
         <x:v>拟新增以 TC-078 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L83" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。</x:v>
       </x:c>
       <x:c r="M83" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: record overlap reconciliation implementation and v2 regression evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rfeb9c85e587c4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R3c595ae9a08c4430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R17a172f9be244a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra26cbfe14e5c4111"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R9a3bdaebd38d4689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R4a66f777b12142ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R06c103b20abd41d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb8bb3a32755242f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2810,7 +2810,7 @@
         <x:v>同会话重复与跨用户独立保留</x:v>
       </x:c>
       <x:c r="G98" s="61" t="str">
-        <x:v>待注册、待验证（缺陷已复现）</x:v>
+        <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="90" customHeight="1">
@@ -2833,7 +2833,7 @@
         <x:v>无法关联冲突与三处报表权限一致</x:v>
       </x:c>
       <x:c r="G99" s="64" t="str">
-        <x:v>待注册、待验证；TC-093 验冲突计量及 viewer 状态/报表覆盖/诊断 IPC、概览与诊断 UI、可选反馈附件的双 owner 隔离和未知语义</x:v>
+        <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="95" customHeight="1">
@@ -2856,7 +2856,7 @@
         <x:v>服务上报与本地冲突计量同口径</x:v>
       </x:c>
       <x:c r="G100" s="67" t="str">
-        <x:v>待注册、待验证；另验历史 v1 迁移 legacy/unverified、旧客户端追加、授权 v2 重算、同设备 v1 回滚拒绝与 owner 范围</x:v>
+        <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3307,7 +3307,8 @@
       </x:c>
       <x:c r="H19" s="10" t="str">
         <x:v>docs/design.md §5、§6；A9；src/main/report.ts
-当前 d18bb47 的 tests/next-report.test.ts TC-029 与 src/main/report.ts 为 10 列；工作簿旧“9 列”仅为历史描述。本轮不改已通过的 v1 导出或 TC-029 证据；v2 尚未实现。</x:v>
+当前 d18bb47 的 tests/next-report.test.ts TC-029 与 src/main/report.ts 为 10 列；工作簿旧“9 列”仅为历史描述。本轮不改已通过的 v1 导出或 TC-029 证据；v2 尚未实现。
+47b03d5：TC-023 新增冲突 v2 十四列项目/模型公式转义独立单元绑定，文档会话单编号两项及 gate 57 单元/22 Electron/82 入口均通过；无冲突 v1 十列保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -4021,7 +4022,8 @@
       </x:c>
       <x:c r="H46" s="58" t="str">
         <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
-2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。</x:v>
+2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。
+47b03d5：TC-079 追加 v1→冲突 v2、扫描入库后旧 snapshotId 拒绝及刷新小计 99→104；文档会话单元+Electron 与 gate 独立通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="150" customHeight="1">
@@ -4201,7 +4203,7 @@
         <x:v>缺陷修复（已复现）</x:v>
       </x:c>
       <x:c r="E53" s="61" t="str">
-        <x:v>待修复/待验证</x:v>
+        <x:v>已编码；TC-092–094 自动子范围通过，正向精确去重/TC-093 补断言/生产迁移待验证</x:v>
       </x:c>
       <x:c r="F53" s="61" t="str">
         <x:v>DEV-057</x:v>
@@ -4214,7 +4216,9 @@
 2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 有独立同日排除 SQL，src/server/server.ts 的 UsageSnapshot/字段白名单无冲突状态；上报路径尚未动态复现。TC-094 单独验收版本 2 快照、旧协议、旧待传与权限/隐私。
 2026-10-03 旧 v1 服务聚合由已知同日误排除规则生成，不得自动视为完整；TC-094 增加历史库迁移与 v1 回滚验收。当前仅设计，尚无实现/通过证据。
 2026-10-03 静态审查发现 sources:statuses 与报表 coverage 返回全局 scanner.statuses()，概览/报表显示全局计数与采集时间；TC-093 增双 owner IPC/UI 验收。尚未动态复现、修复或通过。
-同日补充静态发现：诊断 IPC/可选反馈附件按 provider 保留整条全局诊断，TC-093 扩至两入口；尚无动态验证。</x:v>
+同日补充静态发现：诊断 IPC/可选反馈附件按 provider 保留整条全局诊断，TC-093 扩至两入口；尚无动态验证。
+2026-10-03 代码 8157e2d：授权 owner 调和替代按日整批排除；冲突仅显示已确认小计，明细保留待核对，CSV v1 十列/v2 十四列，服务 accountingVersion 2、旧 v1 状态 legacy_unknown，viewer 来源状态/诊断/附件按本人或未知。文档会话独立 test:gate 82 入口、56 单元、22 Electron 通过；TC-092–094 单编号通过。未证共同事件 ID 正向去重、TC-093 的概览 B 值/sources:scan 直调、v2 TC-023/079、真实生产库迁移和旧服务真实版本。REQ-040 管理员筛选覆盖独立待验。
+47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5455,7 +5459,8 @@
       <x:c r="G55" s="58" t="str">
         <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。
-78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。</x:v>
+78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。
+47b03d5：TC-079 原单元新增冲突 v2 快照身份回归：新增遥测使旧 ID 拒绝、刷新小计 99，继续新增事实又拒绝，刷新小计 104；单编号 unit/Electron 与完整门禁独立通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="155" customHeight="1">
@@ -5613,13 +5618,10 @@
         <x:v>TC-092、TC-093、TC-094</x:v>
       </x:c>
       <x:c r="E62" s="61" t="str">
-        <x:v>src/main/report.ts；usage_facts/source_identities 关联键；src/main/database.ts（如需可追溯冲突状态）；tests/report-overlap.test.ts；scripts/test-cases.mjs
-src/main/usage-sync.ts；src/server/server.ts（版本 2 快照校验/存储/查询）；tests/usage-sync-overlap.test.ts；服务隔离集成测试
-viewer 元数据路径：src/main/index.ts 的 sources:statuses、src/main/report.ts 的 coverage、src/renderer/overview.tsx 与 report.tsx；src/shared/types.ts 的 SourceStatus；对应 IPC/UI 测试。
-另查 src/main/index.ts 的 sources:diagnostics 与 feedback:submit、src/renderer/diagnostics.tsx、src/shared/types.ts 的 CollectionDiagnostic。</x:v>
+        <x:v>src/main/reconcile.ts、report.ts、usage-sync.ts、index.ts；src/server/server.ts；src/shared/types.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；tests/reconciliation.test.ts、sync-reconciliation.test.ts、e2e/overlap-privacy.spec.ts；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
-        <x:v>待开发；故障已在隔离 SQLite 复现</x:v>
+        <x:v>已实现；TC-092–094 自动子范围通过（8157e2d），剩余断言和真实迁移待验证</x:v>
       </x:c>
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
@@ -5627,7 +5629,9 @@
 CSV 版本迁移：无冲突 v1 十列不变；含冲突显式 v2 十四列并改导出标签/文件名，前十列同顺序、冲突数值列空、末四列只给逐组小计与状态/来源/条数；旧消费者按表头或文件名识别版本。TC-029 仍验 v1，TC-093 验两个冲突组小计不重复，TC-023/079 扩到两版。现有本地/OTel 无共同事件 ID，TC-092 当前只验不误删/标冲突；同事件正向去重待双方真实具备并证明共同稳定 ID 后再验。
 升级服务先为旧 aggregates/source_coverage 标 legacy/unverified 并保留原值；同设备未收 v2 前若仍收 v1，也只能维持未核实。首次授权 v2 原子替换后，可证范围才 confirmed，冲突范围 uncertain；此后任何 v1（含更高 revision）须拒绝且聚合、覆盖、状态和 device_revisions 均不变。
 在主进程按登录态/授权查询范围构造 viewer 来源状态；不能仅前端隐藏全局 fileCount/factCount/telemetryFactCount、lastTelemetry/lastScan、detail 或由全局状态推导真零。无法证明 owner 归属则未知/空值；对齐来源状态 IPC、报表 coverage 与概览/报表 UI，管理员全局视图标明范围。TC-093 双 owner IPC/UI 回归，关联 TC-021/045/046/077/078。当前仅静态审查。
-诊断 IPC 和可选反馈附件必须复用按 owner 授权后的视图；通用 suggestion 可留，跨 owner location/reason、文件/事实/未归属/异常计数、lastScan/lastSuccess 不能经 IPC、UI 或反馈载荷泄露。</x:v>
+诊断 IPC 和可选反馈附件必须复用按 owner 授权后的视图；通用 suggestion 可留，跨 owner location/reason、文件/事实/未归属/异常计数、lastScan/lastSuccess 不能经 IPC、UI 或反馈载荷泄露。
+8157e2d：本地/OTel 按授权 owner 和会话调和；冲突候选不冒充已证重复，查询范围外同会话候选仍影响状态。报表/概览已确认小计、明细待核对原行、v2 十四列逐组小计及同快照导出；服务 v2 旧值 legacy_unknown/confirmedSubtotal=null、v2 后拒 v1、旧 outbox 重算/旧协议待传；viewer 来源状态/诊断/反馈附件隔离。文档会话 gate 82/56/22 全过；共同事件 ID 正向去重、TC-093 部分 IPC/UI 与 v2 公式/快照、生产迁移仍待补。管理员全局状态不代表 DEV-049 完成。
+47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5672,7 +5676,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–094 已分配；TC-001–076 与 TC-079–081 已注册，TC-077–078、TC-082–094 待注册/待验证。TC-076 仅合成旧版自动成功子范围通过；TC-028 真实签名公证与异机、TC-072 目标 Mac 权限仍待人工证据。</x:v>
+        <x:v>TC-001–094 已分配；TC-001–076、TC-079–081、TC-092–094 已注册（82 个），TC-077–078、TC-082–091 待注册（12 个）。TC-092–094 在 8157e2d 的自动子范围通过，完整边界见各行；TC-028/072 目标环境仍待人工证据。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -6662,22 +6666,25 @@
         <x:v>表格软件不会将该字段作为公式执行。</x:v>
       </x:c>
       <x:c r="H28" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；v1 原绑定及 v2 公式转义新绑定均通过（47b03d5）</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
-        <x:v>tests/report.test.ts</x:v>
+        <x:v>tests/report.test.ts
+2026-10-03 文档会话固定 47b03d5 独立运行 TC-023：原 v1 与新增 v2 项目/模型公式转义两项单元均通过、退出码 0；完整 gate 82 注册入口、57 单元、22 Electron 通过。</x:v>
       </x:c>
       <x:c r="J28" s="9" t="str">
         <x:v>npm run test:case -- TC-023</x:v>
       </x:c>
       <x:c r="K28" s="9" t="str">
-        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属</x:v>
+        <x:v>tests/report.test.ts：报表按本地时区与 ISO 周汇总，并限制普通用户归属
+47b03d5 extraRuns 新绑 tests/report-snapshot.test.ts 的 TC-023 CSV v2 待核对行的模型和项目名称仍转义公式，测试 +unsafe-project 与 =SUM(1,2)。</x:v>
       </x:c>
       <x:c r="L28" s="9" t="str">
-        <x:v>共享测试；非独立断言</x:v>
+        <x:v>原共享测试覆盖 v1 公式防注入；47b03d5 新增独立 v2 冲突行项目/模型公式转义。其他 CSV 文本组合和实际电子表格客户端行为未逐项验证。</x:v>
       </x:c>
       <x:c r="M28" s="9" t="str">
-        <x:v>保存共享 Vitest 函数日志及脱敏 CSV 字段断言。</x:v>
+        <x:v>保存共享 Vitest 函数日志及脱敏 CSV 字段断言。
+47b03d5；macOS 本机专用临时库；TC-023 两单元绑定退出码 0，门禁 82 入口/57 单元/22 Electron 退出码 0。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -9001,11 +9008,12 @@
 授权查询和选中事实的 SHA-256 快照 ID；事实变化后旧 ID 拒绝并提示刷新，刷新后 12→111 Token；不同筛选/角色的旧 ID 拒绝。Electron 最终只显示 B，加载中禁用导出，IPC 携带 B 筛选及 B ID。</x:v>
       </x:c>
       <x:c r="H84" s="55" t="str">
-        <x:v>已注册；单元 1/1 + Electron 1/1 通过（78b3a3b，本机隔离样本）</x:v>
+        <x:v>已注册；v1/v2 快照单元及 Electron 子范围通过（47b03d5）</x:v>
       </x:c>
       <x:c r="I84" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。</x:v>
+2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。
+47b03d5 文档会话独立运行 TC-079：单元与 Electron 均通过、退出码 0；单元增加 v1→v2 冲突、扫描后旧 snapshotId 拒绝和刷新小计 99→104；完整 gate 82/57/22 通过。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
         <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
@@ -9014,11 +9022,11 @@
         <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。</x:v>
       </x:c>
       <x:c r="L84" s="55" t="str">
-        <x:v>测试为本机隔离临时库/合成事实及 Electron 模拟 IPC；snapshotId 基于查询和选中事实，不是全库 revision。TC-079 不覆盖 REQ-040 历史覆盖、其他打磨需求或打包安装。CSV 原 10 列由 TC-029、公式转义由 TC-023 回归。
-DEV-057 后须回归 v1/v2 两版同授权查询快照；当前 TC-079 仅测 v1。</x:v>
+        <x:v>当前已在单元测试覆盖 v1 与冲突 v2 的扫描后旧 snapshotId 拒绝；Electron 仍侧重快速筛选切换与导出等待当前快照。snapshotId 是授权查询+事实集合身份，不是全库 revision；REQ-040 历史覆盖及目标安装环境仍未由此证明。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
-        <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。</x:v>
+        <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。
+47b03d5；macOS 本机隔离合成库；TC-079 单元/Electron 各 1/1、退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="185" customHeight="1">
@@ -9534,28 +9542,28 @@
         <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F97" s="61" t="str">
-        <x:v>独立临时库构造同提供方同 UTC 日本地用户 A 12 Token、遥测用户 B 99 Token；另造有共同稳定事件 ID 的重复、仅同会话但无共同事件 ID 的候选，以及同用户不同会话。</x:v>
+        <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
-        <x:v>A/B 独立事实各按权限保留；可证同事件只计主来源；仅同会话的候选标冲突且不当成已证重复；同日存在本地事实不能整批屏蔽遥测。</x:v>
+        <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
-        <x:v>待注册、待验证（已复现缺陷）</x:v>
+        <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
       </x:c>
       <x:c r="I97" s="61" t="str">
-        <x:v>2026-10-03 仅在一次性 SQLite 以现有 selectFacts SQL 复现 owner B 的 99 Token 被误排除；尚无修复代码、独立函数或通过证据。</x:v>
+        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-092：单元 1/1、退出码 0；管理员初值 111，owner B 99，A 不同会话 19，同会话后已确认小计 7/状态 uncertain。test:gate 82 注册入口、56 单元、22 Electron 通过。</x:v>
       </x:c>
       <x:c r="J97" s="61" t="str">
-        <x:v>npm run test:case -- TC-092（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-092（已注册；文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K97" s="61" t="str">
-        <x:v>拟新增 tests/report-overlap.test.ts 中以 TC-092 开头的独立函数并在 scripts/test-cases.mjs 注册。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/reconciliation.test.ts 中以 TC-092 开头的独立 Vitest 函数。</x:v>
       </x:c>
       <x:c r="L97" s="61" t="str">
-        <x:v>专用临时数据库和无正文合成记录；不得使用生产库。需核对不同用户授权及 Codex/Claude 各自来源身份。</x:v>
+        <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
-        <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>
+        <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="185" customHeight="1">
@@ -9572,7 +9580,7 @@
         <x:v>无法关联冲突与三处报表权限一致</x:v>
       </x:c>
       <x:c r="E98" s="64" t="str">
-        <x:v>单元/集成</x:v>
+        <x:v>单元/集成 + Electron</x:v>
       </x:c>
       <x:c r="F98" s="64" t="str">
         <x:v>独立库构造无法确认关联的本地/遥测重叠、多用户筛选、时区边界和 CSV；核对授权汇总、分页明细、导出各状态及数值。
@@ -9587,25 +9595,24 @@
 只按 provider 相同不得泄露 B 的文件/事实/未归属/异常计数、位置/原因、扫描/成功时间；通用指引和 A 可证字段可保留，无法归属字段未知/省略，反馈附件不增加权限。</x:v>
       </x:c>
       <x:c r="H98" s="64" t="str">
-        <x:v>待注册、待验证（已复现缺陷）</x:v>
+        <x:v>已注册；单元+Electron 自动子范围通过（47b03d5），真实冲突事实完整 E2E/生产环境待验证</x:v>
       </x:c>
       <x:c r="I98" s="64" t="str">
-        <x:v>2026-10-03 仅在一次性 SQLite 以现有 selectFacts SQL 复现 owner B 的 99 Token 被误排除；尚无修复代码、独立函数或通过证据。</x:v>
+        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-093：Vitest 1/1、Electron 1/1、退出码 0；单元 v2 十四列三组小计 5/7/0，总计 12，冲突明细保留 5 条，跨窗候选仍标冲突。Electron 真实 IPC/反馈附件双 owner 隔离；冲突 UI 文案采用注入响应。test:gate 82/56/22 全过。
+47b03d5 文档会话独立复跑 TC-093：unit 1/1、Electron 1/1、退出码 0；Electron 新验 viewer 直调 sources:scan 被拒、概览 Codex 卡本人 1 条且不含 B 的 2 条及 B 遥测时间。TC-023/079 v2 回归亦独立通过，gate 82/57/22。</x:v>
       </x:c>
       <x:c r="J98" s="64" t="str">
-        <x:v>npm run test:case -- TC-093（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-093（已注册；文档会话单元+Electron 退出码 0）</x:v>
       </x:c>
       <x:c r="K98" s="64" t="str">
-        <x:v>拟新增 tests/report-overlap.test.ts 中以 TC-093 开头的独立函数并在 scripts/test-cases.mjs 注册。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/reconciliation.test.ts 中 TC-093 Vitest 函数；tests/e2e/overlap-privacy.spec.ts 中 TC-093 Electron 函数。</x:v>
       </x:c>
       <x:c r="L98" s="64" t="str">
-        <x:v>专用临时数据库与无正文合成记录；当前本地/遥测没有通用事件 ID，同会话不能证明逐事件重复。不得使用生产库，不得用未知代替已证零，也不得把已确认小计称为完整总量。
-v2 仍待开发；TC-029 的既有自动通过只覆盖 v1 十列。TC-023 公式转义与 TC-079 同快照约束需扩到 v2。
-静态审查发现全局状态暴露路径；尚未动态复现或验收。验收必须在主进程 IPC 层断言，不以 UI 隐藏代替。
-反馈载荷用隔离接收器或桩验收，不提交真实反馈；不能只看诊断 UI，必须核主进程 IPC/附件。</x:v>
+        <x:v>当前已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
-        <x:v>实施后保存固定提交、环境、单编号命令/退出码和脱敏事实集合/冲突状态；旧 TC-016 的历史通过不能代替。</x:v>
+        <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
+47b03d5；macOS 本机隔离临时库/Electron；TC-093 unit/E2E 各 1/1 退出码 0，TC-023 两单元、TC-079 unit/E2E 均退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="195" customHeight="1">
@@ -9622,7 +9629,7 @@
         <x:v>服务上报与本地冲突计量同口径</x:v>
       </x:c>
       <x:c r="E99" s="67" t="str">
-        <x:v>集成</x:v>
+        <x:v>隔离服务集成单元</x:v>
       </x:c>
       <x:c r="F99" s="67" t="str">
         <x:v>隔离客户端和服务库构造同日跨 owner 本地/遥测、同 owner 疑似重叠；检查扫描后的版本 2 快照、服务端存储/查询、旧完整聚合清除、旧 outbox、旧协议拒绝/恢复重传、设备令牌范围与 TC-088 状态。
@@ -9633,23 +9640,22 @@
 迁移及旧客户端追加均显示 legacy/unverified，不把旧数值当完整；v2 原子替换后仅可证范围 confirmed、冲突 uncertain；收过 v2 的设备拒绝所有 v1，拒绝前后 aggregates/coverage/状态/revision 完全相同，跨 owner 授权仍拒绝。</x:v>
       </x:c>
       <x:c r="H99" s="67" t="str">
-        <x:v>待注册、待验证（静态代码核对）</x:v>
+        <x:v>已注册；隔离服务自动子范围 1/1 通过（8157e2d），真实迁移待验证</x:v>
       </x:c>
       <x:c r="I99" s="67" t="str">
-        <x:v>2026-10-03 静态核对 src/main/usage-sync.ts aggregate() 另有 provider+UTC 日 NOT EXISTS；src/server/server.ts 的 UsageSnapshot/白名单无冲突状态。尚未动态复现、无新协议或通过证据。</x:v>
+        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-094：单元 1/1、退出码 0。合成旧表迁移、旧 v1 续传 legacy_unknown/GET confirmedSubtotal=null、v2 重算及冲突、跨 owner/白名单拒绝、v1 回滚状态不变、旧 outbox 重算及协议不兼容待传后恢复。完整 gate 82/56/22 通过。</x:v>
       </x:c>
       <x:c r="J99" s="67" t="str">
-        <x:v>npm run test:case -- TC-094（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-094（已注册；文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K99" s="67" t="str">
-        <x:v>拟新增 tests/usage-sync-overlap.test.ts 中以 TC-094 开头的独立函数、服务隔离集成用例，在 scripts/test-cases.mjs 注册。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/sync-reconciliation.test.ts 中以 TC-094 开头的独立 Vitest 函数，使用合成客户端与隔离本机服务库。</x:v>
       </x:c>
       <x:c r="L99" s="67" t="str">
-        <x:v>专用临时客户端/服务数据库，无正文合成事实与假设备令牌；不得使用生产库或密钥。版本 2 协议需兼容/迁移设计，旧服务不能静默接收小计。
-当前 v1 数据已知可能跨 owner 误排除；TC-094 必须用历史库实测降级边界，不能仅测新 v2 干净库，也不能从旧 200/ready 推断完整。当前尚未注册或执行。</x:v>
+        <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
-        <x:v>实施后保存固定提交、环境、单编号命令/退出码、版本 2 快照白名单/权限/冲突/旧协议/旧 outbox/恢复重传的脱敏证据；关联复跑 TC-038–040、TC-047、TC-074、TC-088。</x:v>
+        <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: scope conservative coverage before complete evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R9a3bdaebd38d4689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R4a66f777b12142ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R06c103b20abd41d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb8bb3a32755242f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R8f3de3763f344507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7ea882c0945e4c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcc4040f400e74dd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R02bf31dab1eb46ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2465,7 +2465,7 @@
         <x:v>所选范围覆盖真值表</x:v>
       </x:c>
       <x:c r="G83" s="55" t="str">
-        <x:v>待注册、待验证；管理员双 owner+未归属，API/UI 按所选范围判未知/部分/真零；全局诊断单独标识</x:v>
+        <x:v>待注册、待验证；本轮只排 owner+工具+时区+区间未知/部分与假零阻断；完整空窗真零正例待证据方案</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="85" customHeight="1">
@@ -2488,7 +2488,7 @@
         <x:v>区间比较可比性门禁</x:v>
       </x:c>
       <x:c r="G84" s="58" t="str">
-        <x:v>待注册、待验证；管理员筛选范围两期同截止且完整才比较，全局 ready/其他 owner 时间不得补证</x:v>
+        <x:v>待注册、待验证；本轮只排同范围保守不可比较负例；同 as-of 双完整窗口同比正例待证据方案</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -3979,13 +3979,14 @@
       </x:c>
       <x:c r="C45" s="55" t="str">
         <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。
-管理员选具体用户或“未归属”后，来源卡、报表 coverage、真零与比较只按该用户+所选工具/IANA 时区/区间的可证覆盖判定。全局 ready/计数/最近扫描时间只能另标“全局”诊断，不能补全选中范围；全局 ready 而所选用户空且缺证据时为未知/部分，不是已确认零。</x:v>
+管理员选具体用户或“未归属”后，来源卡、报表 coverage、真零与比较只按该用户+所选工具/IANA 时区/区间的可证覆盖判定。全局 ready/计数/最近扫描时间只能另标“全局”诊断，不能补全选中范围；全局 ready 而所选用户空且缺证据时为未知/部分，不是已确认零。
+本轮部分范围：先按授权 owner（含未归属）+工具+IANA 时区+区间生成保守未知/可证部分覆盖；全局 ready/计数/时间、最早事实与成功空扫描都不构成完整证明。无事实不宣称已确认零；仅 pending 事实可显示已确认小计 0，但完整总量未知；比较不可比较。完整空窗真零和同 as-of 同口径同比正例待可证留存/连续采集方案。</x:v>
       </x:c>
       <x:c r="D45" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E45" s="55" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>待实现/待验证；本轮仅排保守未知/部分子范围，完整正例待证据方案</x:v>
       </x:c>
       <x:c r="F45" s="55" t="str">
         <x:v>DEV-049</x:v>
@@ -3995,7 +3996,8 @@
       </x:c>
       <x:c r="H45" s="55" t="str">
         <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
-2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。</x:v>
+2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。
+2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -5430,11 +5432,12 @@
 另核 src/renderer/report.tsx 的 coverage 与 src/main/index.ts 的授权报表 IPC；全局诊断若保留需显式标范围。</x:v>
       </x:c>
       <x:c r="F54" s="55" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>待开发；先实施保守未知/部分覆盖子范围，完整真零/同比正例待证据方案</x:v>
       </x:c>
       <x:c r="G54" s="55" t="str">
         <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。</x:v>
+管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。
+下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -8913,14 +8916,16 @@
       </x:c>
       <x:c r="F82" s="55" t="str">
         <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。
-构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。</x:v>
+构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。
+本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
         <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
-B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。</x:v>
+B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。
+缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；保守负例可先实施，完整真零正例待证据方案</x:v>
       </x:c>
       <x:c r="I82" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
@@ -8933,7 +8938,8 @@
       </x:c>
       <x:c r="L82" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。</x:v>
+计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。
+当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
@@ -8957,14 +8963,16 @@
       </x:c>
       <x:c r="F83" s="58" t="str">
         <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。
-管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。</x:v>
+管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。
+本轮先造管理员选定 owner/未归属两期、全局 ready 但选中范围缺证、今天进行中与扫描滞后；核 API/界面保持不可比较。完整同 as-of 正例等待证据方案。</x:v>
       </x:c>
       <x:c r="G83" s="58" t="str">
         <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。
-全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。</x:v>
+全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。
+没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；保守不可比较负例可先实施，完整同比正例待证据方案</x:v>
       </x:c>
       <x:c r="I83" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
@@ -8977,7 +8985,8 @@
       </x:c>
       <x:c r="L83" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。</x:v>
+计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。
+现有采集记录不能证明历史留存及连续采集；没有真实可得的同 as-of 双完整窗口，正向同比用例待需求会话决定证据来源。负例通过后整项仍待验证。</x:v>
       </x:c>
       <x:c r="M83" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: cite missing-source coverage limits
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R8f3de3763f344507"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7ea882c0945e4c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcc4040f400e74dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R02bf31dab1eb46ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R59088db07b21452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rff7f1c132fe14e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rdd62ebcab8424dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R085c8dad2ce0459d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3997,7 +3997,8 @@
       <x:c r="H45" s="55" t="str">
         <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。
-2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。</x:v>
+2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。
+2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -5437,7 +5438,8 @@
       <x:c r="G54" s="55" t="str">
         <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。
-下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。</x:v>
+下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。
+官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -8917,7 +8919,8 @@
       <x:c r="F82" s="55" t="str">
         <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。
 构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。
-本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。</x:v>
+本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。
+以无正文合成缺失输入模拟 Codex ephemeral 不落文件及 Claude OTel 未启用/exporter=none；核本地文件/OTel 缺记录仍未知，不宣称工具没用或真零。真实工具端到端验证另行安排。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
         <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
@@ -8939,7 +8942,8 @@
       <x:c r="L82" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。
-当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。</x:v>
+当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。
+外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
@@ -8986,7 +8990,8 @@
       <x:c r="L83" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。
-现有采集记录不能证明历史留存及连续采集；没有真实可得的同 as-of 双完整窗口，正向同比用例待需求会话决定证据来源。负例通过后整项仍待验证。</x:v>
+现有采集记录不能证明历史留存及连续采集；没有真实可得的同 as-of 双完整窗口，正向同比用例待需求会话决定证据来源。负例通过后整项仍待验证。
+TC-077 两类官方缺失来源反例存在时，两期均无记录仍不可比较；这些资料不提供同 as-of 双完整窗口的正例证据，正向同比继续待方案。</x:v>
       </x:c>
       <x:c r="M83" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: record scoped coverage validation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R59088db07b21452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rff7f1c132fe14e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rdd62ebcab8424dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R085c8dad2ce0459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R7b3c50001e164822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb56b72905f5f4dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R160b3f2831634cbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb1150e333acc421a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2465,7 +2465,7 @@
         <x:v>所选范围覆盖真值表</x:v>
       </x:c>
       <x:c r="G83" s="55" t="str">
-        <x:v>待注册、待验证；本轮只排 owner+工具+时区+区间未知/部分与假零阻断；完整空窗真零正例待证据方案</x:v>
+        <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="85" customHeight="1">
@@ -2488,7 +2488,7 @@
         <x:v>区间比较可比性门禁</x:v>
       </x:c>
       <x:c r="G84" s="58" t="str">
-        <x:v>待注册、待验证；本轮只排同范围保守不可比较负例；同 as-of 双完整窗口同比正例待证据方案</x:v>
+        <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -3986,7 +3986,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E45" s="55" t="str">
-        <x:v>待实现/待验证；本轮仅排保守未知/部分子范围，完整正例待证据方案</x:v>
+        <x:v>保守未知/防假零子范围已实现并独立复验（ef7a3de、c10bbf3）；整项待验证，完整真零/同比正例待证据方案</x:v>
       </x:c>
       <x:c r="F45" s="55" t="str">
         <x:v>DEV-049</x:v>
@@ -3998,7 +3998,8 @@
         <x:v>承接 REQ-010/028/029；需来源留存/游标/时间边界可证明的覆盖证据，缺证据降级未知或部分。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。
 2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。
-2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。</x:v>
+2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。
+2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -5433,13 +5434,14 @@
 另核 src/renderer/report.tsx 的 coverage 与 src/main/index.ts 的授权报表 IPC；全局诊断若保留需显式标范围。</x:v>
       </x:c>
       <x:c r="F54" s="55" t="str">
-        <x:v>待开发；先实施保守未知/部分覆盖子范围，完整真零/同比正例待证据方案</x:v>
+        <x:v>保守防假零/防假同比子范围已实现并独立复验（ef7a3de、c10bbf3）；完整覆盖证据与正例待开发/待验证</x:v>
       </x:c>
       <x:c r="G54" s="55" t="str">
         <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。
 下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。
-官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。</x:v>
+官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。
+2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -7596,7 +7598,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I50" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-045，unit 1/1，退出码 0；仅现有绑定断言。</x:v>
       </x:c>
       <x:c r="J50" s="14" t="str">
         <x:v>npm run test:case -- TC-045</x:v>
@@ -7608,7 +7611,8 @@
         <x:v>零/错误状态；未测全部界面缺失/权限状态</x:v>
       </x:c>
       <x:c r="M50" s="14" t="str">
-        <x:v>记录 TC-045 命令、退出码、提交、环境和脱敏日志；覆盖与限制：零/错误状态；未测全部界面缺失/权限状态。</x:v>
+        <x:v>记录 TC-045 命令、退出码、提交、环境和脱敏日志；覆盖与限制：零/错误状态；未测全部界面缺失/权限状态。
+c10bbf3；macOS x86_64 隔离合成样本；TC-045 unit 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="70" customHeight="1">
@@ -7637,7 +7641,8 @@
         <x:v>已验证（自动；边界待验）</x:v>
       </x:c>
       <x:c r="I51" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md</x:v>
+        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
+2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-046，unit 1/1，退出码 0；仅现有绑定断言。</x:v>
       </x:c>
       <x:c r="J51" s="35" t="str">
         <x:v>npm run test:case -- TC-046</x:v>
@@ -7649,7 +7654,8 @@
         <x:v>事实数/扫描时间/缺目录；未测全部状态卡片</x:v>
       </x:c>
       <x:c r="M51" s="35" t="str">
-        <x:v>记录 TC-046 命令、退出码、提交、环境和脱敏日志；覆盖与限制：事实数/扫描时间/缺目录；未测全部状态卡片。</x:v>
+        <x:v>记录 TC-046 命令、退出码、提交、环境和脱敏日志；覆盖与限制：事实数/扫描时间/缺目录；未测全部状态卡片。
+c10bbf3；macOS x86_64 隔离合成样本；TC-046 unit 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="146" customHeight="1">
@@ -8900,7 +8906,7 @@
 文档会话独立复跑 TC-076 1/1、TC-036 2/2、TC-034/035/059 各 1/1 和 76 入口检查，均退出码 0；开发会话报告 test:gate 52 单元/18 E2E。0.3.5 未签名 DMG 只在当前 Mac 核验；真实签名公证、目标 Mac 属 TC-028。</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="185" customHeight="1">
+    <x:row r="82" ht="300" customHeight="1">
       <x:c r="A82" s="55" t="str">
         <x:v>TC-077</x:v>
       </x:c>
@@ -8928,28 +8934,31 @@
 缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
-        <x:v>待注册、待验证；保守负例可先实施，完整真零正例待证据方案</x:v>
+        <x:v>已注册；防假零保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
       </x:c>
       <x:c r="I82" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-077：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。</x:v>
       </x:c>
       <x:c r="J82" s="55" t="str">
-        <x:v>npm run test:case -- TC-077（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-077（已注册；单元 1/1、Electron 1/1，文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K82" s="55" t="str">
-        <x:v>拟新增以 TC-077 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/coverage-window.test.ts 中 TC-077 Vitest 函数；tests/e2e/coverage-window.spec.ts 中 TC-077 Electron 函数。</x:v>
       </x:c>
       <x:c r="L82" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。
 当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。
-外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。</x:v>
+外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。
+现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="83" ht="185" customHeight="1">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
+ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="300" customHeight="1">
       <x:c r="A83" s="58" t="str">
         <x:v>TC-078</x:v>
       </x:c>
@@ -8976,25 +8985,28 @@
 没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
-        <x:v>待注册、待验证；保守不可比较负例可先实施，完整同比正例待证据方案</x:v>
+        <x:v>已注册；防假同比保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
       </x:c>
       <x:c r="I83" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-078：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。</x:v>
       </x:c>
       <x:c r="J83" s="58" t="str">
-        <x:v>npm run test:case -- TC-078（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-078（已注册；单元 1/1、Electron 1/1，文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K83" s="58" t="str">
-        <x:v>拟新增以 TC-078 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/coverage-window.test.ts 中 TC-078 Vitest 函数；tests/e2e/coverage-window.spec.ts 中 TC-078 Electron 函数。</x:v>
       </x:c>
       <x:c r="L83" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。
 现有采集记录不能证明历史留存及连续采集；没有真实可得的同 as-of 双完整窗口，正向同比用例待需求会话决定证据来源。负例通过后整项仍待验证。
-TC-077 两类官方缺失来源反例存在时，两期均无记录仍不可比较；这些资料不提供同 as-of 双完整窗口的正例证据，正向同比继续待方案。</x:v>
+TC-077 两类官方缺失来源反例存在时，两期均无记录仍不可比较；这些资料不提供同 as-of 双完整窗口的正例证据，正向同比继续待方案。
+Asia/Shanghai 与 UTC 边界、真实隔离 local/OTel 待核对 UI 子断言已过；仅 pending 时已确认小计 0 而完整总量未知，比较不可比。双完整窗口同 as-of 正例和扫描延迟证据仍未取得。</x:v>
       </x:c>
       <x:c r="M83" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
+ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="185" customHeight="1">
@@ -9070,7 +9082,8 @@
       </x:c>
       <x:c r="I85" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-2026-10-03 文档会话在固定代码 d18bb47 独立运行 npm run test:case -- TC-080，Electron 1/1 退出码 0；受影响 TC-054 1/1、TC-021 三绑定及完整 test:gate（79 入口、53 unit、21 E2E）均退出码 0。</x:v>
+2026-10-03 文档会话在固定代码 d18bb47 独立运行 npm run test:case -- TC-080，Electron 1/1 退出码 0；受影响 TC-054 1/1、TC-021 三绑定及完整 test:gate（79 入口、53 unit、21 E2E）均退出码 0。
+2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-080，Electron 1/1，退出码 0；仅现有绑定断言。</x:v>
       </x:c>
       <x:c r="J85" s="58" t="str">
         <x:v>npm run test:case -- TC-080（已注册；文档会话 2026-10-03 退出码 0）</x:v>
@@ -9082,7 +9095,8 @@
         <x:v>UTC 当前日期隔离合成事实覆盖 90/30/7、管理员 viewer、工具/时区、趋势桶、第二页、面包屑筛选与趋势按钮回焦；未造 DST、扫描延迟量化、所有键盘/VoiceOver 路径。</x:v>
       </x:c>
       <x:c r="M85" s="58" t="str">
-        <x:v>固定代码 d18bb47；macOS 本机隔离合成工作区；单编号 1/1、相关 TC-054 1/1、TC-021 三绑定、test:gate 79 入口/53 unit/21 E2E 均退出码 0。真实生产数据、目标 Mac、完整无障碍边界未验证。</x:v>
+        <x:v>固定代码 d18bb47；macOS 本机隔离合成工作区；单编号 1/1、相关 TC-054 1/1、TC-021 三绑定、test:gate 79 入口/53 unit/21 E2E 均退出码 0。真实生产数据、目标 Mac、完整无障碍边界未验证。
+c10bbf3；macOS x86_64 隔离合成样本；TC-080 Electron 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="185" customHeight="1">
@@ -9613,7 +9627,8 @@
       </x:c>
       <x:c r="I98" s="64" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-093：Vitest 1/1、Electron 1/1、退出码 0；单元 v2 十四列三组小计 5/7/0，总计 12，冲突明细保留 5 条，跨窗候选仍标冲突。Electron 真实 IPC/反馈附件双 owner 隔离；冲突 UI 文案采用注入响应。test:gate 82/56/22 全过。
-47b03d5 文档会话独立复跑 TC-093：unit 1/1、Electron 1/1、退出码 0；Electron 新验 viewer 直调 sources:scan 被拒、概览 Codex 卡本人 1 条且不含 B 的 2 条及 B 遥测时间。TC-023/079 v2 回归亦独立通过，gate 82/57/22。</x:v>
+47b03d5 文档会话独立复跑 TC-093：unit 1/1、Electron 1/1、退出码 0；Electron 新验 viewer 直调 sources:scan 被拒、概览 Codex 卡本人 1 条且不含 B 的 2 条及 B 遥测时间。TC-023/079 v2 回归亦独立通过，gate 82/57/22。
+2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-093，unit 1/1、Electron 1/1，退出码 0；仅现有绑定断言。</x:v>
       </x:c>
       <x:c r="J98" s="64" t="str">
         <x:v>npm run test:case -- TC-093（已注册；文档会话单元+Electron 退出码 0）</x:v>
@@ -9626,7 +9641,8 @@
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
-47b03d5；macOS 本机隔离临时库/Electron；TC-093 unit/E2E 各 1/1 退出码 0，TC-023 两单元、TC-079 unit/E2E 均退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。</x:v>
+47b03d5；macOS 本机隔离临时库/Electron；TC-093 unit/E2E 各 1/1 退出码 0，TC-023 两单元、TC-079 unit/E2E 均退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
+c10bbf3；macOS x86_64 隔离合成样本；TC-093 unit 1/1、Electron 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="195" customHeight="1">

</xml_diff>

<commit_message>
docs: scope empty-state work before implementation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R7b3c50001e164822"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb56b72905f5f4dc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R160b3f2831634cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb1150e333acc421a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5e5b76f30e144044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd1bd6a063ea4495d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd97a4ab0298f4ef6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rccf7dd01df9d4d5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2626,7 +2626,7 @@
         <x:v>六类空状态与可操作下一步</x:v>
       </x:c>
       <x:c r="G90" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-084 待注册、待验证；本轮先测保守空状态/行动，真零正例待 REQ-040 的 complete 证据方案，REQ-044 整项待验</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -2649,7 +2649,7 @@
         <x:v>长扫描进展与诊断重试</x:v>
       </x:c>
       <x:c r="G91" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-085 待注册、待验证；本轮可先测长扫描真实阶段/心跳与诊断修复重试，不证明真零或完整覆盖</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="85" customHeight="1">
@@ -4091,7 +4091,8 @@
         <x:v>可操作空状态与扫描反馈</x:v>
       </x:c>
       <x:c r="C49" s="55" t="str">
-        <x:v>真零、未扫描、权限不足、格式不支持、筛选无匹配和部分覆盖分别说明原因与下一步；诊断原因指向相应授权/重扫/调整筛选动作。长扫描持续显示阶段与最近进展，不伪造百分比，失败可重试。</x:v>
+        <x:v>真零、未扫描、权限不足、格式不支持、筛选无匹配和部分覆盖分别说明原因与下一步；诊断原因指向相应授权/重扫/调整筛选动作。长扫描持续显示阶段与最近进展，不伪造百分比，失败可重试。
+本轮只排可证的分型和行动：未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知及有已观测记录但完整性未知；真零保留为未来同一授权筛选范围 coverage.complete 且事实为空的受控分支。</x:v>
       </x:c>
       <x:c r="D49" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4106,7 +4107,8 @@
         <x:v>TC-084、TC-085</x:v>
       </x:c>
       <x:c r="H49" s="55" t="str">
-        <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5537,7 +5539,8 @@
         <x:v>待开发；关联新 TC 待注册/待验证</x:v>
       </x:c>
       <x:c r="G58" s="55" t="str">
-        <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -9240,13 +9243,15 @@
         <x:v>单元/Electron</x:v>
       </x:c>
       <x:c r="F89" s="58" t="str">
-        <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。</x:v>
+        <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。
+2026-10-03 本轮先逐项造未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知、已观测但完整性未知；核授权范围、文案与行动。真零正例等待可证完整空窗，不在本轮造数或注入 complete。</x:v>
       </x:c>
       <x:c r="G89" s="58" t="str">
-        <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。</x:v>
+        <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。
+保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；本轮仅排保守空状态负例，真零正例待 REQ-040 证据方案，整项待验</x:v>
       </x:c>
       <x:c r="I89" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
@@ -9258,7 +9263,8 @@
         <x:v>拟新增以 TC-084 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L89" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+SOP-001/002 本轮范围决议：当前 REQ-040 没有完整空窗证据；不得用全局 ready、成功空扫描、空事实或伪造 complete 让“真零”通过。用隔离库和 Electron 分别检查各保守状态的原因、角色/筛选范围和实际行动。</x:v>
       </x:c>
       <x:c r="M89" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
@@ -9281,13 +9287,15 @@
         <x:v>Electron 端到端</x:v>
       </x:c>
       <x:c r="F90" s="55" t="str">
-        <x:v>慢速合成扫描、阶段停顿、解析错误及随后修复重试。</x:v>
+        <x:v>慢速合成扫描、阶段停顿、解析错误及随后修复重试。
+本轮在专用临时目录注入慢扫描、真实阶段停顿与解析失败，再修复输入后重扫；记录阶段、最近已处理量或心跳及诊断/重试结果，不造伪百分比。</x:v>
       </x:c>
       <x:c r="G90" s="55" t="str">
-        <x:v>期间持续反馈真实阶段/最近进展，无假百分比或无响应；原因→下一步→重试后状态更新。</x:v>
+        <x:v>期间持续反馈真实阶段/最近进展，无假百分比或无响应；原因→下一步→重试后状态更新。
+进展、诊断和操作须与真实扫描状态一致；重试后旧错误不继续占位。该子范围不证明完整覆盖、真零或 TC-084 正例。</x:v>
       </x:c>
       <x:c r="H90" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证；长扫描/修复重试子范围可先实施，整项按实际证据验收</x:v>
       </x:c>
       <x:c r="I90" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
@@ -9299,7 +9307,8 @@
         <x:v>拟新增以 TC-085 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L90" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+SOP-001/002 本轮范围决议：TC-085 可独立于完整空窗证据先测真实扫描反馈和修复重试；需独立命名函数、专用临时库/用户目录，未运行前不写通过。</x:v>
       </x:c>
       <x:c r="M90" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: record onboarding validation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5e5b76f30e144044"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd1bd6a063ea4495d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rd97a4ab0298f4ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rccf7dd01df9d4d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1aa0951b5a144427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb91c00c6557043db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2063d7b95ded4ea8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5274d6854b3647c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2580,7 +2580,7 @@
         <x:v>管理员四步引导与跳过恢复</x:v>
       </x:c>
       <x:c r="G88" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-082 已注册；2 单元+1 Electron 隔离自动子范围通过（3bbaf15）；真实生产/打包环境待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="85" customHeight="1">
@@ -2603,7 +2603,7 @@
         <x:v>普通用户引导角色边界</x:v>
       </x:c>
       <x:c r="G89" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-083 已注册；1 单元+1 Electron 隔离自动子范围通过（3bbaf15）；真实生产/打包环境待验证</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="85" customHeight="1">
@@ -3999,7 +3999,8 @@
 2026-10-03 静态审查：概览以全局 sources 判断 ready/no_records，报表 coverage 返回全局状态；TC-077/078 新增管理员双 owner+未归属反例。当前未动态复现或验收，DEV-057 管理员可见全局诊断不代表本需求通过。
 2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。
 2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。
-2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。</x:v>
+2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。
+3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -4071,7 +4072,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E48" s="58" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>已实现；隔离自动子范围通过（3bbaf15），真实生产数据/打包环境待验证</x:v>
       </x:c>
       <x:c r="F48" s="58" t="str">
         <x:v>DEV-052</x:v>
@@ -4080,7 +4081,8 @@
         <x:v>TC-082、TC-083</x:v>
       </x:c>
       <x:c r="H48" s="58" t="str">
-        <x:v>独立新能力；与现有首次建账及角色授权兼容。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>独立新能力；与现有首次建账及角色授权兼容。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 代码 3bbaf15：主进程 onboarding:status 授权四步，管理员成功空扫描可完成扫描步、重扫不倒退；viewer 仅本人归属/用量，扫描步因来源级不可归属而保持未知。零 Token/同会话 local+OTel 待核对不算首笔，须已确认正 Token。按用户跳过/重开，已绑定且有正用量的 viewer 概览不常驻催促。文档会话独立复跑 TC-082/083 与回归和完整门禁，通过范围见 docs/validation.md；生产/打包/工具版本未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="150" customHeight="1">
@@ -5510,13 +5512,14 @@
         <x:v>TC-082、TC-083</x:v>
       </x:c>
       <x:c r="E57" s="58" t="str">
-        <x:v>src/renderer/；src/main/index.ts；独立用户数据与角色 Electron 测试</x:v>
+        <x:v>src/main/onboarding.ts；src/main/index.ts 授权 IPC；src/preload/index.ts、src/renderer/index.tsx、onboarding.tsx、style.css；tests/onboarding.test.ts、tests/e2e/onboarding.spec.ts</x:v>
       </x:c>
       <x:c r="F57" s="58" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>已实现；隔离自动子范围通过（3bbaf15），真实生产数据/打包环境待验证</x:v>
       </x:c>
       <x:c r="G57" s="58" t="str">
-        <x:v>四步只读真实状态；跳过可重开；viewer 不出现管理员绑定动作，任何状态写入受主进程角色校验。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>四步只读真实状态；跳过可重开；viewer 不出现管理员绑定动作，任何状态写入受主进程角色校验。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+3bbaf15：onboarding:status 仅按登录态查本人或管理员范围；成功扫描/重扫状态稳定，首笔须已确认正 Token，零 Token 和 pending 不算。概览提示可跳过，当前 Electron userData 的 localStorage 按应用 user.id 保存；侧栏可重开，viewer 完成归属和首笔后不常驻催促。状态只在登录、进入概览/引导、手动扫描/归属/刷新时重算；2500 条合成事实单次状态调用 &lt;2 秒断言。TC-082/083 独立复验通过，门禁 86 入口/62 unit/26 Electron；真实环境待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="155" customHeight="1">
@@ -8941,7 +8944,8 @@
       </x:c>
       <x:c r="I82" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-077：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。</x:v>
+2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-077：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。
+3bbaf15 文档会话复跑 TC-077 单元 1/1、Electron 1/1、退出码 0；新增无事实 reason 的“没有已观测记录”断言。</x:v>
       </x:c>
       <x:c r="J82" s="55" t="str">
         <x:v>npm run test:case -- TC-077（已注册；单元 1/1、Electron 1/1，文档会话退出码 0）</x:v>
@@ -8954,11 +8958,13 @@
 计划用例，未注册或执行；不得以 DEV-057 的管理员全局状态返回、TC-080/081 的筛选下钻通过或空事实集合冒充范围完整。
 当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。
 外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。
-现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。</x:v>
+现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。
+3bbaf15 已修正原“未归属”筛选下无事实 reason 的“已归属”措辞；仍不证明完整覆盖。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
-ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。</x:v>
+ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。
+3bbaf15；TC-077 单元 1/1、Electron 1/1、退出码 0；门禁 86 入口/62 unit/26 Electron 通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="300" customHeight="1">
@@ -9144,7 +9150,7 @@
         <x:v>固定代码 d18bb47；macOS 本机隔离合成工作区；单编号 1/1、相关 TC-054 1/1、TC-021 三绑定、test:gate 79 入口/53 unit/21 E2E 均退出码 0。真实生产数据、目标 Mac、完整无障碍边界未验证。</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" ht="185" customHeight="1">
+    <x:row r="87" ht="250" customHeight="1">
       <x:c r="A87" s="58" t="str">
         <x:v>TC-082</x:v>
       </x:c>
@@ -9167,25 +9173,28 @@
         <x:v>四步状态与真实数据一致，跳过不产生归属/采集副作用，重开可继续。</x:v>
       </x:c>
       <x:c r="H87" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；隔离自动子范围通过（3bbaf15），真实生产/打包环境待验证</x:v>
       </x:c>
       <x:c r="I87" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在固定代码 3bbaf15、macOS x86_64 / Node v24.15.0 / npm 11.12.1 独立运行 npm run test:case -- TC-082：2 unit + 1 Electron 全通过、退出码 0；test:gate 86 入口/62 unit/26 Electron 通过。</x:v>
       </x:c>
       <x:c r="J87" s="58" t="str">
-        <x:v>npm run test:case -- TC-082（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-082（已注册；文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K87" s="58" t="str">
-        <x:v>拟新增以 TC-082 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/onboarding.test.ts 中 TC-082 独立 Vitest 函数；tests/e2e/onboarding.spec.ts 中 TC-082 Electron 函数。另有第二个性能 Vitest 绑定。</x:v>
       </x:c>
       <x:c r="L87" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+管理员四步及 2500 条合成事实状态响应两项单元；管理员跳过/重开和真实采集归属更新一项 Electron。 四步状态、成功空扫描、重扫不倒退、零 Token 非首笔、已确认正 Token、跳过无归属副作用与重载后侧栏重开；2500 条单次调用 &lt;2 秒，仅限合成样本。 未使用真实生产用户数据或打包 App，不从自动断言推断所有工具版本。</x:v>
       </x:c>
       <x:c r="M87" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="185" customHeight="1">
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
+3bbaf15；macOS x86_64、Node v24.15.0，独立临时 SQLite/用户目录和无正文合成事实；2 unit + 1 Electron，单编号退出码 0；完整门禁 86 入口/62 unit/26 Electron 退出码 0。见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="250" customHeight="1">
       <x:c r="A88" s="55" t="str">
         <x:v>TC-083</x:v>
       </x:c>
@@ -9208,22 +9217,25 @@
         <x:v>普通用户仅见授权结果和请求管理员指引，不能从 UI/IPC 绑定来源；跳过和首笔用量状态正确。</x:v>
       </x:c>
       <x:c r="H88" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；隔离自动子范围通过（3bbaf15），真实生产/打包环境待验证</x:v>
       </x:c>
       <x:c r="I88" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-03 文档会话在固定代码 3bbaf15、macOS x86_64 / Node v24.15.0 / npm 11.12.1 独立运行 npm run test:case -- TC-083：1 unit + 1 Electron 全通过、退出码 0；test:gate 86 入口/62 unit/26 Electron 通过。</x:v>
       </x:c>
       <x:c r="J88" s="55" t="str">
-        <x:v>npm run test:case -- TC-083（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-083（已注册；文档会话退出码 0）</x:v>
       </x:c>
       <x:c r="K88" s="55" t="str">
-        <x:v>拟新增以 TC-083 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>scripts/test-cases.mjs：tests/onboarding.test.ts 中 TC-083 独立 Vitest 函数；tests/e2e/onboarding.spec.ts 中 TC-083 Electron 函数。</x:v>
       </x:c>
       <x:c r="L88" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+viewer 本人归属/待核对冲突单元；多用户角色隔离、扫描/绑定 IPC 拒绝、按用户跳过和非催促 Electron。 其他 owner 扫描/事实不进入 viewer 状态；扫描步未知并指引管理员，同会话 local/OTel pending 不算首笔；绑定且正用量后概览不常驻催促，详情仍未知。 未使用真实生产用户数据或打包 App，不从自动断言推断所有工具版本。</x:v>
       </x:c>
       <x:c r="M88" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
+3bbaf15；macOS x86_64、Node v24.15.0，独立临时 SQLite/用户目录和无正文合成事实；1 unit + 1 Electron，单编号退出码 0；完整门禁 86 入口/62 unit/26 Electron 退出码 0。见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="185" customHeight="1">

</xml_diff>

<commit_message>
docs: scope source rebinding preview and audit
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1aa0951b5a144427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb91c00c6557043db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2063d7b95ded4ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5274d6854b3647c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3aad6868576046b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1b504f87c7024e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2fc1b22772ef499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R22a5d49168754c4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2672,7 +2672,8 @@
         <x:v>来源重绑预览与确认范围</x:v>
       </x:c>
       <x:c r="G92" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-086 待注册/待验；草稿/授权预览、同筛选双 owner 可见范围、取消/Escape、确认、重扫后过期基线和 viewer 越权
+在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -2695,7 +2696,8 @@
         <x:v>来源重绑失败回滚与最小审计</x:v>
       </x:c>
       <x:c r="G93" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>TC-087 待注册/待验；业务拒绝、事务/审计失败、数据库不可写、原子回滚与不透明审计引用及旧日志脱敏
+离线重绑须留新 revision/待传，旧 owner 队列失效，恢复后重试。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="85" customHeight="1">
@@ -2718,7 +2720,8 @@
         <x:v>本机采集与可选服务状态分离</x:v>
       </x:c>
       <x:c r="G94" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证（规划目标）
+与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="85" customHeight="1">
@@ -4121,7 +4124,9 @@
         <x:v>来源重新绑定预览确认与最小审计</x:v>
       </x:c>
       <x:c r="C50" s="58" t="str">
-        <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、来源稳定键、前后用户 ID、数量和结果码，不含路径/正文。</x:v>
+        <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、来源稳定键、前后用户 ID、数量和结果码，不含路径/正文。
+选择候选只留 UI 草稿；主进程预览须显示原/新 owner、来源全部受影响事实数及相同筛选下两侧授权可见事实范围/待核对状态。确认时在事务中复验权限、来源、目标活跃性、原 owner 和预览事实集合基线；重扫或目标变化后旧预览失效，须重取。取消/Escape 无写入；失败恢复 UI 原值并给可操作错误。审计只存持久随机不透明来源引用，不存原始 key/标签/路径/账号/正文；旧审计展示/导出前脱敏。
+重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。</x:v>
       </x:c>
       <x:c r="D50" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4136,7 +4141,9 @@
         <x:v>TC-086、TC-087</x:v>
       </x:c>
       <x:c r="H50" s="58" t="str">
-        <x:v>承接 REQ-011；归属与报表权限应在同一提交边界生效。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-011；归属与报表权限应在同一提交边界生效。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 SOP-001/002 实施前静态核对：当前来源下拉 onChange 立即 bind；scanner.identities().factCount 为来源全部 usage_facts 条数，不能当选定筛选后可见集；scanner.bindIdentity() 当前把原始 key 写 audit_events.target_id。新预览和审计白名单按 docs/design.md §20.3 实施，未改代码、未运行新用例。
+当前 sources:bind 只调用 bindIdentity，没有显式生成 usage-sync 新快照；TC-086/087 分别验在线旧 owner 清除和离线队列，TC-088 回归本地与服务状态分离。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -5567,7 +5574,9 @@
       </x:c>
       <x:c r="G59" s="58" t="str">
         <x:v>预览受影响事实数/可见范围，确认后主进程复验权限和版本；事务提交归属及最小审计，失败不改变归属；审计不保存路径/正文。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-需求复核补充：成功绑定与最小审计同事务；业务拒绝可另记结果，DB 不可写时绑定不变且不得声称审计已持久化。</x:v>
+需求复核补充：成功绑定与最小审计同事务；业务拒绝可另记结果，DB 不可写时绑定不变且不得声称审计已持久化。
+实施前补充：改下拉为草稿→授权预览→确认，预览含原/新 owner、来源全体受影响事实数与同筛选两侧报表可见集合/待核对状态；带归属和事实集合的不可伪造基线。确认在事务内重验 actor、来源、活跃目标、旧 owner 与基线，重扫新增/改写事实须拒绝旧预览。成功归属+最小审计同事务并刷新 UI/报表；取消/Escape 无写入，失败 UI 回原值。审计引用用持久随机不透明 ID，历史 raw key 展示/导出前脱敏；DB 不可写时不宣称审计持久。TC-086/087 分别测一致性/权限与失败回滚/隐私。
+绑定成功后创建持久版本 2 新 revision/待传义务，停止上传旧 owner 队列；在线替换/清除旧 owner 服务聚合，离线显示本地已变而服务待传并可重试。不得回退 DEV-057 v2 授权/冲突口径，交叉回归 TC-088。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -9326,7 +9335,7 @@
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="185" customHeight="1">
+    <x:row r="91" ht="320" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9343,10 +9352,14 @@
         <x:v>集成/Electron</x:v>
       </x:c>
       <x:c r="F91" s="58" t="str">
-        <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。</x:v>
+        <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。
+本轮补造已确认与待核对事实、筛选内外事实；选候选只成草稿，预览原/新 owner、全部受影响数、同筛选两侧授权可见集合。取消/Escape、确认后刷新、viewer 预览/确认 IPC 越权；预览后重扫增删/改写事实或目标停用再确认，旧基线必须失效。
+在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
-        <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。</x:v>
+        <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
+预览数量须与实际转移授权可见性的事实集合一致，不能以来源总 factCount 充当筛选后可见总量；取消/Escape 无归属/报表/成功审计变化。确认时同事务复验，过期预览拒绝并提示刷新；成功后恰好所示范围变化且 UI/报表同步，viewer IPC 拒绝。
+预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9361,13 +9374,15 @@
         <x:v>拟新增以 TC-086 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L91" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+当前 UI 下拉 onChange 直绑，需改为草稿/预览/确认。来源全体条数与相同筛选可见事实数须分列；pending 不称已确认总量。用专用临时库并在预览后注入新扫描/目标状态变化检验竞态，未实施前不登记通过。
+用独立测试服务和合成聚合核对在线同步；不把本地成功等同服务成功。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="185" customHeight="1">
+    <x:row r="92" ht="320" customHeight="1">
       <x:c r="A92" s="55" t="str">
         <x:v>TC-087</x:v>
       </x:c>
@@ -9384,10 +9399,14 @@
         <x:v>集成</x:v>
       </x:c>
       <x:c r="F92" s="55" t="str">
-        <x:v>在业务规则拒绝、事务写入失败及数据库不可写处分别注入异常，检查归属/报表；成功路径检查审计字段。</x:v>
+        <x:v>在业务规则拒绝、事务写入失败及数据库不可写处分别注入异常，检查归属/报表；成功路径检查审计字段。
+本轮补验成功归属与最小审计同事务；注入业务拒绝、归属写入/审计写入失败、数据库不可写。检查下拉恢复、可操作错误、旧 owner 报表不变及审计是否实际持久化；审计展示/导出扫描当前和历史行的原始来源 key/标签/路径/账号/会话/事实 ID/正文泄漏。
+离线确认后检查新 revision/待传快照持久、旧 owner 旧队列失效；恢复后重试新授权快照。</x:v>
       </x:c>
       <x:c r="G92" s="55" t="str">
-        <x:v>成功绑定与最小审计同事务；各失败均保持旧归属/统计。业务拒绝可单记最小结果；数据库不可写时不要求持久审计，但不得误报成功或更改归属；审计无路径/正文。</x:v>
+        <x:v>成功绑定与最小审计同事务；各失败均保持旧归属/统计。业务拒绝可单记最小结果；数据库不可写时不要求持久审计，但不得误报成功或更改归属；审计无路径/正文。
+成功审计限时间、actor/旧新 owner 应用用户 ID、持久随机不透明来源引用、受影响事实数和结果码；不能把原始 key 写 target_id。审计写失败则归属回滚；业务拒绝仅可在 DB 可写时另记最小结果，不可写时不宣称持久审计。所有失败 UI/报表恢复旧状态。
+本地重绑成功但服务离线时分别显示本地已变和服务待传/重试；恢复后按版本 2 口径上传，旧 owner 聚合清除且旧快照不再发送。</x:v>
       </x:c>
       <x:c r="H92" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9402,13 +9421,15 @@
         <x:v>拟新增以 TC-087 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L92" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+scanner.bindIdentity() 当前 audit_events.target_id 写原始 key，是需修正的旧行为；旧行任何展示/导出前也须脱敏。独立合成用户/来源，不提交真实账户、路径、会话正文或凭证；测试注入失败后清理。
+模拟断网、旧队列与恢复，审计与同步失败分别断言，DEV-057 v2 冲突口径保持。</x:v>
       </x:c>
       <x:c r="M92" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="185" customHeight="1">
+    <x:row r="93" ht="320" customHeight="1">
       <x:c r="A93" s="58" t="str">
         <x:v>TC-088</x:v>
       </x:c>
@@ -9426,11 +9447,13 @@
       </x:c>
       <x:c r="F93" s="58" t="str">
         <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。
-追加用量冲突与旧上报协议不兼容两类状态，观察本地报表和服务状态。</x:v>
+追加用量冲突与旧上报协议不兼容两类状态，观察本地报表和服务状态。
+交叉回归来源重绑后在线与离线场景，核本地授权即时变化、服务旧 owner 聚合清除/待传。</x:v>
       </x:c>
       <x:c r="G93" s="58" t="str">
         <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。
-本地统计仍可用；冲突/协议不兼容显示“待核对/未同步”及原因，不误写网络离线、零用量或扫描失败；与 TC-094 的服务快照结果一致。</x:v>
+本地统计仍可用；冲突/协议不兼容显示“待核对/未同步”及原因，不误写网络离线、零用量或扫描失败；与 TC-094 的服务快照结果一致。
+在线服务状态只在旧 owner 聚合已替换/清除后显示同步；离线保留本地报表正常和服务待传，恢复重试不上传旧队列。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9445,7 +9468,8 @@
         <x:v>拟新增以 TC-088 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L93" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+与 TC-086/087 共享同一预期语义，但独立运行 TC-088；DEV-057 版本 2 授权和冲突口径须保持。</x:v>
       </x:c>
       <x:c r="M93" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: validate empty states and scan progress
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3aad6868576046b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1b504f87c7024e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2fc1b22772ef499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R22a5d49168754c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5de37a15c3584da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd1be8e0cde5446f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R484b6f83d2cf4150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R19e39c65484840e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2626,7 +2626,7 @@
         <x:v>六类空状态与可操作下一步</x:v>
       </x:c>
       <x:c r="G90" s="58" t="str">
-        <x:v>TC-084 待注册、待验证；本轮先测保守空状态/行动，真零正例待 REQ-040 的 complete 证据方案，REQ-044 整项待验</x:v>
+        <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -2649,7 +2649,7 @@
         <x:v>长扫描进展与诊断重试</x:v>
       </x:c>
       <x:c r="G91" s="55" t="str">
-        <x:v>TC-085 待注册、待验证；本轮可先测长扫描真实阶段/心跳与诊断修复重试，不证明真零或完整覆盖</x:v>
+        <x:v>TC-085 已注册：单元+Electron 进度/修复重试子范围通过；取消/续扫未实现，整项待验</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="85" customHeight="1">
@@ -4103,7 +4103,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E49" s="55" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>部分实现；保守空状态与进度/重试自动子范围通过，真零及取消待验</x:v>
       </x:c>
       <x:c r="F49" s="55" t="str">
         <x:v>DEV-053</x:v>
@@ -4113,7 +4113,8 @@
       </x:c>
       <x:c r="H49" s="55" t="str">
         <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
-2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。</x:v>
+2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。
+2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5546,11 +5547,12 @@
         <x:v>src/collectors/scanner.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；状态测试</x:v>
       </x:c>
       <x:c r="F58" s="55" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>部分实现；TC-084/085 已注册，保守子范围通过，真零与取消待补</x:v>
       </x:c>
       <x:c r="G58" s="55" t="str">
         <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。</x:v>
+本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。
+代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -9247,7 +9249,7 @@
 3bbaf15；macOS x86_64、Node v24.15.0，独立临时 SQLite/用户目录和无正文合成事实；1 unit + 1 Electron，单编号退出码 0；完整门禁 86 入口/62 unit/26 Electron 退出码 0。见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" ht="185" customHeight="1">
+    <x:row r="89" ht="340" customHeight="1">
       <x:c r="A89" s="58" t="str">
         <x:v>TC-084</x:v>
       </x:c>
@@ -9272,26 +9274,27 @@
 保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
-        <x:v>待注册、待验证；本轮仅排保守空状态负例，真零正例待 REQ-040 证据方案，整项待验</x:v>
+        <x:v>已注册；保守空状态自动子范围通过，真零正例待 REQ-040 完整覆盖证据，整项待验</x:v>
       </x:c>
       <x:c r="I89" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。仅保守状态与筛选无匹配 UI 行动；完整空窗真零未验。此前“待注册/不可运行”是实施前记录。</x:v>
       </x:c>
       <x:c r="J89" s="58" t="str">
-        <x:v>npm run test:case -- TC-084（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-084（2026-10-03 独立通过）</x:v>
       </x:c>
       <x:c r="K89" s="58" t="str">
-        <x:v>拟新增以 TC-084 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/empty-state.test.ts：TC-084 未扫描权限格式筛选无匹配及已观测未知各给出独立行动且不造真零；tests/e2e/empty-state.spec.ts：TC-084 报表筛选无匹配保持覆盖未知并可清除筛选进入诊断</x:v>
       </x:c>
       <x:c r="L89" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-SOP-001/002 本轮范围决议：当前 REQ-040 没有完整空窗证据；不得用全局 ready、成功空扫描、空事实或伪造 complete 让“真零”通过。用隔离库和 Electron 分别检查各保守状态的原因、角色/筛选范围和实际行动。</x:v>
+SOP-001/002 本轮范围决议：当前 REQ-040 没有完整空窗证据；不得用全局 ready、成功空扫描、空事实或伪造 complete 让“真零”通过。用隔离库和 Electron 分别检查各保守状态的原因、角色/筛选范围和实际行动。
+Electron 仅走筛选无匹配→清除→诊断；其他状态的逐类 UI 行动与真零正例未覆盖。</x:v>
       </x:c>
       <x:c r="M89" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="185" customHeight="1">
+        <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。REQ-040 尚无 complete 证据，TC-084 整项待验；docs/validation.md 对应记录。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="340" customHeight="1">
       <x:c r="A90" s="55" t="str">
         <x:v>TC-085</x:v>
       </x:c>
@@ -9309,30 +9312,33 @@
       </x:c>
       <x:c r="F90" s="55" t="str">
         <x:v>慢速合成扫描、阶段停顿、解析错误及随后修复重试。
-本轮在专用临时目录注入慢扫描、真实阶段停顿与解析失败，再修复输入后重扫；记录阶段、最近已处理量或心跳及诊断/重试结果，不造伪百分比。</x:v>
+本轮在专用临时目录注入慢扫描、真实阶段停顿与解析失败，再修复输入后重扫；记录阶段、最近已处理量或心跳及诊断/重试结果，不造伪百分比。
+后续补慢文件取消、重复点击、当前文件事务结束、已处理事实/游标与覆盖未知、重新扫描续跑及 viewer IPC 拒绝；不得以重试通过替代取消。</x:v>
       </x:c>
       <x:c r="G90" s="55" t="str">
         <x:v>期间持续反馈真实阶段/最近进展，无假百分比或无响应；原因→下一步→重试后状态更新。
-进展、诊断和操作须与真实扫描状态一致；重试后旧错误不继续占位。该子范围不证明完整覆盖、真零或 TC-084 正例。</x:v>
+进展、诊断和操作须与真实扫描状态一致；重试后旧错误不继续占位。该子范围不证明完整覆盖、真零或 TC-084 正例。
+取消后不接收新文件，当前文件事实/游标原子完成；本轮为已取消/覆盖未知，不作完整成功或完整同步；从游标续跑且不并发。若立即中断单文件，该文件事实/游标均回滚。</x:v>
       </x:c>
       <x:c r="H90" s="55" t="str">
-        <x:v>待注册、待验证；长扫描/修复重试子范围可先实施，整项按实际证据验收</x:v>
+        <x:v>已注册；真实进度与修复重试自动子范围通过，取消/续扫未实现，整项待验</x:v>
       </x:c>
       <x:c r="I90" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。当前无取消 IPC/UI/扫描器状态，此前“待注册/不可运行”是实施前记录。</x:v>
       </x:c>
       <x:c r="J90" s="55" t="str">
-        <x:v>npm run test:case -- TC-085（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-085（2026-10-03 进度/重试子范围通过）</x:v>
       </x:c>
       <x:c r="K90" s="55" t="str">
-        <x:v>拟新增以 TC-085 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/m6-diagnostics.test.ts：TC-085 慢扫描真实处理数及解析失败修复重试；tests/e2e/empty-state.spec.ts：TC-085 慢速合成扫描在诊断页显示中间进展且完成后清除</x:v>
       </x:c>
       <x:c r="L90" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-SOP-001/002 本轮范围决议：TC-085 可独立于完整空窗证据先测真实扫描反馈和修复重试；需独立命名函数、专用临时库/用户目录，未运行前不写通过。</x:v>
+SOP-001/002 本轮范围决议：TC-085 可独立于完整空窗证据先测真实扫描反馈和修复重试；需独立命名函数、专用临时库/用户目录，未运行前不写通过。
+当前产品无取消入口和状态，自动绑定只验进度/重试；取消语义及测试见 docs/test-case-acceptance.md。</x:v>
       </x:c>
       <x:c r="M90" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。取消/续扫未实现，TC-085 整项待验；docs/validation.md 对应记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="320" customHeight="1">

</xml_diff>

<commit_message>
docs: scope service states and telemetry copy
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5de37a15c3584da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd1be8e0cde5446f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R484b6f83d2cf4150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R19e39c65484840e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf2ca425b6da64727"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R60deb1d913f34e90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R0ef9e64e5bbc4e7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra4b8d5a5e1be4788"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2721,7 +2721,8 @@
       </x:c>
       <x:c r="G94" s="58" t="str">
         <x:v>待注册、待验证（规划目标）
-与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。</x:v>
+与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。
+TC-088 增默认内置/未配置远端/远端离线拒权旧协议与恢复；配置来源须显式，状态与本地报表分离。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="85" customHeight="1">
@@ -2790,7 +2791,8 @@
         <x:v>关键文案与动作逐状态走查</x:v>
       </x:c>
       <x:c r="G97" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证（规划目标）
+TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="90" customHeight="1">
@@ -4156,7 +4158,8 @@
       </x:c>
       <x:c r="C51" s="55" t="str">
         <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。
-若某范围因用量冲突或上报协议不兼容而暂停同步，显示“待核对/未同步”及原因，不归入网络离线、零用量或扫描失败。</x:v>
+若某范围因用量冲突或上报协议不兼容而暂停同步，显示“待核对/未同步”及原因，不归入网络离线、零用量或扫描失败。
+服务状态须由主进程明确配置来源/类型判定，区分默认内置回环服务、未配置远端、远端已配置在线/离线/授权失败/旧协议、积压与待核对；不能仅从 hasToken 或 online 猜远端配置。设置页和页头须与真实服务状态一致，本地扫描/报表独立。</x:v>
       </x:c>
       <x:c r="D51" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4171,7 +4174,8 @@
         <x:v>TC-088</x:v>
       </x:c>
       <x:c r="H51" s="55" t="str">
-        <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 静态核对：ServerConnection 默认启动本机服务，status() 仅返回 url/online/error/hasToken；设置页统称未连接、页头离线写本机运行。仅规划修正，TC-088 未注册/未运行。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="150" customHeight="1">
@@ -4182,7 +4186,8 @@
         <x:v>窄窗口与无障碍精确值</x:v>
       </x:c>
       <x:c r="C52" s="58" t="str">
-        <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。</x:v>
+        <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
+设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。</x:v>
       </x:c>
       <x:c r="D52" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4197,7 +4202,8 @@
         <x:v>TC-089、TC-090、TC-091</x:v>
       </x:c>
       <x:c r="H52" s="58" t="str">
-        <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。</x:v>
+        <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="170" customHeight="1">
@@ -5602,7 +5608,8 @@
       </x:c>
       <x:c r="G60" s="55" t="str">
         <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。</x:v>
+REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。
+主进程增加可核的服务配置来源/类型状态，明确默认内置回环与远端未配置；远端已配置再分别报告连接、授权、协议、待传。UI 不用 hasToken=false 当未配置，不用在线内置服务冒充远端配置；修正设置页“未连接”和页头“本机运行”的歧义。TC-088 各状态独立模拟，保护本地报表。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="155" customHeight="1">
@@ -5625,7 +5632,8 @@
         <x:v>待开发；关联新 TC 待注册/待验证</x:v>
       </x:c>
       <x:c r="G61" s="58" t="str">
-        <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -9435,7 +9443,7 @@
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="320" customHeight="1">
+    <x:row r="93" ht="350" customHeight="1">
       <x:c r="A93" s="58" t="str">
         <x:v>TC-088</x:v>
       </x:c>
@@ -9454,12 +9462,14 @@
       <x:c r="F93" s="58" t="str">
         <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。
 追加用量冲突与旧上报协议不兼容两类状态，观察本地报表和服务状态。
-交叉回归来源重绑后在线与离线场景，核本地授权即时变化、服务旧 owner 聚合清除/待传。</x:v>
+交叉回归来源重绑后在线与离线场景，核本地授权即时变化、服务旧 owner 聚合清除/待传。
+追加默认内置回环服务、未显式配置远端、远端离线、拒权、旧协议不兼容与恢复；核主进程配置来源/服务类型，设置页和页头状态。</x:v>
       </x:c>
       <x:c r="G93" s="58" t="str">
         <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。
 本地统计仍可用；冲突/协议不兼容显示“待核对/未同步”及原因，不误写网络离线、零用量或扫描失败；与 TC-094 的服务快照结果一致。
-在线服务状态只在旧 owner 聚合已替换/清除后显示同步；离线保留本地报表正常和服务待传，恢复重试不上传旧队列。</x:v>
+在线服务状态只在旧 owner 聚合已替换/清除后显示同步；离线保留本地报表正常和服务待传，恢复重试不上传旧队列。
+hasToken=false 不能直接显示远端未配置，内置服务在线不能显示远端已配置；远端故障不得被“本机运行”遮蔽，未配置/离线/拒权/协议/待传各有正确状态且本地报表正常。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9475,7 +9485,8 @@
       </x:c>
       <x:c r="L93" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-与 TC-086/087 共享同一预期语义，但独立运行 TC-088；DEV-057 版本 2 授权和冲突口径须保持。</x:v>
+与 TC-086/087 共享同一预期语义，但独立运行 TC-088；DEV-057 版本 2 授权和冲突口径须保持。
+独立临时客户端/服务目录造默认内置与远端配置路径；当前只有 url/online/error/hasToken，无显式来源字段。静态发现，不算 TC-088 通过。</x:v>
       </x:c>
       <x:c r="M93" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
@@ -9563,7 +9574,7 @@
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="185" customHeight="1">
+    <x:row r="96" ht="300" customHeight="1">
       <x:c r="A96" s="55" t="str">
         <x:v>TC-091</x:v>
       </x:c>
@@ -9580,10 +9591,12 @@
         <x:v>Electron/人工</x:v>
       </x:c>
       <x:c r="F96" s="55" t="str">
-        <x:v>逐项触发首次引导、六类空状态、诊断重试与自动升级失败状态，核对文案及对应按钮。</x:v>
+        <x:v>逐项触发首次引导、六类空状态、诊断重试与自动升级失败状态，核对文案及对应按钮。
+追加设置页遥测说明、概览/报表/CSV 在不同 owner/会话与疑似重叠时的逐文案核对；触发相关下一步。</x:v>
       </x:c>
       <x:c r="G96" s="55" t="str">
-        <x:v>每条文案与实际状态、权限和可执行下一步一致；不把未配置服务、未知覆盖、更新失败写为采集为零或成功。</x:v>
+        <x:v>每条文案与实际状态、权限和可执行下一步一致；不把未配置服务、未知覆盖、更新失败写为采集为零或成功。
+不得再出现“同一天有本地记录时，报表采用本地记录”的整日覆盖承诺；说明独立事实保留、疑似重叠待核对、完整总量不可确认，实际动作可达。</x:v>
       </x:c>
       <x:c r="H96" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9598,7 +9611,8 @@
         <x:v>拟新增以 TC-091 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L96" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+当前 settings.tsx 仍有旧文案；与 DEV-057/TC-092–094 已实现调和结果对照，TC-091 未注册/未运行。</x:v>
       </x:c>
       <x:c r="M96" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: detail accessibility acceptance for third batch
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf2ca425b6da64727"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R60deb1d913f34e90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R0ef9e64e5bbc4e7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra4b8d5a5e1be4788"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rb7912f3385ac428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R113384ff6d84404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra5776e50c14a4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd71ef8045b2947b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2745,7 +2745,8 @@
         <x:v>窄窗口键盘与 VoiceOver 主路径</x:v>
       </x:c>
       <x:c r="G95" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证（规划目标）
+第三批：TC-089 键盘主路径、模态背景实际隔离、取消/Escape/失败回焦与目标 Mac VoiceOver 人工证据，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="85" customHeight="1">
@@ -2768,7 +2769,8 @@
         <x:v>精确 Token 与覆盖状态非悬浮可读</x:v>
       </x:c>
       <x:c r="G96" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>待注册、待验证（规划目标）
+第三批：TC-090 所有 Token 字段精确整数非 hover 可读、覆盖未知与小计 0 不造真零，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="85" customHeight="1">
@@ -2792,7 +2794,8 @@
       </x:c>
       <x:c r="G97" s="55" t="str">
         <x:v>待注册、待验证（规划目标）
-TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。</x:v>
+TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。
+第三批：TC-091 引导、空状态、诊断取消/重试、重绑/服务/更新及遥测冲突逐状态文案与动作，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="90" customHeight="1">
@@ -4187,7 +4190,8 @@
       </x:c>
       <x:c r="C52" s="58" t="str">
         <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
-设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。</x:v>
+设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。
+来源重绑预览弹窗须实际隔离背景键盘操作，焦点进入弹窗并留在其中；取消/Escape/失败后焦点回触发控件，成功刷新移除触发控件时回来源列表稳定标题。标准与窄窗口主路径焦点顺序可见。概览、趋势、排行、报表、明细所有 Token 精确整数及覆盖状态须非悬浮可读；引导、空状态、诊断、重绑、服务、更新文案与真实角色/状态/动作一致。</x:v>
       </x:c>
       <x:c r="D52" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4203,7 +4207,8 @@
       </x:c>
       <x:c r="H52" s="58" t="str">
         <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
-2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。</x:v>
+2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。
+2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="170" customHeight="1">
@@ -5633,7 +5638,8 @@
       </x:c>
       <x:c r="G61" s="58" t="str">
         <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。</x:v>
+修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。
+第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -9492,7 +9498,7 @@
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="185" customHeight="1">
+    <x:row r="94" ht="360" customHeight="1">
       <x:c r="A94" s="55" t="str">
         <x:v>TC-089</x:v>
       </x:c>
@@ -9509,10 +9515,12 @@
         <x:v>Electron/目标 Mac 人工</x:v>
       </x:c>
       <x:c r="F94" s="55" t="str">
-        <x:v>覆盖窄宽窗口、Tab/Shift+Tab、Enter/Escape、面包屑与主要控件；目标 Mac 用 VoiceOver 逐项朗读。</x:v>
+        <x:v>覆盖窄宽窗口、Tab/Shift+Tab、Enter/Escape、面包屑与主要控件；目标 Mac 用 VoiceOver 逐项朗读。
+标准与窄窗口仅键盘走登录→导航→来源重绑弹窗→概览下钻→明细返回→诊断/设置；Tab/Shift+Tab、Enter/Space、Escape。另在目标 Mac 用 VoiceOver 人工朗读名称、状态、错误和动作。</x:v>
       </x:c>
       <x:c r="G94" s="55" t="str">
-        <x:v>无控件遮挡，焦点可见、顺序与动作合理；名称/角色/状态可读，人工证据不由自动布局测试替代。</x:v>
+        <x:v>无控件遮挡，焦点可见、顺序与动作合理；名称/角色/状态可读，人工证据不由自动布局测试替代。
+焦点顺序随可见布局、始终可见且不被固定栏遮挡；重绑弹窗打开后焦点进入、Tab 不到背景，aria-modal 与真实行为一致。取消/Escape 无写入并回触发控件；失败错误可读，关闭回焦；成功触发控件消失时回来源列表稳定标题。VoiceOver 人工与 Electron 自动证据分别记录。</x:v>
       </x:c>
       <x:c r="H94" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9527,13 +9535,14 @@
         <x:v>拟新增以 TC-089 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L94" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+仅用键盘验证实际背景隔离，不以 aria-modal 属性存在代替；独立目标 Mac 记录系统版本、应用构建与脱敏朗读证据。</x:v>
       </x:c>
       <x:c r="M94" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="185" customHeight="1">
+    <x:row r="95" ht="360" customHeight="1">
       <x:c r="A95" s="58" t="str">
         <x:v>TC-090</x:v>
       </x:c>
@@ -9550,10 +9559,12 @@
         <x:v>Electron 端到端</x:v>
       </x:c>
       <x:c r="F95" s="58" t="str">
-        <x:v>无 hover、仅键盘/朗读方式查看概览、趋势、模型排行及明细。</x:v>
+        <x:v>无 hover、仅键盘/朗读方式查看概览、趋势、模型排行及明细。
+以 0、1023、1024、超过 1M、待核对合成事实，在无 hover 条件下查概览总量/输入输出、每个趋势桶、排行、报表指标、明细输入/输出/缓存/总量及覆盖状态。</x:v>
       </x:c>
       <x:c r="G95" s="58" t="str">
-        <x:v>精确原值与覆盖状态有可见文本或可聚焦可读入口，不仅藏在 title/tooltip。</x:v>
+        <x:v>精确原值与覆盖状态有可见文本或可聚焦可读入口，不仅藏在 title/tooltip。
+每个 Token 精确整数可见或在键盘可聚焦且有名称的详情入口读取；K/M/P 仅视觉摘要，title/tooltip 与 CSV 不可为唯一精确值来源。覆盖未知/总量不可确认可读，已确认小计 0 不作完整真零。</x:v>
       </x:c>
       <x:c r="H95" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9568,13 +9579,14 @@
         <x:v>拟新增以 TC-090 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
       </x:c>
       <x:c r="L95" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。</x:v>
+        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+当前 overview.tsx/report.tsx 多处精确值仅 title；核所有字段和边界值，不只看主指标。</x:v>
       </x:c>
       <x:c r="M95" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="300" customHeight="1">
+    <x:row r="96" ht="360" customHeight="1">
       <x:c r="A96" s="55" t="str">
         <x:v>TC-091</x:v>
       </x:c>
@@ -9592,11 +9604,13 @@
       </x:c>
       <x:c r="F96" s="55" t="str">
         <x:v>逐项触发首次引导、六类空状态、诊断重试与自动升级失败状态，核对文案及对应按钮。
-追加设置页遥测说明、概览/报表/CSV 在不同 owner/会话与疑似重叠时的逐文案核对；触发相关下一步。</x:v>
+追加设置页遥测说明、概览/报表/CSV 在不同 owner/会话与疑似重叠时的逐文案核对；触发相关下一步。
+建立状态/角色/动作表逐项触发引导、未扫描/权限/格式/筛选无匹配/覆盖未知/已观测未知、诊断取消/失败/重试、重绑失败、服务未配置/离线/待传、更新失败及遥测待核对。真零正例待 REQ-040 有完整覆盖证据另补。</x:v>
       </x:c>
       <x:c r="G96" s="55" t="str">
         <x:v>每条文案与实际状态、权限和可执行下一步一致；不把未配置服务、未知覆盖、更新失败写为采集为零或成功。
-不得再出现“同一天有本地记录时，报表采用本地记录”的整日覆盖承诺；说明独立事实保留、疑似重叠待核对、完整总量不可确认，实际动作可达。</x:v>
+不得再出现“同一天有本地记录时，报表采用本地记录”的整日覆盖承诺；说明独立事实保留、疑似重叠待核对、完整总量不可确认，实际动作可达。
+每条文案与实际状态和角色一致，按钮实际到达对应页面/操作；viewer 无管理员动作。未知/待核对不写成已确认零或完整成功，失败不写成成功；不能用虚构 complete 造真零。</x:v>
       </x:c>
       <x:c r="H96" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9612,7 +9626,8 @@
       </x:c>
       <x:c r="L96" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-当前 settings.tsx 仍有旧文案；与 DEV-057/TC-092–094 已实现调和结果对照，TC-091 未注册/未运行。</x:v>
+当前 settings.tsx 仍有旧文案；与 DEV-057/TC-092–094 已实现调和结果对照，TC-091 未注册/未运行。
+诊断取消当前尚未实现；TC-091 相关状态待实现后执行，不以现有重试自动测试替代。</x:v>
       </x:c>
       <x:c r="M96" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>

</xml_diff>

<commit_message>
docs: validate source rebinding implementation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rb7912f3385ac428e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R113384ff6d84404a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra5776e50c14a4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rd71ef8045b2947b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R26f6acbce3764bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra80027a4a3f842fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb2d0b3b1426149f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R7d334bf7fc594d47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2673,7 +2673,8 @@
       </x:c>
       <x:c r="G92" s="58" t="str">
         <x:v>TC-086 待注册/待验；草稿/授权预览、同筛选双 owner 可见范围、取消/Escape、确认、重扫后过期基线和 viewer 越权
-在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。</x:v>
+在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。
+代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -2697,7 +2698,8 @@
       </x:c>
       <x:c r="G93" s="55" t="str">
         <x:v>TC-087 待注册/待验；业务拒绝、事务/审计失败、数据库不可写、原子回滚与不透明审计引用及旧日志脱敏
-离线重绑须留新 revision/待传，旧 owner 队列失效，恢复后重试。</x:v>
+离线重绑须留新 revision/待传，旧 owner 队列失效，恢复后重试。
+代码 01a7095：TC-087 已注册，单元+Electron 自动子范围独立通过；回滚、旧日志合成迁移、离线新队列已证，生产迁移/打包待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="85" customHeight="1">
@@ -4130,7 +4132,7 @@
         <x:v>来源重新绑定预览确认与最小审计</x:v>
       </x:c>
       <x:c r="C50" s="58" t="str">
-        <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、来源稳定键、前后用户 ID、数量和结果码，不含路径/正文。
+        <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、持久随机不透明来源引用、前后用户 ID、数量和结果码，不含路径/正文。
 选择候选只留 UI 草稿；主进程预览须显示原/新 owner、来源全部受影响事实数及相同筛选下两侧授权可见事实范围/待核对状态。确认时在事务中复验权限、来源、目标活跃性、原 owner 和预览事实集合基线；重扫或目标变化后旧预览失效，须重取。取消/Escape 无写入；失败恢复 UI 原值并给可操作错误。审计只存持久随机不透明来源引用，不存原始 key/标签/路径/账号/正文；旧审计展示/导出前脱敏。
 重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。</x:v>
       </x:c>
@@ -4138,7 +4140,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E50" s="58" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>已实现；隔离自动子范围通过，生产库迁移/打包应用待验</x:v>
       </x:c>
       <x:c r="F50" s="58" t="str">
         <x:v>DEV-054</x:v>
@@ -4149,7 +4151,8 @@
       <x:c r="H50" s="58" t="str">
         <x:v>承接 REQ-011；归属与报表权限应在同一提交边界生效。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 SOP-001/002 实施前静态核对：当前来源下拉 onChange 立即 bind；scanner.identities().factCount 为来源全部 usage_facts 条数，不能当选定筛选后可见集；scanner.bindIdentity() 当前把原始 key 写 audit_events.target_id。新预览和审计白名单按 docs/design.md §20.3 实施，未改代码、未运行新用例。
-当前 sources:bind 只调用 bindIdentity，没有显式生成 usage-sync 新快照；TC-086/087 分别验在线旧 owner 清除和离线队列，TC-088 回归本地与服务状态分离。</x:v>
+当前 sources:bind 只调用 bindIdentity，没有显式生成 usage-sync 新快照；TC-086/087 分别验在线旧 owner 清除和离线队列，TC-088 回归本地与服务状态分离。
+2026-10-03 代码 01a7095：文档会话独立复跑 TC-086/087 各单元+Electron、TC-074/080/093 及完整门禁（90 入口、66 单元、30 Electron）通过。五分钟一次性预览/基线、耐久事务审计与 v2 新队列有隔离证据；真实生产库迁移、打包安装、TC-088/089 仍待验。此前待实现文字为阶段历史。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -5580,16 +5583,17 @@
         <x:v>TC-086、TC-087</x:v>
       </x:c>
       <x:c r="E59" s="58" t="str">
-        <x:v>src/main/database.ts、index.ts；src/renderer/index.tsx；受控 IPC；事务与 Electron 测试</x:v>
+        <x:v>src/main/source-binding.ts、database.ts、index.ts、usage-sync.ts；src/collectors/scanner.ts；src/server/server.ts；src/renderer/index.tsx、source-binding.tsx；tests/source-binding.test.ts、tests/e2e/source-binding.spec.ts</x:v>
       </x:c>
       <x:c r="F59" s="58" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>已开发；TC-086/087 已注册并通过隔离自动子范围，生产/打包待验</x:v>
       </x:c>
       <x:c r="G59" s="58" t="str">
         <x:v>预览受影响事实数/可见范围，确认后主进程复验权限和版本；事务提交归属及最小审计，失败不改变归属；审计不保存路径/正文。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 需求复核补充：成功绑定与最小审计同事务；业务拒绝可另记结果，DB 不可写时绑定不变且不得声称审计已持久化。
 实施前补充：改下拉为草稿→授权预览→确认，预览含原/新 owner、来源全体受影响事实数与同筛选两侧报表可见集合/待核对状态；带归属和事实集合的不可伪造基线。确认在事务内重验 actor、来源、活跃目标、旧 owner 与基线，重扫新增/改写事实须拒绝旧预览。成功归属+最小审计同事务并刷新 UI/报表；取消/Escape 无写入，失败 UI 回原值。审计引用用持久随机不透明 ID，历史 raw key 展示/导出前脱敏；DB 不可写时不宣称审计持久。TC-086/087 分别测一致性/权限与失败回滚/隐私。
-绑定成功后创建持久版本 2 新 revision/待传义务，停止上传旧 owner 队列；在线替换/清除旧 owner 服务聚合，离线显示本地已变而服务待传并可重试。不得回退 DEV-057 v2 授权/冲突口径，交叉回归 TC-088。</x:v>
+绑定成功后创建持久版本 2 新 revision/待传义务，停止上传旧 owner 队列；在线替换/清除旧 owner 服务聚合，离线显示本地已变而服务待传并可重试。不得回退 DEV-057 v2 授权/冲突口径，交叉回归 TC-088。
+代码 01a7095 已实现草稿→预览→确认、五分钟一次性基线、主进程重验、耐久事务归属+不透明审计+v2 新 outbox。旧审计原始 key 初始化迁移；在线清设备历史授权旧 owner 聚合、保留历史未授权行，离线新 revision 替换旧队列；审计/磁盘失败回滚。文档会话独立复验 TC-086/087、TC-074/080/093 与完整门禁通过。生产库迁移、打包应用、TC-088/089 尚未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -9355,7 +9359,7 @@
         <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。取消/续扫未实现，TC-085 整项待验；docs/validation.md 对应记录。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="320" customHeight="1">
+    <x:row r="91" ht="380" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9382,27 +9386,28 @@
 预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；单元+Electron 自动子范围通过，完整键盘/生产打包待验</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
       </x:c>
       <x:c r="J91" s="58" t="str">
-        <x:v>npm run test:case -- TC-086（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-086（2026-10-03 独立通过）</x:v>
       </x:c>
       <x:c r="K91" s="58" t="str">
-        <x:v>拟新增以 TC-086 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/source-binding.test.ts：TC-086 预览双侧授权范围取消过期和在线确认清除旧归属；tests/e2e/source-binding.spec.ts：TC-086 草稿预览键盘取消与确认后权限转移</x:v>
       </x:c>
       <x:c r="L91" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 UI 下拉 onChange 直绑，需改为草稿/预览/确认。来源全体条数与相同筛选可见事实数须分列；pending 不称已确认总量。用专用临时库并在预览后注入新扫描/目标状态变化检验竞态，未实施前不登记通过。
-用独立测试服务和合成聚合核对在线同步；不把本地成功等同服务成功。</x:v>
+用独立测试服务和合成聚合核对在线同步；不把本地成功等同服务成功。
+在线服务旧 owner 聚合清理由隔离服务器验证；UI 仅测少量 Tab/Escape，完整背景隔离/失败回焦和目标 Mac VoiceOver 属 TC-089。未测打包 App。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92" ht="320" customHeight="1">
+        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="380" customHeight="1">
       <x:c r="A92" s="55" t="str">
         <x:v>TC-087</x:v>
       </x:c>
@@ -9416,7 +9421,7 @@
         <x:v>来源重绑失败回滚与最小审计</x:v>
       </x:c>
       <x:c r="E92" s="55" t="str">
-        <x:v>集成</x:v>
+        <x:v>单元/Electron</x:v>
       </x:c>
       <x:c r="F92" s="55" t="str">
         <x:v>在业务规则拒绝、事务写入失败及数据库不可写处分别注入异常，检查归属/报表；成功路径检查审计字段。
@@ -9429,24 +9434,25 @@
 本地重绑成功但服务离线时分别显示本地已变和服务待传/重试；恢复后按版本 2 口径上传，旧 owner 聚合清除且旧快照不再发送。</x:v>
       </x:c>
       <x:c r="H92" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；单元+Electron 自动子范围通过，生产迁移/打包待验</x:v>
       </x:c>
       <x:c r="I92" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。TC-074 回归证明历史未授权服务行保留；完整门禁 90 入口、66 单元、30 Electron 通过。此前“待注册/不可运行”为实施前历史。</x:v>
       </x:c>
       <x:c r="J92" s="55" t="str">
-        <x:v>npm run test:case -- TC-087（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-087（2026-10-03 独立通过）</x:v>
       </x:c>
       <x:c r="K92" s="55" t="str">
-        <x:v>拟新增以 TC-087 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/source-binding.test.ts：TC-087 停用旧归属仍可迁出事务故障回滚离线新快照覆盖旧队列；tests/e2e/source-binding.spec.ts：TC-087 预览后重扫变化确认拒绝且界面恢复旧归属</x:v>
       </x:c>
       <x:c r="L92" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 scanner.bindIdentity() 当前 audit_events.target_id 写原始 key，是需修正的旧行为；旧行任何展示/导出前也须脱敏。独立合成用户/来源，不提交真实账户、路径、会话正文或凭证；测试注入失败后清理。
-模拟断网、旧队列与恢复，审计与同步失败分别断言，DEV-057 v2 冲突口径保持。</x:v>
+模拟断网、旧队列与恢复，审计与同步失败分别断言，DEV-057 v2 冲突口径保持。
+旧审计原始 key 仅以隔离合成旧行验证初始化迁移；注入审计和磁盘持久化失败并验回滚，离线新 v2 队列恢复。真实生产库迁移/打包未验。</x:v>
       </x:c>
       <x:c r="M92" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产库迁移、打包应用未验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="350" customHeight="1">

</xml_diff>

<commit_message>
docs: review service states and keyboard copy gaps
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R26f6acbce3764bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra80027a4a3f842fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb2d0b3b1426149f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R7d334bf7fc594d47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rbde08366f00e49fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf7364048ca5349ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2fb0f44ced504652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf06258e3b3784175"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2724,7 +2724,8 @@
       <x:c r="G94" s="58" t="str">
         <x:v>待注册、待验证（规划目标）
 与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。
-TC-088 增默认内置/未配置远端/远端离线拒权旧协议与恢复；配置来源须显式，状态与本地报表分离。</x:v>
+TC-088 增默认内置/未配置远端/远端离线拒权旧协议与恢复；配置来源须显式，状态与本地报表分离。
+基线 4b3ff02：TC-088 加当前 revision 与内置/远端、网络/认证/协议、待传/待核对、本地覆盖正交组合，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="85" customHeight="1">
@@ -2748,7 +2749,8 @@
       </x:c>
       <x:c r="G95" s="55" t="str">
         <x:v>待注册、待验证（规划目标）
-第三批：TC-089 键盘主路径、模态背景实际隔离、取消/Escape/失败回焦与目标 Mac VoiceOver 人工证据，待注册/待验。</x:v>
+第三批：TC-089 键盘主路径、模态背景实际隔离、取消/Escape/失败回焦与目标 Mac VoiceOver 人工证据，待注册/待验。
+基线 4b3ff02：TC-089 加重绑弹窗背景 VoiceOver 导航隔离；自动与人工证据分开，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="85" customHeight="1">
@@ -2772,7 +2774,8 @@
       </x:c>
       <x:c r="G96" s="58" t="str">
         <x:v>待注册、待验证（规划目标）
-第三批：TC-090 所有 Token 字段精确整数非 hover 可读、覆盖未知与小计 0 不造真零，待注册/待验。</x:v>
+第三批：TC-090 所有 Token 字段精确整数非 hover 可读、覆盖未知与小计 0 不造真零，待注册/待验。
+基线 4b3ff02：TC-090 加纯键盘复制所有 Token 精确整数与粘贴比对，未知不复制假零，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="85" customHeight="1">
@@ -2797,7 +2800,8 @@
       <x:c r="G97" s="55" t="str">
         <x:v>待注册、待验证（规划目标）
 TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。
-第三批：TC-091 引导、空状态、诊断取消/重试、重绑/服务/更新及遥测冲突逐状态文案与动作，待注册/待验。</x:v>
+第三批：TC-091 引导、空状态、诊断取消/重试、重绑/服务/更新及遥测冲突逐状态文案与动作，待注册/待验。
+基线 4b3ff02：TC-091 加服务正交组合与当前 revision 文案/动作，待注册/待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="90" customHeight="1">
@@ -4165,7 +4169,8 @@
       <x:c r="C51" s="55" t="str">
         <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。
 若某范围因用量冲突或上报协议不兼容而暂停同步，显示“待核对/未同步”及原因，不归入网络离线、零用量或扫描失败。
-服务状态须由主进程明确配置来源/类型判定，区分默认内置回环服务、未配置远端、远端已配置在线/离线/授权失败/旧协议、积压与待核对；不能仅从 hasToken 或 online 猜远端配置。设置页和页头须与真实服务状态一致，本地扫描/报表独立。</x:v>
+服务状态须由主进程明确配置来源/类型判定，区分默认内置回环服务、未配置远端、远端已配置在线/离线/授权失败/旧协议、积压与待核对；不能仅从 hasToken 或 online 猜远端配置。设置页和页头须与真实服务状态一致，本地扫描/报表独立。
+服务类型/显式远端配置、网络/认证/协议、当前 revision 待传/已确认、待核对聚合、本地扫描与历史覆盖为正交状态；旧 lastSuccess 或 pending=0 不能单独证明当前 revision 已同步。并存状态须同时可见。</x:v>
       </x:c>
       <x:c r="D51" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4181,7 +4186,8 @@
       </x:c>
       <x:c r="H51" s="55" t="str">
         <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
-2026-10-03 静态核对：ServerConnection 默认启动本机服务，status() 仅返回 url/online/error/hasToken；设置页统称未连接、页头离线写本机运行。仅规划修正，TC-088 未注册/未运行。</x:v>
+2026-10-03 静态核对：ServerConnection 默认启动本机服务，status() 仅返回 url/online/error/hasToken；设置页统称未连接、页头离线写本机运行。仅规划修正，TC-088 未注册/未运行。
+2026-10-03 基线 4b3ff02 静态核对：ServerStatus 无显式远端配置与当前 revision，UploadStatus.pending 为 outbox 批数、uncertainRows 为待核对聚合数，概览优先级文案隐藏并存状态。TC-088 组合待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="150" customHeight="1">
@@ -4194,7 +4200,8 @@
       <x:c r="C52" s="58" t="str">
         <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
 设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。
-来源重绑预览弹窗须实际隔离背景键盘操作，焦点进入弹窗并留在其中；取消/Escape/失败后焦点回触发控件，成功刷新移除触发控件时回来源列表稳定标题。标准与窄窗口主路径焦点顺序可见。概览、趋势、排行、报表、明细所有 Token 精确整数及覆盖状态须非悬浮可读；引导、空状态、诊断、重绑、服务、更新文案与真实角色/状态/动作一致。</x:v>
+来源重绑预览弹窗须实际隔离背景键盘操作，焦点进入弹窗并留在其中；取消/Escape/失败后焦点回触发控件，成功刷新移除触发控件时回来源列表稳定标题。标准与窄窗口主路径焦点顺序可见。概览、趋势、排行、报表、明细所有 Token 精确整数及覆盖状态须非悬浮可读；引导、空状态、诊断、重绑、服务、更新文案与真实角色/状态/动作一致。
+精确 Token 原始十进制整数还须能纯键盘复制；可选可选中文本或有字段/范围名称的复制按钮，带可读反馈和合理焦点。缩写、title 或 CSV 不是复制入口；未知/待核对不可复制假完整总量。重绑弹窗背景对辅助技术导航也不可达。</x:v>
       </x:c>
       <x:c r="D52" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4211,7 +4218,8 @@
       <x:c r="H52" s="58" t="str">
         <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。
-2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。</x:v>
+2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。
+2026-10-03 基线 4b3ff02 静态核对：概览/报表多处精确值只在 title，无纯键盘复制路径；弹窗目前仅少量 Tab/Escape 自动断言，VoiceOver 背景隔离待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="170" customHeight="1">
@@ -5618,7 +5626,8 @@
       <x:c r="G60" s="55" t="str">
         <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。
-主进程增加可核的服务配置来源/类型状态，明确默认内置回环与远端未配置；远端已配置再分别报告连接、授权、协议、待传。UI 不用 hasToken=false 当未配置，不用在线内置服务冒充远端配置；修正设置页“未连接”和页头“本机运行”的歧义。TC-088 各状态独立模拟，保护本地报表。</x:v>
+主进程增加可核的服务配置来源/类型状态，明确默认内置回环与远端未配置；远端已配置再分别报告连接、授权、协议、待传。UI 不用 hasToken=false 当未配置，不用在线内置服务冒充远端配置；修正设置页“未连接”和页头“本机运行”的歧义。TC-088 各状态独立模拟，保护本地报表。
+增加当前设备/owner 的最新 revision 确认与显式配置来源状态；同时呈现网络/认证/协议、待传、待核对及本地扫描/覆盖。TC-088 交叉测在线+待核对、离线+待传+待核对、拒权/旧协议+待传、恢复后 revision 已确认但仍待核对，以及本地覆盖未知/扫描失败与服务状态。旧 lastSuccess/pending=0 不作当前同步证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="155" customHeight="1">
@@ -5643,7 +5652,8 @@
       <x:c r="G61" s="58" t="str">
         <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。
-第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。</x:v>
+第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。
+为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -9455,7 +9465,7 @@
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产库迁移、打包应用未验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="350" customHeight="1">
+    <x:row r="93" ht="400" customHeight="1">
       <x:c r="A93" s="58" t="str">
         <x:v>TC-088</x:v>
       </x:c>
@@ -9475,13 +9485,15 @@
         <x:v>分别未配置服务、服务离线、恢复并补传；本机合成用量持续扫描。
 追加用量冲突与旧上报协议不兼容两类状态，观察本地报表和服务状态。
 交叉回归来源重绑后在线与离线场景，核本地授权即时变化、服务旧 owner 聚合清除/待传。
-追加默认内置回环服务、未显式配置远端、远端离线、拒权、旧协议不兼容与恢复；核主进程配置来源/服务类型，设置页和页头状态。</x:v>
+追加默认内置回环服务、未显式配置远端、远端离线、拒权、旧协议不兼容与恢复；核主进程配置来源/服务类型，设置页和页头状态。
+增加正交组合：内置本地/远端配置、在线+待核对、断网+待传+待核对、认证失败+待传、旧协议+待传、恢复后当前 revision 确认但待核对仍在；本地覆盖未知与服务在线、扫描失败与服务在线。</x:v>
       </x:c>
       <x:c r="G93" s="58" t="str">
         <x:v>未配置显示未配置而非故障；离线时本机覆盖/报表正常，积压与重试单列，恢复后状态正确。
 本地统计仍可用；冲突/协议不兼容显示“待核对/未同步”及原因，不误写网络离线、零用量或扫描失败；与 TC-094 的服务快照结果一致。
 在线服务状态只在旧 owner 聚合已替换/清除后显示同步；离线保留本地报表正常和服务待传，恢复重试不上传旧队列。
-hasToken=false 不能直接显示远端未配置，内置服务在线不能显示远端已配置；远端故障不得被“本机运行”遮蔽，未配置/离线/拒权/协议/待传各有正确状态且本地报表正常。</x:v>
+hasToken=false 不能直接显示远端未配置，内置服务在线不能显示远端已配置；远端故障不得被“本机运行”遮蔽，未配置/离线/拒权/协议/待传各有正确状态且本地报表正常。
+概览/设置同时展示服务类型、连接/认证/协议、当前 revision 待传/已确认、待核对、本地扫描/覆盖；旧 lastSuccess 或 pending=0 不误报当前同步，重绑后尤其检查。服务正常不证明本地历史完整，扫描失败不被服务在线遮蔽。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9498,13 +9510,14 @@
       <x:c r="L93" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 与 TC-086/087 共享同一预期语义，但独立运行 TC-088；DEV-057 版本 2 授权和冲突口径须保持。
-独立临时客户端/服务目录造默认内置与远端配置路径；当前只有 url/online/error/hasToken，无显式来源字段。静态发现，不算 TC-088 通过。</x:v>
+独立临时客户端/服务目录造默认内置与远端配置路径；当前只有 url/online/error/hasToken，无显式来源字段。静态发现，不算 TC-088 通过。
+独立临时客户端/服务记录设备/owner 的 revision 和服务应答；逐组合检查 UI 文案与真实状态，不只检查 pending 批数。当前缺主进程显式远端配置/当前 revision 状态，仍待实现。</x:v>
       </x:c>
       <x:c r="M93" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="360" customHeight="1">
+    <x:row r="94" ht="400" customHeight="1">
       <x:c r="A94" s="55" t="str">
         <x:v>TC-089</x:v>
       </x:c>
@@ -9522,11 +9535,13 @@
       </x:c>
       <x:c r="F94" s="55" t="str">
         <x:v>覆盖窄宽窗口、Tab/Shift+Tab、Enter/Escape、面包屑与主要控件；目标 Mac 用 VoiceOver 逐项朗读。
-标准与窄窗口仅键盘走登录→导航→来源重绑弹窗→概览下钻→明细返回→诊断/设置；Tab/Shift+Tab、Enter/Space、Escape。另在目标 Mac 用 VoiceOver 人工朗读名称、状态、错误和动作。</x:v>
+标准与窄窗口仅键盘走登录→导航→来源重绑弹窗→概览下钻→明细返回→诊断/设置；Tab/Shift+Tab、Enter/Space、Escape。另在目标 Mac 用 VoiceOver 人工朗读名称、状态、错误和动作。
+在重绑弹窗打开时分别用 Tab 与目标 Mac VoiceOver 导航尝试到达背景控件，并核关闭/失败回焦。</x:v>
       </x:c>
       <x:c r="G94" s="55" t="str">
         <x:v>无控件遮挡，焦点可见、顺序与动作合理；名称/角色/状态可读，人工证据不由自动布局测试替代。
-焦点顺序随可见布局、始终可见且不被固定栏遮挡；重绑弹窗打开后焦点进入、Tab 不到背景，aria-modal 与真实行为一致。取消/Escape 无写入并回触发控件；失败错误可读，关闭回焦；成功触发控件消失时回来源列表稳定标题。VoiceOver 人工与 Electron 自动证据分别记录。</x:v>
+焦点顺序随可见布局、始终可见且不被固定栏遮挡；重绑弹窗打开后焦点进入、Tab 不到背景，aria-modal 与真实行为一致。取消/Escape 无写入并回触发控件；失败错误可读，关闭回焦；成功触发控件消失时回来源列表稳定标题。VoiceOver 人工与 Electron 自动证据分别记录。
+背景在键盘及辅助技术导航均不可达；aria-modal 与实际隔离一致，不能只靠两次 Tab/Escape 断言推全路径通过。</x:v>
       </x:c>
       <x:c r="H94" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9542,13 +9557,14 @@
       </x:c>
       <x:c r="L94" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-仅用键盘验证实际背景隔离，不以 aria-modal 属性存在代替；独立目标 Mac 记录系统版本、应用构建与脱敏朗读证据。</x:v>
+仅用键盘验证实际背景隔离，不以 aria-modal 属性存在代替；独立目标 Mac 记录系统版本、应用构建与脱敏朗读证据。
+TC-086 现有 Electron 仅测少量 Tab/Escape；TC-089 的目标 Mac VoiceOver 背景隔离仍单列人工证据。</x:v>
       </x:c>
       <x:c r="M94" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="360" customHeight="1">
+    <x:row r="95" ht="400" customHeight="1">
       <x:c r="A95" s="58" t="str">
         <x:v>TC-090</x:v>
       </x:c>
@@ -9566,11 +9582,13 @@
       </x:c>
       <x:c r="F95" s="58" t="str">
         <x:v>无 hover、仅键盘/朗读方式查看概览、趋势、模型排行及明细。
-以 0、1023、1024、超过 1M、待核对合成事实，在无 hover 条件下查概览总量/输入输出、每个趋势桶、排行、报表指标、明细输入/输出/缓存/总量及覆盖状态。</x:v>
+以 0、1023、1024、超过 1M、待核对合成事实，在无 hover 条件下查概览总量/输入输出、每个趋势桶、排行、报表指标、明细输入/输出/缓存/总量及覆盖状态。
+对概览、趋势、排行、报表指标和明细所有 Token 字段，仅用键盘复制精确整数并粘贴核对；覆盖 0、1023、1024、超过 1M 和待核对。</x:v>
       </x:c>
       <x:c r="G95" s="58" t="str">
         <x:v>精确原值与覆盖状态有可见文本或可聚焦可读入口，不仅藏在 title/tooltip。
-每个 Token 精确整数可见或在键盘可聚焦且有名称的详情入口读取；K/M/P 仅视觉摘要，title/tooltip 与 CSV 不可为唯一精确值来源。覆盖未知/总量不可确认可读，已确认小计 0 不作完整真零。</x:v>
+每个 Token 精确整数可见或在键盘可聚焦且有名称的详情入口读取；K/M/P 仅视觉摘要，title/tooltip 与 CSV 不可为唯一精确值来源。覆盖未知/总量不可确认可读，已确认小计 0 不作完整真零。
+复制结果为当前授权范围该字段的原始十进制整数，不是 K/M/P、title 或整页文本；操作反馈可读且焦点合理。未知/总量不可确认时不提供假完整总量 0。</x:v>
       </x:c>
       <x:c r="H95" s="58" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>
@@ -9586,13 +9604,14 @@
       </x:c>
       <x:c r="L95" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
-当前 overview.tsx/report.tsx 多处精确值仅 title；核所有字段和边界值，不只看主指标。</x:v>
+当前 overview.tsx/report.tsx 多处精确值仅 title；核所有字段和边界值，不只看主指标。
+当前 title 是多处唯一精确值来源；需自动读取隔离剪贴板或等价粘贴结果，核每类字段及状态。</x:v>
       </x:c>
       <x:c r="M95" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" ht="360" customHeight="1">
+    <x:row r="96" ht="400" customHeight="1">
       <x:c r="A96" s="55" t="str">
         <x:v>TC-091</x:v>
       </x:c>
@@ -9611,12 +9630,14 @@
       <x:c r="F96" s="55" t="str">
         <x:v>逐项触发首次引导、六类空状态、诊断重试与自动升级失败状态，核对文案及对应按钮。
 追加设置页遥测说明、概览/报表/CSV 在不同 owner/会话与疑似重叠时的逐文案核对；触发相关下一步。
-建立状态/角色/动作表逐项触发引导、未扫描/权限/格式/筛选无匹配/覆盖未知/已观测未知、诊断取消/失败/重试、重绑失败、服务未配置/离线/待传、更新失败及遥测待核对。真零正例待 REQ-040 有完整覆盖证据另补。</x:v>
+建立状态/角色/动作表逐项触发引导、未扫描/权限/格式/筛选无匹配/覆盖未知/已观测未知、诊断取消/失败/重试、重绑失败、服务未配置/离线/待传、更新失败及遥测待核对。真零正例待 REQ-040 有完整覆盖证据另补。
+加入服务在线/离线/拒权/旧协议与待传/待核对、当前 revision、新旧成功时间及本地扫描覆盖的并存文案/动作。</x:v>
       </x:c>
       <x:c r="G96" s="55" t="str">
         <x:v>每条文案与实际状态、权限和可执行下一步一致；不把未配置服务、未知覆盖、更新失败写为采集为零或成功。
 不得再出现“同一天有本地记录时，报表采用本地记录”的整日覆盖承诺；说明独立事实保留、疑似重叠待核对、完整总量不可确认，实际动作可达。
-每条文案与实际状态和角色一致，按钮实际到达对应页面/操作；viewer 无管理员动作。未知/待核对不写成已确认零或完整成功，失败不写成成功；不能用虚构 complete 造真零。</x:v>
+每条文案与实际状态和角色一致，按钮实际到达对应页面/操作；viewer 无管理员动作。未知/待核对不写成已确认零或完整成功，失败不写成成功；不能用虚构 complete 造真零。
+并存状态均可辨，不能因一个优先级标签隐去其他故障/待核对；按钮指向对应修复路径，旧成功不得说新 revision 已同步。</x:v>
       </x:c>
       <x:c r="H96" s="55" t="str">
         <x:v>待注册、待验证（规划目标）</x:v>

</xml_diff>

<commit_message>
docs: validate scan cancellation and resumption
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rbde08366f00e49fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf7364048ca5349ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2fb0f44ced504652"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf06258e3b3784175"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rae5b377940be4421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re55ac8d246444bf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rde1412d7f6894933"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R60dff80b17814781"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2649,7 +2649,8 @@
         <x:v>长扫描进展与诊断重试</x:v>
       </x:c>
       <x:c r="G91" s="55" t="str">
-        <x:v>TC-085 已注册：单元+Electron 进度/修复重试子范围通过；取消/续扫未实现，整项待验</x:v>
+        <x:v>TC-085 已注册：单元+Electron 进度/修复重试子范围通过；取消/续扫未实现，整项待验
+90338f4：TC-085 已注册 5 单元+2 Electron，取消/续扫隔离自动目标独立通过；生产/打包未验，REQ-044 真零仍待 TC-084/REQ-040。</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="85" customHeight="1">
@@ -4114,7 +4115,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E49" s="55" t="str">
-        <x:v>部分实现；保守空状态与进度/重试自动子范围通过，真零及取消待验</x:v>
+        <x:v>部分实现；保守空状态与进度/取消/重试自动子范围通过，真零待 REQ-040 证据</x:v>
       </x:c>
       <x:c r="F49" s="55" t="str">
         <x:v>DEV-053</x:v>
@@ -4125,7 +4126,8 @@
       <x:c r="H49" s="55" t="str">
         <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。
-2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。</x:v>
+2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。
+2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5569,12 +5571,13 @@
         <x:v>src/collectors/scanner.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；状态测试</x:v>
       </x:c>
       <x:c r="F58" s="55" t="str">
-        <x:v>部分实现；TC-084/085 已注册，保守子范围通过，真零与取消待补</x:v>
+        <x:v>部分实现；TC-085 进度/取消/续扫隔离自动目标通过，TC-084 真零待证</x:v>
       </x:c>
       <x:c r="G58" s="55" t="str">
         <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。
-代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。</x:v>
+代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。
+90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -9322,7 +9325,7 @@
         <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。REQ-040 尚无 complete 证据，TC-084 整项待验；docs/validation.md 对应记录。</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" ht="340" customHeight="1">
+    <x:row r="90" ht="410" customHeight="1">
       <x:c r="A90" s="55" t="str">
         <x:v>TC-085</x:v>
       </x:c>
@@ -9336,7 +9339,7 @@
         <x:v>长扫描进展与诊断重试</x:v>
       </x:c>
       <x:c r="E90" s="55" t="str">
-        <x:v>Electron 端到端</x:v>
+        <x:v>单元/Electron</x:v>
       </x:c>
       <x:c r="F90" s="55" t="str">
         <x:v>慢速合成扫描、阶段停顿、解析错误及随后修复重试。
@@ -9349,24 +9352,25 @@
 取消后不接收新文件，当前文件事实/游标原子完成；本轮为已取消/覆盖未知，不作完整成功或完整同步；从游标续跑且不并发。若立即中断单文件，该文件事实/游标均回滚。</x:v>
       </x:c>
       <x:c r="H90" s="55" t="str">
-        <x:v>已注册；真实进度与修复重试自动子范围通过，取消/续扫未实现，整项待验</x:v>
+        <x:v>已注册；5 单元+2 Electron 隔离自动目标通过，生产/打包待验</x:v>
       </x:c>
       <x:c r="I90" s="55" t="str">
-        <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。当前无取消 IPC/UI/扫描器状态，此前“待注册/不可运行”是实施前记录。</x:v>
+        <x:v>2026-10-03 文档会话在代码 90338f4、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：TC-085 单元 5/5、Electron 2/2，退出码 0；TC-087 回归通过，完整门禁 90 入口、70 单元、31 Electron 通过。旧“取消未实现”为 000372b 阶段事实。</x:v>
       </x:c>
       <x:c r="J90" s="55" t="str">
-        <x:v>npm run test:case -- TC-085（2026-10-03 进度/重试子范围通过）</x:v>
+        <x:v>npm run test:case -- TC-085（2026-10-03 独立通过）</x:v>
       </x:c>
       <x:c r="K90" s="55" t="str">
-        <x:v>tests/m6-diagnostics.test.ts：TC-085 慢扫描真实处理数及解析失败修复重试；tests/e2e/empty-state.spec.ts：TC-085 慢速合成扫描在诊断页显示中间进展且完成后清除</x:v>
+        <x:v>tests/m6-diagnostics.test.ts：TC-085 真实进度/修复重试、当前文件提交后取消续扫、第二工具取消、目录发现取消、文件落盘失败回滚，共 5 单元；tests/e2e/empty-state.spec.ts：TC-085 进度与 viewer IPC、取消 UI/覆盖未知/重扫，共 2 Electron</x:v>
       </x:c>
       <x:c r="L90" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 SOP-001/002 本轮范围决议：TC-085 可独立于完整空窗证据先测真实扫描反馈和修复重试；需独立命名函数、专用临时库/用户目录，未运行前不写通过。
-当前产品无取消入口和状态，自动绑定只验进度/重试；取消语义及测试见 docs/test-case-acceptance.md。</x:v>
+当前产品无取消入口和状态，自动绑定只验进度/重试；取消语义及测试见 docs/test-case-acceptance.md。
+已用合成慢文件和注入落盘失败验事实/游标一致、停止后续文件/工具、取消不触发完整上报；未测真实生产库、打包 App 或系统强制终止。</x:v>
       </x:c>
       <x:c r="M90" s="55" t="str">
-        <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。取消/续扫未实现，TC-085 整项待验；docs/validation.md 对应记录。</x:v>
+        <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="380" customHeight="1">

</xml_diff>

<commit_message>
docs: validate service status and telemetry copy scope
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rae5b377940be4421"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re55ac8d246444bf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rde1412d7f6894933"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R60dff80b17814781"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra86c223b860b41e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R122a03d302a24af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce4caa6c66ff43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re948103e5e2b489d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="68">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -405,6 +405,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2722,11 +2728,13 @@
       <x:c r="F94" s="58" t="str">
         <x:v>本机采集与可选服务状态分离</x:v>
       </x:c>
-      <x:c r="G94" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）
+      <x:c r="G94" s="68" t="str">
+        <x:v>当前：TC-088 已注册，6 单元+2 Electron 隔离自动通过；重绑提示误报风险及真实远端/打包待验。
+待注册、待验证（规划目标）
 与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。
 TC-088 增默认内置/未配置远端/远端离线拒权旧协议与恢复；配置来源须显式，状态与本地报表分离。
-基线 4b3ff02：TC-088 加当前 revision 与内置/远端、网络/认证/协议、待传/待核对、本地覆盖正交组合，待注册/待验。</x:v>
+基线 4b3ff02：TC-088 加当前 revision 与内置/远端、网络/认证/协议、待传/待核对、本地覆盖正交组合，待注册/待验。
+当前代码 41838d8：TC-088 已注册并独立通过 6 单元+2 Electron；服务状态自动子范围通过，重绑提示 pending=0 误报风险、真实远端与打包仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="85" customHeight="1">
@@ -2798,11 +2806,13 @@
       <x:c r="F97" s="55" t="str">
         <x:v>关键文案与动作逐状态走查</x:v>
       </x:c>
-      <x:c r="G97" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）
+      <x:c r="G97" s="69" t="str">
+        <x:v>当前：TC-091 已注册，1 单元+1 Electron 遥测说明子范围通过；完整文案矩阵待验，TC-089/090 未注册。
+待注册、待验证（规划目标）
 TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。
 第三批：TC-091 引导、空状态、诊断取消/重试、重绑/服务/更新及遥测冲突逐状态文案与动作，待注册/待验。
-基线 4b3ff02：TC-091 加服务正交组合与当前 revision 文案/动作，待注册/待验。</x:v>
+基线 4b3ff02：TC-091 加服务正交组合与当前 revision 文案/动作，待注册/待验。
+当前代码 41838d8：TC-091 已注册并独立通过 1 单元+1 Electron，仅遥测说明与冲突报表/CSV v2 子范围；其余文案矩阵待验，TC-089/090 未注册。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="90" customHeight="1">
@@ -4178,7 +4188,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E51" s="55" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>部分实现；TC-088 隔离自动子范围通过，待提示缺口修复与发布验收</x:v>
       </x:c>
       <x:c r="F51" s="55" t="str">
         <x:v>DEV-055</x:v>
@@ -4189,7 +4199,8 @@
       <x:c r="H51" s="55" t="str">
         <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态核对：ServerConnection 默认启动本机服务，status() 仅返回 url/online/error/hasToken；设置页统称未连接、页头离线写本机运行。仅规划修正，TC-088 未注册/未运行。
-2026-10-03 基线 4b3ff02 静态核对：ServerStatus 无显式远端配置与当前 revision，UploadStatus.pending 为 outbox 批数、uncertainRows 为待核对聚合数，概览优先级文案隐藏并存状态。TC-088 组合待验。</x:v>
+2026-10-03 基线 4b3ff02 静态核对：ServerStatus 无显式远端配置与当前 revision，UploadStatus.pending 为 outbox 批数、uncertainRows 为待核对聚合数，概览优先级文案隐藏并存状态。TC-088 组合待验。
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-088 6 单元+2 Electron。重绑提示仍有 pending=0 未核 currentConfirmed 的误报风险，待修并补回归。</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="150" customHeight="1">
@@ -4209,7 +4220,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E52" s="58" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>部分实现；TC-091 遥测说明子范围通过，整项待验</x:v>
       </x:c>
       <x:c r="F52" s="58" t="str">
         <x:v>DEV-056</x:v>
@@ -4221,7 +4232,8 @@
         <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。
 2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。
-2026-10-03 基线 4b3ff02 静态核对：概览/报表多处精确值只在 title，无纯键盘复制路径；弹窗目前仅少量 Tab/Escape 自动断言，VoiceOver 背景隔离待验。</x:v>
+2026-10-03 基线 4b3ff02 静态核对：概览/报表多处精确值只在 title，无纯键盘复制路径；弹窗目前仅少量 Tab/Escape 自动断言，VoiceOver 背景隔离待验。
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 1 单元+1 Electron；TC-089/090 未注册，TC-091 其余文案动作矩阵未覆盖。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="170" customHeight="1">
@@ -5624,13 +5636,14 @@
         <x:v>src/main/usage-sync.ts、server-connection.ts；src/renderer/overview.tsx、settings.tsx；离线测试</x:v>
       </x:c>
       <x:c r="F60" s="55" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>已实现服务状态子范围；TC-088 隔离自动通过，待提示缺口修复与发布验收</x:v>
       </x:c>
       <x:c r="G60" s="55" t="str">
         <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。
 主进程增加可核的服务配置来源/类型状态，明确默认内置回环与远端未配置；远端已配置再分别报告连接、授权、协议、待传。UI 不用 hasToken=false 当未配置，不用在线内置服务冒充远端配置；修正设置页“未连接”和页头“本机运行”的歧义。TC-088 各状态独立模拟，保护本地报表。
-增加当前设备/owner 的最新 revision 确认与显式配置来源状态；同时呈现网络/认证/协议、待传、待核对及本地扫描/覆盖。TC-088 交叉测在线+待核对、离线+待传+待核对、拒权/旧协议+待传、恢复后 revision 已确认但仍待核对，以及本地覆盖未知/扫描失败与服务状态。旧 lastSuccess/pending=0 不作当前同步证据。</x:v>
+增加当前设备/owner 的最新 revision 确认与显式配置来源状态；同时呈现网络/认证/协议、待传、待核对及本地扫描/覆盖。TC-088 交叉测在线+待核对、离线+待传+待核对、拒权/旧协议+待传、恢复后 revision 已确认但仍待核对，以及本地覆盖未知/扫描失败与服务状态。旧 lastSuccess/pending=0 不作当前同步证据。
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 主进程配置来源/类型、授权/协议、当前 revision 确认与 UI 正交状态已落地；重绑提示仍仅凭 pending=0 可误报服务端已同步，须补 currentConfirmed 守卫和 TC-088 断言。</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="155" customHeight="1">
@@ -5650,13 +5663,14 @@
         <x:v>src/renderer/、style.css；Electron 键盘/布局测试；目标 Mac VoiceOver 人工证据</x:v>
       </x:c>
       <x:c r="F61" s="58" t="str">
-        <x:v>待开发；关联新 TC 待注册/待验证</x:v>
+        <x:v>遥测说明子范围已实现并通过；键盘/VoiceOver/精确值及完整文案矩阵待开发验收</x:v>
       </x:c>
       <x:c r="G61" s="58" t="str">
         <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。
 第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。
-为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。</x:v>
+为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 遥测文案与疑似重叠报表/CSV v2 已测；TC-089/090 未注册。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -9500,25 +9514,26 @@
 概览/设置同时展示服务类型、连接/认证/协议、当前 revision 待传/已确认、待核对、本地扫描/覆盖；旧 lastSuccess 或 pending=0 不误报当前同步，重绑后尤其检查。服务正常不证明本地历史完整，扫描失败不被服务在线遮蔽。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；隔离自动子范围通过，整项待补验</x:v>
       </x:c>
       <x:c r="I93" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
       </x:c>
       <x:c r="J93" s="58" t="str">
-        <x:v>npm run test:case -- TC-088（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-088（2026-10-03 实测退出码 0）</x:v>
       </x:c>
       <x:c r="K93" s="58" t="str">
-        <x:v>拟新增以 TC-088 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/service-state.test.ts：6 个 TC-088 单元；tests/e2e/service-state.spec.ts：2 个 TC-088 Electron；scripts/test-cases.mjs 已注册。</x:v>
       </x:c>
       <x:c r="L93" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 与 TC-086/087 共享同一预期语义，但独立运行 TC-088；DEV-057 版本 2 授权和冲突口径须保持。
 独立临时客户端/服务目录造默认内置与远端配置路径；当前只有 url/online/error/hasToken，无显式来源字段。静态发现，不算 TC-088 通过。
-独立临时客户端/服务记录设备/owner 的 revision 和服务应答；逐组合检查 UI 文案与真实状态，不只检查 pending 批数。当前缺主进程显式远端配置/当前 revision 状态，仍待实现。</x:v>
+独立临时客户端/服务记录设备/owner 的 revision 和服务应答；逐组合检查 UI 文案与真实状态，不只检查 pending 批数。当前缺主进程显式远端配置/当前 revision 状态，仍待实现。
+当前重绑提示仅凭 pending=0 可能误称已同步，未被本次绑定覆盖；须增加 currentConfirmed=false 且 pending=0 的 UI 回归。真实远端/生产库/打包应用未验。</x:v>
       </x:c>
       <x:c r="M93" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-088 6/6 单元、2/2 Electron；静态发现提示缺口，整项待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="400" customHeight="1">
@@ -9644,24 +9659,25 @@
 并存状态均可辨，不能因一个优先级标签隐去其他故障/待核对；按钮指向对应修复路径，旧成功不得说新 revision 已同步。</x:v>
       </x:c>
       <x:c r="H96" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>已注册；遥测说明与冲突报表/CSV v2 子范围通过，整项待验</x:v>
       </x:c>
       <x:c r="I96" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
       </x:c>
       <x:c r="J96" s="55" t="str">
-        <x:v>npm run test:case -- TC-091（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-091（2026-10-03 实测退出码 0）</x:v>
       </x:c>
       <x:c r="K96" s="55" t="str">
-        <x:v>拟新增以 TC-091 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/reconciliation.test.ts：1 个 TC-091 单元；tests/e2e/settings-copy.spec.ts：1 个 TC-091 Electron；scripts/test-cases.mjs 已注册。</x:v>
       </x:c>
       <x:c r="L96" s="55" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 settings.tsx 仍有旧文案；与 DEV-057/TC-092–094 已实现调和结果对照，TC-091 未注册/未运行。
-诊断取消当前尚未实现；TC-091 相关状态待实现后执行，不以现有重试自动测试替代。</x:v>
+诊断取消当前尚未实现；TC-091 相关状态待实现后执行，不以现有重试自动测试替代。
+引导、六类空状态、诊断取消/重试、重绑、服务、更新及逐角色动作矩阵未逐项绑定；真零正例待 REQ-040 覆盖证据。</x:v>
       </x:c>
       <x:c r="M96" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 1/1 单元、1/1 Electron；仅遥测说明及报表/CSV 冲突子范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="185" customHeight="1">

</xml_diff>

<commit_message>
docs: validate keyboard accessibility and exact token copy
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Ra86c223b860b41e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R122a03d302a24af4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce4caa6c66ff43a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re948103e5e2b489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R22e4a74d5c40453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R195ab0e84afc4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra1c7963f17ca47e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rdd6dd99c1d16402c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -639,7 +639,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>每行对应一条测试用例；编号明细、状态和证据见后三页。</x:v>
+        <x:v>代码 6a194ea：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2729,12 +2729,7 @@
         <x:v>本机采集与可选服务状态分离</x:v>
       </x:c>
       <x:c r="G94" s="68" t="str">
-        <x:v>当前：TC-088 已注册，6 单元+2 Electron 隔离自动通过；重绑提示误报风险及真实远端/打包待验。
-待注册、待验证（规划目标）
-与 TC-086/087 交叉回归重绑后在线旧 owner 清除、离线待传及本地/服务状态分离；仍待注册/待验。
-TC-088 增默认内置/未配置远端/远端离线拒权旧协议与恢复；配置来源须显式，状态与本地报表分离。
-基线 4b3ff02：TC-088 加当前 revision 与内置/远端、网络/认证/协议、待传/待核对、本地覆盖正交组合，待注册/待验。
-当前代码 41838d8：TC-088 已注册并独立通过 6 单元+2 Electron；服务状态自动子范围通过，重绑提示 pending=0 误报风险、真实远端与打包仍待验。</x:v>
+        <x:v>自动子范围通过；重绑误报已修；真实远端/打包待验</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="85" customHeight="1">
@@ -2756,10 +2751,8 @@
       <x:c r="F95" s="55" t="str">
         <x:v>窄窗口键盘与 VoiceOver 主路径</x:v>
       </x:c>
-      <x:c r="G95" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）
-第三批：TC-089 键盘主路径、模态背景实际隔离、取消/Escape/失败回焦与目标 Mac VoiceOver 人工证据，待注册/待验。
-基线 4b3ff02：TC-089 加重绑弹窗背景 VoiceOver 导航隔离；自动与人工证据分开，待注册/待验。</x:v>
+      <x:c r="G95" s="69" t="str">
+        <x:v>键盘自动子范围通过；VoiceOver 人工待验</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="85" customHeight="1">
@@ -2781,10 +2774,8 @@
       <x:c r="F96" s="58" t="str">
         <x:v>精确 Token 与覆盖状态非悬浮可读</x:v>
       </x:c>
-      <x:c r="G96" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）
-第三批：TC-090 所有 Token 字段精确整数非 hover 可读、覆盖未知与小计 0 不造真零，待注册/待验。
-基线 4b3ff02：TC-090 加纯键盘复制所有 Token 精确整数与粘贴比对，未知不复制假零，待注册/待验。</x:v>
+      <x:c r="G96" s="68" t="str">
+        <x:v>精确值复制自动子范围通过；打包/真实工具待验</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="85" customHeight="1">
@@ -2807,12 +2798,7 @@
         <x:v>关键文案与动作逐状态走查</x:v>
       </x:c>
       <x:c r="G97" s="69" t="str">
-        <x:v>当前：TC-091 已注册，1 单元+1 Electron 遥测说明子范围通过；完整文案矩阵待验，TC-089/090 未注册。
-待注册、待验证（规划目标）
-TC-091 增设置页旧“同日采用本地记录”文案修正及 owner/会话独立保留、疑似重叠待核对的逐状态验证。
-第三批：TC-091 引导、空状态、诊断取消/重试、重绑/服务/更新及遥测冲突逐状态文案与动作，待注册/待验。
-基线 4b3ff02：TC-091 加服务正交组合与当前 revision 文案/动作，待注册/待验。
-当前代码 41838d8：TC-091 已注册并独立通过 1 单元+1 Electron，仅遥测说明与冲突报表/CSV v2 子范围；其余文案矩阵待验，TC-089/090 未注册。</x:v>
+        <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="90" customHeight="1">
@@ -2920,7 +2906,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–039；REQ-006 / DEV-047 的 fallback 归并和大会话启动性能回归已在 0.3.4 本机候选验证；生产库仅用临时副本启动，真实安装/目标 Mac 待验。</x:v>
+        <x:v>REQ-001–048 共 48 条；状态与 DEV/TC 关联见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -4188,7 +4174,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E51" s="55" t="str">
-        <x:v>部分实现；TC-088 隔离自动子范围通过，待提示缺口修复与发布验收</x:v>
+        <x:v>部分实现；服务状态自动子范围通过，重绑误报已修，真实远端/打包待验</x:v>
       </x:c>
       <x:c r="F51" s="55" t="str">
         <x:v>DEV-055</x:v>
@@ -4196,8 +4182,9 @@
       <x:c r="G51" s="55" t="str">
         <x:v>TC-088</x:v>
       </x:c>
-      <x:c r="H51" s="55" t="str">
-        <x:v>承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+      <x:c r="H51" s="69" t="str">
+        <x:v>当前 6a194ea：重绑提示仅以 currentConfirmed 报当前版本获确认，TC-091 新单元+Electron 通过；REQ-046 真实远端/生产库/打包仍待验。
+承接 REQ-021/026；不得把服务状态算入本地历史覆盖。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态核对：ServerConnection 默认启动本机服务，status() 仅返回 url/online/error/hasToken；设置页统称未连接、页头离线写本机运行。仅规划修正，TC-088 未注册/未运行。
 2026-10-03 基线 4b3ff02 静态核对：ServerStatus 无显式远端配置与当前 revision，UploadStatus.pending 为 outbox 批数、uncertainRows 为待核对聚合数，概览优先级文案隐藏并存状态。TC-088 组合待验。
 2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-088 6 单元+2 Electron。重绑提示仍有 pending=0 未核 currentConfirmed 的误报风险，待修并补回归。</x:v>
@@ -4220,7 +4207,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E52" s="58" t="str">
-        <x:v>部分实现；TC-091 遥测说明子范围通过，整项待验</x:v>
+        <x:v>部分实现；TC-089/090/091 隔离自动子范围通过，人工 VoiceOver/真零/发布待验</x:v>
       </x:c>
       <x:c r="F52" s="58" t="str">
         <x:v>DEV-056</x:v>
@@ -4228,8 +4215,9 @@
       <x:c r="G52" s="58" t="str">
         <x:v>TC-089、TC-090、TC-091</x:v>
       </x:c>
-      <x:c r="H52" s="58" t="str">
-        <x:v>承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
+      <x:c r="H52" s="68" t="str">
+        <x:v>当前 6a194ea：TC-089 1 Electron、TC-090 2 Electron 与 TC-091 扩展组合独立通过；目标 Mac VoiceOver、REQ-040 真零及真实打包待验。
+承接 REQ-033 和更新状态；目标 Mac 人工可访问性证据与自动布局断言分开。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。
 2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。
 2026-10-03 基线 4b3ff02 静态核对：概览/报表多处精确值只在 title，无纯键盘复制路径；弹窗目前仅少量 Tab/Escape 自动断言，VoiceOver 背景隔离待验。
@@ -4307,7 +4295,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码落点以 2026-10-03 仓库为准；DEV-047 在 aa6d91b 修复 fallback 归并、7abd640 修复大会话启动性能，0.3.4 有自动与隔离生产库副本证据；DEV-048 的 0.3.3 设备授权证据保留。真实安装与目标环境待验。</x:v>
+        <x:v>DEV-001–057 共 57 项；状态与 REQ/TC 关联见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -5636,10 +5624,11 @@
         <x:v>src/main/usage-sync.ts、server-connection.ts；src/renderer/overview.tsx、settings.tsx；离线测试</x:v>
       </x:c>
       <x:c r="F60" s="55" t="str">
-        <x:v>已实现服务状态子范围；TC-088 隔离自动通过，待提示缺口修复与发布验收</x:v>
-      </x:c>
-      <x:c r="G60" s="55" t="str">
-        <x:v>未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+        <x:v>服务状态自动子范围已实现；重绑误报已修，真实远端/发布待验</x:v>
+      </x:c>
+      <x:c r="G60" s="69" t="str">
+        <x:v>当前 6a194ea：pending=0 但 currentConfirmed=false 不再提示服务端已同步，TC-091 单元+Electron 补证。
+未配置/已连接/离线/积压/重试单列服务状态；本地扫描与报表无服务仍可用，服务错误不覆盖本地来源状态。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 REQ-048 版本 2 快照如因冲突/协议不兼容暂停某范围上报，状态须明确“待核对/未同步”及原因；不与网络离线、无用量或扫描失败混同，TC-088 与 TC-094 联动回归。
 主进程增加可核的服务配置来源/类型状态，明确默认内置回环与远端未配置；远端已配置再分别报告连接、授权、协议、待传。UI 不用 hasToken=false 当未配置，不用在线内置服务冒充远端配置；修正设置页“未连接”和页头“本机运行”的歧义。TC-088 各状态独立模拟，保护本地报表。
 增加当前设备/owner 的最新 revision 确认与显式配置来源状态；同时呈现网络/认证/协议、待传、待核对及本地扫描/覆盖。TC-088 交叉测在线+待核对、离线+待传+待核对、拒权/旧协议+待传、恢复后 revision 已确认但仍待核对，以及本地覆盖未知/扫描失败与服务状态。旧 lastSuccess/pending=0 不作当前同步证据。
@@ -5663,10 +5652,11 @@
         <x:v>src/renderer/、style.css；Electron 键盘/布局测试；目标 Mac VoiceOver 人工证据</x:v>
       </x:c>
       <x:c r="F61" s="58" t="str">
-        <x:v>遥测说明子范围已实现并通过；键盘/VoiceOver/精确值及完整文案矩阵待开发验收</x:v>
-      </x:c>
-      <x:c r="G61" s="58" t="str">
-        <x:v>验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+        <x:v>键盘/精确值/文案自动子范围已实现；人工 VoiceOver 与发布验收待验</x:v>
+      </x:c>
+      <x:c r="G61" s="68" t="str">
+        <x:v>当前 6a194ea：TC-089 1180/760/700px 弹窗与焦点；TC-090 两项剪贴板原始整数；TC-091 组合回归。目标 Mac VoiceOver、可证真零及打包待验。
+验证窄宽窗口、Tab 顺序/焦点可见与角色动作；精确 Token 文本及状态非 hover-only；逐状态文案和按钮动作对照。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。
 第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。
 为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。
@@ -5745,7 +5735,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–094 已分配；TC-001–076、TC-079–081、TC-092–094 已注册（82 个），TC-077–078、TC-082–091 待注册（12 个）。TC-092–094 在 8157e2d 的自动子范围通过，完整边界见各行；TC-028/072 目标环境仍待人工证据。</x:v>
+        <x:v>TC-001–094 共 94 个编号，均已注册；人工与发布验收按各行证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -9514,7 +9504,7 @@
 概览/设置同时展示服务类型、连接/认证/协议、当前 revision 待传/已确认、待核对、本地扫描/覆盖；旧 lastSuccess 或 pending=0 不误报当前同步，重绑后尤其检查。服务正常不证明本地历史完整，扫描失败不被服务在线遮蔽。</x:v>
       </x:c>
       <x:c r="H93" s="58" t="str">
-        <x:v>已注册；隔离自动子范围通过，整项待补验</x:v>
+        <x:v>已注册；服务状态隔离自动子范围通过，重绑提示误报已修，真实环境待验</x:v>
       </x:c>
       <x:c r="I93" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
@@ -9532,8 +9522,9 @@
 独立临时客户端/服务记录设备/owner 的 revision 和服务应答；逐组合检查 UI 文案与真实状态，不只检查 pending 批数。当前缺主进程显式远端配置/当前 revision 状态，仍待实现。
 当前重绑提示仅凭 pending=0 可能误称已同步，未被本次绑定覆盖；须增加 currentConfirmed=false 且 pending=0 的 UI 回归。真实远端/生产库/打包应用未验。</x:v>
       </x:c>
-      <x:c r="M93" s="58" t="str">
-        <x:v>2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-088 6/6 单元、2/2 Electron；静态发现提示缺口，整项待补。</x:v>
+      <x:c r="M93" s="68" t="str">
+        <x:v>当前 6a194ea：TC-091 补证 pending=0/currentConfirmed=false 不报同步；TC-088 既有 6 单元+2 Electron 状态范围不变。
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-088 6/6 单元、2/2 Electron；静态发现提示缺口，整项待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="400" customHeight="1">
@@ -9563,24 +9554,26 @@
 背景在键盘及辅助技术导航均不可达；aria-modal 与实际隔离一致，不能只靠两次 Tab/Escape 断言推全路径通过。</x:v>
       </x:c>
       <x:c r="H94" s="55" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
-      </x:c>
-      <x:c r="I94" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>已注册；键盘/弹窗焦点隔离自动子范围通过，目标 Mac VoiceOver 待验</x:v>
+      </x:c>
+      <x:c r="I94" s="69" t="str">
+        <x:v>当前 6a194ea：文档会话单编号 Electron 1/1；1180/760/700px、弹窗背景 inert/aria-hidden、Tab/Escape、失败错误聚焦。
+2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
       </x:c>
       <x:c r="J94" s="55" t="str">
-        <x:v>npm run test:case -- TC-089（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-089（2026-10-03 独立实测退出码 0）</x:v>
       </x:c>
       <x:c r="K94" s="55" t="str">
-        <x:v>拟新增以 TC-089 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
-      </x:c>
-      <x:c r="L94" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+        <x:v>scripts/test-cases.mjs：tests/e2e/accessibility.spec.ts 1 个 TC-089 Electron 独立绑定。</x:v>
+      </x:c>
+      <x:c r="L94" s="69" t="str">
+        <x:v>当前自动边界：可访问树/键盘自动断言通过；目标 Mac VoiceOver 真实导航/朗读、整条主路径和打包 App 待验。
+只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 仅用键盘验证实际背景隔离，不以 aria-modal 属性存在代替；独立目标 Mac 记录系统版本、应用构建与脱敏朗读证据。
 TC-086 现有 Electron 仅测少量 Tab/Escape；TC-089 的目标 Mac VoiceOver 背景隔离仍单列人工证据。</x:v>
       </x:c>
       <x:c r="M94" s="55" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，TC-089 Electron 1/1 退出码 0；目标 Mac VoiceOver 脱敏人工证据待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="400" customHeight="1">
@@ -9610,24 +9603,26 @@
 复制结果为当前授权范围该字段的原始十进制整数，不是 K/M/P、title 或整页文本；操作反馈可读且焦点合理。未知/总量不可确认时不提供假完整总量 0。</x:v>
       </x:c>
       <x:c r="H95" s="58" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
-      </x:c>
-      <x:c r="I95" s="58" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>已注册；原始整数键盘复制隔离自动子范围通过，打包/真实工具待验</x:v>
+      </x:c>
+      <x:c r="I95" s="68" t="str">
+        <x:v>当前 6a194ea：文档会话单编号 Electron 2/2；实际剪贴板 0/1023/1024/1050000、字段 Tab 顺序、700px 无横溢、待核对/未知边界。
+2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
       </x:c>
       <x:c r="J95" s="58" t="str">
-        <x:v>npm run test:case -- TC-090（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-090（2026-10-03 独立实测退出码 0）</x:v>
       </x:c>
       <x:c r="K95" s="58" t="str">
-        <x:v>拟新增以 TC-090 开头的独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
-      </x:c>
-      <x:c r="L95" s="58" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+        <x:v>scripts/test-cases.mjs：tests/e2e/exact-tokens.spec.ts 2 个 TC-090 Electron 独立绑定。</x:v>
+      </x:c>
+      <x:c r="L95" s="68" t="str">
+        <x:v>当前自动边界：概览/趋势/排行/项目模型/报表指标/明细原始整数可复制；真实工具格式、打包 App 与目标 Mac 辅助技术待验。
+只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 overview.tsx/report.tsx 多处精确值仅 title；核所有字段和边界值，不只看主指标。
 当前 title 是多处唯一精确值来源；需自动读取隔离剪贴板或等价粘贴结果，核每类字段及状态。</x:v>
       </x:c>
       <x:c r="M95" s="58" t="str">
-        <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。</x:v>
+        <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，TC-090 Electron 2/2 退出码 0；无安装包或目标 Mac 人工证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="400" customHeight="1">
@@ -9659,25 +9654,27 @@
 并存状态均可辨，不能因一个优先级标签隐去其他故障/待核对；按钮指向对应修复路径，旧成功不得说新 revision 已同步。</x:v>
       </x:c>
       <x:c r="H96" s="55" t="str">
-        <x:v>已注册；遥测说明与冲突报表/CSV v2 子范围通过，整项待验</x:v>
-      </x:c>
-      <x:c r="I96" s="55" t="str">
-        <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+        <x:v>已注册；遥测/重绑提示及关联文案自动组合通过，真零与发布验收待验</x:v>
+      </x:c>
+      <x:c r="I96" s="69" t="str">
+        <x:v>当前 6a194ea：文档会话单编号退出码 0；新增 pending=0/currentConfirmed=false 单元与 Electron，复用引导/空状态/取消/重绑/服务/权限/更新/调和既有断言。
+2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
       </x:c>
       <x:c r="J96" s="55" t="str">
-        <x:v>npm run test:case -- TC-091（2026-10-03 实测退出码 0）</x:v>
+        <x:v>npm run test:case -- TC-091（2026-10-03 独立实测退出码 0）</x:v>
       </x:c>
       <x:c r="K96" s="55" t="str">
-        <x:v>tests/reconciliation.test.ts：1 个 TC-091 单元；tests/e2e/settings-copy.spec.ts：1 个 TC-091 Electron；scripts/test-cases.mjs 已注册。</x:v>
-      </x:c>
-      <x:c r="L96" s="55" t="str">
-        <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
+        <x:v>scripts/test-cases.mjs：原遥测说明 Electron，新增重绑提示单元+Electron，并串行绑定 TC-082/083/084/085/087/088/061/059/093 既有断言。</x:v>
+      </x:c>
+      <x:c r="L96" s="69" t="str">
+        <x:v>当前自动边界：复用既有用例防回退，未逐条证明全部状态×角色×动作矩阵；REQ-040 可证真零正例、人工与打包待验。
+只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 settings.tsx 仍有旧文案；与 DEV-057/TC-092–094 已实现调和结果对照，TC-091 未注册/未运行。
 诊断取消当前尚未实现；TC-091 相关状态待实现后执行，不以现有重试自动测试替代。
 引导、六类空状态、诊断取消/重试、重绑、服务、更新及逐角色动作矩阵未逐项绑定；真零正例待 REQ-040 覆盖证据。</x:v>
       </x:c>
       <x:c r="M96" s="55" t="str">
-        <x:v>2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 1/1 单元、1/1 Electron；仅遥测说明及报表/CSV 冲突子范围。</x:v>
+        <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，单编号退出码 0；完整门禁 94 入口、77 单元、38 Electron；真零与人工证据待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="185" customHeight="1">

</xml_diff>

<commit_message>
docs: validate real 0.3.5 to 0.3.6 upgrade
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R22e4a74d5c40453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R195ab0e84afc4250"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra1c7963f17ca47e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rdd6dd99c1d16402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R977c14bccc6a46b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd98389b4017a43d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re7210f36d0034c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R74be06d948ce408d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="70">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -410,6 +410,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -639,7 +642,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码 6a194ea：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。</x:v>
+        <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1459,7 +1462,7 @@
         <x:v>更新版本判断与下载校验</x:v>
       </x:c>
       <x:c r="G39" s="35" t="str">
-        <x:v>0.3.5 自动子范围通过；边界待验</x:v>
+        <x:v>0.3.6 TC-034 回归通过；异常边界待验</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="62" customHeight="1">
@@ -1482,7 +1485,7 @@
         <x:v>更新服务故障恢复</x:v>
       </x:c>
       <x:c r="G40" s="14" t="str">
-        <x:v>0.3.5 自动子范围通过；边界待验</x:v>
+        <x:v>0.3.6 TC-035 回归通过；异常边界待验</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="62" customHeight="1">
@@ -1505,7 +1508,7 @@
         <x:v>自动安装控制与回退</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>0.3.5 单元控制/回滚通过；真实制品边界待验</x:v>
+        <x:v>0.3.6 TC-036 合成回滚回归通过；打包故障待验</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2034,7 +2037,7 @@
         <x:v>更新入口可发现</x:v>
       </x:c>
       <x:c r="G64" s="36" t="str">
-        <x:v>0.3.5 自动 E2E 子范围通过；真实安装待验</x:v>
+        <x:v>0.3.6 TC-059 回归通过；真实安装状态待验</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="66" customHeight="1">
@@ -2057,7 +2060,7 @@
         <x:v>更新状态与失败恢复</x:v>
       </x:c>
       <x:c r="G65" s="37" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>0.3.6 TC-059 回归通过；真实安装状态待验</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="66" customHeight="1">
@@ -2448,7 +2451,7 @@
         <x:v>实际打包 App 隔离自动升级</x:v>
       </x:c>
       <x:c r="G82" s="52" t="str">
-        <x:v>已注册；合成旧版自动成功链路部分验证</x:v>
+        <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="85" customHeight="1">
@@ -3525,7 +3528,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>已编码（0.3.5 检查/下载与坏摘要拒绝自动通过；超时/空间不足等新增边界待验）</x:v>
+        <x:v>已编码；0.3.6 回归通过版本/摘要自动子范围，超时/空间不足等待验</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
         <x:v>DEV-024</x:v>
@@ -3533,8 +3536,9 @@
       <x:c r="G27" s="35" t="str">
         <x:v>TC-034、TC-035</x:v>
       </x:c>
-      <x:c r="H27" s="35" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
+      <x:c r="H27" s="69" t="str">
+        <x:v>当前 1e70412：TC-034/035 与 TC-059 独立回归退出码 0，TC-076 真实 DMG 成功链路通过；异常边界仍按各 TC 待验。
+docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
 2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。</x:v>
       </x:c>
     </x:row>
@@ -3552,7 +3556,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>0.3.5 自动安装代码已落地；合成旧版隔离成功链路/单元回滚通过，真实历史旧版一键过渡与环境边界待验</x:v>
+        <x:v>部分验证；真实 0.3.5→0.3.6 隔离自动成功，系统安装/打包故障回滚待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3560,8 +3564,9 @@
       <x:c r="G28" s="14" t="str">
         <x:v>TC-036、TC-076</x:v>
       </x:c>
-      <x:c r="H28" s="14" t="str">
-        <x:v>历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
+      <x:c r="H28" s="70" t="str">
+        <x:v>当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
+历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
 2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。</x:v>
       </x:c>
     </x:row>
@@ -4891,10 +4896,11 @@
         <x:v>src/main/update-client.ts；src/main/server-connection.ts；更新状态 IPC/界面；tests/next-update.test.ts；scripts/test-cases.mjs 的 TC-034/035 绑定</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
-        <x:v>0.3.5 已编码；TC-034/035/059 自动子范围通过，安装前异常边界待补</x:v>
-      </x:c>
-      <x:c r="G29" s="35" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。
+        <x:v>0.3.6 TC-034/035/059 自动回归通过；异常边界待补</x:v>
+      </x:c>
+      <x:c r="G29" s="69" t="str">
+        <x:v>当前 1e70412：文档会话独立复跑 TC-034/035/059，各 1/1 退出码 0；TC-076 的真实候选下载/摘要通过。
+自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。
 86a4b5b：客户端下载后校验大小/SHA-256 再交自动安装器，坏包不会触发 helper；文档会话 TC-034/035/059 与 76 入口检查退出码 0。超时/磁盘不足与真实用户错误恢复仍待验。</x:v>
       </x:c>
     </x:row>
@@ -4915,10 +4921,11 @@
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>0.3.5 已编码；单元回滚与合成旧版隔离自动成功通过；真实历史旧版/只读 DMG 及目标环境部分待验</x:v>
-      </x:c>
-      <x:c r="G30" s="14" t="str">
-        <x:v>历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
+        <x:v>真实 0.3.5→0.3.6 隔离自动成功链路通过；系统安装/打包故障回滚待验</x:v>
+      </x:c>
+      <x:c r="G30" s="70" t="str">
+        <x:v>当前 1e70412：文档会话构建 0.3.6 x64 目录包并以真实旧/新 DMG、固定哈希独立复跑 TC-076，exit 0；TC-036 2/2 合成单元回归通过。
+历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
 86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。</x:v>
       </x:c>
     </x:row>
@@ -7188,10 +7195,11 @@
         <x:v>只提示匹配的新版本；大小或摘要错误绝不启动安装，临时包清理。</x:v>
       </x:c>
       <x:c r="H39" s="35" t="str">
-        <x:v>0.3.5 自动子范围通过；大小/空间等边界待验</x:v>
-      </x:c>
-      <x:c r="I39" s="35" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：旧通过只覆盖当时的版本/架构/摘要与打开路径，不证明辅助进程从未收到坏包；新增断言待实现。
+        <x:v>0.3.6 自动回归 1/1 通过；原目标边界待验</x:v>
+      </x:c>
+      <x:c r="I39" s="69" t="str">
+        <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-034，1/1、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
+提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：旧通过只覆盖当时的版本/架构/摘要与打开路径，不证明辅助进程从未收到坏包；新增断言待实现。
 86a4b5b：文档会话单编号 TC-034 1/1 退出码 0，坏 SHA-256 无安装回调；版本/架构/摘要为合成包断言。</x:v>
       </x:c>
       <x:c r="J39" s="35" t="str">
@@ -7230,10 +7238,11 @@
         <x:v>错误阶段可见且可重试；无损坏临时包，旧版和本机报表继续可用。</x:v>
       </x:c>
       <x:c r="H40" s="14" t="str">
-        <x:v>0.3.5 自动子范围通过；超时/空间不足待验</x:v>
-      </x:c>
-      <x:c r="I40" s="14" t="str">
-        <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：原停服/重试通过仍有效于旧范围；超时、空间不足、取消和安装前状态/旧版可用性待新增断言。
+        <x:v>0.3.6 自动回归 1/1 通过；原目标边界待验</x:v>
+      </x:c>
+      <x:c r="I40" s="70" t="str">
+        <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-035，1/1、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
+提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md；2026-10-03 新目标：原停服/重试通过仍有效于旧范围；超时、空间不足、取消和安装前状态/旧版可用性待新增断言。
 86a4b5b：文档会话单编号 TC-035 1/1 退出码 0，停服下载失败后重试；未注入超时或磁盘空间不足。</x:v>
       </x:c>
       <x:c r="J40" s="14" t="str">
@@ -7272,10 +7281,11 @@
         <x:v>成功路径自动退出旧版、安装替换并启动新版；失败回滚旧版、保留用户数据、清理挂载/临时文件；权限不足不静默绕过，成功无需 Finder 拖拽。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>0.3.5 自动控制与回滚单元通过；真实历史旧版/制品故障边界待验</x:v>
-      </x:c>
-      <x:c r="I41" s="35" t="str">
-        <x:v>历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。
+        <x:v>0.3.6 合成控制/回滚单元 2/2 回归通过；打包故障回滚待验</x:v>
+      </x:c>
+      <x:c r="I41" s="69" t="str">
+        <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-036，2/2、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
+历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。
 86a4b5b：文档会话单编号 TC-036 两项 2/2 退出码 0：下载校验后交自动安装器及启动失败不退出旧版；合成 Bundle/命令覆盖 /Applications/~/Applications 选择、成功、挂载/复制/替换/重启/健康超时及篡改失败回滚。真实旧二进制、只读 DMG 实测及系统权限未由单元证明。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
@@ -8229,10 +8239,11 @@
         <x:v>每阶段状态准确，错误可恢复；坏包不打开，旧版可用。</x:v>
       </x:c>
       <x:c r="H64" s="36" t="str">
-        <x:v>0.3.5 自动 E2E 子范围通过；真实安装状态边界待验</x:v>
-      </x:c>
-      <x:c r="I64" s="36" t="str">
-        <x:v>提交 6223c30；2026-10-02 14:57:06 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-059.log
+        <x:v>0.3.6 自动回归 1/1 通过；原目标边界待验</x:v>
+      </x:c>
+      <x:c r="I64" s="68" t="str">
+        <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-059，1/1、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
+提交 6223c30；2026-10-02 14:57:06 UTC；darwin-x64 / Node v24.15.0；退出码 0；本机 test-results/acceptance/TC-059.log
 86a4b5b：文档会话单编号 TC-059 1/1 退出码 0；合成坏摘要显示错误，改清单后可重新检查；不执行真实 DMG 安装。</x:v>
       </x:c>
       <x:c r="J64" s="36" t="str">
@@ -8938,24 +8949,25 @@
         <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>已注册；部分验证（0.3.5 合成旧版打包 App 自动成功链路通过）</x:v>
-      </x:c>
-      <x:c r="I81" s="52" t="str">
-        <x:v>2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
+        <x:v>已注册；真实 0.3.5→0.3.6 DMG 隔离自动成功子范围通过，整项待环境/回滚</x:v>
+      </x:c>
+      <x:c r="I81" s="68" t="str">
+        <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
+2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
 86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="str">
-        <x:v>npm run test:case -- TC-076（已注册；文档会话 2026-10-03 退出码 0）</x:v>
+        <x:v>TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff npm run test:case -- TC-076</x:v>
       </x:c>
       <x:c r="K81" s="52" t="str">
-        <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；脚本在隔离目录用当前包复制并改版本元数据模拟前一补丁版本，再运行旧/新 App 自动升级成功链路。</x:v>
-      </x:c>
-      <x:c r="L81" s="52" t="str">
-        <x:v>0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。</x:v>
+        <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；给定 OLD_DMG/OLD_SHA256/NEW_DMG/NEW_SHA256 即验证真实旧/新 DMG；省略参数则为改版本元数据的合成旧版模式。</x:v>
+      </x:c>
+      <x:c r="L81" s="68" t="str">
+        <x:v>当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
+0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
-        <x:v>实施后保存旧/新 DMG SHA-256、macOS/架构、固定代码提交、单编号命令及退出码、脱敏启动/安装/回滚日志；不读取真实会话或生产数据库。真实签名/公证和其他目标 Mac 归 TC-028。
-文档会话独立复跑 TC-076 1/1、TC-036 2/2、TC-034/035/059 各 1/1 和 76 入口检查，均退出码 0；开发会话报告 test:gate 52 单元/18 E2E。0.3.5 未签名 DMG 只在当前 Mac 核验；真实签名公证、目标 Mac 属 TC-028。</x:v>
+        <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">

</xml_diff>

<commit_message>
docs: define scoped coverage evidence contract
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R977c14bccc6a46b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd98389b4017a43d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re7210f36d0034c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R74be06d948ce408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6f3bad9b332c4509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc922a8a12bae43c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rda7d290e335b4ada"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5e3ea7e8599a42b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2474,7 +2474,8 @@
         <x:v>所选范围覆盖真值表</x:v>
       </x:c>
       <x:c r="G83" s="55" t="str">
-        <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验</x:v>
+        <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验
+2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="85" customHeight="1">
@@ -2497,7 +2498,8 @@
         <x:v>区间比较可比性门禁</x:v>
       </x:c>
       <x:c r="G84" s="58" t="str">
-        <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验</x:v>
+        <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验
+2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -2635,7 +2637,8 @@
         <x:v>六类空状态与可操作下一步</x:v>
       </x:c>
       <x:c r="G90" s="58" t="str">
-        <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验</x:v>
+        <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验
+2026-10-03 覆盖证据决议：真零须已关闭同范围完整空窗；合成只验规则，真实来源未证；REQ-044/DEV-053/TC-084 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -3996,7 +3999,8 @@
       <x:c r="C45" s="55" t="str">
         <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。
 管理员选具体用户或“未归属”后，来源卡、报表 coverage、真零与比较只按该用户+所选工具/IANA 时区/区间的可证覆盖判定。全局 ready/计数/最近扫描时间只能另标“全局”诊断，不能补全选中范围；全局 ready 而所选用户空且缺证据时为未知/部分，不是已确认零。
-本轮部分范围：先按授权 owner（含未归属）+工具+IANA 时区+区间生成保守未知/可证部分覆盖；全局 ready/计数/时间、最早事实与成功空扫描都不构成完整证明。无事实不宣称已确认零；仅 pending 事实可显示已确认小计 0，但完整总量未知；比较不可比较。完整空窗真零和同 as-of 同口径同比正例待可证留存/连续采集方案。</x:v>
+本轮部分范围：先按授权 owner（含未归属）+工具+IANA 时区+区间生成保守未知/可证部分覆盖；全局 ready/计数/时间、最早事实与成功空扫描都不构成完整证明。无事实不宣称已确认零；仅 pending 事实可显示已确认小计 0，但完整总量未知；比较不可比较。完整空窗真零和同 as-of 同口径同比正例待可证留存/连续采集方案。
+2026-10-03 覆盖证据决议：仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。窗口关闭且同一事实集为空才可显示“已确认零（所选已监测来源）”；不得声称服务商账单或全设备零。比较需两窗等长、同范围/时区/as-of 且双方完整。</x:v>
       </x:c>
       <x:c r="D45" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4016,7 +4020,8 @@
 2026-10-03 静态检查 src/collectors/scanner.ts：source_status 只有当前状态、最近扫描/成功时间，source_cursors 只有现存文件偏移/更新时间；usage_facts 仅证已观察事件，均无历史留存起点/连续采集证明。SOP-001 部分范围已定义，未改代码或注册测试；完整正例由需求会话待决。
 2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。
 2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。
-3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。</x:v>
+3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。
+2026-10-03 覆盖证据决议：现有状态/游标/事实仅证已观察；受控合成正例只验规则，不证明真实 Codex/Claude 来源完整。真实来源机制未落实，整项仍待验。官方：https://learn.chatgpt.com/docs/developer-commands?surface=cli 与 https://code.claude.com/docs/en/monitoring-usage</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -4110,7 +4115,8 @@
       </x:c>
       <x:c r="C49" s="55" t="str">
         <x:v>真零、未扫描、权限不足、格式不支持、筛选无匹配和部分覆盖分别说明原因与下一步；诊断原因指向相应授权/重扫/调整筛选动作。长扫描持续显示阶段与最近进展，不伪造百分比，失败可重试。
-本轮只排可证的分型和行动：未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知及有已观测记录但完整性未知；真零保留为未来同一授权筛选范围 coverage.complete 且事实为空的受控分支。</x:v>
+本轮只排可证的分型和行动：未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知及有已观测记录但完整性未知；真零保留为未来同一授权筛选范围 coverage.complete 且事实为空的受控分支。
+2026-10-03 覆盖证据决议：真零依赖 REQ-040 的 仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。仅窗口关闭且同一授权筛选事实集为空可标限定真零。</x:v>
       </x:c>
       <x:c r="D49" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4128,7 +4134,8 @@
         <x:v>承接 REQ-010/036；服务上传故障不得误写为本机扫描失败。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。
 2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。
-2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。</x:v>
+2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。
+2026-10-03 覆盖证据决议：TC-084 可计划受控合成规则正例；真实来源完整性、范围外执行模式和实际空窗未验，REQ-044 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5484,7 +5491,8 @@
 管理员切换具体用户/未归属时，主进程提供按当前授权查询范围的覆盖证据供概览、报表及真零/同比门禁共用；全局扫描诊断另标“全局”并与筛选证据分开，不能以全局 ready、计数或时间证明所选用户完整。TC-077/078 用双 owner+未归属核 API/UI，空而缺证据时未知/部分。DEV-057 的管理员全局返回不构成此任务通过。
 下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。
 官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。
-2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。</x:v>
+2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。
+2026-10-03 覆盖证据决议：增加监测来源边界、留存起点、连续采集/重放水位、错误/缺口、归属和维度解析的可审计证据链，按所选范围判定；关闭空窗限定真零，双窗同口径且完整才比较。合成契约不得提升真实来源状态。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -5584,7 +5592,8 @@
         <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。
 代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。
-90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。</x:v>
+90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。
+2026-10-03 覆盖证据决议：真零 UI 仅消费经 REQ-040/DEV-049 证明的所选来源 complete、已关闭且同事实集为空；范围外模式仍未知。真实来源机制未交付前 DEV-053 整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -8990,12 +8999,14 @@
         <x:v>独立库构造 Codex/Claude 各用户跨历史缺口、成功空扫描、权限拒绝、留存未知；切换工具/用户/时区/区间。
 构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。
 本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。
-以无正文合成缺失输入模拟 Codex ephemeral 不落文件及 Claude OTel 未启用/exporter=none；核本地文件/OTel 缺记录仍未知，不宣称工具没用或真零。真实工具端到端验证另行安排。</x:v>
+以无正文合成缺失输入模拟 Codex ephemeral 不落文件及 Claude OTel 未启用/exporter=none；核本地文件/OTel 缺记录仍未知，不宣称工具没用或真零。真实工具端到端验证另行安排。
+2026-10-03 覆盖证据决议：计划受控合成正例：为所选 owner+provider+窗口逐项提供监测范围、留存起点、连续水位、无错误/缺口、归属及筛选维度证据；分别移除一项作降级反例，并核 API/概览/报表一致。真实工具来源另需独立证据。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
         <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
 B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。
-缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。</x:v>
+缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。
+2026-10-03 覆盖证据决议：仅完整证据链支持所选来源 complete；范围外模式未知。关闭且同事实集空才显示限定“已确认零（所选已监测来源）”，不推服务商账单/全设备零。合成正例不使真实历史通过。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
         <x:v>已注册；防假零保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
@@ -9017,12 +9028,14 @@
 当前 source_status/cursors/usage_facts 无历史留存起点及连续采集证明；最早事实、ready、成功空扫描不能制造 complete。部分负例通过后仍不得标 TC-077 整项通过。
 外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。
 现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。
-3bbaf15 已修正原“未归属”筛选下无事实 reason 的“已归属”措辞；仍不证明完整覆盖。</x:v>
+3bbaf15 已修正原“未归属”筛选下无事实 reason 的“已归属”措辞；仍不证明完整覆盖。
+2026-10-03 覆盖证据决议：现有保守负例结果保留。Codex --ephemeral 可无 rollout，Claude OTel 日志 exporter 可为 none；真实来源留存与连续性未证，TC-077 整项待验。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
 ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。
-3bbaf15；TC-077 单元 1/1、Electron 1/1、退出码 0；门禁 86 入口/62 unit/26 Electron 通过。</x:v>
+3bbaf15；TC-077 单元 1/1、Electron 1/1、退出码 0；门禁 86 入口/62 unit/26 Electron 通过。
+2026-10-03 覆盖证据决议：本次仅修订证据契约/计划，未执行新正例或真实来源验证；旧 c10bbf3/3bbaf15 子断言成绩保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="300" customHeight="1">
@@ -9044,12 +9057,14 @@
       <x:c r="F83" s="58" t="str">
         <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。
 管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。
-本轮先造管理员选定 owner/未归属两期、全局 ready 但选中范围缺证、今天进行中与扫描滞后；核 API/界面保持不可比较。完整同 as-of 正例等待证据方案。</x:v>
+本轮先造管理员选定 owner/未归属两期、全局 ready 但选中范围缺证、今天进行中与扫描滞后；核 API/界面保持不可比较。完整同 as-of 正例等待证据方案。
+2026-10-03 覆盖证据决议：计划受控合成双窗正例及单变量反例：两窗等长、同 owner/provider/筛选/来源范围、同 IANA 时区与 as-of 截止，双方各有完整证据链；破坏任一条件应不可比较。</x:v>
       </x:c>
       <x:c r="G83" s="58" t="str">
         <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。
 全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。
-没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。</x:v>
+没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。
+2026-10-03 覆盖证据决议：只有双方 source-complete 且双窗等长、同范围/时区/as-of 才显示比较；今天未结束、扫描滞后或范围外模式均不可比较。合成正例不证明真实历史。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
         <x:v>已注册；防假同比保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
@@ -9069,11 +9084,13 @@
 计划用例，未注册或执行；全局 as-of 与当前用户范围 as-of 必须区分。
 现有采集记录不能证明历史留存及连续采集；没有真实可得的同 as-of 双完整窗口，正向同比用例待需求会话决定证据来源。负例通过后整项仍待验证。
 TC-077 两类官方缺失来源反例存在时，两期均无记录仍不可比较；这些资料不提供同 as-of 双完整窗口的正例证据，正向同比继续待方案。
-Asia/Shanghai 与 UTC 边界、真实隔离 local/OTel 待核对 UI 子断言已过；仅 pending 时已确认小计 0 而完整总量未知，比较不可比。双完整窗口同 as-of 正例和扫描延迟证据仍未取得。</x:v>
+Asia/Shanghai 与 UTC 边界、真实隔离 local/OTel 待核对 UI 子断言已过；仅 pending 时已确认小计 0 而完整总量未知，比较不可比。双完整窗口同 as-of 正例和扫描延迟证据仍未取得。
+2026-10-03 覆盖证据决议：现有防假同比成绩保留；真实 Codex/Claude 双窗完整性机制及同截止证据未落实，TC-078 整项待验。</x:v>
       </x:c>
       <x:c r="M83" s="58" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
-ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。</x:v>
+ef7a3de、语义修正 c10bbf3；macOS x86_64 / Node 24.15.0；独立临时 SQLite/用户目录、无正文合成事实；单编号 unit 1/1、Electron 1/1、退出码 0；test:gate 84 入口/59 unit/24 Electron 通过。详见 docs/validation.md。
+2026-10-03 覆盖证据决议：本次仅修订验收计划，未执行新双完整窗口正例；旧 c10bbf3 子断言成绩保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="185" customHeight="1">
@@ -9314,11 +9331,13 @@
       </x:c>
       <x:c r="F89" s="58" t="str">
         <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。
-2026-10-03 本轮先逐项造未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知、已观测但完整性未知；核授权范围、文案与行动。真零正例等待可证完整空窗，不在本轮造数或注入 complete。</x:v>
+2026-10-03 本轮先逐项造未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知、已观测但完整性未知；核授权范围、文案与行动。真零正例等待可证完整空窗，不在本轮造数或注入 complete。
+2026-10-03 覆盖证据决议：计划受控合成正例须经 REQ-040 所选 owner+provider+窗口的完整证据链，窗口已关闭且同一授权筛选事实集为空；逐项撤证及范围外模式作为负例。真实来源另验。</x:v>
       </x:c>
       <x:c r="G89" s="58" t="str">
         <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。
-保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。</x:v>
+保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。
+2026-10-03 覆盖证据决议：仅显示限定“已确认零（所选已监测来源）”；不宣称服务商账单/全设备零。未关闭、待核对、缺证或范围外模式不得真零。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
         <x:v>已注册；保守空状态自动子范围通过，真零正例待 REQ-040 完整覆盖证据，整项待验</x:v>
@@ -9335,10 +9354,12 @@
       <x:c r="L89" s="58" t="str">
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 SOP-001/002 本轮范围决议：当前 REQ-040 没有完整空窗证据；不得用全局 ready、成功空扫描、空事实或伪造 complete 让“真零”通过。用隔离库和 Electron 分别检查各保守状态的原因、角色/筛选范围和实际行动。
-Electron 仅走筛选无匹配→清除→诊断；其他状态的逐类 UI 行动与真零正例未覆盖。</x:v>
+Electron 仅走筛选无匹配→清除→诊断；其他状态的逐类 UI 行动与真零正例未覆盖。
+2026-10-03 覆盖证据决议：保守空状态子断言通过记录保留；合成 complete 仅能验规则，真实 Codex/Claude 来源完整性机制未落实，TC-084 整项待验。</x:v>
       </x:c>
       <x:c r="M89" s="58" t="str">
-        <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。REQ-040 尚无 complete 证据，TC-084 整项待验；docs/validation.md 对应记录。</x:v>
+        <x:v>代码 000372b；单元 1/1、Electron 1/1，单编号命令退出码 0。REQ-040 尚无 complete 证据，TC-084 整项待验；docs/validation.md 对应记录。
+2026-10-03 覆盖证据决议：本次只更新证据门槛，未执行新真零正例；旧 000372b 结果保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="410" customHeight="1">

</xml_diff>

<commit_message>
docs: record verified upgrade fault coverage and retry
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6f3bad9b332c4509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc922a8a12bae43c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rda7d290e335b4ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5e3ea7e8599a42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R379dabd84b574342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R048738006a0a4766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9bc88177812646f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R007ba0acec3346db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1508,7 +1508,8 @@
         <x:v>自动安装控制与回退</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>0.3.6 TC-036 合成回滚回归通过；打包故障待验</x:v>
+        <x:v>0.3.6 TC-036 合成回滚回归通过；打包故障待验
+2026-10-04 / 80e7f10→0eac84b：TC-036 路径别名合成单元 2/2 独立通过；模块故障见 TC-076，打包 helper/UI 回滚仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="62" customHeight="1">
@@ -2451,7 +2452,8 @@
         <x:v>实际打包 App 隔离自动升级</x:v>
       </x:c>
       <x:c r="G82" s="52" t="str">
-        <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验</x:v>
+        <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
+2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="85" customHeight="1">
@@ -3542,7 +3544,8 @@
       <x:c r="H27" s="69" t="str">
         <x:v>当前 1e70412：TC-034/035 与 TC-059 独立回归退出码 0，TC-076 真实 DMG 成功链路通过；异常边界仍按各 TC 待验。
 docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
-2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。</x:v>
+2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。
+2026-10-04 / 80e7f10→0eac84b：当前候选 DMG 新 SHA-256 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c、142591838 字节，两包 hdiutil verify VALID；原 27aae018… 为 1e70412 历史候选。此批主要验安装，TC-034/035 的原异常边界不据此提升。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="62" customHeight="1">
@@ -3559,7 +3562,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>部分验证；真实 0.3.5→0.3.6 隔离自动成功，系统安装/打包故障回滚待验</x:v>
+        <x:v>部分验证；真实 0.3.5→0.3.6 隔离自动升级及 installer 模块五故障回退/重试子范围通过；系统安装/打包 helper 故障与安装中取消待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3570,7 +3573,8 @@
       <x:c r="H28" s="70" t="str">
         <x:v>当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
 历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
-2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。</x:v>
+2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。
+2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4908,7 +4912,8 @@
       <x:c r="G29" s="69" t="str">
         <x:v>当前 1e70412：文档会话独立复跑 TC-034/035/059，各 1/1 退出码 0；TC-076 的真实候选下载/摘要通过。
 自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md；2026-10-03 新目标：在校验大小/SHA-256、架构及版本后才允许启动辅助安装；停服、下载中断、空间不足和摘要错误逐阶段可恢复，坏包绝不安装。TC-034/035 既有通过保留历史，新增断言与状态待实现。
-86a4b5b：客户端下载后校验大小/SHA-256 再交自动安装器，坏包不会触发 helper；文档会话 TC-034/035/059 与 76 入口检查退出码 0。超时/磁盘不足与真实用户错误恢复仍待验。</x:v>
+86a4b5b：客户端下载后校验大小/SHA-256 再交自动安装器，坏包不会触发 helper；文档会话 TC-034/035/059 与 76 入口检查退出码 0。超时/磁盘不足与真实用户错误恢复仍待验。
+2026-10-04 / 80e7f10→0eac84b：本批新候选摘要已对账；下载/校验与安装分层，不能由 installer 故障回退推 TC-034/035 的超时/空间不足下载边界已验。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="62" customHeight="1">
@@ -4928,12 +4933,13 @@
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>真实 0.3.5→0.3.6 隔离自动成功链路通过；系统安装/打包故障回滚待验</x:v>
+        <x:v>部分实现/验证；真实 DMG 隔离成功升级、五种生产 installer 模块 hooks 故障回退及重试通过；系统安装目标、打包 helper/UI 故障、安装中取消待验</x:v>
       </x:c>
       <x:c r="G30" s="70" t="str">
         <x:v>当前 1e70412：文档会话构建 0.3.6 x64 目录包并以真实旧/新 DMG、固定哈希独立复跑 TC-076，exit 0；TC-036 2/2 合成单元回归通过。
 历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
-86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。</x:v>
+86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。
+2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -7284,18 +7290,20 @@
         <x:v>单元/辅助进程故障注入</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
-        <x:v>注入已校验包的辅助进程启动、旧进程退出、挂载、替换、重启和健康确认成功/失败；测试取消及不可写安装位置。</x:v>
+        <x:v>注入已校验包的辅助进程启动、旧进程退出、挂载、替换、重启和健康确认成功/失败；测试取消及不可写安装位置。
+2026-10-04 / 80e7f10→0eac84b：增加父目录符号链接别名健康标记样本（/var 与 /private/var 可指同一 App），保留叶子 App 非符号链接约束。</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
         <x:v>成功路径自动退出旧版、安装替换并启动新版；失败回滚旧版、保留用户数据、清理挂载/临时文件；权限不足不静默绕过，成功无需 Finder 拖拽。</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
-        <x:v>0.3.6 合成控制/回滚单元 2/2 回归通过；打包故障回滚待验</x:v>
+        <x:v>0.3.6 合成控制/回滚单元 2/2 独立通过，含路径别名；真实 DMG 的模块故障子范围由 TC-076 另验，打包 helper/UI 回滚仍待验</x:v>
       </x:c>
       <x:c r="I41" s="69" t="str">
         <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-036，2/2、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
 历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。
-86a4b5b：文档会话单编号 TC-036 两项 2/2 退出码 0：下载校验后交自动安装器及启动失败不退出旧版；合成 Bundle/命令覆盖 /Applications/~/Applications 选择、成功、挂载/复制/替换/重启/健康超时及篡改失败回滚。真实旧二进制、只读 DMG 实测及系统权限未由单元证明。</x:v>
+86a4b5b：文档会话单编号 TC-036 两项 2/2 退出码 0：下载校验后交自动安装器及启动失败不退出旧版；合成 Bundle/命令覆盖 /Applications/~/Applications 选择、成功、挂载/复制/替换/重启/健康超时及篡改失败回滚。真实旧二进制、只读 DMG 实测及系统权限未由单元证明。
+2026-10-04 / 80e7f10→0eac84b：文档工作树 macOS 15.7.4 x86_64、Node 24.15.0：npm run test:case -- TC-036，2/2、exit 0；门禁 94 入口/77 单元/38 Electron、打包版 38/38 均 exit 0。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str">
         <x:v>单元：npm run test:case -- TC-036；本机链路：npm run test:upgrade:local -- /绝对路径/Token-0.2.0.dmg /绝对路径/Token-0.3.0.dmg</x:v>
@@ -7305,10 +7313,12 @@
       </x:c>
       <x:c r="L41" s="35" t="str">
         <x:v>2026-10-02：本机隔离下载打开、ditto 替换、受信登录及合成 1280 Token 通过。2026-10-03：打开后不替换并重启旧版，版本/登录/已采集数据保留；单元注入打开失败时旧文件不变；旧 0.2.0→0.3.0 可复用链路继续通过，普通 0.3.0→0.3.1 隔离升级由开发会话报告通过。Finder 真实失败回退、手动安装未测。；新目标的自动替换、重启、权限/回滚未验证；真实制品见待注册 TC-076。
-0.3.5 合成测试覆盖 helper 控制流和路径选择；不等于真实只读 DMG、不可写系统安装或历史 0.3.0/0.3.4 UI 一键升级。</x:v>
+0.3.5 合成测试覆盖 helper 控制流和路径选择；不等于真实只读 DMG、不可写系统安装或历史 0.3.0/0.3.4 UI 一键升级。
+2026-10-04 / 80e7f10→0eac84b：路径别名新断言是合成 App 的 installer 模块测试，不证明真实系统安装目标或打包 helper/UI 失败恢复。</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。；2026-10-03 起旧 Finder 手动安装不再是自动成功路径目标；原缺口与证据作为历史保留。</x:v>
+        <x:v>旧/新 0.2.0→0.3.0 DMG SHA-256：49ae49eebc26502dd4f017cab47e06d7dda6b1cbb73601ea179cafb7151b0ff6 / 64917685d073d0c631ef492df58eb3a3bec96657f15372177af466c68a34fec8；0.3.1 候选包见 TC-073、docs/validation.md；生产库迁移、签名公证及目标 Mac 另验。；2026-10-03 起旧 Finder 手动安装不再是自动成功路径目标；原缺口与证据作为历史保留。
+2026-10-04 / 80e7f10→0eac84b：0eac84b 固定代码；TC-036 2/2 exit 0。80e7f10 新产品路径修复，测试脚本后续修正不改变该产品语义。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="70" customHeight="1">
@@ -8952,31 +8962,37 @@
         <x:v>打包应用/本机隔离</x:v>
       </x:c>
       <x:c r="F81" s="52" t="str">
-        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。分别注入取消、磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。</x:v>
+        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。分别注入取消、磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
+2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。</x:v>
       </x:c>
       <x:c r="G81" s="52" t="str">
-        <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。</x:v>
+        <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。
+2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>已注册；真实 0.3.5→0.3.6 DMG 隔离自动成功子范围通过，整项待环境/回滚</x:v>
+        <x:v>已注册；真实 DMG 隔离成功升级、只读旧包初始启动、五种生产 installer 模块故障回退及重试自动子范围独立通过；系统目标/打包 helper/UI/安装中取消待验</x:v>
       </x:c>
       <x:c r="I81" s="68" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
 2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
-86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。</x:v>
+86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。
+2026-10-04 / 80e7f10→0eac84b：80e7f10 文档独立首次全命令：成功段、只读初始启动、五故障回退输出通过；末次重试读取已被 UI 消费的一次性 last-install.json 得 undefined，exit 1。0eac84b 修脚本后同 DMG 再跑，全命令 exit 0；旧包 142557541 字节 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 142591838 字节 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c，两包 verify VALID。旧 27aae018… 只属历史候选。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="str">
-        <x:v>TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff npm run test:case -- TC-076</x:v>
+        <x:v>TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c npm run test:case -- TC-076</x:v>
       </x:c>
       <x:c r="K81" s="52" t="str">
-        <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；给定 OLD_DMG/OLD_SHA256/NEW_DMG/NEW_SHA256 即验证真实旧/新 DMG；省略参数则为改版本元数据的合成旧版模式。</x:v>
+        <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；给定 OLD_DMG/OLD_SHA256/NEW_DMG/NEW_SHA256 即验证真实旧/新 DMG；省略参数则为改版本元数据的合成旧版模式。
+2026-10-04 / 80e7f10→0eac84b：现另绑定 scripts/verify-auto-upgrade-faults.mjs；仅给出四个真实 DMG/摘要参数才运行真实制品故障路径；此脚本直接调用生产 installer 模块，非打包 helper 进程。</x:v>
       </x:c>
       <x:c r="L81" s="68" t="str">
         <x:v>当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
-0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。</x:v>
+0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。
+2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
-        <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。</x:v>
+        <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
+2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">

</xml_diff>

<commit_message>
docs: decide managed coverage evidence and record reconciliation validation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R379dabd84b574342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R048738006a0a4766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9bc88177812646f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R007ba0acec3346db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ca160ef7cd541d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8d2c0aed88124511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R19fbb98ecdad444f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb0546ac5d2a64f08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -221,7 +221,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="73">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -414,6 +414,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -626,7 +632,7 @@
     <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="57.779998779296875" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="28" customHeight="1">
@@ -2456,7 +2462,7 @@
 2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="85" customHeight="1">
+    <x:row r="83" ht="135" customHeight="1">
       <x:c r="A83" s="55" t="str">
         <x:v>REQ-040</x:v>
       </x:c>
@@ -2475,12 +2481,13 @@
       <x:c r="F83" s="55" t="str">
         <x:v>所选范围覆盖真值表</x:v>
       </x:c>
-      <x:c r="G83" s="55" t="str">
+      <x:c r="G83" s="71" t="str">
         <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验
-2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="84" ht="85" customHeight="1">
+2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
+2026-10-04 受管持续采集设计已决，TC-077 受控和真实 CLI 正例未实施；整项待验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="135" customHeight="1">
       <x:c r="A84" s="58" t="str">
         <x:v>REQ-040</x:v>
       </x:c>
@@ -2499,9 +2506,10 @@
       <x:c r="F84" s="58" t="str">
         <x:v>区间比较可比性门禁</x:v>
       </x:c>
-      <x:c r="G84" s="58" t="str">
+      <x:c r="G84" s="72" t="str">
         <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验
-2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。</x:v>
+2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
+2026-10-04 TC-078 双关闭等长完整窗口受控/真实正例待实施，范围外未知；整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -2619,7 +2627,7 @@
         <x:v>TC-083 已注册；1 单元+1 Electron 隔离自动子范围通过（3bbaf15）；真实生产/打包环境待验证</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" ht="85" customHeight="1">
+    <x:row r="90" ht="135" customHeight="1">
       <x:c r="A90" s="58" t="str">
         <x:v>REQ-044</x:v>
       </x:c>
@@ -2638,9 +2646,10 @@
       <x:c r="F90" s="58" t="str">
         <x:v>六类空状态与可操作下一步</x:v>
       </x:c>
-      <x:c r="G90" s="58" t="str">
+      <x:c r="G90" s="72" t="str">
         <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验
-2026-10-03 覆盖证据决议：真零须已关闭同范围完整空窗；合成只验规则，真实来源未证；REQ-044/DEV-053/TC-084 整项待验。</x:v>
+2026-10-03 覆盖证据决议：真零须已关闭同范围完整空窗；合成只验规则，真实来源未证；REQ-044/DEV-053/TC-084 整项待验。
+2026-10-04 TC-084 受管关闭空窗真零正例待实施，固定快照/空心跳不能补证；整项待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -2809,7 +2818,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="90" customHeight="1">
+    <x:row r="98" ht="135" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2828,11 +2837,12 @@
       <x:c r="F98" s="61" t="str">
         <x:v>同会话重复与跨用户独立保留</x:v>
       </x:c>
-      <x:c r="G98" s="61" t="str">
-        <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="90" customHeight="1">
+      <x:c r="G98" s="71" t="str">
+        <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证
+2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="135" customHeight="1">
       <x:c r="A99" s="64" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2851,8 +2861,9 @@
       <x:c r="F99" s="64" t="str">
         <x:v>无法关联冲突与三处报表权限一致</x:v>
       </x:c>
-      <x:c r="G99" s="64" t="str">
-        <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验</x:v>
+      <x:c r="G99" s="72" t="str">
+        <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验
+2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="95" customHeight="1">
@@ -4025,7 +4036,8 @@
 2026-10-03 官方来源核对：Codex exec --ephemeral 不持久化 session rollout 文件（https://learn.chatgpt.com/docs/developer-commands#codex-exec）；Claude Code OTel 要 CLAUDE_CODE_ENABLE_TELEMETRY=1，指标/日志 exporter 可为 none（https://code.claude.com/docs/en/monitoring-usage）。推论仅为本地文件/OTel 未观察到不能证明真零或完整，非完整覆盖正例。REQ-040 状态不变。
 2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。
 3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。
-2026-10-03 覆盖证据决议：现有状态/游标/事实仅证已观察；受控合成正例只验规则，不证明真实 Codex/Claude 来源完整。真实来源机制未落实，整项仍待验。官方：https://learn.chatgpt.com/docs/developer-commands?surface=cli 与 https://code.claude.com/docs/en/monitoring-usage</x:v>
+2026-10-03 覆盖证据决议：现有状态/游标/事实仅证已观察；受控合成正例只验规则，不证明真实 Codex/Claude 来源完整。真实来源机制未落实，整项仍待验。官方：https://learn.chatgpt.com/docs/developer-commands?surface=cli 与 https://code.claude.com/docs/en/monitoring-usage
+2026-10-04 设计决议：用户主动启用受管会话；持久启动/结束账本、逐事件用量与守护连续水位按 owner/provider/模型/项目/IANA 时区/关闭窗口 fail closed。文件快照仅证重放；普通本机全部使用量及范围外仍未知。见 docs/coverage-evidence-decision.md；未实施、未验真实正例。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -4139,7 +4151,8 @@
 2026-10-03 SOP-001/002 范围决议：REQ-040 当前不能证明完整空窗，因此 TC-084 真零正例本轮不可构造；无事实、ready 或注入 complete 不能冒充真零。保守空状态和长扫描/修复重试可先开发验收，REQ-044 整项待验。未改代码/测试。
 2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。
 2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。
-2026-10-03 覆盖证据决议：TC-084 可计划受控合成规则正例；真实来源完整性、范围外执行模式和实际空窗未验，REQ-044 整项待验。</x:v>
+2026-10-03 覆盖证据决议：TC-084 可计划受控合成规则正例；真实来源完整性、范围外执行模式和实际空窗未验，REQ-044 整项待验。
+2026-10-04 真零仅限同一授权受管来源关闭空窗、启动账本和连续采集可证、事实集为空；界面标范围外未知。TC-084 受控和真实正例待实现/验收。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -4259,7 +4272,7 @@
         <x:v>缺陷修复（已复现）</x:v>
       </x:c>
       <x:c r="E53" s="61" t="str">
-        <x:v>已编码；TC-092–094 自动子范围通过，正向精确去重/TC-093 补断言/生产迁移待验证</x:v>
+        <x:v>已编码；TC-092–094 自动子范围通过，TC-093 在 81c271b 增真实隔离输入 E2E 并独立复验；跨账户同键碰撞待修，正向精确去重/生产迁移待验证</x:v>
       </x:c>
       <x:c r="F53" s="61" t="str">
         <x:v>DEV-057</x:v>
@@ -4274,7 +4287,8 @@
 2026-10-03 静态审查发现 sources:statuses 与报表 coverage 返回全局 scanner.statuses()，概览/报表显示全局计数与采集时间；TC-093 增双 owner IPC/UI 验收。尚未动态复现、修复或通过。
 同日补充静态发现：诊断 IPC/可选反馈附件按 provider 保留整条全局诊断，TC-093 扩至两入口；尚无动态验证。
 2026-10-03 代码 8157e2d：授权 owner 调和替代按日整批排除；冲突仅显示已确认小计，明细保留待核对，CSV v1 十列/v2 十四列，服务 accountingVersion 2、旧 v1 状态 legacy_unknown，viewer 来源状态/诊断/附件按本人或未知。文档会话独立 test:gate 82 入口、56 单元、22 Electron 通过；TC-092–094 单编号通过。未证共同事件 ID 正向去重、TC-093 的概览 B 值/sources:scan 直调、v2 TC-023/079、真实生产库迁移和旧服务真实版本。REQ-040 管理员筛选覆盖独立待验。
-47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。</x:v>
+47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。
+2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5498,7 +5512,8 @@
 下一笔先按 owner+工具+时区+区间给授权 API/概览/报表统一的未知或可证部分，阻断全局 ready、最早事实、成功空扫描推出假零/假同比；仅 pending 事实时显示已确认小计 0 与完整总量未知。TC-077/078 先注册负例和范围一致性断言。完整空窗真零、同 as-of 两期完整比较需需求会话先决定留存/连续采集证据及旧库策略，不能造假 complete 或将整项标通过。
 官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。
 2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。
-2026-10-03 覆盖证据决议：增加监测来源边界、留存起点、连续采集/重放水位、错误/缺口、归属和维度解析的可审计证据链，按所选范围判定；关闭空窗限定真零，双窗同口径且完整才比较。合成契约不得提升真实来源状态。</x:v>
+2026-10-03 覆盖证据决议：增加监测来源边界、留存起点、连续采集/重放水位、错误/缺口、归属和维度解析的可审计证据链，按所选范围判定；关闭空窗限定真零，双窗同口径且完整才比较。合成契约不得提升真实来源状态。
+2026-10-04 分期：受管入口与持久运行/用量/连续水位账本→授权范围封窗与 UI 标签→TC-077/078 受控正例→真实 CLI 正例；固定快照不升级为完整使用窗口。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -5599,7 +5614,8 @@
 本轮先实现未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知/已观测但完整性未知的原因和行动；长扫描只用真实阶段、处理量或心跳并可修复重试。真零只为未来 coverage.complete 且同一授权筛选范围无事实的受控分支，等 REQ-040 证据方案后再验；不得伪造 complete。TC-084/085 可先测保守子范围，DEV-053 整项待验。
 代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。
 90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。
-2026-10-03 覆盖证据决议：真零 UI 仅消费经 REQ-040/DEV-049 证明的所选来源 complete、已关闭且同事实集为空；范围外模式仍未知。真实来源机制未交付前 DEV-053 整项待验。</x:v>
+2026-10-03 覆盖证据决议：真零 UI 仅消费经 REQ-040/DEV-049 证明的所选来源 complete、已关闭且同事实集为空；范围外模式仍未知。真实来源机制未交付前 DEV-053 整项待验。
+2026-10-04 TC-084 真零依赖受管服务连续有效、关闭空窗及同范围空事实；先受控规则，再真实 CLI/守护服务正例，范围外仍未知。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -5702,7 +5718,7 @@
         <x:v>src/main/reconcile.ts、report.ts、usage-sync.ts、index.ts；src/server/server.ts；src/shared/types.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；tests/reconciliation.test.ts、sync-reconciliation.test.ts、e2e/overlap-privacy.spec.ts；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
-        <x:v>已实现；TC-092–094 自动子范围通过（8157e2d），剩余断言和真实迁移待验证</x:v>
+        <x:v>已实现调和子范围；TC-093 真实隔离输入 E2E 通过（81c271b）；TC-092 跨账户同键碰撞待修，正向精确去重/真实迁移待验证</x:v>
       </x:c>
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
@@ -5712,7 +5728,8 @@
 在主进程按登录态/授权查询范围构造 viewer 来源状态；不能仅前端隐藏全局 fileCount/factCount/telemetryFactCount、lastTelemetry/lastScan、detail 或由全局状态推导真零。无法证明 owner 归属则未知/空值；对齐来源状态 IPC、报表 coverage 与概览/报表 UI，管理员全局视图标明范围。TC-093 双 owner IPC/UI 回归，关联 TC-021/045/046/077/078。当前仅静态审查。
 诊断 IPC 和可选反馈附件必须复用按 owner 授权后的视图；通用 suggestion 可留，跨 owner location/reason、文件/事实/未归属/异常计数、lastScan/lastSuccess 不能经 IPC、UI 或反馈载荷泄露。
 8157e2d：本地/OTel 按授权 owner 和会话调和；冲突候选不冒充已证重复，查询范围外同会话候选仍影响状态。报表/概览已确认小计、明细待核对原行、v2 十四列逐组小计及同快照导出；服务 v2 旧值 legacy_unknown/confirmedSubtotal=null、v2 后拒 v1、旧 outbox 重算/旧协议待传；viewer 来源状态/诊断/反馈附件隔离。文档会话 gate 82/56/22 全过；共同事件 ID 正向去重、TC-093 部分 IPC/UI 与 v2 公式/快照、生产迁移仍待补。管理员全局状态不代表 DEV-049 完成。
-47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。</x:v>
+47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。
+2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9016,13 +9033,15 @@
 构造管理员可选 A/B 两个 owner 与未归属事实，令全局 scanner.ready 且 A 有事实，选无事实 B 与未归属；切换工具、时区、区间，核授权 API、概览来源卡和报表 coverage。另造 B 所选范围确实完整且空的正例。
 本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。
 以无正文合成缺失输入模拟 Codex ephemeral 不落文件及 Claude OTel 未启用/exporter=none；核本地文件/OTel 缺记录仍未知，不宣称工具没用或真零。真实工具端到端验证另行安排。
-2026-10-03 覆盖证据决议：计划受控合成正例：为所选 owner+provider+窗口逐项提供监测范围、留存起点、连续水位、无错误/缺口、归属及筛选维度证据；分别移除一项作降级反例，并核 API/概览/报表一致。真实工具来源另需独立证据。</x:v>
+2026-10-03 覆盖证据决议：计划受控合成正例：为所选 owner+provider+窗口逐项提供监测范围、留存起点、连续水位、无错误/缺口、归属及筛选维度证据；分别移除一项作降级反例，并核 API/概览/报表一致。真实工具来源另需独立证据。
+2026-10-04 待补受控持久运行账本正例与真实受管 Codex/Claude CLI（含 ephemeral/无持久会话）端到端；撤掉留存起点、启动/结束、连续水位、身份/维度、无错误条件逐项降级。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
         <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
 B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。
 缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。
-2026-10-03 覆盖证据决议：仅完整证据链支持所选来源 complete；范围外模式未知。关闭且同事实集空才显示限定“已确认零（所选已监测来源）”，不推服务商账单/全设备零。合成正例不使真实历史通过。</x:v>
+2026-10-03 覆盖证据决议：仅完整证据链支持所选来源 complete；范围外模式未知。关闭且同事实集空才显示限定“已确认零（所选已监测来源）”，不推服务商账单/全设备零。合成正例不使真实历史通过。
+仅在主动启用的受管来源、窗口封闭且 owner/provider/模型/项目/时区等全部可证时 complete；固定快照和范围外执行未知。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
         <x:v>已注册；防假零保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
@@ -9045,7 +9064,8 @@
 外部依据：https://learn.chatgpt.com/docs/developer-commands#codex-exec 说明 --ephemeral 不落 rollout；https://code.claude.com/docs/en/monitoring-usage 说明 OTel 显式开启且 exporter 可 none。仅支持“未观察到≠真零”，不能用合成缺失样本证明全部真实入口。
 现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。
 3bbaf15 已修正原“未归属”筛选下无事实 reason 的“已归属”措辞；仍不证明完整覆盖。
-2026-10-03 覆盖证据决议：现有保守负例结果保留。Codex --ephemeral 可无 rollout，Claude OTel 日志 exporter 可为 none；真实来源留存与连续性未证，TC-077 整项待验。</x:v>
+2026-10-03 覆盖证据决议：现有保守负例结果保留。Codex --ephemeral 可无 rollout，Claude OTel 日志 exporter 可为 none；真实来源留存与连续性未证，TC-077 整项待验。
+真实 CLI 版本、结束语义、子代理及模型/项目字段、受管服务连续性尚需外部环境；不得以受控样本升真实覆盖。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
@@ -9074,13 +9094,15 @@
         <x:v>同范围等长两期分别构造双方完整、一方部分、范围变化、时区边界、今天进行中与扫描滞后，并记录最近成功采集的 as-of。
 管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。
 本轮先造管理员选定 owner/未归属两期、全局 ready 但选中范围缺证、今天进行中与扫描滞后；核 API/界面保持不可比较。完整同 as-of 正例等待证据方案。
-2026-10-03 覆盖证据决议：计划受控合成双窗正例及单变量反例：两窗等长、同 owner/provider/筛选/来源范围、同 IANA 时区与 as-of 截止，双方各有完整证据链；破坏任一条件应不可比较。</x:v>
+2026-10-03 覆盖证据决议：计划受控合成双窗正例及单变量反例：两窗等长、同 owner/provider/筛选/来源范围、同 IANA 时区与 as-of 截止，双方各有完整证据链；破坏任一条件应不可比较。
+2026-10-04 待补两段真实受管关闭窗口，及受控等长/同范围/同 as-of 正例；注入掉线、晚到结束、时区实际不等长和范围外运行。</x:v>
       </x:c>
       <x:c r="G83" s="58" t="str">
         <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。
 全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。
 没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。
-2026-10-03 覆盖证据决议：只有双方 source-complete 且双窗等长、同范围/时区/as-of 才显示比较；今天未结束、扫描滞后或范围外模式均不可比较。合成正例不证明真实历史。</x:v>
+2026-10-03 覆盖证据决议：只有双方 source-complete 且双窗等长、同范围/时区/as-of 才显示比较；今天未结束、扫描滞后或范围外模式均不可比较。合成正例不证明真实历史。
+两窗各自完整且实际 UTC 时长相等、同 owner/provider/模式/模型/项目/IANA 时区及 as-of 才显示差值。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
         <x:v>已注册；防假同比保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
@@ -9348,12 +9370,14 @@
       <x:c r="F89" s="58" t="str">
         <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。
 2026-10-03 本轮先逐项造未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知、已观测但完整性未知；核授权范围、文案与行动。真零正例等待可证完整空窗，不在本轮造数或注入 complete。
-2026-10-03 覆盖证据决议：计划受控合成正例须经 REQ-040 所选 owner+provider+窗口的完整证据链，窗口已关闭且同一授权筛选事实集为空；逐项撤证及范围外模式作为负例。真实来源另验。</x:v>
+2026-10-03 覆盖证据决议：计划受控合成正例须经 REQ-040 所选 owner+provider+窗口的完整证据链，窗口已关闭且同一授权筛选事实集为空；逐项撤证及范围外模式作为负例。真实来源另验。
+2026-10-04 待补受控和真实守护服务连续有效、启动账本无运行的关闭空窗正例；范围外另运行真实命令核标签。</x:v>
       </x:c>
       <x:c r="G89" s="58" t="str">
         <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。
 保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。
-2026-10-03 覆盖证据决议：仅显示限定“已确认零（所选已监测来源）”；不宣称服务商账单/全设备零。未关闭、待核对、缺证或范围外模式不得真零。</x:v>
+2026-10-03 覆盖证据决议：仅显示限定“已确认零（所选已监测来源）”；不宣称服务商账单/全设备零。未关闭、待核对、缺证或范围外模式不得真零。
+仅显示“已确认零（所选受管来源）”并列范围外未知；空心跳、空扫描、空快照、未知模型/项目不得真零。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
         <x:v>已注册；保守空状态自动子范围通过，真零正例待 REQ-040 完整覆盖证据，整项待验</x:v>
@@ -9743,10 +9767,12 @@
         <x:v>单元/集成</x:v>
       </x:c>
       <x:c r="F97" s="61" t="str">
-        <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。</x:v>
+        <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。
+2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
-        <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。</x:v>
+        <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
+双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9761,7 +9787,8 @@
         <x:v>scripts/test-cases.mjs：tests/reconciliation.test.ts 中以 TC-092 开头的独立 Vitest 函数。</x:v>
       </x:c>
       <x:c r="L97" s="61" t="str">
-        <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。</x:v>
+        <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。
+静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
@@ -9796,7 +9823,8 @@
 只按 provider 相同不得泄露 B 的文件/事实/未归属/异常计数、位置/原因、扫描/成功时间；通用指引和 A 可证字段可保留，无法归属字段未知/省略，反馈附件不增加权限。</x:v>
       </x:c>
       <x:c r="H98" s="64" t="str">
-        <x:v>已注册；单元+Electron 自动子范围通过（47b03d5），真实冲突事实完整 E2E/生产环境待验证</x:v>
+        <x:v>已注册；单元+Electron 自动子范围通过（47b03d5），真实冲突事实完整 E2E/生产环境待验证
+已注册；81c271b 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路及原隐私 Electron、单元子范围经文档会话独立复验通过；生产迁移/共同 ID 正向去重仍待证</x:v>
       </x:c>
       <x:c r="I98" s="64" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-093：Vitest 1/1、Electron 1/1、退出码 0；单元 v2 十四列三组小计 5/7/0，总计 12，冲突明细保留 5 条，跨窗候选仍标冲突。Electron 真实 IPC/反馈附件双 owner 隔离；冲突 UI 文案采用注入响应。test:gate 82/56/22 全过。
@@ -9810,12 +9838,14 @@
         <x:v>scripts/test-cases.mjs：tests/reconciliation.test.ts 中 TC-093 Vitest 函数；tests/e2e/overlap-privacy.spec.ts 中 TC-093 Electron 函数。</x:v>
       </x:c>
       <x:c r="L98" s="64" t="str">
-        <x:v>当前已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。</x:v>
+        <x:v>47b03d5 阶段已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。47b03d5 阶段 TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。
+2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
 47b03d5；macOS 本机隔离临时库/Electron；TC-093 unit/E2E 各 1/1 退出码 0，TC-023 两单元、TC-079 unit/E2E 均退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
-c10bbf3；macOS x86_64 隔离合成样本；TC-093 unit 1/1、Electron 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。</x:v>
+c10bbf3；macOS x86_64 隔离合成样本；TC-093 unit 1/1、Electron 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。
+81c271b；文档会话独立 npm run test:case -- TC-093：unit 1/1、Electron 2/2、exit 0；真实隔离输入 A 本地 12/5、OTel 14，B OTel 99；A 已确认 5、待核对 2、明细 [5,12,14]、CSV v2 14 列/B 仅 99。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="195" customHeight="1">

</xml_diff>

<commit_message>
docs: capture telemetry event identity and source key risks
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ca160ef7cd541d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8d2c0aed88124511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R19fbb98ecdad444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb0546ac5d2a64f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1e145e87b56c4d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc0ed8740deac4dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc7a05a03f0eb49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R54ba9b4fce7b4bb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2818,7 +2818,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="135" customHeight="1">
+    <x:row r="98" ht="210" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2839,7 +2839,8 @@
       </x:c>
       <x:c r="G98" s="71" t="str">
         <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证
-2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。</x:v>
+2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="135" customHeight="1">
@@ -4288,7 +4289,8 @@
 同日补充静态发现：诊断 IPC/可选反馈附件按 provider 保留整条全局诊断，TC-093 扩至两入口；尚无动态验证。
 2026-10-03 代码 8157e2d：授权 owner 调和替代按日整批排除；冲突仅显示已确认小计，明细保留待核对，CSV v1 十列/v2 十四列，服务 accountingVersion 2、旧 v1 状态 legacy_unknown，viewer 来源状态/诊断/附件按本人或未知。文档会话独立 test:gate 82 入口、56 单元、22 Electron 通过；TC-092–094 单编号通过。未证共同事件 ID 正向去重、TC-093 的概览 B 值/sources:scan 直调、v2 TC-023/079、真实生产库迁移和旧服务真实版本。REQ-040 管理员筛选覆盖独立待验。
 47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。
-2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。</x:v>
+2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5729,7 +5731,8 @@
 诊断 IPC 和可选反馈附件必须复用按 owner 授权后的视图；通用 suggestion 可留，跨 owner location/reason、文件/事实/未归属/异常计数、lastScan/lastSuccess 不能经 IPC、UI 或反馈载荷泄露。
 8157e2d：本地/OTel 按授权 owner 和会话调和；冲突候选不冒充已证重复，查询范围外同会话候选仍影响状态。报表/概览已确认小计、明细待核对原行、v2 十四列逐组小计及同快照导出；服务 v2 旧值 legacy_unknown/confirmedSubtotal=null、v2 后拒 v1、旧 outbox 重算/旧协议待传；viewer 来源状态/诊断/反馈附件隔离。文档会话 gate 82/56/22 全过；共同事件 ID 正向去重、TC-093 部分 IPC/UI 与 v2 公式/快照、生产迁移仍待补。管理员全局状态不代表 DEV-049 完成。
 47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。
-2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。</x:v>
+2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9768,11 +9771,13 @@
       </x:c>
       <x:c r="F97" s="61" t="str">
         <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。
-2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。</x:v>
+2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
-双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。</x:v>
+双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9788,7 +9793,8 @@
       </x:c>
       <x:c r="L97" s="61" t="str">
         <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。
-静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。</x:v>
+静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>

</xml_diff>

<commit_message>
docs: validate packaged update helper fault recovery
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1e145e87b56c4d35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc0ed8740deac4dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc7a05a03f0eb49b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R54ba9b4fce7b4bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R8c5edf2aaeb142ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf1223480509e4fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3676f496478d448e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R9cf486e008274b45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2438,7 +2438,7 @@
         <x:v>已验证（自动；模拟预检、命令构造与五处核验失败清理）</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="100" customHeight="1">
+    <x:row r="82" ht="195" customHeight="1">
       <x:c r="A82" s="52" t="str">
         <x:v>REQ-023</x:v>
       </x:c>
@@ -2459,7 +2459,8 @@
       </x:c>
       <x:c r="G82" s="52" t="str">
         <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
-2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。</x:v>
+2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。
+2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -2818,7 +2819,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="210" customHeight="1">
+    <x:row r="98" ht="292.5" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2840,7 +2841,8 @@
       <x:c r="G98" s="71" t="str">
         <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证
 2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="135" customHeight="1">
@@ -3574,7 +3576,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>部分验证；真实 0.3.5→0.3.6 隔离自动升级及 installer 模块五故障回退/重试子范围通过；系统安装/打包 helper 故障与安装中取消待验</x:v>
+        <x:v>部分验证；真实 0.3.5→0.3.6 隔离升级、installer 模块与打包 helper 五故障回退/重试子范围独立通过；真实系统目录/满盘/崩溃/安装中取消/签名异机待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3586,7 +3588,8 @@
         <x:v>当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
 历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
 2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。
-2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。</x:v>
+2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。
+2026-10-04 1961de3：TC-076 新增隔离打包 helper 五故障。文档会话真实旧/新 DMG 固定哈希完整命令 exit 0；旧 UI 触发 helper，mount/space/replace/launch/health 每次回退旧版、受信登录/1280 Token/清理，最后重试新版。注入为专用临时目录预加载，非真实满盘/崩溃或系统安装。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4290,7 +4293,8 @@
 2026-10-03 代码 8157e2d：授权 owner 调和替代按日整批排除；冲突仅显示已确认小计，明细保留待核对，CSV v1 十列/v2 十四列，服务 accountingVersion 2、旧 v1 状态 legacy_unknown，viewer 来源状态/诊断/附件按本人或未知。文档会话独立 test:gate 82 入口、56 单元、22 Electron 通过；TC-092–094 单编号通过。未证共同事件 ID 正向去重、TC-093 的概览 B 值/sources:scan 直调、v2 TC-023/079、真实生产库迁移和旧服务真实版本。REQ-040 管理员筛选覆盖独立待验。
 47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。
 2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4949,13 +4953,14 @@
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>部分实现/验证；真实 DMG 隔离成功升级、五种生产 installer 模块 hooks 故障回退及重试通过；系统安装目标、打包 helper/UI 故障、安装中取消待验</x:v>
+        <x:v>部分实现/验证；真实 DMG 隔离升级、installer 模块及打包 helper 五故障回退/重试通过；真实系统目录、满盘/崩溃、安装中取消待验</x:v>
       </x:c>
       <x:c r="G30" s="70" t="str">
         <x:v>当前 1e70412：文档会话构建 0.3.6 x64 目录包并以真实旧/新 DMG、固定哈希独立复跑 TC-076，exit 0；TC-036 2/2 合成单元回归通过。
 历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
 86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。
-2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。</x:v>
+2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。
+2026-10-04 1961de3：TC-076 三段集成绑定中的新增 scripts/verify-packaged-helper-faults.mjs 在隔离临时目录经旧 UI 触发真实打包 helper；文档会话完整命令 exit 0、TC-036 两项单元 exit 0。未测真实满盘/进程崩溃/系统安装/签名公证异机。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -5732,7 +5737,8 @@
 8157e2d：本地/OTel 按授权 owner 和会话调和；冲突候选不冒充已证重复，查询范围外同会话候选仍影响状态。报表/概览已确认小计、明细待核对原行、v2 十四列逐组小计及同快照导出；服务 v2 旧值 legacy_unknown/confirmedSubtotal=null、v2 后拒 v1、旧 outbox 重算/旧协议待传；viewer 来源状态/诊断/反馈附件隔离。文档会话 gate 82/56/22 全过；共同事件 ID 正向去重、TC-093 部分 IPC/UI 与 v2 公式/快照、生产迁移仍待补。管理员全局状态不代表 DEV-049 完成。
 47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。
 2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8990,7 +8996,7 @@
 2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>已注册；真实 DMG 隔离成功升级、只读旧包初始启动、五种生产 installer 模块故障回退及重试自动子范围独立通过；系统目标/打包 helper/UI/安装中取消待验</x:v>
+        <x:v>已注册；1961de3 真实 DMG 隔离成功升级、只读旧包初始启动、installer 模块及打包 helper 五故障回退/重试自动子范围独立通过；真实系统目录/满盘/崩溃/安装中取消待验</x:v>
       </x:c>
       <x:c r="I81" s="68" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
@@ -9003,16 +9009,20 @@
       </x:c>
       <x:c r="K81" s="52" t="str">
         <x:v>scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；给定 OLD_DMG/OLD_SHA256/NEW_DMG/NEW_SHA256 即验证真实旧/新 DMG；省略参数则为改版本元数据的合成旧版模式。
-2026-10-04 / 80e7f10→0eac84b：现另绑定 scripts/verify-auto-upgrade-faults.mjs；仅给出四个真实 DMG/摘要参数才运行真实制品故障路径；此脚本直接调用生产 installer 模块，非打包 helper 进程。</x:v>
+2026-10-04 / 80e7f10→0eac84b：现另绑定 scripts/verify-auto-upgrade-faults.mjs；仅给出四个真实 DMG/摘要参数才运行真实制品故障路径；此脚本直接调用生产 installer 模块，非打包 helper 进程。
+1961de3 新增 integration scripts/verify-packaged-helper-faults.mjs；仅给定真实 OLD/NEW DMG+SHA 执行，NODE_OPTIONS 预加载限专用临时目录的打包 update-helper.cjs，五故障和最后重试逐项核。</x:v>
       </x:c>
       <x:c r="L81" s="68" t="str">
         <x:v>当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
 0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。
-2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。</x:v>
+2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。
+2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
-2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。</x:v>
+2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。
+1961de3；文档会话独立 TC-076 完整命令 exit 0，真实旧/新 DMG SHA-256 分别 ae1b8e80…、d99d7af9…，两包 hdiutil verify VALID；打包 helper mount/space/replace/launch/health 各回退、受信登录/1280 Token/清理及最后重试均通过；TC-036 两单元 exit 0。
+1961de3 文档会话独立 test:gate 类型检查、94 入口、77/77 单元、39/39 Electron exit 0；未另跑打包版全量。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">
@@ -9772,12 +9782,14 @@
       <x:c r="F97" s="61" t="str">
         <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。
 2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
 双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9794,7 +9806,8 @@
       <x:c r="L97" s="61" t="str">
         <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。
 静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。
-2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。</x:v>
+2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>

</xml_diff>

<commit_message>
docs: specify in-progress update cancellation contract
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R8c5edf2aaeb142ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf1223480509e4fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3676f496478d448e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R9cf486e008274b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2a181b34e7494eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1b6a3ee198894dd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf97cf909a7cc46aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rca4248ad276e4703"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2438,7 +2438,7 @@
         <x:v>已验证（自动；模拟预检、命令构造与五处核验失败清理）</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" ht="195" customHeight="1">
+    <x:row r="82" ht="337.5" customHeight="1">
       <x:c r="A82" s="52" t="str">
         <x:v>REQ-023</x:v>
       </x:c>
@@ -2460,7 +2460,9 @@
       <x:c r="G82" s="52" t="str">
         <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
 2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。
-2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。</x:v>
+2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。
+2026-10-04 安装中取消设计已决：独立控制窗口+helper 阶段回执、替换后回滚和 userData 隔离健康探测，TC-076 分阶段打包 UI 真取消待实现/验收；既有成功/故障证据不变。
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -3570,7 +3572,8 @@
         <x:v>应用内自动安装升级</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。取消或挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。</x:v>
+        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。取消或挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
+2026-10-04 新增安装中取消：下载/校验前可立即取消；旧版退出后挂载/暂存于安全检查点取消；旧版已移动至成功耐久提交前取消必须完整恢复旧版和未改真实 userData；提交后拒绝迟到取消。控制窗口持续可见并给权威回执，崩溃/断电边界详见 docs/install-cancellation-decision.md。</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>M5（计划）</x:v>
@@ -3589,7 +3592,9 @@
 历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
 2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。
 2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。
-2026-10-04 1961de3：TC-076 新增隔离打包 helper 五故障。文档会话真实旧/新 DMG 固定哈希完整命令 exit 0；旧 UI 触发 helper，mount/space/replace/launch/health 每次回退旧版、受信登录/1280 Token/清理，最后重试新版。注入为专用临时目录预加载，非真实满盘/崩溃或系统安装。</x:v>
+2026-10-04 1961de3：TC-076 新增隔离打包 helper 五故障。文档会话真实旧/新 DMG 固定哈希完整命令 exit 0；旧 UI 触发 helper，mount/space/replace/launch/health 每次回退旧版、受信登录/1280 Token/清理，最后重试新版。注入为专用临时目录预加载，非真实满盘/崩溃或系统安装。
+2026-10-04 取消设计决议：当前没有旧 App 退出后的可见取消入口，健康标记前新版会打开真实 userData。独立控制进程、helper 阶段 journal/取消能力、隔离健康探测与结果持久反馈待实现；1961de3 五故障通过不代证取消。
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4960,7 +4965,9 @@
 历史自动测试 96e99be；2026-10-02 44a96e8 本机升级脚本通过；2026-10-03 b224dde 隔离取消和打开失败补验，开发工作树 test-results/manual/evidence/TC-036-cancel.log；边界见 docs/validation.md；2026-10-03 新计划：辅助进程限制包和目标路径、等待旧 PID 退出、挂载已校验 DMG、同卷暂存/备份/替换、启动新版并确认健康；失败还原旧版并卸载清理。只读 DMG 运行须告知目标：当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启 ~/Applications/Token.app；已有不可写系统安装须明确授权或报错，不能静默迁址；用户数据不随 App 包删除。重写 TC-036 单元断言，新增 TC-076 真正旧/新打包 App 独立隔离测试；受信登录/safeStorage 必须实测，不能借用旧脚本。
 86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。
 2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。
-2026-10-04 1961de3：TC-076 三段集成绑定中的新增 scripts/verify-packaged-helper-faults.mjs 在隔离临时目录经旧 UI 触发真实打包 helper；文档会话完整命令 exit 0、TC-036 两项单元 exit 0。未测真实满盘/进程崩溃/系统安装/签名公证异机。</x:v>
+2026-10-04 1961de3：TC-076 三段集成绑定中的新增 scripts/verify-packaged-helper-faults.mjs 在隔离临时目录经旧 UI 触发真实打包 helper；文档会话完整命令 exit 0、TC-036 两项单元 exit 0。未测真实满盘/进程崩溃/系统安装/签名公证异机。
+2026-10-04 下一任务：管理员授权的一次性取消能力及独立更新控制窗口；下载 AbortController、helper 阶段/回执/安全检查点、替换后回滚、隔离健康探测防真实 userData 迁移、终态可重启读取和中断恢复。成功提交后取消 too_late；系统级断电自动恢复若承诺须另有 bundle 外恢复入口。
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -8989,11 +8996,15 @@
       </x:c>
       <x:c r="F81" s="52" t="str">
         <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。分别注入取消、磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
-2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。</x:v>
+2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。
+2026-10-04 待新增打包版真点击取消：下载中、校验交接前、旧版退出后挂载/暂存、旧版移动后、健康探测中；另造阻塞步骤等待、重复点击、viewer/伪造请求、成功前后竞态及隔离强杀后的 journal 恢复。
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
       <x:c r="G81" s="52" t="str">
         <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。
-2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。</x:v>
+2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。
+仅 helper 完成回执后称已取消；前段保留旧 App，替换后恢复旧版与受信登录/1280 Token，真实 userData 不受候选探测写入；无挂载/备份/下载残留。成功提交后拒绝迟到取消且新版保持；恢复失败保存备份并提示人工处理。
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
         <x:v>已注册；1961de3 真实 DMG 隔离成功升级、只读旧包初始启动、installer 模块及打包 helper 五故障回退/重试自动子范围独立通过；真实系统目录/满盘/崩溃/安装中取消待验</x:v>
@@ -9016,7 +9027,8 @@
         <x:v>当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
 0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。
 2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。
-2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。</x:v>
+2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。
+2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。

</xml_diff>

<commit_message>
docs: define unknown telemetry identity authorization boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2a181b34e7494eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1b6a3ee198894dd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf97cf909a7cc46aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rca4248ad276e4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R26e51d242ba043bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8946cae60a974770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf00dcd6c9bea4df9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb882f9890ed5446b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2821,7 +2821,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="292.5" customHeight="1">
+    <x:row r="98" ht="337.5" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2844,10 +2844,11 @@
         <x:v>8157e2d 已注册；TC-092 单元 1/1 自动子范围通过；共同稳定事件 ID 正向去重待证
 2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="135" customHeight="1">
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+2026-10-04 TC-092 缺 account_id fallback 及同键旧绑定迁移目标已补；未知来源不可绑定，viewer 隔离/管理员提示/脱敏审计待动态复现和修复。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="225" customHeight="1">
       <x:c r="A99" s="64" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2868,10 +2869,11 @@
       </x:c>
       <x:c r="G99" s="72" t="str">
         <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验
-2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="95" customHeight="1">
+2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。
+2026-10-04 TC-093 关联 viewer 报表/明细/CSV/来源状态、诊断与通用提示回归待补，不改变既有通过子范围。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="225" customHeight="1">
       <x:c r="A100" s="67" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2891,7 +2893,8 @@
         <x:v>服务上报与本地冲突计量同口径</x:v>
       </x:c>
       <x:c r="G100" s="67" t="str">
-        <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验</x:v>
+        <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验
+2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4275,7 +4278,8 @@
 CSV 冲突契约：v2 沿用时间桶+提供方+模型+项目键一组一行，逐组只填该组已确认小计，不在多个冲突行重复全查询小计；冲突行旧数值列空，末四列状态/小计/白名单来源/条数，整份文件显式标 v2。无冲突仍用 v1 十列。
 服务 v2 旧值：迁移历史 v1 聚合/覆盖先标 legacy/unverified，旧客户端继续上报也不得标 confirmed；同设备成功接收 v2 后拒绝任何 v1（包括更高 revision），且旧聚合/覆盖/状态/修订不变。只有授权 v2 当前事实重算后按证据变为 confirmed 或 uncertain。
 viewer 来源状态隔离：报表 coverage、sources:statuses 和概览/报表来源信息只能含当前登录用户及授权查询范围可证明归属的记录数、扫描/遥测时间、状态和诊断细节；不能返回其他 owner 的全局元数据。来源级证据无法归属时显示未知/未覆盖及空值，不得伪装成真零；管理员全局范围须明确。
-同一授权边界覆盖 sources:diagnostics 与 feedback:submit 可选诊断附件；按 provider 筛选不能代表按 owner 隔离。viewer 可得通用修复建议和本人可证状态，跨 owner 位置、原因、各类计数与时间须过滤或未知；勾选附件不扩大读取权限。</x:v>
+同一授权边界覆盖 sources:diagnostics 与 feedback:submit 可选诊断附件；按 provider 筛选不能代表按 owner 隔离。viewer 可得通用修复建议和本人可证状态，跨 owner 位置、原因、各类计数与时间须过滤或未知；勾选附件不扩大读取权限。
+2026-10-04 身份边界：Codex OTel 缺可证 user.account_id 时不得以 macOS username 归属；新事实进入独立 unknown 来源，旧 fallback 已绑定需审计证据并保守暂停不可拆分的历史归属。普通用户报表/明细/CSV/来源状态与上报均不得获得未知事实；管理员诊断显示“账户身份无法验证，历史归属已暂停”及重新启用带 account_id 遥测的行动。受影响 viewer 仅有通用提示，审计不含原始 account/session。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4299,7 +4303,8 @@
 47b03d5：TC-093 Electron 增 viewer sources:scan 直调拒绝、概览同提供方 B 计数/遥测时间不出现；TC-023 v2 公式转义第二绑定、TC-079 v2 旧快照拒绝均已独立复跑通过。固定提交 gate 82 入口/57 单元/22 Electron 通过。真实冲突事实完整 Electron UI、共同事件 ID 正向去重、生产迁移及 REQ-040 仍待验。
 2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5745,7 +5750,8 @@
 47b03d5：TC-093 补概览 B 值隔离和 sources:scan viewer 拒绝；TC-023/079 补 v2 公式转义与旧快照拒绝。文档会话三编号及 gate 82 入口/57 unit/22 E2E 均退出码 0；真实生产迁移/共同事件 ID 正向去重/REQ-040 仍独立待验。
 2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+缺 account_id 不可用 hash(os.username) 作可绑定来源：新写入独立 unknown 命名空间，主进程预览/确认拒绑定；旧绑定逐来源审计，无法区分 account_id==username 同键时撤销归属并记录影响。重算本地查询、v2 待传和服务旧 owner 聚合；管理员/受影响 viewer 按角色给行动与通用提示，最小脱敏审计。历史事实不可自动重建。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9795,13 +9801,15 @@
         <x:v>隔离库同日构造 owner A 本地 12、owner B 遥测 99；同 owner 不同会话 7、同会话 14 和未知会话 5，按管理员及两个 viewer 查询。
 2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+待新增无 user.account_id Codex OTel 同机 A/B 账户样本；另有真实 account_id==macOS username 与缺 ID 同键旧库、已绑定 fallback owner A；迁移后分别以 viewer A/B、管理员调用报表/明细/CSV/来源状态/诊断/绑定预览确认及在线/离线上报。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
 双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+缺身份事实未归属且不可重绑，普通用户各路径无此事实或跨 owner 元数据；管理员可见身份未知与重新启用含 account_id 遥测行动，受影响 viewer 有通用提示；旧混合键无法拆分则保守暂停并记录可能合法事实受影响。迁移幂等、旧 owner 服务聚合清理或待传、脱敏审计无原始 account/session。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9819,7 +9827,8 @@
         <x:v>当前本地与 OTel 无共同稳定事件 ID；同会话只标待核对，不作正向精确去重通过声明。仅隔离合成库。
 静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
-2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。</x:v>
+2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
+新身份边界未动态复现/修复或执行新断言；旧 TC-092 自动子结果不覆盖缺 ID fallback、同键 account_id==username、旧绑定撤销与 viewer/服务回归。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
@@ -9870,7 +9879,8 @@
       </x:c>
       <x:c r="L98" s="64" t="str">
         <x:v>47b03d5 阶段已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。47b03d5 阶段 TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。
-2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。</x:v>
+2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。
+关联 TC-093 回归：缺身份/旧绑定撤销后，viewer 概览/报表/明细/CSV v2、来源状态、诊断和可选反馈附件不得泄露未知事实；受影响本人仅见通用提示。新断言未执行。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
@@ -9916,7 +9926,8 @@
         <x:v>scripts/test-cases.mjs：tests/sync-reconciliation.test.ts 中以 TC-094 开头的独立 Vitest 函数，使用合成客户端与隔离本机服务库。</x:v>
       </x:c>
       <x:c r="L99" s="67" t="str">
-        <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。</x:v>
+        <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。
+关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>

</xml_diff>

<commit_message>
docs: define legacy source rescan and startup sync acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R26e51d242ba043bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8946cae60a974770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf00dcd6c9bea4df9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rb882f9890ed5446b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re8882e34f65c4fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rad6713bdcc4f4c91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4c59bb3ccb494227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5cadbd78707d4762"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2821,7 +2821,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="337.5" customHeight="1">
+    <x:row r="98" ht="465" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2845,10 +2845,11 @@
 2026-10-04 TC-092 新增跨账户同字段 OTel source_key 碰撞与迁移幂等目标；静态发现，代码未修、测试未运行，历史覆盖未知。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-2026-10-04 TC-092 缺 account_id fallback 及同键旧绑定迁移目标已补；未知来源不可绑定，viewer 隔离/管理员提示/脱敏审计待动态复现和修复。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="225" customHeight="1">
+2026-10-04 TC-092 缺 account_id fallback 及同键旧绑定迁移目标已补；未知来源不可绑定，viewer 隔离/管理员提示/脱敏审计待动态复现和修复。
+2026-10-04 旧本地 legacy-unverified 迁移、重扫成功/失败提示、清理与真实启动首次 flush 顺序补入 TC-092；凡影响授权或已确认小计/状态，旧 v1/v2 outbox 均先持久替换；同 owner 旧 OTel confirmed 降 uncertain，待动态验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="277.5" customHeight="1">
       <x:c r="A99" s="64" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2870,10 +2871,11 @@
       <x:c r="G99" s="72" t="str">
         <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验
 2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。
-2026-10-04 TC-093 关联 viewer 报表/明细/CSV/来源状态、诊断与通用提示回归待补，不改变既有通过子范围。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="225" customHeight="1">
+2026-10-04 TC-093 关联 viewer 报表/明细/CSV/来源状态、诊断与通用提示回归待补，不改变既有通过子范围。
+2026-10-04 TC-093 关联迁移期/失败/恢复后的 viewer 页面、CSV、来源状态通用提示与隔离，待验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="270" customHeight="1">
       <x:c r="A100" s="67" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2894,7 +2896,8 @@
       </x:c>
       <x:c r="G100" s="67" t="str">
         <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验
-2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。</x:v>
+2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。
+2026-10-04 TC-094 关联真实主进程启动与在线服务：首次 flush 前受影响的旧 v1/v2 outbox 替换、旧 owner 聚合删除和同 owner 旧 OTel confirmed 降 uncertain；手动排队单测不足，待验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4279,7 +4282,8 @@
 服务 v2 旧值：迁移历史 v1 聚合/覆盖先标 legacy/unverified，旧客户端继续上报也不得标 confirmed；同设备成功接收 v2 后拒绝任何 v1（包括更高 revision），且旧聚合/覆盖/状态/修订不变。只有授权 v2 当前事实重算后按证据变为 confirmed 或 uncertain。
 viewer 来源状态隔离：报表 coverage、sources:statuses 和概览/报表来源信息只能含当前登录用户及授权查询范围可证明归属的记录数、扫描/遥测时间、状态和诊断细节；不能返回其他 owner 的全局元数据。来源级证据无法归属时显示未知/未覆盖及空值，不得伪装成真零；管理员全局范围须明确。
 同一授权边界覆盖 sources:diagnostics 与 feedback:submit 可选诊断附件；按 provider 筛选不能代表按 owner 隔离。viewer 可得通用修复建议和本人可证状态，跨 owner 位置、原因、各类计数与时间须过滤或未知；勾选附件不扩大读取权限。
-2026-10-04 身份边界：Codex OTel 缺可证 user.account_id 时不得以 macOS username 归属；新事实进入独立 unknown 来源，旧 fallback 已绑定需审计证据并保守暂停不可拆分的历史归属。普通用户报表/明细/CSV/来源状态与上报均不得获得未知事实；管理员诊断显示“账户身份无法验证，历史归属已暂停”及重新启用带 account_id 遥测的行动。受影响 viewer 仅有通用提示，审计不含原始 account/session。</x:v>
+2026-10-04 身份边界：Codex OTel 缺可证 user.account_id 时不得以 macOS username 归属；新事实进入独立 unknown 来源，旧 fallback 已绑定需审计证据并保守暂停不可拆分的历史归属。普通用户报表/明细/CSV/来源状态与上报均不得获得未知事实；管理员诊断显示“账户身份无法验证，历史归属已暂停”及重新启用带 account_id 遥测的行动。受影响 viewer 仅有通用提示，审计不含原始 account/session。
+2026-10-04 旧本地来源迁移：旧 Codex/Claude 事实暂入 legacy-unverified 未归属期间，受影响 viewer 须见不含来源细节的“历史归属正在核对”；缺文件、拒权或无法解析而重扫失败时，显示“无法完成重扫/历史仍待核对”，不能默默显示真零。管理员须有重扫与权限授权后重试行动；仅可证身份及授权归属后恢复。成功后清除无事实临时来源，保留脱敏审计。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4304,7 +4308,8 @@
 2026-10-04 81c271b 增 TC-093 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路；文档会话单编号 unit 1/1、Electron 2/2 通过。另静态发现不同 account_id 的同 session/时间/模型/Token OTel 事件 source_key 碰撞，第二条可被 INSERT OR IGNORE 丢弃；DEV-057/TC-092 待修/待新增正例。旧库已丢事实不可重建，历史覆盖未知。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。</x:v>
+旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。
+旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5751,7 +5756,8 @@
 2026-10-04 81c271b/TC-093 已补真实隔离输入端到端。待修 Codex OTel 跨账户事实键碰撞：将不可逆账户身份纳入幂等键，迁移/新旧键别名保证同一历史事件重送不双计、项目关联/授权归属保留；旧键碰撞丢失事实不可重建、覆盖未知。TC-092 增双账户同字段各自入库及同账户重发幂等。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-缺 account_id 不可用 hash(os.username) 作可绑定来源：新写入独立 unknown 命名空间，主进程预览/确认拒绑定；旧绑定逐来源审计，无法区分 account_id==username 同键时撤销归属并记录影响。重算本地查询、v2 待传和服务旧 owner 聚合；管理员/受影响 viewer 按角色给行动与通用提示，最小脱敏审计。历史事实不可自动重建。</x:v>
+缺 account_id 不可用 hash(os.username) 作可绑定来源：新写入独立 unknown 命名空间，主进程预览/确认拒绑定；旧绑定逐来源审计，无法区分 account_id==username 同键时撤销归属并记录影响。重算本地查询、v2 待传和服务旧 owner 聚合；管理员/受影响 viewer 按角色给行动与通用提示，最小脱敏审计。历史事实不可自动重建。
+旧本地来源迁移需保存待核对/重扫失败状态，按角色给 viewer 通用提示与管理员重扫/权限动作；可证重归属后清理零事实 legacy-unverified 来源行/绑定候选，保留不透明审计引用；重试幂等。启动时任何影响授权或已确认小计/状态的迁移后，先持久重算替换旧 v1/v2 outbox，失败阻断旧包，随后才允许 UsageSync 首次 flush；旧 owner 聚合清除，同 owner 旧 OTel 键转 legacy_otel_identity_unknown 时旧 confirmed 降 uncertain。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9802,14 +9808,16 @@
 2026-10-04 待补 Codex OTel 双 account_id、同 session/UTC 时间/模型/输入/输出/缓存双事件，绑定不同 owner 并重发同账户事件；旧库键迁移重放及缺身份反例。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-待新增无 user.account_id Codex OTel 同机 A/B 账户样本；另有真实 account_id==macOS username 与缺 ID 同键旧库、已绑定 fallback owner A；迁移后分别以 viewer A/B、管理员调用报表/明细/CSV/来源状态/诊断/绑定预览确认及在线/离线上报。</x:v>
+待新增无 user.account_id Codex OTel 同机 A/B 账户样本；另有真实 account_id==macOS username 与缺 ID 同键旧库、已绑定 fallback owner A；迁移后分别以 viewer A/B、管理员调用报表/明细/CSV/来源状态/诊断/绑定预览确认及在线/离线上报。
+新增旧库：Codex/Claude 已绑定 viewer 的历史事实和旧 v1/v2 outbox，触发 legacy-unverified 迁移；分别模拟可证重扫成功、文件缺失、权限拒绝、不可读/无法解析、取消和重启重试；另造有 account_id、owner 不变但旧 OTel 键被迁为 legacy_otel_identity_unknown 的 confirmed 快照；真实主进程启动并连接在线服务。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
 双账户事实各自入库且 viewer 授权隔离；同账户重发幂等；新旧键重放不双计，项目关联/归属不丢；旧碰撞丢失不可重建，历史覆盖未知。原始账户/会话 ID 不外露。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-缺身份事实未归属且不可重绑，普通用户各路径无此事实或跨 owner 元数据；管理员可见身份未知与重新启用含 account_id 遥测行动，受影响 viewer 有通用提示；旧混合键无法拆分则保守暂停并记录可能合法事实受影响。迁移幂等、旧 owner 服务聚合清理或待传、脱敏审计无原始 account/session。</x:v>
+缺身份事实未归属且不可重绑，普通用户各路径无此事实或跨 owner 元数据；管理员可见身份未知与重新启用含 account_id 遥测行动，受影响 viewer 有通用提示；旧混合键无法拆分则保守暂停并记录可能合法事实受影响。迁移幂等、旧 owner 服务聚合清理或待传、脱敏审计无原始 account/session。
+迁移期间 viewer 旧历史暂不可见但有“历史归属正在核对”通用提示，失败后显示“无法完成重扫/历史仍待核对”，管理员有可操作重扫/权限行动；仅可证授权后恢复，不重复计量或泄露。成功后零事实临时来源不留归属表/候选，脱敏审计保留。任何影响授权或已确认小计/状态的迁移后，首次 flush 前持久替换旧 outbox 为重算的 v2；旧包从未发送，在线旧 owner 聚合删除，同 owner 旧 OTel confirmed 降 uncertain。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9828,7 +9836,8 @@
 静态发现 source_key 未含账户身份而 identity 含账户哈希，usage_facts 主键 + INSERT OR IGNORE 可静默丢第二账户；新断言未实现/未运行。
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
-新身份边界未动态复现/修复或执行新断言；旧 TC-092 自动子结果不覆盖缺 ID fallback、同键 account_id==username、旧绑定撤销与 viewer/服务回归。</x:v>
+新身份边界未动态复现/修复或执行新断言；旧 TC-092 自动子结果不覆盖缺 ID fallback、同键 account_id==username、旧绑定撤销与 viewer/服务回归。
+旧来源重扫 UX、零事实清理及任何影响授权或已确认小计/状态的迁移后，主进程启动/首次上传顺序为新增待验断言；手动调用 queueSnapshot 单测不能证明，既有 TC-092 通过子范围不覆盖。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
@@ -9880,7 +9889,8 @@
       <x:c r="L98" s="64" t="str">
         <x:v>47b03d5 阶段已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。47b03d5 阶段 TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。
 2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。
-关联 TC-093 回归：缺身份/旧绑定撤销后，viewer 概览/报表/明细/CSV v2、来源状态、诊断和可选反馈附件不得泄露未知事实；受影响本人仅见通用提示。新断言未执行。</x:v>
+关联 TC-093 回归：缺身份/旧绑定撤销后，viewer 概览/报表/明细/CSV v2、来源状态、诊断和可选反馈附件不得泄露未知事实；受影响本人仅见通用提示。新断言未执行。
+关联 TC-093：迁移中/重扫失败时概览、报表、明细、CSV、来源状态给本人通用提示，不泄露来源或其他用户；成功恢复后数值与提示同步。待验。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
@@ -9927,7 +9937,8 @@
       </x:c>
       <x:c r="L99" s="67" t="str">
         <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。
-关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。</x:v>
+关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。
+关联 TC-094：预置旧 v1/v2 outbox，任何影响授权或已确认小计/状态的迁移，真实启动首次 flush 前持久替换；在线服务删除旧 owner 聚合，同 owner 旧 OTel confirmed 降 uncertain；离线/替换失败时旧包不能外传，恢复后只传新 v2。待验。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>

</xml_diff>

<commit_message>
docs: extend telemetry identity acceptance to Claude
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re8882e34f65c4fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rad6713bdcc4f4c91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4c59bb3ccb494227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5cadbd78707d4762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ce0ea4a7f184a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R16d983a73bac4161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rff39693aa8f04836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R6ced2c92eeea4bf5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2821,7 +2821,7 @@
         <x:v>文案组合自动子范围通过；真零/发布待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" ht="465" customHeight="1">
+    <x:row r="98" ht="615" customHeight="1">
       <x:c r="A98" s="61" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2846,10 +2846,12 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 2026-10-04 TC-092 缺 account_id fallback 及同键旧绑定迁移目标已补；未知来源不可绑定，viewer 隔离/管理员提示/脱敏审计待动态复现和修复。
-2026-10-04 旧本地 legacy-unverified 迁移、重扫成功/失败提示、清理与真实启动首次 flush 顺序补入 TC-092；凡影响授权或已确认小计/状态，旧 v1/v2 outbox 均先持久替换；同 owner 旧 OTel confirmed 降 uncertain，待动态验收。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99" ht="277.5" customHeight="1">
+2026-10-04 旧本地 legacy-unverified 迁移、重扫成功/失败提示、清理与真实启动首次 flush 顺序补入 TC-092；凡影响授权或已确认小计/状态，旧 v1/v2 outbox 均先持久替换；同 owner 旧 OTel confirmed 降 uncertain，待动态验收。
+2026-10-04 TC-092 新增 Claude 缺/空/无效/超长 user.id、安装 ID 非账户、旧混合键及双账户同 stream/time 累计游标碰撞反例；无法证重送标 uncertain，待验。
+2026-10-04 Codex unknown 两账户同字段双 POST 与真正重送对照待验；缺稳定 ID 保留观测并标 uncertain，旧身份可证子范围不变。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="330" customHeight="1">
       <x:c r="A99" s="64" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2872,10 +2874,11 @@
         <x:v>47b03d5 已注册；TC-093 单元+Electron 各 1/1 自动子范围通过，概览 B 值/sources:scan 与 v2 公式/快照回归已补；真实冲突事实完整 E2E/生产待验
 2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。
 2026-10-04 TC-093 关联 viewer 报表/明细/CSV/来源状态、诊断与通用提示回归待补，不改变既有通过子范围。
-2026-10-04 TC-093 关联迁移期/失败/恢复后的 viewer 页面、CSV、来源状态通用提示与隔离，待验。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100" ht="270" customHeight="1">
+2026-10-04 TC-093 关联迁移期/失败/恢复后的 viewer 页面、CSV、来源状态通用提示与隔离，待验。
+2026-10-04 TC-093 新增 Claude unknown 与旧归属撤销后的 viewer 页面/CSV/来源状态/诊断附件隔离，待验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="322.5" customHeight="1">
       <x:c r="A100" s="67" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2897,7 +2900,8 @@
       <x:c r="G100" s="67" t="str">
         <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验
 2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。
-2026-10-04 TC-094 关联真实主进程启动与在线服务：首次 flush 前受影响的旧 v1/v2 outbox 替换、旧 owner 聚合删除和同 owner 旧 OTel confirmed 降 uncertain；手动排队单测不足，待验。</x:v>
+2026-10-04 TC-094 关联真实主进程启动与在线服务：首次 flush 前受影响的旧 v1/v2 outbox 替换、旧 owner 聚合删除和同 owner 旧 OTel confirmed 降 uncertain；手动排队单测不足，待验。
+2026-10-04 TC-094 新增 Claude unknown 或累计降级后的首次 flush 前快照重算与在线旧聚合清理/降级，待验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4283,7 +4287,9 @@
 viewer 来源状态隔离：报表 coverage、sources:statuses 和概览/报表来源信息只能含当前登录用户及授权查询范围可证明归属的记录数、扫描/遥测时间、状态和诊断细节；不能返回其他 owner 的全局元数据。来源级证据无法归属时显示未知/未覆盖及空值，不得伪装成真零；管理员全局范围须明确。
 同一授权边界覆盖 sources:diagnostics 与 feedback:submit 可选诊断附件；按 provider 筛选不能代表按 owner 隔离。viewer 可得通用修复建议和本人可证状态，跨 owner 位置、原因、各类计数与时间须过滤或未知；勾选附件不扩大读取权限。
 2026-10-04 身份边界：Codex OTel 缺可证 user.account_id 时不得以 macOS username 归属；新事实进入独立 unknown 来源，旧 fallback 已绑定需审计证据并保守暂停不可拆分的历史归属。普通用户报表/明细/CSV/来源状态与上报均不得获得未知事实；管理员诊断显示“账户身份无法验证，历史归属已暂停”及重新启用带 account_id 遥测的行动。受影响 viewer 仅有通用提示，审计不含原始 account/session。
-2026-10-04 旧本地来源迁移：旧 Codex/Claude 事实暂入 legacy-unverified 未归属期间，受影响 viewer 须见不含来源细节的“历史归属正在核对”；缺文件、拒权或无法解析而重扫失败时，显示“无法完成重扫/历史仍待核对”，不能默默显示真零。管理员须有重扫与权限授权后重试行动；仅可证身份及授权归属后恢复。成功后清除无事实临时来源，保留脱敏审计。</x:v>
+2026-10-04 旧本地来源迁移：旧 Codex/Claude 事实暂入 legacy-unverified 未归属期间，受影响 viewer 须见不含来源细节的“历史归属正在核对”；缺文件、拒权或无法解析而重扫失败时，显示“无法完成重扫/历史仍待核对”，不能默默显示真零。管理员须有重扫与权限授权后重试行动；仅可证身份及授权归属后恢复。成功后清除无事实临时来源，保留脱敏审计。
+2026-10-04 Claude OTel：缺失、空白、非字符串、超长 user.id 或仅有安装级 user.id 均不足以证明 Claude 账户归属，新事实进入独立 unknown 且不可绑定；旧 username/hash(空串)/安装 ID 混合来源无法拆分时撤销归属。viewer 页面/CSV/来源状态/上报隔离，管理员可见脱敏诊断。累计游标与事实键不得跨账户静默合并/错算；无法证重送则保留观测并标待核对，不报完整总量。
+Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4309,7 +4315,8 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。
-旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。</x:v>
+旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。
+Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5757,7 +5764,9 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 缺 account_id 不可用 hash(os.username) 作可绑定来源：新写入独立 unknown 命名空间，主进程预览/确认拒绑定；旧绑定逐来源审计，无法区分 account_id==username 同键时撤销归属并记录影响。重算本地查询、v2 待传和服务旧 owner 聚合；管理员/受影响 viewer 按角色给行动与通用提示，最小脱敏审计。历史事实不可自动重建。
-旧本地来源迁移需保存待核对/重扫失败状态，按角色给 viewer 通用提示与管理员重扫/权限动作；可证重归属后清理零事实 legacy-unverified 来源行/绑定候选，保留不透明审计引用；重试幂等。启动时任何影响授权或已确认小计/状态的迁移后，先持久重算替换旧 v1/v2 outbox，失败阻断旧包，随后才允许 UsageSync 首次 flush；旧 owner 聚合清除，同 owner 旧 OTel 键转 legacy_otel_identity_unknown 时旧 confirmed 降 uncertain。</x:v>
+旧本地来源迁移需保存待核对/重扫失败状态，按角色给 viewer 通用提示与管理员重扫/权限动作；可证重归属后清理零事实 legacy-unverified 来源行/绑定候选，保留不透明审计引用；重试幂等。启动时任何影响授权或已确认小计/状态的迁移后，先持久重算替换旧 v1/v2 outbox，失败阻断旧包，随后才允许 UsageSync 首次 flush；旧 owner 聚合清除，同 owner 旧 OTel 键转 legacy_otel_identity_unknown 时旧 confirmed 降 uncertain。
+Claude telemetry.ts 的 string() 接受空串而 hash(空串) 可绑定，缺/无效/超长退回 os.username；改为按可证认证账户属性或经验证网关 subject 判归属，其余 unknown。旧混合键保守撤销并重算本地/服务授权；隔离累计 stream、otel_metric_cursors 和事实键，避免双账户缺 ID 同 stream/time 的丢点或错算。无法证重送保留观测并标 uncertain；首次 flush 前持久替换受影响快照。
+开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9809,7 +9818,9 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 待新增无 user.account_id Codex OTel 同机 A/B 账户样本；另有真实 account_id==macOS username 与缺 ID 同键旧库、已绑定 fallback owner A；迁移后分别以 viewer A/B、管理员调用报表/明细/CSV/来源状态/诊断/绑定预览确认及在线/离线上报。
-新增旧库：Codex/Claude 已绑定 viewer 的历史事实和旧 v1/v2 outbox，触发 legacy-unverified 迁移；分别模拟可证重扫成功、文件缺失、权限拒绝、不可读/无法解析、取消和重启重试；另造有 account_id、owner 不变但旧 OTel 键被迁为 legacy_otel_identity_unknown 的 confirmed 快照；真实主进程启动并连接在线服务。</x:v>
+新增旧库：Codex/Claude 已绑定 viewer 的历史事实和旧 v1/v2 outbox，触发 legacy-unverified 迁移；分别模拟可证重扫成功、文件缺失、权限拒绝、不可读/无法解析、取消和重启重试；另造有 account_id、owner 不变但旧 OTel 键被迁为 legacy_otel_identity_unknown 的 confirmed 快照；真实主进程启动并连接在线服务。
+新增 Claude OTel 同机账户 A/B：user.id 缺失、空串、空白、非字符串、超过 200 字符及两账户共用安装 ID；对照有可验证认证账户属性或网关 OIDC subject 的样本。旧库预绑 username/hash(空串) 混合键。两账户缺 ID 且 session/model/category/start/time 全同，累计值不同，再给各自后续点与真正重送。
+再造 Codex 账户 A/B 均无 user.account_id，分两次 POST 且 session/rawTime/model/Token 全同；另造同一真实事件的重送对照。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
@@ -9817,7 +9828,9 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 缺身份事实未归属且不可重绑，普通用户各路径无此事实或跨 owner 元数据；管理员可见身份未知与重新启用含 account_id 遥测行动，受影响 viewer 有通用提示；旧混合键无法拆分则保守暂停并记录可能合法事实受影响。迁移幂等、旧 owner 服务聚合清理或待传、脱敏审计无原始 account/session。
-迁移期间 viewer 旧历史暂不可见但有“历史归属正在核对”通用提示，失败后显示“无法完成重扫/历史仍待核对”，管理员有可操作重扫/权限行动；仅可证授权后恢复，不重复计量或泄露。成功后零事实临时来源不留归属表/候选，脱敏审计保留。任何影响授权或已确认小计/状态的迁移后，首次 flush 前持久替换旧 outbox 为重算的 v2；旧包从未发送，在线旧 owner 聚合删除，同 owner 旧 OTel confirmed 降 uncertain。</x:v>
+迁移期间 viewer 旧历史暂不可见但有“历史归属正在核对”通用提示，失败后显示“无法完成重扫/历史仍待核对”，管理员有可操作重扫/权限行动；仅可证授权后恢复，不重复计量或泄露。成功后零事实临时来源不留归属表/候选，脱敏审计保留。任何影响授权或已确认小计/状态的迁移后，首次 flush 前持久替换旧 outbox 为重算的 v2；旧包从未发送，在线旧 owner 聚合删除，同 owner 旧 OTel confirmed 降 uncertain。
+仅安装 ID 不能证明账户；缺/空/无效/超长来源 unknown、不可绑定，旧混合键保守撤销，viewer A/B 全路径隔离、管理员脱敏诊断。相同 stream/time 的不同账户点不得静默丢失，后续累计点不得跨账户差分；无法证重送时保留观测并标 uncertain，已丢历史仍未知。受影响 v2 快照首次 flush 前重算，旧 owner 聚合清除或状态降级。
+不可仅因 unknown:hash(mac username) 键同而静默去重；无法证同一事件时两次观测均保留、计量 uncertain，viewer/上报不称确定总量。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9837,7 +9850,9 @@
 2026-10-04 补同 owner 事件身份与本地跨来源键空间边界：Codex OTel 纳秒截为毫秒，账户哈希仍不足以区分同账户同毫秒同用量不同事件；无稳定事件 ID 时保留观测并标计量不确定，不得静默丢弃或确认单条为总量。本地 Codex session+response、Claude session+request 键未含来源身份，不同来源/owner 同值 ID 需各自保留并授权隔离；旧键迁移/重放须幂等，项目关联不串户。现仅静态风险和测试设计，未执行新正例。
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 新身份边界未动态复现/修复或执行新断言；旧 TC-092 自动子结果不覆盖缺 ID fallback、同键 account_id==username、旧绑定撤销与 viewer/服务回归。
-旧来源重扫 UX、零事实清理及任何影响授权或已确认小计/状态的迁移后，主进程启动/首次上传顺序为新增待验断言；手动调用 queueSnapshot 单测不能证明，既有 TC-092 通过子范围不覆盖。</x:v>
+旧来源重扫 UX、零事实清理及任何影响授权或已确认小计/状态的迁移后，主进程启动/首次上传顺序为新增待验断言；手动调用 queueSnapshot 单测不能证明，既有 TC-092 通过子范围不覆盖。
+Claude user.id 安装级语义及缺/空/无效/超长、双账户同 stream/time 游标碰撞是新增待验反例；现有 TC-092 自动子结果不覆盖，未动态复现或修复。
+Codex unknown 同键双 POST 与真正重送的新反例未动态运行；身份可证旧通过子范围结论不变。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
@@ -9890,7 +9905,8 @@
         <x:v>47b03d5 阶段已证 viewer 状态/诊断/反馈附件 IPC、概览同提供方 B 值排除、sources:scan 拒绝，以及 v2 CSV 单元、TC-023 v2 公式转义、TC-079 v2 旧快照拒绝。47b03d5 阶段 TC-093 冲突 UI 文案仍用注入响应，真实冲突事实完整 Electron 流程、生产数据与共同事件 ID 正向去重未验。
 2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。
 关联 TC-093 回归：缺身份/旧绑定撤销后，viewer 概览/报表/明细/CSV v2、来源状态、诊断和可选反馈附件不得泄露未知事实；受影响本人仅见通用提示。新断言未执行。
-关联 TC-093：迁移中/重扫失败时概览、报表、明细、CSV、来源状态给本人通用提示，不泄露来源或其他用户；成功恢复后数值与提示同步。待验。</x:v>
+关联 TC-093：迁移中/重扫失败时概览、报表、明细、CSV、来源状态给本人通用提示，不泄露来源或其他用户；成功恢复后数值与提示同步。待验。
+关联 TC-093：Claude unknown 或旧混合键撤销后 viewer 概览/报表/明细/CSV/来源状态/诊断附件无其他账户事实，仅通用提示；新断言待验。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
@@ -9938,7 +9954,8 @@
       <x:c r="L99" s="67" t="str">
         <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。
 关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。
-关联 TC-094：预置旧 v1/v2 outbox，任何影响授权或已确认小计/状态的迁移，真实启动首次 flush 前持久替换；在线服务删除旧 owner 聚合，同 owner 旧 OTel confirmed 降 uncertain；离线/替换失败时旧包不能外传，恢复后只传新 v2。待验。</x:v>
+关联 TC-094：预置旧 v1/v2 outbox，任何影响授权或已确认小计/状态的迁移，真实启动首次 flush 前持久替换；在线服务删除旧 owner 聚合，同 owner 旧 OTel confirmed 降 uncertain；离线/替换失败时旧包不能外传，恢复后只传新 v2。待验。
+关联 TC-094：Claude 旧混合键归属撤销或累计状态降 uncertain 后，真实启动首次 flush 前替换 v1/v2 outbox，在线清旧 owner 聚合或降状态；未知事实不按旧 owner 上传。待验。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>

</xml_diff>

<commit_message>
docs: track in-flight snapshot drain failure
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6ce0ea4a7f184a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R16d983a73bac4161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rff39693aa8f04836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R6ced2c92eeea4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf00897d63a81411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcefcae8d227c4478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R41ace9e714664575"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0bc7ca2e1ea9465c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1587,7 +1587,7 @@
         <x:v>已验证（自动；范围见文档）</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="62" customHeight="1">
+    <x:row r="45" ht="142.5" customHeight="1">
       <x:c r="A45" s="35" t="str">
         <x:v>REQ-026</x:v>
       </x:c>
@@ -1607,7 +1607,8 @@
         <x:v>离线重试与状态</x:v>
       </x:c>
       <x:c r="G45" s="35" t="str">
-        <x:v>已验证（自动；范围见文档）</x:v>
+        <x:v>已验证（自动；范围见文档）
+2026-10-04 TC-040 新增发送中排快照立即顺序 drain 与失败退避/状态断言；开发会话真实启动诊断 pending=1、修订未确认，当前失败待修，旧自动通过子范围保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="62" customHeight="1">
@@ -2878,7 +2879,7 @@
 2026-10-04 TC-093 新增 Claude unknown 与旧归属撤销后的 viewer 页面/CSV/来源状态/诊断附件隔离，待验。</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="322.5" customHeight="1">
+    <x:row r="100" ht="375" customHeight="1">
       <x:c r="A100" s="67" t="str">
         <x:v>REQ-048</x:v>
       </x:c>
@@ -2901,7 +2902,8 @@
         <x:v>8157e2d 已注册；TC-094 隔离服务单元 1/1 自动子范围通过；旧值 legacy_unknown，真实生产迁移/旧服务互操作待验
 2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。
 2026-10-04 TC-094 关联真实主进程启动与在线服务：首次 flush 前受影响的旧 v1/v2 outbox 替换、旧 owner 聚合删除和同 owner 旧 OTel confirmed 降 uncertain；手动排队单测不足，待验。
-2026-10-04 TC-094 新增 Claude unknown 或累计降级后的首次 flush 前快照重算与在线旧聚合清理/降级，待验。</x:v>
+2026-10-04 TC-094 新增 Claude unknown 或累计降级后的首次 flush 前快照重算与在线旧聚合清理/降级，待验。
+2026-10-04 TC-094 真实 Electron 启动发送竞态当前失败：迁移首包成功后扫描新 revision 未立即续传；需自动 drain 到服务确认最新 revision 并清旧 owner 聚合，不靠 60 秒定时器。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3659,7 +3661,7 @@
         <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="62" customHeight="1">
+    <x:row r="31" ht="112.5" customHeight="1">
       <x:c r="A31" s="35" t="str">
         <x:v>REQ-026</x:v>
       </x:c>
@@ -3667,7 +3669,8 @@
         <x:v>聚合幂等、重试和状态</x:v>
       </x:c>
       <x:c r="C31" s="35" t="str">
-        <x:v>同一设备、归属用户、统计区间及数据修订只计入一次；重复上报更新快照而不累加；服务不可用时保留待传队列，有限退避重试，并显示最近成功/失败与积压。</x:v>
+        <x:v>同一设备、归属用户、统计区间及数据修订只计入一次；重复上报更新快照而不累加；服务不可用时保留待传队列，有限退避重试，并显示最近成功/失败与积压。
+2026-10-04 发送中排入更高 revision：旧包成功后应立即顺序 drain 最新持久待传快照，最终由服务确认；失败仍守有限退避，待传/错误/确认状态可观察，不靠 60 秒定时器或人工重试。</x:v>
       </x:c>
       <x:c r="D31" s="35" t="str">
         <x:v>M5（计划）</x:v>
@@ -3682,7 +3685,8 @@
         <x:v>TC-039、TC-040</x:v>
       </x:c>
       <x:c r="H31" s="35" t="str">
-        <x:v>docs/design.md §9–13；docs/development-plan.md §7</x:v>
+        <x:v>docs/design.md §9–13；docs/development-plan.md §7
+开发会话真实 Electron 启动诊断：首包成功后留下 pending=1、localRevision&gt;confirmedRevision、lastError=null，直到 60 秒定时器；新交错当前失败待修，旧 TC-040 自动通过仅覆盖原离线补传样本。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -4289,7 +4293,8 @@
 2026-10-04 身份边界：Codex OTel 缺可证 user.account_id 时不得以 macOS username 归属；新事实进入独立 unknown 来源，旧 fallback 已绑定需审计证据并保守暂停不可拆分的历史归属。普通用户报表/明细/CSV/来源状态与上报均不得获得未知事实；管理员诊断显示“账户身份无法验证，历史归属已暂停”及重新启用带 account_id 遥测的行动。受影响 viewer 仅有通用提示，审计不含原始 account/session。
 2026-10-04 旧本地来源迁移：旧 Codex/Claude 事实暂入 legacy-unverified 未归属期间，受影响 viewer 须见不含来源细节的“历史归属正在核对”；缺文件、拒权或无法解析而重扫失败时，显示“无法完成重扫/历史仍待核对”，不能默默显示真零。管理员须有重扫与权限授权后重试行动；仅可证身份及授权归属后恢复。成功后清除无事实临时来源，保留脱敏审计。
 2026-10-04 Claude OTel：缺失、空白、非字符串、超长 user.id 或仅有安装级 user.id 均不足以证明 Claude 账户归属，新事实进入独立 unknown 且不可绑定；旧 username/hash(空串)/安装 ID 混合来源无法拆分时撤销归属。viewer 页面/CSV/来源状态/上报隔离，管理员可见脱敏诊断。累计游标与事实键不得跨账户静默合并/错算；无法证重送则保留观测并标待核对，不报完整总量。
-Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。</x:v>
+Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。
+迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4316,7 +4321,8 @@
 2026-10-04 静态补充：scanner.ts 同 source_key 冲突时，新 totalTokens 较小可被丢弃，较大可覆盖数值但保留首次 source_identity_key，使 B 数值计入 A；fact_projects 可能跟键错配。TC-092 需测 B 较小/较大、项目与授权归属、旧库迁移；已污染历史无法凭现存事实确证恢复。
 旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。
 旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。
-Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。</x:v>
+Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。
+2026-10-04 真实 Electron 启动诊断发现迁移首包成功后更新快照停在 outbox，需等 60 秒定时器；TC-094 新交错为当前失败待修，现有单元通过不能覆盖。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5033,7 +5039,7 @@
         <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="62" customHeight="1">
+    <x:row r="33" ht="131.25" customHeight="1">
       <x:c r="A33" s="35" t="str">
         <x:v>DEV-028</x:v>
       </x:c>
@@ -5053,7 +5059,8 @@
         <x:v>已编码（自动覆盖；边界待验）</x:v>
       </x:c>
       <x:c r="G33" s="35" t="str">
-        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md</x:v>
+        <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md
+修复 UsageSync.flush 发送中排队竞态：旧包成功后比较当前持久 outbox revision 并立即顺序 drain，避免并发重复发送；失败保留错误与待传，按有限退避重试。pending=1 且本地 revision 高于确认 revision 时不得显示已同步。TC-040 增可控延迟/失败断言。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -5766,7 +5773,8 @@
 缺 account_id 不可用 hash(os.username) 作可绑定来源：新写入独立 unknown 命名空间，主进程预览/确认拒绑定；旧绑定逐来源审计，无法区分 account_id==username 同键时撤销归属并记录影响。重算本地查询、v2 待传和服务旧 owner 聚合；管理员/受影响 viewer 按角色给行动与通用提示，最小脱敏审计。历史事实不可自动重建。
 旧本地来源迁移需保存待核对/重扫失败状态，按角色给 viewer 通用提示与管理员重扫/权限动作；可证重归属后清理零事实 legacy-unverified 来源行/绑定候选，保留不透明审计引用；重试幂等。启动时任何影响授权或已确认小计/状态的迁移后，先持久重算替换旧 v1/v2 outbox，失败阻断旧包，随后才允许 UsageSync 首次 flush；旧 owner 聚合清除，同 owner 旧 OTel 键转 legacy_otel_identity_unknown 时旧 confirmed 降 uncertain。
 Claude telemetry.ts 的 string() 接受空串而 hash(空串) 可绑定，缺/无效/超长退回 os.username；改为按可证认证账户属性或经验证网关 subject 判归属，其余 unknown。旧混合键保守撤销并重算本地/服务授权；隔离累计 stream、otel_metric_cursors 和事实键，避免双账户缺 ID 同 stream/time 的丢点或错算。无法证重送保留观测并标 uncertain；首次 flush 前持久替换受影响快照。
-开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。</x:v>
+开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。
+迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7501,7 +7509,7 @@
         <x:v>记录 TC-039 命令、退出码、提交、环境和脱敏日志；覆盖与限制：重复快照和修订替换；未测多设备并发。</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="70" customHeight="1">
+    <x:row r="45" ht="195" customHeight="1">
       <x:c r="A45" s="35" t="str">
         <x:v>TC-040</x:v>
       </x:c>
@@ -7518,13 +7526,15 @@
         <x:v>单元</x:v>
       </x:c>
       <x:c r="F45" s="35" t="str">
-        <x:v>停服完成扫描，检查积压并恢复服务。</x:v>
+        <x:v>停服完成扫描，检查积压并恢复服务。
+旧快照上传响应保持未完成时排入更高 revision，先让旧包成功；另注入上传失败并排入新快照，观察自动续传、退避和状态。</x:v>
       </x:c>
       <x:c r="G45" s="35" t="str">
-        <x:v>有限退避补传，最近错误/成功及积压数量可见。</x:v>
+        <x:v>有限退避补传，最近错误/成功及积压数量可见。
+成功后单发送器立即顺序 drain 最新快照且服务确认最新 revision；失败保留 pending/lastError、守有限退避，恢复后自动补传，无忙循环或 60 秒定时器/人工重试依赖。</x:v>
       </x:c>
       <x:c r="H45" s="35" t="str">
-        <x:v>已验证（自动；边界待验）</x:v>
+        <x:v>旧离线补传自动子范围通过；发送中排新快照未立即续传，当前失败待修</x:v>
       </x:c>
       <x:c r="I45" s="35" t="str">
         <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
@@ -7537,7 +7547,8 @@
         <x:v>tests/next-sync.test.ts：test('TC-040 停服后待传快照持久化并恢复补传')</x:v>
       </x:c>
       <x:c r="L45" s="35" t="str">
-        <x:v>持久待传和恢复补传；未长时间运行验证退避</x:v>
+        <x:v>持久待传和恢复补传；未长时间运行验证退避
+开发会话真实 Electron 启动诊断残留 pending=1、localRevision&gt;confirmedRevision、lastError=null 至 60 秒定时器；新断言未修/未独立复验，旧 TC-040 通过不覆盖。</x:v>
       </x:c>
       <x:c r="M45" s="35" t="str">
         <x:v>记录 TC-040 命令、退出码、提交、环境和脱敏日志；覆盖与限制：持久待传和恢复补传；未长时间运行验证退避。</x:v>
@@ -9915,7 +9926,7 @@
 81c271b；文档会话独立 npm run test:case -- TC-093：unit 1/1、Electron 2/2、exit 0；真实隔离输入 A 本地 12/5、OTel 14，B OTel 99；A 已确认 5、待核对 2、明细 [5,12,14]、CSV v2 14 列/B 仅 99。</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="195" customHeight="1">
+    <x:row r="99" ht="315" customHeight="1">
       <x:c r="A99" s="67" t="str">
         <x:v>TC-094</x:v>
       </x:c>
@@ -9933,14 +9944,16 @@
       </x:c>
       <x:c r="F99" s="67" t="str">
         <x:v>隔离客户端和服务库构造同日跨 owner 本地/遥测、同 owner 疑似重叠；检查扫描后的版本 2 快照、服务端存储/查询、旧完整聚合清除、旧 outbox、旧协议拒绝/恢复重传、设备令牌范围与 TC-088 状态。
-预置有跨 owner 误排除风险的 v1 历史 aggregates/coverage，升级服务后依次发送旧客户端 v1 追加、授权 v2 重算、同设备更高 revision 的 v1 回滚，并另测越权 owner。</x:v>
+预置有跨 owner 误排除风险的 v1 历史 aggregates/coverage，升级服务后依次发送旧客户端 v1 追加、授权 v2 重算、同设备更高 revision 的 v1 回滚，并另测越权 owner。
+真实 Electron 启动预置在线服务旧 owner 聚合；迁移首包上传时延迟响应，扫描排入更高 revision，依次释放服务响应并观察首次上传链路。</x:v>
       </x:c>
       <x:c r="G99" s="67" t="str">
         <x:v>上报与页面/明细/CSV 共用调和版本和授权事实集；跨 owner 独立保留，冲突只传白名单已确认小计、待核对来源/条数及总量不可确认，旧 totalTokens 不冒充完整总量；旧服务安全拒绝并保留待传，旧 outbox 重算或阻断，恢复后 revision 幂等重传。旧完整聚合被清除，越权 403 不改状态，无原始账户、会话 ID、路径或正文；待核对/未同步不混成网络离线/零/扫描失败。
-迁移及旧客户端追加均显示 legacy/unverified，不把旧数值当完整；v2 原子替换后仅可证范围 confirmed、冲突 uncertain；收过 v2 的设备拒绝所有 v1，拒绝前后 aggregates/coverage/状态/revision 完全相同，跨 owner 授权仍拒绝。</x:v>
+迁移及旧客户端追加均显示 legacy/unverified，不把旧数值当完整；v2 原子替换后仅可证范围 confirmed、冲突 uncertain；收过 v2 的设备拒绝所有 v1，拒绝前后 aggregates/coverage/状态/revision 完全相同，跨 owner 授权仍拒绝。
+首包成功后立即顺序 drain 更新 v2，不靠定时器/人工重试；服务确认最新 revision 并删除旧 owner 聚合。失败时保持退避和可观察待传，不把旧包确认误作最新确认。</x:v>
       </x:c>
       <x:c r="H99" s="67" t="str">
-        <x:v>已注册；隔离服务自动子范围 1/1 通过（8157e2d），真实迁移待验证</x:v>
+        <x:v>旧隔离服务自动子范围 1/1 通过（8157e2d）；真实 Electron 启动发送中排新快照未续传，当前失败待修</x:v>
       </x:c>
       <x:c r="I99" s="67" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-094：单元 1/1、退出码 0。合成旧表迁移、旧 v1 续传 legacy_unknown/GET confirmedSubtotal=null、v2 重算及冲突、跨 owner/白名单拒绝、v1 回滚状态不变、旧 outbox 重算及协议不兼容待传后恢复。完整 gate 82/56/22 通过。</x:v>
@@ -9955,7 +9968,8 @@
         <x:v>实际状态名 legacy_unknown，旧 GET confirmedSubtotal=null；测试以合成旧表与模拟旧服务 400 验边界。真实生产库迁移演练、真实旧服务互操作及目标设备未验；旧 200/ready 不证明完整。
 关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。
 关联 TC-094：预置旧 v1/v2 outbox，任何影响授权或已确认小计/状态的迁移，真实启动首次 flush 前持久替换；在线服务删除旧 owner 聚合，同 owner 旧 OTel confirmed 降 uncertain；离线/替换失败时旧包不能外传，恢复后只传新 v2。待验。
-关联 TC-094：Claude 旧混合键归属撤销或累计状态降 uncertain 后，真实启动首次 flush 前替换 v1/v2 outbox，在线清旧 owner 聚合或降状态；未知事实不按旧 owner 上传。待验。</x:v>
+关联 TC-094：Claude 旧混合键归属撤销或累计状态降 uncertain 后，真实启动首次 flush 前替换 v1/v2 outbox，在线清旧 owner 聚合或降状态；未知事实不按旧 owner 上传。待验。
+开发会话真实 Electron 启动诊断：迁移首包成功，扫描在发送中排新 revision；flush 仅等旧 promise，剩 pending=1、localRevision&gt;confirmedRevision、lastError=null，直至 60 秒定时器。本交错当前失败，修复及独立复验待做。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>

</xml_diff>

<commit_message>
docs: clarify Claude local file identity boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf00897d63a81411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rcefcae8d227c4478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R41ace9e714664575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0bc7ca2e1ea9465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rcdc50a26e00346d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb6247ec7d62a4174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb4768ca902054631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R13ec8f4464ba4ea5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2680,7 +2680,7 @@
 90338f4：TC-085 已注册 5 单元+2 Electron，取消/续扫隔离自动目标独立通过；生产/打包未验，REQ-044 真零仍待 TC-084/REQ-040。</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="85" customHeight="1">
+    <x:row r="92" ht="172.5" customHeight="1">
       <x:c r="A92" s="58" t="str">
         <x:v>REQ-045</x:v>
       </x:c>
@@ -2702,7 +2702,8 @@
       <x:c r="G92" s="58" t="str">
         <x:v>TC-086 待注册/待验；草稿/授权预览、同筛选双 owner 可见范围、取消/Escape、确认、重扫后过期基线和 viewer 越权
 在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。
-代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。</x:v>
+代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。
+2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -2849,7 +2850,8 @@
 2026-10-04 TC-092 缺 account_id fallback 及同键旧绑定迁移目标已补；未知来源不可绑定，viewer 隔离/管理员提示/脱敏审计待动态复现和修复。
 2026-10-04 旧本地 legacy-unverified 迁移、重扫成功/失败提示、清理与真实启动首次 flush 顺序补入 TC-092；凡影响授权或已确认小计/状态，旧 v1/v2 outbox 均先持久替换；同 owner 旧 OTel confirmed 降 uncertain，待动态验收。
 2026-10-04 TC-092 新增 Claude 缺/空/无效/超长 user.id、安装 ID 非账户、旧混合键及双账户同 stream/time 累计游标碰撞反例；无法证重送标 uncertain，待验。
-2026-10-04 Codex unknown 两账户同字段双 POST 与真正重送对照待验；缺稳定 ID 保留观测并标 uncertain，旧身份可证子范围不变。</x:v>
+2026-10-04 Codex unknown 两账户同字段双 POST 与真正重送对照待验；缺稳定 ID 保留观测并标 uncertain，旧身份可证子范围不变。
+2026-10-04 Claude 跨 owner 正例限定可证不同 UID/上下文；同 UID 两文件同键默认未归属。待验每文件不透明来源+事实键、逐文件绑定成本、移动/轮转/跨文件重放与旧库迁移；文件不等于账号。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="330" customHeight="1">
@@ -4294,7 +4296,8 @@
 2026-10-04 旧本地来源迁移：旧 Codex/Claude 事实暂入 legacy-unverified 未归属期间，受影响 viewer 须见不含来源细节的“历史归属正在核对”；缺文件、拒权或无法解析而重扫失败时，显示“无法完成重扫/历史仍待核对”，不能默默显示真零。管理员须有重扫与权限授权后重试行动；仅可证身份及授权归属后恢复。成功后清除无事实临时来源，保留脱敏审计。
 2026-10-04 Claude OTel：缺失、空白、非字符串、超长 user.id 或仅有安装级 user.id 均不足以证明 Claude 账户归属，新事实进入独立 unknown 且不可绑定；旧 username/hash(空串)/安装 ID 混合来源无法拆分时撤销归属。viewer 页面/CSV/来源状态/上报隔离，管理员可见脱敏诊断。累计游标与事实键不得跨账户静默合并/错算；无法证重送则保留观测并标待核对，不报完整总量。
 Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。
-迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。</x:v>
+迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。
+2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态筛选或分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4322,7 +4325,8 @@
 旧 fallback key 可与真实 account_id 恰等于 macOS username 的事件同键，现存键不足以逐条还原；混合键无法拆分时保守未归属，合法历史也可能被暂停，覆盖与总量未知。当前仅静态路径/验收设计，动态复现和修复待开发确认。
 旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。
 Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。
-2026-10-04 真实 Electron 启动诊断发现迁移首包成功后更新快照停在 outbox，需等 60 秒定时器；TC-094 新交错为当前失败待修，现有单元通过不能覆盖。</x:v>
+2026-10-04 真实 Electron 启动诊断发现迁移首包成功后更新快照停在 outbox，需等 60 秒定时器；TC-094 新交错为当前失败待修，现有单元通过不能覆盖。
+现行 claude.ts 的 sourceIdentityKey=context.fallbackIdentityKey，scanner.ts fallback 为 claude:macos:&lt;uid&gt;，事实键 claude:session:request；同 UID 多文件缺账号证据。开发报告未提交工作树 test:gate 94 入口/89 单元/40 Electron 退出码 0，无固定提交供文档会话复验，状态不升。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5774,7 +5778,8 @@
 旧本地来源迁移需保存待核对/重扫失败状态，按角色给 viewer 通用提示与管理员重扫/权限动作；可证重归属后清理零事实 legacy-unverified 来源行/绑定候选，保留不透明审计引用；重试幂等。启动时任何影响授权或已确认小计/状态的迁移后，先持久重算替换旧 v1/v2 outbox，失败阻断旧包，随后才允许 UsageSync 首次 flush；旧 owner 聚合清除，同 owner 旧 OTel 键转 legacy_otel_identity_unknown 时旧 confirmed 降 uncertain。
 Claude telemetry.ts 的 string() 接受空串而 hash(空串) 可绑定，缺/无效/超长退回 os.username；改为按可证认证账户属性或经验证网关 subject 判归属，其余 unknown。旧混合键保守撤销并重算本地/服务授权；隔离累计 stream、otel_metric_cursors 和事实键，避免双账户缺 ID 同 stream/time 的丢点或错算。无法证重送保留观测并标 uncertain；首次 flush 前持久替换受影响快照。
 开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。
-迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。</x:v>
+迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。
+Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态筛选或分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9507,7 +9512,7 @@
         <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="380" customHeight="1">
+    <x:row r="91" ht="247.5" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9526,12 +9531,14 @@
       <x:c r="F91" s="58" t="str">
         <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。
 本轮补造已确认与待核对事实、筛选内外事实；选候选只成草稿，预览原/新 owner、全部受影响数、同筛选两侧授权可见集合。取消/Escape、确认后刷新、viewer 预览/确认 IPC 越权；预览后重扫增删/改写事实或目标停用再确认，旧基线必须失效。
-在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。</x:v>
+在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。
+关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
         <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
 预览数量须与实际转移授权可见性的事实集合一致，不能以来源总 factCount 充当筛选后可见总量；取消/Escape 无归属/报表/成功审计变化。确认时同事务复验，过期预览拒绝并提示刷新；成功后恰好所示范围变化且 UI/报表同步，viewer IPC 拒绝。
-预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。</x:v>
+预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。
+管理员可逐文件核对、保留暂不归属；不能仅按同 UID 批量绑定或把文件来源叫账号，列表/预览/审计无原始路径、正文、账户/会话 ID。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
         <x:v>已注册；单元+Electron 自动子范围通过，完整键盘/生产打包待验</x:v>
@@ -9549,7 +9556,8 @@
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 UI 下拉 onChange 直绑，需改为草稿/预览/确认。来源全体条数与相同筛选可见事实数须分列；pending 不称已确认总量。用专用临时库并在预览后注入新扫描/目标状态变化检验竞态，未实施前不登记通过。
 用独立测试服务和合成聚合核对在线同步；不把本地成功等同服务成功。
-在线服务旧 owner 聚合清理由隔离服务器验证；UI 仅测少量 Tab/Escape，完整背景隔离/失败回焦和目标 Mac VoiceOver 属 TC-089。未测打包 App。</x:v>
+在线服务旧 owner 聚合清理由隔离服务器验证；UI 仅测少量 Tab/Escape，完整背景隔离/失败回焦和目标 Mac VoiceOver 属 TC-089。未测打包 App。
+Claude 每文件来源队列 UX 是新增待验子范围；既有 TC-086 少量来源的自动通过不覆盖大量历史文件管理成本。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>
@@ -9807,7 +9815,7 @@
         <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，单编号退出码 0；完整门禁 94 入口、77 单元、38 Electron；真零与人工证据待补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="185" customHeight="1">
+    <x:row r="97" ht="281.25" customHeight="1">
       <x:c r="A97" s="61" t="str">
         <x:v>TC-092</x:v>
       </x:c>
@@ -9831,7 +9839,8 @@
 待新增无 user.account_id Codex OTel 同机 A/B 账户样本；另有真实 account_id==macOS username 与缺 ID 同键旧库、已绑定 fallback owner A；迁移后分别以 viewer A/B、管理员调用报表/明细/CSV/来源状态/诊断/绑定预览确认及在线/离线上报。
 新增旧库：Codex/Claude 已绑定 viewer 的历史事实和旧 v1/v2 outbox，触发 legacy-unverified 迁移；分别模拟可证重扫成功、文件缺失、权限拒绝、不可读/无法解析、取消和重启重试；另造有 account_id、owner 不变但旧 OTel 键被迁为 legacy_otel_identity_unknown 的 confirmed 快照；真实主进程启动并连接在线服务。
 新增 Claude OTel 同机账户 A/B：user.id 缺失、空串、空白、非字符串、超过 200 字符及两账户共用安装 ID；对照有可验证认证账户属性或网关 OIDC subject 的样本。旧库预绑 username/hash(空串) 混合键。两账户缺 ID 且 session/model/category/start/time 全同，累计值不同，再给各自后续点与真正重送。
-再造 Codex 账户 A/B 均无 user.account_id，分两次 POST 且 session/rawTime/model/Token 全同；另造同一真实事件的重送对照。</x:v>
+再造 Codex 账户 A/B 均无 user.account_id，分两次 POST 且 session/rawTime/model/Token 全同；另造同一真实事件的重送对照。
+Claude 本地同 session/request：先用不同合成 UID/可证上下文造跨 owner 正例；再用同一 UID 下两个 JSONL 模拟多账号且同键、Token 大小互换，另造移动/轮转与同请求跨文件重放、旧 UID 已绑定库。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
@@ -9841,7 +9850,8 @@
 缺身份事实未归属且不可重绑，普通用户各路径无此事实或跨 owner 元数据；管理员可见身份未知与重新启用含 account_id 遥测行动，受影响 viewer 有通用提示；旧混合键无法拆分则保守暂停并记录可能合法事实受影响。迁移幂等、旧 owner 服务聚合清理或待传、脱敏审计无原始 account/session。
 迁移期间 viewer 旧历史暂不可见但有“历史归属正在核对”通用提示，失败后显示“无法完成重扫/历史仍待核对”，管理员有可操作重扫/权限行动；仅可证授权后恢复，不重复计量或泄露。成功后零事实临时来源不留归属表/候选，脱敏审计保留。任何影响授权或已确认小计/状态的迁移后，首次 flush 前持久替换旧 outbox 为重算的 v2；旧包从未发送，在线旧 owner 聚合删除，同 owner 旧 OTel confirmed 降 uncertain。
 仅安装 ID 不能证明账户；缺/空/无效/超长来源 unknown、不可绑定，旧混合键保守撤销，viewer A/B 全路径隔离、管理员脱敏诊断。相同 stream/time 的不同账户点不得静默丢失，后续累计点不得跨账户差分；无法证重送时保留观测并标 uncertain，已丢历史仍未知。受影响 v2 快照首次 flush 前重算，旧 owner 聚合清除或状态降级。
-不可仅因 unknown:hash(mac username) 键同而静默去重；无法证同一事件时两次观测均保留、计量 uncertain，viewer/上报不称确定总量。</x:v>
+不可仅因 unknown:hash(mac username) 键同而静默去重；无法证同一事件时两次观测均保留、计量 uncertain，viewer/上报不称确定总量。
+跨 owner 正例仅在来源和 owner 均可证时分别可见；同 UID 两文件应保留两条独立事实/项目关联但文件来源默认未归属，viewer A/B 均不得因 UID 自动看见。UI 仅称文件来源，管理员逐文件凭额外证据预览/确认；无原始路径/正文/ID。重扫/迁移幂等；跨文件重复仅在可证同事件时去重，否则 uncertain；旧无法拆分绑定保守撤销。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9863,7 +9873,8 @@
 新身份边界未动态复现/修复或执行新断言；旧 TC-092 自动子结果不覆盖缺 ID fallback、同键 account_id==username、旧绑定撤销与 viewer/服务回归。
 旧来源重扫 UX、零事实清理及任何影响授权或已确认小计/状态的迁移后，主进程启动/首次上传顺序为新增待验断言；手动调用 queueSnapshot 单测不能证明，既有 TC-092 通过子范围不覆盖。
 Claude user.id 安装级语义及缺/空/无效/超长、双账户同 stream/time 游标碰撞是新增待验反例；现有 TC-092 自动子结果不覆盖，未动态复现或修复。
-Codex unknown 同键双 POST 与真正重送的新反例未动态运行；身份可证旧通过子范围结论不变。</x:v>
+Codex unknown 同键双 POST 与真正重送的新反例未动态运行；身份可证旧通过子范围结论不变。
+现行 Claude JSONL 不能证同 UID 多账号分别属于不同 owner；不可通过预先手工分配 owner 伪造 TC-092。文件级来源及管理员逐文件绑定/TC-086 UI 成本、移动/轮转和重放新断言待实现/运行；未提交 gate 结果不提升状态。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>

</xml_diff>

<commit_message>
docs: define Claude file generation acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rcdc50a26e00346d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb6247ec7d62a4174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb4768ca902054631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R13ec8f4464ba4ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R211be0194ee8480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf4cc64b3d2b74371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R68c5f074e6274a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R3513a67ee5844a25"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2851,7 +2851,8 @@
 2026-10-04 旧本地 legacy-unverified 迁移、重扫成功/失败提示、清理与真实启动首次 flush 顺序补入 TC-092；凡影响授权或已确认小计/状态，旧 v1/v2 outbox 均先持久替换；同 owner 旧 OTel confirmed 降 uncertain，待动态验收。
 2026-10-04 TC-092 新增 Claude 缺/空/无效/超长 user.id、安装 ID 非账户、旧混合键及双账户同 stream/time 累计游标碰撞反例；无法证重送标 uncertain，待验。
 2026-10-04 Codex unknown 两账户同字段双 POST 与真正重送对照待验；缺稳定 ID 保留观测并标 uncertain，旧身份可证子范围不变。
-2026-10-04 Claude 跨 owner 正例限定可证不同 UID/上下文；同 UID 两文件同键默认未归属。待验每文件不透明来源+事实键、逐文件绑定成本、移动/轮转/跨文件重放与旧库迁移；文件不等于账号。</x:v>
+2026-10-04 Claude 跨 owner 正例限定可证不同 UID/上下文；同 UID 两文件同键默认未归属。待验每文件不透明来源+事实键、逐文件绑定成本、移动/轮转/跨文件重放与旧库迁移；文件不等于账号。
+2026-10-04 同文件改名保持身份与旧文件删除后新代次同路径/UID/dev/ino/size/tailHash、birthtime 不同须越过旧游标短路且不继承 owner 的对照待验；旧事实/项目/审计/服务隔离及迁移幂等。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="330" customHeight="1">
@@ -4297,7 +4298,8 @@
 2026-10-04 Claude OTel：缺失、空白、非字符串、超长 user.id 或仅有安装级 user.id 均不足以证明 Claude 账户归属，新事实进入独立 unknown 且不可绑定；旧 username/hash(空串)/安装 ID 混合来源无法拆分时撤销归属。viewer 页面/CSV/来源状态/上报隔离，管理员可见脱敏诊断。累计游标与事实键不得跨账户静默合并/错算；无法证重送则保留观测并标待核对，不报完整总量。
 Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。
 迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。
-2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态筛选或分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。</x:v>
+2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态筛选或分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。
+2026-10-04 文件代次：同一 Claude JSONL 改名/移动且可证连续时保持来源；旧文件删除后新文件即使复用 UID/dev/ino，也必须新建未归属“文件来源”，不得继承旧 owner/审计或将新事实按旧 owner 展示/上报。仅 sha256(uid:dev:ino) 不足以证明代次。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
@@ -4326,7 +4328,8 @@
 旧本地历史可能因暂时未归属而从原 viewer 报表消失，缺文件时不能保证恢复。任何影响授权或已确认小计/状态的迁移后，已有 v1/v2 待传快照必须于首次 flush 前持久替换成重算的 v2 快照；旧 owner 聚合删除，旧 OTel 有 account_id、owner 不变但旧键标 legacy_otel_identity_unknown 时，旧 confirmed 降 uncertain。此为待验收，不是已实现。
 Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。
 2026-10-04 真实 Electron 启动诊断发现迁移首包成功后更新快照停在 outbox，需等 60 秒定时器；TC-094 新交错为当前失败待修，现有单元通过不能覆盖。
-现行 claude.ts 的 sourceIdentityKey=context.fallbackIdentityKey，scanner.ts fallback 为 claude:macos:&lt;uid&gt;，事实键 claude:session:request；同 UID 多文件缺账号证据。开发报告未提交工作树 test:gate 94 入口/89 单元/40 Electron 退出码 0，无固定提交供文档会话复验，状态不升。</x:v>
+现行 claude.ts 的 sourceIdentityKey=context.fallbackIdentityKey，scanner.ts fallback 为 claude:macos:&lt;uid&gt;，事实键 claude:session:request；同 UID 多文件缺账号证据。开发报告未提交工作树 test:gate 94 入口/89 单元/40 Electron 退出码 0，无固定提交供文档会话复验，状态不升。
+开发中 sha256(uid:dev:ino) 方案尚无固定提交可独立验收；inode 可复用，需同文件改名与不同代次同元组对照。现仅修订验收口径，状态不升。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5779,7 +5782,8 @@
 Claude telemetry.ts 的 string() 接受空串而 hash(空串) 可绑定，缺/无效/超长退回 os.username；改为按可证认证账户属性或经验证网关 subject 判归属，其余 unknown。旧混合键保守撤销并重算本地/服务授权；隔离累计 stream、otel_metric_cursors 和事实键，避免双账户缺 ID 同 stream/time 的丢点或错算。无法证重送保留观测并标 uncertain；首次 flush 前持久替换受影响快照。
 开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。
 迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。
-Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态筛选或分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。</x:v>
+Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态筛选或分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。
+文件来源身份加入可验证代次/连续性判断：同文件改名保持身份与幂等；删除/轮转后的新代次即使 UID/dev/ino 复用也须先于 stat.size===start 游标短路识别并重扫，再新建未归属来源，证据不足时不得沿用 owner。旧事实/项目/脱敏审计与 v2 outbox/服务聚合按授权迁移，TC-092/093/094 回归。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9815,7 +9819,7 @@
         <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，单编号退出码 0；完整门禁 94 入口、77 单元、38 Electron；真零与人工证据待补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="281.25" customHeight="1">
+    <x:row r="97" ht="352.5" customHeight="1">
       <x:c r="A97" s="61" t="str">
         <x:v>TC-092</x:v>
       </x:c>
@@ -9840,7 +9844,8 @@
 新增旧库：Codex/Claude 已绑定 viewer 的历史事实和旧 v1/v2 outbox，触发 legacy-unverified 迁移；分别模拟可证重扫成功、文件缺失、权限拒绝、不可读/无法解析、取消和重启重试；另造有 account_id、owner 不变但旧 OTel 键被迁为 legacy_otel_identity_unknown 的 confirmed 快照；真实主进程启动并连接在线服务。
 新增 Claude OTel 同机账户 A/B：user.id 缺失、空串、空白、非字符串、超过 200 字符及两账户共用安装 ID；对照有可验证认证账户属性或网关 OIDC subject 的样本。旧库预绑 username/hash(空串) 混合键。两账户缺 ID 且 session/model/category/start/time 全同，累计值不同，再给各自后续点与真正重送。
 再造 Codex 账户 A/B 均无 user.account_id，分两次 POST 且 session/rawTime/model/Token 全同；另造同一真实事件的重送对照。
-Claude 本地同 session/request：先用不同合成 UID/可证上下文造跨 owner 正例；再用同一 UID 下两个 JSONL 模拟多账号且同键、Token 大小互换，另造移动/轮转与同请求跨文件重放、旧 UID 已绑定库。</x:v>
+Claude 本地同 session/request：先用不同合成 UID/可证上下文造跨 owner 正例；再用同一 UID 下两个 JSONL 模拟多账号且同键、Token 大小互换，另造移动/轮转与同请求跨文件重放、旧 UID 已绑定库。
+文件 F1 已绑定 owner A、含事实/项目/审计；同 F1 改名后重扫；删除 F1 后用元数据注入造 F2 同路径、UID/dev/ino、size、tailHash 但 birthtime 不同，session/request 可同旧事实；另跑真实移动/轮转。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
@@ -9851,7 +9856,8 @@
 迁移期间 viewer 旧历史暂不可见但有“历史归属正在核对”通用提示，失败后显示“无法完成重扫/历史仍待核对”，管理员有可操作重扫/权限行动；仅可证授权后恢复，不重复计量或泄露。成功后零事实临时来源不留归属表/候选，脱敏审计保留。任何影响授权或已确认小计/状态的迁移后，首次 flush 前持久替换旧 outbox 为重算的 v2；旧包从未发送，在线旧 owner 聚合删除，同 owner 旧 OTel confirmed 降 uncertain。
 仅安装 ID 不能证明账户；缺/空/无效/超长来源 unknown、不可绑定，旧混合键保守撤销，viewer A/B 全路径隔离、管理员脱敏诊断。相同 stream/time 的不同账户点不得静默丢失，后续累计点不得跨账户差分；无法证重送时保留观测并标 uncertain，已丢历史仍未知。受影响 v2 快照首次 flush 前重算，旧 owner 聚合清除或状态降级。
 不可仅因 unknown:hash(mac username) 键同而静默去重；无法证同一事件时两次观测均保留、计量 uncertain，viewer/上报不称确定总量。
-跨 owner 正例仅在来源和 owner 均可证时分别可见；同 UID 两文件应保留两条独立事实/项目关联但文件来源默认未归属，viewer A/B 均不得因 UID 自动看见。UI 仅称文件来源，管理员逐文件凭额外证据预览/确认；无原始路径/正文/ID。重扫/迁移幂等；跨文件重复仅在可证同事件时去重，否则 uncertain；旧无法拆分绑定保守撤销。</x:v>
+跨 owner 正例仅在来源和 owner 均可证时分别可见；同 UID 两文件应保留两条独立事实/项目关联但文件来源默认未归属，viewer A/B 均不得因 UID 自动看见。UI 仅称文件来源，管理员逐文件凭额外证据预览/确认；无原始路径/正文/ID。重扫/迁移幂等；跨文件重复仅在可证同事件时去重，否则 uncertain；旧无法拆分绑定保守撤销。
+可证同文件改名沿用来源且不增量；F2 必须在 stat.size===start 旧游标短路前重置并重新读取，新建未归属来源，不继承 A 绑定/审计，不覆盖 F1 事实/项目，viewer/CSV/来源状态/服务均不按 A 计 F2。重启迁移/重扫幂等，管理员不能凭同 inode 自动绑定。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
         <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
@@ -9874,7 +9880,8 @@
 旧来源重扫 UX、零事实清理及任何影响授权或已确认小计/状态的迁移后，主进程启动/首次上传顺序为新增待验断言；手动调用 queueSnapshot 单测不能证明，既有 TC-092 通过子范围不覆盖。
 Claude user.id 安装级语义及缺/空/无效/超长、双账户同 stream/time 游标碰撞是新增待验反例；现有 TC-092 自动子结果不覆盖，未动态复现或修复。
 Codex unknown 同键双 POST 与真正重送的新反例未动态运行；身份可证旧通过子范围结论不变。
-现行 Claude JSONL 不能证同 UID 多账号分别属于不同 owner；不可通过预先手工分配 owner 伪造 TC-092。文件级来源及管理员逐文件绑定/TC-086 UI 成本、移动/轮转和重放新断言待实现/运行；未提交 gate 结果不提升状态。</x:v>
+现行 Claude JSONL 不能证同 UID 多账号分别属于不同 owner；不可通过预先手工分配 owner 伪造 TC-092。文件级来源及管理员逐文件绑定/TC-086 UI 成本、移动/轮转和重放新断言待实现/运行；未提交 gate 结果不提升状态。
+inode 复用难在真实文件系统稳定强制，可用受控元数据注入测同路径/大小/尾哈希、birthtime 不同的新代次反例；仅 fact-key helper 测试不足以验游标短路；另留真实改名/轮转集成。开发方案未有固定提交，本反例未运行，旧通过子范围不覆盖。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>

</xml_diff>

<commit_message>
docs: define Claude migration and binding evidence cases
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R211be0194ee8480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rf4cc64b3d2b74371"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R68c5f074e6274a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R3513a67ee5844a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1c66345efbd74bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd597216a37ef4b17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf3342f710fc74dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R46d01d8408524939"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2703,7 +2703,9 @@
         <x:v>TC-086 待注册/待验；草稿/授权预览、同筛选双 owner 可见范围、取消/Escape、确认、重扫后过期基线和 viewer 越权
 在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。
 代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。
-2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。</x:v>
+2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。
+2026-10-04 Claude 逐文件确认补 controlled_account_file_mapping、external_managed_registry、evr_+32 位小写十六进制引用和显式人工声明；空/路径式/非白名单 UI 与 IPC 均拒绝并保持未归属，审计最小脱敏且标人工确认，TC-086 新增子范围待验。
+拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -2852,7 +2854,9 @@
 2026-10-04 TC-092 新增 Claude 缺/空/无效/超长 user.id、安装 ID 非账户、旧混合键及双账户同 stream/time 累计游标碰撞反例；无法证重送标 uncertain，待验。
 2026-10-04 Codex unknown 两账户同字段双 POST 与真正重送对照待验；缺稳定 ID 保留观测并标 uncertain，旧身份可证子范围不变。
 2026-10-04 Claude 跨 owner 正例限定可证不同 UID/上下文；同 UID 两文件同键默认未归属。待验每文件不透明来源+事实键、逐文件绑定成本、移动/轮转/跨文件重放与旧库迁移；文件不等于账号。
-2026-10-04 同文件改名保持身份与旧文件删除后新代次同路径/UID/dev/ino/size/tailHash、birthtime 不同须越过旧游标短路且不继承 owner 的对照待验；旧事实/项目/审计/服务隔离及迁移幂等。</x:v>
+2026-10-04 同文件改名保持身份与旧文件删除后新代次同路径/UID/dev/ino/size/tailHash、birthtime 不同须越过旧游标短路且不继承 owner 的对照待验；旧事实/项目/审计/服务隔离及迁移幂等。
+2026-10-04 单文件 S1/S2、游标仅 S2 须逐事实隔离/一一调和；临时副本不重复计量，歧义留原因/未知总量且不自动恢复旧 owner；TC-092 待验。
+旧游标仅 dev:ino 或 birthtime_ms=0 时不可用 F2 当前 birthtime 倒填；F1 待核对不清除、F2 未归属、首包清旧 owner，TC-092 待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="330" customHeight="1">
@@ -4191,13 +4195,15 @@
       <x:c r="C50" s="58" t="str">
         <x:v>变更来源归属前展示受影响事实数、旧/新用户可见范围，确认后才提交；主进程复验角色与来源，失败不改归属或报表。成功变更与最小审计同事务；业务拒绝可单记最小结果，数据库不可写时不得声称持久审计。审计字段限时间、操作者、持久随机不透明来源引用、前后用户 ID、数量和结果码，不含路径/正文。
 选择候选只留 UI 草稿；主进程预览须显示原/新 owner、来源全部受影响事实数及相同筛选下两侧授权可见事实范围/待核对状态。确认时在事务中复验权限、来源、目标活跃性、原 owner 和预览事实集合基线；重扫或目标变化后旧预览失效，须重取。取消/Escape 无写入；失败恢复 UI 原值并给可操作错误。审计只存持久随机不透明来源引用，不存原始 key/标签/路径/账号/正文；旧审计展示/导出前脱敏。
-重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。</x:v>
+重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。
+2026-10-04 Claude 逐文件归属：项目/时间/UID/文件来源和管理员点击不足以证明账号。确认前逐项声明受控账号-文件映射证据类别、受控出处的不透明引用并显式确认已核对；无证据保持未归属，主进程拒绝。只以最小脱敏审计记录人工判断，不称提供方验证。
+证据字段首个白名单为 controlled_account_file_mapping / external_managed_registry / evr_ 加 32 位小写十六进制及单独确认位。真实登记未证实可用时，合成登记仅验机制；主进程可据合法声明提交标为“管理员人工确认”的事务，但不验证真实性。管理员无外部证据应选暂不归属，真实归属正例待外部复核。</x:v>
       </x:c>
       <x:c r="D50" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E50" s="58" t="str">
-        <x:v>已实现；隔离自动子范围通过，生产库迁移/打包应用待验</x:v>
+        <x:v>既有重绑子范围已实现且隔离自动通过；Claude 逐文件证据门槛待实现/待验，真实受控出处待证；生产库迁移/打包应用待验</x:v>
       </x:c>
       <x:c r="F50" s="58" t="str">
         <x:v>DEV-054</x:v>
@@ -4209,7 +4215,9 @@
         <x:v>承接 REQ-011；归属与报表权限应在同一提交边界生效。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 SOP-001/002 实施前静态核对：当前来源下拉 onChange 立即 bind；scanner.identities().factCount 为来源全部 usage_facts 条数，不能当选定筛选后可见集；scanner.bindIdentity() 当前把原始 key 写 audit_events.target_id。新预览和审计白名单按 docs/design.md §20.3 实施，未改代码、未运行新用例。
 当前 sources:bind 只调用 bindIdentity，没有显式生成 usage-sync 新快照；TC-086/087 分别验在线旧 owner 清除和离线队列，TC-088 回归本地与服务状态分离。
-2026-10-03 代码 01a7095：文档会话独立复跑 TC-086/087 各单元+Electron、TC-074/080/093 及完整门禁（90 入口、66 单元、30 Electron）通过。五分钟一次性预览/基线、耐久事务审计与 v2 新队列有隔离证据；真实生产库迁移、打包安装、TC-088/089 仍待验。此前待实现文字为阶段历史。</x:v>
+2026-10-03 代码 01a7095：文档会话独立复跑 TC-086/087 各单元+Electron、TC-074/080/093 及完整门禁（90 入口、66 单元、30 Electron）通过。五分钟一次性预览/基线、耐久事务审计与 v2 新队列有隔离证据；真实生产库迁移、打包安装、TC-088/089 仍待验。此前待实现文字为阶段历史。
+Claude 文件来源独立证据声明为新增待验门槛；旧 TC-086/087 通过不覆盖。
+真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -4299,13 +4307,15 @@
 Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。
 迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。
 2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态筛选或分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。
-2026-10-04 文件代次：同一 Claude JSONL 改名/移动且可证连续时保持来源；旧文件删除后新文件即使复用 UID/dev/ino，也必须新建未归属“文件来源”，不得继承旧 owner/审计或将新事实按旧 owner 展示/上报。仅 sha256(uid:dev:ino) 不足以证明代次。</x:v>
+2026-10-04 文件代次：同一 Claude JSONL 改名/移动且可证连续时保持来源；旧文件删除后新文件即使复用 UID/dev/ino，也必须新建未归属“文件来源”，不得继承旧 owner/审计或将新事实按旧 owner 展示/上报。仅 sha256(uid:dev:ino) 不足以证明代次。
+2026-10-04 旧 UID 绑定单 JSONL 可有 S1/S2 两事实而游标只记 S2：迁移须逐事实隔离、可证重扫一一调和，已匹配临时副本不再有效计量；歧义留待核对原因与未知总量，文件本身不恢复账号 owner。逐文件人工绑定另须独立可复核证据声明，否则未归属。
+旧游标只有 file_id=dev:ino 或 birthtime_ms=0 时，不得把当前 F2 的 stat.birthtimeMs 回填为旧 F1 连续性证据；F1 待核对临时事实不清除，F2 同路径/inode/payload 仍未归属，旧 owner 确认总量不恢复。</x:v>
       </x:c>
       <x:c r="D53" s="61" t="str">
         <x:v>缺陷修复（已复现）</x:v>
       </x:c>
       <x:c r="E53" s="61" t="str">
-        <x:v>已编码；TC-092–094 自动子范围通过，TC-093 在 81c271b 增真实隔离输入 E2E 并独立复验；跨账户同键碰撞待修，正向精确去重/生产迁移待验证</x:v>
+        <x:v>已编码；TC-092–094 自动子范围通过，TC-093 在 81c271b 增真实隔离输入 E2E 并独立复验；跨账户同键碰撞待修，正向精确去重/生产迁移待验证；新增 Claude 文件代次、多 session 与旧游标倒填反例待实现/待验</x:v>
       </x:c>
       <x:c r="F53" s="61" t="str">
         <x:v>DEV-057</x:v>
@@ -4329,7 +4339,9 @@
 Claude 官方监测属性说明：普通 user.id 为保存在 ~/.claude.json 的安装级匿名值，不源于 Claude 账户；网关 OIDC 下可变为 IdP subject，认证账户属性仅在可用时存在。身份来源与实际版本须验，不可把 user.id 直接等同 Codex account_id。https://code.claude.com/docs/en/monitoring-usage；当前仅静态风险。
 2026-10-04 真实 Electron 启动诊断发现迁移首包成功后更新快照停在 outbox，需等 60 秒定时器；TC-094 新交错为当前失败待修，现有单元通过不能覆盖。
 现行 claude.ts 的 sourceIdentityKey=context.fallbackIdentityKey，scanner.ts fallback 为 claude:macos:&lt;uid&gt;，事实键 claude:session:request；同 UID 多文件缺账号证据。开发报告未提交工作树 test:gate 94 入口/89 单元/40 Electron 退出码 0，无固定提交供文档会话复验，状态不升。
-开发中 sha256(uid:dev:ino) 方案尚无固定提交可独立验收；inode 可复用，需同文件改名与不同代次同元组对照。现仅修订验收口径，状态不升。</x:v>
+开发中 sha256(uid:dev:ino) 方案尚无固定提交可独立验收；inode 可复用，需同文件改名与不同代次同元组对照。现仅修订验收口径，状态不升。
+单文件多 session 旧库迁移和逐文件独立证据声明为新增待验范围；现无固定实现及动态通过。
+旧游标代次倒填反例待验：仅旧持久连续性证据和逐事实映射充分才归档 F1；首包 v2 须清旧 owner 聚合。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5680,14 +5692,16 @@
         <x:v>src/main/source-binding.ts、database.ts、index.ts、usage-sync.ts；src/collectors/scanner.ts；src/server/server.ts；src/renderer/index.tsx、source-binding.tsx；tests/source-binding.test.ts、tests/e2e/source-binding.spec.ts</x:v>
       </x:c>
       <x:c r="F59" s="58" t="str">
-        <x:v>已开发；TC-086/087 已注册并通过隔离自动子范围，生产/打包待验</x:v>
+        <x:v>既有重绑流程已开发且 TC-086/087 隔离自动子范围通过；Claude 独立证据声明待实现/待验，生产/打包待验</x:v>
       </x:c>
       <x:c r="G59" s="58" t="str">
         <x:v>预览受影响事实数/可见范围，确认后主进程复验权限和版本；事务提交归属及最小审计，失败不改变归属；审计不保存路径/正文。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 需求复核补充：成功绑定与最小审计同事务；业务拒绝可另记结果，DB 不可写时绑定不变且不得声称审计已持久化。
 实施前补充：改下拉为草稿→授权预览→确认，预览含原/新 owner、来源全体受影响事实数与同筛选两侧报表可见集合/待核对状态；带归属和事实集合的不可伪造基线。确认在事务内重验 actor、来源、活跃目标、旧 owner 与基线，重扫新增/改写事实须拒绝旧预览。成功归属+最小审计同事务并刷新 UI/报表；取消/Escape 无写入，失败 UI 回原值。审计引用用持久随机不透明 ID，历史 raw key 展示/导出前脱敏；DB 不可写时不宣称审计持久。TC-086/087 分别测一致性/权限与失败回滚/隐私。
 绑定成功后创建持久版本 2 新 revision/待传义务，停止上传旧 owner 队列；在线替换/清除旧 owner 服务聚合，离线显示本地已变而服务待传并可重试。不得回退 DEV-057 v2 授权/冲突口径，交叉回归 TC-088。
-代码 01a7095 已实现草稿→预览→确认、五分钟一次性基线、主进程重验、耐久事务归属+不透明审计+v2 新 outbox。旧审计原始 key 初始化迁移；在线清设备历史授权旧 owner 聚合、保留历史未授权行，离线新 revision 替换旧队列；审计/磁盘失败回滚。文档会话独立复验 TC-086/087、TC-074/080/093 与完整门禁通过。生产库迁移、打包应用、TC-088/089 尚未验。</x:v>
+代码 01a7095 已实现草稿→预览→确认、五分钟一次性基线、主进程重验、耐久事务归属+不透明审计+v2 新 outbox。旧审计原始 key 初始化迁移；在线清设备历史授权旧 owner 聚合、保留历史未授权行，离线新 revision 替换旧队列；审计/磁盘失败回滚。文档会话独立复验 TC-086/087、TC-074/080/093 与完整门禁通过。生产库迁移、打包应用、TC-088/089 尚未验。
+Claude 文件确认 API 增 evidenceCategory=controlled_account_file_mapping、evidenceSource=external_managed_registry、evidenceRef=evr_ 加 32 位小写十六进制及显式人工确认；主进程连同预览基线校验，空/路径式/非白名单值拒绝且不改归属。审计仅留原因码/类别/来源码、不透明引用、操作者/结果，不存原始路径/账号/会话/正文/证据内容。引用真实性由外部受控登记复核，TC-086/087 回归。
+external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -5763,7 +5777,7 @@
         <x:v>src/main/reconcile.ts、report.ts、usage-sync.ts、index.ts；src/server/server.ts；src/shared/types.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；tests/reconciliation.test.ts、sync-reconciliation.test.ts、e2e/overlap-privacy.spec.ts；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
-        <x:v>已实现调和子范围；TC-093 真实隔离输入 E2E 通过（81c271b）；TC-092 跨账户同键碰撞待修，正向精确去重/真实迁移待验证</x:v>
+        <x:v>已实现调和子范围；TC-093 真实隔离输入 E2E 通过（81c271b）；TC-092 跨账户同键碰撞待修，正向精确去重/真实迁移待验证；新增 Claude 文件代次、多 session 与旧游标倒填反例待实现/待验</x:v>
       </x:c>
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
@@ -5783,7 +5797,9 @@
 开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。
 迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。
 Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态筛选或分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。
-文件来源身份加入可验证代次/连续性判断：同文件改名保持身份与幂等；删除/轮转后的新代次即使 UID/dev/ino 复用也须先于 stat.size===start 游标短路识别并重扫，再新建未归属来源，证据不足时不得沿用 owner。旧事实/项目/脱敏审计与 v2 outbox/服务聚合按授权迁移，TC-092/093/094 回归。</x:v>
+文件来源身份加入可验证代次/连续性判断：同文件改名保持身份与幂等；删除/轮转后的新代次即使 UID/dev/ino 复用也须先于 stat.size===start 游标短路识别并重扫，再新建未归属来源，证据不足时不得沿用 owner。旧事实/项目/脱敏审计与 v2 outbox/服务聚合按授权迁移，TC-092/093/094 回归。
+单 JSONL S1/S2 旧事实、游标仅记 S2 时逐事实隔离并与可证重扫一一匹配；已匹配临时副本退出有效计量，歧义保留原因/未知总量，不因文件身份自动恢复旧 owner，项目/审计/服务迁移幂等。逐文件绑定调用 DEV-054 的独立证据声明门槛。
+迁移不能用当前 stat.birthtimeMs 回填旧 file_id=dev:ino 或 birthtime_ms=0；F1 删除后 F2 同路径/inode/payload 也不得归档 F1 或继承 owner，首次 v2 清旧聚合；仅旧持久证据充分且逐事实匹配才归档。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9516,7 +9532,7 @@
         <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="247.5" customHeight="1">
+    <x:row r="91" ht="322.5" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9536,16 +9552,20 @@
         <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。
 本轮补造已确认与待核对事实、筛选内外事实；选候选只成草稿，预览原/新 owner、全部受影响数、同筛选两侧授权可见集合。取消/Escape、确认后刷新、viewer 预览/确认 IPC 越权；预览后重扫增删/改写事实或目标停用再确认，旧基线必须失效。
 在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。
-关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。</x:v>
+关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。
+Claude 文件来源另造项目/时间似乎匹配 owner A：仅选择 A、证据类别缺失/非白名单、来源非白名单、引用空/原始路径式/格式无效、未显式确认时分别尝试 UI 和确认 IPC 直调；正例提交 controlled_account_file_mapping、external_managed_registry、evr_ 加 32 位小写十六进制与确认声明，并由外部登记复核出处。
+用合成登记和外形合法 evr_ 核人工确认事务机制，但不声称真实账号已证；真实账号-文件映射正例另待外部脱敏复核，无证据的管理员选择暂不归属。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
         <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
 预览数量须与实际转移授权可见性的事实集合一致，不能以来源总 factCount 充当筛选后可见总量；取消/Escape 无归属/报表/成功审计变化。确认时同事务复验，过期预览拒绝并提示刷新；成功后恰好所示范围变化且 UI/报表同步，viewer IPC 拒绝。
 预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。
-管理员可逐文件核对、保留暂不归属；不能仅按同 UID 批量绑定或把文件来源叫账号，列表/预览/审计无原始路径、正文、账户/会话 ID。</x:v>
+管理员可逐文件核对、保留暂不归属；不能仅按同 UID 批量绑定或把文件来源叫账号，列表/预览/审计无原始路径、正文、账户/会话 ID。
+无有效独立证据时保持未归属，无成功审计或 viewer/CSV/v2 授权变化；有效声明仅当前文件可人工确认且审计仅留白名单类别/来源码/原因码/不透明引用/操作者/结果，界面不称提供方验证。格式校验不代替外部证据真实性复核。
+合法 evr_ 声明可触发标为人工确认的事务，程序不核外部真实性；合成登记正例不等于真实 Claude 账号归属通过，无外部证据时管理员应选暂不归属。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
-        <x:v>已注册；单元+Electron 自动子范围通过，完整键盘/生产打包待验</x:v>
+        <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
         <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
@@ -9561,7 +9581,9 @@
 当前 UI 下拉 onChange 直绑，需改为草稿/预览/确认。来源全体条数与相同筛选可见事实数须分列；pending 不称已确认总量。用专用临时库并在预览后注入新扫描/目标状态变化检验竞态，未实施前不登记通过。
 用独立测试服务和合成聚合核对在线同步；不把本地成功等同服务成功。
 在线服务旧 owner 聚合清理由隔离服务器验证；UI 仅测少量 Tab/Escape，完整背景隔离/失败回焦和目标 Mac VoiceOver 属 TC-089。未测打包 App。
-Claude 每文件来源队列 UX 是新增待验子范围；既有 TC-086 少量来源的自动通过不覆盖大量历史文件管理成本。</x:v>
+Claude 每文件来源队列 UX 是新增待验子范围；既有 TC-086 少量来源的自动通过不覆盖大量历史文件管理成本。
+独立证据声明的 UI/IPC 与审计断言未运行；旧少量来源自动通过不覆盖，证据真实性须由受控外部来源复核。
+external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>
@@ -9819,7 +9841,7 @@
         <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，单编号退出码 0；完整门禁 94 入口、77 单元、38 Electron；真零与人工证据待补。</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" ht="352.5" customHeight="1">
+    <x:row r="97" ht="570" customHeight="1">
       <x:c r="A97" s="61" t="str">
         <x:v>TC-092</x:v>
       </x:c>
@@ -9845,7 +9867,9 @@
 新增 Claude OTel 同机账户 A/B：user.id 缺失、空串、空白、非字符串、超过 200 字符及两账户共用安装 ID；对照有可验证认证账户属性或网关 OIDC subject 的样本。旧库预绑 username/hash(空串) 混合键。两账户缺 ID 且 session/model/category/start/time 全同，累计值不同，再给各自后续点与真正重送。
 再造 Codex 账户 A/B 均无 user.account_id，分两次 POST 且 session/rawTime/model/Token 全同；另造同一真实事件的重送对照。
 Claude 本地同 session/request：先用不同合成 UID/可证上下文造跨 owner 正例；再用同一 UID 下两个 JSONL 模拟多账号且同键、Token 大小互换，另造移动/轮转与同请求跨文件重放、旧 UID 已绑定库。
-文件 F1 已绑定 owner A、含事实/项目/审计；同 F1 改名后重扫；删除 F1 后用元数据注入造 F2 同路径、UID/dev/ino、size、tailHash 但 birthtime 不同，session/request 可同旧事实；另跑真实移动/轮转。</x:v>
+文件 F1 已绑定 owner A、含事实/项目/审计；同 F1 改名后重扫；删除 F1 后用元数据注入造 F2 同路径、UID/dev/ino、size、tailHash 但 birthtime 不同，session/request 可同旧事实；另跑真实移动/轮转。
+另造单 JSONL S1/S2 两请求，旧 UID 来源均有已绑定事实与项目，持久游标仅 S2；迁移、逐事实可证重扫、重复启动/重扫，并造无法唯一匹配的分支。
+另造旧 F1 游标只含 file_id=dev:ino 与 birthtime_ms=0 两分支；删 F1 后注入同 path/UID/dev/ino/payload 但 birthtime 不同的 F2，启动迁移与首包上报。</x:v>
       </x:c>
       <x:c r="G97" s="61" t="str">
         <x:v>跨 owner/不同会话独立保留；同会话/未知候选标 uncertain，已确认小计与待核对来源/条数分开。共同稳定事件 ID 的正向去重仍需真实双方 ID 才能验。
@@ -9857,10 +9881,12 @@
 仅安装 ID 不能证明账户；缺/空/无效/超长来源 unknown、不可绑定，旧混合键保守撤销，viewer A/B 全路径隔离、管理员脱敏诊断。相同 stream/time 的不同账户点不得静默丢失，后续累计点不得跨账户差分；无法证重送时保留观测并标 uncertain，已丢历史仍未知。受影响 v2 快照首次 flush 前重算，旧 owner 聚合清除或状态降级。
 不可仅因 unknown:hash(mac username) 键同而静默去重；无法证同一事件时两次观测均保留、计量 uncertain，viewer/上报不称确定总量。
 跨 owner 正例仅在来源和 owner 均可证时分别可见；同 UID 两文件应保留两条独立事实/项目关联但文件来源默认未归属，viewer A/B 均不得因 UID 自动看见。UI 仅称文件来源，管理员逐文件凭额外证据预览/确认；无原始路径/正文/ID。重扫/迁移幂等；跨文件重复仅在可证同事件时去重，否则 uncertain；旧无法拆分绑定保守撤销。
-可证同文件改名沿用来源且不增量；F2 必须在 stat.size===start 旧游标短路前重置并重新读取，新建未归属来源，不继承 A 绑定/审计，不覆盖 F1 事实/项目，viewer/CSV/来源状态/服务均不按 A 计 F2。重启迁移/重扫幂等，管理员不能凭同 inode 自动绑定。</x:v>
+可证同文件改名沿用来源且不增量；F2 必须在 stat.size===start 旧游标短路前重置并重新读取，新建未归属来源，不继承 A 绑定/审计，不覆盖 F1 事实/项目，viewer/CSV/来源状态/服务均不按 A 计 F2。重启迁移/重扫幂等，管理员不能凭同 inode 自动绑定。
+S1/S2 均逐条隔离，一一匹配的临时副本不参与重复计量；只记 S2 的游标不得丢 S1。歧义观测保持未归属、明确原因和总量不可确认；不自动恢复旧 owner，项目/审计/服务旧聚合与 viewer/CSV 一致，重启幂等。
+F2 当前 birthtime 不可倒填证明 F1；F1 临时事实继续未归属/待核对且不被清除，F2 新来源未归属，首包 v2 与在线服务无旧 owner 已确认聚合；仅旧持久证据充分时归档。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
-        <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证</x:v>
+        <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证；新增 Claude 文件代次、多 session 与旧游标倒填反例待补/待验</x:v>
       </x:c>
       <x:c r="I97" s="61" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-092：单元 1/1、退出码 0；管理员初值 111，owner B 99，A 不同会话 19，同会话后已确认小计 7/状态 uncertain。test:gate 82 注册入口、56 单元、22 Electron 通过。</x:v>
@@ -9881,7 +9907,9 @@
 Claude user.id 安装级语义及缺/空/无效/超长、双账户同 stream/time 游标碰撞是新增待验反例；现有 TC-092 自动子结果不覆盖，未动态复现或修复。
 Codex unknown 同键双 POST 与真正重送的新反例未动态运行；身份可证旧通过子范围结论不变。
 现行 Claude JSONL 不能证同 UID 多账号分别属于不同 owner；不可通过预先手工分配 owner 伪造 TC-092。文件级来源及管理员逐文件绑定/TC-086 UI 成本、移动/轮转和重放新断言待实现/运行；未提交 gate 结果不提升状态。
-inode 复用难在真实文件系统稳定强制，可用受控元数据注入测同路径/大小/尾哈希、birthtime 不同的新代次反例；仅 fact-key helper 测试不足以验游标短路；另留真实改名/轮转集成。开发方案未有固定提交，本反例未运行，旧通过子范围不覆盖。</x:v>
+inode 复用难在真实文件系统稳定强制，可用受控元数据注入测同路径/大小/尾哈希、birthtime 不同的新代次反例；仅 fact-key helper 测试不足以验游标短路；另留真实改名/轮转集成。开发方案未有固定提交，本反例未运行，旧通过子范围不覆盖。
+单文件 S1/S2、游标仅 S2 的旧库迁移反例未运行；临时副本有效计量清理、歧义原因及旧 owner 服务清理仍待固定提交验证。
+旧 birthtime 缺失/为 0 和 F2 复用同 payload 的倒填反例未运行，不能凭当前 stat 或旧游标末值证明连续性。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
         <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>

</xml_diff>

<commit_message>
docs: specify Claude binding validation retry
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1c66345efbd74bb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd597216a37ef4b17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf3342f710fc74dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R46d01d8408524939"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rc13684a45a9c439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2b50fa6c88e04ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf184eb59682a4652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rbc821dbcab5d44b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2680,7 +2680,7 @@
 90338f4：TC-085 已注册 5 单元+2 Electron，取消/续扫隔离自动目标独立通过；生产/打包未验，REQ-044 真零仍待 TC-084/REQ-040。</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="172.5" customHeight="1">
+    <x:row r="92" ht="255" customHeight="1">
       <x:c r="A92" s="58" t="str">
         <x:v>REQ-045</x:v>
       </x:c>
@@ -2705,7 +2705,8 @@
 代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。
 2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。
 2026-10-04 Claude 逐文件确认补 controlled_account_file_mapping、external_managed_registry、evr_+32 位小写十六进制引用和显式人工声明；空/路径式/非白名单 UI 与 IPC 均拒绝并保持未归属，审计最小脱敏且标人工确认，TC-086 新增子范围待验。
-拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。</x:v>
+拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。
+2026-10-04 REQ-045/DEV-054/TC-086 补字段级错误/焦点、保留弹窗和值、同有效 previewId 修正重试；字段拒绝不改归属/审计/outbox/服务，过期/基线变化/取消/成功仍失效。新增待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -4197,7 +4198,8 @@
 选择候选只留 UI 草稿；主进程预览须显示原/新 owner、来源全部受影响事实数及相同筛选下两侧授权可见事实范围/待核对状态。确认时在事务中复验权限、来源、目标活跃性、原 owner 和预览事实集合基线；重扫或目标变化后旧预览失效，须重取。取消/Escape 无写入；失败恢复 UI 原值并给可操作错误。审计只存持久随机不透明来源引用，不存原始 key/标签/路径/账号/正文；旧审计展示/导出前脱敏。
 重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。
 2026-10-04 Claude 逐文件归属：项目/时间/UID/文件来源和管理员点击不足以证明账号。确认前逐项声明受控账号-文件映射证据类别、受控出处的不透明引用并显式确认已核对；无证据保持未归属，主进程拒绝。只以最小脱敏审计记录人工判断，不称提供方验证。
-证据字段首个白名单为 controlled_account_file_mapping / external_managed_registry / evr_ 加 32 位小写十六进制及单独确认位。真实登记未证实可用时，合成登记仅验机制；主进程可据合法声明提交标为“管理员人工确认”的事务，但不验证真实性。管理员无外部证据应选暂不归属，真实归属正例待外部复核。</x:v>
+证据字段首个白名单为 controlled_account_file_mapping / external_managed_registry / evr_ 加 32 位小写十六进制及单独确认位。真实登记未证实可用时，合成登记仅验机制；主进程可据合法声明提交标为“管理员人工确认”的事务，但不验证真实性。管理员无外部证据应选暂不归属，真实归属正例待外部复核。
+2026-10-04 Claude 证据字段无效时，弹窗保留输入、字段级提示并聚焦首个错误；同一未过期且基线有效的 previewId 可修正重试。主进程字段校验失败不消费预览，不改归属、审计或 v2 上报；过期/基线变化/取消/成功仍失效。</x:v>
       </x:c>
       <x:c r="D50" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4217,7 +4219,8 @@
 当前 sources:bind 只调用 bindIdentity，没有显式生成 usage-sync 新快照；TC-086/087 分别验在线旧 owner 清除和离线队列，TC-088 回归本地与服务状态分离。
 2026-10-03 代码 01a7095：文档会话独立复跑 TC-086/087 各单元+Electron、TC-074/080/093 及完整门禁（90 入口、66 单元、30 Electron）通过。五分钟一次性预览/基线、耐久事务审计与 v2 新队列有隔离证据；真实生产库迁移、打包安装、TC-088/089 仍待验。此前待实现文字为阶段历史。
 Claude 文件来源独立证据声明为新增待验门槛；旧 TC-086/087 通过不覆盖。
-真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。</x:v>
+真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。
+证据字段纠错与同预览重试为新增待实现/待验子范围，旧 TC-086 自动通过不覆盖。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -5701,7 +5704,8 @@
 绑定成功后创建持久版本 2 新 revision/待传义务，停止上传旧 owner 队列；在线替换/清除旧 owner 服务聚合，离线显示本地已变而服务待传并可重试。不得回退 DEV-057 v2 授权/冲突口径，交叉回归 TC-088。
 代码 01a7095 已实现草稿→预览→确认、五分钟一次性基线、主进程重验、耐久事务归属+不透明审计+v2 新 outbox。旧审计原始 key 初始化迁移；在线清设备历史授权旧 owner 聚合、保留历史未授权行，离线新 revision 替换旧队列；审计/磁盘失败回滚。文档会话独立复验 TC-086/087、TC-074/080/093 与完整门禁通过。生产库迁移、打包应用、TC-088/089 尚未验。
 Claude 文件确认 API 增 evidenceCategory=controlled_account_file_mapping、evidenceSource=external_managed_registry、evidenceRef=evr_ 加 32 位小写十六进制及显式人工确认；主进程连同预览基线校验，空/路径式/非白名单值拒绝且不改归属。审计仅留原因码/类别/来源码、不透明引用、操作者/结果，不存原始路径/账号/会话/正文/证据内容。引用真实性由外部受控登记复核，TC-086/087 回归。
-external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。</x:v>
+external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。
+Claude 确认先核预览有效/基线及证据字段；字段非法返回可定位错误且保留 pending，不写归属/审计/outbox/服务。renderer 保留弹窗和值并聚焦首个错误字段，修正后同 previewId 重试；过期、基线变化、取消与成功按原规则失效。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -9532,7 +9536,7 @@
         <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="322.5" customHeight="1">
+    <x:row r="91" ht="382.5" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9554,7 +9558,8 @@
 在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。
 关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。
 Claude 文件来源另造项目/时间似乎匹配 owner A：仅选择 A、证据类别缺失/非白名单、来源非白名单、引用空/原始路径式/格式无效、未显式确认时分别尝试 UI 和确认 IPC 直调；正例提交 controlled_account_file_mapping、external_managed_registry、evr_ 加 32 位小写十六进制与确认声明，并由外部登记复核出处。
-用合成登记和外形合法 evr_ 核人工确认事务机制，但不声称真实账号已证；真实账号-文件映射正例另待外部脱敏复核，无证据的管理员选择暂不归属。</x:v>
+用合成登记和外形合法 evr_ 核人工确认事务机制，但不声称真实账号已证；真实账号-文件映射正例另待外部脱敏复核，无证据的管理员选择暂不归属。
+在同一 Claude 预览中依次提交空/路径式 evidenceRef、未确认位，分别走 UI 与确认 IPC；检查字段级错误和焦点、原输入与 pending preview 保留，再修正后沿同 ID 成功。另在纠错时模拟五分钟过期、重扫/目标变化及取消。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
         <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
@@ -9562,10 +9567,12 @@
 预览提示本地范围即时变化、服务可能待传；在线重绑后旧 owner 服务聚合确实清除/替换，不能继续上传旧 owner 快照。
 管理员可逐文件核对、保留暂不归属；不能仅按同 UID 批量绑定或把文件来源叫账号，列表/预览/审计无原始路径、正文、账户/会话 ID。
 无有效独立证据时保持未归属，无成功审计或 viewer/CSV/v2 授权变化；有效声明仅当前文件可人工确认且审计仅留白名单类别/来源码/原因码/不透明引用/操作者/结果，界面不称提供方验证。格式校验不代替外部证据真实性复核。
-合法 evr_ 声明可触发标为人工确认的事务，程序不核外部真实性；合成登记正例不等于真实 Claude 账号归属通过，无外部证据时管理员应选暂不归属。</x:v>
+合法 evr_ 声明可触发标为人工确认的事务，程序不核外部真实性；合成登记正例不等于真实 Claude 账号归属通过，无外部证据时管理员应选暂不归属。
+字段非法时弹窗不关闭、值不丢、聚焦首个错误字段；同预览有效重试只提交一次。拒绝期间归属、任何审计、v2 outbox revision 和在线服务聚合均不变；过期/基线变化/取消及成功使原 ID 失效。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
-        <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验</x:v>
+        <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验
+证据字段纠错与同预览重试新增待补/待验；既有自动子范围不覆盖。</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
         <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
@@ -9583,7 +9590,8 @@
 在线服务旧 owner 聚合清理由隔离服务器验证；UI 仅测少量 Tab/Escape，完整背景隔离/失败回焦和目标 Mac VoiceOver 属 TC-089。未测打包 App。
 Claude 每文件来源队列 UX 是新增待验子范围；既有 TC-086 少量来源的自动通过不覆盖大量历史文件管理成本。
 独立证据声明的 UI/IPC 与审计断言未运行；旧少量来源自动通过不覆盖，证据真实性须由受控外部来源复核。
-external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。</x:v>
+external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。
+现行 confirm() 提前删除 pending，renderer 失败后关闭弹窗；本次字段纠错反例未运行，须与真正过期/基线变化错误区分。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>

</xml_diff>

<commit_message>
docs: scope Claude source deferrals per admin
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rc13684a45a9c439e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2b50fa6c88e04ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rf184eb59682a4652"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rbc821dbcab5d44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R720ed699fde14b7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8429afe8fe5742e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R53520eb3c2e74034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R87a33ee37d464a13"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2680,7 +2680,7 @@
 90338f4：TC-085 已注册 5 单元+2 Electron，取消/续扫隔离自动目标独立通过；生产/打包未验，REQ-044 真零仍待 TC-084/REQ-040。</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="255" customHeight="1">
+    <x:row r="92" ht="303.75" customHeight="1">
       <x:c r="A92" s="58" t="str">
         <x:v>REQ-045</x:v>
       </x:c>
@@ -2706,7 +2706,8 @@
 2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。
 2026-10-04 Claude 逐文件确认补 controlled_account_file_mapping、external_managed_registry、evr_+32 位小写十六进制引用和显式人工声明；空/路径式/非白名单 UI 与 IPC 均拒绝并保持未归属，审计最小脱敏且标人工确认，TC-086 新增子范围待验。
 拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。
-2026-10-04 REQ-045/DEV-054/TC-086 补字段级错误/焦点、保留弹窗和值、同有效 previewId 修正重试；字段拒绝不改归属/审计/outbox/服务，过期/基线变化/取消/成功仍失效。新增待验。</x:v>
+2026-10-04 REQ-045/DEV-054/TC-086 补字段级错误/焦点、保留弹窗和值、同有效 previewId 修正重试；字段拒绝不改归属/审计/outbox/服务，过期/基线变化/取消/成功仍失效。新增待验。
+2026-10-04 暂不归属按管理员内部 ID 持久隔离；切换/重启重算个人待办与筛选，A 不影响 B、解除恢复，未归属总数不变；暂缓不改 owner/viewer/审计/v2 服务，TC-086 待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -4199,7 +4200,8 @@
 重绑导致本地授权即刻变化；预览须提示服务同步可能待传。确认后创建持久的版本 2 新 revision/同步义务，旧 owner 快照不得继续上传；在线须替换或清除服务端旧 owner 聚合，离线须保存待传与重试原因。
 2026-10-04 Claude 逐文件归属：项目/时间/UID/文件来源和管理员点击不足以证明账号。确认前逐项声明受控账号-文件映射证据类别、受控出处的不透明引用并显式确认已核对；无证据保持未归属，主进程拒绝。只以最小脱敏审计记录人工判断，不称提供方验证。
 证据字段首个白名单为 controlled_account_file_mapping / external_managed_registry / evr_ 加 32 位小写十六进制及单独确认位。真实登记未证实可用时，合成登记仅验机制；主进程可据合法声明提交标为“管理员人工确认”的事务，但不验证真实性。管理员无外部证据应选暂不归属，真实归属正例待外部复核。
-2026-10-04 Claude 证据字段无效时，弹窗保留输入、字段级提示并聚焦首个错误；同一未过期且基线有效的 previewId 可修正重试。主进程字段校验失败不消费预览，不改归属、审计或 v2 上报；过期/基线变化/取消/成功仍失效。</x:v>
+2026-10-04 Claude 证据字段无效时，弹窗保留输入、字段级提示并聚焦首个错误；同一未过期且基线有效的 previewId 可修正重试。主进程字段校验失败不消费预览，不改归属、审计或 v2 上报；过期/基线变化/取消/成功仍失效。
+2026-10-04 Claude “暂不归属”仅是当前管理员持久待办偏好，按认证管理员内部 ID 隔离；未归属总数不减，个人待办数/筛选排除本人暂缓项。切换/重启即时加载对应视图，解除暂缓恢复本人计数，A 暂缓不影响 B；不改 owner、viewer、审计或 v2 服务。</x:v>
       </x:c>
       <x:c r="D50" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4220,7 +4222,8 @@
 2026-10-03 代码 01a7095：文档会话独立复跑 TC-086/087 各单元+Electron、TC-074/080/093 及完整门禁（90 入口、66 单元、30 Electron）通过。五分钟一次性预览/基线、耐久事务审计与 v2 新队列有隔离证据；真实生产库迁移、打包安装、TC-088/089 仍待验。此前待实现文字为阶段历史。
 Claude 文件来源独立证据声明为新增待验门槛；旧 TC-086/087 通过不覆盖。
 真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。
-证据字段纠错与同预览重试为新增待实现/待验子范围，旧 TC-086 自动通过不覆盖。</x:v>
+证据字段纠错与同预览重试为新增待实现/待验子范围，旧 TC-086 自动通过不覆盖。
+Claude 暂缓跨管理员隔离为新增待实现/待验子范围；开发草稿全局 localStorage 键不是有效证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -5705,7 +5708,8 @@
 代码 01a7095 已实现草稿→预览→确认、五分钟一次性基线、主进程重验、耐久事务归属+不透明审计+v2 新 outbox。旧审计原始 key 初始化迁移；在线清设备历史授权旧 owner 聚合、保留历史未授权行，离线新 revision 替换旧队列；审计/磁盘失败回滚。文档会话独立复验 TC-086/087、TC-074/080/093 与完整门禁通过。生产库迁移、打包应用、TC-088/089 尚未验。
 Claude 文件确认 API 增 evidenceCategory=controlled_account_file_mapping、evidenceSource=external_managed_registry、evidenceRef=evr_ 加 32 位小写十六进制及显式人工确认；主进程连同预览基线校验，空/路径式/非白名单值拒绝且不改归属。审计仅留原因码/类别/来源码、不透明引用、操作者/结果，不存原始路径/账号/会话/正文/证据内容。引用真实性由外部受控登记复核，TC-086/087 回归。
 external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。
-Claude 确认先核预览有效/基线及证据字段；字段非法返回可定位错误且保留 pending，不写归属/审计/outbox/服务。renderer 保留弹窗和值并聚焦首个错误字段，修正后同 previewId 重试；过期、基线变化、取消与成功按原规则失效。</x:v>
+Claude 确认先核预览有效/基线及证据字段；字段非法返回可定位错误且保留 pending，不写归属/审计/outbox/服务。renderer 保留弹窗和值并聚焦首个错误字段，修正后同 previewId 重试；过期、基线变化、取消与成功按原规则失效。
+将暂缓集合按当前管理员内部 ID 持久分区，禁止设备全局 token-deferred-source-keys；切换身份/重启重算未归属总数与个人待办/筛选/分页，解除暂缓恢复。仅存不透明来源引用；已归属/消失来源不计待办。暂缓/解除不触发绑定、审计、viewer 或 v2 outbox/服务变化。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -9536,7 +9540,7 @@
         <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="382.5" customHeight="1">
+    <x:row r="91" ht="405" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9559,7 +9563,8 @@
 关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。
 Claude 文件来源另造项目/时间似乎匹配 owner A：仅选择 A、证据类别缺失/非白名单、来源非白名单、引用空/原始路径式/格式无效、未显式确认时分别尝试 UI 和确认 IPC 直调；正例提交 controlled_account_file_mapping、external_managed_registry、evr_ 加 32 位小写十六进制与确认声明，并由外部登记复核出处。
 用合成登记和外形合法 evr_ 核人工确认事务机制，但不声称真实账号已证；真实账号-文件映射正例另待外部脱敏复核，无证据的管理员选择暂不归属。
-在同一 Claude 预览中依次提交空/路径式 evidenceRef、未确认位，分别走 UI 与确认 IPC；检查字段级错误和焦点、原输入与 pending preview 保留，再修正后沿同 ID 成功。另在纠错时模拟五分钟过期、重扫/目标变化及取消。</x:v>
+在同一 Claude 预览中依次提交空/路径式 evidenceRef、未确认位，分别走 UI 与确认 IPC；检查字段级错误和焦点、原输入与 pending preview 保留，再修正后沿同 ID 成功。另在纠错时模拟五分钟过期、重扫/目标变化及取消。
+再造管理员 A/B 与未归属 Claude F1/F2：A 暂缓 F1，核 A/B 待办计数与项目/最近时间/状态筛选；切 B、切回 A、重启，A 解除暂缓；另使 F1 已归属或消失，核陈旧引用。各步读取 owner/事实/审计、viewer、v2 outbox revision 与隔离服务。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
         <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
@@ -9568,11 +9573,13 @@
 管理员可逐文件核对、保留暂不归属；不能仅按同 UID 批量绑定或把文件来源叫账号，列表/预览/审计无原始路径、正文、账户/会话 ID。
 无有效独立证据时保持未归属，无成功审计或 viewer/CSV/v2 授权变化；有效声明仅当前文件可人工确认且审计仅留白名单类别/来源码/原因码/不透明引用/操作者/结果，界面不称提供方验证。格式校验不代替外部证据真实性复核。
 合法 evr_ 声明可触发标为人工确认的事务，程序不核外部真实性；合成登记正例不等于真实 Claude 账号归属通过，无外部证据时管理员应选暂不归属。
-字段非法时弹窗不关闭、值不丢、聚焦首个错误字段；同预览有效重试只提交一次。拒绝期间归属、任何审计、v2 outbox revision 和在线服务聚合均不变；过期/基线变化/取消及成功使原 ID 失效。</x:v>
+字段非法时弹窗不关闭、值不丢、聚焦首个错误字段；同预览有效重试只提交一次。拒绝期间归属、任何审计、v2 outbox revision 和在线服务聚合均不变；过期/基线变化/取消及成功使原 ID 失效。
+未归属总数不因暂缓减；A 的待办数减一且 F1 进 A 暂缓视图，B 待办/筛选仍含 F1；切换/重启不串显，解除恢复 A。陈旧项不计数；暂缓/解除不改 owner、事实、viewer/来源状态、审计、outbox 或服务聚合。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
         <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验
-证据字段纠错与同预览重试新增待补/待验；既有自动子范围不覆盖。</x:v>
+证据字段纠错与同预览重试新增待补/待验；既有自动子范围不覆盖。
+按管理员隔离“暂不归属”的双账户/重启反例新增待补/待验。</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
         <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
@@ -9591,7 +9598,8 @@
 Claude 每文件来源队列 UX 是新增待验子范围；既有 TC-086 少量来源的自动通过不覆盖大量历史文件管理成本。
 独立证据声明的 UI/IPC 与审计断言未运行；旧少量来源自动通过不覆盖，证据真实性须由受控外部来源复核。
 external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。
-现行 confirm() 提前删除 pending，renderer 失败后关闭弹窗；本次字段纠错反例未运行，须与真正过期/基线变化错误区分。</x:v>
+现行 confirm() 提前删除 pending，renderer 失败后关闭弹窗；本次字段纠错反例未运行，须与真正过期/基线变化错误区分。
+开发草稿全局 token-deferred-source-keys localStorage 可能串管理员；双账户暂缓/解除及无副作用断言未运行，旧 TC-086 通过不覆盖。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>

</xml_diff>

<commit_message>
docs: require Claude queue project and date filters
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R720ed699fde14b7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R8429afe8fe5742e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R53520eb3c2e74034"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R87a33ee37d464a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re80f2d519dcc4084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R67448edf2f844065"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfcf9645924e04cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5d7575b929874df0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2680,7 +2680,7 @@
 90338f4：TC-085 已注册 5 单元+2 Electron，取消/续扫隔离自动目标独立通过；生产/打包未验，REQ-044 真零仍待 TC-084/REQ-040。</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="303.75" customHeight="1">
+    <x:row r="92" ht="401.25" customHeight="1">
       <x:c r="A92" s="58" t="str">
         <x:v>REQ-045</x:v>
       </x:c>
@@ -2703,11 +2703,12 @@
         <x:v>TC-086 待注册/待验；草稿/授权预览、同筛选双 owner 可见范围、取消/Escape、确认、重扫后过期基线和 viewer 越权
 在线重绑须替换/清除旧 owner 服务聚合；本地授权即时变化，服务状态据实显示。
 代码 01a7095：TC-086 已注册，单元+Electron 自动子范围独立通过；在线旧 owner 清理，完整键盘/生产打包待验。
-2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态筛选或分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。
+2026-10-04 关联 Claude 文件来源：待归属数量、项目/最近时间/状态组合筛选及分页、逐项证据预览和“暂不归属”待验；不能按 UID 一键归属。
 2026-10-04 Claude 逐文件确认补 controlled_account_file_mapping、external_managed_registry、evr_+32 位小写十六进制引用和显式人工声明；空/路径式/非白名单 UI 与 IPC 均拒绝并保持未归属，审计最小脱敏且标人工确认，TC-086 新增子范围待验。
 拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。
 2026-10-04 REQ-045/DEV-054/TC-086 补字段级错误/焦点、保留弹窗和值、同有效 previewId 修正重试；字段拒绝不改归属/审计/outbox/服务，过期/基线变化/取消/成功仍失效。新增待验。
-2026-10-04 暂不归属按管理员内部 ID 持久隔离；切换/重启重算个人待办与筛选，A 不影响 B、解除恢复，未归属总数不变；暂缓不改 owner/viewer/审计/v2 服务，TC-086 待验。</x:v>
+2026-10-04 暂不归属按管理员内部 ID 持久隔离；切换/重启重算个人待办与筛选，A 不影响 B、解除恢复，未归属总数不变；暂缓不改 owner/viewer/审计/v2 服务，TC-086 待验。
+2026-10-04 本轮项目展示名精确、最近记录本机日期闭区间、状态组合筛选+分页均必需；未知时间单列、倒置报错、切换条件回首页、25+ 文件第二页/空结果/命中数，TC-086 待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -4201,7 +4202,8 @@
 2026-10-04 Claude 逐文件归属：项目/时间/UID/文件来源和管理员点击不足以证明账号。确认前逐项声明受控账号-文件映射证据类别、受控出处的不透明引用并显式确认已核对；无证据保持未归属，主进程拒绝。只以最小脱敏审计记录人工判断，不称提供方验证。
 证据字段首个白名单为 controlled_account_file_mapping / external_managed_registry / evr_ 加 32 位小写十六进制及单独确认位。真实登记未证实可用时，合成登记仅验机制；主进程可据合法声明提交标为“管理员人工确认”的事务，但不验证真实性。管理员无外部证据应选暂不归属，真实归属正例待外部复核。
 2026-10-04 Claude 证据字段无效时，弹窗保留输入、字段级提示并聚焦首个错误；同一未过期且基线有效的 previewId 可修正重试。主进程字段校验失败不消费预览，不改归属、审计或 v2 上报；过期/基线变化/取消/成功仍失效。
-2026-10-04 Claude “暂不归属”仅是当前管理员持久待办偏好，按认证管理员内部 ID 隔离；未归属总数不减，个人待办数/筛选排除本人暂缓项。切换/重启即时加载对应视图，解除暂缓恢复本人计数，A 暂缓不影响 B；不改 owner、viewer、审计或 v2 服务。</x:v>
+2026-10-04 Claude “暂不归属”仅是当前管理员持久待办偏好，按认证管理员内部 ID 隔离；未归属总数不减，个人待办数/筛选排除本人暂缓项。切换/重启即时加载对应视图，解除暂缓恢复本人计数，A 暂缓不影响 B；不改 owner、viewer、审计或 v2 服务。
+2026-10-04 Claude 队列本轮须有状态、脱敏项目展示名精确匹配、最近事实本机日期起止闭区间三种真实筛选控件，取交集后分页。未知时间无日期筛选可见、有日期时不匹配但单列数量/清除日期入口；倒置区间报错。条件、管理员或暂缓变化重置首页，区分未归属总数、我的待办数和筛选命中数。</x:v>
       </x:c>
       <x:c r="D50" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -4223,7 +4225,8 @@
 Claude 文件来源独立证据声明为新增待验门槛；旧 TC-086/087 通过不覆盖。
 真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。
 证据字段纠错与同预览重试为新增待实现/待验子范围，旧 TC-086 自动通过不覆盖。
-Claude 暂缓跨管理员隔离为新增待实现/待验子范围；开发草稿全局 localStorage 键不是有效证据。</x:v>
+Claude 暂缓跨管理员隔离为新增待实现/待验子范围；开发草稿全局 localStorage 键不是有效证据。
+项目/日期/状态组合筛选与分页是本轮真实控件要求；项目/时间仅展示或仅状态+分页不算通过，TC-086 新反例待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -4312,7 +4315,7 @@
 2026-10-04 Claude OTel：缺失、空白、非字符串、超长 user.id 或仅有安装级 user.id 均不足以证明 Claude 账户归属，新事实进入独立 unknown 且不可绑定；旧 username/hash(空串)/安装 ID 混合来源无法拆分时撤销归属。viewer 页面/CSV/来源状态/上报隔离，管理员可见脱敏诊断。累计游标与事实键不得跨账户静默合并/错算；无法证重送则保留观测并标待核对，不报完整总量。
 Codex 无 user.account_id 的两账户同字段观测不能只因 unknown 键相同就确定去重；若无可证稳定事件 ID，保留观测、标计量不确定，viewer/上报不展示确定总量。
 迁移首包发送期间若扫描排入更新 revision，应自动续传最新授权 v2 快照；服务最终确认该 revision 且清除旧 owner 聚合。旧包成功不等于启动迁移已完成。
-2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态筛选或分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。
+2026-10-04 Claude 本地 JSONL：采用每文件不透明哈希“文件来源”及包含该身份的事实键，以隔离同 UID 同 session/request；新文件默认未归属。文件分隔不证明 Claude 账号；同 UID 多账号不得自动归属或伪造跨 owner 正例，保持身份未知/覆盖限制。管理员逐文件依据额外可证证据预览绑定，UI 明示文件来源、待归属数量、项目/最近时间/状态组合筛选及分页及“暂不归属”，不暴露原始路径/内容/账户/会话 ID。移动/轮转和跨文件重放须可证去重，否则保留观测并标 uncertain。
 2026-10-04 文件代次：同一 Claude JSONL 改名/移动且可证连续时保持来源；旧文件删除后新文件即使复用 UID/dev/ino，也必须新建未归属“文件来源”，不得继承旧 owner/审计或将新事实按旧 owner 展示/上报。仅 sha256(uid:dev:ino) 不足以证明代次。
 2026-10-04 旧 UID 绑定单 JSONL 可有 S1/S2 两事实而游标只记 S2：迁移须逐事实隔离、可证重扫一一调和，已匹配临时副本不再有效计量；歧义留待核对原因与未知总量，文件本身不恢复账号 owner。逐文件人工绑定另须独立可复核证据声明，否则未归属。
 旧游标只有 file_id=dev:ino 或 birthtime_ms=0 时，不得把当前 F2 的 stat.birthtimeMs 回填为旧 F1 连续性证据；F1 待核对临时事实不清除，F2 同路径/inode/payload 仍未归属，旧 owner 确认总量不恢复。</x:v>
@@ -5709,7 +5712,8 @@
 Claude 文件确认 API 增 evidenceCategory=controlled_account_file_mapping、evidenceSource=external_managed_registry、evidenceRef=evr_ 加 32 位小写十六进制及显式人工确认；主进程连同预览基线校验，空/路径式/非白名单值拒绝且不改归属。审计仅留原因码/类别/来源码、不透明引用、操作者/结果，不存原始路径/账号/会话/正文/证据内容。引用真实性由外部受控登记复核，TC-086/087 回归。
 external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。
 Claude 确认先核预览有效/基线及证据字段；字段非法返回可定位错误且保留 pending，不写归属/审计/outbox/服务。renderer 保留弹窗和值并聚焦首个错误字段，修正后同 previewId 重试；过期、基线变化、取消与成功按原规则失效。
-将暂缓集合按当前管理员内部 ID 持久分区，禁止设备全局 token-deferred-source-keys；切换身份/重启重算未归属总数与个人待办/筛选/分页，解除暂缓恢复。仅存不透明来源引用；已归属/消失来源不计待办。暂缓/解除不触发绑定、审计、viewer 或 v2 outbox/服务变化。</x:v>
+将暂缓集合按当前管理员内部 ID 持久分区，禁止设备全局 token-deferred-source-keys；切换身份/重启重算未归属总数与个人待办/筛选/分页，解除暂缓恢复。仅存不透明来源引用；已归属/消失来源不计待办。暂缓/解除不触发绑定、审计、viewer 或 v2 outbox/服务变化。
+做脱敏项目展示名精确筛选（同名均命中）、最近事实按本机日期闭区间、状态筛选及组合分页；未知时间单列，日期筛选时排除并给清除入口，倒置日期字段错误。筛选、管理员、暂缓变化回第一页，显示分页前命中数，不混同未归属总数/本人待办数。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -5804,7 +5808,7 @@
 Claude telemetry.ts 的 string() 接受空串而 hash(空串) 可绑定，缺/无效/超长退回 os.username；改为按可证认证账户属性或经验证网关 subject 判归属，其余 unknown。旧混合键保守撤销并重算本地/服务授权；隔离累计 stream、otel_metric_cursors 和事实键，避免双账户缺 ID 同 stream/time 的丢点或错算。无法证重送保留观测并标 uncertain；首次 flush 前持久替换受影响快照。
 开发中 Codex v2 unknown:hash(mac username) 键须防两账户同 session/rawTime/model/Token 的分次 POST 被 INSERT OR IGNORE 丢第二观测；与真正重送区分不明时保留观测并降级计量。
 迁移首包与扫描新快照交错时，DEV-028 发送器须自动续传最新授权 v2；TC-094 用真实主进程启动和在线服务验证最新 revision 确认及旧 owner 聚合清除，不能以首包成功或手动 queueSnapshot 代替。当前 Electron 诊断失败待修。
-Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态筛选或分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。
+Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态组合筛选及分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。
 文件来源身份加入可验证代次/连续性判断：同文件改名保持身份与幂等；删除/轮转后的新代次即使 UID/dev/ino 复用也须先于 stat.size===start 游标短路识别并重扫，再新建未归属来源，证据不足时不得沿用 owner。旧事实/项目/脱敏审计与 v2 outbox/服务聚合按授权迁移，TC-092/093/094 回归。
 单 JSONL S1/S2 旧事实、游标仅记 S2 时逐事实隔离并与可证重扫一一匹配；已匹配临时副本退出有效计量，歧义保留原因/未知总量，不因文件身份自动恢复旧 owner，项目/审计/服务迁移幂等。逐文件绑定调用 DEV-054 的独立证据声明门槛。
 迁移不能用当前 stat.birthtimeMs 回填旧 file_id=dev:ino 或 birthtime_ms=0；F1 删除后 F2 同路径/inode/payload 也不得归档 F1 或继承 owner，首次 v2 清旧聚合；仅旧持久证据充分且逐事实匹配才归档。</x:v>
@@ -9540,7 +9544,7 @@
         <x:v>代码 90338f4；单元 5/5、Electron 2/2，单编号命令退出码 0。仅隔离自动目标通过；生产/打包未验，TC-084 真零与 REQ-044/DEV-053 整项仍待验。详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" ht="405" customHeight="1">
+    <x:row r="91" ht="408.75" customHeight="1">
       <x:c r="A91" s="58" t="str">
         <x:v>TC-086</x:v>
       </x:c>
@@ -9560,11 +9564,12 @@
         <x:v>临时库两用户/一来源已有事实；预览旧/新可见数量，取消与确认分别核对报表。
 本轮补造已确认与待核对事实、筛选内外事实；选候选只成草稿，预览原/新 owner、全部受影响数、同筛选两侧授权可见集合。取消/Escape、确认后刷新、viewer 预览/确认 IPC 越权；预览后重扫增删/改写事实或目标停用再确认，旧基线必须失效。
 在线确认时验证本地授权范围即时更新，版本 2 服务快照替换或清除旧 owner 聚合；不依赖新扫描触发同步。
-关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态筛选或分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。
+关联 Claude 大量历史 JSONL 迁移：文件来源列表展示待归属数量，可按项目/最近时间/状态组合筛选及分页，逐项预览可证上下文，选择“暂不归属”并核无授权变化。
 Claude 文件来源另造项目/时间似乎匹配 owner A：仅选择 A、证据类别缺失/非白名单、来源非白名单、引用空/原始路径式/格式无效、未显式确认时分别尝试 UI 和确认 IPC 直调；正例提交 controlled_account_file_mapping、external_managed_registry、evr_ 加 32 位小写十六进制与确认声明，并由外部登记复核出处。
 用合成登记和外形合法 evr_ 核人工确认事务机制，但不声称真实账号已证；真实账号-文件映射正例另待外部脱敏复核，无证据的管理员选择暂不归属。
 在同一 Claude 预览中依次提交空/路径式 evidenceRef、未确认位，分别走 UI 与确认 IPC；检查字段级错误和焦点、原输入与 pending preview 保留，再修正后沿同 ID 成功。另在纠错时模拟五分钟过期、重扫/目标变化及取消。
-再造管理员 A/B 与未归属 Claude F1/F2：A 暂缓 F1，核 A/B 待办计数与项目/最近时间/状态筛选；切 B、切回 A、重启，A 解除暂缓；另使 F1 已归属或消失，核陈旧引用。各步读取 owner/事实/审计、viewer、v2 outbox revision 与隔离服务。</x:v>
+再造管理员 A/B 与未归属 Claude F1/F2：A 暂缓 F1，核 A/B 待办计数与项目/最近时间/状态筛选；切 B、切回 A、重启，A 解除暂缓；另使 F1 已归属或消失，核陈旧引用。各步读取 owner/事实/审计、viewer、v2 outbox revision 与隔离服务。
+另造 25+ 文件且第二页有记录，含同名脱敏项目、不同项目、本机起止边界日、最近时间未知和 A/B 暂缓；依次组合项目精确、最近记录起止日期和状态，测试第二页改条件、倒置日期、空结果及清除条件。</x:v>
       </x:c>
       <x:c r="G91" s="58" t="str">
         <x:v>取消不改归属；确认后恰好所示事实改为新用户可见，普通用户不能确认。
@@ -9574,12 +9579,14 @@
 无有效独立证据时保持未归属，无成功审计或 viewer/CSV/v2 授权变化；有效声明仅当前文件可人工确认且审计仅留白名单类别/来源码/原因码/不透明引用/操作者/结果，界面不称提供方验证。格式校验不代替外部证据真实性复核。
 合法 evr_ 声明可触发标为人工确认的事务，程序不核外部真实性；合成登记正例不等于真实 Claude 账号归属通过，无外部证据时管理员应选暂不归属。
 字段非法时弹窗不关闭、值不丢、聚焦首个错误字段；同预览有效重试只提交一次。拒绝期间归属、任何审计、v2 outbox revision 和在线服务聚合均不变；过期/基线变化/取消及成功使原 ID 失效。
-未归属总数不因暂缓减；A 的待办数减一且 F1 进 A 暂缓视图，B 待办/筛选仍含 F1；切换/重启不串显，解除恢复 A。陈旧项不计数；暂缓/解除不改 owner、事实、viewer/来源状态、审计、outbox 或服务聚合。</x:v>
+未归属总数不因暂缓减；A 的待办数减一且 F1 进 A 暂缓视图，B 待办/筛选仍含 F1；切换/重启不串显，解除恢复 A。陈旧项不计数；暂缓/解除不改 owner、事实、viewer/来源状态、审计、outbox 或服务聚合。
+三条件先取交集再分页；同项目展示名均命中，日期两端包含。未知时间无日期时可见、有日期时不命中但另列数量和清除入口。显示分页前命中数；改条件/管理员/暂缓重置首页，A/B 不串；空结果给清除动作而不称无来源。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
         <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验
 证据字段纠错与同预览重试新增待补/待验；既有自动子范围不覆盖。
-按管理员隔离“暂不归属”的双账户/重启反例新增待补/待验。</x:v>
+按管理员隔离“暂不归属”的双账户/重启反例新增待补/待验。
+项目/最近日期真实控件、25+ 文件第二页、未知时间与空结果等组合断言新增待补/待验。</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
         <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
@@ -9599,7 +9606,8 @@
 独立证据声明的 UI/IPC 与审计断言未运行；旧少量来源自动通过不覆盖，证据真实性须由受控外部来源复核。
 external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。
 现行 confirm() 提前删除 pending，renderer 失败后关闭弹窗；本次字段纠错反例未运行，须与真正过期/基线变化错误区分。
-开发草稿全局 token-deferred-source-keys localStorage 可能串管理员；双账户暂缓/解除及无副作用断言未运行，旧 TC-086 通过不覆盖。</x:v>
+开发草稿全局 token-deferred-source-keys localStorage 可能串管理员；双账户暂缓/解除及无副作用断言未运行，旧 TC-086 通过不覆盖。
+开发未提交工作树报告项目/日期控件与 25 文件 E2E 阶段性通过；倒置日期、未知时间/清除入口、空结果动作及命中数尚缺，未固定提交或独立复验。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
         <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>

</xml_diff>

<commit_message>
docs: record independent 508851a validation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re80f2d519dcc4084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R67448edf2f844065"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfcf9645924e04cad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5d7575b929874df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5f6238c0b9a540c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R207c983698084e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9a00f672c4dc40db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R28695be9a4174483"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -648,7 +648,8 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。</x:v>
+        <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
+当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1608,7 +1609,8 @@
       </x:c>
       <x:c r="G45" s="35" t="str">
         <x:v>已验证（自动；范围见文档）
-2026-10-04 TC-040 新增发送中排快照立即顺序 drain 与失败退避/状态断言；开发会话真实启动诊断 pending=1、修订未确认，当前失败待修，旧自动通过子范围保留。</x:v>
+2026-10-04 TC-040 新增发送中排快照立即顺序 drain 与失败退避/状态断言；开发会话真实启动诊断 pending=1、修订未确认，当前失败待修，旧自动通过子范围保留。
+508851a：TC-040 4 个单元绑定独立通过；真实长期退避/生产环境待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="62" customHeight="1">
@@ -2463,7 +2465,8 @@
 2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。
 2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。
 2026-10-04 安装中取消设计已决：独立控制窗口+helper 阶段回执、替换后回滚和 userData 隔离健康探测，TC-076 分阶段打包 UI 真取消待实现/验收；既有成功/故障证据不变。
-2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
+508851a：历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -2708,7 +2711,8 @@
 拟定登记枚举未有真实可用性证据；合成 evr_ 仅验机制，真实逐文件归属及整项验收待外部可复核来源。
 2026-10-04 REQ-045/DEV-054/TC-086 补字段级错误/焦点、保留弹窗和值、同有效 previewId 修正重试；字段拒绝不改归属/审计/outbox/服务，过期/基线变化/取消/成功仍失效。新增待验。
 2026-10-04 暂不归属按管理员内部 ID 持久隔离；切换/重启重算个人待办与筛选，A 不影响 B、解除恢复，未归属总数不变；暂缓不改 owner/viewer/审计/v2 服务，TC-086 待验。
-2026-10-04 本轮项目展示名精确、最近记录本机日期闭区间、状态组合筛选+分页均必需；未知时间单列、倒置报错、切换条件回首页、25+ 文件第二页/空结果/命中数，TC-086 待验。</x:v>
+2026-10-04 本轮项目展示名精确、最近记录本机日期闭区间、状态组合筛选+分页均必需；未知时间单列、倒置报错、切换条件回首页、25+ 文件第二页/空结果/命中数，TC-086 待验。
+508851a：TC-086 3 单元+4 Electron 隔离自动通过；真实外部受控登记/生产打包待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="85" customHeight="1">
@@ -2733,7 +2737,8 @@
       <x:c r="G93" s="55" t="str">
         <x:v>TC-087 待注册/待验；业务拒绝、事务/审计失败、数据库不可写、原子回滚与不透明审计引用及旧日志脱敏
 离线重绑须留新 revision/待传，旧 owner 队列失效，恢复后重试。
-代码 01a7095：TC-087 已注册，单元+Electron 自动子范围独立通过；回滚、旧日志合成迁移、离线新队列已证，生产迁移/打包待验。</x:v>
+代码 01a7095：TC-087 已注册，单元+Electron 自动子范围独立通过；回滚、旧日志合成迁移、离线新队列已证，生产迁移/打包待验。
+508851a：TC-087 单元/Electron 各 1 独立通过；生产迁移/打包全量待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="85" customHeight="1">
@@ -2859,7 +2864,8 @@
 2026-10-04 Claude 跨 owner 正例限定可证不同 UID/上下文；同 UID 两文件同键默认未归属。待验每文件不透明来源+事实键、逐文件绑定成本、移动/轮转/跨文件重放与旧库迁移；文件不等于账号。
 2026-10-04 同文件改名保持身份与旧文件删除后新代次同路径/UID/dev/ino/size/tailHash、birthtime 不同须越过旧游标短路且不继承 owner 的对照待验；旧事实/项目/审计/服务隔离及迁移幂等。
 2026-10-04 单文件 S1/S2、游标仅 S2 须逐事实隔离/一一调和；临时副本不重复计量，歧义留原因/未知总量且不自动恢复旧 owner；TC-092 待验。
-旧游标仅 dev:ino 或 birthtime_ms=0 时不可用 F2 当前 birthtime 倒填；F1 待核对不清除、F2 未归属、首包清旧 owner，TC-092 待验。</x:v>
+旧游标仅 dev:ino 或 birthtime_ms=0 时不可用 F2 当前 birthtime 倒填；F1 待核对不清除、F2 未归属、首包清旧 owner，TC-092 待验。
+508851a：TC-092 15 个单元绑定独立通过；真实历史来源/外部映射待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="330" customHeight="1">
@@ -2886,7 +2892,8 @@
 2026-10-04 81c271b TC-093 真实隔离 JSONL+回环 OTel+归属+UI/CSV v2 单元 1/1、Electron 2/2 独立通过；共同 ID 去重/生产迁移仍待证。
 2026-10-04 TC-093 关联 viewer 报表/明细/CSV/来源状态、诊断与通用提示回归待补，不改变既有通过子范围。
 2026-10-04 TC-093 关联迁移期/失败/恢复后的 viewer 页面、CSV、来源状态通用提示与隔离，待验。
-2026-10-04 TC-093 新增 Claude unknown 与旧归属撤销后的 viewer 页面/CSV/来源状态/诊断附件隔离，待验。</x:v>
+2026-10-04 TC-093 新增 Claude unknown 与旧归属撤销后的 viewer 页面/CSV/来源状态/诊断附件隔离，待验。
+508851a：TC-093 单元 1/1、Electron 2/2 独立通过；真实历史/异机待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="375" customHeight="1">
@@ -2913,7 +2920,8 @@
 2026-10-04 TC-094 关联旧 owner 聚合清理、v2 待传/恢复与未知身份不上报的回归待补。
 2026-10-04 TC-094 关联真实主进程启动与在线服务：首次 flush 前受影响的旧 v1/v2 outbox 替换、旧 owner 聚合删除和同 owner 旧 OTel confirmed 降 uncertain；手动排队单测不足，待验。
 2026-10-04 TC-094 新增 Claude unknown 或累计降级后的首次 flush 前快照重算与在线旧聚合清理/降级，待验。
-2026-10-04 TC-094 真实 Electron 启动发送竞态当前失败：迁移首包成功后扫描新 revision 未立即续传；需自动 drain 到服务确认最新 revision 并清旧 owner 聚合，不靠 60 秒定时器。</x:v>
+2026-10-04 TC-094 真实 Electron 启动发送竞态当前失败：迁移首包成功后扫描新 revision 未立即续传；需自动 drain 到服务确认最新 revision 并清旧 owner 聚合，不靠 60 秒定时器。
+508851a：TC-094 单元 2/2、Electron 1/1 独立通过；真实生产迁移/旧服务待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3686,7 +3694,7 @@
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E31" s="35" t="str">
-        <x:v>代码已落地（自动覆盖；边界待验）</x:v>
+        <x:v>已编码且 TC-040 发送中续传隔离自动通过；长期运行/生产待验</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
         <x:v>DEV-028、DEV-023</x:v>
@@ -3696,7 +3704,8 @@
       </x:c>
       <x:c r="H31" s="35" t="str">
         <x:v>docs/design.md §9–13；docs/development-plan.md §7
-开发会话真实 Electron 启动诊断：首包成功后留下 pending=1、localRevision&gt;confirmedRevision、lastError=null，直到 60 秒定时器；新交错当前失败待修，旧 TC-040 自动通过仅覆盖原离线补传样本。</x:v>
+开发会话真实 Electron 启动诊断：首包成功后留下 pending=1、localRevision&gt;confirmedRevision、lastError=null，直到 60 秒定时器；新交错当前失败待修，旧 TC-040 自动通过仅覆盖原离线补传样本。
+508851a：发送中新增 revision、末次队列读取竞态和失败退避已在固定提交独立通过。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -4209,7 +4218,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E50" s="58" t="str">
-        <x:v>既有重绑子范围已实现且隔离自动通过；Claude 逐文件证据门槛待实现/待验，真实受控出处待证；生产库迁移/打包应用待验</x:v>
+        <x:v>已编码且 TC-086/087 隔离自动子范围通过；真实外部受控登记/生产待验</x:v>
       </x:c>
       <x:c r="F50" s="58" t="str">
         <x:v>DEV-054</x:v>
@@ -4226,7 +4235,8 @@
 真实受控账号-文件登记尚无可复核证据；TC-086 真实逐文件归属正例待外部来源，不能以合成 evr_ 升整项状态。
 证据字段纠错与同预览重试为新增待实现/待验子范围，旧 TC-086 自动通过不覆盖。
 Claude 暂缓跨管理员隔离为新增待实现/待验子范围；开发草稿全局 localStorage 键不是有效证据。
-项目/日期/状态组合筛选与分页是本轮真实控件要求；项目/时间仅展示或仅状态+分页不算通过，TC-086 新反例待验。</x:v>
+项目/日期/状态组合筛选与分页是本轮真实控件要求；项目/时间仅展示或仅状态+分页不算通过，TC-086 新反例待验。
+508851a：Claude 证据声明格式、同预览纠错、个人暂缓与项目/日期/状态组合筛选已测；人工声明不证明外部登记真实。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="150" customHeight="1">
@@ -4324,7 +4334,7 @@
         <x:v>缺陷修复（已复现）</x:v>
       </x:c>
       <x:c r="E53" s="61" t="str">
-        <x:v>已编码；TC-092–094 自动子范围通过，TC-093 在 81c271b 增真实隔离输入 E2E 并独立复验；跨账户同键碰撞待修，正向精确去重/生产迁移待验证；新增 Claude 文件代次、多 session 与旧游标倒填反例待实现/待验</x:v>
+        <x:v>已编码且 TC-092–094 隔离自动子范围通过；真实生产迁移/历史身份待验</x:v>
       </x:c>
       <x:c r="F53" s="61" t="str">
         <x:v>DEV-057</x:v>
@@ -4350,7 +4360,8 @@
 现行 claude.ts 的 sourceIdentityKey=context.fallbackIdentityKey，scanner.ts fallback 为 claude:macos:&lt;uid&gt;，事实键 claude:session:request；同 UID 多文件缺账号证据。开发报告未提交工作树 test:gate 94 入口/89 单元/40 Electron 退出码 0，无固定提交供文档会话复验，状态不升。
 开发中 sha256(uid:dev:ino) 方案尚无固定提交可独立验收；inode 可复用，需同文件改名与不同代次同元组对照。现仅修订验收口径，状态不升。
 单文件多 session 旧库迁移和逐文件独立证据声明为新增待验范围；现无固定实现及动态通过。
-旧游标代次倒填反例待验：仅旧持久连续性证据和逐事实映射充分才归档 F1；首包 v2 须清旧 owner 聚合。</x:v>
+旧游标代次倒填反例待验：仅旧持久连续性证据和逐事实映射充分才归档 F1；首包 v2 须清旧 owner 聚合。
+508851a：本地/OTel 键隔离、保守旧来源迁移与首次 v2 清旧 owner 聚合已测；旧历史事实不可凭合成样本重建。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5084,11 +5095,12 @@
         <x:v>src/main/usage-sync.ts；src/server/server.ts；tests/next-sync.test.ts</x:v>
       </x:c>
       <x:c r="F33" s="35" t="str">
-        <x:v>已编码（自动覆盖；边界待验）</x:v>
+        <x:v>已编码；TC-040 发送中续传/失败退避隔离自动通过，长期运行待验</x:v>
       </x:c>
       <x:c r="G33" s="35" t="str">
         <x:v>自动测试见 TC 关联；提交 96e99be；完整验收限制见 docs/test-case-acceptance.md
-修复 UsageSync.flush 发送中排队竞态：旧包成功后比较当前持久 outbox revision 并立即顺序 drain，避免并发重复发送；失败保留错误与待传，按有限退避重试。pending=1 且本地 revision 高于确认 revision 时不得显示已同步。TC-040 增可控延迟/失败断言。</x:v>
+修复 UsageSync.flush 发送中排队竞态：旧包成功后比较当前持久 outbox revision 并立即顺序 drain，避免并发重复发送；失败保留错误与待传，按有限退避重试。pending=1 且本地 revision 高于确认 revision 时不得显示已同步。TC-040 增可控延迟/失败断言。
+508851a：4 个 TC-040 单元绑定独立通过；不靠 60 秒定时器才能继续传。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="62" customHeight="1">
@@ -5701,7 +5713,7 @@
         <x:v>src/main/source-binding.ts、database.ts、index.ts、usage-sync.ts；src/collectors/scanner.ts；src/server/server.ts；src/renderer/index.tsx、source-binding.tsx；tests/source-binding.test.ts、tests/e2e/source-binding.spec.ts</x:v>
       </x:c>
       <x:c r="F59" s="58" t="str">
-        <x:v>既有重绑流程已开发且 TC-086/087 隔离自动子范围通过；Claude 独立证据声明待实现/待验，生产/打包待验</x:v>
+        <x:v>已编码；TC-086/087 Claude 证据、个人队列与重绑隔离自动通过；外部登记/生产待验</x:v>
       </x:c>
       <x:c r="G59" s="58" t="str">
         <x:v>预览受影响事实数/可见范围，确认后主进程复验权限和版本；事务提交归属及最小审计，失败不改变归属；审计不保存路径/正文。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5713,7 +5725,8 @@
 external_managed_registry 仅为拟定出处码；主进程只核 evr_ 声明格式，不在线验证外部记录；合法声明可提交标为人工确认的事务。无真实登记时管理员应选暂不归属，合成登记只验 IPC/事务/审计，真实正例待外部复核。
 Claude 确认先核预览有效/基线及证据字段；字段非法返回可定位错误且保留 pending，不写归属/审计/outbox/服务。renderer 保留弹窗和值并聚焦首个错误字段，修正后同 previewId 重试；过期、基线变化、取消与成功按原规则失效。
 将暂缓集合按当前管理员内部 ID 持久分区，禁止设备全局 token-deferred-source-keys；切换身份/重启重算未归属总数与个人待办/筛选/分页，解除暂缓恢复。仅存不透明来源引用；已归属/消失来源不计待办。暂缓/解除不触发绑定、审计、viewer 或 v2 outbox/服务变化。
-做脱敏项目展示名精确筛选（同名均命中）、最近事实按本机日期闭区间、状态筛选及组合分页；未知时间单列，日期筛选时排除并给清除入口，倒置日期字段错误。筛选、管理员、暂缓变化回第一页，显示分页前命中数，不混同未归属总数/本人待办数。</x:v>
+做脱敏项目展示名精确筛选（同名均命中）、最近事实按本机日期闭区间、状态筛选及组合分页；未知时间单列，日期筛选时排除并给清除入口，倒置日期字段错误。筛选、管理员、暂缓变化回第一页，显示分页前命中数，不混同未归属总数/本人待办数。
+508851a：TC-086 3 单元+4 Electron；TC-087 1 单元+1 Electron，均 exit 0；外部证据仅合成格式。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="155" customHeight="1">
@@ -5789,7 +5802,7 @@
         <x:v>src/main/reconcile.ts、report.ts、usage-sync.ts、index.ts；src/server/server.ts；src/shared/types.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；tests/reconciliation.test.ts、sync-reconciliation.test.ts、e2e/overlap-privacy.spec.ts；scripts/test-cases.mjs</x:v>
       </x:c>
       <x:c r="F62" s="61" t="str">
-        <x:v>已实现调和子范围；TC-093 真实隔离输入 E2E 通过（81c271b）；TC-092 跨账户同键碰撞待修，正向精确去重/真实迁移待验证；新增 Claude 文件代次、多 session 与旧游标倒填反例待实现/待验</x:v>
+        <x:v>已编码；TC-092–094 身份隔离/保守迁移/服务清理自动通过；生产待验</x:v>
       </x:c>
       <x:c r="G62" s="61" t="str">
         <x:v>先以 TC-092 复现同日跨用户被误排除。建立授权 owner 过滤后的共同调和函数：仅按可证共同事件身份去重；不同用户/明确不同会话保留；仅同会话或身份不明的重叠不得臆定重复或完整，应标冲突。输出已确认小计、授权范围内待核对来源/条数及“总量不可确认”状态，报表/明细/CSV 同口径；不改 Codex/Claude 原始事实或 Token 分类，不泄露其他用户/原始身份。兼容旧库，复跑 TC-016、TC-021–023、TC-038、TC-092–093 和门禁。
@@ -5811,7 +5824,8 @@
 Claude 本地来源改为每 JSONL 不透明哈希文件身份并纳入事实键；新来源默认未归属，文件/UID 不等于账号。旧 claude:macos:uid 绑定和同键事实保守幂等迁移，无法逐条证明则撤销 owner；移动/轮转别名、跨文件同事件重放须可证去重，否则 uncertain。UI 称“文件来源”，管理员逐文件凭额外证据预览/绑定，待归属数量及项目/最近时间/状态组合筛选及分页可操作，保留“暂不归属”，不泄露路径/正文/原始 ID；TC-086 回归管理成本与审计，TC-094 回归服务旧聚合。
 文件来源身份加入可验证代次/连续性判断：同文件改名保持身份与幂等；删除/轮转后的新代次即使 UID/dev/ino 复用也须先于 stat.size===start 游标短路识别并重扫，再新建未归属来源，证据不足时不得沿用 owner。旧事实/项目/脱敏审计与 v2 outbox/服务聚合按授权迁移，TC-092/093/094 回归。
 单 JSONL S1/S2 旧事实、游标仅记 S2 时逐事实隔离并与可证重扫一一匹配；已匹配临时副本退出有效计量，歧义保留原因/未知总量，不因文件身份自动恢复旧 owner，项目/审计/服务迁移幂等。逐文件绑定调用 DEV-054 的独立证据声明门槛。
-迁移不能用当前 stat.birthtimeMs 回填旧 file_id=dev:ino 或 birthtime_ms=0；F1 删除后 F2 同路径/inode/payload 也不得归档 F1 或继承 owner，首次 v2 清旧聚合；仅旧持久证据充分且逐事实匹配才归档。</x:v>
+迁移不能用当前 stat.birthtimeMs 回填旧 file_id=dev:ino 或 birthtime_ms=0；F1 删除后 F2 同路径/inode/payload 也不得归档 F1 或继承 owner，首次 v2 清旧聚合；仅旧持久证据充分且逐事实匹配才归档。
+508851a：TC-092 15 单元；TC-093 1 单元+2 Electron；TC-094 2 单元+1 Electron，均 exit 0。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7571,11 +7585,12 @@
 成功后单发送器立即顺序 drain 最新快照且服务确认最新 revision；失败保留 pending/lastError、守有限退避，恢复后自动补传，无忙循环或 60 秒定时器/人工重试依赖。</x:v>
       </x:c>
       <x:c r="H45" s="35" t="str">
-        <x:v>旧离线补传自动子范围通过；发送中排新快照未立即续传，当前失败待修</x:v>
+        <x:v>TC-040 4 个单元绑定独立通过；真实长期退避/生产环境待验</x:v>
       </x:c>
       <x:c r="I45" s="35" t="str">
         <x:v>提交 96e99be；逐项日志见 test-results/acceptance/（本机，未提交）；门禁结果见 docs/validation.md
-2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。</x:v>
+2026-10-03：DEV-048 受影响回归，文档会话在 533992e 独立复跑单编号退出码 0；原样本与覆盖边界仍见 L/M 列。
+508851a：4 个单元绑定逐项 exit 0；发送中追加、末次读取竞态、失败退避。</x:v>
       </x:c>
       <x:c r="J45" s="35" t="str">
         <x:v>npm run test:case -- TC-040</x:v>
@@ -7585,10 +7600,12 @@
       </x:c>
       <x:c r="L45" s="35" t="str">
         <x:v>持久待传和恢复补传；未长时间运行验证退避
-开发会话真实 Electron 启动诊断残留 pending=1、localRevision&gt;confirmedRevision、lastError=null 至 60 秒定时器；新断言未修/未独立复验，旧 TC-040 通过不覆盖。</x:v>
+开发会话真实 Electron 启动诊断残留 pending=1、localRevision&gt;confirmedRevision、lastError=null 至 60 秒定时器；新断言未修/未独立复验，旧 TC-040 通过不覆盖。
+旧“当前失败待修”是 508851a 前阶段；新固定提交已通过隔离反例。</x:v>
       </x:c>
       <x:c r="M45" s="35" t="str">
-        <x:v>记录 TC-040 命令、退出码、提交、环境和脱敏日志；覆盖与限制：持久待传和恢复补传；未长时间运行验证退避。</x:v>
+        <x:v>记录 TC-040 命令、退出码、提交、环境和脱敏日志；覆盖与限制：持久待传和恢复补传；未长时间运行验证退避。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；4 个单元绑定逐项 exit 0；发送中追加、末次读取竞态、失败退避。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="70" customHeight="1">
@@ -9076,13 +9093,14 @@
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>已注册；1961de3 真实 DMG 隔离成功升级、只读旧包初始启动、installer 模块及打包 helper 五故障回退/重试自动子范围独立通过；真实系统目录/满盘/崩溃/安装中取消待验</x:v>
+        <x:v>历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过</x:v>
       </x:c>
       <x:c r="I81" s="68" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
 2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
 86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。
-2026-10-04 / 80e7f10→0eac84b：80e7f10 文档独立首次全命令：成功段、只读初始启动、五故障回退输出通过；末次重试读取已被 UI 消费的一次性 last-install.json 得 undefined，exit 1。0eac84b 修脚本后同 DMG 再跑，全命令 exit 0；旧包 142557541 字节 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 142591838 字节 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c，两包 verify VALID。旧 27aae018… 只属历史候选。</x:v>
+2026-10-04 / 80e7f10→0eac84b：80e7f10 文档独立首次全命令：成功段、只读初始启动、五故障回退输出通过；末次重试读取已被 UI 消费的一次性 last-install.json 得 undefined，exit 1。0eac84b 修脚本后同 DMG 再跑，全命令 exit 0；旧包 142557541 字节 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 142591838 字节 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c，两包 verify VALID。旧 27aae018… 只属历史候选。
+508851a：TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="str">
         <x:v>TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c npm run test:case -- TC-076</x:v>
@@ -9097,13 +9115,15 @@
 0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。
 2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。
 2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。
-2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。</x:v>
+2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。
+本次并未复跑真实旧/新 DMG 与固定 SHA 的故障链；历史 1961de3 证据另列。系统安装、签名公证及安装中取消未验。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
 2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。
 1961de3；文档会话独立 TC-076 完整命令 exit 0，真实旧/新 DMG SHA-256 分别 ae1b8e80…、d99d7af9…，两包 hdiutil verify VALID；打包 helper mount/space/replace/launch/health 各回退、受信登录/1280 Token/清理及最后重试均通过；TC-036 两单元 exit 0。
-1961de3 文档会话独立 test:gate 类型检查、94 入口、77/77 单元、39/39 Electron exit 0；未另跑打包版全量。</x:v>
+1961de3 文档会话独立 test:gate 类型检查、94 入口、77/77 单元、39/39 Electron exit 0；未另跑打包版全量。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">
@@ -9583,13 +9603,11 @@
 三条件先取交集再分页；同项目展示名均命中，日期两端包含。未知时间无日期时可见、有日期时不命中但另列数量和清除入口。显示分页前命中数；改条件/管理员/暂缓重置首页，A/B 不串；空结果给清除动作而不称无来源。</x:v>
       </x:c>
       <x:c r="H91" s="58" t="str">
-        <x:v>已注册；既有单元+Electron 子范围通过；Claude 证据门槛与大量文件 UX 待补/待验，真实外部证据待取；完整键盘/生产打包待验
-证据字段纠错与同预览重试新增待补/待验；既有自动子范围不覆盖。
-按管理员隔离“暂不归属”的双账户/重启反例新增待补/待验。
-项目/最近日期真实控件、25+ 文件第二页、未知时间与空结果等组合断言新增待补/待验。</x:v>
+        <x:v>TC-086 3 单元+4 Electron 隔离自动通过；真实外部受控登记/生产打包待验</x:v>
       </x:c>
       <x:c r="I91" s="58" t="str">
-        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。</x:v>
+        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。完整门禁 90 入口、66 单元、30 Electron 通过。前述“待注册/不可运行”为实施前历史。
+508851a：3 个单元与 4 个 Electron 绑定逐项 exit 0；证据字段纠错、同预览重试、25 文件分页、组合筛选、未知日期及 A/B 管理员暂缓隔离。</x:v>
       </x:c>
       <x:c r="J91" s="58" t="str">
         <x:v>npm run test:case -- TC-086（2026-10-03 独立通过）</x:v>
@@ -9607,10 +9625,12 @@
 external_managed_registry 暂无真实可用性证据；真实人工归属正例及 TC-086 整项仍待外部证据。
 现行 confirm() 提前删除 pending，renderer 失败后关闭弹窗；本次字段纠错反例未运行，须与真正过期/基线变化错误区分。
 开发草稿全局 token-deferred-source-keys localStorage 可能串管理员；双账户暂缓/解除及无副作用断言未运行，旧 TC-086 通过不覆盖。
-开发未提交工作树报告项目/日期控件与 25 文件 E2E 阶段性通过；倒置日期、未知时间/清除入口、空结果动作及命中数尚缺，未固定提交或独立复验。</x:v>
+开发未提交工作树报告项目/日期控件与 25 文件 E2E 阶段性通过；倒置日期、未知时间/清除入口、空结果动作及命中数尚缺，未固定提交或独立复验。
+旧“待补/待验”描述为固定提交前阶段。外部登记只用合成 evr_ 引用，真实性未验证；打包全量另有偶发失败。</x:v>
       </x:c>
       <x:c r="M91" s="58" t="str">
-        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。</x:v>
+        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产数据/打包与 TC-089 单独待验。详见 docs/validation.md。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；3 个单元与 4 个 Electron 绑定逐项 exit 0；证据字段纠错、同预览重试、25 文件分页、组合筛选、未知日期及 A/B 管理员暂缓隔离。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="380" customHeight="1">
@@ -9640,10 +9660,11 @@
 本地重绑成功但服务离线时分别显示本地已变和服务待传/重试；恢复后按版本 2 口径上传，旧 owner 聚合清除且旧快照不再发送。</x:v>
       </x:c>
       <x:c r="H92" s="55" t="str">
-        <x:v>已注册；单元+Electron 自动子范围通过，生产迁移/打包待验</x:v>
+        <x:v>TC-087 单元/Electron 各 1 独立通过；生产迁移/打包全量待验</x:v>
       </x:c>
       <x:c r="I92" s="55" t="str">
-        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。TC-074 回归证明历史未授权服务行保留；完整门禁 90 入口、66 单元、30 Electron 通过。此前“待注册/不可运行”为实施前历史。</x:v>
+        <x:v>2026-10-03 文档会话在代码 01a7095、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0。TC-074 回归证明历史未授权服务行保留；完整门禁 90 入口、66 单元、30 Electron 通过。此前“待注册/不可运行”为实施前历史。
+508851a：单元 1/1、Electron 1/1，exit 0；回滚、审计和旧基线回归。</x:v>
       </x:c>
       <x:c r="J92" s="55" t="str">
         <x:v>npm run test:case -- TC-087（2026-10-03 独立通过）</x:v>
@@ -9655,10 +9676,12 @@
         <x:v>只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 scanner.bindIdentity() 当前 audit_events.target_id 写原始 key，是需修正的旧行为；旧行任何展示/导出前也须脱敏。独立合成用户/来源，不提交真实账户、路径、会话正文或凭证；测试注入失败后清理。
 模拟断网、旧队列与恢复，审计与同步失败分别断言，DEV-057 v2 冲突口径保持。
-旧审计原始 key 仅以隔离合成旧行验证初始化迁移；注入审计和磁盘持久化失败并验回滚，离线新 v2 队列恢复。真实生产库迁移/打包未验。</x:v>
+旧审计原始 key 仅以隔离合成旧行验证初始化迁移；注入审计和磁盘持久化失败并验回滚，离线新 v2 队列恢复。真实生产库迁移/打包未验。
+生产历史审计数据、打包全量稳定性未由本次单编号证明。</x:v>
       </x:c>
       <x:c r="M92" s="55" t="str">
-        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产库迁移、打包应用未验。详见 docs/validation.md。</x:v>
+        <x:v>代码 01a7095；单元 1/1、Electron 1/1，命令退出码 0。仅隔离自动子范围通过；生产库迁移、打包应用未验。详见 docs/validation.md。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 1/1、Electron 1/1，exit 0；回滚、审计和旧基线回归。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="400" customHeight="1">
@@ -9910,10 +9933,11 @@
 F2 当前 birthtime 不可倒填证明 F1；F1 临时事实继续未归属/待核对且不被清除，F2 新来源未归属，首包 v2 与在线服务无旧 owner 已确认聚合；仅旧持久证据充分时归档。</x:v>
       </x:c>
       <x:c r="H97" s="61" t="str">
-        <x:v>已注册；单元自动子范围 1/1 通过（8157e2d），正向精确去重待证；新增 Claude 文件代次、多 session 与旧游标倒填反例待补/待验</x:v>
+        <x:v>TC-092 15 个单元绑定独立通过；真实历史来源/外部映射待验</x:v>
       </x:c>
       <x:c r="I97" s="61" t="str">
-        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-092：单元 1/1、退出码 0；管理员初值 111，owner B 99，A 不同会话 19，同会话后已确认小计 7/状态 uncertain。test:gate 82 注册入口、56 单元、22 Electron 通过。</x:v>
+        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-092：单元 1/1、退出码 0；管理员初值 111，owner B 99，A 不同会话 19，同会话后已确认小计 7/状态 uncertain。test:gate 82 注册入口、56 单元、22 Electron 通过。
+508851a：15 个单元绑定逐项 exit 0；同键/同毫秒、缺身份、旧 UID 多 session、文件代次/游标、重扫及幂等迁移。</x:v>
       </x:c>
       <x:c r="J97" s="61" t="str">
         <x:v>npm run test:case -- TC-092（已注册；文档会话退出码 0）</x:v>
@@ -9933,10 +9957,12 @@
 现行 Claude JSONL 不能证同 UID 多账号分别属于不同 owner；不可通过预先手工分配 owner 伪造 TC-092。文件级来源及管理员逐文件绑定/TC-086 UI 成本、移动/轮转和重放新断言待实现/运行；未提交 gate 结果不提升状态。
 inode 复用难在真实文件系统稳定强制，可用受控元数据注入测同路径/大小/尾哈希、birthtime 不同的新代次反例；仅 fact-key helper 测试不足以验游标短路；另留真实改名/轮转集成。开发方案未有固定提交，本反例未运行，旧通过子范围不覆盖。
 单文件 S1/S2、游标仅 S2 的旧库迁移反例未运行；临时副本有效计量清理、歧义原因及旧 owner 服务清理仍待固定提交验证。
-旧 birthtime 缺失/为 0 和 F2 复用同 payload 的倒填反例未运行，不能凭当前 stat 或旧游标末值证明连续性。</x:v>
+旧 birthtime 缺失/为 0 和 F2 复用同 payload 的倒填反例未运行，不能凭当前 stat 或旧游标末值证明连续性。
+旧“待补/待修”是固定提交前状态；真实碰撞已丢事实不可重建，生产历史覆盖未知；共同稳定事件 ID 正向去重仍缺。</x:v>
       </x:c>
       <x:c r="M97" s="61" t="str">
-        <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。</x:v>
+        <x:v>8157e2d；macOS 本机专用临时 SQLite；单编号单元 1/1 退出码 0，完整门禁 82 入口/56 单元/22 Electron 退出码 0。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；15 个单元绑定逐项 exit 0；同键/同毫秒、缺身份、旧 UID 多 session、文件代次/游标、重扫及幂等迁移。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="185" customHeight="1">
@@ -9968,13 +9994,13 @@
 只按 provider 相同不得泄露 B 的文件/事实/未归属/异常计数、位置/原因、扫描/成功时间；通用指引和 A 可证字段可保留，无法归属字段未知/省略，反馈附件不增加权限。</x:v>
       </x:c>
       <x:c r="H98" s="64" t="str">
-        <x:v>已注册；单元+Electron 自动子范围通过（47b03d5），真实冲突事实完整 E2E/生产环境待验证
-已注册；81c271b 真实隔离 JSONL+OTel+归属+页面/明细/CSV v2 Electron 链路及原隐私 Electron、单元子范围经文档会话独立复验通过；生产迁移/共同 ID 正向去重仍待证</x:v>
+        <x:v>TC-093 单元 1/1、Electron 2/2 独立通过；真实历史/异机待验</x:v>
       </x:c>
       <x:c r="I98" s="64" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-093：Vitest 1/1、Electron 1/1、退出码 0；单元 v2 十四列三组小计 5/7/0，总计 12，冲突明细保留 5 条，跨窗候选仍标冲突。Electron 真实 IPC/反馈附件双 owner 隔离；冲突 UI 文案采用注入响应。test:gate 82/56/22 全过。
 47b03d5 文档会话独立复跑 TC-093：unit 1/1、Electron 1/1、退出码 0；Electron 新验 viewer 直调 sources:scan 被拒、概览 Codex 卡本人 1 条且不含 B 的 2 条及 B 遥测时间。TC-023/079 v2 回归亦独立通过，gate 82/57/22。
-2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-093，unit 1/1、Electron 1/1，退出码 0；仅现有绑定断言。</x:v>
+2026-10-03 c10bbf3 受影响回归：文档会话独立运行 npm run test:case -- TC-093，unit 1/1、Electron 1/1，退出码 0；仅现有绑定断言。
+508851a：单元 1/1、Electron 2/2，exit 0；真实隔离 JSONL/回环 OTel 与 viewer/CSV 授权链。</x:v>
       </x:c>
       <x:c r="J98" s="64" t="str">
         <x:v>npm run test:case -- TC-093（已注册；文档会话单元+Electron 退出码 0）</x:v>
@@ -9987,13 +10013,15 @@
 2026-10-04 新测试使用独立临时库的真实本机 JSONL 扫描与回环 OTel 接收、正式归属 IPC、两 viewer UI/CSV；旧注入响应测试保留为不同证据层。非第三方生产历史，跨账户完全同键碰撞仍归 TC-092 待修。
 关联 TC-093 回归：缺身份/旧绑定撤销后，viewer 概览/报表/明细/CSV v2、来源状态、诊断和可选反馈附件不得泄露未知事实；受影响本人仅见通用提示。新断言未执行。
 关联 TC-093：迁移中/重扫失败时概览、报表、明细、CSV、来源状态给本人通用提示，不泄露来源或其他用户；成功恢复后数值与提示同步。待验。
-关联 TC-093：Claude unknown 或旧混合键撤销后 viewer 概览/报表/明细/CSV/来源状态/诊断附件无其他账户事实，仅通用提示；新断言待验。</x:v>
+关联 TC-093：Claude unknown 或旧混合键撤销后 viewer 概览/报表/明细/CSV/来源状态/诊断附件无其他账户事实，仅通用提示；新断言待验。
+仅合成输入与本机回环，不代替真实生产历史。</x:v>
       </x:c>
       <x:c r="M98" s="64" t="str">
         <x:v>8157e2d；macOS 本机专用临时库与 Electron；单编号 unit 1/1、E2E 1/1 退出码 0，门禁 82 入口/56 unit/22 E2E 通过。
 47b03d5；macOS 本机隔离临时库/Electron；TC-093 unit/E2E 各 1/1 退出码 0，TC-023 两单元、TC-079 unit/E2E 均退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
 c10bbf3；macOS x86_64 隔离合成样本；TC-093 unit 1/1、Electron 1/1、单编号退出码 0；完整门禁 84 入口/59 unit/24 Electron 通过。
-81c271b；文档会话独立 npm run test:case -- TC-093：unit 1/1、Electron 2/2、exit 0；真实隔离输入 A 本地 12/5、OTel 14，B OTel 99；A 已确认 5、待核对 2、明细 [5,12,14]、CSV v2 14 列/B 仅 99。</x:v>
+81c271b；文档会话独立 npm run test:case -- TC-093：unit 1/1、Electron 2/2、exit 0；真实隔离输入 A 本地 12/5、OTel 14，B OTel 99；A 已确认 5、待核对 2、明细 [5,12,14]、CSV v2 14 列/B 仅 99。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 1/1、Electron 2/2，exit 0；真实隔离 JSONL/回环 OTel 与 viewer/CSV 授权链。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="315" customHeight="1">
@@ -10023,10 +10051,11 @@
 首包成功后立即顺序 drain 更新 v2，不靠定时器/人工重试；服务确认最新 revision 并删除旧 owner 聚合。失败时保持退避和可观察待传，不把旧包确认误作最新确认。</x:v>
       </x:c>
       <x:c r="H99" s="67" t="str">
-        <x:v>旧隔离服务自动子范围 1/1 通过（8157e2d）；真实 Electron 启动发送中排新快照未续传，当前失败待修</x:v>
+        <x:v>TC-094 单元 2/2、Electron 1/1 独立通过；真实生产迁移/旧服务待验</x:v>
       </x:c>
       <x:c r="I99" s="67" t="str">
-        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-094：单元 1/1、退出码 0。合成旧表迁移、旧 v1 续传 legacy_unknown/GET confirmedSubtotal=null、v2 重算及冲突、跨 owner/白名单拒绝、v1 回滚状态不变、旧 outbox 重算及协议不兼容待传后恢复。完整 gate 82/56/22 通过。</x:v>
+        <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-094：单元 1/1、退出码 0。合成旧表迁移、旧 v1 续传 legacy_unknown/GET confirmedSubtotal=null、v2 重算及冲突、跨 owner/白名单拒绝、v1 回滚状态不变、旧 outbox 重算及协议不兼容待传后恢复。完整 gate 82/56/22 通过。
+508851a：单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。</x:v>
       </x:c>
       <x:c r="J99" s="67" t="str">
         <x:v>npm run test:case -- TC-094（已注册；文档会话退出码 0）</x:v>
@@ -10039,10 +10068,12 @@
 关联 TC-094 回归：迁移撤销旧 fallback owner 后，v2 快照/旧 owner 服务聚合清理、离线待传与恢复、白名单/授权边界；未知身份不得上传成已归属用量。新断言未执行。
 关联 TC-094：预置旧 v1/v2 outbox，任何影响授权或已确认小计/状态的迁移，真实启动首次 flush 前持久替换；在线服务删除旧 owner 聚合，同 owner 旧 OTel confirmed 降 uncertain；离线/替换失败时旧包不能外传，恢复后只传新 v2。待验。
 关联 TC-094：Claude 旧混合键归属撤销或累计状态降 uncertain 后，真实启动首次 flush 前替换 v1/v2 outbox，在线清旧 owner 聚合或降状态；未知事实不按旧 owner 上传。待验。
-开发会话真实 Electron 启动诊断：迁移首包成功，扫描在发送中排新 revision；flush 仅等旧 promise，剩 pending=1、localRevision&gt;confirmedRevision、lastError=null，直至 60 秒定时器。本交错当前失败，修复及独立复验待做。</x:v>
+开发会话真实 Electron 启动诊断：迁移首包成功，扫描在发送中排新 revision；flush 仅等旧 promise，剩 pending=1、localRevision&gt;confirmedRevision、lastError=null，直至 60 秒定时器。本交错当前失败，修复及独立复验待做。
+使用合成旧库/本机服务；真实旧服务版本互操作和生产库迁移未验。</x:v>
       </x:c>
       <x:c r="M99" s="67" t="str">
-        <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。</x:v>
+        <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: track version progress and packaged date failure
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5f6238c0b9a540c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R207c983698084e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9a00f672c4dc40db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R28695be9a4174483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1cb780518bc24605"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R50d39b0bfc5b4d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R369da6f6681243d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf3fdea548cc84f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R953e0762189c40fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -56,8 +57,24 @@
       <x:color rgb="FF243247"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF25465D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="37">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -209,19 +226,67 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153C59"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF167D87"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9F3FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="5">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
         <x:color rgb="FFC5D2DF"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E3E8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E3E8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E3E8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9E3E8"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="73">
+  <x:cellXfs count="91">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -419,6 +484,44 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="33" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="34" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="35" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -649,7 +752,8 @@
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
         <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
-当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。</x:v>
+当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。
+2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -733,7 +837,8 @@
         <x:v>首次创建与重启登录</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
@@ -779,7 +884,8 @@
         <x:v>用户创建与权限隔离</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -802,7 +908,8 @@
         <x:v>管理 IPC 拒绝越权</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -917,7 +1024,8 @@
         <x:v>重复扫描和重启幂等</x:v>
       </x:c>
       <x:c r="G15" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="38" customHeight="1">
@@ -1124,7 +1232,8 @@
         <x:v>绑定后权限和报表更新</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="38" customHeight="1">
@@ -1193,7 +1302,8 @@
         <x:v>CSV 与页面结果一致</x:v>
       </x:c>
       <x:c r="G27" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
@@ -1285,7 +1395,8 @@
         <x:v>跨进程权限和数据边界</x:v>
       </x:c>
       <x:c r="G31" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）
+2026-10-04 打包共用 app.spec.ts 重复 3/5，日期字段回退；该打包路径待修/复验，历史自动子范围证据保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
@@ -2539,7 +2650,8 @@
         <x:v>异步筛选与 CSV 快照一致</x:v>
       </x:c>
       <x:c r="G85" s="55" t="str">
-        <x:v>78b3a3b 已注册；TC-079 单元 1/1 + Electron 1/1 通过；仅 REQ-041 同事实集合查询/导出子范围</x:v>
+        <x:v>78b3a3b 已注册；TC-079 单元 1/1 + Electron 1/1 通过；仅 REQ-041 同事实集合查询/导出子范围
+2026-10-04 REQ-041→DEV-050→TC-079 新增双日期连续快速修改/最终组合/无错误/CSV 同屏验收；当前打包共用路径重复 3/5，2 次失败，待修/复验。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="85" customHeight="1">
@@ -4090,13 +4202,14 @@
         <x:v>筛选异步加载与 CSV 同一查询</x:v>
       </x:c>
       <x:c r="C46" s="58" t="str">
-        <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。</x:v>
+        <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。
+2026-10-04 打包缺陷验收补充：在用量报表连续快速修改开始和结束日期，两输入值均须保持最终选择；查询只使用最终起止日期组合，无倒置范围错误。当前屏显结果与 CSV 必须使用同一授权筛选、时区和快照，期间旧请求不得覆写新组合。</x:v>
       </x:c>
       <x:c r="D46" s="58" t="str">
         <x:v>下一轮产品打磨（第一批 B 阶段实现）</x:v>
       </x:c>
       <x:c r="E46" s="58" t="str">
-        <x:v>已实现；同事实集合查询/导出子范围验证通过（78b3a3b，本机隔离样本）</x:v>
+        <x:v>原异步/快照子范围通过；0.3.6 打包日期双字段快速修改反例当前失败，待修/复验</x:v>
       </x:c>
       <x:c r="F46" s="58" t="str">
         <x:v>DEV-050</x:v>
@@ -4107,7 +4220,8 @@
       <x:c r="H46" s="58" t="str">
         <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。
-47b03d5：TC-079 追加 v1→冲突 v2、扫描入库后旧 snapshotId 拒绝及刷新小计 99→104；文档会话单元+Electron 与 gate 独立通过。</x:v>
+47b03d5：TC-079 追加 v1→冲突 v2、扫描入库后旧 snapshotId 拒绝及刷新小计 99→104；文档会话单元+Electron 与 gate 独立通过。
+508851a 未签名目录包共用报表 E2E 重复 5 次中 2 次开始日期回退；验收补充先于开发修改。旧 TC-079 源码态通过不覆盖打包连续修改。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="150" customHeight="1">
@@ -5611,13 +5725,14 @@
         <x:v>src/main/report.ts、index.ts；src/preload/index.ts；src/renderer/report.tsx；src/shared/types.ts；tests/report-snapshot.test.ts、tests/e2e/report-snapshot.spec.ts；scripts/test-cases.mjs、run-test-case.mjs</x:v>
       </x:c>
       <x:c r="F55" s="58" t="str">
-        <x:v>已实现；TC-079 单元/Electron 各 1/1 通过（78b3a3b）</x:v>
+        <x:v>既有异步快照子范围已实现；0.3.6 打包日期双字段反例当前失败，待修/复验</x:v>
       </x:c>
       <x:c r="G55" s="58" t="str">
         <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。
 78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。
-47b03d5：TC-079 原单元新增冲突 v2 快照身份回归：新增遥测使旧 ID 拒绝、刷新小计 99，继续新增事实又拒绝，刷新小计 104；单编号 unit/Electron 与完整门禁独立通过。</x:v>
+47b03d5：TC-079 原单元新增冲突 v2 快照身份回归：新增遥测使旧 ID 拒绝、刷新小计 99，继续新增事实又拒绝，刷新小计 104；单编号 unit/Electron 与完整门禁独立通过。
+2026-10-04 新修复目标：排查日期输入状态/异步请求竞态，确保连续快速填写两端后值保持、只查询最终组合、无日期范围错误，CSV 与屏显同快照；TC-079 加打包反例，TC-021 管理员主流程回归。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="155" customHeight="1">
@@ -5997,10 +6112,11 @@
         <x:v>账户与既有数据保留。</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I7" s="10" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A1</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A1
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J7" s="27" t="str">
         <x:v>npm run test:case -- TC-002</x:v>
@@ -6012,7 +6128,8 @@
         <x:v>共享测试；非独立断言</x:v>
       </x:c>
       <x:c r="M7" s="27" t="str">
-        <x:v>保存命令、退出码和 Playwright 脱敏日志；记录提交及 macOS 环境。</x:v>
+        <x:v>保存命令、退出码和 Playwright 脱敏日志；记录提交及 macOS 环境。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60" customHeight="1">
@@ -6079,10 +6196,11 @@
         <x:v>仅可见已归属用量，不出现管理入口。</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I9" s="10" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J9" s="27" t="str">
         <x:v>npm run test:case -- TC-004</x:v>
@@ -6094,7 +6212,8 @@
         <x:v>共享测试；非独立断言</x:v>
       </x:c>
       <x:c r="M9" s="27" t="str">
-        <x:v>保存共享 Playwright 函数的命令与退出码；说明本编号没有独立测试函数。</x:v>
+        <x:v>保存共享 Playwright 函数的命令与退出码；说明本编号没有独立测试函数。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="60" customHeight="1">
@@ -6120,10 +6239,11 @@
         <x:v>所有未授权调用被拒绝。</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
         <x:v>npm run test:case -- TC-005</x:v>
@@ -6135,7 +6255,8 @@
         <x:v>共享测试；非独立断言</x:v>
       </x:c>
       <x:c r="M10" s="9" t="str">
-        <x:v>保存共享 Playwright 函数的命令与退出码；标注三项 IPC 结果。</x:v>
+        <x:v>保存共享 Playwright 函数的命令与退出码；标注三项 IPC 结果。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="60" customHeight="1">
@@ -6325,10 +6446,11 @@
         <x:v>事实数与总量不增加。</x:v>
       </x:c>
       <x:c r="H15" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I15" s="10" t="str">
-        <x:v>tests/collector.test.ts；tests/e2e/app.spec.ts；A5</x:v>
+        <x:v>tests/collector.test.ts；tests/e2e/app.spec.ts；A5
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J15" s="27" t="str">
         <x:v>npm run test:case -- TC-010</x:v>
@@ -6341,7 +6463,8 @@
         <x:v>共享测试；非独立断言</x:v>
       </x:c>
       <x:c r="M15" s="27" t="str">
-        <x:v>保留同一 TC 命令的两段测试日志及退出码；说明两个绑定函数均通过。</x:v>
+        <x:v>保留同一 TC 命令的两段测试日志及退出码；说明两个绑定函数均通过。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="60" customHeight="1">
@@ -6696,10 +6819,11 @@
         <x:v>该用户可见绑定来源，其他来源仍不可见。</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A7</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A7
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
         <x:v>npm run test:case -- TC-019</x:v>
@@ -6711,7 +6835,8 @@
         <x:v>共享测试；非独立断言</x:v>
       </x:c>
       <x:c r="M24" s="9" t="str">
-        <x:v>保存共享 Playwright 函数命令、退出码和 12/14 权限对比。</x:v>
+        <x:v>保存共享 Playwright 函数命令、退出码和 12/14 权限对比。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
@@ -6781,7 +6906,8 @@
         <x:v>已验证（自动；独立翻页）</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。 后续：961c96c 补启动失败清理；8234dcc 补样本写入/数据库关闭异常清理。开发会话在 8234dcc 上报告类型检查、TC-021 单编号及完整门禁通过（73 入口/42 单元/18 Electron）；文档会话独立复跑四个绑定退出码 0；见 docs/validation.md。</x:v>
+        <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。 后续：961c96c 补启动失败清理；8234dcc 补样本写入/数据库关闭异常清理。开发会话在 8234dcc 上报告类型检查、TC-021 单编号及完整门禁通过（73 入口/42 单元/18 Electron）；文档会话独立复跑四个绑定退出码 0；见 docs/validation.md。
+2026-10-04 作为 REQ-041/TC-079 日期回退修复的管理员筛选与分页回归；新目标修复后按编号单独复跑，不能用既有结果替代。</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
         <x:v>npm run test:case -- TC-021</x:v>
@@ -6793,7 +6919,8 @@
         <x:v>共享旧测试继续运行。独立单元：123 条事实分页 50/50/23、ID 不重复、总 Token 与报表一致；普通用户仅见 61 条、第二页 11 条，用户/提供方/模型/项目/日期筛选贯穿分页。独立 Electron：61 条合成 Codex 记录首屏 50、第二页 11，切换第二模型后回首页并显示 10。未用生产库或新版安装包；TC-047 跨用户服务授权未验。</x:v>
       </x:c>
       <x:c r="M26" s="9" t="str">
-        <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。 8234dcc 使测试异常时的一次性目录清理更完整；产品行为、断言和绑定未变。</x:v>
+        <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。 8234dcc 使测试异常时的一次性目录清理更完整；产品行为、断言和绑定未变。
+TC-021 为关联回归，尚未针对新日期缺陷复跑；主验收归 TC-079。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -6819,10 +6946,11 @@
         <x:v>示例两行 12、14 Token，与页面 26 一致。</x:v>
       </x:c>
       <x:c r="H27" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I27" s="10" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A9</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A9
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J27" s="27" t="str">
         <x:v>npm run test:case -- TC-022</x:v>
@@ -6834,7 +6962,8 @@
         <x:v>共享测试；非独立断言；CSV 列结构未测试</x:v>
       </x:c>
       <x:c r="M27" s="27" t="str">
-        <x:v>保存共享 Playwright 日志和脱敏 CSV 数值；当前测试没有检查表头 8/9 列错位，见 TC-029。</x:v>
+        <x:v>保存共享 Playwright 日志和脱敏 CSV 数值；当前测试没有检查表头 8/9 列错位，见 TC-029。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -6986,10 +7115,11 @@
         <x:v>主进程拒绝越权；样本无会话正文或密钥。</x:v>
       </x:c>
       <x:c r="H31" s="10" t="str">
-        <x:v>已验证（自动）</x:v>
+        <x:v>已验证（自动）；当前打包共用用例重复运行不稳定，待修/复验</x:v>
       </x:c>
       <x:c r="I31" s="10" t="str">
-        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2</x:v>
+        <x:v>tests/e2e/app.spec.ts；docs/validation.md A2
+2026-10-04 同一 508851a 未签名目录包 app.asar 8a687bf6…：开发会话运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1；文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05，结束日期 2026-01-02，报日期范围无效。待定位应用状态/测试时序；历史源码态通过不等于打包稳定。</x:v>
       </x:c>
       <x:c r="J31" s="27" t="str">
         <x:v>npm run test:case -- TC-026</x:v>
@@ -7001,7 +7131,8 @@
         <x:v>共享测试；非独立断言；磁盘隐私未测试</x:v>
       </x:c>
       <x:c r="M31" s="27" t="str">
-        <x:v>保存共享 Playwright 日志；现有测试未断言磁盘/导出中不存在正文或密钥。</x:v>
+        <x:v>保存共享 Playwright 日志；现有测试未断言磁盘/导出中不存在正文或密钥。
+同一共用 Electron 用例对应多个 TC；失败发生在日期报表断言，不能直接判每个前置步骤失败，也不能把打包版整项标稳定通过。详细复现见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="60" customHeight="1">
@@ -9263,19 +9394,22 @@
       </x:c>
       <x:c r="F84" s="55" t="str">
         <x:v>独立库快速切换 A/B 筛选并延迟 A 返回；B 查询完成后再扫描入库，分别在 B 加载、完成及新扫描后导出。
-已注册单元以专用临时 SQLite 在查询后插入同筛选事实并重算快照；Electron 以延迟 IPC 模拟 A→B 快速切换与过期导出。</x:v>
+已注册单元以专用临时 SQLite 在查询后插入同筛选事实并重算快照；Electron 以延迟 IPC 模拟 A→B 快速切换与过期导出。
+0.3.6 打包补例：进入管理员用量报表，连续快速填写开始 2026-01-01、结束 2026-01-02；重复运行至少 5 次并检查字段最终值、查询参数/页面数字和 CSV；再造两端不同快速变化及旧请求晚返回。关联 TC-021 管理员主流程回归。</x:v>
       </x:c>
       <x:c r="G84" s="55" t="str">
         <x:v>旧响应不覆盖 B；加载时导出禁用或等待 B；页面和 CSV 的授权查询键、数据库 revision/快照身份及逐事实集合一致；新扫描不能造成旧页面/新 CSV 错配。
-授权查询和选中事实的 SHA-256 快照 ID；事实变化后旧 ID 拒绝并提示刷新，刷新后 12→111 Token；不同筛选/角色的旧 ID 拒绝。Electron 最终只显示 B，加载中禁用导出，IPC 携带 B 筛选及 B ID。</x:v>
+授权查询和选中事实的 SHA-256 快照 ID；事实变化后旧 ID 拒绝并提示刷新，刷新后 12→111 Token；不同筛选/角色的旧 ID 拒绝。Electron 最终只显示 B，加载中禁用导出，IPC 携带 B 筛选及 B ID。
+两个日期输入最终值稳定为用户最后选择；查询只取新的有效日期组合、无“日期范围无效”；屏显指标/明细和 CSV 使用同一授权查询与事实快照；旧响应不能回退任何日期或结果。</x:v>
       </x:c>
       <x:c r="H84" s="55" t="str">
-        <x:v>已注册；v1/v2 快照单元及 Electron 子范围通过（47b03d5）</x:v>
+        <x:v>既有源码态 v1/v2 快照子范围通过；0.3.6 打包双日期快速修改新反例当前失败，待修/复验</x:v>
       </x:c>
       <x:c r="I84" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。
-47b03d5 文档会话独立运行 TC-079：单元与 Electron 均通过、退出码 0；单元增加 v1→v2 冲突、扫描后旧 snapshotId 拒绝和刷新小计 99→104；完整 gate 82/57/22 通过。</x:v>
+47b03d5 文档会话独立运行 TC-079：单元与 Electron 均通过、退出码 0；单元增加 v1→v2 冲突、扫描后旧 snapshotId 拒绝和刷新小计 99→104；完整 gate 82/57/22 通过。
+2026-10-04 固定代码 508851a、app.asar SHA-256 8a687bf6…：开发会话在文档工作树运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1。文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05、结束 2026-01-02，报日期范围无效；新增 TC-079 断言尚未实现，当前失败不能写通过。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
         <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
@@ -9284,11 +9418,13 @@
         <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。</x:v>
       </x:c>
       <x:c r="L84" s="55" t="str">
-        <x:v>当前已在单元测试覆盖 v1 与冲突 v2 的扫描后旧 snapshotId 拒绝；Electron 仍侧重快速筛选切换与导出等待当前快照。snapshotId 是授权查询+事实集合身份，不是全库 revision；REQ-040 历史覆盖及目标安装环境仍未由此证明。</x:v>
+        <x:v>当前已在单元测试覆盖 v1 与冲突 v2 的扫描后旧 snapshotId 拒绝；Electron 仍侧重快速筛选切换与导出等待当前快照。snapshotId 是授权查询+事实集合身份，不是全库 revision；REQ-040 历史覆盖及目标安装环境仍未由此证明。
+本次打包共用 app.spec.ts 只复现异常，尚未有专属 TC-079 双日期快速修改绑定；失败根因未定，应用状态与测试时序需区分。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
         <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。
-47b03d5；macOS 本机隔离合成库；TC-079 单元/Electron 各 1/1、退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。</x:v>
+47b03d5；macOS 本机隔离合成库；TC-079 单元/Electron 各 1/1、退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
+0.3.6 打包日期新验收当前失败 2/5；修复后必须单编号运行 TC-079、TC-021 回归，再重复打包用例并跑打包全量。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="185" customHeight="1">
@@ -10079,4 +10215,426 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF167D87"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14.220000267028809" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="40" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="36.11000061035156" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="27.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="39.439998626708984" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="37.779998779296875" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="31.5" customHeight="1">
+      <x:c r="A1" s="74" t="str">
+        <x:v>Token 版本规划与迭代状态</x:v>
+      </x:c>
+      <x:c r="B1" s="74"/>
+      <x:c r="C1" s="74"/>
+      <x:c r="D1" s="74"/>
+      <x:c r="E1" s="74"/>
+      <x:c r="F1" s="74"/>
+      <x:c r="G1" s="74"/>
+      <x:c r="H1" s="74"/>
+      <x:c r="I1" s="74"/>
+      <x:c r="J1" s="74"/>
+      <x:c r="K1" s="74"/>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="77" t="str">
+        <x:v>截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。历史本机候选不等于公开发布；“待定”不承诺版本号或日期。进度按已取得证据填写，未完成项不能由源码门禁自动转为版本完成。</x:v>
+      </x:c>
+      <x:c r="B2" s="77"/>
+      <x:c r="C2" s="77"/>
+      <x:c r="D2" s="77"/>
+      <x:c r="E2" s="77"/>
+      <x:c r="F2" s="77"/>
+      <x:c r="G2" s="77"/>
+      <x:c r="H2" s="77"/>
+      <x:c r="I2" s="77"/>
+      <x:c r="J2" s="77"/>
+      <x:c r="K2" s="77"/>
+    </x:row>
+    <x:row r="3" ht="21" customHeight="1">
+      <x:c r="A3" s="77"/>
+      <x:c r="B3" s="77"/>
+      <x:c r="C3" s="77"/>
+      <x:c r="D3" s="77"/>
+      <x:c r="E3" s="77"/>
+      <x:c r="F3" s="77"/>
+      <x:c r="G3" s="77"/>
+      <x:c r="H3" s="77"/>
+      <x:c r="I3" s="77"/>
+      <x:c r="J3" s="77"/>
+      <x:c r="K3" s="77"/>
+    </x:row>
+    <x:row r="5" ht="25.5" customHeight="1">
+      <x:c r="A5" s="86" t="str">
+        <x:v>版本跟踪ID</x:v>
+      </x:c>
+      <x:c r="B5" s="86" t="str">
+        <x:v>版本/候选</x:v>
+      </x:c>
+      <x:c r="C5" s="86" t="str">
+        <x:v>迭代范围</x:v>
+      </x:c>
+      <x:c r="D5" s="86" t="str">
+        <x:v>版本主要功能点</x:v>
+      </x:c>
+      <x:c r="E5" s="86" t="str">
+        <x:v>关联需求</x:v>
+      </x:c>
+      <x:c r="F5" s="86" t="str">
+        <x:v>关联开发任务</x:v>
+      </x:c>
+      <x:c r="G5" s="86" t="str">
+        <x:v>关联测试用例</x:v>
+      </x:c>
+      <x:c r="H5" s="86" t="str">
+        <x:v>迭代进度（已证阶段）</x:v>
+      </x:c>
+      <x:c r="I5" s="86" t="str">
+        <x:v>版本完成状态</x:v>
+      </x:c>
+      <x:c r="J5" s="86" t="str">
+        <x:v>固定证据</x:v>
+      </x:c>
+      <x:c r="K5" s="86" t="str">
+        <x:v>剩余事项/下一步</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="84" customHeight="1">
+      <x:c r="A6" s="87" t="str">
+        <x:v>VER-001</x:v>
+      </x:c>
+      <x:c r="B6" s="87" t="str">
+        <x:v>0.2.0</x:v>
+      </x:c>
+      <x:c r="C6" s="87" t="str">
+        <x:v>首版与 M5 基础</x:v>
+      </x:c>
+      <x:c r="D6" s="87" t="str">
+        <x:v>本机账户与两家工具采集、报表/CSV；受信登录、独立服务、聚合上报和更新基础</x:v>
+      </x:c>
+      <x:c r="E6" s="87" t="str">
+        <x:v>REQ-001–030</x:v>
+      </x:c>
+      <x:c r="F6" s="87" t="str">
+        <x:v>DEV-001–033</x:v>
+      </x:c>
+      <x:c r="G6" s="87" t="str">
+        <x:v>TC-001–049</x:v>
+      </x:c>
+      <x:c r="H6" s="87" t="str">
+        <x:v>代码与本机候选已形成；逐项验收见各 TC</x:v>
+      </x:c>
+      <x:c r="I6" s="87" t="str">
+        <x:v>历史本机候选；外部验收不完整</x:v>
+      </x:c>
+      <x:c r="J6" s="87" t="str">
+        <x:v>96e99be；package.json 历史版本提交；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K6" s="87" t="str">
+        <x:v>按逐项 TC 继续核真实来源、生产环境与目标 Mac</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="84" customHeight="1">
+      <x:c r="A7" s="88" t="str">
+        <x:v>VER-002</x:v>
+      </x:c>
+      <x:c r="B7" s="88" t="str">
+        <x:v>0.3.0</x:v>
+      </x:c>
+      <x:c r="C7" s="88" t="str">
+        <x:v>M6 产品扩展</x:v>
+      </x:c>
+      <x:c r="D7" s="88" t="str">
+        <x:v>项目分析、导航、诊断、反馈与固定超级管理员</x:v>
+      </x:c>
+      <x:c r="E7" s="88" t="str">
+        <x:v>REQ-031–039</x:v>
+      </x:c>
+      <x:c r="F7" s="88" t="str">
+        <x:v>DEV-034–046</x:v>
+      </x:c>
+      <x:c r="G7" s="88" t="str">
+        <x:v>TC-050–072</x:v>
+      </x:c>
+      <x:c r="H7" s="88" t="str">
+        <x:v>代码/编号入口已落地；本机未签名包有子范围证据</x:v>
+      </x:c>
+      <x:c r="I7" s="88" t="str">
+        <x:v>历史本机候选；未完成外部分发</x:v>
+      </x:c>
+      <x:c r="J7" s="88" t="str">
+        <x:v>0f10cec；docs/development-plan.md §8；TC-027 本机证据</x:v>
+      </x:c>
+      <x:c r="K7" s="88" t="str">
+        <x:v>TC-028/072 及生产账号/权限环境继续待验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="84" customHeight="1">
+      <x:c r="A8" s="87" t="str">
+        <x:v>VER-003</x:v>
+      </x:c>
+      <x:c r="B8" s="87" t="str">
+        <x:v>0.3.1</x:v>
+      </x:c>
+      <x:c r="C8" s="87" t="str">
+        <x:v>Codex fallback 修复</x:v>
+      </x:c>
+      <x:c r="D8" s="87" t="str">
+        <x:v>跨扫描 fallback 被正式记录替代；旧库幂等清理</x:v>
+      </x:c>
+      <x:c r="E8" s="87" t="str">
+        <x:v>REQ-006</x:v>
+      </x:c>
+      <x:c r="F8" s="87" t="str">
+        <x:v>DEV-047</x:v>
+      </x:c>
+      <x:c r="G8" s="87" t="str">
+        <x:v>TC-010、TC-073</x:v>
+      </x:c>
+      <x:c r="H8" s="87" t="str">
+        <x:v>单编号/目录包与 0.3.0→0.3.1 同库隔离升级已证</x:v>
+      </x:c>
+      <x:c r="I8" s="87" t="str">
+        <x:v>历史本机候选；生产迁移待验</x:v>
+      </x:c>
+      <x:c r="J8" s="87" t="str">
+        <x:v>aa6d91b、867a03a；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K8" s="87" t="str">
+        <x:v>真实生产账户安装与签名目标 Mac 待验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="84" customHeight="1">
+      <x:c r="A9" s="88" t="str">
+        <x:v>VER-004</x:v>
+      </x:c>
+      <x:c r="B9" s="88" t="str">
+        <x:v>0.3.2</x:v>
+      </x:c>
+      <x:c r="C9" s="88" t="str">
+        <x:v>服务上传授权初版</x:v>
+      </x:c>
+      <x:c r="D9" s="88" t="str">
+        <x:v>设备令牌、owner 写库前授权和客户端凭据保存</x:v>
+      </x:c>
+      <x:c r="E9" s="88" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="F9" s="88" t="str">
+        <x:v>DEV-023、DEV-048</x:v>
+      </x:c>
+      <x:c r="G9" s="88" t="str">
+        <x:v>TC-047、TC-074</x:v>
+      </x:c>
+      <x:c r="H9" s="88" t="str">
+        <x:v>隔离授权测试已证；随后发现服务切换竞态</x:v>
+      </x:c>
+      <x:c r="I9" s="88" t="str">
+        <x:v>历史候选，已被 0.3.3 修正</x:v>
+      </x:c>
+      <x:c r="J9" s="88" t="str">
+        <x:v>ca0f37f；docs/development-plan.md §10</x:v>
+      </x:c>
+      <x:c r="K9" s="88" t="str">
+        <x:v>不作为最终交付结论；采用 0.3.3 及后续证据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="84" customHeight="1">
+      <x:c r="A10" s="87" t="str">
+        <x:v>VER-005</x:v>
+      </x:c>
+      <x:c r="B10" s="87" t="str">
+        <x:v>0.3.3</x:v>
+      </x:c>
+      <x:c r="C10" s="87" t="str">
+        <x:v>服务切换修正</x:v>
+      </x:c>
+      <x:c r="D10" s="87" t="str">
+        <x:v>配置代次阻止旧登记响应与令牌跨服务使用</x:v>
+      </x:c>
+      <x:c r="E10" s="87" t="str">
+        <x:v>REQ-021</x:v>
+      </x:c>
+      <x:c r="F10" s="87" t="str">
+        <x:v>DEV-048</x:v>
+      </x:c>
+      <x:c r="G10" s="87" t="str">
+        <x:v>TC-047、TC-074</x:v>
+      </x:c>
+      <x:c r="H10" s="87" t="str">
+        <x:v>竞态回归/本机候选及隔离升级已证</x:v>
+      </x:c>
+      <x:c r="I10" s="87" t="str">
+        <x:v>历史本机候选；生产部署待验</x:v>
+      </x:c>
+      <x:c r="J10" s="87" t="str">
+        <x:v>3d60b5e；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K10" s="87" t="str">
+        <x:v>可信证书异机、真实生产账户/库待验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="84" customHeight="1">
+      <x:c r="A11" s="88" t="str">
+        <x:v>VER-006</x:v>
+      </x:c>
+      <x:c r="B11" s="88" t="str">
+        <x:v>0.3.4</x:v>
+      </x:c>
+      <x:c r="C11" s="88" t="str">
+        <x:v>大会话启动性能</x:v>
+      </x:c>
+      <x:c r="D11" s="88" t="str">
+        <x:v>只检查真实 fallback 会话；6000 条无 fallback 样本和生产库临时副本启动</x:v>
+      </x:c>
+      <x:c r="E11" s="88" t="str">
+        <x:v>REQ-006</x:v>
+      </x:c>
+      <x:c r="F11" s="88" t="str">
+        <x:v>DEV-047</x:v>
+      </x:c>
+      <x:c r="G11" s="88" t="str">
+        <x:v>TC-010、TC-027、TC-073</x:v>
+      </x:c>
+      <x:c r="H11" s="88" t="str">
+        <x:v>单编号、隔离副本启动、DMG 与本机人工子范围已证</x:v>
+      </x:c>
+      <x:c r="I11" s="88" t="str">
+        <x:v>历史本机候选；异机与签名待验</x:v>
+      </x:c>
+      <x:c r="J11" s="88" t="str">
+        <x:v>7abd640；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K11" s="88" t="str">
+        <x:v>生产原库安装和目标 Mac 未由临时副本证明</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="84" customHeight="1">
+      <x:c r="A12" s="87" t="str">
+        <x:v>VER-007</x:v>
+      </x:c>
+      <x:c r="B12" s="87" t="str">
+        <x:v>0.3.5</x:v>
+      </x:c>
+      <x:c r="C12" s="87" t="str">
+        <x:v>自动安装机制</x:v>
+      </x:c>
+      <x:c r="D12" s="87" t="str">
+        <x:v>下载后 helper 自动退出、替换、启动及回滚基础</x:v>
+      </x:c>
+      <x:c r="E12" s="87" t="str">
+        <x:v>REQ-022、REQ-023</x:v>
+      </x:c>
+      <x:c r="F12" s="87" t="str">
+        <x:v>DEV-024、DEV-025</x:v>
+      </x:c>
+      <x:c r="G12" s="87" t="str">
+        <x:v>TC-034–036、TC-059、TC-076</x:v>
+      </x:c>
+      <x:c r="H12" s="87" t="str">
+        <x:v>本机未签名 DMG/合成旧版本升级子范围已证</x:v>
+      </x:c>
+      <x:c r="I12" s="87" t="str">
+        <x:v>历史本机候选；真实系统安装待验</x:v>
+      </x:c>
+      <x:c r="J12" s="87" t="str">
+        <x:v>86a4b5b；0.3.5 DMG 摘要见 docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K12" s="87" t="str">
+        <x:v>原 0.3.4 UI 不能直接调用新 helper；安装中取消待验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="84" customHeight="1">
+      <x:c r="A13" s="89" t="str">
+        <x:v>VER-008</x:v>
+      </x:c>
+      <x:c r="B13" s="89" t="str">
+        <x:v>0.3.6</x:v>
+      </x:c>
+      <x:c r="C13" s="89" t="str">
+        <x:v>当前修复与产品打磨</x:v>
+      </x:c>
+      <x:c r="D13" s="89" t="str">
+        <x:v>真实 0.3.5→0.3.6 隔离升级；来源身份隔离、Claude 逐文件队列、v2 迁移、快照续传</x:v>
+      </x:c>
+      <x:c r="E13" s="89" t="str">
+        <x:v>REQ-023、REQ-026、REQ-040–048</x:v>
+      </x:c>
+      <x:c r="F13" s="89" t="str">
+        <x:v>DEV-025、DEV-028、DEV-049–057</x:v>
+      </x:c>
+      <x:c r="G13" s="89" t="str">
+        <x:v>TC-040、TC-076–094</x:v>
+      </x:c>
+      <x:c r="H13" s="89" t="str">
+        <x:v>508851a 源码门禁 94 入口/97 单元/43 Electron；未签名目录包已构建</x:v>
+      </x:c>
+      <x:c r="I13" s="89" t="str">
+        <x:v>验证中；打包日期用例当前失败</x:v>
+      </x:c>
+      <x:c r="J13" s="89" t="str">
+        <x:v>app.asar SHA-256 8a687bf6…；打包全量 42/43；同用例重复 3/5，exit 1；REQ-041/TC-079 当前反例失败；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K13" s="89" t="str">
+        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装中取消、签名/目标 Mac 待验</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="84" customHeight="1">
+      <x:c r="A14" s="90" t="str">
+        <x:v>VER-009</x:v>
+      </x:c>
+      <x:c r="B14" s="90" t="str">
+        <x:v>待定</x:v>
+      </x:c>
+      <x:c r="C14" s="90" t="str">
+        <x:v>下一轮，尚未承诺版号/日期</x:v>
+      </x:c>
+      <x:c r="D14" s="90" t="str">
+        <x:v>修复打包日期报表不稳定；补真实受控归属、生产迁移、目标 Mac 和发布证据</x:v>
+      </x:c>
+      <x:c r="E14" s="90" t="str">
+        <x:v>REQ-023、REQ-041、REQ-045、REQ-048</x:v>
+      </x:c>
+      <x:c r="F14" s="90" t="str">
+        <x:v>DEV-025、DEV-050、DEV-054、DEV-057</x:v>
+      </x:c>
+      <x:c r="G14" s="90" t="str">
+        <x:v>TC-021、TC-028、TC-072、TC-076、TC-079、TC-086、TC-092–094</x:v>
+      </x:c>
+      <x:c r="H14" s="90" t="str">
+        <x:v>已确认日期缺陷；其余仅剩余事项整理，未形成新候选</x:v>
+      </x:c>
+      <x:c r="I14" s="90" t="str">
+        <x:v>规划中；范围/版号待决定</x:v>
+      </x:c>
+      <x:c r="J14" s="90" t="str">
+        <x:v>2026-10-04 TC-079 打包反例 3/5；docs/validation.md</x:v>
+      </x:c>
+      <x:c r="K14" s="90" t="str">
+        <x:v>先修日期回退并复跑 TC-079 单编号/TC-021 回归及打包全量；不预设完成日期</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K1"/>
+    <x:mergeCell ref="A2:K3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: keep current iteration scope in version plan
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1cb780518bc24605"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R50d39b0bfc5b4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R369da6f6681243d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf3fdea548cc84f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R953e0762189c40fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R58fdbd4662fe4cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R62c31ef0d5284048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R5ec83e17dc4c47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R9059ea4d811d491e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R0032437a21ea4d1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="37">
+  <x:fills count="38">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -256,6 +256,11 @@
         <x:fgColor rgb="FFE9F3FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF0F3F6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -286,7 +291,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="91">
+  <x:cellXfs count="95">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -524,6 +529,16 @@
     <x:xf numFmtId="0" fontId="9" fillId="36" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -753,7 +768,8 @@
       <x:c r="A3" s="4" t="str">
         <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
 当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。
-2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。</x:v>
+2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。
+版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -10254,7 +10270,7 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="77" t="str">
-        <x:v>截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。历史本机候选不等于公开发布；“待定”不承诺版本号或日期。进度按已取得证据填写，未完成项不能由源码门禁自动转为版本完成。</x:v>
+        <x:v>截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。</x:v>
       </x:c>
       <x:c r="B2" s="77"/>
       <x:c r="C2" s="77"/>
@@ -10595,39 +10611,74 @@
         <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装中取消、签名/目标 Mac 待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="84" customHeight="1">
+    <x:row r="14" ht="99" customHeight="1">
       <x:c r="A14" s="90" t="str">
         <x:v>VER-009</x:v>
       </x:c>
       <x:c r="B14" s="90" t="str">
-        <x:v>待定</x:v>
+        <x:v>待定（当前目标收尾）</x:v>
       </x:c>
       <x:c r="C14" s="90" t="str">
-        <x:v>下一轮，尚未承诺版号/日期</x:v>
+        <x:v>三批打磨及当前发布门槛</x:v>
       </x:c>
       <x:c r="D14" s="90" t="str">
-        <x:v>修复打包日期报表不稳定；补真实受控归属、生产迁移、目标 Mac 和发布证据</x:v>
+        <x:v>修复打包日期回退；补完整覆盖/真零与同比、空状态、真实服务状态、VoiceOver、Claude 外部归属、生产迁移、安装中取消与目标 Mac 发布证据</x:v>
       </x:c>
       <x:c r="E14" s="90" t="str">
-        <x:v>REQ-023、REQ-041、REQ-045、REQ-048</x:v>
+        <x:v>REQ-023、REQ-040–048</x:v>
       </x:c>
       <x:c r="F14" s="90" t="str">
-        <x:v>DEV-025、DEV-050、DEV-054、DEV-057</x:v>
+        <x:v>DEV-025、DEV-049–057</x:v>
       </x:c>
       <x:c r="G14" s="90" t="str">
-        <x:v>TC-021、TC-028、TC-072、TC-076、TC-079、TC-086、TC-092–094</x:v>
+        <x:v>TC-021、TC-028、TC-072、TC-076–094</x:v>
       </x:c>
       <x:c r="H14" s="90" t="str">
-        <x:v>已确认日期缺陷；其余仅剩余事项整理，未形成新候选</x:v>
+        <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>规划中；范围/版号待决定</x:v>
+        <x:v>当前目标收尾中；完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
-        <x:v>2026-10-04 TC-079 打包反例 3/5；docs/validation.md</x:v>
+        <x:v>2026-10-04 TC-079 打包日期反例 3/5；各 TC 的自动通过与未验边界分别见原编号行及 docs/validation.md</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
-        <x:v>先修日期回退并复跑 TC-079 单编号/TC-021 回归及打包全量；不预设完成日期</x:v>
+        <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="84" customHeight="1">
+      <x:c r="A15" s="94" t="str">
+        <x:v>VER-010</x:v>
+      </x:c>
+      <x:c r="B15" s="94" t="str">
+        <x:v>待定（后续方向）</x:v>
+      </x:c>
+      <x:c r="C15" s="94" t="str">
+        <x:v>下一轮候选，尚未立项</x:v>
+      </x:c>
+      <x:c r="D15" s="94" t="str">
+        <x:v>CodexBar 式菜单栏入口与速览；交互和范围待需求决策</x:v>
+      </x:c>
+      <x:c r="E15" s="94" t="str">
+        <x:v>未分配</x:v>
+      </x:c>
+      <x:c r="F15" s="94" t="str">
+        <x:v>未分配</x:v>
+      </x:c>
+      <x:c r="G15" s="94" t="str">
+        <x:v>未分配</x:v>
+      </x:c>
+      <x:c r="H15" s="94" t="str">
+        <x:v>仅记录方向；尚无 REQ/DEV/TC、实现或验收计划</x:v>
+      </x:c>
+      <x:c r="I15" s="94" t="str">
+        <x:v>未排期，不属于当前交付完成项</x:v>
+      </x:c>
+      <x:c r="J15" s="94" t="str">
+        <x:v>用户提出的下一轮方向；需后续按 SOP-001 定义需求与验收</x:v>
+      </x:c>
+      <x:c r="K15" s="94" t="str">
+        <x:v>当前三批打磨及发布门槛先收尾；未来明确范围后再定版本号、任务和用例</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record temporary local release boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R58fdbd4662fe4cf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R62c31ef0d5284048"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R5ec83e17dc4c47a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R9059ea4d811d491e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R0032437a21ea4d1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R839cba28ff294324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R678d1426ef7f4d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R92b009efb9c44c20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rc109652b23fb49c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R86975e53f6414bc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1458,7 +1458,8 @@
         <x:v>签名公证及目标 Mac 验收</x:v>
       </x:c>
       <x:c r="G33" s="12" t="str">
-        <x:v>待验证</x:v>
+        <x:v>待验证
+2026-10-04 当前无正式签名/公证环境及第二台目标 Mac；本机未签名临时测试可继续，本人工项仍待验证，原 REQ 目标保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="38" customHeight="1">
@@ -2496,7 +2497,8 @@
         <x:v>目标 Mac 文件授权手工验收</x:v>
       </x:c>
       <x:c r="G78" s="36" t="str">
-        <x:v>待验证（人工）</x:v>
+        <x:v>待验证（人工）
+2026-10-04 当前无正式签名/公证环境及第二台目标 Mac；本机未签名临时测试可继续，本人工项仍待验证，原 REQ 目标保留。</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="76" customHeight="1">
@@ -3608,7 +3610,8 @@
       <x:c r="H23" s="10" t="str">
         <x:v>docs/design.md §7；docs/development-plan.md 外部分发计划；docs/test-case-acceptance.md TC-028/TC-075；docs/validation.md。2026-10-03：签名脚本与自动预检均未实现，缺有效签名身份及另一台目标 Mac；不得把未签名 0.3.4 DMG 或将来的 TC-075 模拟通过写成外部分发通过。
 2026-10-03 后续：dc37b8b 实现 pack:signed、预检与同候选制品核验脚本，TC-075 一项自动绑定；文档会话独立复跑 1/1、75 编号检查，缺凭据构建前退出码 1 且无 signed 制品。DEV-018 仅部分落地；没有真实签名/公证、票据或目标 Mac 证据，TC-028 仍待验证。见 docs/validation.md。
-2026-10-03 继续：2f43b00 为 TC-075 补四项核验命令与 Developer ID 身份核对共五个模拟失败分支；文档会话独立复跑同一函数 1/1、75 入口和类型检查通过。模拟失败只证明停止发布与清理，真实签名、公证及异机 TC-028 未执行；REQ-018 仍为部分实现。</x:v>
+2026-10-03 继续：2f43b00 为 TC-075 补四项核验命令与 Developer ID 身份核对共五个模拟失败分支；文档会话独立复跑同一函数 1/1、75 入口和类型检查通过。模拟失败只证明停止发布与清理，真实签名、公证及异机 TC-028 未执行；REQ-018 仍为部分实现。
+2026-10-04 当前无正式 Developer ID/公证环境及第二台目标 Mac；本机未签名临时候选可继续测试，REQ-018 的签名/公证/异机交付条件未取消，TC-028 待验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="62" customHeight="1">
@@ -4067,7 +4070,8 @@
         <x:v>TC-060、TC-061、TC-072</x:v>
       </x:c>
       <x:c r="H40" s="36" t="str">
-        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 明确目标 Mac 拒绝→授予→撤销→重扫闭环；原自动模拟结果不代替真实系统证据。</x:v>
+        <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 明确目标 Mac 拒绝→授予→撤销→重扫闭环；原自动模拟结果不代替真实系统证据。
+2026-10-04 当前无第二台目标 Mac；TC-072 拒绝/授予/撤销/重扫人工闭环仍待验证，现阶段本机临时测试不改变 REQ-035 目标。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -7218,10 +7222,11 @@
         <x:v>签名和公证通过，目标设备安装/启动/采集通过。</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
-        <x:v>待验证</x:v>
+        <x:v>待验证（正式签名/公证与另一台目标 Mac 环境暂缺）</x:v>
       </x:c>
       <x:c r="I33" s="10" t="str">
-        <x:v>历史：实施前无签名、公证和目标 Mac 证据。2026-10-03 dc37b8b 已新增 pack:signed，但当前 Mac 无有效签名身份/公证凭据；文档会话运行 TC-028 人工清单，退出码 2，未登记 pass。尚无真实签名、公证票据、Gatekeeper 或另一台 Mac 的安装/启动/登录/采集结果；TC-075 自动通过不能替代本项。</x:v>
+        <x:v>历史：实施前无签名、公证和目标 Mac 证据。2026-10-03 dc37b8b 已新增 pack:signed，但当前 Mac 无有效签名身份/公证凭据；文档会话运行 TC-028 人工清单，退出码 2，未登记 pass。尚无真实签名、公证票据、Gatekeeper 或另一台 Mac 的安装/启动/登录/采集结果；TC-075 自动通过不能替代本项。
+2026-10-04 项目沟通确认：当前无可用正式 Developer ID/公证环境，也没有第二台目标 Mac。现阶段仅本机未签名临时候选继续测试；尚未执行新的签名票据/Gatekeeper/异机安装、登录、采集人工验收，不登记 pass。资源具备后按本编号清单补脱敏证据。</x:v>
       </x:c>
       <x:c r="J33" s="27" t="str">
         <x:v>npm run test:case -- TC-028</x:v>
@@ -7230,10 +7235,12 @@
         <x:v>scripts/test-cases.mjs：TC-028 人工清单；已更新为先运行 pack:signed、核对 release/signed 证据，再在另一台目标 Mac 安装与验证；无自动通过断言。</x:v>
       </x:c>
       <x:c r="L33" s="30" t="str">
-        <x:v>人工入口；待验证</x:v>
+        <x:v>人工入口；待验证
+当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。</x:v>
       </x:c>
       <x:c r="M33" s="27" t="str">
-        <x:v>运行 npm run test:case -- TC-028 仅输出人工清单、退出码 2；实际验收需同一签名候选的 App/DMG、脱敏 Developer ID 身份、公证和票据/Gatekeeper 核验、包大小/SHA-256、目标 Mac 版本/架构与安装、启动、登录、采集记录。当前无 pass 证据，不得借用 TC-075 1/1 或 0.3.4 未签名包。</x:v>
+        <x:v>运行 npm run test:case -- TC-028 仅输出人工清单、退出码 2；实际验收需同一签名候选的 App/DMG、脱敏 Developer ID 身份、公证和票据/Gatekeeper 核验、包大小/SHA-256、目标 Mac 版本/架构与安装、启动、登录、采集记录。当前无 pass 证据，不得借用 TC-075 1/1 或 0.3.4 未签名包。
+2026-10-04 资源确认；未运行新增人工验收，状态待验证；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="60" customHeight="1">
@@ -9061,10 +9068,11 @@
         <x:v>拒绝时来源未知且不越权；授予后恢复可观察用量；撤销后重新显示权限不足/未知，不保留伪零；指引与系统设置路径可执行。</x:v>
       </x:c>
       <x:c r="H77" s="37" t="str">
-        <x:v>待验证（人工）</x:v>
+        <x:v>待验证（第二台目标 Mac 暂缺，人工授权闭环未执行）</x:v>
       </x:c>
       <x:c r="I77" s="37" t="str">
-        <x:v>已注册人工清单；截至 2026-10-02 尚无目标 Mac 拒绝、授予、撤销文件访问权限的脱敏证据；不得登记 pass。 2026-10-03 验收口径补充撤销后的重扫与回到未知；当前仍无目标 Mac 证据。</x:v>
+        <x:v>已注册人工清单；截至 2026-10-02 尚无目标 Mac 拒绝、授予、撤销文件访问权限的脱敏证据；不得登记 pass。 2026-10-03 验收口径补充撤销后的重扫与回到未知；当前仍无目标 Mac 证据。
+2026-10-04 项目沟通确认：目前没有第二台目标 Mac。本机未签名候选可继续隔离测试，但不能替代目标 Mac 独立账户上的拒绝→授予→撤销权限及逐步重扫；本轮无新人工执行或 pass 证据。</x:v>
       </x:c>
       <x:c r="J77" s="37" t="str">
         <x:v>npm run test:case -- TC-072</x:v>
@@ -9073,10 +9081,12 @@
         <x:v>scripts/test-cases.mjs：TC-072 人工清单（非自动断言）</x:v>
       </x:c>
       <x:c r="L77" s="37" t="str">
-        <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。；新增目标还须实测撤销后的状态/重扫。</x:v>
+        <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。；新增目标还须实测撤销后的状态/重扫。
+当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。</x:v>
       </x:c>
       <x:c r="M77" s="37" t="str">
-        <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。</x:v>
+        <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。
+2026-10-04 资源确认；未运行新增人工验收，状态待验证；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="152" customHeight="1">
@@ -10576,7 +10586,7 @@
         <x:v>原 0.3.4 UI 不能直接调用新 helper；安装中取消待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="84" customHeight="1">
+    <x:row r="13" ht="120" customHeight="1">
       <x:c r="A13" s="89" t="str">
         <x:v>VER-008</x:v>
       </x:c>
@@ -10605,13 +10615,15 @@
         <x:v>验证中；打包日期用例当前失败</x:v>
       </x:c>
       <x:c r="J13" s="89" t="str">
-        <x:v>app.asar SHA-256 8a687bf6…；打包全量 42/43；同用例重复 3/5，exit 1；REQ-041/TC-079 当前反例失败；docs/validation.md</x:v>
+        <x:v>app.asar SHA-256 8a687bf6…；打包全量 42/43；同用例重复 3/5，exit 1；REQ-041/TC-079 当前反例失败；docs/validation.md
+当前资源确认：没有正式 Developer ID/公证环境及第二台目标 Mac；本机未签名候选继续测试，不增加 TC-028/072 通过证据。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
-        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装中取消、签名/目标 Mac 待验</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="99" customHeight="1">
+        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装中取消、签名/目标 Mac 待验
+临时可用范围限当前 Mac；签名、公证、异机与目标 Mac 授权待具备资源后分别按 TC-028/072 验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" customHeight="1">
       <x:c r="A14" s="90" t="str">
         <x:v>VER-009</x:v>
       </x:c>
@@ -10637,13 +10649,15 @@
         <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>当前目标收尾中；完整交付门槛未通过</x:v>
+        <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
-        <x:v>2026-10-04 TC-079 打包日期反例 3/5；各 TC 的自动通过与未验边界分别见原编号行及 docs/validation.md</x:v>
+        <x:v>2026-10-04 TC-079 打包日期反例 3/5；各 TC 的自动通过与未验边界分别见原编号行及 docs/validation.md
+2026-10-04 项目沟通确认：暂缺正式 Developer ID/公证环境和第二台目标 Mac，TC-028/072 无新增执行证据。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
-        <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据</x:v>
+        <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
+当前只要求本机未签名临时候选可用；资源具备后仍须完成 TC-028/072，REQ-018/035 目标未删除。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: update install scope and version evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R839cba28ff294324"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R678d1426ef7f4d9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R92b009efb9c44c20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rc109652b23fb49c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R86975e53f6414bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rb3fffa3542574da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R44275fddba9e4b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rda9a2eaf0ef94721"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf440f08e8ab54d9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R72afee60c6824b35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2595,7 +2595,9 @@
 2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。
 2026-10-04 安装中取消设计已决：独立控制窗口+helper 阶段回执、替换后回滚和 userData 隔离健康探测，TC-076 分阶段打包 UI 真取消待实现/验收；既有成功/故障证据不变。
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
-508851a：历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
+508851a：历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过；详情见测试用例 I/L/M 列与 docs/validation.md。
+2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 新包隔离升级及两层五故障回退动态子范围通过；完整系统/生产验收待补；历史取消设计保留备选。
+当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2 TC-076 真实双 DMG 脚本 exit 0；范围与限制见测试用例 I/M 列。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -3733,14 +3735,14 @@
         <x:v>应用内自动安装升级</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。取消或挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
-2026-10-04 新增安装中取消：下载/校验前可立即取消；旧版退出后挂载/暂存于安全检查点取消；旧版已移动至成功耐久提交前取消必须完整恢复旧版和未改真实 userData；提交后拒绝迟到取消。控制窗口持续可见并给权威回执，崩溃/断电边界详见 docs/install-cancellation-decision.md。</x:v>
+        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
+2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：未点击更新前可放弃；点击后下载并校验，通过后自动退出旧版、原位替换和启动新版；开始执行替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>部分验证；真实 0.3.5→0.3.6 隔离升级、installer 模块与打包 helper 五故障回退/重试子范围独立通过；真实系统目录/满盘/崩溃/安装中取消/签名异机待验</x:v>
+        <x:v>部分验证；当前新 DMG 真实旧/新隔离升级、installer/打包 helper 各五故障回退与重试通过；系统目录、真实故障和生产数据仍待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3755,7 +3757,9 @@
 2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。
 2026-10-04 1961de3：TC-076 新增隔离打包 helper 五故障。文档会话真实旧/新 DMG 固定哈希完整命令 exit 0；旧 UI 触发 helper，mount/space/replace/launch/health 每次回退旧版、受信登录/1280 Token/清理，最后重试新版。注入为专用临时目录预加载，非真实满盘/崩溃或系统安装。
 2026-10-04 取消设计决议：当前没有旧 App 退出后的可见取消入口，健康标记前新版会打开真实 userData。独立控制进程、helper 阶段 journal/取消能力、隔离健康探测与结果持久反馈待实现；1961de3 五故障通过不代证取消。
-2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
+2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 当前新包取干净 main 9af351a，SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；旧 d99d7af9 包的 TC-076 故障证据不外推。
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -5154,7 +5158,7 @@
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>部分实现/验证；真实 DMG 隔离升级、installer 模块及打包 helper 五故障回退/重试通过；真实系统目录、满盘/崩溃、安装中取消待验</x:v>
+        <x:v>部分实现/验证；当前简化范围为安装前可放弃、安装开始后不可取消、失败自动回退；新包隔离升级及双路径五故障回退通过，真实系统/生产场景待验</x:v>
       </x:c>
       <x:c r="G30" s="70" t="str">
         <x:v>当前 1e70412：文档会话构建 0.3.6 x64 目录包并以真实旧/新 DMG、固定哈希独立复跑 TC-076，exit 0；TC-036 2/2 合成单元回归通过。
@@ -5163,7 +5167,9 @@
 2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。
 2026-10-04 1961de3：TC-076 三段集成绑定中的新增 scripts/verify-packaged-helper-faults.mjs 在隔离临时目录经旧 UI 触发真实打包 helper；文档会话完整命令 exit 0、TC-036 两项单元 exit 0。未测真实满盘/进程崩溃/系统安装/签名公证异机。
 2026-10-04 下一任务：管理员授权的一次性取消能力及独立更新控制窗口；下载 AbortController、helper 阶段/回执/安全检查点、替换后回滚、隔离健康探测防真实 userData 迁移、终态可重启读取和中断恢复。成功提交后取消 too_late；系统级断电自动恢复若承诺须另有 bundle 外恢复入口。
-2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
+2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
+2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 前文“独立窗口/阶段取消”为旧计划；开发工作树未提交实验不算候选。当前新包 SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，包校验通过，安装功能新证据待补。
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -9238,26 +9244,26 @@
         <x:v>打包应用/本机隔离</x:v>
       </x:c>
       <x:c r="F81" s="52" t="str">
-        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。分别注入取消、磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
+        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。安装前未确认时放弃，另注入磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
 2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。
-2026-10-04 待新增打包版真点击取消：下载中、校验交接前、旧版退出后挂载/暂存、旧版移动后、健康探测中；另造阻塞步骤等待、重复点击、viewer/伪造请求、成功前后竞态及隔离强杀后的 journal 恢复。
-2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
+2026-10-04 当前简化操作：安装前放弃不得触发替换；一旦开始执行替换/安装，不提供取消动作；分别注入挂载、空间、替换、启动与健康故障，核自动恢复旧版/数据及重试。下载阶段取消非本轮必需，不能无代码证据写成通过。</x:v>
       </x:c>
       <x:c r="G81" s="52" t="str">
         <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。
 2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。
-仅 helper 完成回执后称已取消；前段保留旧 App，替换后恢复旧版与受信登录/1280 Token，真实 userData 不受候选探测写入；无挂载/备份/下载残留。成功提交后拒绝迟到取消且新版保持；恢复失败保存备份并提示人工处理。
-2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。</x:v>
+2026-10-04 当前预期：安装前不确认则旧版保持；安装开始后不可主动取消，正常成功自动替换/重启；故障自动回退旧版、保留用户数据与受信状态并清理残留。此口径新包隔离升级和故障回退子范围后续已动态验证，系统目录及生产数据仍待验。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过</x:v>
+        <x:v>部分验证：新 DMG 真实旧/新隔离升级、installer/打包 helper 各五故障自动回退与重试通过；安装前放弃、真实系统目录/生产数据和真实故障仍待验</x:v>
       </x:c>
       <x:c r="I81" s="68" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
 2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
 86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。
 2026-10-04 / 80e7f10→0eac84b：80e7f10 文档独立首次全命令：成功段、只读初始启动、五故障回退输出通过；末次重试读取已被 UI 消费的一次性 last-install.json 得 undefined，exit 1。0eac84b 修脚本后同 DMG 再跑，全命令 exit 0；旧包 142557541 字节 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 142591838 字节 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c，两包 verify VALID。旧 27aae018… 只属历史候选。
-508851a：TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。</x:v>
+508851a：TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。
+2026-10-04 用户决议：开始执行应用替换/安装后不可取消，安装前可放弃，失败自动恢复；原五阶段取消要求撤出本轮。新候选从干净 main 9af351a 构建，未签名 mac x64 DMG SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；需求会话报告 pack:dmg exit 0，文档会话独立重算 SHA-256 与 hdiutil verify VALID。新包成功/故障隔离动态子范围后续已测，详见本列最新证据，旧 d99d7af9 包证据不外推。
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="str">
         <x:v>TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c npm run test:case -- TC-076</x:v>
@@ -9273,14 +9279,17 @@
 2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。
 2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。
 2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。
-本次并未复跑真实旧/新 DMG 与固定 SHA 的故障链；历史 1961de3 证据另列。系统安装、签名公证及安装中取消未验。</x:v>
+本次并未复跑真实旧/新 DMG 与固定 SHA 的故障链；历史 1961de3 证据另列。系统安装、签名公证及安装中取消未验。
+2026-10-04 用户已撤出安装中取消交付要求；前文独立控制窗口/五阶段点击取消及“取消未验”属于历史阶段，不再构成当前简化目标的待验项。新包仍须按简化范围重新核安装成功、自动失败回退和数据连续性。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
 2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。
 1961de3；文档会话独立 TC-076 完整命令 exit 0，真实旧/新 DMG SHA-256 分别 ae1b8e80…、d99d7af9…，两包 hdiutil verify VALID；打包 helper mount/space/replace/launch/health 各回退、受信登录/1280 Token/清理及最后重试均通过；TC-036 两单元 exit 0。
 1961de3 文档会话独立 test:gate 类型检查、94 入口、77/77 单元、39/39 Electron exit 0；未另跑打包版全量。
-508851a；macOS 15.7.4 x86_64、Node v24.15.0；TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。
+后续新包 TC-076 隔离动态子范围已由需求会话执行通过，详见 I 列最新证据；整项仍部分验证。
+新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 exit 0，打包 Electron 43/43，test:gate 97/97 单元+43/43 Electron；均由需求会话报告，文档会话未独立复跑。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">
@@ -9435,7 +9444,8 @@
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。
 47b03d5 文档会话独立运行 TC-079：单元与 Electron 均通过、退出码 0；单元增加 v1→v2 冲突、扫描后旧 snapshotId 拒绝和刷新小计 99→104；完整 gate 82/57/22 通过。
-2026-10-04 固定代码 508851a、app.asar SHA-256 8a687bf6…：开发会话在文档工作树运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1。文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05、结束 2026-01-02，报日期范围无效；新增 TC-079 断言尚未实现，当前失败不能写通过。</x:v>
+2026-10-04 固定代码 508851a、app.asar SHA-256 8a687bf6…：开发会话在文档工作树运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1。文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05、结束 2026-01-02，报日期范围无效；新增 TC-079 断言尚未实现，当前失败不能写通过。
+2026-10-04 新 DMG 8773dd38… 已构建/校验，但未针对双日期快速输入反例单独复测；508851a 目录包 2/5 失败仍是已知风险，不能以构建或旧包结果改成通过。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
         <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
@@ -10586,7 +10596,7 @@
         <x:v>原 0.3.4 UI 不能直接调用新 helper；安装中取消待验</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="120" customHeight="1">
+    <x:row r="13" ht="142.5" customHeight="1">
       <x:c r="A13" s="89" t="str">
         <x:v>VER-008</x:v>
       </x:c>
@@ -10609,21 +10619,24 @@
         <x:v>TC-040、TC-076–094</x:v>
       </x:c>
       <x:c r="H13" s="89" t="str">
-        <x:v>508851a 源码门禁 94 入口/97 单元/43 Electron；未签名目录包已构建</x:v>
+        <x:v>0.3.6 本机未签名候选：打包与完整性通过；同包源码门禁、TC-076 真实双 DMG 隔离子范围及打包 Electron 43/43 通过；TC-079 日期反例、系统/生产/外部验收待补</x:v>
       </x:c>
       <x:c r="I13" s="89" t="str">
-        <x:v>验证中；打包日期用例当前失败</x:v>
+        <x:v>本机临时候选部分验证；主要自动子范围通过，TC-079 已知回归及完整验收未通过</x:v>
       </x:c>
       <x:c r="J13" s="89" t="str">
         <x:v>app.asar SHA-256 8a687bf6…；打包全量 42/43；同用例重复 3/5，exit 1；REQ-041/TC-079 当前反例失败；docs/validation.md
-当前资源确认：没有正式 Developer ID/公证环境及第二台目标 Mac；本机未签名候选继续测试，不增加 TC-028/072 通过证据。</x:v>
+当前资源确认：没有正式 Developer ID/公证环境及第二台目标 Mac；本机未签名候选继续测试，不增加 TC-028/072 通过证据。
+2026-10-04 干净 main 9af351a 新 DMG SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，hdiutil verify VALID；历史 d99d7af9 故障证据不外推，新包 TC-076 隔离子范围后续通过；TC-079 日期反例待复测。
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
-        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装中取消、签名/目标 Mac 待验
-临时可用范围限当前 Mac；签名、公证、异机与目标 Mac 授权待具备资源后分别按 TC-028/072 验收。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="120" customHeight="1">
+        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装失败自动回退、签名/目标 Mac 待验
+临时可用范围限当前 Mac；签名、公证、异机与目标 Mac 授权待具备资源后分别按 TC-028/072 验收。
+当前安装前可放弃，开始执行替换/安装后不可取消；新包成功/故障回退隔离子范围已测；TC-079 日期反例仍需单独修复复测。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="142.5" customHeight="1">
       <x:c r="A14" s="90" t="str">
         <x:v>VER-009</x:v>
       </x:c>
@@ -10634,7 +10647,7 @@
         <x:v>三批打磨及当前发布门槛</x:v>
       </x:c>
       <x:c r="D14" s="90" t="str">
-        <x:v>修复打包日期回退；补完整覆盖/真零与同比、空状态、真实服务状态、VoiceOver、Claude 外部归属、生产迁移、安装中取消与目标 Mac 发布证据</x:v>
+        <x:v>修复打包日期回退；补完整覆盖/真零与同比、空状态、真实服务状态、VoiceOver、Claude 外部归属、生产迁移、安装开始后不可取消、失败自动回退和目标 Mac 发布证据</x:v>
       </x:c>
       <x:c r="E14" s="90" t="str">
         <x:v>REQ-023、REQ-040–048</x:v>
@@ -10646,18 +10659,21 @@
         <x:v>TC-021、TC-028、TC-072、TC-076–094</x:v>
       </x:c>
       <x:c r="H14" s="90" t="str">
-        <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺</x:v>
+        <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺
+当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
         <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
         <x:v>2026-10-04 TC-079 打包日期反例 3/5；各 TC 的自动通过与未验边界分别见原编号行及 docs/validation.md
-2026-10-04 项目沟通确认：暂缺正式 Developer ID/公证环境和第二台目标 Mac，TC-028/072 无新增执行证据。</x:v>
+2026-10-04 项目沟通确认：暂缺正式 Developer ID/公证环境和第二台目标 Mac，TC-028/072 无新增执行证据。
+新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 真实双 DMG 隔离脚本 exit 0，打包 Electron 43/43；TC-079 重复失败记录继续有效，不宣称版本完成。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
-当前只要求本机未签名临时候选可用；资源具备后仍须完成 TC-028/072，REQ-018/035 目标未删除。</x:v>
+当前只要求本机未签名临时候选可用；资源具备后仍须完成 TC-028/072，REQ-018/035 目标未删除。
+REQ-023/TC-076 按用户决议收敛：安装前可放弃、安装开始后不可取消、失败自动恢复；独立取消控制窗口不属本轮。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: correct TC-079 packaged date failure attribution
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rb3fffa3542574da3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R44275fddba9e4b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rda9a2eaf0ef94721"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rf440f08e8ab54d9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R72afee60c6824b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3874106da2874b86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R655cfcbea0de4550"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc033b6eb87564067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5561639d72a6499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Raae18bcbf9ab4a61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2671,7 +2671,8 @@
       </x:c>
       <x:c r="G85" s="55" t="str">
         <x:v>78b3a3b 已注册；TC-079 单元 1/1 + Electron 1/1 通过；仅 REQ-041 同事实集合查询/导出子范围
-2026-10-04 REQ-041→DEV-050→TC-079 新增双日期连续快速修改/最终组合/无错误/CSV 同屏验收；当前打包共用路径重复 3/5，2 次失败，待修/复验。</x:v>
+2026-10-04 REQ-041→DEV-050→TC-079 新增双日期连续快速修改/最终组合/无错误/CSV 同屏验收；当前打包共用路径重复 3/5，2 次失败，待修/复验。
+2026-10-04 根因修订：共用打包测试跨页模糊标签误选来源页日期；原生报表控件不改。旧 2/5、新报告 1/5 失败记录保留；专属真实查询/CSV 和无重试打包复验待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="85" customHeight="1">
@@ -4227,13 +4228,14 @@
       </x:c>
       <x:c r="C46" s="58" t="str">
         <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。
-2026-10-04 打包缺陷验收补充：在用量报表连续快速修改开始和结束日期，两输入值均须保持最终选择；查询只使用最终起止日期组合，无倒置范围错误。当前屏显结果与 CSV 必须使用同一授权筛选、时区和快照，期间旧请求不得覆写新组合。</x:v>
+2026-10-04 打包缺陷验收补充：在用量报表连续快速修改开始和结束日期，两输入值均须保持最终选择；查询只使用最终起止日期组合，无倒置范围错误。当前屏显结果与 CSV 必须使用同一授权筛选、时区和快照，期间旧请求不得覆写新组合。
+2026-10-04 当前澄清：保持原生日期输入与现有范围校验；最终报表查询及页面、明细、CSV 同授权筛选/时区/snapshotId 的原要求不变。打包异常先按跨页模糊测试定位修复，不增设文本输入或双日期提交产品需求。</x:v>
       </x:c>
       <x:c r="D46" s="58" t="str">
         <x:v>下一轮产品打磨（第一批 B 阶段实现）</x:v>
       </x:c>
       <x:c r="E46" s="58" t="str">
-        <x:v>原异步/快照子范围通过；0.3.6 打包日期双字段快速修改反例当前失败，待修/复验</x:v>
+        <x:v>异步/快照子范围已通过；打包共用测试日期定位错误待修并复验，产品日期控件异常未证实</x:v>
       </x:c>
       <x:c r="F46" s="58" t="str">
         <x:v>DEV-050</x:v>
@@ -4245,7 +4247,8 @@
         <x:v>承接 REQ-013/014；不改变 CSV 原值、列结构、公式转义及主进程授权。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
 2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。
 47b03d5：TC-079 追加 v1→冲突 v2、扫描入库后旧 snapshotId 拒绝及刷新小计 99→104；文档会话单元+Electron 与 gate 独立通过。
-508851a 未签名目录包共用报表 E2E 重复 5 次中 2 次开始日期回退；验收补充先于开发修改。旧 TC-079 源码态通过不覆盖打包连续修改。</x:v>
+508851a 未签名目录包共用报表 E2E 重复 5 次中 2 次开始日期回退；验收补充先于开发修改。旧 TC-079 源码态通过不覆盖打包连续修改。
+2026-10-04 复核修订：需求/开发会话报告，新目录包 5 次无重试执行仍 1 次失败；失败时操作快照在“工作台 / 数据来源”。共用 app.spec.ts 在切到报表后立即用 page.getByLabel("开始日期")，它会模糊匹配来源页“最近记录开始日期”；当前代码中两个标签并存，且该测试未等待 .report-page 可见。此前固定 508851a 包 3/5 通过、2/5 失败的错误页面显示报表日期倒置，但该末态不足以证明报表控件自行回退。定位结论为测试跨页误选，保留历史失败次数，产品日期控件缺陷待有效测试判定；不要求改为文本输入。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="150" customHeight="1">
@@ -5751,14 +5754,15 @@
         <x:v>src/main/report.ts、index.ts；src/preload/index.ts；src/renderer/report.tsx；src/shared/types.ts；tests/report-snapshot.test.ts、tests/e2e/report-snapshot.spec.ts；scripts/test-cases.mjs、run-test-case.mjs</x:v>
       </x:c>
       <x:c r="F55" s="58" t="str">
-        <x:v>既有异步快照子范围已实现；0.3.6 打包日期双字段反例当前失败，待修/复验</x:v>
+        <x:v>异步/快照子范围已实现；打包共用 E2E 先修跨页日期定位并复验，产品日期控件不改</x:v>
       </x:c>
       <x:c r="G55" s="58" t="str">
         <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 需求复核补充：导出须绑定数据库 revision/快照身份；TC-079 须在查询完成后再次扫描，再核屏显与 CSV 逐事实集合。
 78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。
 47b03d5：TC-079 原单元新增冲突 v2 快照身份回归：新增遥测使旧 ID 拒绝、刷新小计 99，继续新增事实又拒绝，刷新小计 104；单编号 unit/Electron 与完整门禁独立通过。
-2026-10-04 新修复目标：排查日期输入状态/异步请求竞态，确保连续快速填写两端后值保持、只查询最终组合、无日期范围错误，CSV 与屏显同快照；TC-079 加打包反例，TC-021 管理员主流程回归。</x:v>
+2026-10-04 新修复目标：排查日期输入状态/异步请求竞态，确保连续快速填写两端后值保持、只查询最终组合、无日期范围错误，CSV 与屏显同快照；TC-079 加打包反例，TC-021 管理员主流程回归。
+2026-10-04 当前最小修复：保留原生日期控件，先等待 .report-page 可见，再在该容器内以 getByLabel("开始日期",{exact:true})、结束日期精确定位；TC-079 专属绑定核真实授权查询参数、页面/明细与 CSV 同一已应用查询及 snapshotId。禁止用失败重试掩盖共用打包反例。既有“排查输入状态”段落为定位前计划。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="155" customHeight="1">
@@ -9430,22 +9434,26 @@
       <x:c r="F84" s="55" t="str">
         <x:v>独立库快速切换 A/B 筛选并延迟 A 返回；B 查询完成后再扫描入库，分别在 B 加载、完成及新扫描后导出。
 已注册单元以专用临时 SQLite 在查询后插入同筛选事实并重算快照；Electron 以延迟 IPC 模拟 A→B 快速切换与过期导出。
-0.3.6 打包补例：进入管理员用量报表，连续快速填写开始 2026-01-01、结束 2026-01-02；重复运行至少 5 次并检查字段最终值、查询参数/页面数字和 CSV；再造两端不同快速变化及旧请求晚返回。关联 TC-021 管理员主流程回归。</x:v>
+0.3.6 打包补例：进入管理员用量报表，连续快速填写开始 2026-01-01、结束 2026-01-02；重复运行至少 5 次并检查字段最终值、查询参数/页面数字和 CSV；再造两端不同快速变化及旧请求晚返回。关联 TC-021 管理员主流程回归。
+2026-10-04 修订步骤：真实打包 App 从数据来源页点击用量报表后等待 .report-page 可见，并在该容器内精确按“开始日期”“结束日期”标签输入 2026-01-01/02；不用模糊全页标签命中“最近记录开始日期”。用独立 TC-079 断言真实查询参数、页面数字/明细和 CSV 均为该已应用授权查询及同一 snapshotId；保留共用 app.spec.ts --repeat-each=5 --retries=0，无失败重试；同时复验 TC-021 与打包全量。</x:v>
       </x:c>
       <x:c r="G84" s="55" t="str">
         <x:v>旧响应不覆盖 B；加载时导出禁用或等待 B；页面和 CSV 的授权查询键、数据库 revision/快照身份及逐事实集合一致；新扫描不能造成旧页面/新 CSV 错配。
 授权查询和选中事实的 SHA-256 快照 ID；事实变化后旧 ID 拒绝并提示刷新，刷新后 12→111 Token；不同筛选/角色的旧 ID 拒绝。Electron 最终只显示 B，加载中禁用导出，IPC 携带 B 筛选及 B ID。
-两个日期输入最终值稳定为用户最后选择；查询只取新的有效日期组合、无“日期范围无效”；屏显指标/明细和 CSV 使用同一授权查询与事实快照；旧响应不能回退任何日期或结果。</x:v>
+两个日期输入最终值稳定为用户最后选择；查询只取新的有效日期组合、无“日期范围无效”；屏显指标/明细和 CSV 使用同一授权查询与事实快照；旧响应不能回退任何日期或结果。
+2026-10-04 修订预期：切页完成前不输入，两个日期只写报表控件；最终有效组合产生真实查询，旧响应不得覆盖，页面/明细/CSV 同授权范围、时区和 snapshotId。五次无重试共用打包路径与专属 TC-079 均通过后，才更新本子范围状态；末态错误页不能单独证明产品控件回退。</x:v>
       </x:c>
       <x:c r="H84" s="55" t="str">
-        <x:v>既有源码态 v1/v2 快照子范围通过；0.3.6 打包双日期快速修改新反例当前失败，待修/复验</x:v>
+        <x:v>既有源码态快照子范围通过；打包共用 E2E 日期定位错误待修复验，产品日期控件缺陷未证实</x:v>
       </x:c>
       <x:c r="I84" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 2026-10-03 文档会话独立执行 npm run test:case -- TC-079：tests/report-snapshot.test.ts 1/1、tests/e2e/report-snapshot.spec.ts 1/1，退出码 0；TC-029 1/1、TC-023 1/1 退出码 0。完整 test:gate 独立复跑 typecheck、77 已注册入口检查、53/53 单元、19/19 Electron，退出码 0。
 47b03d5 文档会话独立运行 TC-079：单元与 Electron 均通过、退出码 0；单元增加 v1→v2 冲突、扫描后旧 snapshotId 拒绝和刷新小计 99→104；完整 gate 82/57/22 通过。
 2026-10-04 固定代码 508851a、app.asar SHA-256 8a687bf6…：开发会话在文档工作树运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1。文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05、结束 2026-01-02，报日期范围无效；新增 TC-079 断言尚未实现，当前失败不能写通过。
-2026-10-04 新 DMG 8773dd38… 已构建/校验，但未针对双日期快速输入反例单独复测；508851a 目录包 2/5 失败仍是已知风险，不能以构建或旧包结果改成通过。</x:v>
+2026-10-04 新 DMG 8773dd38… 已构建/校验，但未针对双日期快速输入反例单独复测；508851a 目录包 2/5 失败仍是已知风险，不能以构建或旧包结果改成通过。
+2026-10-04 复核修订：需求/开发会话报告，新目录包 5 次无重试执行仍 1 次失败；失败时操作快照在“工作台 / 数据来源”。共用 app.spec.ts 在切到报表后立即用 page.getByLabel("开始日期")，它会模糊匹配来源页“最近记录开始日期”；当前代码中两个标签并存，且该测试未等待 .report-page 可见。此前固定 508851a 包 3/5 通过、2/5 失败的错误页面显示报表日期倒置，但该末态不足以证明报表控件自行回退。定位结论为测试跨页误选，保留历史失败次数，产品日期控件缺陷待有效测试判定；不要求改为文本输入。
+2026-10-04 开发会话随后报告已撤回日期产品改动并仅修共用测试为报表容器内 exact 标签：源码管理员流程重复 20 次 exit 0，重构目录包同用例重复 5 次 exit 0，TC-079 单编号 exit 0。此时尚无固定提交/制品 SHA 与完整门禁、打包全量结果；文档会话未独立复跑，不把暂存通过登记为整项通过。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
         <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
@@ -9455,12 +9463,15 @@
       </x:c>
       <x:c r="L84" s="55" t="str">
         <x:v>当前已在单元测试覆盖 v1 与冲突 v2 的扫描后旧 snapshotId 拒绝；Electron 仍侧重快速筛选切换与导出等待当前快照。snapshotId 是授权查询+事实集合身份，不是全库 revision；REQ-040 历史覆盖及目标安装环境仍未由此证明。
-本次打包共用 app.spec.ts 只复现异常，尚未有专属 TC-079 双日期快速修改绑定；失败根因未定，应用状态与测试时序需区分。</x:v>
+本次打包共用 app.spec.ts 只复现异常，尚未有专属 TC-079 双日期快速修改绑定；失败根因未定，应用状态与测试时序需区分。
+当前根因修订覆盖前文“日期字段回退/根因未定”的推断：共用脚本全页模糊标签在报表页出现前可误选来源页控件。专属 TC-079 的真实查询/CSV 断言及修正后打包复验尚无通过证据。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
         <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。
 47b03d5；macOS 本机隔离合成库；TC-079 单元/Electron 各 1/1、退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
-0.3.6 打包日期新验收当前失败 2/5；修复后必须单编号运行 TC-079、TC-021 回归，再重复打包用例并跑打包全量。</x:v>
+0.3.6 打包日期新验收当前失败 2/5；修复后必须单编号运行 TC-079、TC-021 回归，再重复打包用例并跑打包全量。
+待固定测试修复提交与候选包 SHA 后，记录 TC-079、TC-021、无重试真实打包重复五次及打包全量的命令/退出码；本轮只修订追溯，不改测试结果为通过。
+开发会话工作树初步结果：源码管理员流程 20/20、重构目录包共用报表 5/5、TC-079 单编号 exit 0；固定提交、包 SHA、完整门禁与打包全量待补。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="185" customHeight="1">
@@ -10619,21 +10630,16 @@
         <x:v>TC-040、TC-076–094</x:v>
       </x:c>
       <x:c r="H13" s="89" t="str">
-        <x:v>0.3.6 本机未签名候选：打包与完整性通过；同包源码门禁、TC-076 真实双 DMG 隔离子范围及打包 Electron 43/43 通过；TC-079 日期反例、系统/生产/外部验收待补</x:v>
+        <x:v>0.3.6 本机未签名候选：打包与完整性通过；同包门禁、TC-076 隔离子范围及打包 Electron 43/43 通过；TC-079 共用测试定位修复与专属复验、系统/生产/外部验收待补</x:v>
       </x:c>
       <x:c r="I13" s="89" t="str">
-        <x:v>本机临时候选部分验证；主要自动子范围通过，TC-079 已知回归及完整验收未通过</x:v>
+        <x:v>本机临时候选部分验证；TC-079 打包共用测试定位待修复验，完整验收未通过</x:v>
       </x:c>
       <x:c r="J13" s="89" t="str">
-        <x:v>app.asar SHA-256 8a687bf6…；打包全量 42/43；同用例重复 3/5，exit 1；REQ-041/TC-079 当前反例失败；docs/validation.md
-当前资源确认：没有正式 Developer ID/公证环境及第二台目标 Mac；本机未签名候选继续测试，不增加 TC-028/072 通过证据。
-2026-10-04 干净 main 9af351a 新 DMG SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，hdiutil verify VALID；历史 d99d7af9 故障证据不外推，新包 TC-076 隔离子范围后续通过；TC-079 日期反例待复测。
-2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
+        <x:v>新 DMG 8773dd38…：门禁 94/97/43、打包 43/43、TC-076 隔离通过。TC-079 旧包 3/5，新包需求会话报告 4/5；脚本跨页模糊定位，产品缺陷未证。TC-028/072 待环境。详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
-        <x:v>修复日期双字段回退并复跑 TC-079/021；外部受控登记、生产迁移、安装失败自动回退、签名/目标 Mac 待验
-临时可用范围限当前 Mac；签名、公证、异机与目标 Mac 授权待具备资源后分别按 TC-028/072 验收。
-当前安装前可放弃，开始执行替换/安装后不可取消；新包成功/故障回退隔离子范围已测；TC-079 日期反例仍需单独修复复测。</x:v>
+        <x:v>先修共用 E2E 报表容器/精确标签并增加 TC-079 真实查询与 CSV；复验 TC-021、打包五次无重试及全量。生产迁移、系统安装、TC-028/072 待证。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="142.5" customHeight="1">
@@ -10660,15 +10666,14 @@
       </x:c>
       <x:c r="H14" s="90" t="str">
         <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺
-当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。</x:v>
+当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。
+当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
         <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
-        <x:v>2026-10-04 TC-079 打包日期反例 3/5；各 TC 的自动通过与未验边界分别见原编号行及 docs/validation.md
-2026-10-04 项目沟通确认：暂缺正式 Developer ID/公证环境和第二台目标 Mac，TC-028/072 无新增执行证据。
-新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 真实双 DMG 隔离脚本 exit 0，打包 Electron 43/43；TC-079 重复失败记录继续有效，不宣称版本完成。</x:v>
+        <x:v>三批完整范围见关联编号；TC-079 共用脚本定位待修复验，TC-076 隔离通过、系统/生产待验，TC-028/072 缺资源。各项证据见测试用例及 docs/validation.md。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据

</xml_diff>

<commit_message>
docs: record independent date test and package validation
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R3874106da2874b86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R655cfcbea0de4550"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc033b6eb87564067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R5561639d72a6499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Raae18bcbf9ab4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2e34e840fafd400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6ff9b0bb65be4aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc1ea221fc5ab4ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R468754ee2c3d4062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rd547c07231db49df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2672,7 +2672,8 @@
       <x:c r="G85" s="55" t="str">
         <x:v>78b3a3b 已注册；TC-079 单元 1/1 + Electron 1/1 通过；仅 REQ-041 同事实集合查询/导出子范围
 2026-10-04 REQ-041→DEV-050→TC-079 新增双日期连续快速修改/最终组合/无错误/CSV 同屏验收；当前打包共用路径重复 3/5，2 次失败，待修/复验。
-2026-10-04 根因修订：共用打包测试跨页模糊标签误选来源页日期；原生报表控件不改。旧 2/5、新报告 1/5 失败记录保留；专属真实查询/CSV 和无重试打包复验待补。</x:v>
+2026-10-04 根因修订：共用打包测试跨页模糊标签误选来源页日期；原生报表控件不改。旧 2/5、新报告 1/5 失败记录保留；专属真实查询/CSV 和无重试打包复验待补。
+7fd0ce7：文档会话独立 TC-079 1 单元+2 Electron、打包管理员无重试 5/5、打包全量 44/44，均 exit 0；旧 2/5 与开发新包 1/5 失败为修复前测试误选历史，产品代码未改。</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="85" customHeight="1">
@@ -4235,7 +4236,7 @@
         <x:v>下一轮产品打磨（第一批 B 阶段实现）</x:v>
       </x:c>
       <x:c r="E46" s="58" t="str">
-        <x:v>异步/快照子范围已通过；打包共用测试日期定位错误待修并复验，产品日期控件异常未证实</x:v>
+        <x:v>异步/快照及修正定位后的日期自动子范围通过；产品原生日期控件未改，真实生产/系统验收未覆盖</x:v>
       </x:c>
       <x:c r="F46" s="58" t="str">
         <x:v>DEV-050</x:v>
@@ -4248,7 +4249,8 @@
 2026-10-03 78b3a3b：授权查询及选中事实生成 SHA-256 snapshotId（事实集合身份，非全库 revision），汇总/明细/CSV 共同核对；新事实改变该筛选内集合时旧 ID 拒绝导出并提示刷新。React 快速 A→B 旧响应不覆盖、加载禁用导出，IPC 带 B 筛选及 B ID；界面显示范围/时区/筛选摘要，CSV 原 10 列顺序保留。文档会话独立复跑 TC-079 单元 1/1、Electron 1/1、TC-029、TC-023 和 test:gate（77 入口、53 单元、19 Electron），均退出码 0。只支持本条已测子范围；REQ-040/042–048 未据此通过。
 47b03d5：TC-079 追加 v1→冲突 v2、扫描入库后旧 snapshotId 拒绝及刷新小计 99→104；文档会话单元+Electron 与 gate 独立通过。
 508851a 未签名目录包共用报表 E2E 重复 5 次中 2 次开始日期回退；验收补充先于开发修改。旧 TC-079 源码态通过不覆盖打包连续修改。
-2026-10-04 复核修订：需求/开发会话报告，新目录包 5 次无重试执行仍 1 次失败；失败时操作快照在“工作台 / 数据来源”。共用 app.spec.ts 在切到报表后立即用 page.getByLabel("开始日期")，它会模糊匹配来源页“最近记录开始日期”；当前代码中两个标签并存，且该测试未等待 .report-page 可见。此前固定 508851a 包 3/5 通过、2/5 失败的错误页面显示报表日期倒置，但该末态不足以证明报表控件自行回退。定位结论为测试跨页误选，保留历史失败次数，产品日期控件缺陷待有效测试判定；不要求改为文本输入。</x:v>
+2026-10-04 复核修订：需求/开发会话报告，新目录包 5 次无重试执行仍 1 次失败；失败时操作快照在“工作台 / 数据来源”。共用 app.spec.ts 在切到报表后立即用 page.getByLabel("开始日期")，它会模糊匹配来源页“最近记录开始日期”；当前代码中两个标签并存，且该测试未等待 .report-page 可见。此前固定 508851a 包 3/5 通过、2/5 失败的错误页面显示报表日期倒置，但该末态不足以证明报表控件自行回退。定位结论为测试跨页误选，保留历史失败次数，产品日期控件缺陷待有效测试判定；不要求改为文本输入。
+7fd0ce7 只修改测试定位/断言；文档会话独立复验 TC-079、TC-021 与源码/打包全量，结果见测试用例 I/M 列及 docs/validation.md。旧错误末态不证明产品控件回退。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="150" customHeight="1">
@@ -5754,7 +5756,7 @@
         <x:v>src/main/report.ts、index.ts；src/preload/index.ts；src/renderer/report.tsx；src/shared/types.ts；tests/report-snapshot.test.ts、tests/e2e/report-snapshot.spec.ts；scripts/test-cases.mjs、run-test-case.mjs</x:v>
       </x:c>
       <x:c r="F55" s="58" t="str">
-        <x:v>异步/快照子范围已实现；打包共用 E2E 先修跨页日期定位并复验，产品日期控件不改</x:v>
+        <x:v>既有查询/快照实现与测试定位修复的自动子范围通过；7fd0ce7 未改产品日期控件，生产环境待验</x:v>
       </x:c>
       <x:c r="G55" s="58" t="str">
         <x:v>为筛选/授权/时区/区间建立稳定请求键或代次；取消或丢弃旧响应，导出绑定已显示查询，加载中不可导出旧/新混合。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5762,7 +5764,8 @@
 78b3a3b：ReportService 用授权查询和选中事实字段生成 SHA-256 snapshotId，明细/CSV 重算拒绝过期 ID；React 筛选匹配与请求代次防止迟到 A 覆盖 B，加载禁用导出，IPC 带筛选和 ID；显示导出范围摘要。快照不是全库 revision，所选事实不变时 ID 可不变。文档会话独立执行 TC-079 1 unit+1 Electron、TC-029、TC-023、test:gate（77 入口、53 unit、19 E2E），均退出码 0。
 47b03d5：TC-079 原单元新增冲突 v2 快照身份回归：新增遥测使旧 ID 拒绝、刷新小计 99，继续新增事实又拒绝，刷新小计 104；单编号 unit/Electron 与完整门禁独立通过。
 2026-10-04 新修复目标：排查日期输入状态/异步请求竞态，确保连续快速填写两端后值保持、只查询最终组合、无日期范围错误，CSV 与屏显同快照；TC-079 加打包反例，TC-021 管理员主流程回归。
-2026-10-04 当前最小修复：保留原生日期控件，先等待 .report-page 可见，再在该容器内以 getByLabel("开始日期",{exact:true})、结束日期精确定位；TC-079 专属绑定核真实授权查询参数、页面/明细与 CSV 同一已应用查询及 snapshotId。禁止用失败重试掩盖共用打包反例。既有“排查输入状态”段落为定位前计划。</x:v>
+2026-10-04 当前最小修复：保留原生日期控件，先等待 .report-page 可见，再在该容器内以 getByLabel("开始日期",{exact:true})、结束日期精确定位；TC-079 专属绑定核真实授权查询参数、页面/明细与 CSV 同一已应用查询及 snapshotId。禁止用失败重试掩盖共用打包反例。既有“排查输入状态”段落为定位前计划。
+7fd0ce7 将 app.spec.ts 限定 .report-page 且精确标签，TC-079 加独立真实隔离库双日期/错误/CSV Electron 绑定，TC-094 首次管理员建立后等概览再关 App；文档会话独立复验，详见 TC-079/021/094。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="155" customHeight="1">
@@ -6937,7 +6940,8 @@
       </x:c>
       <x:c r="I26" s="9" t="str">
         <x:v>历史：tests/report.test.ts、tests/e2e/app.spec.ts、A8 的共享测试通过；当时未测第二页。2026-10-03 f7fcdee：新增独立单元和 Electron 分页测试；开发会话报告 TC-021 与门禁通过（73 入口/42 单元/18 Electron）；文档会话单编号独立复跑四个绑定均通过，退出码 0。详见 docs/validation.md。 后续：961c96c 补启动失败清理；8234dcc 补样本写入/数据库关闭异常清理。开发会话在 8234dcc 上报告类型检查、TC-021 单编号及完整门禁通过（73 入口/42 单元/18 Electron）；文档会话独立复跑四个绑定退出码 0；见 docs/validation.md。
-2026-10-04 作为 REQ-041/TC-079 日期回退修复的管理员筛选与分页回归；新目标修复后按编号单独复跑，不能用既有结果替代。</x:v>
+2026-10-04 作为 REQ-041/TC-079 日期回退修复的管理员筛选与分页回归；新目标修复后按编号单独复跑，不能用既有结果替代。
+2026-10-04 固定 7fd0ce7 文档会话独立运行 npm run test:case -- TC-021：共享管理员 app.spec.ts、独立分页单元及 Electron 共 1 单元+2 Electron，exit 0；同提交源码门禁 94/97/44、打包管理员无重试 5/5、打包全量 44/44。</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
         <x:v>npm run test:case -- TC-021</x:v>
@@ -6950,7 +6954,8 @@
       </x:c>
       <x:c r="M26" s="9" t="str">
         <x:v>tests/support/test-workspace.ts 为单元临时 token.sqlite 和 Electron 临时用户数据分别隔离，合成 JSONL 无正文且以 turn_context 标注模型，结束清理。开发首轮因无效 payload.model 造数失败，修正后完整重跑通过；文档会话独立复跑单编号退出码 0。TC-028/TC-072 目标环境仍待验；证据见 docs/validation.md。 8234dcc 使测试异常时的一次性目录清理更完整；产品行为、断言和绑定未变。
-TC-021 为关联回归，尚未针对新日期缺陷复跑；主验收归 TC-079。</x:v>
+TC-021 为关联回归，尚未针对新日期缺陷复跑；主验收归 TC-079。
+7fd0ce7；macOS 15.7.4 x86_64、Node v24.15.0；TC-021 单编号 exit 0（1 单元+2 Electron），本机临时库/无正文样本；产品真实账户未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -9444,7 +9449,7 @@
 2026-10-04 修订预期：切页完成前不输入，两个日期只写报表控件；最终有效组合产生真实查询，旧响应不得覆盖，页面/明细/CSV 同授权范围、时区和 snapshotId。五次无重试共用打包路径与专属 TC-079 均通过后，才更新本子范围状态；末态错误页不能单独证明产品控件回退。</x:v>
       </x:c>
       <x:c r="H84" s="55" t="str">
-        <x:v>既有源码态快照子范围通过；打包共用 E2E 日期定位错误待修复验，产品日期控件缺陷未证实</x:v>
+        <x:v>修正定位后自动子范围通过：固定 7fd0ce7 单编号 1 单元+2 Electron、真实打包共用用例无重试 5/5、打包全量 44/44；生产/系统环境未验</x:v>
       </x:c>
       <x:c r="I84" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -9453,25 +9458,30 @@
 2026-10-04 固定代码 508851a、app.asar SHA-256 8a687bf6…：开发会话在文档工作树运行 npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5，3/5 通过、2/5 失败，exit 1。文档会话复核 repeat3/4 错误快照，开始日期回退至 2026-09-05、结束 2026-01-02，报日期范围无效；新增 TC-079 断言尚未实现，当前失败不能写通过。
 2026-10-04 新 DMG 8773dd38… 已构建/校验，但未针对双日期快速输入反例单独复测；508851a 目录包 2/5 失败仍是已知风险，不能以构建或旧包结果改成通过。
 2026-10-04 复核修订：需求/开发会话报告，新目录包 5 次无重试执行仍 1 次失败；失败时操作快照在“工作台 / 数据来源”。共用 app.spec.ts 在切到报表后立即用 page.getByLabel("开始日期")，它会模糊匹配来源页“最近记录开始日期”；当前代码中两个标签并存，且该测试未等待 .report-page 可见。此前固定 508851a 包 3/5 通过、2/5 失败的错误页面显示报表日期倒置，但该末态不足以证明报表控件自行回退。定位结论为测试跨页误选，保留历史失败次数，产品日期控件缺陷待有效测试判定；不要求改为文本输入。
-2026-10-04 开发会话随后报告已撤回日期产品改动并仅修共用测试为报表容器内 exact 标签：源码管理员流程重复 20 次 exit 0，重构目录包同用例重复 5 次 exit 0，TC-079 单编号 exit 0。此时尚无固定提交/制品 SHA 与完整门禁、打包全量结果；文档会话未独立复跑，不把暂存通过登记为整项通过。</x:v>
+2026-10-04 开发会话随后报告已撤回日期产品改动并仅修共用测试为报表容器内 exact 标签：源码管理员流程重复 20 次 exit 0，重构目录包同用例重复 5 次 exit 0，TC-079 单编号 exit 0。此时尚无固定提交/制品 SHA 与完整门禁、打包全量结果；文档会话未独立复跑，不把暂存通过登记为整项通过。
+2026-10-04 固定代码 7fd0ce7；文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 独立运行：test:cases:check 94 入口；npm run test:case -- TC-079 为 1 单元+2 Electron，TC-021 为 1 单元+2 Electron，TC-094 为 2 单元+1 Electron，均 exit 0；npm run test:gate 为类型检查、94 入口、97/97 单元、44/44 Electron，exit 0。重新 pack:dir 后 app.asar SHA-256 8a687bf692b150e59615e338b57e75f94db516477fad5b9e30f98b70d66eb460，管理员共用打包用例 --repeat-each=5 --retries=0 为 5/5，打包全量 44/44，均 exit 0。旧固定包 2/5 失败、新目录包开发自测 1/5 失败仍为修复前测试误选记录；未执行真实生产账户或系统安装。</x:v>
       </x:c>
       <x:c r="J84" s="55" t="str">
-        <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）</x:v>
+        <x:v>npm run test:case -- TC-079（已注册；文档会话 2026-10-03 退出码 0）
+npm run test:e2e:packaged -- tests/e2e/app.spec.ts --repeat-each=5 --retries=0；npm run test:e2e:packaged；npm run test:gate</x:v>
       </x:c>
       <x:c r="K84" s="55" t="str">
-        <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。</x:v>
+        <x:v>scripts/test-cases.mjs：unit 绑定 tests/report-snapshot.test.ts 的 TC-079 查询后新增事实必须刷新快照才能导出相同事实集合；extraRuns 绑定 tests/e2e/report-snapshot.spec.ts 的 TC-079 快速切换筛选时旧响应不覆盖且导出等待当前快照。
+7fd0ce7 新增 tests/e2e/report-snapshot.spec.ts 的 TC-079 双日期独立 Electron 绑定：倒置范围报错/导出禁用、连续输入最终日期、真实隔离样本 42 Token 与 CSV 日期/模型。原单元及 A→B Electron 继续验证授权快照/旧响应；共用 app.spec.ts 在 .report-page 内精确定位。</x:v>
       </x:c>
       <x:c r="L84" s="55" t="str">
         <x:v>当前已在单元测试覆盖 v1 与冲突 v2 的扫描后旧 snapshotId 拒绝；Electron 仍侧重快速筛选切换与导出等待当前快照。snapshotId 是授权查询+事实集合身份，不是全库 revision；REQ-040 历史覆盖及目标安装环境仍未由此证明。
 本次打包共用 app.spec.ts 只复现异常，尚未有专属 TC-079 双日期快速修改绑定；失败根因未定，应用状态与测试时序需区分。
-当前根因修订覆盖前文“日期字段回退/根因未定”的推断：共用脚本全页模糊标签在报表页出现前可误选来源页控件。专属 TC-079 的真实查询/CSV 断言及修正后打包复验尚无通过证据。</x:v>
+当前根因修订覆盖前文“日期字段回退/根因未定”的推断：共用脚本全页模糊标签在报表页出现前可误选来源页控件。专属 TC-079 的真实查询/CSV 断言及修正后打包复验尚无通过证据。
+新双日期 Electron 用例不单独截取 IPC 的 snapshotId；同编号既有单元/A→B Electron 负责旧 ID 拒绝与同快照导出断言。5/5 只针对本机未签名目录包和合成数据，不代表真实生产账户、系统安装或外部分发。</x:v>
       </x:c>
       <x:c r="M84" s="55" t="str">
         <x:v>固定代码 78b3a3b；macOS 本机；单编号 TC-079 unit/E2E 各 1/1、TC-029 与 TC-023 各 1/1、test:gate 53 unit/19 E2E/77 入口，均退出码 0。无生产数据或真实打包安装证据。
 47b03d5；macOS 本机隔离合成库；TC-079 单元/Electron 各 1/1、退出码 0；完整 gate 82 入口/57 unit/22 E2E 通过。
 0.3.6 打包日期新验收当前失败 2/5；修复后必须单编号运行 TC-079、TC-021 回归，再重复打包用例并跑打包全量。
 待固定测试修复提交与候选包 SHA 后，记录 TC-079、TC-021、无重试真实打包重复五次及打包全量的命令/退出码；本轮只修订追溯，不改测试结果为通过。
-开发会话工作树初步结果：源码管理员流程 20/20、重构目录包共用报表 5/5、TC-079 单编号 exit 0；固定提交、包 SHA、完整门禁与打包全量待补。</x:v>
+开发会话工作树初步结果：源码管理员流程 20/20、重构目录包共用报表 5/5、TC-079 单编号 exit 0；固定提交、包 SHA、完整门禁与打包全量待补。
+2026-10-04 固定代码 7fd0ce7；文档会话在 macOS 15.7.4 x86_64、Node v24.15.0 独立运行：test:cases:check 94 入口；npm run test:case -- TC-079 为 1 单元+2 Electron，TC-021 为 1 单元+2 Electron，TC-094 为 2 单元+1 Electron，均 exit 0；npm run test:gate 为类型检查、94 入口、97/97 单元、44/44 Electron，exit 0。重新 pack:dir 后 app.asar SHA-256 8a687bf692b150e59615e338b57e75f94db516477fad5b9e30f98b70d66eb460，管理员共用打包用例 --repeat-each=5 --retries=0 为 5/5，打包全量 44/44，均 exit 0。旧固定包 2/5 失败、新目录包开发自测 1/5 失败仍为修复前测试误选记录；未执行真实生产账户或系统安装。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="185" customHeight="1">
@@ -10238,7 +10248,8 @@
       </x:c>
       <x:c r="I99" s="67" t="str">
         <x:v>2026-10-03 文档会话固定 8157e2d 独立运行 TC-094：单元 1/1、退出码 0。合成旧表迁移、旧 v1 续传 legacy_unknown/GET confirmedSubtotal=null、v2 重算及冲突、跨 owner/白名单拒绝、v1 回滚状态不变、旧 outbox 重算及协议不兼容待传后恢复。完整 gate 82/56/22 通过。
-508851a：单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。</x:v>
+508851a：单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。
+2026-10-04 7fd0ce7 仅在首次创建管理员后等概览可见再关闭测试 App，消除测试自身竞态；文档会话独立 TC-094 2 单元+1 Electron exit 0，源码门禁与打包全量 44/44。修复前开发全量 43/44（首次重启登录失败）为历史失败，不能抹去。</x:v>
       </x:c>
       <x:c r="J99" s="67" t="str">
         <x:v>npm run test:case -- TC-094（已注册；文档会话退出码 0）</x:v>
@@ -10256,7 +10267,8 @@
       </x:c>
       <x:c r="M99" s="67" t="str">
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。
-508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。</x:v>
+508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。
+7fd0ce7；macOS 15.7.4 x86_64、Node v24.15.0；TC-094 单编号 2 单元+1 Electron、test:gate 94/97/44、打包全量 44/44，均 exit 0；生产迁移/真实旧服务仍未验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10630,16 +10642,16 @@
         <x:v>TC-040、TC-076–094</x:v>
       </x:c>
       <x:c r="H13" s="89" t="str">
-        <x:v>0.3.6 本机未签名候选：打包与完整性通过；同包门禁、TC-076 隔离子范围及打包 Electron 43/43 通过；TC-079 共用测试定位修复与专属复验、系统/生产/外部验收待补</x:v>
+        <x:v>0.3.6 本机未签名候选：7fd0ce7 测试定位修复后 TC-079/021/094 与源码门禁、目录包无重试五次及全量通过；TC-076 隔离升级/回退已证；系统/生产/外部验收待补</x:v>
       </x:c>
       <x:c r="I13" s="89" t="str">
-        <x:v>本机临时候选部分验证；TC-079 打包共用测试定位待修复验，完整验收未通过</x:v>
+        <x:v>本机候选自动与打包子范围通过；完整版本/公开分发验收未完成</x:v>
       </x:c>
       <x:c r="J13" s="89" t="str">
-        <x:v>新 DMG 8773dd38…：门禁 94/97/43、打包 43/43、TC-076 隔离通过。TC-079 旧包 3/5，新包需求会话报告 4/5；脚本跨页模糊定位，产品缺陷未证。TC-028/072 待环境。详见 docs/validation.md。</x:v>
+        <x:v>7fd0ce7 仅改测试：文档独立门禁 94/97/44、打包 5/5 与 44/44，通过。旧 2/5 和开发报告 1/5 为修复前测试失败。服务包 8773dd38… 完整性通过；TC-028/072 未验。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
-        <x:v>先修共用 E2E 报表容器/精确标签并增加 TC-079 真实查询与 CSV；复验 TC-021、打包五次无重试及全量。生产迁移、系统安装、TC-028/072 待证。</x:v>
+        <x:v>补真实生产账户/系统安装、来源归属和迁移验收；具备签名、公证、另一台目标 Mac 后执行 TC-028/072。保留旧失败及对应固定提交证据。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="142.5" customHeight="1">
@@ -10667,13 +10679,14 @@
       <x:c r="H14" s="90" t="str">
         <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺
 当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。
-当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。</x:v>
+当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。
+7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
         <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
-        <x:v>三批完整范围见关联编号；TC-079 共用脚本定位待修复验，TC-076 隔离通过、系统/生产待验，TC-028/072 缺资源。各项证据见测试用例及 docs/validation.md。</x:v>
+        <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据

</xml_diff>

<commit_message>
docs: align upgrade boundary and managed CLI acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R2e34e840fafd400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6ff9b0bb65be4aa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc1ea221fc5ab4ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R468754ee2c3d4062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rd547c07231db49df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R522a0b8c159947f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb8ab2579fdba499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3451773e901a4009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rde4d62ac0b334cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Reb0ff4778a7b4169"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2597,7 +2597,8 @@
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
 508851a：历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过；详情见测试用例 I/L/M 列与 docs/validation.md。
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 新包隔离升级及两层五故障回退动态子范围通过；完整系统/生产验收待补；历史取消设计保留备选。
-当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2 TC-076 真实双 DMG 脚本 exit 0；范围与限制见测试用例 I/M 列。</x:v>
+当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2 TC-076 真实双 DMG 脚本 exit 0；范围与限制见测试用例 I/M 列。
+2026-10-04 最新用户决议：点击开始前可放弃；点击后下载/校验/交接/安装全程无取消，直到成功或失败自动恢复。独立窗口、取消协议/journal、分阶段点击取消不属本轮；旧隔离成功/五故障证据保留，系统/生产/目标 Mac 仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -2622,7 +2623,8 @@
       <x:c r="G83" s="71" t="str">
         <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验
 2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
-2026-10-04 受管持续采集设计已决，TC-077 受控和真实 CLI 正例未实施；整项待验。</x:v>
+2026-10-04 受管持续采集设计已决，TC-077 受控和真实 CLI 正例未实施；整项待验。
+2026-10-04 TC-077：阶段一新增管理员受限 CLI、viewer/越界拒绝、actor≠owner、账本失效负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="135" customHeight="1">
@@ -2647,7 +2649,8 @@
       <x:c r="G84" s="72" t="str">
         <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验
 2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
-2026-10-04 TC-078 双关闭等长完整窗口受控/真实正例待实施，范围外未知；整项待验。</x:v>
+2026-10-04 TC-078 双关闭等长完整窗口受控/真实正例待实施，范围外未知；整项待验。
+2026-10-04 TC-078：阶段一新增未知 owner/水位缺口仍不可比负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -2790,7 +2793,8 @@
       <x:c r="G90" s="72" t="str">
         <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验
 2026-10-03 覆盖证据决议：真零须已关闭同范围完整空窗；合成只验规则，真实来源未证；REQ-044/DEV-053/TC-084 整项待验。
-2026-10-04 TC-084 受管关闭空窗真零正例待实施，固定快照/空心跳不能补证；整项待验。</x:v>
+2026-10-04 TC-084 受管关闭空窗真零正例待实施，固定快照/空心跳不能补证；整项待验。
+2026-10-04 TC-084：阶段一新增管理员结果可见、正文仅内存与空状态负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -3737,14 +3741,15 @@
         <x:v>应用内自动安装升级</x:v>
       </x:c>
       <x:c r="C28" s="14" t="str">
-        <x:v>用户在应用内确认新版后，已校验 DMG 由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
-2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：未点击更新前可放弃；点击后下载并校验，通过后自动退出旧版、原位替换和启动新版；开始执行替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。</x:v>
+        <x:v>用户在应用内点击“开始升级”后下载并校验 DMG，由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
+2026-10-04 前次决议（已被下方最新点击边界取代，仅供追溯）：未点击更新前可放弃；点击后下载并校验，通过后自动退出旧版、原位替换和启动新版；开始执行替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。
+2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。</x:v>
       </x:c>
       <x:c r="D28" s="14" t="str">
         <x:v>M5（计划）</x:v>
       </x:c>
       <x:c r="E28" s="14" t="str">
-        <x:v>部分验证；当前新 DMG 真实旧/新隔离升级、installer/打包 helper 各五故障回退与重试通过；系统目录、真实故障和生产数据仍待验</x:v>
+        <x:v>部分验证；点击前可放弃、点击后下载至安装不可取消为当前决议，真实双 DMG 隔离升级与双路径五故障回退通过；全阶段无取消 UI/系统目录/生产数据待验</x:v>
       </x:c>
       <x:c r="F28" s="14" t="str">
         <x:v>DEV-025</x:v>
@@ -3761,7 +3766,8 @@
 2026-10-04 取消设计决议：当前没有旧 App 退出后的可见取消入口，健康标记前新版会打开真实 userData。独立控制进程、helper 阶段 journal/取消能力、隔离健康探测与结果持久反馈待实现；1961de3 五故障通过不代证取消。
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 当前新包取干净 main 9af351a，SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；旧 d99d7af9 包的 TC-076 故障证据不外推。
-2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
+2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 当前隔离成功/五故障自动恢复证据继续有效；未知的系统目录、真实满盘/断电与目标 Mac 不升为通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4195,13 +4201,14 @@
         <x:v>按所选工具、用户、IANA 时区和时间区间分别判定完整、部分、未知/未覆盖与已确认零；必须有可证明的来源留存、扫描及时间窗口，当前 SourceStatus=ready 不足以证明完整历史。近 7/30/90 天包含今天；今天进行中须标截至最近成功采集时间（as-of）及扫描延迟，不可算完整日。上期与本期须同范围、等长、同截止口径且双方相应窗口可证覆盖才显示增减比例，任一不足显示不可比较，不把空区间当零。
 管理员选具体用户或“未归属”后，来源卡、报表 coverage、真零与比较只按该用户+所选工具/IANA 时区/区间的可证覆盖判定。全局 ready/计数/最近扫描时间只能另标“全局”诊断，不能补全选中范围；全局 ready 而所选用户空且缺证据时为未知/部分，不是已确认零。
 本轮部分范围：先按授权 owner（含未归属）+工具+IANA 时区+区间生成保守未知/可证部分覆盖；全局 ready/计数/时间、最早事实与成功空扫描都不构成完整证明。无事实不宣称已确认零；仅 pending 事实可显示已确认小计 0，但完整总量未知；比较不可比较。完整空窗真零和同 as-of 同口径同比正例待可证留存/连续采集方案。
-2026-10-03 覆盖证据决议：仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。窗口关闭且同一事实集为空才可显示“已确认零（所选已监测来源）”；不得声称服务商账单或全设备零。比较需两窗等长、同范围/时区/as-of 且双方完整。</x:v>
+2026-10-03 覆盖证据决议：仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。窗口关闭且同一事实集为空才可显示“已确认零（所选已监测来源）”；不得声称服务商账单或全设备零。比较需两窗等长、同范围/时区/as-of 且双方完整。
+2026-10-04 受管账本阶段一（计划，尚未实现/执行）：用户主动启用受管入口后，仅管理员可从明确授权的本机工作目录启动固定 Codex/Claude CLI 的只读或计划模式；主进程/服务按应用角色、受控路径及符号链接实际目标、固定可执行文件/参数/环境白名单复核，viewer 即使与管理员共用 macOS 账户凭证也不可通过界面或 IPC 启动，拒绝发生在 spawn 前。actor 只是发起者；CLI 账号归属须由可验证的提供方身份和有效绑定版本证明，不能由点击者、macOS UID、凭证目录推定。缺证据时 owner_verified=false、owner 为空，运行/用量不进入报表事实或完整覆盖。仅耐久保存 run/event/heartbeat/水位、白名单计量与错误状态；提示词、回复和原始流正文只在发起者当前窗口的有界内存显示，退出/切换用户清除，不写数据库、日志、反馈附件。解析、落盘、服务中断或重启未能核对的运行和窗口 fail closed。阶段一不产出 source-complete、真零或同比正例。</x:v>
       </x:c>
       <x:c r="D45" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E45" s="55" t="str">
-        <x:v>保守未知/防假零子范围已实现并独立复验（ef7a3de、c10bbf3）；整项待验证，完整真零/同比正例待证据方案</x:v>
+        <x:v>保守未知/防假零自动子范围已证；受管 CLI 阶段一授权/归属/账本未实现，完整覆盖与同比正例待验</x:v>
       </x:c>
       <x:c r="F45" s="55" t="str">
         <x:v>DEV-049</x:v>
@@ -4217,7 +4224,8 @@
 2026-10-03 代码 ef7a3de、语义修正 c10bbf3：按授权 owner+工具+模型+项目+IANA 时区+区间的已观察事实生成覆盖；有无事实均标未知，有事实保留本范围计数和最近观察时间，asOf/来源级 lastScan 空值。文档会话独立复跑 TC-077/078 与相关回归及完整门禁通过；ef7a3de 的“有事实即部分”已由 c10bbf3 修正；单条事实不证明连续区间完整。真零/同比正例未验，REQ-040 整项待验证。详见 docs/validation.md。
 3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。
 2026-10-03 覆盖证据决议：现有状态/游标/事实仅证已观察；受控合成正例只验规则，不证明真实 Codex/Claude 来源完整。真实来源机制未落实，整项仍待验。官方：https://learn.chatgpt.com/docs/developer-commands?surface=cli 与 https://code.claude.com/docs/en/monitoring-usage
-2026-10-04 设计决议：用户主动启用受管会话；持久启动/结束账本、逐事件用量与守护连续水位按 owner/provider/模型/项目/IANA 时区/关闭窗口 fail closed。文件快照仅证重放；普通本机全部使用量及范围外仍未知。见 docs/coverage-evidence-decision.md；未实施、未验真实正例。</x:v>
+2026-10-04 设计决议：用户主动启用受管会话；持久启动/结束账本、逐事件用量与守护连续水位按 owner/provider/模型/项目/IANA 时区/关闭窗口 fail closed。文件快照仅证重放；普通本机全部使用量及范围外仍未知。见 docs/coverage-evidence-decision.md；未实施、未验真实正例。
+阶段一沿用 REQ-040→DEV-049→TC-077/078；CLI 执行安全与可证 owner 是受管来源范围成立的前置条件，新增断言仍待注册/执行。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -4317,13 +4325,14 @@
       <x:c r="C49" s="55" t="str">
         <x:v>真零、未扫描、权限不足、格式不支持、筛选无匹配和部分覆盖分别说明原因与下一步；诊断原因指向相应授权/重扫/调整筛选动作。长扫描持续显示阶段与最近进展，不伪造百分比，失败可重试。
 本轮只排可证的分型和行动：未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知及有已观测记录但完整性未知；真零保留为未来同一授权筛选范围 coverage.complete 且事实为空的受控分支。
-2026-10-03 覆盖证据决议：真零依赖 REQ-040 的 仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。仅窗口关闭且同一授权筛选事实集为空可标限定真零。</x:v>
+2026-10-03 覆盖证据决议：真零依赖 REQ-040 的 仅对所选 owner（含未归属）+provider+时间窗及筛选的明确监测来源范围，在可核验留存起点、连续采集/重放水位、无缺口/丢弃/权限或格式错误、身份归属可证、所选模型/项目等维度完整解析时，才允许 source-complete。范围外执行模式写未知；全局 ready、空扫描、最早事实和单次缓存盘点均不补证。仅窗口关闭且同一授权筛选事实集为空可标限定真零。
+2026-10-04 阶段一新增结果体验与隐私：管理员发起受管命令后，在当前已授权窗口可见完成状态和有界结果正文，或获得明确、安全且仅本会话有效的打开结果动作；关闭窗口/退出/切换用户后正文丢弃，不能由 viewer 读取。无结果或异常须说明原因与下一步，不把身份未知、空账本或受管命令无用量称真零；正文不得写数据库、日志、反馈附件。</x:v>
       </x:c>
       <x:c r="D49" s="55" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E49" s="55" t="str">
-        <x:v>部分实现；保守空状态与进度/取消/重试自动子范围通过，真零待 REQ-040 证据</x:v>
+        <x:v>保守空状态与进度/取消/重试自动子范围通过；受管结果可见/正文隐私阶段一未实现，真零待 REQ-040 证据</x:v>
       </x:c>
       <x:c r="F49" s="55" t="str">
         <x:v>DEV-053</x:v>
@@ -4337,7 +4346,8 @@
 2026-10-03 代码 000372b：文档会话独立复跑 TC-084/085 各单元+Electron、六项回归及完整门禁（88 入口、64 单元、28 Electron）通过。TC-084 无同范围 complete 真零正例；TC-085 无可取消状态/续扫，整项待验。
 2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。
 2026-10-03 覆盖证据决议：TC-084 可计划受控合成规则正例；真实来源完整性、范围外执行模式和实际空窗未验，REQ-044 整项待验。
-2026-10-04 真零仅限同一授权受管来源关闭空窗、启动账本和连续采集可证、事实集为空；界面标范围外未知。TC-084 受控和真实正例待实现/验收。</x:v>
+2026-10-04 真零仅限同一授权受管来源关闭空窗、启动账本和连续采集可证、事实集为空；界面标范围外未知。TC-084 受控和真实正例待实现/验收。
+阶段一沿用 REQ-044→DEV-053→TC-084；结果可见性/短暂内存与空状态为现有用户可操作性目标的细化，不新增编号；真实 CLI 与真零正例仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5163,7 +5173,7 @@
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>部分实现/验证；当前简化范围为安装前可放弃、安装开始后不可取消、失败自动回退；新包隔离升级及双路径五故障回退通过，真实系统/生产场景待验</x:v>
+        <x:v>部分实现/验证；本轮点击前可放弃，点击开始后下载/校验/交接/安装全程不可取消、失败自动回退；隔离成功与五故障通过，全阶段 UI/系统/生产仍待验</x:v>
       </x:c>
       <x:c r="G30" s="70" t="str">
         <x:v>当前 1e70412：文档会话构建 0.3.6 x64 目录包并以真实旧/新 DMG、固定哈希独立复跑 TC-076，exit 0；TC-036 2/2 合成单元回归通过。
@@ -5171,10 +5181,11 @@
 86a4b5b：Node 模式辅助进程等待旧版退出，验证 DMG 与 Bundle 身份/架构/版本，安装同卷暂存并备份原 App，启动新版等待健康标记，失败回滚/尝试重开旧版；DMG 只读来源按权限选 /Applications 或 ~/Applications。文档会话 TC-036 2/2、TC-076 1/1、hdiutil verify 0.3.5 VALID、SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。TC-076 旧版仅由 0.3.5 元数据改号，真实旧二进制不是该测试对象；开发会话另报告生产安装 0.3.0 由新 helper 一次性人工接管，先备份 userData、原位更新至 0.3.5 并自动启动，未人工验完整账号/真实数据。
 2026-10-04 / 80e7f10→0eac84b：健康标记的 /var 与 /private/var 父目录别名以真实路径比较，叶子 App 符号链接仍拒绝；TC-036 2/2。TC-076 的 80e7f10 独立复跑最后状态文件竞态 exit 1，0eac84b 修后同包完整命令 exit 0。生产 installer 模块 hooks 与实际打包 helper/UI 故障必须分开登记。
 2026-10-04 1961de3：TC-076 三段集成绑定中的新增 scripts/verify-packaged-helper-faults.mjs 在隔离临时目录经旧 UI 触发真实打包 helper；文档会话完整命令 exit 0、TC-036 两项单元 exit 0。未测真实满盘/进程崩溃/系统安装/签名公证异机。
-2026-10-04 下一任务：管理员授权的一次性取消能力及独立更新控制窗口；下载 AbortController、helper 阶段/回执/安全检查点、替换后回滚、隔离健康探测防真实 userData 迁移、终态可重启读取和中断恢复。成功提交后取消 too_late；系统级断电自动恢复若承诺须另有 bundle 外恢复入口。
+2026-10-04 历史取消计划（已撤销，不属本轮任务）：管理员授权的一次性取消能力及独立更新控制窗口；下载 AbortController、helper 阶段/回执/安全检查点、替换后回滚、隔离健康探测防真实 userData 迁移、终态可重启读取和中断恢复。成功提交后取消 too_late；系统级断电自动恢复若承诺须另有 bundle 外恢复入口。
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
-2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 前文“独立窗口/阶段取消”为旧计划；开发工作树未提交实验不算候选。当前新包 SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，包校验通过，安装功能新证据待补。
-2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:v>
+2026-10-04 前次决议（已被下方最新点击边界取代，仅供追溯）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 前文“独立窗口/阶段取消”为旧计划；开发工作树未提交实验不算候选。当前新包 SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，包校验通过，安装功能新证据待补。
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
+2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 产品/测试不得把下载阶段可取消写成承诺；旧取消控制窗口、取消协议及取消 journal 不属本轮。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -5727,7 +5738,7 @@
 另核 src/renderer/report.tsx 的 coverage 与 src/main/index.ts 的授权报表 IPC；全局诊断若保留需显式标范围。</x:v>
       </x:c>
       <x:c r="F54" s="55" t="str">
-        <x:v>保守防假零/防假同比子范围已实现并独立复验（ef7a3de、c10bbf3）；完整覆盖证据与正例待开发/待验证</x:v>
+        <x:v>保守防假零/同比子范围已证；受管 CLI 安全入口、可证 owner 与耐久账本阶段一待实现/验证，complete 正例待验</x:v>
       </x:c>
       <x:c r="G54" s="55" t="str">
         <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5736,7 +5747,8 @@
 官方缺失输入反例：Codex ephemeral 无本地 rollout 文件、Claude 未启用 OTel 或 exporter=none 无遥测；将缺记录判未知，不能由 ready/空扫描/最早事实补证完整。详见 REQ-040 H45 的官方 URL。
 2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。
 2026-10-03 覆盖证据决议：增加监测来源边界、留存起点、连续采集/重放水位、错误/缺口、归属和维度解析的可审计证据链，按所选范围判定；关闭空窗限定真零，双窗同口径且完整才比较。合成契约不得提升真实来源状态。
-2026-10-04 分期：受管入口与持久运行/用量/连续水位账本→授权范围封窗与 UI 标签→TC-077/078 受控正例→真实 CLI 正例；固定快照不升级为完整使用窗口。</x:v>
+2026-10-04 分期：受管入口与持久运行/用量/连续水位账本→授权范围封窗与 UI 标签→TC-077/078 受控正例→真实 CLI 正例；固定快照不升级为完整使用窗口。
+2026-10-04 阶段一交付前置：固定 provider CLI、只读/计划模式和经过授权的工作目录，主进程/服务拒绝 viewer、任意命令/标志/环境和越界路径；先记 run_id、actorUserId，再独立核 provider 账号/绑定版，缺证据写 owner_verified=false、owner=null，不生成报表事实或 complete。耐久写 run/event/heartbeat/水位/白名单计量与错误；解析、落盘、异常退出/重启不一致时 fail closed。提示词/回复/原始流不得持久化。TC-077/078 独立临时库/假 CLI 验收；本期不开放完整窗正例。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -5833,7 +5845,7 @@
         <x:v>src/collectors/scanner.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；状态测试</x:v>
       </x:c>
       <x:c r="F58" s="55" t="str">
-        <x:v>部分实现；TC-085 进度/取消/续扫隔离自动目标通过，TC-084 真零待证</x:v>
+        <x:v>保守空状态/扫描反馈自动子范围已证；受管命令结果可见/内存隐私阶段一待实现，真零正例仍待证</x:v>
       </x:c>
       <x:c r="G58" s="55" t="str">
         <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5841,7 +5853,8 @@
 代码 000372b 已提供分型空状态、授权保守措辞、真实扫描阶段/处理数、错误修复重试。UsageScanner.scan() 与 UI 无取消入口；默认取消语义：停止新文件，当前文件事实/游标同事务结束，已处理事实仅算已观测、覆盖未知，重试从游标续扫，重复点击不并发。TC-085 需补该断言；TC-084 真零待 REQ-040 证据。
 90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。
 2026-10-03 覆盖证据决议：真零 UI 仅消费经 REQ-040/DEV-049 证明的所选来源 complete、已关闭且同事实集为空；范围外模式仍未知。真实来源机制未交付前 DEV-053 整项待验。
-2026-10-04 TC-084 真零依赖受管服务连续有效、关闭空窗及同范围空事实；先受控规则，再真实 CLI/守护服务正例，范围外仍未知。</x:v>
+2026-10-04 TC-084 真零依赖受管服务连续有效、关闭空窗及同范围空事实；先受控规则，再真实 CLI/守护服务正例，范围外仍未知。
+2026-10-04 阶段一：仅向发起管理员当前会话呈现受管任务状态与有界内存结果，或提供同会话安全打开动作；关闭/登出/切换用户清理正文，viewer 不可查看。DB、结构化日志、反馈附件只含脱敏状态/计量，不含提示词、回复或原始流；失败/身份未知给明确下一步，空结果不冒充真零。TC-084 用独立假 CLI/临时库和 UI/反馈附件核对。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -9253,17 +9266,19 @@
         <x:v>打包应用/本机隔离</x:v>
       </x:c>
       <x:c r="F81" s="52" t="str">
-        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；从隔离更新服务检查、下载及校验新版 DMG，点击升级后由应用自动退出旧版、安装替换并启动实际新版。安装前未确认时放弃，另注入磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
+        <x:v>独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；点击开始升级后从隔离更新服务检查、下载及校验新版 DMG，再由应用自动退出旧版、安装替换并启动实际新版。点击前退出或放弃，另注入磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
 2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。
-2026-10-04 当前简化操作：安装前放弃不得触发替换；一旦开始执行替换/安装，不提供取消动作；分别注入挂载、空间、替换、启动与健康故障，核自动恢复旧版/数据及重试。下载阶段取消非本轮必需，不能无代码证据写成通过。</x:v>
+2026-10-04 前次简化操作（已由下方最新操作取代）：安装前放弃不得触发替换；一旦开始执行替换/安装，不提供取消动作；分别注入挂载、空间、替换、启动与健康故障，核自动恢复旧版/数据及重试。下载阶段取消非本轮必需，不能无代码证据写成通过。
+2026-10-04 当前新增操作：点击开始前退出须保留旧版；点击开始后覆盖下载、校验、交接、安装直至成功/失败自动回退，不设计或点击中途取消控制。继续分别注入挂载、空间、替换、启动、健康故障核自动恢复旧版/数据、清理及重试；不新增五阶段取消正例。</x:v>
       </x:c>
       <x:c r="G81" s="52" t="str">
         <x:v>无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。
 2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。
-2026-10-04 当前预期：安装前不确认则旧版保持；安装开始后不可主动取消，正常成功自动替换/重启；故障自动回退旧版、保留用户数据与受信状态并清理残留。此口径新包隔离升级和故障回退子范围后续已动态验证，系统目录及生产数据仍待验。</x:v>
+2026-10-04 前次预期（已由下方最新预期取代）：安装前不确认则旧版保持；安装开始后不可主动取消，正常成功自动替换/重启；故障自动回退旧版、保留用户数据与受信状态并清理残留。此口径新包隔离升级和故障回退子范围后续已动态验证，系统目录及生产数据仍待验。
+2026-10-04 最新预期：点击前放弃不触发升级；点击后全程没有可用中途取消，正常成功旧版退出/替换/新版启动，故障自动回退且用户数据和受信状态连续。此无取消边界仍须按真实打包 UI/服务检查；既有隔离五故障通过不代证系统目录/生产。</x:v>
       </x:c>
       <x:c r="H81" s="52" t="str">
-        <x:v>部分验证：新 DMG 真实旧/新隔离升级、installer/打包 helper 各五故障自动回退与重试通过；安装前放弃、真实系统目录/生产数据和真实故障仍待验</x:v>
+        <x:v>部分验证：当前新 DMG 隔离成功升级、installer/打包 helper 各五故障回退与重试通过；点击后全阶段无取消 UI、真实系统目录/生产数据与真实故障待验</x:v>
       </x:c>
       <x:c r="I81" s="68" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
@@ -9289,7 +9304,8 @@
 2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。
 2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。
 本次并未复跑真实旧/新 DMG 与固定 SHA 的故障链；历史 1961de3 证据另列。系统安装、签名公证及安装中取消未验。
-2026-10-04 用户已撤出安装中取消交付要求；前文独立控制窗口/五阶段点击取消及“取消未验”属于历史阶段，不再构成当前简化目标的待验项。新包仍须按简化范围重新核安装成功、自动失败回退和数据连续性。</x:v>
+2026-10-04 用户已撤出安装中取消交付要求；前文独立控制窗口/五阶段点击取消及“取消未验”属于历史阶段，不再构成当前简化目标的待验项。新包仍须按简化范围重新核安装成功、自动失败回退和数据连续性。
+2026-10-04 用户最新决议：取消交付义务的边界从“开始替换/安装”前移至点击“开始升级”；下载/校验/交接/安装均不可中断取消。上方“下载取消待核实/安装中取消待验”及阶段取消正例只属历史；本轮只验点击前放弃、正常完成与失败自动回退。</x:v>
       </x:c>
       <x:c r="M81" s="52" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
@@ -9323,17 +9339,19 @@
 本轮先造 A/B/未归属及 viewer 范围负例：全局 ready、成功空扫描、最早事实、无事实用户、仅 pending 事实；按 owner+工具+时区+区间核主进程 API、概览卡、报表覆盖。完整空窗正例等待可证证据方案。
 以无正文合成缺失输入模拟 Codex ephemeral 不落文件及 Claude OTel 未启用/exporter=none；核本地文件/OTel 缺记录仍未知，不宣称工具没用或真零。真实工具端到端验证另行安排。
 2026-10-03 覆盖证据决议：计划受控合成正例：为所选 owner+provider+窗口逐项提供监测范围、留存起点、连续水位、无错误/缺口、归属及筛选维度证据；分别移除一项作降级反例，并核 API/概览/报表一致。真实工具来源另需独立证据。
-2026-10-04 待补受控持久运行账本正例与真实受管 Codex/Claude CLI（含 ephemeral/无持久会话）端到端；撤掉留存起点、启动/结束、连续水位、身份/维度、无错误条件逐项降级。</x:v>
+2026-10-04 待补受控持久运行账本正例与真实受管 Codex/Claude CLI（含 ephemeral/无持久会话）端到端；撤掉留存起点、启动/结束、连续水位、身份/维度、无错误条件逐项降级。
+2026-10-04 阶段一新增隔离合成脚本（计划命令 npm run test:case -- TC-077）：独立临时 SQLite/用户目录、固定假 CLI/无正文计量流；同一 macOS UID 下用管理员/普通 app 用户直调受管启动 IPC，依次尝试任意可执行文件、写入模式、额外标志/环境、未授权目录及符号链接逃逸。管理员在授权目录以固定只读/计划模式启动；对照可证/缺失/错配 provider 账号，重启服务并注入事件解析、落盘、心跳、水位故障。</x:v>
       </x:c>
       <x:c r="G82" s="55" t="str">
         <x:v>仅可证完整且无事实为真零；缺历史证据为部分/未知，不因其他工具成功而扩大所选范围。
 B/未归属无可证覆盖时为未知/部分而非真零；全局计数和最近扫描只能在另标“全局”的诊断中出现，不得充当当前筛选覆盖。只有所选用户/工具/时区/区间可证完整且空时才为已确认零；API/UI 一致。
 缺历史留存/连续采集证明时只能未知或有可证子区间时部分；空事实不写已确认零。仅 pending 事实允许已确认小计 0，但完整总量未知/不可确认；全局状态不补证。完整空窗真零属于最终目标，当前不构造或判通过。
 2026-10-03 覆盖证据决议：仅完整证据链支持所选来源 complete；范围外模式未知。关闭且同事实集空才显示限定“已确认零（所选已监测来源）”，不推服务商账单/全设备零。合成正例不使真实历史通过。
-仅在主动启用的受管来源、窗口封闭且 owner/provider/模型/项目/时区等全部可证时 complete；固定快照和范围外执行未知。</x:v>
+仅在主动启用的受管来源、窗口封闭且 owner/provider/模型/项目/时区等全部可证时 complete；固定快照和范围外执行未知。
+阶段一预期：viewer/越界或任意任务参数在 spawn 前拒绝，不借共享 macOS 凭证执行；actor 与 owner 分列，仅可证 provider 账号+绑定版本允许 owner_verified=true，缺证据为 false/空 owner，计量不进报表事实或 complete。run/event/heartbeat/水位持久，异常与不一致降级未知；无提示词/回复/原始流落盘。即使合成账本健康，本期仍无 complete 正例。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
-        <x:v>已注册；防假零保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
+        <x:v>旧保守防假零自动子断言已证；受管 CLI 阶段一授权/归属/账本新范围待实现和单编号复验，完整覆盖正例待验</x:v>
       </x:c>
       <x:c r="I82" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -9354,7 +9372,8 @@
 现行有无事实均标未知，有事实保留本范围计数/最近观察时间；单条事实不证明连续子区间完整；全局 ready 下双 owner+未归属及 viewer 的 API/UI 空事实防假零子断言已过。未验完整空窗真零、真实 Codex ephemeral/Claude OTel 缺输入端到端与全部来源路径。无事实 reason 在“未归属”筛选下仍称“没有已归属记录”，措辞待修。
 3bbaf15 已修正原“未归属”筛选下无事实 reason 的“已归属”措辞；仍不证明完整覆盖。
 2026-10-03 覆盖证据决议：现有保守负例结果保留。Codex --ephemeral 可无 rollout，Claude OTel 日志 exporter 可为 none；真实来源留存与连续性未证，TC-077 整项待验。
-真实 CLI 版本、结束语义、子代理及模型/项目字段、受管服务连续性尚需外部环境；不得以受控样本升真实覆盖。</x:v>
+真实 CLI 版本、结束语义、子代理及模型/项目字段、受管服务连续性尚需外部环境；不得以受控样本升真实覆盖。
+阶段一假 CLI 只验证授权、归属与账本 fail closed；真实 Codex/Claude 账户身份、输出协议、子代理/模型/项目字段和完整关闭窗留待后续真实工具正例，不能以合成状态提升覆盖。</x:v>
       </x:c>
       <x:c r="M82" s="55" t="str">
         <x:v>执行后记录固定提交、macOS/架构、测试数据版本、单编号命令、退出码和脱敏结果；当前无通过证据。
@@ -9384,17 +9403,19 @@
 管理员双 owner+未归属切换筛选：全局 ready、其他 owner 有最近成功扫描，而选中用户两个等长窗口之一缺证据或无事实；对照所选范围 API/as-of 和界面比较。
 本轮先造管理员选定 owner/未归属两期、全局 ready 但选中范围缺证、今天进行中与扫描滞后；核 API/界面保持不可比较。完整同 as-of 正例等待证据方案。
 2026-10-03 覆盖证据决议：计划受控合成双窗正例及单变量反例：两窗等长、同 owner/provider/筛选/来源范围、同 IANA 时区与 as-of 截止，双方各有完整证据链；破坏任一条件应不可比较。
-2026-10-04 待补两段真实受管关闭窗口，及受控等长/同范围/同 as-of 正例；注入掉线、晚到结束、时区实际不等长和范围外运行。</x:v>
+2026-10-04 待补两段真实受管关闭窗口，及受控等长/同范围/同 as-of 正例；注入掉线、晚到结束、时区实际不等长和范围外运行。
+2026-10-04 阶段一新增隔离合成脚本（计划命令 npm run test:case -- TC-078）：独立临时 SQLite/用户目录，用假 CLI 建两段已结束账本，分别使 owner_verified=false、仅 actor 可知、身份错配、事件/心跳缺口及服务重启水位不连续；按 owner/provider/窗口在授权 API 和 UI 查询比较。</x:v>
       </x:c>
       <x:c r="G83" s="58" t="str">
         <x:v>仅同来源/用户/时区、同长度、同 as-of 截止口径且可证覆盖时显示增减；不能用完整上期比未结束今天或扫描滞后的本期，否则显示不可比较。
 全局 ready/其他 owner 时间不能使当前筛选两期可比；缺覆盖显示不可比较。只有同用户范围/工具/时区、等长且同 as-of、两期完整才显示增减。
 没有双方完整且同截止的可证窗口时均显示不可比较，不能借别的 owner、全局最近扫描或最早事实补证。同比正例属最终目标，当前不伪造 complete。
 2026-10-03 覆盖证据决议：只有双方 source-complete 且双窗等长、同范围/时区/as-of 才显示比较；今天未结束、扫描滞后或范围外模式均不可比较。合成正例不证明真实历史。
-两窗各自完整且实际 UTC 时长相等、同 owner/provider/模式/模型/项目/IANA 时区及 as-of 才显示差值。</x:v>
+两窗各自完整且实际 UTC 时长相等、同 owner/provider/模式/模型/项目/IANA 时区及 as-of 才显示差值。
+阶段一预期：即使 run/event 已耐久且两窗等长，只要 provider owner 未可证或连续证据不全，比较一律不可比较，不能从 actor、macOS UID、空账本或一次合成运行推 complete；同比正例本期不判通过。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
-        <x:v>已注册；防假同比保守自动子断言通过（ef7a3de、语义修正 c10bbf3）；完整覆盖正例待验证，整项待验</x:v>
+        <x:v>旧保守防假同比自动子断言已证；受管账本/未知 owner 比较降级新范围待实现和单编号复验，双完整窗正例待验</x:v>
       </x:c>
       <x:c r="I83" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -9678,16 +9699,18 @@
         <x:v>独立库分别制造真零、未扫描、权限不足、格式不支持、筛选无匹配、部分覆盖。
 2026-10-03 本轮先逐项造未扫描、权限不足、格式不支持、筛选无匹配、覆盖未知、已观测但完整性未知；核授权范围、文案与行动。真零正例等待可证完整空窗，不在本轮造数或注入 complete。
 2026-10-03 覆盖证据决议：计划受控合成正例须经 REQ-040 所选 owner+provider+窗口的完整证据链，窗口已关闭且同一授权筛选事实集为空；逐项撤证及范围外模式作为负例。真实来源另验。
-2026-10-04 待补受控和真实守护服务连续有效、启动账本无运行的关闭空窗正例；范围外另运行真实命令核标签。</x:v>
+2026-10-04 待补受控和真实守护服务连续有效、启动账本无运行的关闭空窗正例；范围外另运行真实命令核标签。
+2026-10-04 阶段一新增隔离合成脚本（计划命令 npm run test:case -- TC-084）：独立临时 SQLite/用户目录、假 CLI 输出无正文标记；管理员发起后核当前窗口有完成/失败状态和可见结果或同会话安全打开动作，viewer 直调结果 IPC 拒绝；登出/切用户/关窗/重启后正文消失。检查 SQLite、诊断/应用日志和可选反馈附件无提示词、回复或原始流标记；身份未知、空账本、故障均显示覆盖未知及下一步。</x:v>
       </x:c>
       <x:c r="G89" s="58" t="str">
         <x:v>六类文案和操作不同；真零须完整覆盖证据；权限/格式/筛选动作指向可执行路径。
 保守子范围不得将筛选无匹配/空事实/单条已观测事实称真零或部分覆盖。真零未来须同一授权筛选范围 coverage.complete 且事实为空、有独立覆盖证据后另验。
 2026-10-03 覆盖证据决议：仅显示限定“已确认零（所选已监测来源）”；不宣称服务商账单/全设备零。未关闭、待核对、缺证或范围外模式不得真零。
-仅显示“已确认零（所选受管来源）”并列范围外未知；空心跳、空扫描、空快照、未知模型/项目不得真零。</x:v>
+仅显示“已确认零（所选受管来源）”并列范围外未知；空心跳、空扫描、空快照、未知模型/项目不得真零。
+阶段一预期：发起者可在当前授权会话看到结果/安全打开，异常有明确说明；正文只在有界内存，viewer 与持久库/日志/反馈附件不可得。受管身份未知或失败不能显示已确认零；真正关闭完整空窗正例仍待后续 REQ-040 证据。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
-        <x:v>已注册；保守空状态自动子范围通过，真零正例待 REQ-040 完整覆盖证据，整项待验</x:v>
+        <x:v>保守空状态自动子范围已证；受管结果可见/正文隐私阶段一待实现和单编号复验，完整空窗真零正例待验</x:v>
       </x:c>
       <x:c r="I89" s="58" t="str">
         <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。仅保守状态与筛选无匹配 UI 行动；完整空窗真零未验。此前“待注册/不可运行”是实施前记录。</x:v>
@@ -10651,7 +10674,8 @@
         <x:v>7fd0ce7 仅改测试：文档独立门禁 94/97/44、打包 5/5 与 44/44，通过。旧 2/5 和开发报告 1/5 为修复前测试失败。服务包 8773dd38… 完整性通过；TC-028/072 未验。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
-        <x:v>补真实生产账户/系统安装、来源归属和迁移验收；具备签名、公证、另一台目标 Mac 后执行 TC-028/072。保留旧失败及对应固定提交证据。</x:v>
+        <x:v>补真实生产账户/系统安装、来源归属和迁移验收；具备签名、公证、另一台目标 Mac 后执行 TC-028/072。保留旧失败及对应固定提交证据。
+REQ-023/TC-076 另需核点击开始后下载至安装均无取消与故障自动回退；真实系统/生产环境待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="142.5" customHeight="1">
@@ -10680,18 +10704,21 @@
         <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺
 当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。
 当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。
-7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。</x:v>
+7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。
+受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
         <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
-        <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。</x:v>
+        <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。
+2026-10-04 仅补 REQ-040/044→DEV-049/053→TC-077/078/084 阶段一合同；无新代码、无新增动态通过。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
 当前只要求本机未签名临时候选可用；资源具备后仍须完成 TC-028/072，REQ-018/035 目标未删除。
-REQ-023/TC-076 按用户决议收敛：安装前可放弃、安装开始后不可取消、失败自动恢复；独立取消控制窗口不属本轮。</x:v>
+REQ-023/TC-076 前次决议（由下方点击边界取代）：安装前可放弃、安装开始后不可取消、失败自动恢复；独立取消控制窗口不属本轮。
+REQ-023/TC-076 最新边界为点击开始前可放弃、点击后直到成功/回退均不可取消；不交付取消控制窗口/协议/journal/分阶段正例。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: define current Mac acceptance and TC-095
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R522a0b8c159947f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb8ab2579fdba499e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3451773e901a4009"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rde4d62ac0b334cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Reb0ff4778a7b4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rfe2c651a5ad449b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1e08cc5f7e87486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa235d39cf7b4ce6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Red4c17a792c44616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rc68ab3c536344ebf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="38">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -261,6 +261,11 @@
         <x:fgColor rgb="FFF0F3F6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -291,7 +296,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="98">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -539,6 +544,13 @@
     <x:xf numFmtId="0" fontId="9" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -769,7 +781,8 @@
         <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
 当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。
 2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。
-版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。</x:v>
+版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。
+2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3060,6 +3073,30 @@
 2026-10-04 TC-094 新增 Claude unknown 或累计降级后的首次 flush 前快照重算与在线旧聚合清理/降级，待验。
 2026-10-04 TC-094 真实 Electron 启动发送竞态当前失败：迁移首包成功后扫描新 revision 未立即续传；需自动 drain 到服务确认最新 revision 并清旧 owner 聚合，不靠 60 秒定时器。
 508851a：TC-094 单元 2/2、Electron 1/1 独立通过；真实生产迁移/旧服务待验；详情见测试用例 I/L/M 列与 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="170" customHeight="1">
+      <x:c r="A101" s="97" t="str">
+        <x:v>REQ-017（关联 REQ-002、REQ-004、REQ-005、REQ-006、REQ-011–015、REQ-023、REQ-035）</x:v>
+      </x:c>
+      <x:c r="B101" s="97" t="str">
+        <x:v>本机开发版打包及当前 Mac 实装可用</x:v>
+      </x:c>
+      <x:c r="C101" s="97" t="str">
+        <x:v>DEV-017（关联 DEV-002、DEV-004、DEV-005、DEV-006、DEV-011–015、DEV-025、DEV-040）</x:v>
+      </x:c>
+      <x:c r="D101" s="97" t="str">
+        <x:v>构建并验证本机 DMG 与关联功能</x:v>
+      </x:c>
+      <x:c r="E101" s="97" t="str">
+        <x:v>TC-095</x:v>
+      </x:c>
+      <x:c r="F101" s="97" t="str">
+        <x:v>当前 Mac 实际安装与本机可用人工验收</x:v>
+      </x:c>
+      <x:c r="G101" s="97" t="str">
+        <x:v>2026-10-04 新增独立本机发布验收；入口待注册、人工未执行，真实安装/登录/权限/采集/报表/CSV/升级故障恢复/数据保留与回退均待证。TC-028/072 不属本次本机门槛，仍各自待验。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3580,17 +3617,19 @@
         <x:v>M4</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>已验证（0.3.4 本机隔离挂载/复制与主流程；Finder、生产安装待验）</x:v>
+        <x:v>本机隔离 DMG 子范围已验证；当前 Mac 实际安装与完整可用流程 TC-095 待注册/待人工验收</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
         <x:v>DEV-017</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
-        <x:v>TC-027</x:v>
+        <x:v>TC-027、TC-095</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
         <x:v>历史：docs/validation.md A10；v0.3.0：同文 TC-027 新批次，本机未签名 DMG 人工 pass（2026-10-02）
-2026-10-03：代码 7abd640 的 0.3.4 未签名 DMG 在 macOS 15.7.4 x86_64 以独立临时库/人工 Codex JSONL 挂载、ditto 复制、启动，受信登录、扫描和 1280 Token 报表通过；TC-027 人工 pass 登记时间 2026-10-02T20:46:08.228Z，证据见 docs/validation.md。Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 待验。</x:v>
+2026-10-03：代码 7abd640 的 0.3.4 未签名 DMG 在 macOS 15.7.4 x86_64 以独立临时库/人工 Codex JSONL 挂载、ditto 复制、启动，受信登录、扫描和 1280 Token 报表通过；TC-027 人工 pass 登记时间 2026-10-02T20:46:08.228Z，证据见 docs/validation.md。Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 待验。
+2026-10-04 本机交付决议：REQ-017 不以其他 Mac/Developer ID/公证为当前门槛；新增 TC-095 独立核当前 Mac 真实安装、启动、管理员登录、来源权限/采集、报表/CSV、升级故障恢复、用户数据保留和可用旧版回退。既有 TC-027 隔离子范围不代证真实安装；生产 userData 不得由自动测试改写。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -3755,7 +3794,7 @@
         <x:v>DEV-025</x:v>
       </x:c>
       <x:c r="G28" s="14" t="str">
-        <x:v>TC-036、TC-076</x:v>
+        <x:v>TC-036、TC-076、TC-095</x:v>
       </x:c>
       <x:c r="H28" s="70" t="str">
         <x:v>当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
@@ -3767,7 +3806,8 @@
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 当前新包取干净 main 9af351a，SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；旧 d99d7af9 包的 TC-076 故障证据不外推。
 2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
-2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 当前隔离成功/五故障自动恢复证据继续有效；未知的系统目录、真实满盘/断电与目标 Mac 不升为通过。</x:v>
+2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 当前隔离成功/五故障自动恢复证据继续有效；未知的系统目录、真实满盘/断电与目标 Mac 不升为通过。
+2026-10-04 TC-095 负责当前 Mac 真实安装/更新故障恢复与数据保留的人工发布验收；TC-076 隔离自动故障证据继续有效，不替代系统位置和现有用户数据保护。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -4073,17 +4113,18 @@
         <x:v>M6（本机实现）</x:v>
       </x:c>
       <x:c r="E40" s="36" t="str">
-        <x:v>代码已落地（TC-072 目标 Mac 待验）</x:v>
+        <x:v>代码已落地；当前 Mac 权限/采集人工 TC-095 待验，异机 TC-072 保留未来待验</x:v>
       </x:c>
       <x:c r="F40" s="36" t="str">
         <x:v>DEV-040</x:v>
       </x:c>
       <x:c r="G40" s="36" t="str">
-        <x:v>TC-060、TC-061、TC-072</x:v>
+        <x:v>TC-060、TC-061、TC-072、TC-095</x:v>
       </x:c>
       <x:c r="H40" s="36" t="str">
         <x:v>代码 6223c30；自动覆盖见 docs/validation.md；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 明确目标 Mac 拒绝→授予→撤销→重扫闭环；原自动模拟结果不代替真实系统证据。
-2026-10-04 当前无第二台目标 Mac；TC-072 拒绝/授予/撤销/重扫人工闭环仍待验证，现阶段本机临时测试不改变 REQ-035 目标。</x:v>
+2026-10-04 当前无第二台目标 Mac；TC-072 拒绝/授予/撤销/重扫人工闭环仍待验证，现阶段本机临时测试不改变 REQ-035 目标。
+2026-10-04 TC-095 另核当前 Mac 授权/拒绝/重扫与可观察采集；TC-072 仍保留第二台目标 Mac 独立账户权限闭环，退出当前本机交付门槛且待验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="66" customHeight="1">
@@ -4972,17 +5013,18 @@
         <x:v>REQ-017</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>TC-027</x:v>
+        <x:v>TC-027、TC-095</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
         <x:v>scripts/package-dmg.mjs；package.json；release/</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>已完成（0.3.4 本机隔离子范围人工通过；Finder、生产安装待验）</x:v>
+        <x:v>0.3.4 本机隔离打包子范围已证；当前 Mac 实际安装与完整可用流程 TC-095 待注册/验收</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
         <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md
-0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。</x:v>
+0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。
+2026-10-04 本机交付任务：在 scripts/test-cases.mjs 注册独立 TC-095 人工清单；冻结候选代码/未签名 DMG 与 SHA/架构，隔离副本先做升级故障回退，当前 Mac 实装与 UI 人工核对另留脱敏证据。不得让自动脚本指向或改写现有生产 userData。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5167,7 +5209,7 @@
         <x:v>REQ-023</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>TC-036、TC-076</x:v>
+        <x:v>TC-036、TC-076、TC-095</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
         <x:v>src/main/update-client.ts、update-launch.ts、update-helper.ts、update-install.ts、index.ts；tests/next-update.test.ts、update-install.test.ts；scripts/verify-auto-upgrade.mjs；scripts/test-cases.mjs；本机 0.3.5 未签名 DMG 和隔离/人工接管记录</x:v>
@@ -5185,7 +5227,8 @@
 2026-10-04 审阅收紧：原 REQ-023 与 TC-076 已含取消/回退，沿用编号。空 userData 仅证二进制可启动；成功提交前须在 owner-only 真实 userData 一致副本演练旧库迁移、受信状态和用量可读，取消时真实目录不变，副本演练失败须在替换前中止。正式迁移若仍失败，保留 bundle 外恢复入口与真实数据备份，不把探测通过称完整保证。
 2026-10-04 前次决议（已被下方最新点击边界取代，仅供追溯）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 前文“独立窗口/阶段取消”为旧计划；开发工作树未提交实验不算候选。当前新包 SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2，包校验通过，安装功能新证据待补。
 2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
-2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 产品/测试不得把下载阶段可取消写成承诺；旧取消控制窗口、取消协议及取消 journal 不属本轮。</x:v>
+2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 产品/测试不得把下载阶段可取消写成承诺；旧取消控制窗口、取消协议及取消 journal 不属本轮。
+2026-10-04 TC-095 本机实装门槛：发布候选的正常更新与故障后旧版可用/数据保留须在当前 Mac 人工核查；真实故障注入先在隔离 App/userData 副本中验证，不对生产目录执行自动注入。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="62" customHeight="1">
@@ -5523,16 +5566,17 @@
         <x:v>REQ-035</x:v>
       </x:c>
       <x:c r="D45" s="37" t="str">
-        <x:v>TC-060、TC-061、TC-072</x:v>
+        <x:v>TC-060、TC-061、TC-072、TC-095</x:v>
       </x:c>
       <x:c r="E45" s="37" t="str">
         <x:v>src/renderer/settings.tsx；src/main/index.ts；tests/e2e/m6-settings.spec.ts</x:v>
       </x:c>
       <x:c r="F45" s="37" t="str">
-        <x:v>已编码（TC-072 人工待验）</x:v>
+        <x:v>已编码；当前 Mac TC-095 人工权限/采集待验，异机 TC-072 待验</x:v>
       </x:c>
       <x:c r="G45" s="37" t="str">
-        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 真实目标 Mac 文件权限拒绝、授予、撤销及重扫继续待验，所需系统版本/截图/日志须脱敏。</x:v>
+        <x:v>提交 6223c30；TC-050–071 逐编号自动日志见 test-results/acceptance/；完整边界见 docs/test-case-acceptance.md；2026-10-03 批次三：TC-072 真实目标 Mac 文件权限拒绝、授予、撤销及重扫继续待验，所需系统版本/截图/日志须脱敏。
+2026-10-04 当前 Mac 文件权限和来源可用性由 TC-095 手工留证；不将 TC-072 异机拒绝/授予/撤销变成此次本机门槛或已通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="66" customHeight="1">
@@ -6031,7 +6075,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–094 共 94 个编号，均已注册；人工与发布验收按各行证据判定。</x:v>
+        <x:v>TC-001–095 共 95 个编号；TC-001–094 已注册，TC-095 为待注册本机人工用例。人工与发布验收按各行证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -7264,7 +7308,8 @@
       </x:c>
       <x:c r="L33" s="30" t="str">
         <x:v>人工入口；待验证
-当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。</x:v>
+当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。
+2026-10-04 外部分发 TC-028 不属当前 Mac 未签名本机交付门槛；真实 Developer ID、公证、Gatekeeper 和异机仍待验证，不得标 pass。</x:v>
       </x:c>
       <x:c r="M33" s="27" t="str">
         <x:v>运行 npm run test:case -- TC-028 仅输出人工清单、退出码 2；实际验收需同一签名候选的 App/DMG、脱敏 Developer ID 身份、公证和票据/Gatekeeper 核验、包大小/SHA-256、目标 Mac 版本/架构与安装、启动、登录、采集记录。当前无 pass 证据，不得借用 TC-075 1/1 或 0.3.4 未签名包。
@@ -9110,7 +9155,8 @@
       </x:c>
       <x:c r="L77" s="37" t="str">
         <x:v>入口仅显示操作步骤；未执行目标 Mac 授权、撤销和重新扫描。；新增目标还须实测撤销后的状态/重扫。
-当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。</x:v>
+当前资源边界仅影响可执行环境，不删除原用例目标，也不把未签名/本机测试当作目标设备验收。
+2026-10-04 异机 TC-072 不属当前 Mac 未签名本机交付门槛；第二台 Mac 独立账户权限闭环仍待验证，不得标 pass。</x:v>
       </x:c>
       <x:c r="M77" s="37" t="str">
         <x:v>目标 Mac 的独立测试账户/专用 token-test-db-tc072-*；先拒绝，再手动授予、重扫并撤销；保存脱敏截图和系统版本。
@@ -10292,6 +10338,49 @@
         <x:v>8157e2d；macOS 本机专用临时客户端/服务 SQLite；单编号 1/1 退出码 0，门禁 82 入口/56 单元/22 Electron 通过。
 508851a；macOS 15.7.4 x86_64、Node v24.15.0；单元 2/2、Electron 1/1，exit 0；首次真实 Electron 启动前重算 v2 待传，在线清旧 owner 聚合。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。
 7fd0ce7；macOS 15.7.4 x86_64、Node v24.15.0；TC-094 单编号 2 单元+1 Electron、test:gate 94/97/44、打包全量 44/44，均 exit 0；生产迁移/真实旧服务仍未验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="315" customHeight="1">
+      <x:c r="A100" s="97" t="str">
+        <x:v>TC-095</x:v>
+      </x:c>
+      <x:c r="B100" s="97" t="str">
+        <x:v>REQ-017；关联 REQ-002、REQ-004、REQ-005、REQ-006、REQ-011–015、REQ-023、REQ-035</x:v>
+      </x:c>
+      <x:c r="C100" s="97" t="str">
+        <x:v>DEV-017；关联 DEV-002、DEV-004、DEV-005、DEV-006、DEV-011–015、DEV-025、DEV-040</x:v>
+      </x:c>
+      <x:c r="D100" s="97" t="str">
+        <x:v>当前 Mac 实际安装与本机可用人工验收</x:v>
+      </x:c>
+      <x:c r="E100" s="97" t="str">
+        <x:v>当前 Mac 人工／真实安装</x:v>
+      </x:c>
+      <x:c r="F100" s="97" t="str">
+        <x:v>固定代码、版本、架构和未签名 DMG SHA-256/hdiutil；确认此 Mac 安装目标及原 App/数据备份位置。仅用授权的人工操作从 DMG 安装到实际 /Applications 或 ~/Applications，启动并登录管理员；以当前账户可访问的授权来源检查无权限/授权后重扫、Codex/Claude 可观察记录、来源归属、报表筛选/明细与 CSV 同一快照。用专用隔离 App/userData 副本做更新坏包与五故障恢复，核旧版可启动/数据可读并可重试；生产 App 如升级，只在备份确认后人工点击“开始升级”，核点击前可放弃、点击后无取消直到成功/自动回退。升级前后以脱敏计数/只读校验核现有数据保留；回退旧版只用已验证兼容备份或明确人工恢复路径，不直接以旧程序打开已迁移的新库。不得由自动脚本写现有生产 userData。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+      </x:c>
+      <x:c r="G100" s="97" t="str">
+        <x:v>同一固定候选在当前 Mac 完成实际安装、启动、管理员登录；权限拒绝/授权后的状态和重扫正确，采集与归属不越权，报表/明细/CSV 一致且未知不写零。安装/更新失败后旧版可用、数据和受信状态保留或明确重新登录；无残留误报，备份与兼容回退路径可执行。失败/空数据有可操作说明；任何缺证项为待验，不以隔离测试替代实际安装。</x:v>
+      </x:c>
+      <x:c r="H100" s="97" t="str">
+        <x:v>待注册、待人工执行；当前本机交付门槛未通过</x:v>
+      </x:c>
+      <x:c r="I100" s="97" t="str">
+        <x:v>2026-10-04 SOP-001 文档立项，未修改产品/测试代码，未触碰生产 userData；既有 TC-027/076 的本机隔离结果不能代证 TC-095。当前 /Applications/Token.app 曾核为 0.3.5，0.3.6 候选包 SHA 8773dd38…；以执行当天冻结制品为准。</x:v>
+      </x:c>
+      <x:c r="J100" s="97" t="str">
+        <x:v>计划：npm run test:case -- TC-095；完成人工验收后 npm run test:case -- TC-095 pass /绝对路径/脱敏证据文件（失败用 fail）；注册前不可执行或登记 pass</x:v>
+      </x:c>
+      <x:c r="K100" s="97" t="str">
+        <x:v>待开发会话在 scripts/test-cases.mjs 注册 manual 清单；只输出步骤并记录人工证据，不执行安装、授权、生产库写入或故障注入</x:v>
+      </x:c>
+      <x:c r="L100" s="97" t="str">
+        <x:v>无自动通过；需分别记录真实当前 Mac 安装路径与 UI、隔离故障回退及生产数据只读前后核对。TC-028/072 仍为未来外部分发待验，不据本项通过。</x:v>
+      </x:c>
+      <x:c r="M100" s="97" t="str">
+        <x:v>证据建议 test-results/manual/evidence/TC-095-local-mac-acceptance.md（被 Git 忽略的绝对路径）；记录固定提交/DMG SHA、macOS/架构、安装前后版本与路径、脱敏截图、权限/采集/报表/CSV 的范围和数值、备份摘要、隔离故障回退结果及原 App/数据恢复步骤；不存真实 JSONL/SQLite/密钥/提示词正文。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10653,29 +10742,36 @@
         <x:v>当前修复与产品打磨</x:v>
       </x:c>
       <x:c r="D13" s="89" t="str">
-        <x:v>真实 0.3.5→0.3.6 隔离升级；来源身份隔离、Claude 逐文件队列、v2 迁移、快照续传</x:v>
+        <x:v>真实 0.3.5→0.3.6 隔离升级；来源身份隔离、Claude 逐文件队列、v2 迁移、快照续传
+当前 Mac 实际安装、管理员登录、授权来源采集、报表/CSV 与升级数据保留/回退另列 TC-095；未完成。</x:v>
       </x:c>
       <x:c r="E13" s="89" t="str">
-        <x:v>REQ-023、REQ-026、REQ-040–048</x:v>
+        <x:v>REQ-023、REQ-026、REQ-040–048
+REQ-017/035；关联 REQ-002/004/005/006/011–015</x:v>
       </x:c>
       <x:c r="F13" s="89" t="str">
-        <x:v>DEV-025、DEV-028、DEV-049–057</x:v>
+        <x:v>DEV-025、DEV-028、DEV-049–057
+DEV-017/040；关联 DEV-002/004/005/006/011–015</x:v>
       </x:c>
       <x:c r="G13" s="89" t="str">
-        <x:v>TC-040、TC-076–094</x:v>
+        <x:v>TC-040、TC-076–094
+TC-095（待注册/人工执行）</x:v>
       </x:c>
       <x:c r="H13" s="89" t="str">
-        <x:v>0.3.6 本机未签名候选：7fd0ce7 测试定位修复后 TC-079/021/094 与源码门禁、目录包无重试五次及全量通过；TC-076 隔离升级/回退已证；系统/生产/外部验收待补</x:v>
+        <x:v>0.3.6 本机未签名候选：7fd0ce7 测试定位修复后 TC-079/021/094 与源码门禁、目录包无重试五次及全量通过；TC-076 隔离升级/回退已证；系统/生产/外部验收待补
+TC-095 当前 Mac 真实安装与完整可用流程待人工验收；TC-028/072 异机不属此次本机门槛。</x:v>
       </x:c>
       <x:c r="I13" s="89" t="str">
-        <x:v>本机候选自动与打包子范围通过；完整版本/公开分发验收未完成</x:v>
+        <x:v>本机自动/隔离打包子范围通过；当前 Mac 实际安装 TC-095 未验，故本机交付未完成；外部分发独立待验</x:v>
       </x:c>
       <x:c r="J13" s="89" t="str">
         <x:v>7fd0ce7 仅改测试：文档独立门禁 94/97/44、打包 5/5 与 44/44，通过。旧 2/5 和开发报告 1/5 为修复前测试失败。服务包 8773dd38… 完整性通过；TC-028/072 未验。</x:v>
       </x:c>
       <x:c r="K13" s="89" t="str">
         <x:v>补真实生产账户/系统安装、来源归属和迁移验收；具备签名、公证、另一台目标 Mac 后执行 TC-028/072。保留旧失败及对应固定提交证据。
-REQ-023/TC-076 另需核点击开始后下载至安装均无取消与故障自动回退；真实系统/生产环境待验。</x:v>
+REQ-023/TC-076 另需核点击开始后下载至安装均无取消与故障自动回退；真实系统/生产环境待验。
+先注册并执行 TC-095 本机人工验收，留固定候选和脱敏证据；生产库只读核对，自动测试仅用隔离副本。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="142.5" customHeight="1">
@@ -10689,16 +10785,20 @@
         <x:v>三批打磨及当前发布门槛</x:v>
       </x:c>
       <x:c r="D14" s="90" t="str">
-        <x:v>修复打包日期回退；补完整覆盖/真零与同比、空状态、真实服务状态、VoiceOver、Claude 外部归属、生产迁移、安装开始后不可取消、失败自动回退和目标 Mac 发布证据</x:v>
+        <x:v>修复打包日期回退；补完整覆盖/真零与同比、空状态、真实服务状态、VoiceOver、Claude 外部归属、生产迁移、安装开始后不可取消、失败自动回退和目标 Mac 发布证据
+2026-10-04 当前交付目标收窄为这台 Mac 的未签名本机可用；具体真实安装、管理员登录、权限、采集、报表/CSV、更新故障和数据保留/回退由 TC-095 判定。旧异机发布文字仅为未来目标。</x:v>
       </x:c>
       <x:c r="E14" s="90" t="str">
-        <x:v>REQ-023、REQ-040–048</x:v>
+        <x:v>REQ-023、REQ-040–048
+当前本机门槛关联 REQ-017/023/035；REQ-018 外部分发目标保留但不在本次门槛。</x:v>
       </x:c>
       <x:c r="F14" s="90" t="str">
-        <x:v>DEV-025、DEV-049–057</x:v>
+        <x:v>DEV-025、DEV-049–057
+当前本机门槛关联 DEV-017/025/040；DEV-018 外部分发任务保留但不在本次门槛。</x:v>
       </x:c>
       <x:c r="G14" s="90" t="str">
-        <x:v>TC-021、TC-028、TC-072、TC-076–094</x:v>
+        <x:v>TC-021、TC-028、TC-072、TC-076–094
+TC-095 当前 Mac 独立人工验收；TC-028/072 保留未来待验，不纳入本次本机通过判定。</x:v>
       </x:c>
       <x:c r="H14" s="90" t="str">
         <x:v>当前三批全范围代码/自动子范围持续推进；TC-080–083/085/090 等已有隔离证据，外部/打包与部分完整验收仍缺
@@ -10708,17 +10808,20 @@
 受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>当前目标收尾中；本机临时可用可继续测试，完整交付门槛未通过</x:v>
+        <x:v>当前 Mac 未签名本机交付待验：TC-095 未注册/未执行，实际安装与生产数据保护未证；外部分发仍待验</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
         <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。
-2026-10-04 仅补 REQ-040/044→DEV-049/053→TC-077/078/084 阶段一合同；无新代码、无新增动态通过。</x:v>
+2026-10-04 仅补 REQ-040/044→DEV-049/053→TC-077/078/084 阶段一合同；无新代码、无新增动态通过。
+2026-10-04 仅调整范围和追溯、分配 TC-095；无本机实装或生产数据动态通过。TC-028/072 均保持待验。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
 当前只要求本机未签名临时候选可用；资源具备后仍须完成 TC-028/072，REQ-018/035 目标未删除。
 REQ-023/TC-076 前次决议（由下方点击边界取代）：安装前可放弃、安装开始后不可取消、失败自动恢复；独立取消控制窗口不属本轮。
-REQ-023/TC-076 最新边界为点击开始前可放弃、点击后直到成功/回退均不可取消；不交付取消控制窗口/协议/journal/分阶段正例。</x:v>
+REQ-023/TC-076 最新边界为点击开始前可放弃、点击后直到成功/回退均不可取消；不交付取消控制窗口/协议/journal/分阶段正例。
+当前优先注册并人工执行 TC-095；同一候选完成当前 Mac 真安装、权限、采集、报表/CSV、升级恢复、只读数据核对和兼容回退证据。Developer ID/公证/第二台 Mac 资源具备后另走 TC-028/072。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: define TC-095 legacy migration acceptance and candidate evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rfe2c651a5ad449b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R1e08cc5f7e87486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa235d39cf7b4ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Red4c17a792c44616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rc68ab3c536344ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R34bd07ab2b764a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra88eeef5f91646e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7e392d2da15a47ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rddbc88359f274872"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R805c400df00345b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2637,7 +2637,8 @@
         <x:v>TC-077 已注册；防假零保守单元+Electron 子断言通过（ef7a3de）；完整空窗真零正例待证据方案，REQ-040 整项待验
 2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
 2026-10-04 受管持续采集设计已决，TC-077 受控和真实 CLI 正例未实施；整项待验。
-2026-10-04 TC-077：阶段一新增管理员受限 CLI、viewer/越界拒绝、actor≠owner、账本失效负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
+2026-10-04 TC-077：阶段一新增管理员受限 CLI、viewer/越界拒绝、actor≠owner、账本失效负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。
+2026-10-04 c359e6a 受管 CLI 阶段一相应单编号由开发会话报告通过；真实 provider owner/complete/真零/同比正例仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="135" customHeight="1">
@@ -2663,7 +2664,8 @@
         <x:v>TC-078 已注册；防假同比保守单元+Electron 子断言通过（ef7a3de）；同 as-of 双完整窗口正例待证据方案，REQ-040 整项待验
 2026-10-03 覆盖证据决议：真实来源完整性仍未证明；受控合成只验规则。REQ-040/DEV-049/TC-077/078 整项待验。
 2026-10-04 TC-078 双关闭等长完整窗口受控/真实正例待实施，范围外未知；整项待验。
-2026-10-04 TC-078：阶段一新增未知 owner/水位缺口仍不可比负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
+2026-10-04 TC-078：阶段一新增未知 owner/水位缺口仍不可比负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。
+2026-10-04 c359e6a 受管 CLI 阶段一相应单编号由开发会话报告通过；真实 provider owner/complete/真零/同比正例仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="85" customHeight="1">
@@ -2807,7 +2809,8 @@
         <x:v>TC-084 已注册：单元+Electron 保守空状态子范围通过；同范围 complete 真零正例待 REQ-040，整项待验
 2026-10-03 覆盖证据决议：真零须已关闭同范围完整空窗；合成只验规则，真实来源未证；REQ-044/DEV-053/TC-084 整项待验。
 2026-10-04 TC-084 受管关闭空窗真零正例待实施，固定快照/空心跳不能补证；整项待验。
-2026-10-04 TC-084：阶段一新增管理员结果可见、正文仅内存与空状态负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。</x:v>
+2026-10-04 TC-084：阶段一新增管理员结果可见、正文仅内存与空状态负例；待实现/执行。 不新增编号，complete/真零/同比正例未验。
+2026-10-04 c359e6a 受管 CLI 阶段一相应单编号由开发会话报告通过；真实 provider owner/complete/真零/同比正例仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="85" customHeight="1">
@@ -3095,8 +3098,12 @@
         <x:v>当前 Mac 实际安装与本机可用人工验收</x:v>
       </x:c>
       <x:c r="G101" s="97" t="str">
-        <x:v>2026-10-04 新增独立本机发布验收；入口待注册、人工未执行，真实安装/登录/权限/采集/报表/CSV/升级故障恢复/数据保留与回退均待证。TC-028/072 不属本次本机门槛，仍各自待验。
-2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+        <x:v>2026-10-04 立项时新增独立本机发布验收、入口待注册；c359e6a 已注册人工入口，至今未人工执行，真实安装/登录/权限/采集/报表/CSV/升级故障恢复/数据保留与回退均待证。TC-028/072 不属本次本机门槛，仍各自待验。
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
+2026-10-04 TC-095 旧库隔离副本启动出现 source_identities 净变化；目前仅知 users/facts/cursors 数量不变及 integrity_check=ok，未证明逐键/归属/报表安全。脚本全表计数全等断言需改为可解释白名单迁移对账，TC-095 仍待验。
+2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
+证据来源：需求会话独立做旧/新打包 App 同一备份副本对照；开发会话核代码/SQL。c359e6a 已注册 TC-095 人工清单，但实际本机安装与完整验收待执行。
+TC-095 保守迁移允许旧本机键→scoped v2、旧 claude:macos 退役/待核对和有因游标清零；逐事实/权限/界面及兼容备份仍是通过条件，不因摘要一致升为完整验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3629,7 +3636,8 @@
         <x:v>历史：docs/validation.md A10；v0.3.0：同文 TC-027 新批次，本机未签名 DMG 人工 pass（2026-10-02）
 2026-10-03：代码 7abd640 的 0.3.4 未签名 DMG 在 macOS 15.7.4 x86_64 以独立临时库/人工 Codex JSONL 挂载、ditto 复制、启动，受信登录、扫描和 1280 Token 报表通过；TC-027 人工 pass 登记时间 2026-10-02T20:46:08.228Z，证据见 docs/validation.md。Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 待验。
 2026-10-04 本机交付决议：REQ-017 不以其他 Mac/Developer ID/公证为当前门槛；新增 TC-095 独立核当前 Mac 真实安装、启动、管理员登录、来源权限/采集、报表/CSV、升级故障恢复、用户数据保留和可用旧版回退。既有 TC-027 隔离子范围不代证真实安装；生产 userData 不得由自动测试改写。
-2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
+2026-10-04 TC-095 旧生产库副本允许可证 legacy-unverified 身份隔离导致身份行变化，但逐事实数值、归属权限与报表范围须对账；单纯完整性 ok/数量不变不构成通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -4249,7 +4257,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E45" s="55" t="str">
-        <x:v>保守未知/防假零自动子范围已证；受管 CLI 阶段一授权/归属/账本未实现，完整覆盖与同比正例待验</x:v>
+        <x:v>保守防假零子范围及受管 CLI 阶段一隔离自动子范围通过（开发报告 c359e6a）；可证 owner、完整窗/同比正例待验</x:v>
       </x:c>
       <x:c r="F45" s="55" t="str">
         <x:v>DEV-049</x:v>
@@ -4266,7 +4274,8 @@
 3bbaf15 将无事实原因改为“没有已观测记录”，适用于管理员“未归属”筛选；文档会话独立复跑 TC-077 单元+Electron 通过。REQ-040 的完整历史覆盖与真零/同比正例仍待验。
 2026-10-03 覆盖证据决议：现有状态/游标/事实仅证已观察；受控合成正例只验规则，不证明真实 Codex/Claude 来源完整。真实来源机制未落实，整项仍待验。官方：https://learn.chatgpt.com/docs/developer-commands?surface=cli 与 https://code.claude.com/docs/en/monitoring-usage
 2026-10-04 设计决议：用户主动启用受管会话；持久启动/结束账本、逐事件用量与守护连续水位按 owner/provider/模型/项目/IANA 时区/关闭窗口 fail closed。文件快照仅证重放；普通本机全部使用量及范围外仍未知。见 docs/coverage-evidence-decision.md；未实施、未验真实正例。
-阶段一沿用 REQ-040→DEV-049→TC-077/078；CLI 执行安全与可证 owner 是受管来源范围成立的前置条件，新增断言仍待注册/执行。</x:v>
+阶段一沿用 REQ-040→DEV-049→TC-077/078；CLI 执行安全与可证 owner 是受管来源范围成立的前置条件，新增断言仍待注册/执行。
+2026-10-04 c359e6a（开发会话报告，文档会话待独立复跑）：0.3.7 管理员显式启用的受限只读/计划 Codex/Claude CLI 入口、受控目录与符号链接复核、固定参数/环境、run/event/heartbeat/水位耐久账本、未知 owner 不进报表、正文仅当前窗口并在登出/关窗清除已编码；TC-077/078/084 各单编号通过。有效 provider owner 身份、真实 CLI 正例、source-complete/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="150" customHeight="1">
@@ -4373,7 +4382,7 @@
         <x:v>下一轮产品打磨（计划）</x:v>
       </x:c>
       <x:c r="E49" s="55" t="str">
-        <x:v>保守空状态与进度/取消/重试自动子范围通过；受管结果可见/正文隐私阶段一未实现，真零待 REQ-040 证据</x:v>
+        <x:v>保守空状态及受管结果仅当前窗口子范围通过（开发报告 c359e6a）；真实完整空窗真零待验</x:v>
       </x:c>
       <x:c r="F49" s="55" t="str">
         <x:v>DEV-053</x:v>
@@ -4388,7 +4397,8 @@
 2026-10-03 代码 90338f4：文档会话独立复跑 TC-085 5 单元+2 Electron、TC-087 及完整门禁（90 入口、70 单元、31 Electron）通过。取消/续扫已实现，TC-084 真零仍待同授权范围完整覆盖证据；生产库/打包未验。
 2026-10-03 覆盖证据决议：TC-084 可计划受控合成规则正例；真实来源完整性、范围外执行模式和实际空窗未验，REQ-044 整项待验。
 2026-10-04 真零仅限同一授权受管来源关闭空窗、启动账本和连续采集可证、事实集为空；界面标范围外未知。TC-084 受控和真实正例待实现/验收。
-阶段一沿用 REQ-044→DEV-053→TC-084；结果可见性/短暂内存与空状态为现有用户可操作性目标的细化，不新增编号；真实 CLI 与真零正例仍待验。</x:v>
+阶段一沿用 REQ-044→DEV-053→TC-084；结果可见性/短暂内存与空状态为现有用户可操作性目标的细化，不新增编号；真实 CLI 与真零正例仍待验。
+2026-10-04 c359e6a（开发会话报告，文档会话待独立复跑）：0.3.7 管理员显式启用的受限只读/计划 Codex/Claude CLI 入口、受控目录与符号链接复核、固定参数/环境、run/event/heartbeat/水位耐久账本、未知 owner 不进报表、正文仅当前窗口并在登出/关窗清除已编码；TC-077/078/084 各单编号通过。有效 provider owner 身份、真实 CLI 正例、source-complete/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="150" customHeight="1">
@@ -5024,7 +5034,8 @@
       <x:c r="G22" s="9" t="str">
         <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md
 0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。
-2026-10-04 本机交付任务：在 scripts/test-cases.mjs 注册独立 TC-095 人工清单；冻结候选代码/未签名 DMG 与 SHA/架构，隔离副本先做升级故障回退，当前 Mac 实装与 UI 人工核对另留脱敏证据。不得让自动脚本指向或改写现有生产 userData。</x:v>
+2026-10-04 本机交付任务：在 scripts/test-cases.mjs 注册独立 TC-095 人工清单；冻结候选代码/未签名 DMG 与 SHA/架构，隔离副本先做升级故障回退，当前 Mac 实装与 UI 人工核对另留脱敏证据。不得让自动脚本指向或改写现有生产 userData。
+2026-10-04 verify-production-copy.mjs 原指纹要求 identities 全等，当前隔离副本报告 净变化；开发应仅在有逐条 legacy-unverified 映射、事实/小计/权限和旧版兼容备份证据时调整断言，不能允许任意新行。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5782,7 +5793,7 @@
 另核 src/renderer/report.tsx 的 coverage 与 src/main/index.ts 的授权报表 IPC；全局诊断若保留需显式标范围。</x:v>
       </x:c>
       <x:c r="F54" s="55" t="str">
-        <x:v>保守防假零/同比子范围已证；受管 CLI 安全入口、可证 owner 与耐久账本阶段一待实现/验证，complete 正例待验</x:v>
+        <x:v>受限受管 CLI 入口、未知 owner 与耐久账本阶段一已编码并有开发单编号结果；真实账号验证及 complete 正例待验</x:v>
       </x:c>
       <x:c r="G54" s="55" t="str">
         <x:v>记录来源可证覆盖区间/留存边界；查询按提供方、授权用户、时区与区间求交，完整与真实零需证据；记录今天 as-of，扫描滞后不当完整日，同比须同截止口径；仅双方完整同范围可比较。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5792,7 +5803,8 @@
 2026-10-03 ef7a3de 落地、c10bbf3 修正：src/main/report.ts 的 scopedCoverage 从授权筛选后的事实给 unknown，不输出 partial/complete；有事实保留本范围计数和最近观察时间；概览/报表使用本范围结果，空事实不称真零，仅 pending 显示已确认小计 0/完整总量未知。TC-077/078 单元+Electron 独立通过，完整门禁 84 入口/59 unit/24 Electron 通过。历史留存/连续采集证明与同 as-of 正例仍待方案；无事实 reason 在“未归属”筛选下仍误称“没有已归属记录”；DEV-049 整项未完成。
 2026-10-03 覆盖证据决议：增加监测来源边界、留存起点、连续采集/重放水位、错误/缺口、归属和维度解析的可审计证据链，按所选范围判定；关闭空窗限定真零，双窗同口径且完整才比较。合成契约不得提升真实来源状态。
 2026-10-04 分期：受管入口与持久运行/用量/连续水位账本→授权范围封窗与 UI 标签→TC-077/078 受控正例→真实 CLI 正例；固定快照不升级为完整使用窗口。
-2026-10-04 阶段一交付前置：固定 provider CLI、只读/计划模式和经过授权的工作目录，主进程/服务拒绝 viewer、任意命令/标志/环境和越界路径；先记 run_id、actorUserId，再独立核 provider 账号/绑定版，缺证据写 owner_verified=false、owner=null，不生成报表事实或 complete。耐久写 run/event/heartbeat/水位/白名单计量与错误；解析、落盘、异常退出/重启不一致时 fail closed。提示词/回复/原始流不得持久化。TC-077/078 独立临时库/假 CLI 验收；本期不开放完整窗正例。</x:v>
+2026-10-04 阶段一交付前置：固定 provider CLI、只读/计划模式和经过授权的工作目录，主进程/服务拒绝 viewer、任意命令/标志/环境和越界路径；先记 run_id、actorUserId，再独立核 provider 账号/绑定版，缺证据写 owner_verified=false、owner=null，不生成报表事实或 complete。耐久写 run/event/heartbeat/水位/白名单计量与错误；解析、落盘、异常退出/重启不一致时 fail closed。提示词/回复/原始流不得持久化。TC-077/078 独立临时库/假 CLI 验收；本期不开放完整窗正例。
+2026-10-04 c359e6a（开发会话报告，文档会话待独立复跑）：0.3.7 管理员显式启用的受限只读/计划 Codex/Claude CLI 入口、受控目录与符号链接复核、固定参数/环境、run/event/heartbeat/水位耐久账本、未知 owner 不进报表、正文仅当前窗口并在登出/关窗清除已编码；TC-077/078/084 各单编号通过。有效 provider owner 身份、真实 CLI 正例、source-complete/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="155" customHeight="1">
@@ -5889,7 +5901,7 @@
         <x:v>src/collectors/scanner.ts；src/renderer/overview.tsx、report.tsx、diagnostics.tsx；状态测试</x:v>
       </x:c>
       <x:c r="F58" s="55" t="str">
-        <x:v>保守空状态/扫描反馈自动子范围已证；受管命令结果可见/内存隐私阶段一待实现，真零正例仍待证</x:v>
+        <x:v>当前会话结果可见/正文不持久化阶段一已编码并有开发单编号结果；真实真零正例待验</x:v>
       </x:c>
       <x:c r="G58" s="55" t="str">
         <x:v>六类空状态与下一步映射；长扫描显示阶段/心跳或已处理数量而非伪百分比；错误恢复与重试。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -5898,7 +5910,8 @@
 90338f4 已实现管理员取消 IPC、取消中/已取消 UI、停止下一文件与下一工具、当前文件事实/游标耐久提交或同回滚、已处理仅已观测、整轮取消不发完整 afterScan 快照；重扫按游标续跑且不并发。文档会话独立复验 TC-085、TC-087 与完整门禁通过。真实生产库、打包应用、系统强制终止未验；真零待 REQ-040。
 2026-10-03 覆盖证据决议：真零 UI 仅消费经 REQ-040/DEV-049 证明的所选来源 complete、已关闭且同事实集为空；范围外模式仍未知。真实来源机制未交付前 DEV-053 整项待验。
 2026-10-04 TC-084 真零依赖受管服务连续有效、关闭空窗及同范围空事实；先受控规则，再真实 CLI/守护服务正例，范围外仍未知。
-2026-10-04 阶段一：仅向发起管理员当前会话呈现受管任务状态与有界内存结果，或提供同会话安全打开动作；关闭/登出/切换用户清理正文，viewer 不可查看。DB、结构化日志、反馈附件只含脱敏状态/计量，不含提示词、回复或原始流；失败/身份未知给明确下一步，空结果不冒充真零。TC-084 用独立假 CLI/临时库和 UI/反馈附件核对。</x:v>
+2026-10-04 阶段一：仅向发起管理员当前会话呈现受管任务状态与有界内存结果，或提供同会话安全打开动作；关闭/登出/切换用户清理正文，viewer 不可查看。DB、结构化日志、反馈附件只含脱敏状态/计量，不含提示词、回复或原始流；失败/身份未知给明确下一步，空结果不冒充真零。TC-084 用独立假 CLI/临时库和 UI/反馈附件核对。
+2026-10-04 c359e6a（开发会话报告，文档会话待独立复跑）：0.3.7 管理员显式启用的受限只读/计划 Codex/Claude CLI 入口、受控目录与符号链接复核、固定参数/环境、run/event/heartbeat/水位耐久账本、未知 owner 不进报表、正文仅当前窗口并在登出/关窗清除已编码；TC-077/078/084 各单编号通过。有效 provider owner 身份、真实 CLI 正例、source-complete/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="155" customHeight="1">
@@ -9397,12 +9410,13 @@
 阶段一预期：viewer/越界或任意任务参数在 spawn 前拒绝，不借共享 macOS 凭证执行；actor 与 owner 分列，仅可证 provider 账号+绑定版本允许 owner_verified=true，缺证据为 false/空 owner，计量不进报表事实或 complete。run/event/heartbeat/水位持久，异常与不一致降级未知；无提示词/回复/原始流落盘。即使合成账本健康，本期仍无 complete 正例。</x:v>
       </x:c>
       <x:c r="H82" s="55" t="str">
-        <x:v>旧保守防假零自动子断言已证；受管 CLI 阶段一授权/归属/账本新范围待实现和单编号复验，完整覆盖正例待验</x:v>
+        <x:v>c359e6a 阶段一隔离自动子范围由开发会话报告通过；真实 CLI/完整覆盖正例待验</x:v>
       </x:c>
       <x:c r="I82" s="55" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
 2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-077：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。
-3bbaf15 文档会话复跑 TC-077 单元 1/1、Electron 1/1、退出码 0；新增无事实 reason 的“没有已观测记录”断言。</x:v>
+3bbaf15 文档会话复跑 TC-077 单元 1/1、Electron 1/1、退出码 0；新增无事实 reason 的“没有已观测记录”断言。
+2026-10-04 TC-077 管理员入口、路径/参数限制、账本/未知 owner 单编号已由开发会话报告通过；完整覆盖正例待验。 固定代码 c359e6a；文档会话未独立复跑，详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J82" s="55" t="str">
         <x:v>npm run test:case -- TC-077（已注册；单元 1/1、Electron 1/1，文档会话退出码 0）</x:v>
@@ -9461,11 +9475,12 @@
 阶段一预期：即使 run/event 已耐久且两窗等长，只要 provider owner 未可证或连续证据不全，比较一律不可比较，不能从 actor、macOS UID、空账本或一次合成运行推 complete；同比正例本期不判通过。</x:v>
       </x:c>
       <x:c r="H83" s="58" t="str">
-        <x:v>旧保守防假同比自动子断言已证；受管账本/未知 owner 比较降级新范围待实现和单编号复验，双完整窗正例待验</x:v>
+        <x:v>c359e6a 阶段一隔离自动子范围由开发会话报告通过；真实 CLI/完整覆盖正例待验</x:v>
       </x:c>
       <x:c r="I83" s="58" t="str">
         <x:v>2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
-2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-078：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。</x:v>
+2026-10-03 文档会话在最终代码 c10bbf3、macOS x86_64、Node v24.15.0、npm 11.12.1 独立运行 npm run test:case -- TC-078：单元 1/1、Electron 1/1、退出码 0。test:gate 类型检查、84 个入口、59/59 单元、24/24 Electron 退出码 0。仅隔离合成子范围通过。
+2026-10-04 TC-078 未验证 owner/心跳缺口仍不可比单编号已由开发会话报告通过；双完整窗正例待验。 固定代码 c359e6a；文档会话未独立复跑，详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J83" s="58" t="str">
         <x:v>npm run test:case -- TC-078（已注册；单元 1/1、Electron 1/1，文档会话退出码 0）</x:v>
@@ -9756,10 +9771,11 @@
 阶段一预期：发起者可在当前授权会话看到结果/安全打开，异常有明确说明；正文只在有界内存，viewer 与持久库/日志/反馈附件不可得。受管身份未知或失败不能显示已确认零；真正关闭完整空窗正例仍待后续 REQ-040 证据。</x:v>
       </x:c>
       <x:c r="H89" s="58" t="str">
-        <x:v>保守空状态自动子范围已证；受管结果可见/正文隐私阶段一待实现和单编号复验，完整空窗真零正例待验</x:v>
+        <x:v>c359e6a 阶段一隔离自动子范围由开发会话报告通过；真实 CLI/完整覆盖正例待验</x:v>
       </x:c>
       <x:c r="I89" s="58" t="str">
-        <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。仅保守状态与筛选无匹配 UI 行动；完整空窗真零未验。此前“待注册/不可运行”是实施前记录。</x:v>
+        <x:v>2026-10-03 文档会话在代码 000372b、macOS x86_64、Node v24.15.0、npm 11.12.1 独立复跑：单元 1/1、Electron 1/1，退出码 0；完整门禁 88 入口、64 单元、28 Electron 通过。仅保守状态与筛选无匹配 UI 行动；完整空窗真零未验。此前“待注册/不可运行”是实施前记录。
+2026-10-04 TC-084 当前窗口结果隐私/保守空状态单编号已由开发会话报告通过；真实真零正例待验。 固定代码 c359e6a；文档会话未独立复跑，详见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J89" s="58" t="str">
         <x:v>npm run test:case -- TC-084（2026-10-03 独立通过）</x:v>
@@ -10358,29 +10374,39 @@
       </x:c>
       <x:c r="F100" s="97" t="str">
         <x:v>固定代码、版本、架构和未签名 DMG SHA-256/hdiutil；确认此 Mac 安装目标及原 App/数据备份位置。仅用授权的人工操作从 DMG 安装到实际 /Applications 或 ~/Applications，启动并登录管理员；以当前账户可访问的授权来源检查无权限/授权后重扫、Codex/Claude 可观察记录、来源归属、报表筛选/明细与 CSV 同一快照。用专用隔离 App/userData 副本做更新坏包与五故障恢复，核旧版可启动/数据可读并可重试；生产 App 如升级，只在备份确认后人工点击“开始升级”，核点击前可放弃、点击后无取消直到成功/自动回退。升级前后以脱敏计数/只读校验核现有数据保留；回退旧版只用已验证兼容备份或明确人工恢复路径，不直接以旧程序打开已迁移的新库。不得由自动脚本写现有生产 userData。
-2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
+2026-10-04 旧生产库隔离副本验收补充：以 SQLite backup 建一次性副本并禁用真实来源/上传；启动前后均核 integrity_check。允许 source_identities 数量仅因可逐条追溯的 codex/claude:legacy-unverified:* 等保守隔离而变化；逐项列旧身份→新身份、提供方、触发事实、owner 清空/原身份保留或退出、legacy_unverified/碰撞原因和脱敏审计。来源身份行变化须逐条解释，不能从计数或 integrity_check 推通过。逐条以稳定旧键→确定性新键映射核 usage_facts 无丢失/无重复，provider、session、model、occurred_at、input/output/cache_read/cache_creation/total_tokens 均逐值一致；fact_projects 关联不丢。users、事实和游标数量保持，游标若为重扫故意归零须逐项说明，不能把任意状态变化当允许。
+最新范围补充：旧 Codex/Claude 本机 source_key 可按确定性规则转 scoped v2；旧 claude:macos 混合身份按规则退役，旧事实进入 legacy-unverified/待核对。发生旧本机键迁移时，现行迁移可清零本机游标偏移、解析状态和尾哈希以重扫；须核触发范围与重扫后无重复/漏计。不可记录真实来源条数或 Token 私有数值。</x:v>
       </x:c>
       <x:c r="G100" s="97" t="str">
-        <x:v>同一固定候选在当前 Mac 完成实际安装、启动、管理员登录；权限拒绝/授权后的状态和重扫正确，采集与归属不越权，报表/明细/CSV 一致且未知不写零。安装/更新失败后旧版可用、数据和受信状态保留或明确重新登录；无残留误报，备份与兼容回退路径可执行。失败/空数据有可操作说明；任何缺证项为待验，不以隔离测试替代实际安装。</x:v>
+        <x:v>同一固定候选在当前 Mac 完成实际安装、启动、管理员登录；权限拒绝/授权后的状态和重扫正确，采集与归属不越权，报表/明细/CSV 一致且未知不写零。安装/更新失败后旧版可用、数据和受信状态保留或明确重新登录；无残留误报，备份与兼容回退路径可执行。失败/空数据有可操作说明；任何缺证项为待验，不以隔离测试替代实际安装。
+预期：每个新增身份都能对应原身份及旧事实，类型/提供方正确且 legacy-unverified owner 为空；已有可证身份和归属不被串改。旧事实即使转到待核对仍可追溯数值与项目，不能无提示计入其他用户已确认小计；管理员看到待核对范围，viewer 不见他人身份、数量或用量。已确认小计若因隔离下降须与迁出事实逐项对账，不能漏计、伪零或把待核对当完整总量；报表/明细/CSV 同授权范围。任何不明新身份、丢失/重复/数值变化、越权或无法解释的游标变化都阻断通过。旧版回退必须恢复与旧版兼容的升级前数据库备份，不能直接用旧版打开已迁移新库。
+scoped v2 键迁移前后每条事实的五类 Token 数值和项目关联保持，旧归属不能扩大为已确认；界面明确待核对且 viewer 隔离。游标清零只在白名单迁移触发，二次启动幂等；旧版回退须带兼容升级前库备份。</x:v>
       </x:c>
       <x:c r="H100" s="97" t="str">
-        <x:v>待注册、待人工执行；当前本机交付门槛未通过</x:v>
+        <x:v>c359e6a 已注册人工入口；旧库隔离副本有需求会话独立对照子证据，真实本机安装/UI/兼容回退未完成，TC-095 未通过</x:v>
       </x:c>
       <x:c r="I100" s="97" t="str">
-        <x:v>2026-10-04 SOP-001 文档立项，未修改产品/测试代码，未触碰生产 userData；既有 TC-027/076 的本机隔离结果不能代证 TC-095。当前 /Applications/Token.app 曾核为 0.3.5，0.3.6 候选包 SHA 8773dd38…；以执行当天冻结制品为准。</x:v>
+        <x:v>2026-10-04 SOP-001 文档立项，未修改产品/测试代码，未触碰生产 userData；既有 TC-027/076 的本机隔离结果不能代证 TC-095。当前 /Applications/Token.app 曾核为 0.3.5，0.3.6 候选包 SHA 8773dd38…；以执行当天冻结制品为准。
+2026-10-04 需求会话独立对照报告：test:production-copy 的隔离副本启动后 source_identities 净变化，users/usage_facts/source_cursors 数量不变且 integrity_check=ok；旧脚本要求四表计数全等而失败。文档会话仅只读核代码/脚本，未接触原生产库、未核新增身份的具体行、未独立复跑；初次报告时尚不能判定是预期隔离或数据破坏，须按本行 F/G/M 验收。
+2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
+证据来源更正：需求会话在仓库外备份后独立用同一一次性副本运行旧 0.3.5 与新 0.3.7 打包 App，核基本表增量、事实 payload 排序摘要/Token 合计、integrity_check 与二次启动幂等；开发会话另做代码/SQL 核对。原生产库未由测试脚本写入；文档会话未独立复跑。仅为隔离副本子证据，界面待核对提示、权限、兼容备份回退与本机实装未验。</x:v>
       </x:c>
       <x:c r="J100" s="97" t="str">
-        <x:v>计划：npm run test:case -- TC-095；完成人工验收后 npm run test:case -- TC-095 pass /绝对路径/脱敏证据文件（失败用 fail）；注册前不可执行或登记 pass</x:v>
+        <x:v>npm run test:case -- TC-095（c359e6a 已注册 manual 清单；未提交人工结果时退出码 2）；实际通过后 npm run test:case -- TC-095 pass /绝对路径/脱敏证据文件</x:v>
       </x:c>
       <x:c r="K100" s="97" t="str">
-        <x:v>待开发会话在 scripts/test-cases.mjs 注册 manual 清单；只输出步骤并记录人工证据，不执行安装、授权、生产库写入或故障注入</x:v>
+        <x:v>scripts/test-cases.mjs：c359e6a 注册 TC-095 manual 清单，仅输出人工步骤与记录证据；不自动安装、写生产库或注入故障</x:v>
       </x:c>
       <x:c r="L100" s="97" t="str">
-        <x:v>无自动通过；需分别记录真实当前 Mac 安装路径与 UI、隔离故障回退及生产数据只读前后核对。TC-028/072 仍为未来外部分发待验，不据本项通过。</x:v>
+        <x:v>无自动通过；需分别记录真实当前 Mac 安装路径与 UI、隔离故障回退及生产数据只读前后核对。TC-028/072 仍为未来外部分发待验，不据本项通过。
+旧生产库隔离副本的原“所有表计数完全相等”不适合可解释的身份隔离迁移；只允许白名单迁移及逐键/逐数值/权限对账通过，不接受任意新增身份或仅 integrity_check=ok。真实生产目录仍不得由自动脚本改写。</x:v>
       </x:c>
       <x:c r="M100" s="97" t="str">
         <x:v>证据建议 test-results/manual/evidence/TC-095-local-mac-acceptance.md（被 Git 忽略的绝对路径）；记录固定提交/DMG SHA、macOS/架构、安装前后版本与路径、脱敏截图、权限/采集/报表/CSV 的范围和数值、备份摘要、隔离故障回退结果及原 App/数据恢复步骤；不存真实 JSONL/SQLite/密钥/提示词正文。
-2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
+隔离副本同一备份前后报告：各表计数、身份键种类与旧→新映射的脱敏摘要、逐事实数值/项目关联对账、owner/不确定原因/审计、管理员与 viewer 报表/明细/CSV 的已确认小计/待核对对账、游标变化原因；失败保留副本本地证据但不提交真实 SQLite/原始键。旧 App 回退另核升级前兼容备份。
+需求会话独立旧/新打包 App 同一副本对照的脱敏结论可作子证据；新脚本另核确定性 scoped v2 映射、legacy-unverified、游标重扫、UI 待核对/权限与旧版兼容备份。禁止记录真实会话正文、身份原值或私有计数。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10779,7 +10805,7 @@
         <x:v>VER-009</x:v>
       </x:c>
       <x:c r="B14" s="90" t="str">
-        <x:v>待定（当前目标收尾）</x:v>
+        <x:v>0.3.7（当前本机未签名候选；未实装）</x:v>
       </x:c>
       <x:c r="C14" s="90" t="str">
         <x:v>三批打磨及当前发布门槛</x:v>
@@ -10805,15 +10831,20 @@
 当前安装中取消要求已撤出本轮，历史备选设计保留；当前简化目标的新包隔离动态子范围已证，真实系统/生产场景仍待验。
 当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。
 7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。
-受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。</x:v>
+受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。
+c359e6a 阶段一受管 CLI 已编码；开发报告 TC-077/078/084 单编号通过，test:gate 95 入口、103/103 单元、46/46 Electron 通过。0.3.7 x64 DMG SHA-256 86a0817d86c8fac68f2ecc924c166e25f68753dce2e27b576254a12fe8f60f92 且 hdiutil VALID；开发先前打包全量 45/46（TC-038 超时）为历史失败；需求会话随后在同一 c359e6a/0.3.7 目录包独立重跑 npm run test:e2e:packaged 为 46/46、退出码 0，TC-038 末尾约 3.5 秒通过。生产库副本旧身份 verifier 待修，暂停发布/实装。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>当前 Mac 未签名本机交付待验：TC-095 未注册/未执行，实际安装与生产数据保护未证；外部分发仍待验</x:v>
+        <x:v>0.3.7 本机候选代码与隔离阶段一自动子范围有开发证据；生产库副本 verifier 待修、打包全量已由需求会话独立复跑 46/46、TC-095 本机实装未执行，故交付未完成；完整覆盖/真零及外部分发另待验</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
         <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。
 2026-10-04 仅补 REQ-040/044→DEV-049/053→TC-077/078/084 阶段一合同；无新代码、无新增动态通过。
-2026-10-04 仅调整范围和追溯、分配 TC-095；无本机实装或生产数据动态通过。TC-028/072 均保持待验。</x:v>
+2026-10-04 仅调整范围和追溯、分配 TC-095；无本机实装或生产数据动态通过。TC-028/072 均保持待验。
+2026-10-04 旧生产库隔离副本启动报告 source_identities 净变化、users/facts/cursors 数量不变且 integrity_check=ok；旧脚本全表计数断言失败。迁移是否安全未逐键核，TC-095/本机交付不升通过。
+2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
+2026-10-04 固定代码 c359e6a；开发报告 test:gate 95/103/46 通过、TC-077/078/084 各单编号通过，打包全量 45/46+TC-038 单项复跑；当前 0.3.7 DMG SHA 86a0817d…、hdiutil VALID。需求会话独立做旧/新 App 备份副本身份迁移对照；文档会话未独立复验。
+2026-10-04 需求会话独立在 c359e6a/0.3.7 目录包执行 npm run test:e2e:packaged，46/46、退出码 0，TC-038 末尾约 3.5 秒通过；开发先前 45/46 超时保留历史。文档会话未独立复跑，TC-095/生产库副本 verifier 仍待验。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
@@ -10821,7 +10852,9 @@
 REQ-023/TC-076 前次决议（由下方点击边界取代）：安装前可放弃、安装开始后不可取消、失败自动恢复；独立取消控制窗口不属本轮。
 REQ-023/TC-076 最新边界为点击开始前可放弃、点击后直到成功/回退均不可取消；不交付取消控制窗口/协议/journal/分阶段正例。
 当前优先注册并人工执行 TC-095；同一候选完成当前 Mac 真安装、权限、采集、报表/CSV、升级恢复、只读数据核对和兼容回退证据。Developer ID/公证/第二台 Mac 资源具备后另走 TC-028/072。
-2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。</x:v>
+2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
+以同一授权备份副本修订并复跑迁移对账：解释每个新增 legacy-unverified 身份、事实逐键/逐数值、owner/小计/待核对与 viewer 隔离，另核旧版兼容备份回退；不得对生产原库做自动写入。
+先修生产库副本 verifier 并复跑同一备份，重建/冻结最终候选并核同候选打包全量及 TC-095 当前 Mac 人工实装；未完成前不发布。真实 provider 归属、source-complete/真零/同比另按 REQ-040/044 验。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: record TC-095 verifier and final 0.3.7 candidate evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R34bd07ab2b764a36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Ra88eeef5f91646e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R7e392d2da15a47ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rddbc88359f274872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R805c400df00345b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R580f32932d594a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7d29ba8adfa14f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R82540a8512d4498d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R6ceecf662b7b48e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rc97d2fcccba04f42"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3103,7 +3103,8 @@
 2026-10-04 TC-095 旧库隔离副本启动出现 source_identities 净变化；目前仅知 users/facts/cursors 数量不变及 integrity_check=ok，未证明逐键/归属/报表安全。脚本全表计数全等断言需改为可解释白名单迁移对账，TC-095 仍待验。
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
 证据来源：需求会话独立做旧/新打包 App 同一备份副本对照；开发会话核代码/SQL。c359e6a 已注册 TC-095 人工清单，但实际本机安装与完整验收待执行。
-TC-095 保守迁移允许旧本机键→scoped v2、旧 claude:macos 退役/待核对和有因游标清零；逐事实/权限/界面及兼容备份仍是通过条件，不因摘要一致升为完整验收。</x:v>
+TC-095 保守迁移允许旧本机键→scoped v2、旧 claude:macos 退役/待核对和有因游标清零；逐事实/权限/界面及兼容备份仍是通过条件，不因摘要一致升为完整验收。
+ee617f3：开发报告授权副本迁移 verifier 退出 0，逐事实/项目/身份/待核对/游标/幂等脚本子范围已证；最终 0.3.7 包和本机服务清单一致，打包全量 46/46。首轮 TC-073 耗时失败保留。TC-095 当前 Mac 实装、UI/CSV、兼容备份回退仍待人工验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3624,7 +3625,7 @@
         <x:v>M4</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>本机隔离 DMG 子范围已验证；当前 Mac 实际安装与完整可用流程 TC-095 待注册/待人工验收</x:v>
+        <x:v>本机隔离 DMG 与旧库副本迁移脚本子范围有通过证据；TC-095 当前 Mac 实装、UI 授权/CSV 与兼容旧备份回退待人工验收</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
         <x:v>DEV-017</x:v>
@@ -3637,7 +3638,8 @@
 2026-10-03：代码 7abd640 的 0.3.4 未签名 DMG 在 macOS 15.7.4 x86_64 以独立临时库/人工 Codex JSONL 挂载、ditto 复制、启动，受信登录、扫描和 1280 Token 报表通过；TC-027 人工 pass 登记时间 2026-10-02T20:46:08.228Z，证据见 docs/validation.md。Finder /Applications、真实生产账户/库、异机、签名公证、TC-072 待验。
 2026-10-04 本机交付决议：REQ-017 不以其他 Mac/Developer ID/公证为当前门槛；新增 TC-095 独立核当前 Mac 真实安装、启动、管理员登录、来源权限/采集、报表/CSV、升级故障恢复、用户数据保留和可用旧版回退。既有 TC-027 隔离子范围不代证真实安装；生产 userData 不得由自动测试改写。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
-2026-10-04 TC-095 旧生产库副本允许可证 legacy-unverified 身份隔离导致身份行变化，但逐事实数值、归属权限与报表范围须对账；单纯完整性 ok/数量不变不构成通过。</x:v>
+2026-10-04 TC-095 旧生产库副本允许可证 legacy-unverified 身份隔离导致身份行变化，但逐事实数值、归属权限与报表范围须对账；单纯完整性 ok/数量不变不构成通过。
+2026-10-04 ee617f3：开发报告授权仓库外备份副本 test:production-copy 退出 0；文档会话只读核脚本，未读/未复跑副本。旧身份白名单及逐事实/项目/待核对/游标/幂等脚本子范围已证，真实 UI 与旧版回退仍待 TC-095。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5029,13 +5031,14 @@
         <x:v>scripts/package-dmg.mjs；package.json；release/</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>0.3.4 本机隔离打包子范围已证；当前 Mac 实际安装与完整可用流程 TC-095 待注册/验收</x:v>
+        <x:v>TC-095 人工入口已注册；ee617f3 旧库副本迁移 verifier 子任务有开发通过证据，当前 Mac 实装/UI/兼容备份回退待验</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
         <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md
 0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。
 2026-10-04 本机交付任务：在 scripts/test-cases.mjs 注册独立 TC-095 人工清单；冻结候选代码/未签名 DMG 与 SHA/架构，隔离副本先做升级故障回退，当前 Mac 实装与 UI 人工核对另留脱敏证据。不得让自动脚本指向或改写现有生产 userData。
-2026-10-04 verify-production-copy.mjs 原指纹要求 identities 全等，当前隔离副本报告 净变化；开发应仅在有逐条 legacy-unverified 映射、事实/小计/权限和旧版兼容备份证据时调整断言，不能允许任意新行。</x:v>
+2026-10-04 verify-production-copy.mjs 原指纹要求 identities 全等，当前隔离副本报告 净变化；开发应仅在有逐条 legacy-unverified 映射、事实/小计/权限和旧版兼容备份证据时调整断言，不能允许任意新行。
+2026-10-04 ee617f3：verify-production-copy.mjs 改为账户、事实、项目关联、身份白名单、待核对和游标的逐行对账及二次启动幂等；开发会话以仓库外授权备份副本和最终 0.3.7 目录包报告退出码 0。文档会话只读核代码，未接触生产库。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -10384,13 +10387,14 @@
 scoped v2 键迁移前后每条事实的五类 Token 数值和项目关联保持，旧归属不能扩大为已确认；界面明确待核对且 viewer 隔离。游标清零只在白名单迁移触发，二次启动幂等；旧版回退须带兼容升级前库备份。</x:v>
       </x:c>
       <x:c r="H100" s="97" t="str">
-        <x:v>c359e6a 已注册人工入口；旧库隔离副本有需求会话独立对照子证据，真实本机安装/UI/兼容回退未完成，TC-095 未通过</x:v>
+        <x:v>ee617f3 旧库隔离副本迁移脚本子范围由开发会话报告通过；最终 0.3.7 打包全量 46/46。当前 Mac 实装、UI 授权/CSV 与兼容旧备份回退未完成，TC-095 未通过</x:v>
       </x:c>
       <x:c r="I100" s="97" t="str">
         <x:v>2026-10-04 SOP-001 文档立项，未修改产品/测试代码，未触碰生产 userData；既有 TC-027/076 的本机隔离结果不能代证 TC-095。当前 /Applications/Token.app 曾核为 0.3.5，0.3.6 候选包 SHA 8773dd38…；以执行当天冻结制品为准。
 2026-10-04 需求会话独立对照报告：test:production-copy 的隔离副本启动后 source_identities 净变化，users/usage_facts/source_cursors 数量不变且 integrity_check=ok；旧脚本要求四表计数全等而失败。文档会话仅只读核代码/脚本，未接触原生产库、未核新增身份的具体行、未独立复跑；初次报告时尚不能判定是预期隔离或数据破坏，须按本行 F/G/M 验收。
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
-证据来源更正：需求会话在仓库外备份后独立用同一一次性副本运行旧 0.3.5 与新 0.3.7 打包 App，核基本表增量、事实 payload 排序摘要/Token 合计、integrity_check 与二次启动幂等；开发会话另做代码/SQL 核对。原生产库未由测试脚本写入；文档会话未独立复跑。仅为隔离副本子证据，界面待核对提示、权限、兼容备份回退与本机实装未验。</x:v>
+证据来源更正：需求会话在仓库外备份后独立用同一一次性副本运行旧 0.3.5 与新 0.3.7 打包 App，核基本表增量、事实 payload 排序摘要/Token 合计、integrity_check 与二次启动幂等；开发会话另做代码/SQL 核对。原生产库未由测试脚本写入；文档会话未独立复跑。仅为隔离副本子证据，界面待核对提示、权限、兼容备份回退与本机实装未验。
+2026-10-04 最终候选 ee617f36d33670344f9f29ac7d29f997368624c5：开发会话报告 test:production-copy 在仓库外授权备份副本退出码 0，脚本逐事实/项目/身份白名单/待核对/游标与二次启动幂等通过；文档会话仅只读核修订脚本。首轮 test:gate TC-073 耗时阈值失败，单编号和第二轮完整门禁 95 入口、103/103 单元、46/46 Electron 通过，最终重建目录包打包全量 46/46。脚本结果不覆盖 UI/CSV 与旧版回退。</x:v>
       </x:c>
       <x:c r="J100" s="97" t="str">
         <x:v>npm run test:case -- TC-095（c359e6a 已注册 manual 清单；未提交人工结果时退出码 2）；实际通过后 npm run test:case -- TC-095 pass /绝对路径/脱敏证据文件</x:v>
@@ -10406,7 +10410,8 @@
         <x:v>证据建议 test-results/manual/evidence/TC-095-local-mac-acceptance.md（被 Git 忽略的绝对路径）；记录固定提交/DMG SHA、macOS/架构、安装前后版本与路径、脱敏截图、权限/采集/报表/CSV 的范围和数值、备份摘要、隔离故障回退结果及原 App/数据恢复步骤；不存真实 JSONL/SQLite/密钥/提示词正文。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 隔离副本同一备份前后报告：各表计数、身份键种类与旧→新映射的脱敏摘要、逐事实数值/项目关联对账、owner/不确定原因/审计、管理员与 viewer 报表/明细/CSV 的已确认小计/待核对对账、游标变化原因；失败保留副本本地证据但不提交真实 SQLite/原始键。旧 App 回退另核升级前兼容备份。
-需求会话独立旧/新打包 App 同一副本对照的脱敏结论可作子证据；新脚本另核确定性 scoped v2 映射、legacy-unverified、游标重扫、UI 待核对/权限与旧版兼容备份。禁止记录真实会话正文、身份原值或私有计数。</x:v>
+需求会话独立旧/新打包 App 同一副本对照的脱敏结论可作子证据；新脚本另核确定性 scoped v2 映射、legacy-unverified、游标重扫、UI 待核对/权限与旧版兼容备份。禁止记录真实会话正文、身份原值或私有计数。
+最终 0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，文档会话独立只读核大小、哈希、hdiutil VALID 与本机服务 manifest/包一致。服务目录发布不等于当前 Mac 已安装；人工证据仍需真实安装、管理员/viewer 权限和报表/CSV、兼容旧备份回退。只记状态，不记私有计数/原始身份/正文。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10832,10 +10837,11 @@
 当前收尾按原生日期控件和同快照导出验收；TC-079 测试定位修复与打包复验待补。
 7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。
 受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。
-c359e6a 阶段一受管 CLI 已编码；开发报告 TC-077/078/084 单编号通过，test:gate 95 入口、103/103 单元、46/46 Electron 通过。0.3.7 x64 DMG SHA-256 86a0817d86c8fac68f2ecc924c166e25f68753dce2e27b576254a12fe8f60f92 且 hdiutil VALID；开发先前打包全量 45/46（TC-038 超时）为历史失败；需求会话随后在同一 c359e6a/0.3.7 目录包独立重跑 npm run test:e2e:packaged 为 46/46、退出码 0，TC-038 末尾约 3.5 秒通过。生产库副本旧身份 verifier 待修，暂停发布/实装。</x:v>
+c359e6a 阶段一受管 CLI 已编码；开发报告 TC-077/078/084 单编号通过，test:gate 95 入口、103/103 单元、46/46 Electron 通过。0.3.7 x64 DMG SHA-256 86a0817d86c8fac68f2ecc924c166e25f68753dce2e27b576254a12fe8f60f92 且 hdiutil VALID；开发先前打包全量 45/46（TC-038 超时）为历史失败；需求会话随后在同一 c359e6a/0.3.7 目录包独立重跑 npm run test:e2e:packaged 为 46/46、退出码 0，TC-038 末尾约 3.5 秒通过。生产库副本旧身份 verifier 待修，暂停发布/实装。
+ee617f3 最终候选：旧库副本 verifier 已修并有开发侧通过报告；第二轮 test:gate 95 入口/103 单元/46 Electron 通过，最终重建目录包打包全量 46/46。首轮 TC-073 耗时阈值失败保留。0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，本机服务 manifest/包一致；本机实装未验。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>0.3.7 本机候选代码与隔离阶段一自动子范围有开发证据；生产库副本 verifier 待修、打包全量已由需求会话独立复跑 46/46、TC-095 本机实装未执行，故交付未完成；完整覆盖/真零及外部分发另待验</x:v>
+        <x:v>0.3.7 最终候选的旧库隔离副本脚本、源码门禁、打包全量和本机服务制品有通过证据；TC-095 当前 Mac 实装、UI 授权/CSV、兼容旧备份回退待人工验收，故版本交付未完成；真实 CLI owner/完整覆盖/真零/同比和异机发布另待验</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
         <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。
@@ -10844,7 +10850,8 @@
 2026-10-04 旧生产库隔离副本启动报告 source_identities 净变化、users/facts/cursors 数量不变且 integrity_check=ok；旧脚本全表计数断言失败。迁移是否安全未逐键核，TC-095/本机交付不升通过。
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
 2026-10-04 固定代码 c359e6a；开发报告 test:gate 95/103/46 通过、TC-077/078/084 各单编号通过，打包全量 45/46+TC-038 单项复跑；当前 0.3.7 DMG SHA 86a0817d…、hdiutil VALID。需求会话独立做旧/新 App 备份副本身份迁移对照；文档会话未独立复验。
-2026-10-04 需求会话独立在 c359e6a/0.3.7 目录包执行 npm run test:e2e:packaged，46/46、退出码 0，TC-038 末尾约 3.5 秒通过；开发先前 45/46 超时保留历史。文档会话未独立复跑，TC-095/生产库副本 verifier 仍待验。</x:v>
+2026-10-04 需求会话独立在 c359e6a/0.3.7 目录包执行 npm run test:e2e:packaged，46/46、退出码 0，TC-038 末尾约 3.5 秒通过；开发先前 45/46 超时保留历史。文档会话未独立复跑，TC-095/生产库副本 verifier 仍待验。
+2026-10-04 ee617f3：开发报告 test:production-copy 授权备份副本退出 0；首轮 test:gate TC-073 耗时阈值失败，单编号及第二轮 95/103/46 通过；最终重建目录包 test:e2e:packaged 46/46。文档会话未复跑动态测试，独立只读核最终 DMG/本机服务 manifest 大小和 SHA 一致、hdiutil VALID；不记录生产私有计数。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
@@ -10854,7 +10861,8 @@
 当前优先注册并人工执行 TC-095；同一候选完成当前 Mac 真安装、权限、采集、报表/CSV、升级恢复、只读数据核对和兼容回退证据。Developer ID/公证/第二台 Mac 资源具备后另走 TC-028/072。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 以同一授权备份副本修订并复跑迁移对账：解释每个新增 legacy-unverified 身份、事实逐键/逐数值、owner/小计/待核对与 viewer 隔离，另核旧版兼容备份回退；不得对生产原库做自动写入。
-先修生产库副本 verifier 并复跑同一备份，重建/冻结最终候选并核同候选打包全量及 TC-095 当前 Mac 人工实装；未完成前不发布。真实 provider 归属、source-complete/真零/同比另按 REQ-040/044 验。</x:v>
+先修生产库副本 verifier 并复跑同一备份，重建/冻结最终候选并核同候选打包全量及 TC-095 当前 Mac 人工实装；未完成前不发布。真实 provider 归属、source-complete/真零/同比另按 REQ-040/044 验。
+当前下一步：以 ee617f3 /最终 0.3.7 同一候选完成 TC-095 本机实际安装、管理员/viewer UI 与报表/CSV 核对、兼容旧版 App 加升级前库备份回退；取得脱敏人工证据后才判本机交付。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
docs: record TC-095 current Mac acceptance pass
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R580f32932d594a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R7d29ba8adfa14f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R82540a8512d4498d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R6ceecf662b7b48e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rc97d2fcccba04f42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rca59d20063494a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2c087390274843fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcb5990b19daa4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra9349c6b6a4c433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R1914e6945da74986"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3098,13 +3098,15 @@
         <x:v>当前 Mac 实际安装与本机可用人工验收</x:v>
       </x:c>
       <x:c r="G101" s="97" t="str">
-        <x:v>2026-10-04 立项时新增独立本机发布验收、入口待注册；c359e6a 已注册人工入口，至今未人工执行，真实安装/登录/权限/采集/报表/CSV/升级故障恢复/数据保留与回退均待证。TC-028/072 不属本次本机门槛，仍各自待验。
+        <x:v>2026-10-04 立项时新增独立本机发布验收、入口待注册；c359e6a 已注册人工入口，立项当时未人工执行，真实安装/登录/权限/采集/报表/CSV/升级故障恢复/数据保留与回退均待证。TC-028/072 不属本次本机门槛，仍各自待验。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 2026-10-04 TC-095 旧库隔离副本启动出现 source_identities 净变化；目前仅知 users/facts/cursors 数量不变及 integrity_check=ok，未证明逐键/归属/报表安全。脚本全表计数全等断言需改为可解释白名单迁移对账，TC-095 仍待验。
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
 证据来源：需求会话独立做旧/新打包 App 同一备份副本对照；开发会话核代码/SQL。c359e6a 已注册 TC-095 人工清单，但实际本机安装与完整验收待执行。
 TC-095 保守迁移允许旧本机键→scoped v2、旧 claude:macos 退役/待核对和有因游标清零；逐事实/权限/界面及兼容备份仍是通过条件，不因摘要一致升为完整验收。
-ee617f3：开发报告授权副本迁移 verifier 退出 0，逐事实/项目/身份/待核对/游标/幂等脚本子范围已证；最终 0.3.7 包和本机服务清单一致，打包全量 46/46。首轮 TC-073 耗时失败保留。TC-095 当前 Mac 实装、UI/CSV、兼容备份回退仍待人工验收。</x:v>
+ee617f3：开发报告授权副本迁移 verifier 退出 0，逐事实/项目/身份/待核对/游标/幂等脚本子范围已证；最终 0.3.7 包和本机服务清单一致，打包全量 46/46。首轮 TC-073 耗时失败保留。TC-095 当前 Mac 实装、UI/CSV、兼容备份回退仍待人工验收。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。 TC-028/072 不随本机结果升通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3625,7 +3627,7 @@
         <x:v>M4</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>本机隔离 DMG 与旧库副本迁移脚本子范围有通过证据；TC-095 当前 Mac 实装、UI 授权/CSV 与兼容旧备份回退待人工验收</x:v>
+        <x:v>TC-095 当前 Mac 未签名 0.3.7 本机范围通过：实际安装、受信登录、来源/报表与 CSV、旧事实保留、隔离兼容回退及同候选五故障恢复/重试有证据；异机/签名另待验</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
         <x:v>DEV-017</x:v>
@@ -3639,7 +3641,9 @@
 2026-10-04 本机交付决议：REQ-017 不以其他 Mac/Developer ID/公证为当前门槛；新增 TC-095 独立核当前 Mac 真实安装、启动、管理员登录、来源权限/采集、报表/CSV、升级故障恢复、用户数据保留和可用旧版回退。既有 TC-027 隔离子范围不代证真实安装；生产 userData 不得由自动测试改写。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 2026-10-04 TC-095 旧生产库副本允许可证 legacy-unverified 身份隔离导致身份行变化，但逐事实数值、归属权限与报表范围须对账；单纯完整性 ok/数量不变不构成通过。
-2026-10-04 ee617f3：开发报告授权仓库外备份副本 test:production-copy 退出 0；文档会话只读核脚本，未读/未复跑副本。旧身份白名单及逐事实/项目/待核对/游标/幂等脚本子范围已证，真实 UI 与旧版回退仍待 TC-095。</x:v>
+2026-10-04 ee617f3：开发报告授权仓库外备份副本 test:production-copy 退出 0；文档会话只读核脚本，未读/未复跑副本。旧身份白名单及逐事实/项目/待核对/游标/幂等脚本子范围已证，真实 UI 与旧版回退仍待 TC-095。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -5031,14 +5035,16 @@
         <x:v>scripts/package-dmg.mjs；package.json；release/</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>TC-095 人工入口已注册；ee617f3 旧库副本迁移 verifier 子任务有开发通过证据，当前 Mac 实装/UI/兼容备份回退待验</x:v>
+        <x:v>DEV-017 当前 Mac 未签名 0.3.7 交付子范围已验：TC-095 人工 pass；同候选隔离五故障恢复/重试及真实安装主流程已记录，异机外部分发另待</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
         <x:v>历史：2026-10-02 当前 Mac 未签名包；v0.3.0：TC-027 人工 pass，DMG 挂载复制及主流程 1/1，见 docs/validation.md
 0.3.4 代码 7abd640：DMG SHA-256 7b4d8ad523c5afe71f5004fc7d7b4e690144e1f1119af2ab7bb86635888bf588，hdiutil VALID；开发会话再次跑 0.3.3→0.3.4 隔离升级退出码 0，当前 TC-027.json 为 pass，证据摘要 evidence/TC-027-0.3.4.md。文档会话此前独立复跑升级。旧 0.3.0 结果已备份；真实生产账户/库、Finder /Applications、异机、签名公证待验，见 docs/validation.md。
 2026-10-04 本机交付任务：在 scripts/test-cases.mjs 注册独立 TC-095 人工清单；冻结候选代码/未签名 DMG 与 SHA/架构，隔离副本先做升级故障回退，当前 Mac 实装与 UI 人工核对另留脱敏证据。不得让自动脚本指向或改写现有生产 userData。
 2026-10-04 verify-production-copy.mjs 原指纹要求 identities 全等，当前隔离副本报告 净变化；开发应仅在有逐条 legacy-unverified 映射、事实/小计/权限和旧版兼容备份证据时调整断言，不能允许任意新行。
-2026-10-04 ee617f3：verify-production-copy.mjs 改为账户、事实、项目关联、身份白名单、待核对和游标的逐行对账及二次启动幂等；开发会话以仓库外授权备份副本和最终 0.3.7 目录包报告退出码 0。文档会话只读核代码，未接触生产库。</x:v>
+2026-10-04 ee617f3：verify-production-copy.mjs 改为账户、事实、项目关联、身份白名单、待核对和游标的逐行对账及二次启动幂等；开发会话以仓库外授权备份副本和最终 0.3.7 目录包报告退出码 0。文档会话只读核代码，未接触生产库。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -10387,14 +10393,16 @@
 scoped v2 键迁移前后每条事实的五类 Token 数值和项目关联保持，旧归属不能扩大为已确认；界面明确待核对且 viewer 隔离。游标清零只在白名单迁移触发，二次启动幂等；旧版回退须带兼容升级前库备份。</x:v>
       </x:c>
       <x:c r="H100" s="97" t="str">
-        <x:v>ee617f3 旧库隔离副本迁移脚本子范围由开发会话报告通过；最终 0.3.7 打包全量 46/46。当前 Mac 实装、UI 授权/CSV 与兼容旧备份回退未完成，TC-095 未通过</x:v>
+        <x:v>pass（2026-10-04，当前 Mac 未签名 0.3.7 本机范围）；同候选隔离故障/重试与真实安装、来源、报表/CSV、保留/兼容回退已证；不包括 TC-028/072 异机/签名或 REQ-040 完整覆盖正例</x:v>
       </x:c>
       <x:c r="I100" s="97" t="str">
         <x:v>2026-10-04 SOP-001 文档立项，未修改产品/测试代码，未触碰生产 userData；既有 TC-027/076 的本机隔离结果不能代证 TC-095。当前 /Applications/Token.app 曾核为 0.3.5，0.3.6 候选包 SHA 8773dd38…；以执行当天冻结制品为准。
 2026-10-04 需求会话独立对照报告：test:production-copy 的隔离副本启动后 source_identities 净变化，users/usage_facts/source_cursors 数量不变且 integrity_check=ok；旧脚本要求四表计数全等而失败。文档会话仅只读核代码/脚本，未接触原生产库、未核新增身份的具体行、未独立复跑；初次报告时尚不能判定是预期隔离或数据破坏，须按本行 F/G/M 验收。
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
 证据来源更正：需求会话在仓库外备份后独立用同一一次性副本运行旧 0.3.5 与新 0.3.7 打包 App，核基本表增量、事实 payload 排序摘要/Token 合计、integrity_check 与二次启动幂等；开发会话另做代码/SQL 核对。原生产库未由测试脚本写入；文档会话未独立复跑。仅为隔离副本子证据，界面待核对提示、权限、兼容备份回退与本机实装未验。
-2026-10-04 最终候选 ee617f36d33670344f9f29ac7d29f997368624c5：开发会话报告 test:production-copy 在仓库外授权备份副本退出码 0，脚本逐事实/项目/身份白名单/待核对/游标与二次启动幂等通过；文档会话仅只读核修订脚本。首轮 test:gate TC-073 耗时阈值失败，单编号和第二轮完整门禁 95 入口、103/103 单元、46/46 Electron 通过，最终重建目录包打包全量 46/46。脚本结果不覆盖 UI/CSV 与旧版回退。</x:v>
+2026-10-04 最终候选 ee617f36d33670344f9f29ac7d29f997368624c5：开发会话报告 test:production-copy 在仓库外授权备份副本退出码 0，脚本逐事实/项目/身份白名单/待核对/游标与二次启动幂等通过；文档会话仅只读核修订脚本。首轮 test:gate TC-073 耗时阈值失败，单编号和第二轮完整门禁 95 入口、103/103 单元、46/46 Electron 通过，最终重建目录包打包全量 46/46。脚本结果不覆盖 UI/CSV 与旧版回退。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
       <x:c r="J100" s="97" t="str">
         <x:v>npm run test:case -- TC-095（c359e6a 已注册 manual 清单；未提交人工结果时退出码 2）；实际通过后 npm run test:case -- TC-095 pass /绝对路径/脱敏证据文件</x:v>
@@ -10403,15 +10411,16 @@
         <x:v>scripts/test-cases.mjs：c359e6a 注册 TC-095 manual 清单，仅输出人工步骤与记录证据；不自动安装、写生产库或注入故障</x:v>
       </x:c>
       <x:c r="L100" s="97" t="str">
-        <x:v>无自动通过；需分别记录真实当前 Mac 安装路径与 UI、隔离故障回退及生产数据只读前后核对。TC-028/072 仍为未来外部分发待验，不据本项通过。
-旧生产库隔离副本的原“所有表计数完全相等”不适合可解释的身份隔离迁移；只允许白名单迁移及逐键/逐数值/权限对账通过，不接受任意新增身份或仅 integrity_check=ok。真实生产目录仍不得由自动脚本改写。</x:v>
+        <x:v>当前 Mac 未签名 0.3.7 范围人工 pass；实际安装/管理员/来源/报表/CSV/旧事实保留、旧 App+升级前兼容库隔离回退，以及同候选隔离五故障恢复、清理与重试有开发侧脱敏证据。故障注入只在临时目录，不证明真实满盘、断电或生产目录故障；TC-028/072 独立待验，真实 CLI owner/完整覆盖/真零/同比不因本项提升。自动脚本不得改写生产原库。</x:v>
       </x:c>
       <x:c r="M100" s="97" t="str">
         <x:v>证据建议 test-results/manual/evidence/TC-095-local-mac-acceptance.md（被 Git 忽略的绝对路径）；记录固定提交/DMG SHA、macOS/架构、安装前后版本与路径、脱敏截图、权限/采集/报表/CSV 的范围和数值、备份摘要、隔离故障回退结果及原 App/数据恢复步骤；不存真实 JSONL/SQLite/密钥/提示词正文。
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 隔离副本同一备份前后报告：各表计数、身份键种类与旧→新映射的脱敏摘要、逐事实数值/项目关联对账、owner/不确定原因/审计、管理员与 viewer 报表/明细/CSV 的已确认小计/待核对对账、游标变化原因；失败保留副本本地证据但不提交真实 SQLite/原始键。旧 App 回退另核升级前兼容备份。
 需求会话独立旧/新打包 App 同一副本对照的脱敏结论可作子证据；新脚本另核确定性 scoped v2 映射、legacy-unverified、游标重扫、UI 待核对/权限与旧版兼容备份。禁止记录真实会话正文、身份原值或私有计数。
-最终 0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，文档会话独立只读核大小、哈希、hdiutil VALID 与本机服务 manifest/包一致。服务目录发布不等于当前 Mac 已安装；人工证据仍需真实安装、管理员/viewer 权限和报表/CSV、兼容旧备份回退。只记状态，不记私有计数/原始身份/正文。</x:v>
+最终 0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，文档会话独立只读核大小、哈希、hdiutil VALID 与本机服务 manifest/包一致。服务目录发布不等于当前 Mac 已安装；人工证据仍需真实安装、管理员/viewer 权限和报表/CSV、兼容旧备份回退。只记状态，不记私有计数/原始身份/正文。
+本机被 Git 忽略的 test-results/manual/evidence/TC-095-local-mac-acceptance.md 为开发侧脱敏人工记录。文档会话只读核实际 /Applications/Token.app 版本 0.3.7、app.asar SHA-256 3167a5cde8fb1a182616494cc32f938191b7ce6daee40a0420d567dd905108ef 与记录一致、仓库外备份目录存在；未读生产库/秘密，未重跑 UI/回退。后续同候选故障注入/重试另补固定命令、退出码及脱敏结果，不记录生产私有计数或正文。
+开发工作树被 Git 忽略的 test-results/manual/evidence/TC-095-local-mac-acceptance.md 已补同候选 TC-076 五故障/重试；test-results/manual/TC-095.json 为 pass（2026-10-04T08:30:06.633Z）。文档会话只读核这两个文件及本地 99f77b4 与远端 ee617f3 的 Git 文件树相同，未读取生产库/秘密，也未复跑故障脚本。记录不含私有计数/身份原值/正文。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10810,7 +10819,7 @@
         <x:v>VER-009</x:v>
       </x:c>
       <x:c r="B14" s="90" t="str">
-        <x:v>0.3.7（当前本机未签名候选；未实装）</x:v>
+        <x:v>0.3.7（当前 Mac 本机未签名范围通过；完整三批/外部分发另待）</x:v>
       </x:c>
       <x:c r="C14" s="90" t="str">
         <x:v>三批打磨及当前发布门槛</x:v>
@@ -10838,10 +10847,12 @@
 7fd0ce7 已补 TC-079 测试定位和本机自动回归；当前目标完整交付仍缺生产、系统及外部环境证据。
 受管 CLI 账本阶段一安全入口、owner 证明、结果可见与正文隐私已列验收；机制及新增 TC-077/078/084 断言待实施，complete/真零/同比正例不属于本期通过。
 c359e6a 阶段一受管 CLI 已编码；开发报告 TC-077/078/084 单编号通过，test:gate 95 入口、103/103 单元、46/46 Electron 通过。0.3.7 x64 DMG SHA-256 86a0817d86c8fac68f2ecc924c166e25f68753dce2e27b576254a12fe8f60f92 且 hdiutil VALID；开发先前打包全量 45/46（TC-038 超时）为历史失败；需求会话随后在同一 c359e6a/0.3.7 目录包独立重跑 npm run test:e2e:packaged 为 46/46、退出码 0，TC-038 末尾约 3.5 秒通过。生产库副本旧身份 verifier 待修，暂停发布/实装。
-ee617f3 最终候选：旧库副本 verifier 已修并有开发侧通过报告；第二轮 test:gate 95 入口/103 单元/46 Electron 通过，最终重建目录包打包全量 46/46。首轮 TC-073 耗时阈值失败保留。0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，本机服务 manifest/包一致；本机实装未验。</x:v>
+ee617f3 最终候选：旧库副本 verifier 已修并有开发侧通过报告；第二轮 test:gate 95 入口/103 单元/46 Electron 通过，最终重建目录包打包全量 46/46。首轮 TC-073 耗时阈值失败保留。0.3.7 x64 DMG 142585117 字节、SHA-256 dd4c6c46c316d2bf603518ce404dea21134061d0ff50f2b9248d3cbcb94c9ab5，本机服务 manifest/包一致；本机实装未验。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
       <x:c r="I14" s="90" t="str">
-        <x:v>0.3.7 最终候选的旧库隔离副本脚本、源码门禁、打包全量和本机服务制品有通过证据；TC-095 当前 Mac 实装、UI 授权/CSV、兼容旧备份回退待人工验收，故版本交付未完成；真实 CLI owner/完整覆盖/真零/同比和异机发布另待验</x:v>
+        <x:v>0.3.7 当前 Mac 未签名本机交付门槛完成，TC-095 人工 pass：真实安装、受信登录、来源/历史待核对报表与 CSV、旧事实保留、兼容旧版隔离回退和同候选隔离五故障恢复/重试有证据。VER-009 完整三批范围与外部分发仍未全部完成；REQ-040 完整覆盖/真零/同比及 TC-028/072 仍待验</x:v>
       </x:c>
       <x:c r="J14" s="90" t="str">
         <x:v>7fd0ce7 本机门禁 94/97/44、目录包管理员 5/5、打包全量 44/44；TC-076 隔离通过。生产迁移、系统安装、TC-028/072 与完整三批范围仍待验，见 docs/validation.md。
@@ -10851,7 +10862,9 @@
 2026-10-04 需求会话仓库外备份并独立对照报告（文档会话未复验）：同一授权旧库备份副本在 0.3.5 启动时基础表数量稳定；待固定的 0.3.7 候选启动后旧 claude:macos 身份退役，旧事实转 legacy-unverified 待核对，来源身份行有可解释净变化；users/facts/cursors 数量、事实计量字段排序摘要和 Token 合计保持，integrity_check=ok，第二次启动幂等。此报告不含原始身份或私有计数；仍须逐事实映射、UI 待核对与 viewer 隔离、兼容备份回退证据，TC-095 不升通过。
 2026-10-04 固定代码 c359e6a；开发报告 test:gate 95/103/46 通过、TC-077/078/084 各单编号通过，打包全量 45/46+TC-038 单项复跑；当前 0.3.7 DMG SHA 86a0817d…、hdiutil VALID。需求会话独立做旧/新 App 备份副本身份迁移对照；文档会话未独立复验。
 2026-10-04 需求会话独立在 c359e6a/0.3.7 目录包执行 npm run test:e2e:packaged，46/46、退出码 0，TC-038 末尾约 3.5 秒通过；开发先前 45/46 超时保留历史。文档会话未独立复跑，TC-095/生产库副本 verifier 仍待验。
-2026-10-04 ee617f3：开发报告 test:production-copy 授权备份副本退出 0；首轮 test:gate TC-073 耗时阈值失败，单编号及第二轮 95/103/46 通过；最终重建目录包 test:e2e:packaged 46/46。文档会话未复跑动态测试，独立只读核最终 DMG/本机服务 manifest 大小和 SHA 一致、hdiutil VALID；不记录生产私有计数。</x:v>
+2026-10-04 ee617f3：开发报告 test:production-copy 授权备份副本退出 0；首轮 test:gate TC-073 耗时阈值失败，单编号及第二轮 95/103/46 通过；最终重建目录包 test:e2e:packaged 46/46。文档会话未复跑动态测试，独立只读核最终 DMG/本机服务 manifest 大小和 SHA 一致、hdiutil VALID；不记录生产私有计数。
+2026-10-04 当前 Mac 人工子证据（开发侧脱敏记录，文档会话仅只读核安装 App）：固定 ee617f3/0.3.7，从 0.3.5 UI 自动更新至 /Applications/Token.app 0.3.7，管理员受信登录、Codex/Claude 主动扫描、历史 uncertain 报表/pending 明细/CSV v2 待核对与已确认小计对账、旧账户/事实计量保留、旧 App+升级前库+受信秘密隔离回退；实际安装可执行文件权限负例 1/1。文档会话核 App 版本和 app.asar SHA；未读生产库或复跑 UI/回退。缺同一 0.3.7 候选的隔离故障注入及失败后重试，TC-095 未通过。
+2026-10-04 同候选故障补证：开发会话用真实 0.3.6 DMG SHA 8773dd38… 与最终 0.3.7 DMG SHA dd4c6c46…，在隔离临时路径/合成数据执行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，退出码 0；installer 模块和打包 helper 各对 mount/space/replace/launch/health 五故障验证旧版恢复、受信登录、合成报表保留、残留清理与重试。连同当前 Mac 实际安装/来源/待核对报表与 CSV/旧事实保留/兼容旧版隔离回退证据，开发会话登记 npm run test:case -- TC-095 pass，退出码 0；被 Git 忽略的 test-results/manual/TC-095.json 为 pass，文档会话只读核记录，未独立复跑。只认当前 Mac 未签名范围，不声称真实满盘/断电或生产故障；TC-028/072、REQ-040 完整覆盖/真零/同比仍待验。</x:v>
       </x:c>
       <x:c r="K14" s="90" t="str">
         <x:v>保留 REQ-040–048/TC-077–094 全范围；先修 TC-079/021，再逐项补覆盖真零、服务状态、VoiceOver、来源/生产迁移及 TC-076/028/072 发布证据
@@ -10862,7 +10875,9 @@
 2026-10-04 制品代次门槛：当前 /Applications/Token.app 0.3.5 与服务中旧 0.3.6 SHA-256 8773dd…均为既有候选；若验收包含其后新增功能，须先冻结包含该功能的代码提交，按仓库规则给出唯一且高于已安装/已发布候选的版本及新 DMG SHA-256，核 manifest 指向同一新制品后才从当前 Mac 实装验收。具体版本由开发统筹确定，不复用旧 0.3.6 包证新功能。
 以同一授权备份副本修订并复跑迁移对账：解释每个新增 legacy-unverified 身份、事实逐键/逐数值、owner/小计/待核对与 viewer 隔离，另核旧版兼容备份回退；不得对生产原库做自动写入。
 先修生产库副本 verifier 并复跑同一备份，重建/冻结最终候选并核同候选打包全量及 TC-095 当前 Mac 人工实装；未完成前不发布。真实 provider 归属、source-complete/真零/同比另按 REQ-040/044 验。
-当前下一步：以 ee617f3 /最终 0.3.7 同一候选完成 TC-095 本机实际安装、管理员/viewer UI 与报表/CSV 核对、兼容旧版 App 加升级前库备份回退；取得脱敏人工证据后才判本机交付。</x:v>
+当前下一步：以 ee617f3 /最终 0.3.7 同一候选完成 TC-095 本机实际安装、管理员/viewer UI 与报表/CSV 核对、兼容旧版 App 加升级前库备份回退；取得脱敏人工证据后才判本机交付。
+当前唯一 TC-095 收尾缺口：以固定 ee617f3/最终 0.3.7 候选做隔离升级故障注入和失败后重试，核旧版恢复、数据/受信状态、残留清理；留脱敏证据后再判断本机交付。TC-028/072 仍为未来签名/异机验收，不随本次状态提升。
+本机 TC-095 已 pass；后续分别完成 REQ-040 可证完整覆盖/真零/同比与真实 provider owner，完整三批其余待验项，资源具备后另做 TC-028/072 签名/异机验收。隔离故障结果不外推真实满盘/断电。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="84" customHeight="1">

</xml_diff>

<commit_message>
feat: move exact token copy into number hover menu
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rca59d20063494a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R2c087390274843fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rcb5990b19daa4cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Ra9349c6b6a4c433e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R1914e6945da74986"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5166c62f4a0a41b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6b9ec0d695d04934"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R06232375ecb44910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R73465f461c384c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rf659d5a238ab4fcc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4493,7 +4493,8 @@
         <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
 设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。
 来源重绑预览弹窗须实际隔离背景键盘操作，焦点进入弹窗并留在其中；取消/Escape/失败后焦点回触发控件，成功刷新移除触发控件时回来源列表稳定标题。标准与窄窗口主路径焦点顺序可见。概览、趋势、排行、报表、明细所有 Token 精确整数及覆盖状态须非悬浮可读；引导、空状态、诊断、重绑、服务、更新文案与真实角色/状态/动作一致。
-精确 Token 原始十进制整数还须能纯键盘复制；可选可选中文本或有字段/范围名称的复制按钮，带可读反馈和合理焦点。缩写、title 或 CSV 不是复制入口；未知/待核对不可复制假完整总量。重绑弹窗背景对辅助技术导航也不可达。</x:v>
+精确 Token 原始十进制整数还须能纯键盘复制；可选可选中文本或有字段/范围名称的复制按钮，带可读反馈和合理焦点。缩写、title 或 CSV 不是复制入口；未知/待核对不可复制假完整总量。重绑弹窗背景对辅助技术导航也不可达。
+交互细化：缩写 Token 数字悬停时显示完整十进制整数和“复制完整数值”；数字聚焦后同样可打开并键盘复制。常驻“复制原值”按钮移入菜单；未知/未覆盖无假零入口。</x:v>
       </x:c>
       <x:c r="D52" s="58" t="str">
         <x:v>下一轮产品打磨（计划）</x:v>
@@ -6009,7 +6010,8 @@
 修正设置页遥测卡按整日覆盖的过时文案，描述 owner/会话独立事实保留、疑似重叠待核对及完整总量不可确认；与报表/CSV 实际状态和行动一致，TC-091 验。
 第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。
 为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。
-2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 遥测文案与疑似重叠报表/CSV v2 已测；TC-089/090 未注册。</x:v>
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 遥测文案与疑似重叠报表/CSV v2 已测；TC-089/090 未注册。
+本轮交互细化：将概览、趋势、排行、报表指标和明细的常驻复制按钮改为数字悬停/聚焦菜单。保留完整整数、复制反馈和键盘路径，菜单不被滚动容器裁切。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -10093,12 +10095,14 @@
       <x:c r="F95" s="58" t="str">
         <x:v>无 hover、仅键盘/朗读方式查看概览、趋势、模型排行及明细。
 以 0、1023、1024、超过 1M、待核对合成事实，在无 hover 条件下查概览总量/输入输出、每个趋势桶、排行、报表指标、明细输入/输出/缓存/总量及覆盖状态。
-对概览、趋势、排行、报表指标和明细所有 Token 字段，仅用键盘复制精确整数并粘贴核对；覆盖 0、1023、1024、超过 1M 和待核对。</x:v>
+对概览、趋势、排行、报表指标和明细所有 Token 字段，仅用键盘复制精确整数并粘贴核对；覆盖 0、1023、1024、超过 1M 和待核对。
+本轮追加：鼠标悬停数字显示完整数值及复制项；离开时关闭。纯键盘聚焦数字后 Tab 到复制项，Enter 复制整数，Escape 关闭并回到数字；检查 700px 布局及滚动容器不裁切。</x:v>
       </x:c>
       <x:c r="G95" s="58" t="str">
         <x:v>精确原值与覆盖状态有可见文本或可聚焦可读入口，不仅藏在 title/tooltip。
 每个 Token 精确整数可见或在键盘可聚焦且有名称的详情入口读取；K/M/P 仅视觉摘要，title/tooltip 与 CSV 不可为唯一精确值来源。覆盖未知/总量不可确认可读，已确认小计 0 不作完整真零。
-复制结果为当前授权范围该字段的原始十进制整数，不是 K/M/P、title 或整页文本；操作反馈可读且焦点合理。未知/总量不可确认时不提供假完整总量 0。</x:v>
+复制结果为当前授权范围该字段的原始十进制整数，不是 K/M/P、title 或整页文本；操作反馈可读且焦点合理。未知/总量不可确认时不提供假完整总量 0。
+常驻“复制原值”按钮消失；悬停/聚焦菜单显示正确的完整十进制整数并能复制。键盘入口与反馈保留，未知/待核对仍遵守原有边界。</x:v>
       </x:c>
       <x:c r="H95" s="58" t="str">
         <x:v>已注册；原始整数键盘复制隔离自动子范围通过，打包/真实工具待验</x:v>

</xml_diff>

<commit_message>
docs: record 0.3.8 local menu acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5166c62f4a0a41b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R6b9ec0d695d04934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R06232375ecb44910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R73465f461c384c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rf659d5a238ab4fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R1a519b8a255e4979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rdda6c424b21348af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R88bfda2966774243"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R87c66315eaa641e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R438973c536774964"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2961,7 +2961,8 @@
         <x:v>精确 Token 与覆盖状态非悬浮可读</x:v>
       </x:c>
       <x:c r="G96" s="68" t="str">
-        <x:v>精确值复制自动子范围通过；打包/真实工具待验</x:v>
+        <x:v>精确值复制自动子范围通过；打包/真实工具待验
+0.3.8 数字悬停/聚焦菜单已在当前 Mac 安装包的隔离自动子范围通过；真实工具及 VoiceOver 仍待验</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="85" customHeight="1">
@@ -4514,7 +4515,8 @@
 2026-10-03 静态核对 settings.tsx 仍有“同一天有本地记录时，报表采用本地记录”过时文案；纳入 TC-091，未改代码/未运行。
 2026-10-03 第三批实施前细化：当前 overview.tsx/report.tsx 多处精确值仅 title，report.tsx 还写“悬浮可查看精确值”。来源重绑弹窗尚待实现，aria-modal 不足以保证背景 Tab 隔离。TC-089 目标 Mac VoiceOver 人工证据与 Electron 自动子范围分开。未改代码/未执行。
 2026-10-03 基线 4b3ff02 静态核对：概览/报表多处精确值只在 title，无纯键盘复制路径；弹窗目前仅少量 Tab/Escape 自动断言，VoiceOver 背景隔离待验。
-2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 1 单元+1 Electron；TC-089/090 未注册，TC-091 其余文案动作矩阵未覆盖。</x:v>
+2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 1 单元+1 Electron；TC-089/090 未注册，TC-091 其余文案动作矩阵未覆盖。
+2026-10-04 代码 87fa4c6 / 本机未签名 0.3.8：数字悬停及聚焦菜单已装机，TC-090 安装包隔离 2/2；完整 REQ-047 仍受 VoiceOver 人工、真零与全状态走查限制。</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="170" customHeight="1">
@@ -6011,7 +6013,8 @@
 第三批门槛：标准/窄窗口键盘走登录、导航、重绑、概览下钻、明细返回、诊断/设置；焦点顺序、可见性和固定栏遮挡可测。弹窗背景实际 inert/不可 Tab，打开聚焦，Tab 留在弹窗；取消/Escape 无写入、失败错误可读并回焦，成功触发控件消失时聚焦来源列表。概览/趋势/排行/报表/明细每个 Token 精确值有非 hover 可见或可聚焦入口，title/CSV 不能是唯一来源。建立状态/角色/文案/动作矩阵；TC-089 目标 Mac VoiceOver 单独证据。
 为概览、趋势、排行、报表、明细每个 Token 精确值提供可读且可纯键盘复制的原始整数；复制按钮若有须有字段/范围名称、反馈和焦点行为。TC-090 粘贴比对；TC-089 另验来源重绑弹窗背景在辅助技术导航中不可达；TC-091 核状态组合文案和动作。
 2026-10-03 代码 41838d8：文档会话独立复跑单编号与完整门禁；92 个已注册入口、76/76 单元、34/34 Electron，通过。仅隔离合成自动子范围；真实远端、生产库与打包应用未验。 TC-091 遥测文案与疑似重叠报表/CSV v2 已测；TC-089/090 未注册。
-本轮交互细化：将概览、趋势、排行、报表指标和明细的常驻复制按钮改为数字悬停/聚焦菜单。保留完整整数、复制反馈和键盘路径，菜单不被滚动容器裁切。</x:v>
+本轮交互细化：将概览、趋势、排行、报表指标和明细的常驻复制按钮改为数字悬停/聚焦菜单。保留完整整数、复制反馈和键盘路径，菜单不被滚动容器裁切。
+2026-10-04 代码 87fa4c6：常驻复制按钮已移入数字菜单；源码门禁 103/103 单元、46/46 Electron；目录包 46/46；当前 Mac 安装包隔离 TC-090 2/2。</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="165" customHeight="1">
@@ -10105,14 +10108,17 @@
 常驻“复制原值”按钮消失；悬停/聚焦菜单显示正确的完整十进制整数并能复制。键盘入口与反馈保留，未知/待核对仍遵守原有边界。</x:v>
       </x:c>
       <x:c r="H95" s="58" t="str">
-        <x:v>已注册；原始整数键盘复制隔离自动子范围通过，打包/真实工具待验</x:v>
+        <x:v>已注册；原始整数键盘复制隔离自动子范围通过，打包/真实工具待验
+已注册；0.3.8 数字菜单源码、打包及当前 Mac 安装包隔离自动子范围通过；真实工具/VoiceOver 待验</x:v>
       </x:c>
       <x:c r="I95" s="68" t="str">
         <x:v>当前 6a194ea：文档会话单编号 Electron 2/2；实际剪贴板 0/1023/1024/1050000、字段 Tab 顺序、700px 无横溢、待核对/未知边界。
-2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。</x:v>
+2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
+2026-10-04 87fa4c6 / macOS 15.7.4 x86_64 / 0.3.8：TC-090 2/2、TC-048 1/1，test:gate 103/103 单元及 46/46 Electron，test:e2e:packaged 46/46，实际 /Applications/Token.app 的隔离 TC-090 2/2。DMG SHA-256 3eee22fdb510661ee7ada501fd4039850a78510403acd2bbf901b40666a32b44；app.asar 3d0666ff506815e1c68df65504932d99e14a992969781f177c42c6502ff57545。</x:v>
       </x:c>
       <x:c r="J95" s="58" t="str">
-        <x:v>npm run test:case -- TC-090（2026-10-03 独立实测退出码 0）</x:v>
+        <x:v>npm run test:case -- TC-090（2026-10-03 独立实测退出码 0）
+npm run test:case -- TC-090；npm run test:case -- TC-048；npm run test:gate；npm run test:e2e:packaged；TOKEN_E2E_EXECUTABLE=/Applications/Token.app/Contents/MacOS/Token npx playwright test tests/e2e/exact-tokens.spec.ts（均退出码 0，2026-10-04）</x:v>
       </x:c>
       <x:c r="K95" s="58" t="str">
         <x:v>scripts/test-cases.mjs：tests/e2e/exact-tokens.spec.ts 2 个 TC-090 Electron 独立绑定。</x:v>
@@ -10121,7 +10127,8 @@
         <x:v>当前自动边界：概览/趋势/排行/项目模型/报表指标/明细原始整数可复制；真实工具格式、打包 App 与目标 Mac 辅助技术待验。
 只使用独立临时用户数据/SQLite 与无正文合成 Codex/Claude 记录；人工目标 Mac 项另留脱敏系统证据。
 当前 overview.tsx/report.tsx 多处精确值仅 title；核所有字段和边界值，不只看主指标。
-当前 title 是多处唯一精确值来源；需自动读取隔离剪贴板或等价粘贴结果，核每类字段及状态。</x:v>
+当前 title 是多处唯一精确值来源；需自动读取隔离剪贴板或等价粘贴结果，核每类字段及状态。
+2026-10-04 新边界：已在当前 Mac 实际安装的可执行文件用隔离账户/无正文合成样本验证菜单；未以真实私人来源数据做人工菜单走查，也未完成 VoiceOver 人工朗读。旧“打包 App 待验”描述仅适用于 6a194ea 阶段。</x:v>
       </x:c>
       <x:c r="M95" s="58" t="str">
         <x:v>固定代码 6a194ea；macOS x86_64、Node v24.15.0，TC-090 Electron 2/2 退出码 0；无安装包或目标 Mac 人工证据。</x:v>
@@ -10469,7 +10476,8 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="77" t="str">
-        <x:v>截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。</x:v>
+        <x:v>截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。
+2026-10-04 VER-011 为插入的本机 0.3.8 数字菜单修订；VER-010 仍是未立项的后续菜单栏方向。</x:v>
       </x:c>
       <x:c r="B2" s="77"/>
       <x:c r="C2" s="77"/>
@@ -10919,6 +10927,41 @@
         <x:v>当前三批打磨及发布门槛先收尾；未来明确范围后再定版本号、任务和用例</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>VER-011</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>0.3.8（当前 Mac 本机未签名交互修订）</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>数字完整数值菜单</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>将概览、趋势、排行、项目/模型、报表指标及明细的常驻“复制原值”移入数字悬停/聚焦菜单；保持精确整数键盘复制、未知/待核对边界。</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>TC-090；趋势布局交叉回归 TC-048</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>87fa4c6；源码门禁 103/103 单元、46/46 Electron；目录包全量 46/46；当前 Mac 实装包隔离 TC-090 2/2。</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>本机菜单交互自动子范围通过；未签名本机版已安装。完整 REQ-047 与外部分发未完成。</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>2026-10-04 macOS 15.7.4 x86_64；/Applications/Token.app 0.3.8；DMG SHA-256 3eee22fdb510661ee7ada501fd4039850a78510403acd2bbf901b40666a32b44；app.asar SHA-256 3d0666ff506815e1c68df65504932d99e14a992969781f177c42c6502ff57545。0.3.7 App 与升级前用户数据已存本机受限备份。</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>保留 0.3.7 TC-095 的历史范围；0.3.8 仅补本轮菜单及相关回归，真实工具/VoiceOver 和签名公证仍待独立验收。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>

</xml_diff>

<commit_message>
Refine usage pages and ship local 0.3.11
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R0fe93209bb984b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rfe365a0fa5e146cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rbf6f739cc60847c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Redc3287d5d164c89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R0d26bf5254594122"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re92b59e81cdf4f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re6f3cbe9dc8b4417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2676777626584123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R93db8671ef0b423b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R7caa8f15ac6f4a39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="40">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -266,6 +266,11 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F6FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -296,7 +301,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="98">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -549,6 +554,13 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -4573,6 +4585,121 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="103" ht="170" customHeight="1">
+      <x:c r="A103" s="100" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="B103" s="100" t="str">
+        <x:v>本机采集与可选服务上报分离</x:v>
+      </x:c>
+      <x:c r="C103" s="100" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="D103" s="100" t="str">
+        <x:v>分离本机采集与服务上报状态</x:v>
+      </x:c>
+      <x:c r="E103" s="100" t="str">
+        <x:v>TC-097</x:v>
+      </x:c>
+      <x:c r="F103" s="100" t="str">
+        <x:v>页头一行状态与详细诊断</x:v>
+      </x:c>
+      <x:c r="G103" s="100" t="str">
+        <x:v>2026-10-05 TC-097 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="170" customHeight="1">
+      <x:c r="A104" s="100" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="B104" s="100" t="str">
+        <x:v>窄窗口与无障碍精确值</x:v>
+      </x:c>
+      <x:c r="C104" s="100" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D104" s="100" t="str">
+        <x:v>补齐键盘 VoiceOver 精确值及文案走查</x:v>
+      </x:c>
+      <x:c r="E104" s="100" t="str">
+        <x:v>TC-098</x:v>
+      </x:c>
+      <x:c r="F104" s="100" t="str">
+        <x:v>KPI 输入输出完整显示与精确原值</x:v>
+      </x:c>
+      <x:c r="G104" s="100" t="str">
+        <x:v>2026-10-05 TC-098 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="170" customHeight="1">
+      <x:c r="A105" s="100" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="B105" s="100" t="str">
+        <x:v>筛选异步加载与 CSV 同一查询</x:v>
+      </x:c>
+      <x:c r="C105" s="100" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="D105" s="100" t="str">
+        <x:v>统一异步查询键与页面 CSV 快照</x:v>
+      </x:c>
+      <x:c r="E105" s="100" t="str">
+        <x:v>TC-099</x:v>
+      </x:c>
+      <x:c r="F105" s="100" t="str">
+        <x:v>报表筛选摘要与当前快照一致</x:v>
+      </x:c>
+      <x:c r="G105" s="100" t="str">
+        <x:v>2026-10-05 TC-099 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="170" customHeight="1">
+      <x:c r="A106" s="100" t="str">
+        <x:v>REQ-049</x:v>
+      </x:c>
+      <x:c r="B106" s="100" t="str">
+        <x:v>单用户 Mac 的 Claude 本地来源默认归属</x:v>
+      </x:c>
+      <x:c r="C106" s="100" t="str">
+        <x:v>DEV-058</x:v>
+      </x:c>
+      <x:c r="D106" s="100" t="str">
+        <x:v>单用户本机 Claude 来源默认归属</x:v>
+      </x:c>
+      <x:c r="E106" s="100" t="str">
+        <x:v>TC-100</x:v>
+      </x:c>
+      <x:c r="F106" s="100" t="str">
+        <x:v>单用户来源汇总与异常优先列表</x:v>
+      </x:c>
+      <x:c r="G106" s="100" t="str">
+        <x:v>2026-10-05 TC-100 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="170" customHeight="1">
+      <x:c r="A107" s="100" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="B107" s="100" t="str">
+        <x:v>可跳过的首次使用四步引导</x:v>
+      </x:c>
+      <x:c r="C107" s="100" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D107" s="100" t="str">
+        <x:v>实现角色感知的可跳过首次引导</x:v>
+      </x:c>
+      <x:c r="E107" s="100" t="str">
+        <x:v>TC-101</x:v>
+      </x:c>
+      <x:c r="F107" s="100" t="str">
+        <x:v>首次引导下一步与操作后即时进度</x:v>
+      </x:c>
+      <x:c r="G107" s="100" t="str">
+        <x:v>2026-10-05 TC-101 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6419,32 +6546,27 @@
           <x:t xml:space="preserve">筛选异步加载与 CSV 同一查询</x:t>
         </x:is>
       </x:c>
-      <x:c r="C46" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。
+      <x:c r="C46" s="58" t="str">
+        <x:v>用户切换筛选时页面只显示与当前请求键匹配的结果；旧请求晚返回不得覆盖新结果。页面和 CSV 必须使用同一授权筛选、时区及可核对的数据库 revision/快照身份；查询完成后再扫描入库，仍须导出屏显的同一事实集合，或先刷新页面再允许导出；加载期间禁用旧结果导出。
 2026-10-04 打包缺陷验收补充：在用量报表连续快速修改开始和结束日期，两输入值均须保持最终选择；查询只使用最终起止日期组合，无倒置范围错误。当前屏显结果与 CSV 必须使用同一授权筛选、时区和快照，期间旧请求不得覆写新组合。
-2026-10-04 当前澄清：保持原生日期输入与现有范围校验；最终报表查询及页面、明细、CSV 同授权筛选/时区/snapshotId 的原要求不变。打包异常先按跨页模糊测试定位修复，不增设文本输入或双日期提交产品需求。</x:t>
-        </x:is>
+2026-10-04 当前澄清：保持原生日期输入与现有范围校验；最终报表查询及页面、明细、CSV 同授权筛选/时区/snapshotId 的原要求不变。打包异常先按跨页模糊测试定位修复，不增设文本输入或双日期提交产品需求。
+2026-10-05 页面打磨：报表将当前日期、时区、工具、模型、项目、授权用户集中显示为可读筛选摘要；筛选变化和 CSV 导出继续绑定同一当前快照，避免重复的长句说明。</x:v>
       </x:c>
       <x:c r="D46" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">下一轮产品打磨（第一批 B 阶段实现）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E46" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">异步/快照及修正定位后的日期自动子范围通过；产品原生日期控件未改，真实生产/系统验收未覆盖</x:t>
-        </x:is>
+      <x:c r="E46" s="58" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨当前 Mac 隔离自动验收通过，安装后人工状态另记。</x:v>
       </x:c>
       <x:c r="F46" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-050</x:t>
         </x:is>
       </x:c>
-      <x:c r="G46" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-079</x:t>
-        </x:is>
+      <x:c r="G46" s="58" t="str">
+        <x:v>TC-079、TC-099</x:v>
       </x:c>
       <x:c r="H46" s="58" t="inlineStr">
         <x:is>
@@ -6512,7 +6634,8 @@
         </x:is>
       </x:c>
       <x:c r="C48" s="58" t="str">
-        <x:v>首次安装完成初始管理员建账后自动进入检测→扫描→归属→第一笔用量四步引导，可跳过或完成后进入工作台；已有安装升级、再次启动/登录及后建账户不自动显示，侧边栏与概览无常驻入口或提示。每步只显示真实完成状态；管理员可执行来源归属，普通用户只看授权用量及请求管理员操作指引；不自动重绑或读取额外文件。</x:v>
+        <x:v>首次安装完成初始管理员建账后自动进入检测→扫描→归属→第一笔用量四步引导，可跳过或完成后进入工作台；已有安装升级、再次启动/登录及后建账户不自动显示，侧边栏与概览无常驻入口或提示。每步只显示真实完成状态；管理员可执行来源归属，普通用户只看授权用量及请求管理员操作指引；不自动重绑或读取额外文件。
+2026-10-05 页面打磨：首次引导每次突出一个下一步动作；扫描或归属操作后返回引导立即刷新真实进度，完成后可结束，随时可跳过，且不恢复常驻侧栏入口。</x:v>
       </x:c>
       <x:c r="D48" s="58" t="inlineStr">
         <x:is>
@@ -6520,17 +6643,15 @@
         </x:is>
       </x:c>
       <x:c r="E48" s="58" t="str">
-        <x:v>已实现；TC-082/083 隔离与打包自动范围通过；本机 0.3.10 已安装启动</x:v>
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨当前 Mac 隔离自动验收通过，安装后人工状态另记。</x:v>
       </x:c>
       <x:c r="F48" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-052</x:t>
         </x:is>
       </x:c>
-      <x:c r="G48" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-082、TC-083</x:t>
-        </x:is>
+      <x:c r="G48" s="58" t="str">
+        <x:v>TC-082、TC-083、TC-101</x:v>
       </x:c>
       <x:c r="H48" s="58" t="str">
         <x:v>独立新能力；与现有首次建账及角色授权兼容。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。 详见 docs/design.md §20、docs/development-plan.md §12、docs/test-case-acceptance.md。
@@ -6660,33 +6781,28 @@
           <x:t xml:space="preserve">本机采集与可选服务上报分离</x:t>
         </x:is>
       </x:c>
-      <x:c r="C51" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。
+      <x:c r="C51" s="55" t="str">
+        <x:v>本机采集、报表覆盖和可选服务连接/待传上报分别显示状态；未配置服务为未配置而非采集故障，服务离线不阻断本机扫描或报表。配置服务后显示积压与重试，受授权范围限制。
 若某范围因用量冲突或上报协议不兼容而暂停同步，显示“待核对/未同步”及原因，不归入网络离线、零用量或扫描失败。
 服务状态须由主进程明确配置来源/类型判定，区分默认内置回环服务、未配置远端、远端已配置在线/离线/授权失败/旧协议、积压与待核对；不能仅从 hasToken 或 online 猜远端配置。设置页和页头须与真实服务状态一致，本地扫描/报表独立。
-服务类型/显式远端配置、网络/认证/协议、当前 revision 待传/已确认、待核对聚合、本地扫描与历史覆盖为正交状态；旧 lastSuccess 或 pending=0 不能单独证明当前 revision 已同步。并存状态须同时可见。</x:t>
-        </x:is>
+服务类型/显式远端配置、网络/认证/协议、当前 revision 待传/已确认、待核对聚合、本地扫描与历史覆盖为正交状态；旧 lastSuccess 或 pending=0 不能单独证明当前 revision 已同步。并存状态须同时可见。
+2026-10-05 页面打磨：页头把本机采集、授权范围覆盖和服务同步分别压缩为一行可读状态；点击后展开原有详细状态和诊断入口。扫描成功不能冒充历史覆盖完整，服务待传不能冒充本机采集失败。</x:v>
       </x:c>
       <x:c r="D51" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">下一轮产品打磨（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E51" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">部分实现；服务状态自动子范围通过，重绑误报已修，真实远端/打包待验</x:t>
-        </x:is>
+      <x:c r="E51" s="55" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨当前 Mac 隔离自动验收通过，安装后人工状态另记。</x:v>
       </x:c>
       <x:c r="F51" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-055</x:t>
         </x:is>
       </x:c>
-      <x:c r="G51" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-088</x:t>
-        </x:is>
+      <x:c r="G51" s="55" t="str">
+        <x:v>TC-088、TC-097</x:v>
       </x:c>
       <x:c r="H51" s="69" t="inlineStr">
         <x:is>
@@ -6709,34 +6825,29 @@
           <x:t xml:space="preserve">窄窗口与无障碍精确值</x:t>
         </x:is>
       </x:c>
-      <x:c r="C52" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
+      <x:c r="C52" s="58" t="str">
+        <x:v>窄窗口仍可键盘完成主路径，焦点可见且顺序合理，VoiceOver 可读控件名称/状态；Token 精确值及覆盖状态在页面可见文本中可获取，不依赖悬浮。关键引导、空状态、诊断、更新文案与动作一致并经逐项走查。
 设置页遥测说明须符合 DEV-057：不同 owner/会话的独立事实保留，疑似重叠显示待核对与完整总量不可确认；不得声称同日有本地记录即舍弃遥测。
 来源重绑预览弹窗须实际隔离背景键盘操作，焦点进入弹窗并留在其中；取消/Escape/失败后焦点回触发控件，成功刷新移除触发控件时回来源列表稳定标题。标准与窄窗口主路径焦点顺序可见。概览、趋势、排行、报表、明细所有 Token 精确整数及覆盖状态须非悬浮可读；引导、空状态、诊断、重绑、服务、更新文案与真实角色/状态/动作一致。
 精确 Token 原始十进制整数还须能纯键盘复制；可选可选中文本或有字段/范围名称的复制按钮，带可读反馈和合理焦点。缩写、title 或 CSV 不是复制入口；未知/待核对不可复制假完整总量。重绑弹窗背景对辅助技术导航也不可达。
-交互细化：缩写 Token 数字悬停时显示完整十进制整数和“复制完整数值”；数字聚焦后同样可打开并键盘复制。常驻“复制原值”按钮移入菜单；未知/未覆盖无假零入口。</x:t>
-        </x:is>
+交互细化：缩写 Token 数字悬停时显示完整十进制整数和“复制完整数值”；数字聚焦后同样可打开并键盘复制。常驻“复制原值”按钮移入菜单；未知/未覆盖无假零入口。
+2026-10-05 页面打磨：概览及报表 KPI 的输入、输出值在标准及窄窗口完整可见，不以省略号截断；缩写值继续支持悬停、键盘聚焦、复制精确整数。覆盖未知与可证真零保留不同文案。</x:v>
       </x:c>
       <x:c r="D52" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">下一轮产品打磨（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E52" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">部分实现；TC-089/090/091 隔离自动子范围通过，人工 VoiceOver/真零/发布待验</x:t>
-        </x:is>
+      <x:c r="E52" s="58" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨当前 Mac 隔离自动验收通过，安装后人工状态另记。</x:v>
       </x:c>
       <x:c r="F52" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-056</x:t>
         </x:is>
       </x:c>
-      <x:c r="G52" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-089、TC-090、TC-091</x:t>
-        </x:is>
+      <x:c r="G52" s="58" t="str">
+        <x:v>TC-089、TC-090、TC-091、TC-098</x:v>
       </x:c>
       <x:c r="H52" s="68" t="inlineStr">
         <x:is>
@@ -6835,30 +6946,25 @@
           <x:t xml:space="preserve">单用户 Mac 的 Claude 本地来源默认归属</x:t>
         </x:is>
       </x:c>
-      <x:c r="C54" s="61" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">同一 macOS 用户资料下只有一个有效 Token 管理员账户时，当前可读取、文件代次可确认的 Claude 本地文件来源自动归属该账户，已存在的可确认来源在再次进入或扫描后同样处理；不要求逐文件填写外部登记。界面标明这是本机使用者归属，不等于 Claude 提供方账号验证。多 Token 账户、文件代次不明、旧库混合来源、遥测身份未知、手动解除归属和扫描失败保持未归属/待核对，不能变为已确认零；自动归属有脱敏审计，重复扫描幂等，viewer 与服务端仅见授权范围。</x:t>
-        </x:is>
+      <x:c r="C54" s="61" t="str">
+        <x:v>同一 macOS 用户资料下只有一个有效 Token 管理员账户时，当前可读取、文件代次可确认的 Claude 本地文件来源自动归属该账户，已存在的可确认来源在再次进入或扫描后同样处理；不要求逐文件填写外部登记。界面标明这是本机使用者归属，不等于 Claude 提供方账号验证。多 Token 账户、文件代次不明、旧库混合来源、遥测身份未知、手动解除归属和扫描失败保持未归属/待核对，不能变为已确认零；自动归属有脱敏审计，重复扫描幂等，viewer 与服务端仅见授权范围。
+2026-10-05 页面打磨：单用户来源页默认按 Codex 与 Claude Code 汇总已归属来源，展开待处理异常；正常已归属文件默认收起且不逐行显示归属下拉框。手动检查和更改归属仍可进入，未知身份/旧来源不隐藏。</x:v>
       </x:c>
       <x:c r="D54" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">当前交互修订</x:t>
         </x:is>
       </x:c>
-      <x:c r="E54" s="61" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">本机 0.3.9 范围通过；其他 Mac 未验</x:t>
-        </x:is>
+      <x:c r="E54" s="61" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨当前 Mac 隔离自动验收通过，安装后人工状态另记。</x:v>
       </x:c>
       <x:c r="F54" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-058</x:t>
         </x:is>
       </x:c>
-      <x:c r="G54" s="61" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-096</x:t>
-        </x:is>
+      <x:c r="G54" s="61" t="str">
+        <x:v>TC-096、TC-100</x:v>
       </x:c>
       <x:c r="H54" s="61" t="inlineStr">
         <x:is>
@@ -8828,20 +8934,16 @@
           <x:t xml:space="preserve">REQ-041</x:t>
         </x:is>
       </x:c>
-      <x:c r="D55" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-079</x:t>
-        </x:is>
+      <x:c r="D55" s="58" t="str">
+        <x:v>TC-079、TC-099</x:v>
       </x:c>
       <x:c r="E55" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">src/main/report.ts、index.ts；src/preload/index.ts；src/renderer/report.tsx；src/shared/types.ts；tests/report-snapshot.test.ts、tests/e2e/report-snapshot.spec.ts；scripts/test-cases.mjs、run-test-case.mjs</x:t>
         </x:is>
       </x:c>
-      <x:c r="F55" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">既有查询/快照实现与测试定位修复的自动子范围通过；7fd0ce7 未改产品日期控件，生产环境待验</x:t>
-        </x:is>
+      <x:c r="F55" s="58" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨实现并通过独立 TC、源码门槛与打包应用回归。</x:v>
       </x:c>
       <x:c r="G55" s="58" t="inlineStr">
         <x:is>
@@ -8909,10 +9011,8 @@
           <x:t xml:space="preserve">REQ-043</x:t>
         </x:is>
       </x:c>
-      <x:c r="D57" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-082、TC-083</x:t>
-        </x:is>
+      <x:c r="D57" s="58" t="str">
+        <x:v>TC-082、TC-083、TC-101</x:v>
       </x:c>
       <x:c r="E57" s="58" t="inlineStr">
         <x:is>
@@ -8920,7 +9020,7 @@
         </x:is>
       </x:c>
       <x:c r="F57" s="58" t="str">
-        <x:v>已实现；TC-082/083 隔离与打包自动范围通过；本机 0.3.10 已安装启动</x:v>
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨实现并通过独立 TC、源码门槛与打包应用回归。</x:v>
       </x:c>
       <x:c r="G57" s="58" t="str">
         <x:v>四步只读真实状态；跳过可重开；viewer 不出现管理员绑定动作，任何状态写入受主进程角色校验。 2026-10-03 SOP-001/002 前置规划；仅需求/设计/验收口径，尚无产品实现、新测试绑定或通过结果。独立测试须使用各自临时数据库、用户数据与无正文合成样本；执行后另记固定提交、环境、命令、退出码和脱敏证据。
@@ -9036,20 +9136,16 @@
           <x:t xml:space="preserve">REQ-046</x:t>
         </x:is>
       </x:c>
-      <x:c r="D60" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-088</x:t>
-        </x:is>
+      <x:c r="D60" s="55" t="str">
+        <x:v>TC-088、TC-097</x:v>
       </x:c>
       <x:c r="E60" s="55" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">src/main/usage-sync.ts、server-connection.ts；src/renderer/overview.tsx、settings.tsx；离线测试</x:t>
         </x:is>
       </x:c>
-      <x:c r="F60" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">服务状态自动子范围已实现；重绑误报已修，真实远端/发布待验</x:t>
-        </x:is>
+      <x:c r="F60" s="55" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨实现并通过独立 TC、源码门槛与打包应用回归。</x:v>
       </x:c>
       <x:c r="G60" s="69" t="inlineStr">
         <x:is>
@@ -9078,20 +9174,16 @@
           <x:t xml:space="preserve">REQ-047</x:t>
         </x:is>
       </x:c>
-      <x:c r="D61" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-089、TC-090、TC-091</x:t>
-        </x:is>
+      <x:c r="D61" s="58" t="str">
+        <x:v>TC-089、TC-090、TC-091、TC-098</x:v>
       </x:c>
       <x:c r="E61" s="58" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">src/renderer/、style.css；Electron 键盘/布局测试；目标 Mac VoiceOver 人工证据</x:t>
         </x:is>
       </x:c>
-      <x:c r="F61" s="58" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">键盘/精确值/文案自动子范围已实现；人工 VoiceOver 与发布验收待验</x:t>
-        </x:is>
+      <x:c r="F61" s="58" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨实现并通过独立 TC、源码门槛与打包应用回归。</x:v>
       </x:c>
       <x:c r="G61" s="68" t="inlineStr">
         <x:is>
@@ -9179,20 +9271,16 @@
           <x:t xml:space="preserve">REQ-049</x:t>
         </x:is>
       </x:c>
-      <x:c r="D63" s="61" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-096</x:t>
-        </x:is>
+      <x:c r="D63" s="61" t="str">
+        <x:v>TC-096、TC-100</x:v>
       </x:c>
       <x:c r="E63" s="61" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">src/collectors/scanner.ts、src/main/index.ts、src/renderer/index.ts；tests/；docs/design.md</x:t>
         </x:is>
       </x:c>
-      <x:c r="F63" s="61" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">已实现；TC-096 本机与隔离测试通过</x:t>
-        </x:is>
+      <x:c r="F63" s="61" t="str">
+        <x:v>既有能力保留原证据；2026-10-05 0.3.11 页面打磨实现并通过独立 TC、源码门槛与打包应用回归。</x:v>
       </x:c>
       <x:c r="G63" s="61" t="inlineStr">
         <x:is>
@@ -16123,6 +16211,211 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="102" ht="220" customHeight="1">
+      <x:c r="A102" s="100" t="str">
+        <x:v>TC-097</x:v>
+      </x:c>
+      <x:c r="B102" s="100" t="str">
+        <x:v>REQ-046</x:v>
+      </x:c>
+      <x:c r="C102" s="100" t="str">
+        <x:v>DEV-055</x:v>
+      </x:c>
+      <x:c r="D102" s="100" t="str">
+        <x:v>页头一行状态与详细诊断</x:v>
+      </x:c>
+      <x:c r="E102" s="100" t="str">
+        <x:v>Electron</x:v>
+      </x:c>
+      <x:c r="F102" s="100" t="str">
+        <x:v>构造本机正常但覆盖未知、扫描错误、服务待传及当前修订版确认四种隔离状态；查看页头并点击详情。</x:v>
+      </x:c>
+      <x:c r="G102" s="100" t="str">
+        <x:v>页头一行分别表述采集、覆盖和同步；未知不写零或完整，待传不写已同步；点击后可见服务修订、扫描与诊断入口。</x:v>
+      </x:c>
+      <x:c r="H102" s="100" t="str">
+        <x:v>通过（0.3.11 当前 Mac 自动验收）</x:v>
+      </x:c>
+      <x:c r="I102" s="100" t="str">
+        <x:v>2026-10-05 0.3.11 当前 Mac x86_64：独立 npm run test:case 退出码 0；npm run test:gate 104/104 单元、52/52 Electron；目录包内 npm run test:e2e:packaged 52/52；DMG SHA-256 00f2d863aed06bbfe9d67edc69ac056328ae3397b7226cecf6146cfa665852e0，hdiutil verify VALID；/Applications/Token.app 已安装启动，app.asar SHA-256 35e0d26ffa5a331fbe98b973b4b454b4d51473b3348ce4852e2215dc65ee27bc，已安装可执行文件本组五场景 5/5。合成样本与隔离 userData，未触碰真实会话正文。 独立命令：npm run test:case -- TC-097。</x:v>
+      </x:c>
+      <x:c r="J102" s="100" t="str">
+        <x:v>npm run test:case -- TC-097</x:v>
+      </x:c>
+      <x:c r="K102" s="100" t="str">
+        <x:v>tests/e2e/page-refinements.spec.ts 的 TC-097 独立场景；受影响旧用例 TC-079/082/088/090/096 按编号通过。</x:v>
+      </x:c>
+      <x:c r="L102" s="100" t="str">
+        <x:v>只使用隔离用户数据、临时数据库和无正文合成来源；不读取生产会话正文。</x:v>
+      </x:c>
+      <x:c r="M102" s="100" t="str">
+        <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="220" customHeight="1">
+      <x:c r="A103" s="100" t="str">
+        <x:v>TC-098</x:v>
+      </x:c>
+      <x:c r="B103" s="100" t="str">
+        <x:v>REQ-047</x:v>
+      </x:c>
+      <x:c r="C103" s="100" t="str">
+        <x:v>DEV-056</x:v>
+      </x:c>
+      <x:c r="D103" s="100" t="str">
+        <x:v>KPI 输入输出完整显示与精确原值</x:v>
+      </x:c>
+      <x:c r="E103" s="100" t="str">
+        <x:v>Electron</x:v>
+      </x:c>
+      <x:c r="F103" s="100" t="str">
+        <x:v>在标准和窄窗口造大输入/输出 Token、已确认零及覆盖未知；查看概览和报表并仅用键盘操作数字菜单。</x:v>
+      </x:c>
+      <x:c r="G103" s="100" t="str">
+        <x:v>输入输出均完整可见、无省略号；悬停和聚焦可读取并复制原始整数；覆盖未知与可证零不同。</x:v>
+      </x:c>
+      <x:c r="H103" s="100" t="str">
+        <x:v>通过（0.3.11 当前 Mac 自动验收）</x:v>
+      </x:c>
+      <x:c r="I103" s="100" t="str">
+        <x:v>2026-10-05 0.3.11 当前 Mac x86_64：独立 npm run test:case 退出码 0；npm run test:gate 104/104 单元、52/52 Electron；目录包内 npm run test:e2e:packaged 52/52；DMG SHA-256 00f2d863aed06bbfe9d67edc69ac056328ae3397b7226cecf6146cfa665852e0，hdiutil verify VALID；/Applications/Token.app 已安装启动，app.asar SHA-256 35e0d26ffa5a331fbe98b973b4b454b4d51473b3348ce4852e2215dc65ee27bc，已安装可执行文件本组五场景 5/5。合成样本与隔离 userData，未触碰真实会话正文。 独立命令：npm run test:case -- TC-098。</x:v>
+      </x:c>
+      <x:c r="J103" s="100" t="str">
+        <x:v>npm run test:case -- TC-098</x:v>
+      </x:c>
+      <x:c r="K103" s="100" t="str">
+        <x:v>tests/e2e/page-refinements.spec.ts 的 TC-098 独立场景；受影响旧用例 TC-079/082/088/090/096 按编号通过。</x:v>
+      </x:c>
+      <x:c r="L103" s="100" t="str">
+        <x:v>只使用隔离用户数据、临时数据库和无正文合成来源；不读取生产会话正文。</x:v>
+      </x:c>
+      <x:c r="M103" s="100" t="str">
+        <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="220" customHeight="1">
+      <x:c r="A104" s="100" t="str">
+        <x:v>TC-099</x:v>
+      </x:c>
+      <x:c r="B104" s="100" t="str">
+        <x:v>REQ-041</x:v>
+      </x:c>
+      <x:c r="C104" s="100" t="str">
+        <x:v>DEV-050</x:v>
+      </x:c>
+      <x:c r="D104" s="100" t="str">
+        <x:v>报表筛选摘要与当前快照一致</x:v>
+      </x:c>
+      <x:c r="E104" s="100" t="str">
+        <x:v>Electron</x:v>
+      </x:c>
+      <x:c r="F104" s="100" t="str">
+        <x:v>快速修改日期、工具、模型、项目、用户和时区，核筛选摘要与屏显/CSV 同一授权快照；含加载和冲突状态。</x:v>
+      </x:c>
+      <x:c r="G104" s="100" t="str">
+        <x:v>筛选摘要完整、可读且只反映当前查询；加载时不展示旧结果或允许旧快照导出；待核对与未知状态保留。</x:v>
+      </x:c>
+      <x:c r="H104" s="100" t="str">
+        <x:v>通过（0.3.11 当前 Mac 自动验收）</x:v>
+      </x:c>
+      <x:c r="I104" s="100" t="str">
+        <x:v>2026-10-05 0.3.11 当前 Mac x86_64：独立 npm run test:case 退出码 0；npm run test:gate 104/104 单元、52/52 Electron；目录包内 npm run test:e2e:packaged 52/52；DMG SHA-256 00f2d863aed06bbfe9d67edc69ac056328ae3397b7226cecf6146cfa665852e0，hdiutil verify VALID；/Applications/Token.app 已安装启动，app.asar SHA-256 35e0d26ffa5a331fbe98b973b4b454b4d51473b3348ce4852e2215dc65ee27bc，已安装可执行文件本组五场景 5/5。合成样本与隔离 userData，未触碰真实会话正文。 独立命令：npm run test:case -- TC-099。</x:v>
+      </x:c>
+      <x:c r="J104" s="100" t="str">
+        <x:v>npm run test:case -- TC-099</x:v>
+      </x:c>
+      <x:c r="K104" s="100" t="str">
+        <x:v>tests/e2e/page-refinements.spec.ts 的 TC-099 独立场景；受影响旧用例 TC-079/082/088/090/096 按编号通过。</x:v>
+      </x:c>
+      <x:c r="L104" s="100" t="str">
+        <x:v>只使用隔离用户数据、临时数据库和无正文合成来源；不读取生产会话正文。</x:v>
+      </x:c>
+      <x:c r="M104" s="100" t="str">
+        <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="220" customHeight="1">
+      <x:c r="A105" s="100" t="str">
+        <x:v>TC-100</x:v>
+      </x:c>
+      <x:c r="B105" s="100" t="str">
+        <x:v>REQ-049</x:v>
+      </x:c>
+      <x:c r="C105" s="100" t="str">
+        <x:v>DEV-058</x:v>
+      </x:c>
+      <x:c r="D105" s="100" t="str">
+        <x:v>单用户来源汇总与异常优先列表</x:v>
+      </x:c>
+      <x:c r="E105" s="100" t="str">
+        <x:v>Electron</x:v>
+      </x:c>
+      <x:c r="F105" s="100" t="str">
+        <x:v>隔离单用户创建已归属 Codex/Claude 文件、未归属、旧身份未知与多用户对照；展开正常来源并操作预览归属。</x:v>
+      </x:c>
+      <x:c r="G105" s="100" t="str">
+        <x:v>按工具显示已归属数；默认仅展开异常，正常文件无逐行下拉框；手动展开后仍可审查/更改，未知不被折叠为正常；多用户原授权流程保持。</x:v>
+      </x:c>
+      <x:c r="H105" s="100" t="str">
+        <x:v>通过（0.3.11 当前 Mac 自动验收）</x:v>
+      </x:c>
+      <x:c r="I105" s="100" t="str">
+        <x:v>2026-10-05 0.3.11 当前 Mac x86_64：独立 npm run test:case 退出码 0；npm run test:gate 104/104 单元、52/52 Electron；目录包内 npm run test:e2e:packaged 52/52；DMG SHA-256 00f2d863aed06bbfe9d67edc69ac056328ae3397b7226cecf6146cfa665852e0，hdiutil verify VALID；/Applications/Token.app 已安装启动，app.asar SHA-256 35e0d26ffa5a331fbe98b973b4b454b4d51473b3348ce4852e2215dc65ee27bc，已安装可执行文件本组五场景 5/5。合成样本与隔离 userData，未触碰真实会话正文。 独立命令：npm run test:case -- TC-100。</x:v>
+      </x:c>
+      <x:c r="J105" s="100" t="str">
+        <x:v>npm run test:case -- TC-100</x:v>
+      </x:c>
+      <x:c r="K105" s="100" t="str">
+        <x:v>tests/e2e/page-refinements.spec.ts 的 TC-100 独立场景；受影响旧用例 TC-079/082/088/090/096 按编号通过。</x:v>
+      </x:c>
+      <x:c r="L105" s="100" t="str">
+        <x:v>只使用隔离用户数据、临时数据库和无正文合成来源；不读取生产会话正文。</x:v>
+      </x:c>
+      <x:c r="M105" s="100" t="str">
+        <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="220" customHeight="1">
+      <x:c r="A106" s="100" t="str">
+        <x:v>TC-101</x:v>
+      </x:c>
+      <x:c r="B106" s="100" t="str">
+        <x:v>REQ-043</x:v>
+      </x:c>
+      <x:c r="C106" s="100" t="str">
+        <x:v>DEV-052</x:v>
+      </x:c>
+      <x:c r="D106" s="100" t="str">
+        <x:v>首次引导下一步与操作后即时进度</x:v>
+      </x:c>
+      <x:c r="E106" s="100" t="str">
+        <x:v>Electron</x:v>
+      </x:c>
+      <x:c r="F106" s="100" t="str">
+        <x:v>首次建账后依次执行来源扫描与归属，返回引导查看焦点动作和进度；分别跳过、完成、重启。</x:v>
+      </x:c>
+      <x:c r="G106" s="100" t="str">
+        <x:v>任一时刻突出一个待办动作；操作后立即反映真实状态，完成可结束、随时可跳过；侧栏无常驻入口，权限和未知状态不变。</x:v>
+      </x:c>
+      <x:c r="H106" s="100" t="str">
+        <x:v>通过（0.3.11 当前 Mac 自动验收）</x:v>
+      </x:c>
+      <x:c r="I106" s="100" t="str">
+        <x:v>2026-10-05 0.3.11 当前 Mac x86_64：独立 npm run test:case 退出码 0；npm run test:gate 104/104 单元、52/52 Electron；目录包内 npm run test:e2e:packaged 52/52；DMG SHA-256 00f2d863aed06bbfe9d67edc69ac056328ae3397b7226cecf6146cfa665852e0，hdiutil verify VALID；/Applications/Token.app 已安装启动，app.asar SHA-256 35e0d26ffa5a331fbe98b973b4b454b4d51473b3348ce4852e2215dc65ee27bc，已安装可执行文件本组五场景 5/5。合成样本与隔离 userData，未触碰真实会话正文。 独立命令：npm run test:case -- TC-101。</x:v>
+      </x:c>
+      <x:c r="J106" s="100" t="str">
+        <x:v>npm run test:case -- TC-101</x:v>
+      </x:c>
+      <x:c r="K106" s="100" t="str">
+        <x:v>tests/e2e/page-refinements.spec.ts 的 TC-101 独立场景；受影响旧用例 TC-079/082/088/090/096 按编号通过。</x:v>
+      </x:c>
+      <x:c r="L106" s="100" t="str">
+        <x:v>只使用隔离用户数据、临时数据库和无正文合成来源；不读取生产会话正文。</x:v>
+      </x:c>
+      <x:c r="M106" s="100" t="str">
+        <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: plan 0.3.11 page performance traceability
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re92b59e81cdf4f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re6f3cbe9dc8b4417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R2676777626584123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R93db8671ef0b423b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R7caa8f15ac6f4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rbc26dd53433747fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd8d65c841016461c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3988c36403e64268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Reb222aff2cf840f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R70ecbaac2ebc49c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,7 +74,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="40">
+  <x:fills count="41">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -271,6 +271,11 @@
         <x:fgColor rgb="FFF2F6FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4FA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -301,7 +306,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="101">
+  <x:cellXfs count="104">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -561,6 +566,15 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -859,14 +873,13 @@
       <x:c r="G2" s="2" t="n"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
+      <x:c r="A3" s="4" t="str">
+        <x:v>代码 1e70412：48 条需求、57 项任务、94 条用例；94 个编号均已注册，状态按证据判定。
 当前 508851a：94 个注册编号；97/97 单元、43/43 Electron 源码门禁通过；打包全量一次 42/43，单项重跑通过，详见 docs/validation.md。
 2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。
 版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。
-2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。</x:t>
-        </x:is>
+2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。
+2026-10-06 新增 REQ-050→DEV-059→TC-102–104；当前 50 REQ、59 DEV、104 TC；新增三项待注册/待验证。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -4698,6 +4711,75 @@
       </x:c>
       <x:c r="G107" s="100" t="str">
         <x:v>2026-10-05 TC-101 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="86.25" customHeight="1">
+      <x:c r="A108" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="B108" s="103" t="str">
+        <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
+      </x:c>
+      <x:c r="C108" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D108" s="103" t="str">
+        <x:v>测量并修复页面导航与长列表瓶颈</x:v>
+      </x:c>
+      <x:c r="E108" s="103" t="str">
+        <x:v>TC-102</x:v>
+      </x:c>
+      <x:c r="F108" s="103" t="str">
+        <x:v>导航反馈与内容可交互时延</x:v>
+      </x:c>
+      <x:c r="G108" s="103" t="str">
+        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="86.25" customHeight="1">
+      <x:c r="A109" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="B109" s="103" t="str">
+        <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
+      </x:c>
+      <x:c r="C109" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D109" s="103" t="str">
+        <x:v>测量并修复页面导航与长列表瓶颈</x:v>
+      </x:c>
+      <x:c r="E109" s="103" t="str">
+        <x:v>TC-103</x:v>
+      </x:c>
+      <x:c r="F109" s="103" t="str">
+        <x:v>长报表连续滚动帧间隔</x:v>
+      </x:c>
+      <x:c r="G109" s="103" t="str">
+        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="86.25" customHeight="1">
+      <x:c r="A110" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="B110" s="103" t="str">
+        <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
+      </x:c>
+      <x:c r="C110" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D110" s="103" t="str">
+        <x:v>测量并修复页面导航与长列表瓶颈</x:v>
+      </x:c>
+      <x:c r="E110" s="103" t="str">
+        <x:v>TC-104</x:v>
+      </x:c>
+      <x:c r="F110" s="103" t="str">
+        <x:v>慢响应、切用户与报表快照回归</x:v>
+      </x:c>
+      <x:c r="G110" s="103" t="str">
+        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4737,10 +4819,8 @@
       <x:c r="H2" s="2" t="n"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">REQ-001–048 共 48 条；状态与 DEV/TC 关联见本页。</x:t>
-        </x:is>
+      <x:c r="A3" s="4" t="str">
+        <x:v>REQ-001–050 共 50 条；REQ-050 为 0.3.11 页面性能增量计划，状态与 DEV/TC 关联见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -6970,6 +7050,32 @@
         <x:is>
           <x:t xml:space="preserve">2026-10-04 用户明确单人客户端规则及数据来源页截图；本机只使用一个登录账户。</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="157.5" customHeight="1">
+      <x:c r="A55" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="B55" s="103" t="str">
+        <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
+      </x:c>
+      <x:c r="C55" s="103" t="str">
+        <x:v>在当前 Mac 0.3.11 同环境、独立 userData、无正文合成空库与约 35,000 条事实下，标准及 700px 窗口的概览↔报表、数据来源、管理中心冷/热切换各至少 20 次；点击到选中态或骨架屏反馈 P95 ≤150ms，并记录点击到内容可交互的 P50/P95。长报表连续滚动 10 秒，帧间隔 P95 ≤32ms、无 ≥200ms 卡顿。先测基线；若已达标，先复现用户可感知延迟触发条件再修。慢查询时仍能切页并见加载反馈；旧响应不覆盖新页面，不泄露上一用户数据；筛选/焦点、报表 CSV 同一快照、权限、未知≠零、错误重试保持正确。</x:v>
+      </x:c>
+      <x:c r="D55" s="103" t="str">
+        <x:v>0.3.11 页面性能增量（计划）</x:v>
+      </x:c>
+      <x:c r="E55" s="103" t="str">
+        <x:v>待实现/待验证</x:v>
+      </x:c>
+      <x:c r="F55" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="G55" s="103" t="str">
+        <x:v>TC-102、TC-103、TC-104</x:v>
+      </x:c>
+      <x:c r="H55" s="103" t="str">
+        <x:v>承接 REQ-041/043/046/047/049 现有页面和权限语义。2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。 详见 docs/design.md §22、docs/development-plan.md §14、docs/test-case-acceptance.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7007,10 +7113,8 @@
       <x:c r="G2" s="2" t="n"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-001–057 共 57 项；状态与 REQ/TC 关联见本页。</x:t>
-        </x:is>
+      <x:c r="A3" s="4" t="str">
+        <x:v>DEV-001–059 共 59 项；DEV-059 为 0.3.11 页面性能增量计划，状态与 REQ/TC 关联见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9286,6 +9390,29 @@
         <x:is>
           <x:t xml:space="preserve">2026-10-04 0.3.9：源码门禁 96 入口、104/104 单元、47/47 Electron；目录包 47/47。唯一账户下，安装后 14 个可确认 Claude 文件来源由未归属变为本机默认归属，14 条脱敏审计；手动解除、多用户和未知来源隔离通过。</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="150" customHeight="1">
+      <x:c r="A64" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="B64" s="103" t="str">
+        <x:v>测量并修复页面导航与长列表瓶颈</x:v>
+      </x:c>
+      <x:c r="C64" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="D64" s="103" t="str">
+        <x:v>TC-102、TC-103、TC-104</x:v>
+      </x:c>
+      <x:c r="E64" s="103" t="str">
+        <x:v>src/renderer/index.tsx、overview.tsx、report.tsx、style.css；若基线证明必要再改主进程查询/IPC；独立性能与正确性用例</x:v>
+      </x:c>
+      <x:c r="F64" s="103" t="str">
+        <x:v>待开发；新增 TC-102–104 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="G64" s="103" t="str">
+        <x:v>在固定候选与合成空库/35,000 事实建立冷/热切换和长列表滚动基线，记录环境、样本量及 P50/P95；定位主线程渲染、查询、IPC 或列表瓶颈后做最小修复并复测。若基线已达标，先找到可复现延迟。保留旧请求代次、授权快照/CSV、权限和未知状态。2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9331,10 +9458,8 @@
       <x:c r="I2" s="2" t="n"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-001–095 共 95 个编号；TC-001–094 已注册，TC-095 为待注册本机人工用例。人工与发布验收按各行证据判定。</x:t>
-        </x:is>
+      <x:c r="A3" s="4" t="str">
+        <x:v>TC-001–104 共 104 个编号；TC-102–104 为 0.3.11 性能增量计划，待注册/待验证；旧用例状态逐行以证据为准。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -16414,6 +16539,129 @@
       </x:c>
       <x:c r="M106" s="100" t="str">
         <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="176.25" customHeight="1">
+      <x:c r="A107" s="103" t="str">
+        <x:v>TC-102</x:v>
+      </x:c>
+      <x:c r="B107" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="C107" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D107" s="103" t="str">
+        <x:v>导航反馈与内容可交互时延</x:v>
+      </x:c>
+      <x:c r="E107" s="103" t="str">
+        <x:v>当前 Mac Electron/性能</x:v>
+      </x:c>
+      <x:c r="F107" s="103" t="str">
+        <x:v>同一 0.3.11 固定候选、独立 userData；空库和约 35,000 无正文合成事实；标准与 700px 窗口，概览↔报表、数据来源、管理中心冷/热各 20 次；记录点击→选中态/骨架屏和点击→内容可交互的逐次原始时长、P50/P95、环境与数据版本；加入可控慢 IPC。</x:v>
+      </x:c>
+      <x:c r="G107" s="103" t="str">
+        <x:v>每个场景反馈 P95 ≤150ms；内容可交互 P50/P95 均记录并和基线比较。慢 IPC 时切页与加载可用，不等同步查询完成。</x:v>
+      </x:c>
+      <x:c r="H107" s="103" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I107" s="103" t="str">
+        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+      </x:c>
+      <x:c r="J107" s="103" t="str">
+        <x:v>npm run test:case -- TC-102（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K107" s="103" t="str">
+        <x:v>拟新增 TC-102 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L107" s="103" t="str">
+        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+      </x:c>
+      <x:c r="M107" s="103" t="str">
+        <x:v>导航性能基线与复测均需固定提交和同机条件；若初测达标，应另复现用户观察到的可感延迟再定义修复。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="176.25" customHeight="1">
+      <x:c r="A108" s="103" t="str">
+        <x:v>TC-103</x:v>
+      </x:c>
+      <x:c r="B108" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="C108" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D108" s="103" t="str">
+        <x:v>长报表连续滚动帧间隔</x:v>
+      </x:c>
+      <x:c r="E108" s="103" t="str">
+        <x:v>当前 Mac Electron/性能</x:v>
+      </x:c>
+      <x:c r="F108" s="103" t="str">
+        <x:v>约 35,000 无正文合成事实填充长报表，标准与 700px 窗口；每种窗口连续滚动 10 秒，采集 requestAnimationFrame 帧时间戳和交互状态；保留逐帧数据及固定候选/环境。空库只验页面稳定，不作为长列表性能样本。</x:v>
+      </x:c>
+      <x:c r="G108" s="103" t="str">
+        <x:v>两种窗口帧间隔 P95 ≤32ms，且任何帧间隔不达到 200ms；滚动后筛选、焦点和可见明细仍正确。</x:v>
+      </x:c>
+      <x:c r="H108" s="103" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I108" s="103" t="str">
+        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+      </x:c>
+      <x:c r="J108" s="103" t="str">
+        <x:v>npm run test:case -- TC-103（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K108" s="103" t="str">
+        <x:v>拟新增 TC-103 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L108" s="103" t="str">
+        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+      </x:c>
+      <x:c r="M108" s="103" t="str">
+        <x:v>按逐帧间隔计算 P95；不将 FPS 均值当作 P95，也不删去长尾卡顿。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="176.25" customHeight="1">
+      <x:c r="A109" s="103" t="str">
+        <x:v>TC-104</x:v>
+      </x:c>
+      <x:c r="B109" s="103" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="C109" s="103" t="str">
+        <x:v>DEV-059</x:v>
+      </x:c>
+      <x:c r="D109" s="103" t="str">
+        <x:v>慢响应、切用户与报表快照回归</x:v>
+      </x:c>
+      <x:c r="E109" s="103" t="str">
+        <x:v>Electron/集成</x:v>
+      </x:c>
+      <x:c r="F109" s="103" t="str">
+        <x:v>双用户授权隔离与不同数据；延迟旧页面查询后切页、切用户并触发新查询；再覆盖筛选快速切换、返回焦点、报表 CSV 导出、权限直调、未知覆盖及失败重试。全部使用独立临时库和无正文合成事实。</x:v>
+      </x:c>
+      <x:c r="G109" s="103" t="str">
+        <x:v>旧响应不能覆盖新页面或新用户；加载和错误状态可操作；筛选与焦点保持；CSV 和当前授权报表为同一快照；跨用户数据/IPC 均不泄露，未知不显示为零，失败可重试。</x:v>
+      </x:c>
+      <x:c r="H109" s="103" t="str">
+        <x:v>待注册、待验证（规划目标）</x:v>
+      </x:c>
+      <x:c r="I109" s="103" t="str">
+        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+      </x:c>
+      <x:c r="J109" s="103" t="str">
+        <x:v>npm run test:case -- TC-104（计划；当前不可运行）</x:v>
+      </x:c>
+      <x:c r="K109" s="103" t="str">
+        <x:v>拟新增 TC-104 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+      </x:c>
+      <x:c r="L109" s="103" t="str">
+        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+      </x:c>
+      <x:c r="M109" s="103" t="str">
+        <x:v>回归 REQ-041/TC-079、REQ-047/TC-089–090、REQ-048/TC-093、REQ-040/TC-077 的现有边界；新增用例自身独立。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17237,6 +17485,41 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="18" ht="168.75" customHeight="1">
+      <x:c r="A18" s="103" t="str">
+        <x:v>VER-013</x:v>
+      </x:c>
+      <x:c r="B18" s="103" t="str">
+        <x:v>0.3.11（当前 Mac 页面修订；性能增量计划）</x:v>
+      </x:c>
+      <x:c r="C18" s="103" t="str">
+        <x:v>页面概览、来源、报表和引导整理；切换与滚动性能</x:v>
+      </x:c>
+      <x:c r="D18" s="103" t="str">
+        <x:v>现有 0.3.11 页面修订：页头状态、精确数值、报表筛选摘要、单用户来源列表、首次引导。新增性能增量：页面切换反馈、长报表滚动与慢响应下的正确性。</x:v>
+      </x:c>
+      <x:c r="E18" s="103" t="str">
+        <x:v>REQ-046/047/041/049/043；新增 REQ-050</x:v>
+      </x:c>
+      <x:c r="F18" s="103" t="str">
+        <x:v>DEV-055/056/050/058/052；新增 DEV-059</x:v>
+      </x:c>
+      <x:c r="G18" s="103" t="str">
+        <x:v>TC-097–101 已有隔离自动证据；新增 TC-102–104 待注册/待验证</x:v>
+      </x:c>
+      <x:c r="H18" s="103" t="str">
+        <x:v>页面修订在 5902568 分支有既有当前 Mac 隔离自动证据；性能增量本次只完成需求、设计和测试规划，尚未实现或测量基线。</x:v>
+      </x:c>
+      <x:c r="I18" s="103" t="str">
+        <x:v>0.3.11 页面修订的已有子范围按原证据；性能增量未完成。完整版本完成状态待 TC-102–104、受影响回归和固定候选复验后评估。</x:v>
+      </x:c>
+      <x:c r="J18" s="103" t="str">
+        <x:v>2026-10-06；性能基线与修复提交、Mac 环境、原始测量/P50/P95、包与安装证据待补。</x:v>
+      </x:c>
+      <x:c r="K18" s="103" t="str">
+        <x:v>不将 TC-097–101 的通过外推到新性能门槛；未知/未覆盖不当零，权限、查询快照和真实私人数据边界保持。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>

</xml_diff>

<commit_message>
docs: record navigation performance subrange evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rbc26dd53433747fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd8d65c841016461c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R3988c36403e64268"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Reb222aff2cf840f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R70ecbaac2ebc49c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re2934719e0774049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbffc73df048d41ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb4bc964e3d3848ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R483560964650425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R00f0b31ea9404285"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -879,7 +879,8 @@
 2026-10-04 新增“版本规划”页，跟踪 0.2.0–0.3.6 与未定下一轮的主要功能、关联编号、进度和完成状态；不替代逐项 REQ/DEV/TC。
 版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。
 2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。
-2026-10-06 新增 REQ-050→DEV-059→TC-102–104；当前 50 REQ、59 DEV、104 TC；新增三项待注册/待验证。</x:v>
+2026-10-06 新增 REQ-050→DEV-059→TC-102–104；当前 50 REQ、59 DEV、104 TC；新增三项待注册/待验证。
+2026-10-06 / 46111d3 已注册 104 个 TC；TC-102–104 现有自动子范围通过，完整合同待补证。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -3789,9 +3790,8 @@
           <x:t xml:space="preserve">实际打包 App 隔离自动升级</x:t>
         </x:is>
       </x:c>
-      <x:c r="G82" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
+      <x:c r="G82" s="52" t="str">
+        <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
 2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。
 2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。
 2026-10-04 安装中取消设计已决：独立控制窗口+helper 阶段回执、替换后回滚和 userData 隔离健康探测，TC-076 分阶段打包 UI 真取消待实现/验收；既有成功/故障证据不变。
@@ -3799,8 +3799,8 @@
 508851a：历史真实 DMG/打包 helper 故障证据保留；本次合成旧版本成功链通过，真实两包故障子段跳过；详情见测试用例 I/L/M 列与 docs/validation.md。
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 新包隔离升级及两层五故障回退动态子范围通过；完整系统/生产验收待补；历史取消设计保留备选。
 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2 TC-076 真实双 DMG 脚本 exit 0；范围与限制见测试用例 I/M 列。
-2026-10-04 最新用户决议：点击开始前可放弃；点击后下载/校验/交接/安装全程无取消，直到成功或失败自动恢复。独立窗口、取消协议/journal、分阶段点击取消不属本轮；旧隔离成功/五故障证据保留，系统/生产/目标 Mac 仍待验。</x:t>
-        </x:is>
+2026-10-04 最新用户决议：点击开始前可放弃；点击后下载/校验/交接/安装全程无取消，直到成功或失败自动恢复。独立窗口、取消协议/journal、分阶段点击取消不属本轮；旧隔离成功/五故障证据保留，系统/生产/目标 Mac 仍待验。
+46111d3：TC-076 前两次首次引导脚本假设失败、修订后第三次合成旧版链路 exit 0；真实双 DMG 故障本轮未执行，整项仍部分验证。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -4713,7 +4713,7 @@
         <x:v>2026-10-05 TC-101 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="86.25" customHeight="1">
+    <x:row r="108" ht="116.25" customHeight="1">
       <x:c r="A108" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4733,10 +4733,10 @@
         <x:v>导航反馈与内容可交互时延</x:v>
       </x:c>
       <x:c r="G108" s="103" t="str">
-        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="86.25" customHeight="1">
+        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="116.25" customHeight="1">
       <x:c r="A109" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4756,10 +4756,10 @@
         <x:v>长报表连续滚动帧间隔</x:v>
       </x:c>
       <x:c r="G109" s="103" t="str">
-        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110" ht="86.25" customHeight="1">
+        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="116.25" customHeight="1">
       <x:c r="A110" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4779,7 +4779,7 @@
         <x:v>慢响应、切用户与报表快照回归</x:v>
       </x:c>
       <x:c r="G110" s="103" t="str">
-        <x:v>待注册、待验证（0.3.11 性能增量计划）</x:v>
+        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-104 仅快速切页与 viewer 菜单隔离；未显式注入慢 IPC，未验双用户实际数据、CSV 同快照、未知≠零和失败重试。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4820,7 +4820,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–050 共 50 条；REQ-050 为 0.3.11 页面性能增量计划，状态与 DEV/TC 关联见本页。</x:v>
+        <x:v>REQ-001–050 共 50 条；REQ-050 已有 0.3.11 代码与自动子范围证据，完整需求待补证。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -7052,7 +7052,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="55" ht="157.5" customHeight="1">
+    <x:row r="55" ht="195" customHeight="1">
       <x:c r="A55" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -7063,10 +7063,10 @@
         <x:v>在当前 Mac 0.3.11 同环境、独立 userData、无正文合成空库与约 35,000 条事实下，标准及 700px 窗口的概览↔报表、数据来源、管理中心冷/热切换各至少 20 次；点击到选中态或骨架屏反馈 P95 ≤150ms，并记录点击到内容可交互的 P50/P95。长报表连续滚动 10 秒，帧间隔 P95 ≤32ms、无 ≥200ms 卡顿。先测基线；若已达标，先复现用户可感知延迟触发条件再修。慢查询时仍能切页并见加载反馈；旧响应不覆盖新页面，不泄露上一用户数据；筛选/焦点、报表 CSV 同一快照、权限、未知≠零、错误重试保持正确。</x:v>
       </x:c>
       <x:c r="D55" s="103" t="str">
-        <x:v>0.3.11 页面性能增量（计划）</x:v>
+        <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
       <x:c r="E55" s="103" t="str">
-        <x:v>待实现/待验证</x:v>
+        <x:v>代码已实现，自动子范围通过；完整需求待补证</x:v>
       </x:c>
       <x:c r="F55" s="103" t="str">
         <x:v>DEV-059</x:v>
@@ -7075,7 +7075,7 @@
         <x:v>TC-102、TC-103、TC-104</x:v>
       </x:c>
       <x:c r="H55" s="103" t="str">
-        <x:v>承接 REQ-041/043/046/047/049 现有页面和权限语义。2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。 详见 docs/design.md §22、docs/development-plan.md §14、docs/test-case-acceptance.md。</x:v>
+        <x:v>2026-10-06 / 46111d3：导航先反馈、旧响应按页面代次和账号丢弃；TC-102–104 已注册且现有自动子范围通过。35,000 条事实 700px 来源/管理反馈 P95 546.2→12.7ms、965.5→12.4ms；滚动 P95 18.6ms。冷/热原始样本与 TC-104 完整正确性待补；见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7114,7 +7114,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>DEV-001–059 共 59 项；DEV-059 为 0.3.11 页面性能增量计划，状态与 REQ/TC 关联见本页。</x:v>
+        <x:v>DEV-001–059 共 59 项；DEV-059 代码已提交、自动子范围通过，完整验收待补证。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9392,7 +9392,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="64" ht="150" customHeight="1">
+    <x:row r="64" ht="172.5" customHeight="1">
       <x:c r="A64" s="103" t="str">
         <x:v>DEV-059</x:v>
       </x:c>
@@ -9406,13 +9406,13 @@
         <x:v>TC-102、TC-103、TC-104</x:v>
       </x:c>
       <x:c r="E64" s="103" t="str">
-        <x:v>src/renderer/index.tsx、overview.tsx、report.tsx、style.css；若基线证明必要再改主进程查询/IPC；独立性能与正确性用例</x:v>
+        <x:v>src/renderer/index.tsx、overview.tsx、report.tsx；scripts/measure-navigation.mjs、scripts/test-cases.mjs；tests/e2e/navigation-performance.spec.ts；TC-076 升级脚本兼容回归</x:v>
       </x:c>
       <x:c r="F64" s="103" t="str">
-        <x:v>待开发；新增 TC-102–104 待注册/待验证</x:v>
+        <x:v>代码已提交；现有自动子范围通过；完整验收待补证</x:v>
       </x:c>
       <x:c r="G64" s="103" t="str">
-        <x:v>在固定候选与合成空库/35,000 事实建立冷/热切换和长列表滚动基线，记录环境、样本量及 P50/P95；定位主线程渲染、查询、IPC 或列表瓶颈后做最小修复并复测。若基线已达标，先找到可复现延迟。保留旧请求代次、授权快照/CSV、权限和未知状态。2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+        <x:v>46111d3 已提交导航先反馈、加载/重试、旧响应隔离及无变化轮询。文档会话独立核 104 入口、TC-102–104 各 1/1、104/104 单元与 55/55 Electron；性能摘要达阈值。冷/热原始样本与 TC-104 完整场景待补；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9459,7 +9459,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–104 共 104 个编号；TC-102–104 为 0.3.11 性能增量计划，待注册/待验证；旧用例状态逐行以证据为准。</x:v>
+        <x:v>TC-001–104 共 104 个编号，全部已注册；TC-102–104 现有自动子范围通过、完整验收待补证。人工与发布验收按逐行证据判定。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -11975,13 +11975,12 @@
           <x:t xml:space="preserve">0.3.6 合成控制/回滚单元 2/2 独立通过，含路径别名；真实 DMG 的模块故障子范围由 TC-076 另验，打包 helper/UI 回滚仍待验</x:t>
         </x:is>
       </x:c>
-      <x:c r="I41" s="69" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">当前 1e70412：文档会话独立执行 npm run test:case -- TC-036，2/2、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
+      <x:c r="I41" s="69" t="str">
+        <x:v>当前 1e70412：文档会话独立执行 npm run test:case -- TC-036，2/2、退出码 0；完整门禁 94 入口/77 单元/38 Electron 通过。
 历史：96e99be 自动日志；2026-10-02 44a96e8 本机升级通过；2026-10-03 b224dde 单元 1/1、取消替换复验。新增：867a03a 可复用脚本，开发会话复跑 0.2.0→0.3.0 及普通 0.3.0→0.3.1 隔离升级；开发工作树 test-results/manual/evidence/TC-036-reusable.log（Git 忽略），摘要见 docs/validation.md。；2026-10-03 旧结果仅作历史，当前函数仍为“只打开安装包”断言；新辅助进程/回滚断言尚未实现或运行。
 86a4b5b：文档会话单编号 TC-036 两项 2/2 退出码 0：下载校验后交自动安装器及启动失败不退出旧版；合成 Bundle/命令覆盖 /Applications/~/Applications 选择、成功、挂载/复制/替换/重启/健康超时及篡改失败回滚。真实旧二进制、只读 DMG 实测及系统权限未由单元证明。
-2026-10-04 / 80e7f10→0eac84b：文档工作树 macOS 15.7.4 x86_64、Node 24.15.0：npm run test:case -- TC-036，2/2、exit 0；门禁 94 入口/77 单元/38 Electron、打包版 38/38 均 exit 0。</x:t>
-        </x:is>
+2026-10-04 / 80e7f10→0eac84b：文档工作树 macOS 15.7.4 x86_64、Node 24.15.0：npm run test:case -- TC-036，2/2、exit 0；门禁 94 入口/77 单元/38 Electron、打包版 38/38 均 exit 0。
+2026-10-06 / 46111d3：文档会话独立 npm run test:case -- TC-036，两个已注册单元绑定各 1/1，exit 0；仅合成 installer 控制/回滚，不代表真实旧二进制或系统目录。</x:v>
       </x:c>
       <x:c r="J41" s="35" t="inlineStr">
         <x:is>
@@ -14702,16 +14701,15 @@
           <x:t xml:space="preserve">部分验证：当前新 DMG 隔离成功升级、installer/打包 helper 各五故障回退与重试通过；点击后全阶段无取消 UI、真实系统目录/生产数据与真实故障待验</x:t>
         </x:is>
       </x:c>
-      <x:c r="I81" s="68" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
+      <x:c r="I81" s="68" t="str">
+        <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
 2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
 86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。
 2026-10-04 / 80e7f10→0eac84b：80e7f10 文档独立首次全命令：成功段、只读初始启动、五故障回退输出通过；末次重试读取已被 UI 消费的一次性 last-install.json 得 undefined，exit 1。0eac84b 修脚本后同 DMG 再跑，全命令 exit 0；旧包 142557541 字节 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 142591838 字节 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c，两包 verify VALID。旧 27aae018… 只属历史候选。
 508851a：TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。
 2026-10-04 用户决议：开始执行应用替换/安装后不可取消，安装前可放弃，失败自动恢复；原五阶段取消要求撤出本轮。新候选从干净 main 9af351a 构建，未签名 mac x64 DMG SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；需求会话报告 pack:dmg exit 0，文档会话独立重算 SHA-256 与 hdiutil verify VALID。新包成功/故障隔离动态子范围后续已测，详见本列最新证据，旧 d99d7af9 包证据不外推。
-2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。</x:t>
-        </x:is>
+2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
+2026-10-06 / 46111d3：开发会话 TC-076 前两次因旧脚本假设首次建账直达概览失败；修订 verify-auto-upgrade.mjs / verify-auto-upgrade-faults.mjs 等待并可跳过引导，第三次 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076 exit 0。隔离合成旧版（当前包改版本元数据）旧进程退出、原位替换、新版启动、受信登录及合成 1280 Token 保留，无 Finder 拖拽。文档会话只读核脚本差异，未复跑 TC-076；前两次失败保留。</x:v>
       </x:c>
       <x:c r="J81" s="52" t="inlineStr">
         <x:is>
@@ -14737,16 +14735,15 @@
 2026-10-04 用户最新决议：取消交付义务的边界从“开始替换/安装”前移至点击“开始升级”；下载/校验/交接/安装均不可中断取消。上方“下载取消待核实/安装中取消待验”及阶段取消正例只属历史；本轮只验点击前放弃、正常完成与失败自动回退。</x:t>
         </x:is>
       </x:c>
-      <x:c r="M81" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
+      <x:c r="M81" s="52" t="str">
+        <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
 2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。
 1961de3；文档会话独立 TC-076 完整命令 exit 0，真实旧/新 DMG SHA-256 分别 ae1b8e80…、d99d7af9…，两包 hdiutil verify VALID；打包 helper mount/space/replace/launch/health 各回退、受信登录/1280 Token/清理及最后重试均通过；TC-036 两单元 exit 0。
 1961de3 文档会话独立 test:gate 类型检查、94 入口、77/77 单元、39/39 Electron exit 0；未另跑打包版全量。
 508851a；macOS 15.7.4 x86_64、Node v24.15.0；TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。
 后续新包 TC-076 隔离动态子范围已由需求会话执行通过，详见 I 列最新证据；整项仍部分验证。
-新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 exit 0，打包 Electron 43/43，test:gate 97/97 单元+43/43 Electron；均由需求会话报告，文档会话未独立复跑。</x:t>
-        </x:is>
+新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 exit 0，打包 Electron 43/43，test:gate 97/97 单元+43/43 Electron；均由需求会话报告，文档会话未独立复跑。
+2026-10-06 本轮第三次成功只覆盖合成旧版链路，未执行真实旧/新 DMG 故障子范围、系统安装目录或生产用户数据；历史真实 DMG 证据只归属原固定候选。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">
@@ -16541,7 +16538,7 @@
         <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="176.25" customHeight="1">
+    <x:row r="107" ht="195" customHeight="1">
       <x:c r="A107" s="103" t="str">
         <x:v>TC-102</x:v>
       </x:c>
@@ -16564,25 +16561,25 @@
         <x:v>每个场景反馈 P95 ≤150ms；内容可交互 P50/P95 均记录并和基线比较。慢 IPC 时切页与加载可用，不等同步查询完成。</x:v>
       </x:c>
       <x:c r="H107" s="103" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>自动子范围通过；完整验收待补证</x:v>
       </x:c>
       <x:c r="I107" s="103" t="str">
-        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-102 1/1、exit 0；开发侧空库/35,000 事实、1180/700px 重复切换 20 次摘要达反馈 P95≤150ms，700px 来源/管理为 12.7/12.4ms。未保存逐次样本和单列冷/热批次；整项待补。</x:v>
       </x:c>
       <x:c r="J107" s="103" t="str">
-        <x:v>npm run test:case -- TC-102（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-102</x:v>
       </x:c>
       <x:c r="K107" s="103" t="str">
-        <x:v>拟新增 TC-102 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-102 独立 Electron 函数；另由 scripts/measure-navigation.mjs 20 产生重复切换摘要。</x:v>
       </x:c>
       <x:c r="L107" s="103" t="str">
-        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
       </x:c>
       <x:c r="M107" s="103" t="str">
-        <x:v>导航性能基线与复测均需固定提交和同机条件；若初测达标，应另复现用户观察到的可感延迟再定义修复。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="176.25" customHeight="1">
+        <x:v>当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="195" customHeight="1">
       <x:c r="A108" s="103" t="str">
         <x:v>TC-103</x:v>
       </x:c>
@@ -16605,25 +16602,25 @@
         <x:v>两种窗口帧间隔 P95 ≤32ms，且任何帧间隔不达到 200ms；滚动后筛选、焦点和可见明细仍正确。</x:v>
       </x:c>
       <x:c r="H108" s="103" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>自动子范围通过；完整验收待补证</x:v>
       </x:c>
       <x:c r="I108" s="103" t="str">
-        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-103 1/1、exit 0（700px/2.5s）；开发侧 35,000 事实双窗口 10s 滚动 P95 17.8/18.6ms，最大 32.6/18.8ms，≥200ms 长任务 0。逐帧样本与滚后交互待补。</x:v>
       </x:c>
       <x:c r="J108" s="103" t="str">
-        <x:v>npm run test:case -- TC-103（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-103</x:v>
       </x:c>
       <x:c r="K108" s="103" t="str">
-        <x:v>拟新增 TC-103 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-103 独立 Electron 函数；另由 scripts/measure-navigation.mjs 20 产生双窗口 10s 滚动摘要。</x:v>
       </x:c>
       <x:c r="L108" s="103" t="str">
-        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
       </x:c>
       <x:c r="M108" s="103" t="str">
-        <x:v>按逐帧间隔计算 P95；不将 FPS 均值当作 P95，也不删去长尾卡顿。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="176.25" customHeight="1">
+        <x:v>独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="195" customHeight="1">
       <x:c r="A109" s="103" t="str">
         <x:v>TC-104</x:v>
       </x:c>
@@ -16646,22 +16643,22 @@
         <x:v>旧响应不能覆盖新页面或新用户；加载和错误状态可操作；筛选与焦点保持；CSV 和当前授权报表为同一快照；跨用户数据/IPC 均不泄露，未知不显示为零，失败可重试。</x:v>
       </x:c>
       <x:c r="H109" s="103" t="str">
-        <x:v>待注册、待验证（规划目标）</x:v>
+        <x:v>自动子范围通过；完整验收待补证</x:v>
       </x:c>
       <x:c r="I109" s="103" t="str">
-        <x:v>2026-10-06 前置规划；待实现、待注册、待执行。已有 0.3.11 页面用例的通过结果不代表本性能门槛通过。</x:v>
+        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-104 1/1、exit 0；快速切页后旧响应不改回概览，viewer 无来源/管理入口。受控慢 IPC、双用户数据、CSV、未知与失败重试未由此用例覆盖；整项待补。</x:v>
       </x:c>
       <x:c r="J109" s="103" t="str">
-        <x:v>npm run test:case -- TC-104（计划；当前不可运行）</x:v>
+        <x:v>npm run test:case -- TC-104</x:v>
       </x:c>
       <x:c r="K109" s="103" t="str">
-        <x:v>拟新增 TC-104 独立函数并在 scripts/test-cases.mjs 注册；当前无实际绑定。</x:v>
+        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-104 独立 Electron 函数；已有 TC-079/077/093 是各自回归，不替代本编号剩余场景。</x:v>
       </x:c>
       <x:c r="L109" s="103" t="str">
-        <x:v>仅独立 userData/SQLite、无正文合成数据；性能样本与上一用户数据须隔离。</x:v>
+        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
       </x:c>
       <x:c r="M109" s="103" t="str">
-        <x:v>回归 REQ-041/TC-079、REQ-047/TC-089–090、REQ-048/TC-093、REQ-040/TC-077 的现有边界；新增用例自身独立。 执行后登记固定提交、Mac 型号/macOS、窗口、数据版本、单编号命令、退出码和脱敏测量证据；当前无通过证据。</x:v>
+        <x:v>独立 TC-104 仅快速切页与 viewer 菜单隔离；未显式注入慢 IPC，未验双用户实际数据、CSV 同快照、未知≠零和失败重试。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17485,12 +17482,12 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18" ht="168.75" customHeight="1">
+    <x:row r="18" ht="195" customHeight="1">
       <x:c r="A18" s="103" t="str">
         <x:v>VER-013</x:v>
       </x:c>
       <x:c r="B18" s="103" t="str">
-        <x:v>0.3.11（当前 Mac 页面修订；性能增量计划）</x:v>
+        <x:v>0.3.11（当前 Mac 页面修订；性能自动子范围）</x:v>
       </x:c>
       <x:c r="C18" s="103" t="str">
         <x:v>页面概览、来源、报表和引导整理；切换与滚动性能</x:v>
@@ -17505,19 +17502,19 @@
         <x:v>DEV-055/056/050/058/052；新增 DEV-059</x:v>
       </x:c>
       <x:c r="G18" s="103" t="str">
-        <x:v>TC-097–101 已有隔离自动证据；新增 TC-102–104 待注册/待验证</x:v>
+        <x:v>TC-097–101 既有页面修订证据；TC-102–104 已注册且自动子范围通过，完整合同待补</x:v>
       </x:c>
       <x:c r="H18" s="103" t="str">
-        <x:v>页面修订在 5902568 分支有既有当前 Mac 隔离自动证据；性能增量本次只完成需求、设计和测试规划，尚未实现或测量基线。</x:v>
+        <x:v>46111d3 页面导航先反馈、加载/重试、旧响应隔离与无变化轮询已实现。文档会话独立核 104 入口、TC-102–104 各 1/1、门禁 104/104 单元与 55/55 Electron；开发侧打包三项 3/3。35,000 条事实导航与 10s 滚动摘要达阈值；见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="I18" s="103" t="str">
-        <x:v>0.3.11 页面修订的已有子范围按原证据；性能增量未完成。完整版本完成状态待 TC-102–104、受影响回归和固定候选复验后评估。</x:v>
+        <x:v>页面修订与性能现有自动子范围通过；冷/热原始样本及 TC-104 完整正确性待补，VER-013 不标完成。未签名本机开发范围，不等于外部分发。</x:v>
       </x:c>
       <x:c r="J18" s="103" t="str">
-        <x:v>2026-10-06；性能基线与修复提交、Mac 环境、原始测量/P50/P95、包与安装证据待补。</x:v>
+        <x:v>2026-10-06 / 46111d3；当前 Mac macOS 15.7.4 x86_64、Node 24.15.0，独立无正文合成数据。基线/复测 JSON 位于开发工作树 Git 忽略的 test-results；文档会话只读核摘要。</x:v>
       </x:c>
       <x:c r="K18" s="103" t="str">
-        <x:v>不将 TC-097–101 的通过外推到新性能门槛；未知/未覆盖不当零，权限、查询快照和真实私人数据边界保持。</x:v>
+        <x:v>冷/热逐次样本、逐帧数据及 TC-104 受控慢查询、双用户数据、CSV、未知、重试待补；内容加载仍约 0.5–1.6s。未验真实安装、生产数据、签名公证或异机。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record cold navigation benchmark blocker
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Re2934719e0774049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rbffc73df048d41ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rb4bc964e3d3848ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R483560964650425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R00f0b31ea9404285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6d7b4934ea5d4030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R84af0748c6c44998"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc767026821894913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0bb2a85ac97a4059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R0820f2952de94e3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4733,7 +4733,8 @@
         <x:v>导航反馈与内容可交互时延</x:v>
       </x:c>
       <x:c r="G108" s="103" t="str">
-        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。</x:v>
+        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。
+冷切换阻塞待修，整项未通过；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="116.25" customHeight="1">
@@ -4756,7 +4757,8 @@
         <x:v>长报表连续滚动帧间隔</x:v>
       </x:c>
       <x:c r="G109" s="103" t="str">
-        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。</x:v>
+        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。
+冷切换阻塞待修，整项未通过；详见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="116.25" customHeight="1">
@@ -7066,7 +7068,7 @@
         <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
       <x:c r="E55" s="103" t="str">
-        <x:v>代码已实现，自动子范围通过；完整需求待补证</x:v>
+        <x:v>代码已实现，自动子范围通过；冷切换阻塞待修，完整需求未验收</x:v>
       </x:c>
       <x:c r="F55" s="103" t="str">
         <x:v>DEV-059</x:v>
@@ -9409,7 +9411,7 @@
         <x:v>src/renderer/index.tsx、overview.tsx、report.tsx；scripts/measure-navigation.mjs、scripts/test-cases.mjs；tests/e2e/navigation-performance.spec.ts；TC-076 升级脚本兼容回归</x:v>
       </x:c>
       <x:c r="F64" s="103" t="str">
-        <x:v>代码已提交；现有自动子范围通过；完整验收待补证</x:v>
+        <x:v>代码已提交；自动子范围通过；长数据查询阻塞待修</x:v>
       </x:c>
       <x:c r="G64" s="103" t="str">
         <x:v>46111d3 已提交导航先反馈、加载/重试、旧响应隔离及无变化轮询。文档会话独立核 104 入口、TC-102–104 各 1/1、104/104 单元与 55/55 Electron；性能摘要达阈值。冷/热原始样本与 TC-104 完整场景待补；详见 docs/validation.md。</x:v>
@@ -16561,10 +16563,11 @@
         <x:v>每个场景反馈 P95 ≤150ms；内容可交互 P50/P95 均记录并和基线比较。慢 IPC 时切页与加载可用，不等同步查询完成。</x:v>
       </x:c>
       <x:c r="H107" s="103" t="str">
-        <x:v>自动子范围通过；完整验收待补证</x:v>
+        <x:v>自动子范围通过；冷切换阻塞待修，整项未通过</x:v>
       </x:c>
       <x:c r="I107" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-102 1/1、exit 0；开发侧空库/35,000 事实、1180/700px 重复切换 20 次摘要达反馈 P95≤150ms，700px 来源/管理为 12.7/12.4ms。未保存逐次样本和单列冷/热批次；整项待补。</x:v>
+        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-102 1/1、exit 0；开发侧空库/35,000 事实、1180/700px 重复切换 20 次摘要达反馈 P95≤150ms，700px 来源/管理为 12.7/12.4ms。未保存逐次样本和单列冷/热批次；整项待补。
+2026-10-06 补测阻塞：修正导航场景/加载状态定位后，35,000 条事实冷启动整组中隔离测试实例的主进程持续处理报表明细查询，长时间无法退出；开发侧中止无效批次并缩小复现。无新的完整 P95；不推断真实生产升级失败。见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J107" s="103" t="str">
         <x:v>npm run test:case -- TC-102</x:v>
@@ -16602,10 +16605,11 @@
         <x:v>两种窗口帧间隔 P95 ≤32ms，且任何帧间隔不达到 200ms；滚动后筛选、焦点和可见明细仍正确。</x:v>
       </x:c>
       <x:c r="H108" s="103" t="str">
-        <x:v>自动子范围通过；完整验收待补证</x:v>
+        <x:v>自动子范围通过；冷切换阻塞待修，整项未通过</x:v>
       </x:c>
       <x:c r="I108" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-103 1/1、exit 0（700px/2.5s）；开发侧 35,000 事实双窗口 10s 滚动 P95 17.8/18.6ms，最大 32.6/18.8ms，≥200ms 长任务 0。逐帧样本与滚后交互待补。</x:v>
+        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-103 1/1、exit 0（700px/2.5s）；开发侧 35,000 事实双窗口 10s 滚动 P95 17.8/18.6ms，最大 32.6/18.8ms，≥200ms 长任务 0。逐帧样本与滚后交互待补。
+2026-10-06 补测阻塞：修正导航场景/加载状态定位后，35,000 条事实冷启动整组中隔离测试实例的主进程持续处理报表明细查询，长时间无法退出；开发侧中止无效批次并缩小复现。无新的完整 P95；不推断真实生产升级失败。见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J108" s="103" t="str">
         <x:v>npm run test:case -- TC-103</x:v>
@@ -17508,13 +17512,14 @@
         <x:v>46111d3 页面导航先反馈、加载/重试、旧响应隔离与无变化轮询已实现。文档会话独立核 104 入口、TC-102–104 各 1/1、门禁 104/104 单元与 55/55 Electron；开发侧打包三项 3/3。35,000 条事实导航与 10s 滚动摘要达阈值；见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="I18" s="103" t="str">
-        <x:v>页面修订与性能现有自动子范围通过；冷/热原始样本及 TC-104 完整正确性待补，VER-013 不标完成。未签名本机开发范围，不等于外部分发。</x:v>
+        <x:v>页面修订及早期性能自动子范围有证据；35,000 条事实冷启动查询阻塞待修，VER-013 未完成。</x:v>
       </x:c>
       <x:c r="J18" s="103" t="str">
         <x:v>2026-10-06 / 46111d3；当前 Mac macOS 15.7.4 x86_64、Node 24.15.0，独立无正文合成数据。基线/复测 JSON 位于开发工作树 Git 忽略的 test-results；文档会话只读核摘要。</x:v>
       </x:c>
       <x:c r="K18" s="103" t="str">
-        <x:v>冷/热逐次样本、逐帧数据及 TC-104 受控慢查询、双用户数据、CSV、未知、重试待补；内容加载仍约 0.5–1.6s。未验真实安装、生产数据、签名公证或异机。</x:v>
+        <x:v>冷/热逐次样本、逐帧数据及 TC-104 受控慢查询、双用户数据、CSV、未知、重试待补；内容加载仍约 0.5–1.6s。未验真实安装、生产数据、签名公证或异机。
+修正脚本的冷启动整组在长数据报表明细查询处中止，尚无完整 P95；此前错误场景样本不用于验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.11 navigation acceptance evidence
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R6d7b4934ea5d4030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R84af0748c6c44998"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rc767026821894913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0bb2a85ac97a4059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R0820f2952de94e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R45b6f94211e544db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R298d2b5b1c0e4f6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa9499bfd27247ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0f57a557a8c34cc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Ree8cda4e573a42da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4713,7 +4713,7 @@
         <x:v>2026-10-05 TC-101 独立通过；0.3.11 当前 Mac 源码门槛 104/104、52/52，打包应用 52/52；DMG 校验通过。</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="116.25" customHeight="1">
+    <x:row r="108" ht="135" customHeight="1">
       <x:c r="A108" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4733,11 +4733,10 @@
         <x:v>导航反馈与内容可交互时延</x:v>
       </x:c>
       <x:c r="G108" s="103" t="str">
-        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。
-冷切换阻塞待修，整项未通过；详见 docs/validation.md。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="116.25" customHeight="1">
+        <x:v>aa3c510 当前 Mac 合成自动验收通过；源码与打包三项定向各 3/3。原始性能样本见 outputs/20261006-token-navigation-performance/README.md；实际安装与外部分发另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="135" customHeight="1">
       <x:c r="A109" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4757,11 +4756,10 @@
         <x:v>长报表连续滚动帧间隔</x:v>
       </x:c>
       <x:c r="G109" s="103" t="str">
-        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。
-冷切换阻塞待修，整项未通过；详见 docs/validation.md。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110" ht="116.25" customHeight="1">
+        <x:v>aa3c510 当前 Mac 合成自动验收通过；源码与打包三项定向各 3/3。原始性能样本见 outputs/20261006-token-navigation-performance/README.md；实际安装与外部分发另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="135" customHeight="1">
       <x:c r="A110" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4781,7 +4779,7 @@
         <x:v>慢响应、切用户与报表快照回归</x:v>
       </x:c>
       <x:c r="G110" s="103" t="str">
-        <x:v>46111d3 已注册；现有自动子范围通过，完整验收待补证。独立 TC-104 仅快速切页与 viewer 菜单隔离；未显式注入慢 IPC，未验双用户实际数据、CSV 同快照、未知≠零和失败重试。</x:v>
+        <x:v>aa3c510 当前 Mac 合成自动验收通过；源码与打包三项定向各 3/3。原始性能样本见 outputs/20261006-token-navigation-performance/README.md；实际安装与外部分发另验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4822,7 +4820,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–050 共 50 条；REQ-050 已有 0.3.11 代码与自动子范围证据，完整需求待补证。各项关联与状态见本页。</x:v>
+        <x:v>REQ-001–050 共 50 条；REQ-050 当前 Mac 合成自动验收通过，实际安装/生产数据另验。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -7054,7 +7052,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="55" ht="195" customHeight="1">
+    <x:row r="55" ht="198.75" customHeight="1">
       <x:c r="A55" s="103" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -7068,7 +7066,7 @@
         <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
       <x:c r="E55" s="103" t="str">
-        <x:v>代码已实现，自动子范围通过；冷切换阻塞待修，完整需求未验收</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实际安装/交付另验</x:v>
       </x:c>
       <x:c r="F55" s="103" t="str">
         <x:v>DEV-059</x:v>
@@ -7077,7 +7075,7 @@
         <x:v>TC-102、TC-103、TC-104</x:v>
       </x:c>
       <x:c r="H55" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：导航先反馈、旧响应按页面代次和账号丢弃；TC-102–104 已注册且现有自动子范围通过。35,000 条事实 700px 来源/管理反馈 P95 546.2→12.7ms、965.5→12.4ms；滚动 P95 18.6ms。冷/热原始样本与 TC-104 完整正确性待补；见 docs/validation.md。</x:v>
+        <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7116,7 +7114,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>DEV-001–059 共 59 项；DEV-059 代码已提交、自动子范围通过，完整验收待补证。各项关联与状态见本页。</x:v>
+        <x:v>DEV-001–059 共 59 项；DEV-059 当前 Mac 合成自动开发与验证完成，版本交付另验。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9394,7 +9392,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="64" ht="172.5" customHeight="1">
+    <x:row r="64" ht="198.75" customHeight="1">
       <x:c r="A64" s="103" t="str">
         <x:v>DEV-059</x:v>
       </x:c>
@@ -9411,10 +9409,10 @@
         <x:v>src/renderer/index.tsx、overview.tsx、report.tsx；scripts/measure-navigation.mjs、scripts/test-cases.mjs；tests/e2e/navigation-performance.spec.ts；TC-076 升级脚本兼容回归</x:v>
       </x:c>
       <x:c r="F64" s="103" t="str">
-        <x:v>代码已提交；自动子范围通过；长数据查询阻塞待修</x:v>
+        <x:v>代码已提交；当前 Mac 合成自动开发与验证完成</x:v>
       </x:c>
       <x:c r="G64" s="103" t="str">
-        <x:v>46111d3 已提交导航先反馈、加载/重试、旧响应隔离及无变化轮询。文档会话独立核 104 入口、TC-102–104 各 1/1、104/104 单元与 55/55 Electron；性能摘要达阈值。冷/热原始样本与 TC-104 完整场景待补；详见 docs/validation.md。</x:v>
+        <x:v>b8bba1d 修复报表快照重复查询，完整门禁 104 入口、105/105 单元、55/55 Electron；aa3c510 补六方向冷切换、滚后筛选/焦点及双用户权限/CSV，同一代码的源码与打包定向 E2E 各 3/3，typecheck 与入口检查通过。补充提交未重跑全量门禁。原始数据见 outputs/20261006-token-navigation-performance/README.md；实装/生产数据归版本验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9461,7 +9459,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–104 共 104 个编号，全部已注册；TC-102–104 现有自动子范围通过、完整验收待补证。人工与发布验收按逐行证据判定。</x:v>
+        <x:v>TC-001–104 共 104 个编号，全部已注册；TC-102–104 当前 Mac 合成自动验收通过。实装与外部分发另验。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -16540,7 +16538,7 @@
         <x:v>自动测试证明已安装可执行文件在隔离样本下的页面行为；真实数据完整性和正式签名/异机分发不由本用例提升为通过。</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="195" customHeight="1">
+    <x:row r="107" ht="198.75" customHeight="1">
       <x:c r="A107" s="103" t="str">
         <x:v>TC-102</x:v>
       </x:c>
@@ -16563,26 +16561,25 @@
         <x:v>每个场景反馈 P95 ≤150ms；内容可交互 P50/P95 均记录并和基线比较。慢 IPC 时切页与加载可用，不等同步查询完成。</x:v>
       </x:c>
       <x:c r="H107" s="103" t="str">
-        <x:v>自动子范围通过；冷切换阻塞待修，整项未通过</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实装另验</x:v>
       </x:c>
       <x:c r="I107" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-102 1/1、exit 0；开发侧空库/35,000 事实、1180/700px 重复切换 20 次摘要达反馈 P95≤150ms，700px 来源/管理为 12.7/12.4ms。未保存逐次样本和单列冷/热批次；整项待补。
-2026-10-06 补测阻塞：修正导航场景/加载状态定位后，35,000 条事实冷启动整组中隔离测试实例的主进程持续处理报表明细查询，长时间无法退出；开发侧中止无效批次并缩小复现。无新的完整 P95；不推断真实生产升级失败。见 docs/validation.md。</x:v>
+        <x:v>aa3c510：空库/35,000 事实、1180/700px，冷/热六方向各 24 组×20 次；反馈 P95 最高 22.1/18.7ms，内容 P95 最高 934.5/897.0ms。受控 400ms IPC 加载与缓存失效单测；源码/打包定向各通过。文档会话只读复算原始值，见 outputs/20261006-token-navigation-performance/README.md。</x:v>
       </x:c>
       <x:c r="J107" s="103" t="str">
         <x:v>npm run test:case -- TC-102</x:v>
       </x:c>
       <x:c r="K107" s="103" t="str">
-        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-102 独立 Electron 函数；另由 scripts/measure-navigation.mjs 20 产生重复切换摘要。</x:v>
+        <x:v>独立 Electron + 报表缓存失效单测 + 冷/热各 20 次集成脚本；固定绑定见 scripts/test-cases.mjs。</x:v>
       </x:c>
       <x:c r="L107" s="103" t="str">
-        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
+        <x:v>当前 Mac macOS 15.7.4 x86_64、Node v24.15.0；隔离无正文合成数据，outputs/20261006-token-navigation-performance/README.md；开发侧源码/打包定向各 3/3；文档会话只读核证。</x:v>
       </x:c>
       <x:c r="M107" s="103" t="str">
-        <x:v>当前性能输出仅有 P50/P95 摘要，无逐次原始导航样本和单列冷/热各 20 次；独立 TC-102 未注入受控慢 IPC。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108" ht="195" customHeight="1">
+        <x:v>当前 Mac 合成自动合同已通过；真实系统目录安装、生产数据、签名公证及异机不由该用例代证。历史阻塞见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="198.75" customHeight="1">
       <x:c r="A108" s="103" t="str">
         <x:v>TC-103</x:v>
       </x:c>
@@ -16605,26 +16602,25 @@
         <x:v>两种窗口帧间隔 P95 ≤32ms，且任何帧间隔不达到 200ms；滚动后筛选、焦点和可见明细仍正确。</x:v>
       </x:c>
       <x:c r="H108" s="103" t="str">
-        <x:v>自动子范围通过；冷切换阻塞待修，整项未通过</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实装另验</x:v>
       </x:c>
       <x:c r="I108" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-103 1/1、exit 0（700px/2.5s）；开发侧 35,000 事实双窗口 10s 滚动 P95 17.8/18.6ms，最大 32.6/18.8ms，≥200ms 长任务 0。逐帧样本与滚后交互待补。
-2026-10-06 补测阻塞：修正导航场景/加载状态定位后，35,000 条事实冷启动整组中隔离测试实例的主进程持续处理报表明细查询，长时间无法退出；开发侧中止无效批次并缩小复现。无新的完整 P95；不推断真实生产升级失败。见 docs/validation.md。</x:v>
+        <x:v>aa3c510：35,000 事实双窗口各滚动 10 秒、各 601 帧；P95 最高 18.6ms、最大 18.8ms、≥200ms 长任务 0。定向 E2E 滚后核工具筛选、趋势明细、焦点及清除筛选；源码/打包各通过。逐帧原始值见 outputs/20261006-token-navigation-performance/README.md。</x:v>
       </x:c>
       <x:c r="J108" s="103" t="str">
         <x:v>npm run test:case -- TC-103</x:v>
       </x:c>
       <x:c r="K108" s="103" t="str">
-        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-103 独立 Electron 函数；另由 scripts/measure-navigation.mjs 20 产生双窗口 10s 滚动摘要。</x:v>
+        <x:v>独立 Electron 10 秒滚动及滚后交互 + 双窗口 10 秒集成脚本；固定绑定见 scripts/test-cases.mjs。</x:v>
       </x:c>
       <x:c r="L108" s="103" t="str">
-        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
+        <x:v>当前 Mac macOS 15.7.4 x86_64、Node v24.15.0；隔离无正文合成数据，outputs/20261006-token-navigation-performance/README.md；开发侧源码/打包定向各 3/3；文档会话只读核证。</x:v>
       </x:c>
       <x:c r="M108" s="103" t="str">
-        <x:v>独立 TC-103 仅 700px 滚动 2.5s；10s 双窗口由独立性能脚本测得，但未留逐帧样本、滚动后筛选/焦点断言。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109" ht="195" customHeight="1">
+        <x:v>当前 Mac 合成自动合同已通过；真实系统目录安装、生产数据、签名公证及异机不由该用例代证。历史阻塞见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="198.75" customHeight="1">
       <x:c r="A109" s="103" t="str">
         <x:v>TC-104</x:v>
       </x:c>
@@ -16647,22 +16643,22 @@
         <x:v>旧响应不能覆盖新页面或新用户；加载和错误状态可操作；筛选与焦点保持；CSV 和当前授权报表为同一快照；跨用户数据/IPC 均不泄露，未知不显示为零，失败可重试。</x:v>
       </x:c>
       <x:c r="H109" s="103" t="str">
-        <x:v>自动子范围通过；完整验收待补证</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实装另验</x:v>
       </x:c>
       <x:c r="I109" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3：文档会话独立 TC-104 1/1、exit 0；快速切页后旧响应不改回概览，viewer 无来源/管理入口。受控慢 IPC、双用户数据、CSV、未知与失败重试未由此用例覆盖；整项待补。</x:v>
+        <x:v>aa3c510：同一 Electron 用例创建 viewer/viewerB 并绑定来源，注入失败重试及 400ms 旧响应；切账号后 viewerB 覆盖未知、管理员 IPC 拒绝；回到 viewer 核 42 Token、快速筛选及授权 CSV 两行。源码/打包定向各通过；关联 TC-079/080/093/077/086/084 回归绑定。见 docs/validation.md。</x:v>
       </x:c>
       <x:c r="J109" s="103" t="str">
         <x:v>npm run test:case -- TC-104</x:v>
       </x:c>
       <x:c r="K109" s="103" t="str">
-        <x:v>tests/e2e/navigation-performance.spec.ts 的 TC-104 独立 Electron 函数；已有 TC-079/077/093 是各自回归，不替代本编号剩余场景。</x:v>
+        <x:v>独立双用户 Electron + TC-079/080/093/077/086/084 关联 E2E；固定绑定见 scripts/test-cases.mjs。</x:v>
       </x:c>
       <x:c r="L109" s="103" t="str">
-        <x:v>独立临时 userData/SQLite 与无正文合成事实；性能基准输出位于开发工作树 Git 忽略的 test-results，文档会话只读核摘要。</x:v>
+        <x:v>当前 Mac macOS 15.7.4 x86_64、Node v24.15.0；隔离无正文合成数据，outputs/20261006-token-navigation-performance/README.md；开发侧源码/打包定向各 3/3；文档会话只读核证。</x:v>
       </x:c>
       <x:c r="M109" s="103" t="str">
-        <x:v>独立 TC-104 仅快速切页与 viewer 菜单隔离；未显式注入慢 IPC，未验双用户实际数据、CSV 同快照、未知≠零和失败重试。 现有通过仅限自动子范围，完整合同与真实安装/生产数据仍待验；固定证据见 docs/validation.md。</x:v>
+        <x:v>当前 Mac 合成自动合同已通过；真实系统目录安装、生产数据、签名公证及异机不由该用例代证。历史阻塞见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17486,7 +17482,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18" ht="195" customHeight="1">
+    <x:row r="18" ht="198.75" customHeight="1">
       <x:c r="A18" s="103" t="str">
         <x:v>VER-013</x:v>
       </x:c>
@@ -17506,20 +17502,19 @@
         <x:v>DEV-055/056/050/058/052；新增 DEV-059</x:v>
       </x:c>
       <x:c r="G18" s="103" t="str">
-        <x:v>TC-097–101 既有页面修订证据；TC-102–104 已注册且自动子范围通过，完整合同待补</x:v>
+        <x:v>TC-097–101 页面修订既有证据；TC-102–104 当前 Mac 合成自动验收通过；实际安装/外部分发待验</x:v>
       </x:c>
       <x:c r="H18" s="103" t="str">
-        <x:v>46111d3 页面导航先反馈、加载/重试、旧响应隔离与无变化轮询已实现。文档会话独立核 104 入口、TC-102–104 各 1/1、门禁 104/104 单元与 55/55 Electron；开发侧打包三项 3/3。35,000 条事实导航与 10s 滚动摘要达阈值；见 docs/validation.md。</x:v>
+        <x:v>0.3.11 页面修订、导航先反馈、加载/重试、过期响应隔离与报表快照缓存已实现。aa3c510 冷/热六方向各 24 组×20 次反馈 P95 最高 22.1/18.7ms；长报表双窗口滚动 P95 最高 18.6ms。TC-102–104 源码与打包定向各 3/3；详见 outputs/20261006-token-navigation-performance/README.md。</x:v>
       </x:c>
       <x:c r="I18" s="103" t="str">
-        <x:v>页面修订及早期性能自动子范围有证据；35,000 条事实冷启动查询阻塞待修，VER-013 未完成。</x:v>
+        <x:v>页面修订与当前 Mac 合成性能自动范围完成；真实系统目录安装/生产数据和外部分发未验，VER-013 完整交付未完成。</x:v>
       </x:c>
       <x:c r="J18" s="103" t="str">
-        <x:v>2026-10-06 / 46111d3；当前 Mac macOS 15.7.4 x86_64、Node 24.15.0，独立无正文合成数据。基线/复测 JSON 位于开发工作树 Git 忽略的 test-results；文档会话只读核摘要。</x:v>
+        <x:v>aa3c510 基于 b8bba1d；b8bba1d 完整门禁 104 入口、105/105 单元、55/55 Electron；补充提交 typecheck、入口检查及源码/打包 TC-102–104 各 3/3，未重跑全套。macOS 15.7.4 x86_64、Node v24.15.0；空库/35,000 合成事实与逐次/逐帧 JSON 见 outputs/20261006-token-navigation-performance/README.md。</x:v>
       </x:c>
       <x:c r="K18" s="103" t="str">
-        <x:v>冷/热逐次样本、逐帧数据及 TC-104 受控慢查询、双用户数据、CSV、未知、重试待补；内容加载仍约 0.5–1.6s。未验真实安装、生产数据、签名公证或异机。
-修正脚本的冷启动整组在长数据报表明细查询处中止，尚无完整 P95；此前错误场景样本不用于验收。</x:v>
+        <x:v>当前 Mac 合成自动性能合同已满足；内容加载最高 P95 934.5ms，导航即时反馈达标。真实系统目录安装、生产数据、签名公证及异机/外部分发仍待独立验收；本轮未固定安装包/DMG 哈希。历史失败与修复见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record main integration and delivery boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R45b6f94211e544db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R298d2b5b1c0e4f6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rfa9499bfd27247ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0f57a557a8c34cc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Ree8cda4e573a42da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd6e01d1431444c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc4882ce02f9c4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce24cbe73ab943d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re2637877d9b04242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rffe0ccedfa4b45b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16694,11 +16694,10 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
-      <x:c r="A2" s="77" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">截至 2026-10-04。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。
-2026-10-04 VER-011 为插入的本机 0.3.8 数字菜单修订；VER-010 仍是未立项的后续菜单栏方向。</x:t>
-        </x:is>
+      <x:c r="A2" s="77" t="str">
+        <x:v>截至 2026-10-06。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。
+2026-10-04 VER-011 为插入的本机 0.3.8 数字菜单修订；VER-010 仍是未立项的后续菜单栏方向。
+2026-10-06：0.3.8–0.3.11 产品代码及文档已并入远端 main 6352651；0.3.11 合并态自动门禁通过，实际安装及交付状态独立判断。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="21" customHeight="1"/>
@@ -17368,121 +17367,119 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="inlineStr">
+    <x:row r="16" ht="198.75" customHeight="1">
+      <x:c r="A16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">VER-011</x:t>
         </x:is>
       </x:c>
-      <x:c r="B16" t="inlineStr">
+      <x:c r="B16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.3.8（当前 Mac 本机未签名交互修订）</x:t>
         </x:is>
       </x:c>
-      <x:c r="C16" t="inlineStr">
+      <x:c r="C16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">数字完整数值菜单</x:t>
         </x:is>
       </x:c>
-      <x:c r="D16" t="inlineStr">
+      <x:c r="D16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">将概览、趋势、排行、项目/模型、报表指标及明细的常驻“复制原值”移入数字悬停/聚焦菜单；保持精确整数键盘复制、未知/待核对边界。</x:t>
         </x:is>
       </x:c>
-      <x:c r="E16" t="inlineStr">
+      <x:c r="E16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-047</x:t>
         </x:is>
       </x:c>
-      <x:c r="F16" t="inlineStr">
+      <x:c r="F16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-056</x:t>
         </x:is>
       </x:c>
-      <x:c r="G16" t="inlineStr">
+      <x:c r="G16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TC-090；趋势布局交叉回归 TC-048</x:t>
         </x:is>
       </x:c>
-      <x:c r="H16" t="inlineStr">
+      <x:c r="H16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">87fa4c6；源码门禁 103/103 单元、46/46 Electron；目录包全量 46/46；当前 Mac 实装包隔离 TC-090 2/2。</x:t>
         </x:is>
       </x:c>
-      <x:c r="I16" t="inlineStr">
+      <x:c r="I16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">本机菜单交互自动子范围通过；未签名本机版已安装。完整 REQ-047 与外部分发未完成。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-04 macOS 15.7.4 x86_64；/Applications/Token.app 0.3.8；DMG SHA-256 3eee22fdb510661ee7ada501fd4039850a78510403acd2bbf901b40666a32b44；app.asar SHA-256 3d0666ff506815e1c68df65504932d99e14a992969781f177c42c6502ff57545。0.3.7 App 与升级前用户数据已存本机受限备份。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K16" t="inlineStr">
+      <x:c r="J16" s="101" t="str">
+        <x:v>2026-10-04 macOS 15.7.4 x86_64；/Applications/Token.app 0.3.8；DMG SHA-256 3eee22fdb510661ee7ada501fd4039850a78510403acd2bbf901b40666a32b44；app.asar SHA-256 3d0666ff506815e1c68df65504932d99e14a992969781f177c42c6502ff57545。0.3.7 App 与升级前用户数据已存本机受限备份。
+2026-10-06：此版本代码随 0.3.8–0.3.11 集成进入远端 main 6352651；原本机安装/功能验收记录仍按上方固定候选，不由主线合并重算。</x:v>
+      </x:c>
+      <x:c r="K16" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">保留 0.3.7 TC-095 的历史范围；0.3.8 仅补本轮菜单及相关回归，真实工具/VoiceOver 和签名公证仍待独立验收。</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="inlineStr">
+    <x:row r="17" ht="198.75" customHeight="1">
+      <x:c r="A17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">VER-012</x:t>
         </x:is>
       </x:c>
-      <x:c r="B17" t="inlineStr">
+      <x:c r="B17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">0.3.9（当前 Mac 本机未签名单用户来源修订）</x:t>
         </x:is>
       </x:c>
-      <x:c r="C17" t="inlineStr">
+      <x:c r="C17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Claude 本地来源默认归属</x:t>
         </x:is>
       </x:c>
-      <x:c r="D17" t="inlineStr">
+      <x:c r="D17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">当前 macOS 用户资料仅有一个有效 Token 管理员时，可确认的 Claude 本地文件来源自动归属该用户；保留手动解除、多用户、旧混合/未知来源待核对和脱敏审计。</x:t>
         </x:is>
       </x:c>
-      <x:c r="E17" t="inlineStr">
+      <x:c r="E17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-049</x:t>
         </x:is>
       </x:c>
-      <x:c r="F17" t="inlineStr">
+      <x:c r="F17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-058</x:t>
         </x:is>
       </x:c>
-      <x:c r="G17" t="inlineStr">
+      <x:c r="G17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TC-096</x:t>
         </x:is>
       </x:c>
-      <x:c r="H17" t="inlineStr">
+      <x:c r="H17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">源码门禁 96 入口、104/104 单元和 47/47 Electron；目录包全量 47/47；当前 Mac 安装包隔离 TC-096 1/1；现有 14 个来源由未归属变为本机默认归属。</x:t>
         </x:is>
       </x:c>
-      <x:c r="I17" t="inlineStr">
+      <x:c r="I17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">本机单用户功能已装机并验证；未签名开发版，外部分发仍待签名公证与异机验收。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-10-04 macOS 15.7.4 x86_64；/Applications/Token.app 0.3.9；DMG SHA-256 b8fb2cd9d73e20cbd4fc26d6808fc96e1c869fe36289cf1a5f4d85897287a30d；app.asar SHA-256 6dcb9906b5cfc1afc39c4af02446cfdb97666efbfa8e28e6007bf7a882211b9f。0.3.8 App 与升级前用户数据保存在本机受限备份。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K17" t="inlineStr">
+      <x:c r="J17" s="101" t="str">
+        <x:v>2026-10-04 macOS 15.7.4 x86_64；/Applications/Token.app 0.3.9；DMG SHA-256 b8fb2cd9d73e20cbd4fc26d6808fc96e1c869fe36289cf1a5f4d85897287a30d；app.asar SHA-256 6dcb9906b5cfc1afc39c4af02446cfdb97666efbfa8e28e6007bf7a882211b9f。0.3.8 App 与升级前用户数据保存在本机受限备份。
+2026-10-06：此版本代码随 0.3.8–0.3.11 集成进入远端 main 6352651；原本机安装/功能验收记录仍按上方固定候选，不由主线合并重算。</x:v>
+      </x:c>
+      <x:c r="K17" s="101" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">不把本机使用者归属声称为 Claude 提供方账号验证；文件代次不明、旧混合身份、遥测未知仍待核对，覆盖完整性/真零另按 REQ-040 验。</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="18" ht="198.75" customHeight="1">
+    <x:row r="18" ht="255" customHeight="1">
       <x:c r="A18" s="103" t="str">
         <x:v>VER-013</x:v>
       </x:c>
@@ -17505,16 +17502,19 @@
         <x:v>TC-097–101 页面修订既有证据；TC-102–104 当前 Mac 合成自动验收通过；实际安装/外部分发待验</x:v>
       </x:c>
       <x:c r="H18" s="103" t="str">
-        <x:v>0.3.11 页面修订、导航先反馈、加载/重试、过期响应隔离与报表快照缓存已实现。aa3c510 冷/热六方向各 24 组×20 次反馈 P95 最高 22.1/18.7ms；长报表双窗口滚动 P95 最高 18.6ms。TC-102–104 源码与打包定向各 3/3；详见 outputs/20261006-token-navigation-performance/README.md。</x:v>
+        <x:v>0.3.11 页面修订、导航先反馈、加载/重试、过期响应隔离与报表快照缓存已实现。aa3c510 冷/热六方向各 24 组×20 次反馈 P95 最高 22.1/18.7ms；长报表双窗口滚动 P95 最高 18.6ms。TC-102–104 源码与打包定向各 3/3；详见 outputs/20261006-token-navigation-performance/README.md。
+2026-10-06：0.3.8–0.3.11 产品代码与本工作簿已快进并入远端 main 6352651；当前进入主线集成完成、目标环境交付待验阶段。</x:v>
       </x:c>
       <x:c r="I18" s="103" t="str">
-        <x:v>页面修订与当前 Mac 合成性能自动范围完成；真实系统目录安装/生产数据和外部分发未验，VER-013 完整交付未完成。</x:v>
+        <x:v>主线集成完成：远端 main 6352651；当前 Mac 合成自动范围与合并态门禁通过。真实系统目录安装、生产数据和外部分发未验，VER-013 完整交付未完成。</x:v>
       </x:c>
       <x:c r="J18" s="103" t="str">
-        <x:v>aa3c510 基于 b8bba1d；b8bba1d 完整门禁 104 入口、105/105 单元、55/55 Electron；补充提交 typecheck、入口检查及源码/打包 TC-102–104 各 3/3，未重跑全套。macOS 15.7.4 x86_64、Node v24.15.0；空库/35,000 合成事实与逐次/逐帧 JSON 见 outputs/20261006-token-navigation-performance/README.md。</x:v>
+        <x:v>aa3c510 基于 b8bba1d；b8bba1d 完整门禁 104 入口、105/105 单元、55/55 Electron；补充提交 typecheck、入口检查及源码/打包 TC-102–104 各 3/3，未重跑全套。macOS 15.7.4 x86_64、Node v24.15.0；空库/35,000 合成事实与逐次/逐帧 JSON 见 outputs/20261006-token-navigation-performance/README.md。
+2026-10-06：开发统筹在合并态 6352651 运行 npm run test:gate，报告 typecheck、104 个 TC 入口、105/105 单元、55/55 Electron 全通过；文档会话只读核远端哈希，未独立复跑本次门禁。</x:v>
       </x:c>
       <x:c r="K18" s="103" t="str">
-        <x:v>当前 Mac 合成自动性能合同已满足；内容加载最高 P95 934.5ms，导航即时反馈达标。真实系统目录安装、生产数据、签名公证及异机/外部分发仍待独立验收；本轮未固定安装包/DMG 哈希。历史失败与修复见 docs/validation.md。</x:v>
+        <x:v>当前 Mac 合成自动性能合同已满足；内容加载最高 P95 934.5ms，导航即时反馈达标。真实系统目录安装、生产数据、签名公证及异机/外部分发仍待独立验收；本轮未固定安装包/DMG 哈希。历史失败与修复见 docs/validation.md。
+主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: plan report cache and five-minute refresh
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rd6e01d1431444c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rc4882ce02f9c4d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce24cbe73ab943d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re2637877d9b04242"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rffe0ccedfa4b45b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R069d925f5f3545ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb6edd37ea9804ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4e6b4eaecbfc4580"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R577cb45cb44b4764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R54121e6c97444940"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="104">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -576,6 +576,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -880,7 +883,8 @@
 版本规划范围纠正：VER-009 为当前三批打磨与交付门槛收尾；VER-010 为未立项的菜单栏方向。
 2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。
 2026-10-06 新增 REQ-050→DEV-059→TC-102–104；当前 50 REQ、59 DEV、104 TC；新增三项待注册/待验证。
-2026-10-06 / 46111d3 已注册 104 个 TC；TC-102–104 现有自动子范围通过，完整合同待补证。</x:v>
+2026-10-06 / 46111d3 已注册 104 个 TC；TC-102–104 现有自动子范围通过，完整合同待补证。
+2026-10-06：REQ-051→DEV-060→TC-105/106 已规划；新两项待注册、待运行，旧 TC-102–104 结果不替代。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -4780,6 +4784,52 @@
       </x:c>
       <x:c r="G110" s="103" t="str">
         <x:v>aa3c510 当前 Mac 合成自动验收通过；源码与打包三项定向各 3/3。原始性能样本见 outputs/20261006-token-navigation-performance/README.md；实际安装与外部分发另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="78.75" customHeight="1">
+      <x:c r="A111" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="B111" s="104" t="str">
+        <x:v>概览与报表缓存复用及五分钟刷新</x:v>
+      </x:c>
+      <x:c r="C111" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="D111" s="104" t="str">
+        <x:v>实现授权报表共享缓存与刷新调度</x:v>
+      </x:c>
+      <x:c r="E111" s="104" t="str">
+        <x:v>TC-105</x:v>
+      </x:c>
+      <x:c r="F111" s="104" t="str">
+        <x:v>切页缓存与五分钟调度</x:v>
+      </x:c>
+      <x:c r="G111" s="104" t="str">
+        <x:v>需求/设计已登记；独立自动入口待注册、待运行。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="78.75" customHeight="1">
+      <x:c r="A112" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="B112" s="104" t="str">
+        <x:v>概览与报表缓存复用及五分钟刷新</x:v>
+      </x:c>
+      <x:c r="C112" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="D112" s="104" t="str">
+        <x:v>实现授权报表共享缓存与刷新调度</x:v>
+      </x:c>
+      <x:c r="E112" s="104" t="str">
+        <x:v>TC-106</x:v>
+      </x:c>
+      <x:c r="F112" s="104" t="str">
+        <x:v>变更失效、跨用户与失败快照</x:v>
+      </x:c>
+      <x:c r="G112" s="104" t="str">
+        <x:v>需求/设计已登记；独立自动入口待注册、待运行。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4820,7 +4870,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–050 共 50 条；REQ-050 当前 Mac 合成自动验收通过，实际安装/生产数据另验。各项关联与状态见本页。</x:v>
+        <x:v>REQ-001–051 共 51 条；REQ-051 已规划概览/报表缓存与五分钟后台查询，待开发和动态验收。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -7076,6 +7126,32 @@
       </x:c>
       <x:c r="H55" s="103" t="str">
         <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="116.25" customHeight="1">
+      <x:c r="A56" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="B56" s="104" t="str">
+        <x:v>概览与报表缓存复用及五分钟刷新</x:v>
+      </x:c>
+      <x:c r="C56" s="104" t="str">
+        <x:v>仅对同一登录用户、授权范围和完整筛选键复用概览/报表的已成功结果；切回相同条件立即显示缓存值，不因挂载清空或反复显示“加载中/正在计算”。后台用量查询以五分钟为节奏，页面切换不重置计时且不产生重复请求；手动刷新、筛选变化和数据/授权变化应立即取新快照。账号切换隔离并清理上个账号可见缓存。失败保留匹配旧值并显式提示未更新，不能把未知/未覆盖写成零。明细与 CSV 使用当前授权报表快照；不复用过期或跨用户结果。五分钟规则不改变来源扫描、服务状态轮询或自动上报节奏。</x:v>
+      </x:c>
+      <x:c r="D56" s="104" t="str">
+        <x:v>0.3.11 主线后页面体验增量</x:v>
+      </x:c>
+      <x:c r="E56" s="104" t="str">
+        <x:v>需求与验收已定义；待开发，未验证</x:v>
+      </x:c>
+      <x:c r="F56" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="G56" s="104" t="str">
+        <x:v>TC-105、TC-106</x:v>
+      </x:c>
+      <x:c r="H56" s="104" t="str">
+        <x:v>2026-10-06：当前 overview.tsx/report.tsx 挂载即查询且各以 15 秒轮询，概览卸载丢结果，报表重建状态；本轮只立项与设计，无代码或新动态通过。既有 REQ-050/TC-102–104 导航性能证据仍归原范围。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7114,7 +7190,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>DEV-001–059 共 59 项；DEV-059 当前 Mac 合成自动开发与验证完成，版本交付另验。</x:v>
+        <x:v>DEV-001–060 共 60 项；DEV-060 为概览/报表缓存和刷新调度，待实施。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9413,6 +9489,29 @@
       </x:c>
       <x:c r="G64" s="103" t="str">
         <x:v>b8bba1d 修复报表快照重复查询，完整门禁 104 入口、105/105 单元、55/55 Electron；aa3c510 补六方向冷切换、滚后筛选/焦点及双用户权限/CSV，同一代码的源码与打包定向 E2E 各 3/3，typecheck 与入口检查通过。补充提交未重跑全量门禁。原始数据见 outputs/20261006-token-navigation-performance/README.md；实装/生产数据归版本验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="116.25" customHeight="1">
+      <x:c r="A65" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="B65" s="104" t="str">
+        <x:v>实现授权报表共享缓存与刷新调度</x:v>
+      </x:c>
+      <x:c r="C65" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="D65" s="104" t="str">
+        <x:v>TC-105、TC-106</x:v>
+      </x:c>
+      <x:c r="E65" s="104" t="str">
+        <x:v>src/renderer/index.tsx、overview.tsx、report.tsx；src/main/report.ts / IPC 失效通知按方案确定；scripts/test-cases.mjs；隔离单元与 Electron 测试</x:v>
+      </x:c>
+      <x:c r="F65" s="104" t="str">
+        <x:v>待实施；不得复用 TC-102–104 结果判通过</x:v>
+      </x:c>
+      <x:c r="G65" s="104" t="str">
+        <x:v>在登录态上方维护按 actor/授权版本/标准化完整筛选键划分的缓存与单一五分钟调度；首查/手动/筛选变更立即请求，数据或授权变更使对应快照失效并刷新。背景失败保留同键旧值并提示未更新，不静默改写 CSV；切用户/登出清理可见状态和未完成请求，旧响应按代次丢弃。先用 TC-105/106 红灯复现，再实现、单编号与完整门禁。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9459,7 +9558,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–104 共 104 个编号，全部已注册；TC-102–104 当前 Mac 合成自动验收通过。实装与外部分发另验。</x:v>
+        <x:v>TC-001–106 共 106 个编号；TC-105/106 已分配、待注册独立自动入口，尚无动态通过证据。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -16659,6 +16758,88 @@
       </x:c>
       <x:c r="M109" s="103" t="str">
         <x:v>当前 Mac 合成自动合同已通过；真实系统目录安装、生产数据、签名公证及异机不由该用例代证。历史阻塞见 docs/validation.md。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="112.5" customHeight="1">
+      <x:c r="A110" s="104" t="str">
+        <x:v>TC-105</x:v>
+      </x:c>
+      <x:c r="B110" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="C110" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="D110" s="104" t="str">
+        <x:v>切页缓存与五分钟调度</x:v>
+      </x:c>
+      <x:c r="E110" s="104" t="str">
+        <x:v>单元 + Electron/集成</x:v>
+      </x:c>
+      <x:c r="F110" s="104" t="str">
+        <x:v>独立临时 userData/SQLite 与无正文合成事实；可控时钟及 queryUsage 调用计数。首次加载概览/报表后多次往返同账号同筛选；推进至 4 分 59 秒、5 分钟；再手动刷新与修改日期/工具/用户/时区筛选。</x:v>
+      </x:c>
+      <x:c r="G110" s="104" t="str">
+        <x:v>相同授权键切回立即显示缓存值，不闪现加载或正在计算，往返不额外查询且不重置五分钟节奏；未到五分钟不后台查询，到期至多一次且无并发重复；手动/筛选变化立即查询，首次无缓存可显示加载。</x:v>
+      </x:c>
+      <x:c r="H110" s="104" t="str">
+        <x:v>已规划；待注册独立入口与动态验收</x:v>
+      </x:c>
+      <x:c r="I110" s="104" t="str">
+        <x:v>待注册、待运行；使用假时钟/IPC 计数和隔离数据库，不读生产 userData。</x:v>
+      </x:c>
+      <x:c r="J110" s="104" t="str">
+        <x:v>npm run test:case -- TC-105（待注册后运行）</x:v>
+      </x:c>
+      <x:c r="K110" s="104" t="str">
+        <x:v>计划在 scripts/test-cases.mjs 为 TC-105 绑定独立函数；不可只挂共享旧用例。</x:v>
+      </x:c>
+      <x:c r="L110" s="104" t="str">
+        <x:v>独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；测试结束清理。</x:v>
+      </x:c>
+      <x:c r="M110" s="104" t="str">
+        <x:v>当前仅为验收设计；无自动通过证据，不证明真实系统安装或生产数据表现。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="112.5" customHeight="1">
+      <x:c r="A111" s="104" t="str">
+        <x:v>TC-106</x:v>
+      </x:c>
+      <x:c r="B111" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="C111" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="D111" s="104" t="str">
+        <x:v>变更失效、跨用户与失败快照</x:v>
+      </x:c>
+      <x:c r="E111" s="104" t="str">
+        <x:v>单元 + Electron/集成</x:v>
+      </x:c>
+      <x:c r="F111" s="104" t="str">
+        <x:v>独立双用户临时库构造不同授权事实、未知覆盖与真实零；制造数据/归属变更、慢响应及一次后台失败，检查概览/报表/明细/CSV，并切用户、登出、重试。</x:v>
+      </x:c>
+      <x:c r="G111" s="104" t="str">
+        <x:v>数据/授权变更后立即刷新或失效，不让旧响应覆盖；B 不见 A 缓存、IPC、CSV；未知与真零区分。失败时只保留同键旧值并显示未更新/重试，不能声称当前值；明细和 CSV 与最新授权 snapshotId 一致，失效旧快照不得静默导出。</x:v>
+      </x:c>
+      <x:c r="H111" s="104" t="str">
+        <x:v>已规划；待注册独立入口与动态验收</x:v>
+      </x:c>
+      <x:c r="I111" s="104" t="str">
+        <x:v>待注册、待运行；一次性双用户库、失败注入和脱敏断言；无真实会话正文。</x:v>
+      </x:c>
+      <x:c r="J111" s="104" t="str">
+        <x:v>npm run test:case -- TC-106（待注册后运行）</x:v>
+      </x:c>
+      <x:c r="K111" s="104" t="str">
+        <x:v>计划在 scripts/test-cases.mjs 为 TC-106 绑定独立函数；不可只挂共享旧用例。</x:v>
+      </x:c>
+      <x:c r="L111" s="104" t="str">
+        <x:v>独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；测试结束清理。</x:v>
+      </x:c>
+      <x:c r="M111" s="104" t="str">
+        <x:v>当前仅为验收设计；无自动通过证据，不证明真实系统安装或生产数据表现。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16697,7 +16878,8 @@
       <x:c r="A2" s="77" t="str">
         <x:v>截至 2026-10-06。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。
 2026-10-04 VER-011 为插入的本机 0.3.8 数字菜单修订；VER-010 仍是未立项的后续菜单栏方向。
-2026-10-06：0.3.8–0.3.11 产品代码及文档已并入远端 main 6352651；0.3.11 合并态自动门禁通过，实际安装及交付状态独立判断。</x:v>
+2026-10-06：0.3.8–0.3.11 产品代码及文档已并入远端 main 6352651；0.3.11 合并态自动门禁通过，实际安装及交付状态独立判断。
+2026-10-06：VER-014 为版本号待定的缓存/刷新增量规划，REQ-051→DEV-060→TC-105/106 均未实现或验收；不改变 VER-013 已有结论。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="21" customHeight="1"/>
@@ -17517,6 +17699,41 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="84" customHeight="1">
+      <x:c r="A19" s="104" t="str">
+        <x:v>VER-014</x:v>
+      </x:c>
+      <x:c r="B19" s="104" t="str">
+        <x:v>版本号待定（概览/报表缓存与刷新节奏）</x:v>
+      </x:c>
+      <x:c r="C19" s="104" t="str">
+        <x:v>同登录态缓存复用与五分钟后台查询增量</x:v>
+      </x:c>
+      <x:c r="D19" s="104" t="str">
+        <x:v>切回同筛选即时显示授权缓存；五分钟后台查询；手动、筛选和数据变化即时刷新；失败旧值提示；跨用户隔离及明细/CSV 同快照。</x:v>
+      </x:c>
+      <x:c r="E19" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="F19" s="104" t="str">
+        <x:v>DEV-060</x:v>
+      </x:c>
+      <x:c r="G19" s="104" t="str">
+        <x:v>TC-105、TC-106（待注册/待运行）</x:v>
+      </x:c>
+      <x:c r="H19" s="104" t="str">
+        <x:v>2026-10-06 SOP-001/002 规划完成；实现、独立自动测试、打包与安装尚未开始。现有 0.3.11 主线和 REQ-050 性能结果为前置基线。</x:v>
+      </x:c>
+      <x:c r="I19" s="104" t="str">
+        <x:v>规划中；无动态通过证据，版本号与交付状态待确定。</x:v>
+      </x:c>
+      <x:c r="J19" s="104" t="str">
+        <x:v>当前 main 93c6872；静态核对 overview.tsx/report.tsx 每次挂载查询、15 秒轮询及卸载状态。新 REQ/DEV/TC 在工作簿已分配，不推断代码已实现。</x:v>
+      </x:c>
+      <x:c r="K19" s="104" t="str">
+        <x:v>版本号在发布候选冻结前确定；真实安装、生产数据及外部分发另按 SOP-005 验。五分钟用量查询不改变来源扫描/同步/状态周期。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:K1"/>

</xml_diff>

<commit_message>
docs: correct TC-106 coverage evidence boundary
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R069d925f5f3545ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rb6edd37ea9804ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R4e6b4eaecbfc4580"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R577cb45cb44b4764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R54121e6c97444940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rc777b8d8d96e45ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R37ed2fee4e1b4231"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce65bbe2e5e84027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R29c0ab297f574484"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rbcd330aaf4fd44bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16801,7 +16801,7 @@
         <x:v>当前仅为验收设计；无自动通过证据，不证明真实系统安装或生产数据表现。</x:v>
       </x:c>
     </x:row>
-    <x:row r="111" ht="112.5" customHeight="1">
+    <x:row r="111" ht="120" customHeight="1">
       <x:c r="A111" s="104" t="str">
         <x:v>TC-106</x:v>
       </x:c>
@@ -16818,16 +16818,16 @@
         <x:v>单元 + Electron/集成</x:v>
       </x:c>
       <x:c r="F111" s="104" t="str">
-        <x:v>独立双用户临时库构造不同授权事实、未知覆盖与真实零；制造数据/归属变更、慢响应及一次后台失败，检查概览/报表/明细/CSV，并切用户、登出、重试。</x:v>
+        <x:v>独立双用户临时库构造不同授权事实：A 有已确认非零，B 的覆盖未知；保留“已确认小计为 0、完整覆盖仍未知”的现有反例，不伪造 complete 真零。再制造数据/归属变更、慢响应与一次后台失败，检查概览/报表/明细/CSV，并切用户、登出、重试。</x:v>
       </x:c>
       <x:c r="G111" s="104" t="str">
-        <x:v>数据/授权变更后立即刷新或失效，不让旧响应覆盖；B 不见 A 缓存、IPC、CSV；未知与真零区分。失败时只保留同键旧值并显示未更新/重试，不能声称当前值；明细和 CSV 与最新授权 snapshotId 一致，失效旧快照不得静默导出。</x:v>
+        <x:v>数据/授权变更后立即刷新或失效，不让旧响应覆盖；B 不见 A 缓存、IPC、CSV，覆盖未知不得渲染成完整真零。已确认小计为 0 时仍标明完整覆盖未知；失败只保留同键旧值并显示未更新/重试；明细与 CSV 和最新授权 snapshotId 一致，失效旧快照不得静默导出。</x:v>
       </x:c>
       <x:c r="H111" s="104" t="str">
         <x:v>已规划；待注册独立入口与动态验收</x:v>
       </x:c>
       <x:c r="I111" s="104" t="str">
-        <x:v>待注册、待运行；一次性双用户库、失败注入和脱敏断言；无真实会话正文。</x:v>
+        <x:v>2026-10-06 验收合同纠正：现行 ReportService.scopedCoverage 无连续采集证据，所有范围为 unknown，不能合法构造 complete 真零。此处只要求未知不得误报为完整零，并保留已确认小计 0/完整覆盖未知反例；动态结果待固定提交和完整门禁。</x:v>
       </x:c>
       <x:c r="J111" s="104" t="str">
         <x:v>npm run test:case -- TC-106（待注册后运行）</x:v>
@@ -16839,7 +16839,7 @@
         <x:v>独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；测试结束清理。</x:v>
       </x:c>
       <x:c r="M111" s="104" t="str">
-        <x:v>当前仅为验收设计；无自动通过证据，不证明真实系统安装或生产数据表现。</x:v>
+        <x:v>不要求伪造 complete 真零；完整覆盖正例待未来可证连续采集方案另行验收。当前此文档分支不登记 TC-106 动态通过，真实安装/生产数据另验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record report refresh traceability and verification
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rc777b8d8d96e45ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R37ed2fee4e1b4231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Rce65bbe2e5e84027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R29c0ab297f574484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="Rbcd330aaf4fd44bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf08772570dc34c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R23f392ee27d142d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R408e36b6f1524587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0b852ce196344c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R84f58a5ff99b4839"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4786,7 +4786,7 @@
         <x:v>aa3c510 当前 Mac 合成自动验收通过；源码与打包三项定向各 3/3。原始性能样本见 outputs/20261006-token-navigation-performance/README.md；实际安装与外部分发另验。</x:v>
       </x:c>
     </x:row>
-    <x:row r="111" ht="78.75" customHeight="1">
+    <x:row r="111" ht="135" customHeight="1">
       <x:c r="A111" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -4806,10 +4806,10 @@
         <x:v>切页缓存与五分钟调度</x:v>
       </x:c>
       <x:c r="G111" s="104" t="str">
-        <x:v>需求/设计已登记；独立自动入口待注册、待运行。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="112" ht="78.75" customHeight="1">
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：TC-105 独立单编号与完整门禁当前 Mac 合成自动通过；实际安装/交付另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="135" customHeight="1">
       <x:c r="A112" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -4829,7 +4829,7 @@
         <x:v>变更失效、跨用户与失败快照</x:v>
       </x:c>
       <x:c r="G112" s="104" t="str">
-        <x:v>需求/设计已登记；独立自动入口待注册、待运行。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：TC-106 独立单编号与完整门禁当前 Mac 合成自动通过；实际安装/交付另验。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4870,7 +4870,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–051 共 51 条；REQ-051 已规划概览/报表缓存与五分钟后台查询，待开发和动态验收。各项关联与状态见本页。</x:v>
+        <x:v>REQ-001–051 共 51 条；REQ-051 当前 Mac 合成自动范围通过，版本交付另验。各项关联与状态见本页。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -7128,7 +7128,7 @@
         <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" ht="116.25" customHeight="1">
+    <x:row r="56" ht="202.5" customHeight="1">
       <x:c r="A56" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -7142,7 +7142,7 @@
         <x:v>0.3.11 主线后页面体验增量</x:v>
       </x:c>
       <x:c r="E56" s="104" t="str">
-        <x:v>需求与验收已定义；待开发，未验证</x:v>
+        <x:v>已实现；当前 Mac 合成自动范围通过，实装交付待验</x:v>
       </x:c>
       <x:c r="F56" s="104" t="str">
         <x:v>DEV-060</x:v>
@@ -7151,7 +7151,7 @@
         <x:v>TC-105、TC-106</x:v>
       </x:c>
       <x:c r="H56" s="104" t="str">
-        <x:v>2026-10-06：当前 overview.tsx/report.tsx 挂载即查询且各以 15 秒轮询，概览卸载丢结果，报表重建状态；本轮只立项与设计，无代码或新动态通过。既有 REQ-050/TC-102–104 导航性能证据仍归原范围。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：共享缓存按登录用户/角色/完整查询键复用；五分钟到期刷新，手动、筛选及数据修订即时查询；旧值失败提示、跨账号隔离、明细/CSV 同授权快照。TC-105/106 单编号和完整门禁通过；当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7190,7 +7190,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>DEV-001–060 共 60 项；DEV-060 为概览/报表缓存和刷新调度，待实施。各项关联与状态见本页。</x:v>
+        <x:v>DEV-001–060 共 60 项；DEV-060 已编码并通过当前 Mac 合成自动验证，交付另验。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9491,7 +9491,7 @@
         <x:v>b8bba1d 修复报表快照重复查询，完整门禁 104 入口、105/105 单元、55/55 Electron；aa3c510 补六方向冷切换、滚后筛选/焦点及双用户权限/CSV，同一代码的源码与打包定向 E2E 各 3/3，typecheck 与入口检查通过。补充提交未重跑全量门禁。原始数据见 outputs/20261006-token-navigation-performance/README.md；实装/生产数据归版本验收。</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" ht="116.25" customHeight="1">
+    <x:row r="65" ht="225" customHeight="1">
       <x:c r="A65" s="104" t="str">
         <x:v>DEV-060</x:v>
       </x:c>
@@ -9505,13 +9505,13 @@
         <x:v>TC-105、TC-106</x:v>
       </x:c>
       <x:c r="E65" s="104" t="str">
-        <x:v>src/renderer/index.tsx、overview.tsx、report.tsx；src/main/report.ts / IPC 失效通知按方案确定；scripts/test-cases.mjs；隔离单元与 Electron 测试</x:v>
+        <x:v>src/renderer/usage-cache.ts、index.tsx、overview.tsx、report.tsx；src/main/database.ts、report.ts、index.ts；src/preload/index.ts、src/shared/types.ts；scripts/test-cases.mjs；tests/usage-cache.test.ts、tests/e2e/usage-refresh.spec.ts</x:v>
       </x:c>
       <x:c r="F65" s="104" t="str">
-        <x:v>待实施；不得复用 TC-102–104 结果判通过</x:v>
+        <x:v>代码已提交；当前 Mac 合成自动开发与验证完成</x:v>
       </x:c>
       <x:c r="G65" s="104" t="str">
-        <x:v>在登录态上方维护按 actor/授权版本/标准化完整筛选键划分的缓存与单一五分钟调度；首查/手动/筛选变更立即请求，数据或授权变更使对应快照失效并刷新。背景失败保留同键旧值并提示未更新，不静默改写 CSV；切用户/登出清理可见状态和未完成请求，旧响应按代次丢弃。先用 TC-105/106 红灯复现，再实现、单编号与完整门禁。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：缓存成功结果与待完成查询，按账号/角色/查询键隔离；五分钟边界、事实修订失效、登出清理与迟到响应代次控制；失败保留匹配旧值并提示未更新。开发侧 npm run test:gate：106 入口、107/107 单元、57/57 Electron；TC-105/106、关联 TC-079/104、性能 TC-102/103 定向通过；打包 usage-refresh 2/2。当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9558,7 +9558,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–106 共 106 个编号；TC-105/106 已分配、待注册独立自动入口，尚无动态通过证据。</x:v>
+        <x:v>TC-001–106 共 106 个编号；TC-105/106 已注册独立入口，当前 Mac 合成自动范围通过。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -16760,7 +16760,7 @@
         <x:v>当前 Mac 合成自动合同已通过；真实系统目录安装、生产数据、签名公证及异机不由该用例代证。历史阻塞见 docs/validation.md。</x:v>
       </x:c>
     </x:row>
-    <x:row r="110" ht="112.5" customHeight="1">
+    <x:row r="110" ht="225" customHeight="1">
       <x:c r="A110" s="104" t="str">
         <x:v>TC-105</x:v>
       </x:c>
@@ -16783,25 +16783,25 @@
         <x:v>相同授权键切回立即显示缓存值，不闪现加载或正在计算，往返不额外查询且不重置五分钟节奏；未到五分钟不后台查询，到期至多一次且无并发重复；手动/筛选变化立即查询，首次无缓存可显示加载。</x:v>
       </x:c>
       <x:c r="H110" s="104" t="str">
-        <x:v>已规划；待注册独立入口与动态验收</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实装另验</x:v>
       </x:c>
       <x:c r="I110" s="104" t="str">
-        <x:v>待注册、待运行；使用假时钟/IPC 计数和隔离数据库，不读生产 userData。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：同键概览↔报表反复切换，queryUsage 无重复调用、无加载回闪；手动刷新立刻请求；假时钟 4 分 59 秒未查询、五分钟到期查询一次；工具、时区、用户、日期变化立即查询。独立单元验证缓存、边界与数据修订失效。 开发侧单编号、完整门禁及打包定向均通过；文档会话核对固定代码和结果摘要。</x:v>
       </x:c>
       <x:c r="J110" s="104" t="str">
-        <x:v>npm run test:case -- TC-105（待注册后运行）</x:v>
+        <x:v>npm run test:case -- TC-105</x:v>
       </x:c>
       <x:c r="K110" s="104" t="str">
-        <x:v>计划在 scripts/test-cases.mjs 为 TC-105 绑定独立函数；不可只挂共享旧用例。</x:v>
+        <x:v>scripts/test-cases.mjs 独立绑定 tests/e2e/usage-refresh.spec.ts 的 TC-105 场景和 tests/usage-cache.test.ts 对应单元。</x:v>
       </x:c>
       <x:c r="L110" s="104" t="str">
-        <x:v>独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；测试结束清理。</x:v>
+        <x:v>macOS 当前 Mac；独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；开发侧完整门禁 106 入口、107 单元、57 Electron，打包定向 2/2。</x:v>
       </x:c>
       <x:c r="M110" s="104" t="str">
-        <x:v>当前仅为验收设计；无自动通过证据，不证明真实系统安装或生产数据表现。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="111" ht="120" customHeight="1">
+        <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="225" customHeight="1">
       <x:c r="A111" s="104" t="str">
         <x:v>TC-106</x:v>
       </x:c>
@@ -16824,22 +16824,22 @@
         <x:v>数据/授权变更后立即刷新或失效，不让旧响应覆盖；B 不见 A 缓存、IPC、CSV，覆盖未知不得渲染成完整真零。已确认小计为 0 时仍标明完整覆盖未知；失败只保留同键旧值并显示未更新/重试；明细与 CSV 和最新授权 snapshotId 一致，失效旧快照不得静默导出。</x:v>
       </x:c>
       <x:c r="H111" s="104" t="str">
-        <x:v>已规划；待注册独立入口与动态验收</x:v>
+        <x:v>当前 Mac 合成自动验收通过；实装另验</x:v>
       </x:c>
       <x:c r="I111" s="104" t="str">
-        <x:v>2026-10-06 验收合同纠正：现行 ReportService.scopedCoverage 无连续采集证据，所有范围为 unknown，不能合法构造 complete 真零。此处只要求未知不得误报为完整零，并保留已确认小计 0/完整覆盖未知反例；动态结果待固定提交和完整门禁。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：合成事实 42→47 后查询、明细和授权 CSV 同步；注入查询失败保留同键旧值并显示未更新，重试恢复；viewer/viewerB 隔离，慢旧响应不覆盖新账号。viewerB 已确认小计 0 且所有覆盖仍 unknown，不冒充完整真零。独立单元验证跨 actor 缓存与失效后的迟到响应。 开发侧单编号、完整门禁及打包定向均通过；文档会话核对固定代码和结果摘要。</x:v>
       </x:c>
       <x:c r="J111" s="104" t="str">
-        <x:v>npm run test:case -- TC-106（待注册后运行）</x:v>
+        <x:v>npm run test:case -- TC-106</x:v>
       </x:c>
       <x:c r="K111" s="104" t="str">
-        <x:v>计划在 scripts/test-cases.mjs 为 TC-106 绑定独立函数；不可只挂共享旧用例。</x:v>
+        <x:v>scripts/test-cases.mjs 独立绑定 tests/e2e/usage-refresh.spec.ts 的 TC-106 场景和 tests/usage-cache.test.ts 对应单元。</x:v>
       </x:c>
       <x:c r="L111" s="104" t="str">
-        <x:v>独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；测试结束清理。</x:v>
+        <x:v>macOS 当前 Mac；独立临时 userData/SQLite、无正文合成事实、假时钟/IPC 计数；开发侧完整门禁 106 入口、107 单元、57 Electron，打包定向 2/2。</x:v>
       </x:c>
       <x:c r="M111" s="104" t="str">
-        <x:v>不要求伪造 complete 真零；完整覆盖正例待未来可证连续采集方案另行验收。当前此文档分支不登记 TC-106 动态通过，真实安装/生产数据另验。</x:v>
+        <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17699,7 +17699,7 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="84" customHeight="1">
+    <x:row r="19" ht="232.5" customHeight="1">
       <x:c r="A19" s="104" t="str">
         <x:v>VER-014</x:v>
       </x:c>
@@ -17719,19 +17719,19 @@
         <x:v>DEV-060</x:v>
       </x:c>
       <x:c r="G19" s="104" t="str">
-        <x:v>TC-105、TC-106（待注册/待运行）</x:v>
+        <x:v>TC-105、TC-106 已注册并在当前 Mac 合成自动范围通过</x:v>
       </x:c>
       <x:c r="H19" s="104" t="str">
-        <x:v>2026-10-06 SOP-001/002 规划完成；实现、独立自动测试、打包与安装尚未开始。现有 0.3.11 主线和 REQ-050 性能结果为前置基线。</x:v>
+        <x:v>共享授权查询缓存、五分钟刷新、手动/筛选/事实变化即时查询、跨账号隔离、失败保留旧值提示和明细/CSV 快照一致均已编码；当前 Mac 合成自动测试及打包定向完成，待确定正式版本并执行目标安装/交付。</x:v>
       </x:c>
       <x:c r="I19" s="104" t="str">
-        <x:v>规划中；无动态通过证据，版本号与交付状态待确定。</x:v>
+        <x:v>实现与当前 Mac 合成自动范围完成；版本号待定，目标系统目录实际安装、生产数据与外部分发未验；VER-014 完整交付未完成。</x:v>
       </x:c>
       <x:c r="J19" s="104" t="str">
-        <x:v>当前 main 93c6872；静态核对 overview.tsx/report.tsx 每次挂载查询、15 秒轮询及卸载状态。新 REQ/DEV/TC 在工作簿已分配，不推断代码已实现。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced；开发侧 npm run test:gate：106 入口、107/107 单元、57/57 Electron；TC-105/106、079/104、102/103 定向通过，打包 usage-refresh 2/2。35,000 合成事实同键概览→报表热切换 1180/700px 各 20 次，反馈 P95 143.5/130.9ms、内容 P95 203.1/180.4ms；10 秒长报表滚动 P95 17.6/17.5ms，≥200ms 0。数值仅属所测路径、窗口与数据集。</x:v>
       </x:c>
       <x:c r="K19" s="104" t="str">
-        <x:v>版本号在发布候选冻结前确定；真实安装、生产数据及外部分发另按 SOP-005 验。五分钟用量查询不改变来源扫描/同步/状态周期。</x:v>
+        <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: plan 0.3.12 update and installed cache acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rf08772570dc34c7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R23f392ee27d142d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R408e36b6f1524587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R0b852ce196344c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R84f58a5ff99b4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5cbe0e18d0074d1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd151825a83d64475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Reb66ee7cefb247f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rc1578dfa1779498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R17b6ed3ca2f94da7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="105">
+  <x:cellXfs count="108">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -578,6 +578,15 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -884,7 +893,9 @@
 2026-10-04 本机交付范围新增 TC-095：总计 48 REQ、57 DEV、95 TC；前 94 项已注册，TC-095 待注册/执行。旧 94 项门禁证据只对应此前固定提交。
 2026-10-06 新增 REQ-050→DEV-059→TC-102–104；当前 50 REQ、59 DEV、104 TC；新增三项待注册/待验证。
 2026-10-06 / 46111d3 已注册 104 个 TC；TC-102–104 现有自动子范围通过，完整合同待补证。
-2026-10-06：REQ-051→DEV-060→TC-105/106 已规划；新两项待注册、待运行，旧 TC-102–104 结果不替代。</x:v>
+2026-10-06：REQ-051→DEV-060→TC-105/106 已规划；新两项待注册、待运行，旧 TC-102–104 结果不替代。
+2026-10-06：0.3.12 实装链路新增 REQ-022/023→DEV-061→TC-107；REQ-050/051→DEV-062→TC-108，均待实施和验收。
+当前工作簿：51 REQ、62 DEV、108 TC；TC-001–106 已注册，TC-107/108 规划待注册。VER-014 目标 0.3.12，生产安装由用户手动更新验收。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -4830,6 +4841,98 @@
       </x:c>
       <x:c r="G112" s="104" t="str">
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：TC-106 独立单编号与完整门禁当前 Mac 合成自动通过；实际安装/交付另验。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="90" customHeight="1">
+      <x:c r="A113" s="104" t="str">
+        <x:v>REQ-022</x:v>
+      </x:c>
+      <x:c r="B113" s="104" t="str">
+        <x:v>版本检查和安装包下载</x:v>
+      </x:c>
+      <x:c r="C113" s="104" t="str">
+        <x:v>DEV-061</x:v>
+      </x:c>
+      <x:c r="D113" s="104" t="str">
+        <x:v>固定 0.3.12 候选并发布本机更新链路</x:v>
+      </x:c>
+      <x:c r="E113" s="104" t="str">
+        <x:v>TC-107</x:v>
+      </x:c>
+      <x:c r="F113" s="104" t="str">
+        <x:v>当前 Mac 0.3.11 应用内升级到 0.3.12</x:v>
+      </x:c>
+      <x:c r="G113" s="104" t="str">
+        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="90" customHeight="1">
+      <x:c r="A114" s="104" t="str">
+        <x:v>REQ-023</x:v>
+      </x:c>
+      <x:c r="B114" s="104" t="str">
+        <x:v>应用内自动安装升级</x:v>
+      </x:c>
+      <x:c r="C114" s="104" t="str">
+        <x:v>DEV-061</x:v>
+      </x:c>
+      <x:c r="D114" s="104" t="str">
+        <x:v>固定 0.3.12 候选并发布本机更新链路</x:v>
+      </x:c>
+      <x:c r="E114" s="104" t="str">
+        <x:v>TC-107</x:v>
+      </x:c>
+      <x:c r="F114" s="104" t="str">
+        <x:v>当前 Mac 0.3.11 应用内升级到 0.3.12</x:v>
+      </x:c>
+      <x:c r="G114" s="104" t="str">
+        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="90" customHeight="1">
+      <x:c r="A115" s="104" t="str">
+        <x:v>REQ-050</x:v>
+      </x:c>
+      <x:c r="B115" s="104" t="str">
+        <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
+      </x:c>
+      <x:c r="C115" s="104" t="str">
+        <x:v>DEV-062</x:v>
+      </x:c>
+      <x:c r="D115" s="104" t="str">
+        <x:v>修复并验证 0.3.12 实装切页与响应</x:v>
+      </x:c>
+      <x:c r="E115" s="104" t="str">
+        <x:v>TC-108</x:v>
+      </x:c>
+      <x:c r="F115" s="104" t="str">
+        <x:v>已安装 0.3.12 缓存切页与性能</x:v>
+      </x:c>
+      <x:c r="G115" s="104" t="str">
+        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="90" customHeight="1">
+      <x:c r="A116" s="104" t="str">
+        <x:v>REQ-051</x:v>
+      </x:c>
+      <x:c r="B116" s="104" t="str">
+        <x:v>概览与报表缓存复用及五分钟刷新</x:v>
+      </x:c>
+      <x:c r="C116" s="104" t="str">
+        <x:v>DEV-062</x:v>
+      </x:c>
+      <x:c r="D116" s="104" t="str">
+        <x:v>修复并验证 0.3.12 实装切页与响应</x:v>
+      </x:c>
+      <x:c r="E116" s="104" t="str">
+        <x:v>TC-108</x:v>
+      </x:c>
+      <x:c r="F116" s="104" t="str">
+        <x:v>已安装 0.3.12 缓存切页与性能</x:v>
+      </x:c>
+      <x:c r="G116" s="104" t="str">
+        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4870,7 +4973,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>REQ-001–051 共 51 条；REQ-051 当前 Mac 合成自动范围通过，版本交付另验。各项关联与状态见本页。</x:v>
+        <x:v>REQ-001–051 共 51 条；REQ-022/023/050/051 的 0.3.12 实装与升级新增验收待实施。既有合成自动通过仍归原固定提交。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -5834,92 +5937,82 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="27" ht="62" customHeight="1">
-      <x:c r="A27" s="35" t="inlineStr">
+    <x:row r="27" ht="266.25" customHeight="1">
+      <x:c r="A27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-022</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" s="35" t="inlineStr">
+      <x:c r="B27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">版本检查和安装包下载</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" s="35" t="inlineStr">
+      <x:c r="C27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">应用请求已配置服务的版本清单，仅较新且平台/架构匹配时提示；下载到受控临时目录，在安装前校验大小和 SHA-256。停服、超时、中断、空间不足、错误摘要和用户取消须展示阶段与可重试状态，坏包绝不交给安装辅助进程，旧版与本机报表仍可用。</x:t>
         </x:is>
       </x:c>
-      <x:c r="D27" s="35" t="inlineStr">
+      <x:c r="D27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">M5（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E27" s="35" t="inlineStr">
+      <x:c r="E27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">已编码；0.3.6 回归通过版本/摘要自动子范围，超时/空间不足等待验</x:t>
         </x:is>
       </x:c>
-      <x:c r="F27" s="35" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-024</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G27" s="35" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-034、TC-035</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H27" s="69" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">当前 1e70412：TC-034/035 与 TC-059 独立回归退出码 0，TC-076 真实 DMG 成功链路通过；异常边界仍按各 TC 待验。
+      <x:c r="F27" s="106" t="str">
+        <x:v>DEV-024、DEV-061</x:v>
+      </x:c>
+      <x:c r="G27" s="106" t="str">
+        <x:v>TC-034、TC-035、TC-107</x:v>
+      </x:c>
+      <x:c r="H27" s="106" t="str">
+        <x:v>当前 1e70412：TC-034/035 与 TC-059 独立回归退出码 0，TC-076 真实 DMG 成功链路通过；异常边界仍按各 TC 待验。
 docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
 2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。
-2026-10-04 / 80e7f10→0eac84b：当前候选 DMG 新 SHA-256 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c、142591838 字节，两包 hdiutil verify VALID；原 27aae018… 为 1e70412 历史候选。此批主要验安装，TC-034/035 的原异常边界不据此提升。</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="62" customHeight="1">
-      <x:c r="A28" s="14" t="inlineStr">
+2026-10-04 / 80e7f10→0eac84b：当前候选 DMG 新 SHA-256 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c、142591838 字节，两包 hdiutil verify VALID；原 27aae018… 为 1e70412 历史候选。此批主要验安装，TC-034/035 的原异常边界不据此提升。
+0.3.12 增量：在实际已安装 0.3.11 上，应用检查更新须从其配置的本机服务得到高于当前版本且 x64 匹配的 0.3.12 清单；“已是最新”不得掩盖无发布包、离线或鉴权错误。发现新版后才能进入下载。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="266.25" customHeight="1">
+      <x:c r="A28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-023</x:t>
         </x:is>
       </x:c>
-      <x:c r="B28" s="14" t="inlineStr">
+      <x:c r="B28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">应用内自动安装升级</x:t>
         </x:is>
       </x:c>
-      <x:c r="C28" s="14" t="inlineStr">
+      <x:c r="C28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">用户在应用内点击“开始升级”后下载并校验 DMG，由受约束辅助进程在旧进程退出后自动安装或替换并重启新版；正常成功无需 Finder 拖拽。只读 DMG 启动时，当前用户可写 /Applications 则自动复制并重启 /Applications/Token.app，否则自动复制并重启用户可写 ~/Applications/Token.app，均无需 Finder 拖拽；已有不可写系统安装须明确授权或报错，不静默迁址。挂载、替换、重启、健康确认失败时恢复旧版并清理临时文件/挂载，用户数据库和凭证不得丢失；受信登录连续性须以真实打包版验证，必要时明确重新登录。
 2026-10-04 前次决议（已被下方最新点击边界取代，仅供追溯）：未点击更新前可放弃；点击后下载并校验，通过后自动退出旧版、原位替换和启动新版；开始执行替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。
 2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。</x:t>
         </x:is>
       </x:c>
-      <x:c r="D28" s="14" t="inlineStr">
+      <x:c r="D28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">M5（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E28" s="14" t="inlineStr">
+      <x:c r="E28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">部分验证；点击前可放弃、点击后下载至安装不可取消为当前决议，真实双 DMG 隔离升级与双路径五故障回退通过；全阶段无取消 UI/系统目录/生产数据待验</x:t>
         </x:is>
       </x:c>
-      <x:c r="F28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-025</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G28" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TC-036、TC-076、TC-095</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H28" s="70" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
+      <x:c r="F28" s="104" t="str">
+        <x:v>DEV-025、DEV-061</x:v>
+      </x:c>
+      <x:c r="G28" s="104" t="str">
+        <x:v>TC-036、TC-076、TC-095、TC-107</x:v>
+      </x:c>
+      <x:c r="H28" s="104" t="str">
+        <x:v>当前 1e70412：TC-076 使用真实 0.3.5 DMG 旧二进制，经临时更新服务自动替换/重启 0.3.6，受信登录和合成 1280 Token 延续；非生产安装。
 历史：docs/design.md §9–13、docs/development-plan.md §7；2026-10-02 44a96e8 本机交接/替换通过；2026-10-03 b224dde 隔离取消后旧版与数据可用、注入式打开失败无替换；真实 Finder 回退等未验，见 docs/validation.md；2026-10-03 变更：原“只打开 DMG”仅保留为 0.3.4 及更早历史。新自动安装/回滚目标见 docs/design.md §11、docs/development-plan.md §7、docs/test-case-acceptance.md；TC-036 需重写断言，TC-076 待注册。TC-028 外部分发独立待验。
 2026-10-03 86a4b5b：辅助进程、同卷暂存/备份/替换/启动及健康标记落地；TC-036 两项单元、TC-076 合成旧版实际打包 App 成功链路由文档会话独立复跑通过。TC-076 的“旧版”是把同一 0.3.5 App 的版本元数据改为 0.3.4，非真实历史 0.3.4 二进制；旧 0.3.0/0.3.4 原按钮不具备自动升级。开发会话另用 0.3.5 helper 对本机原 0.3.0 安装做一次性人工接管并启动 0.3.5，这不证明旧版一键升级。未签名外部分发/目标 Mac 仍由 TC-028 验收。
 2026-10-04 / 80e7f10→0eac84b：80e7f10 的独立 TC-076 最后状态文件读取竞态使整条命令 exit 1；0eac84b 修复测试脚本后同包完整复跑 exit 0。只读旧 DMG 直接启动初始界面已验，但未从只读卷触发更新或实测系统目标；五故障是生产 installer 模块 hooks，非打包 helper/UI。旧成功证据保留。
@@ -5929,8 +6022,8 @@
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 当前新包取干净 main 9af351a，SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；旧 d99d7af9 包的 TC-076 故障证据不外推。
 2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
 2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 当前隔离成功/五故障自动恢复证据继续有效；未知的系统目录、真实满盘/断电与目标 Mac 不升为通过。
-2026-10-04 TC-095 负责当前 Mac 真实安装/更新故障恢复与数据保留的人工发布验收；TC-076 隔离自动故障证据继续有效，不替代系统位置和现有用户数据保护。</x:t>
-        </x:is>
+2026-10-04 TC-095 负责当前 Mac 真实安装/更新故障恢复与数据保留的人工发布验收；TC-076 隔离自动故障证据继续有效，不替代系统位置和现有用户数据保护。
+0.3.12 增量：先以真实 0.3.11 DMG 复制到隔离目录，在应用内发现、下载、摘要校验、原位替换及重启 0.3.12；失败保留可用旧版和测试数据。生产 /Applications/Token.app 的点击升级由用户自行执行，实际安装结果待用户手动验收，不由隔离链路代证。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -7102,33 +7195,35 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="55" ht="198.75" customHeight="1">
-      <x:c r="A55" s="103" t="str">
+    <x:row r="55" ht="266.25" customHeight="1">
+      <x:c r="A55" s="107" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
-      <x:c r="B55" s="103" t="str">
+      <x:c r="B55" s="107" t="str">
         <x:v>0.3.11 页面切换与长报表滚动响应</x:v>
       </x:c>
-      <x:c r="C55" s="103" t="str">
-        <x:v>在当前 Mac 0.3.11 同环境、独立 userData、无正文合成空库与约 35,000 条事实下，标准及 700px 窗口的概览↔报表、数据来源、管理中心冷/热切换各至少 20 次；点击到选中态或骨架屏反馈 P95 ≤150ms，并记录点击到内容可交互的 P50/P95。长报表连续滚动 10 秒，帧间隔 P95 ≤32ms、无 ≥200ms 卡顿。先测基线；若已达标，先复现用户可感知延迟触发条件再修。慢查询时仍能切页并见加载反馈；旧响应不覆盖新页面，不泄露上一用户数据；筛选/焦点、报表 CSV 同一快照、权限、未知≠零、错误重试保持正确。</x:v>
-      </x:c>
-      <x:c r="D55" s="103" t="str">
+      <x:c r="C55" s="107" t="str">
+        <x:v>在当前 Mac 0.3.11 同环境、独立 userData、无正文合成空库与约 35,000 条事实下，标准及 700px 窗口的概览↔报表、数据来源、管理中心冷/热切换各至少 20 次；点击到选中态或骨架屏反馈 P95 ≤150ms，并记录点击到内容可交互的 P50/P95。长报表连续滚动 10 秒，帧间隔 P95 ≤32ms、无 ≥200ms 卡顿。先测基线；若已达标，先复现用户可感知延迟触发条件再修。慢查询时仍能切页并见加载反馈；旧响应不覆盖新页面，不泄露上一用户数据；筛选/焦点、报表 CSV 同一快照、权限、未知≠零、错误重试保持正确。
+0.3.12 将同一门槛应用于最终候选的隔离安装副本与无正文数据；生产安装新版由用户手动复核，不能用 0.3.11 合成结果替代。</x:v>
+      </x:c>
+      <x:c r="D55" s="107" t="str">
         <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
-      <x:c r="E55" s="103" t="str">
+      <x:c r="E55" s="107" t="str">
         <x:v>当前 Mac 合成自动验收通过；实际安装/交付另验</x:v>
       </x:c>
-      <x:c r="F55" s="103" t="str">
-        <x:v>DEV-059</x:v>
-      </x:c>
-      <x:c r="G55" s="103" t="str">
-        <x:v>TC-102、TC-103、TC-104</x:v>
-      </x:c>
-      <x:c r="H55" s="103" t="str">
-        <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="202.5" customHeight="1">
+      <x:c r="F55" s="107" t="str">
+        <x:v>DEV-059、DEV-062</x:v>
+      </x:c>
+      <x:c r="G55" s="107" t="str">
+        <x:v>TC-102、TC-103、TC-104、TC-108</x:v>
+      </x:c>
+      <x:c r="H55" s="107" t="str">
+        <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。
+0.3.12 增量：以最终 0.3.12 候选可执行文件的隔离安装副本及同环境无正文数据复验 1180/700px、至少 20 次冷热切换反馈 P95≤150ms、长报表 10 秒帧间隔 P95≤32ms 且无≥200ms 停顿；记录内容可交互 P50/P95。生产 /Applications 新版切页由用户升级后手动验收，不能用源码或目录包合成指标代证。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="266.25" customHeight="1">
       <x:c r="A56" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -7136,22 +7231,24 @@
         <x:v>概览与报表缓存复用及五分钟刷新</x:v>
       </x:c>
       <x:c r="C56" s="104" t="str">
-        <x:v>仅对同一登录用户、授权范围和完整筛选键复用概览/报表的已成功结果；切回相同条件立即显示缓存值，不因挂载清空或反复显示“加载中/正在计算”。后台用量查询以五分钟为节奏，页面切换不重置计时且不产生重复请求；手动刷新、筛选变化和数据/授权变化应立即取新快照。账号切换隔离并清理上个账号可见缓存。失败保留匹配旧值并显式提示未更新，不能把未知/未覆盖写成零。明细与 CSV 使用当前授权报表快照；不复用过期或跨用户结果。五分钟规则不改变来源扫描、服务状态轮询或自动上报节奏。</x:v>
+        <x:v>仅对同一登录用户、授权范围和完整筛选键复用概览/报表的已成功结果；切回相同条件立即显示缓存值，不因挂载清空或反复显示“加载中/正在计算”。后台用量查询以五分钟为节奏，页面切换不重置计时且不产生重复请求；手动刷新、筛选变化和数据/授权变化应立即取新快照。账号切换隔离并清理上个账号可见缓存。失败保留匹配旧值并显式提示未更新，不能把未知/未覆盖写成零。明细与 CSV 使用当前授权报表快照；不复用过期或跨用户结果。五分钟规则不改变来源扫描、服务状态轮询或自动上报节奏。
+0.3.12 先以隔离安装副本验缓存命中无首次加载回闪；用户自行升级 /Applications 后再复核实际切页，性能以 REQ-050 门槛独立衡量。</x:v>
       </x:c>
       <x:c r="D56" s="104" t="str">
-        <x:v>0.3.11 主线后页面体验增量</x:v>
+        <x:v>0.3.12 当前 Mac 实装修复候选</x:v>
       </x:c>
       <x:c r="E56" s="104" t="str">
         <x:v>已实现；当前 Mac 合成自动范围通过，实装交付待验</x:v>
       </x:c>
       <x:c r="F56" s="104" t="str">
-        <x:v>DEV-060</x:v>
+        <x:v>DEV-060、DEV-062</x:v>
       </x:c>
       <x:c r="G56" s="104" t="str">
-        <x:v>TC-105、TC-106</x:v>
+        <x:v>TC-105、TC-106、TC-108</x:v>
       </x:c>
       <x:c r="H56" s="104" t="str">
-        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：共享缓存按登录用户/角色/完整查询键复用；五分钟到期刷新，手动、筛选及数据修订即时查询；旧值失败提示、跨账号隔离、明细/CSV 同授权快照。TC-105/106 单编号和完整门禁通过；当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
+        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：共享缓存按登录用户/角色/完整查询键复用；五分钟到期刷新，手动、筛选及数据修订即时查询；旧值失败提示、跨账号隔离、明细/CSV 同授权快照。TC-105/106 单编号和完整门禁通过；当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。
+0.3.12 增量：隔离安装副本与用户手动升级后的生产新版，在同账号、同授权及筛选下概览↔报表切回立即显示缓存结果，不反复出现首次加载、重复发查询或重置五分钟计时；手动/筛选/数据变更及失败状态沿用原合同。旧 0.3.11 实装出现每次加载的用户反馈尚待新版实测。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7190,7 +7287,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>DEV-001–060 共 60 项；DEV-060 已编码并通过当前 Mac 合成自动验证，交付另验。</x:v>
+        <x:v>DEV-001–062 共 62 项；DEV-061/062 为 0.3.12 更新发布和实装页面体验，待实施。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -9512,6 +9609,52 @@
       </x:c>
       <x:c r="G65" s="104" t="str">
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：缓存成功结果与待完成查询，按账号/角色/查询键隔离；五分钟边界、事实修订失效、登出清理与迟到响应代次控制；失败保留匹配旧值并提示未更新。开发侧 npm run test:gate：106 入口、107/107 单元、57/57 Electron；TC-105/106、关联 TC-079/104、性能 TC-102/103 定向通过；打包 usage-refresh 2/2。当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="195" customHeight="1">
+      <x:c r="A66" s="104" t="str">
+        <x:v>DEV-061</x:v>
+      </x:c>
+      <x:c r="B66" s="104" t="str">
+        <x:v>固定 0.3.12 候选并发布本机更新链路</x:v>
+      </x:c>
+      <x:c r="C66" s="104" t="str">
+        <x:v>REQ-022、REQ-023</x:v>
+      </x:c>
+      <x:c r="D66" s="104" t="str">
+        <x:v>TC-107</x:v>
+      </x:c>
+      <x:c r="E66" s="104" t="str">
+        <x:v>package.json；package-lock.json；本机未签名 x64 DMG；scripts/publish-update.mjs；更新服务 manifest、UpdateClient/安装 helper 及打包回归（按定位结果修改）</x:v>
+      </x:c>
+      <x:c r="F66" s="104" t="str">
+        <x:v>已规划；待代码、制品及实装验证</x:v>
+      </x:c>
+      <x:c r="G66" s="104" t="str">
+        <x:v>只读核当前 /Applications 0.3.11 与所连本机服务配置；候选版升至 0.3.12，固定代码、DMG 大小/SHA-256，发布到当前应用连接的本机更新服务并核在线清单/版本/架构/鉴权。以真实 0.3.11 DMG 复制到隔离安装目录验证应用内发现→下载→替换→重启及故障回退。开发不得替用户升级生产 /Applications/Token.app；用户自行点击更新并手动验收。不得读取或提交生产数据库/密钥。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="195" customHeight="1">
+      <x:c r="A67" s="104" t="str">
+        <x:v>DEV-062</x:v>
+      </x:c>
+      <x:c r="B67" s="104" t="str">
+        <x:v>修复并验证 0.3.12 实装切页与响应</x:v>
+      </x:c>
+      <x:c r="C67" s="104" t="str">
+        <x:v>REQ-050、REQ-051</x:v>
+      </x:c>
+      <x:c r="D67" s="104" t="str">
+        <x:v>TC-108</x:v>
+      </x:c>
+      <x:c r="E67" s="104" t="str">
+        <x:v>src/renderer/usage-cache.ts、overview.tsx、report.tsx、index.tsx；src/main/report.ts；独立实装性能/缓存核验脚本与按编号入口（依实际根因定稿）</x:v>
+      </x:c>
+      <x:c r="F67" s="104" t="str">
+        <x:v>已规划；待代码、制品及实装验证</x:v>
+      </x:c>
+      <x:c r="G67" s="104" t="str">
+        <x:v>以最终 0.3.12 可执行文件的隔离安装副本复现同筛选往返与 loading 问题；若仍触发查询/回闪，定位 actor/查询键、缓存生命周期和 IPC/渲染瓶颈并修复。以临时 userData 和无正文合成空库/35,000 事实测 1180/700px 冷热至少 20 次、10 秒长报表；生产 /Applications 新版由用户自行升级后手动确认切页表现。保留旧版本样本与失败记录，禁止测试写生产用户数据。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9558,7 +9701,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>TC-001–106 共 106 个编号；TC-105/106 已注册独立入口，当前 Mac 合成自动范围通过。</x:v>
+        <x:v>TC-001–108 共 108 个编号；TC-107/108 已规划，独立入口待注册、实装证据待取得；TC-105/106 既有合成结果保留。</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n"/>
       <x:c r="C3" s="2" t="n"/>
@@ -16840,6 +16983,88 @@
       </x:c>
       <x:c r="M111" s="104" t="str">
         <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="225" customHeight="1">
+      <x:c r="A112" s="104" t="str">
+        <x:v>TC-107</x:v>
+      </x:c>
+      <x:c r="B112" s="104" t="str">
+        <x:v>REQ-022、REQ-023</x:v>
+      </x:c>
+      <x:c r="C112" s="104" t="str">
+        <x:v>DEV-061</x:v>
+      </x:c>
+      <x:c r="D112" s="104" t="str">
+        <x:v>0.3.11 隔离升级及用户实装验收</x:v>
+      </x:c>
+      <x:c r="E112" s="104" t="str">
+        <x:v>当前 Mac 实装人工 + 隔离集成/性能</x:v>
+      </x:c>
+      <x:c r="F112" s="104" t="str">
+        <x:v>只读固定生产 /Applications/Token.app 为旧版 0.3.11；固定 0.3.12 代码、真实 x64 DMG、大小/SHA-256、hdiutil 与当前 App 所连本机服务清单/在线响应。将真实 0.3.11 DMG 中 App 复制到独立可写安装目录，用临时 userData 在旧版界面检查更新、下载、自动退出、原位替换、重启及合成用量延续；在隔离路径注入失败并核旧版回退。生产 /Applications 的点击与结果由用户自行执行并提供脱敏手动证据。</x:v>
+      </x:c>
+      <x:c r="G112" s="104" t="str">
+        <x:v>隔离旧版及用户随后操作的生产旧版均应发现 0.3.12；不把未发布/离线/拒权写成“已是最新”。隔离升级无 Finder 拖拽，替换后 0.3.12 重启，合成数据保留；故障回退旧版并清理。生产安装仅在用户自行点击后依据脱敏版本、启动、受信状态和既有用量核验，不由开发或隔离结果代替。</x:v>
+      </x:c>
+      <x:c r="H112" s="104" t="str">
+        <x:v>已规划；入口待注册，实际安装与动态验收未执行</x:v>
+      </x:c>
+      <x:c r="I112" s="104" t="str">
+        <x:v>2026-10-06：仅核到 /Applications/Token.app 和 package.json 均为 0.3.11；用户报告旧版切页重复加载且检查更新称最新。0.3.12 尚无固定候选、在线清单、实装或动态通过证据。</x:v>
+      </x:c>
+      <x:c r="J112" s="104" t="str">
+        <x:v>npm run test:case -- TC-107（计划独立入口；隔离自动子范围与用户实装人工证据分别记录）</x:v>
+      </x:c>
+      <x:c r="K112" s="104" t="str">
+        <x:v>计划在 scripts/test-cases.mjs 分配独立人工入口；实装性能脚本须使用当前已安装可执行文件，不能只跑源码构建。</x:v>
+      </x:c>
+      <x:c r="L112" s="104" t="str">
+        <x:v>当前 Mac；隔离合成测试只写临时 userData/SQLite；实际安装步骤仅留脱敏摘要、版本/制品校验与可见结果。</x:v>
+      </x:c>
+      <x:c r="M112" s="104" t="str">
+        <x:v>旧 0.3.11 实装症状与 2e5ee34 源码合成通过可同时成立；不得以源码测试推断 0.3.12 实装已通过。生产数据不复制入库。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="225" customHeight="1">
+      <x:c r="A113" s="104" t="str">
+        <x:v>TC-108</x:v>
+      </x:c>
+      <x:c r="B113" s="104" t="str">
+        <x:v>REQ-050、REQ-051</x:v>
+      </x:c>
+      <x:c r="C113" s="104" t="str">
+        <x:v>DEV-062</x:v>
+      </x:c>
+      <x:c r="D113" s="104" t="str">
+        <x:v>0.3.12 隔离切页性能及用户实装体验</x:v>
+      </x:c>
+      <x:c r="E113" s="104" t="str">
+        <x:v>当前 Mac 实装人工 + 隔离集成/性能</x:v>
+      </x:c>
+      <x:c r="F113" s="104" t="str">
+        <x:v>固定最终 0.3.12 候选可执行文件摘要；以其隔离安装副本及临时 userData、空库/35,000 无正文合成事实，在 1180/700px 对概览↔报表及来源/管理中心冷/热各至少 20 次采逐次反馈与内容时间，并在长报表双窗口各滚 10 秒记录逐帧间隔；核 queryUsage 计数与五分钟边界。用户自行升级生产 App 后，在真实登录态只读观察同账号/同筛选概览↔报表往返缓存显示，不采集正文。</x:v>
+      </x:c>
+      <x:c r="G113" s="104" t="str">
+        <x:v>隔离副本与用户实装新版同键切回均立即显示已授权缓存，不反复出现首次加载或重复用量查询；筛选/手动/数据变化即时更新。隔离性能每场景反馈 P95≤150ms；内容 P50/P95 留基线；双窗口长报表帧间隔 P95≤32ms、无≥200ms 停顿；旧响应与跨用户隔离、未知≠零不退化。用户实装确认前不宣称生产体验完成。</x:v>
+      </x:c>
+      <x:c r="H113" s="104" t="str">
+        <x:v>已规划；入口待注册，实际安装与动态验收未执行</x:v>
+      </x:c>
+      <x:c r="I113" s="104" t="str">
+        <x:v>2026-10-06：仅核到 /Applications/Token.app 和 package.json 均为 0.3.11；用户报告旧版切页重复加载且检查更新称最新。0.3.12 尚无固定候选、在线清单、实装或动态通过证据。</x:v>
+      </x:c>
+      <x:c r="J113" s="104" t="str">
+        <x:v>npm run test:case -- TC-108（计划独立入口；隔离性能与用户实装人工证据分别记录）</x:v>
+      </x:c>
+      <x:c r="K113" s="104" t="str">
+        <x:v>计划在 scripts/test-cases.mjs 分配独立人工入口；实装性能脚本须使用当前已安装可执行文件，不能只跑源码构建。</x:v>
+      </x:c>
+      <x:c r="L113" s="104" t="str">
+        <x:v>当前 Mac；隔离合成测试只写临时 userData/SQLite；实际安装步骤仅留脱敏摘要、版本/制品校验与可见结果。</x:v>
+      </x:c>
+      <x:c r="M113" s="104" t="str">
+        <x:v>旧 0.3.11 实装症状与 2e5ee34 源码合成通过可同时成立；不得以源码测试推断 0.3.12 实装已通过。生产数据不复制入库。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16876,10 +17101,8 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="77" t="str">
-        <x:v>截至 2026-10-06。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。VER-009 是当前目标的未完成收尾，不是顺延；VER-010 才是未立项的下一轮方向。历史本机候选不等于公开发布；未定版号不承诺日期。
-2026-10-04 VER-011 为插入的本机 0.3.8 数字菜单修订；VER-010 仍是未立项的后续菜单栏方向。
-2026-10-06：0.3.8–0.3.11 产品代码及文档已并入远端 main 6352651；0.3.11 合并态自动门禁通过，实际安装及交付状态独立判断。
-2026-10-06：VER-014 为版本号待定的缓存/刷新增量规划，REQ-051→DEV-060→TC-105/106 均未实现或验收；不改变 VER-013 已有结论。</x:v>
+        <x:v>截至 2026-10-06。VER 是版本跟踪行号；REQ/DEV/TC 的唯一编号和逐项状态仍以其他工作表为准。历史本机候选不等于公开发布；未定版号不承诺日期。
+2026-10-06：VER-014 已指定 0.3.12 本机更新与切页体验候选；当前生产 App/package.json 为 0.3.11。DEV-061/062、TC-107/108 已规划，代码、制品、清单及实装证据待完成。开发仅向当前 App 所连服务发布，用户自行点击升级生产 App。REQ-051 的 2e5ee34 证据仍只属 0.3.11 合成自动范围。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="21" customHeight="1"/>
@@ -17699,39 +17922,39 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="232.5" customHeight="1">
+    <x:row r="19" ht="255" customHeight="1">
       <x:c r="A19" s="104" t="str">
         <x:v>VER-014</x:v>
       </x:c>
       <x:c r="B19" s="104" t="str">
-        <x:v>版本号待定（概览/报表缓存与刷新节奏）</x:v>
+        <x:v>0.3.12（当前 Mac 更新与缓存体验候选）</x:v>
       </x:c>
       <x:c r="C19" s="104" t="str">
-        <x:v>同登录态缓存复用与五分钟后台查询增量</x:v>
+        <x:v>0.3.11 应用内更新到 0.3.12；实装缓存切页与性能</x:v>
       </x:c>
       <x:c r="D19" s="104" t="str">
-        <x:v>切回同筛选即时显示授权缓存；五分钟后台查询；手动、筛选和数据变化即时刷新；失败旧值提示；跨用户隔离及明细/CSV 同快照。</x:v>
+        <x:v>固定 0.3.12 未签名本机候选及更新清单；旧版应用内发现、下载、原位替换、重启；新版同键切页即时缓存、五分钟刷新、长报表性能与权限/CSV 边界。</x:v>
       </x:c>
       <x:c r="E19" s="104" t="str">
-        <x:v>REQ-051</x:v>
+        <x:v>REQ-022、REQ-023、REQ-050、REQ-051</x:v>
       </x:c>
       <x:c r="F19" s="104" t="str">
-        <x:v>DEV-060</x:v>
+        <x:v>DEV-024、DEV-025、DEV-059、DEV-060、DEV-061、DEV-062</x:v>
       </x:c>
       <x:c r="G19" s="104" t="str">
-        <x:v>TC-105、TC-106 已注册并在当前 Mac 合成自动范围通过</x:v>
+        <x:v>TC-105/106 合成自动已有证据；新增 TC-107/108 实装/性能待注册与执行；回归 TC-034–036/076/102–104</x:v>
       </x:c>
       <x:c r="H19" s="104" t="str">
-        <x:v>共享授权查询缓存、五分钟刷新、手动/筛选/事实变化即时查询、跨账号隔离、失败保留旧值提示和明细/CSV 快照一致均已编码；当前 Mac 合成自动测试及打包定向完成，待确定正式版本并执行目标安装/交付。</x:v>
+        <x:v>2e5ee34 缓存功能已编码且合成自动通过；当前 /Applications/Token.app 与 package.json 仍为 0.3.11。0.3.12 版本、真实 DMG、本机更新服务发布、隔离旧版 UI 升级及新版切页/性能均待实施。生产 App 由用户自行点击更新与手动验收。</x:v>
       </x:c>
       <x:c r="I19" s="104" t="str">
-        <x:v>实现与当前 Mac 合成自动范围完成；版本号待定，目标系统目录实际安装、生产数据与外部分发未验；VER-014 完整交付未完成。</x:v>
+        <x:v>规划中：0.3.12 尚未固定或发布；TC-107/108 隔离与用户实装均无动态通过证据。VER-014 完整交付未完成。</x:v>
       </x:c>
       <x:c r="J19" s="104" t="str">
-        <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced；开发侧 npm run test:gate：106 入口、107/107 单元、57/57 Electron；TC-105/106、079/104、102/103 定向通过，打包 usage-refresh 2/2。35,000 合成事实同键概览→报表热切换 1180/700px 各 20 次，反馈 P95 143.5/130.9ms、内容 P95 203.1/180.4ms；10 秒长报表滚动 P95 17.6/17.5ms，≥200ms 0。数值仅属所测路径、窗口与数据集。</x:v>
+        <x:v>2026-10-06 只读核 /Applications/Token.app Info.plist 与 package.json 均为 0.3.11。用户报告旧实装切页加载/卡顿、设置称最新；2e5ee34 的 106 入口/107 单元/57 Electron 与打包定向 2/2 仅证明合成范围，不证明旧安装含该实现。0.3.12 待记录代码、DMG 大小/SHA-256、在线 manifest、TC-107/108、目标安装与性能样本。</x:v>
       </x:c>
       <x:c r="K19" s="104" t="str">
-        <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
+        <x:v>“已是最新”也可能表示本机服务尚无新版清单，需核在线响应与鉴权后定位。开发仅发布到当前 App 所连本机服务，不替用户升级生产 /Applications。用户自行升级并手动验收前，不标实装完成；生产数据只留脱敏摘要。签名公证及异机外部分发仍属独立门槛。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.12 release and isolated acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R5cbe0e18d0074d1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rd151825a83d64475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Reb66ee7cefb247f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rc1578dfa1779498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R17b6ed3ca2f94da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rcc0f0f611d124764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re701dbfbcaee41e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re09c970c4cfa423f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R22ae91b5014949b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R25a67b63f04443b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4843,7 +4843,7 @@
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：TC-106 独立单编号与完整门禁当前 Mac 合成自动通过；实际安装/交付另验。</x:v>
       </x:c>
     </x:row>
-    <x:row r="113" ht="90" customHeight="1">
+    <x:row r="113" ht="108.75" customHeight="1">
       <x:c r="A113" s="104" t="str">
         <x:v>REQ-022</x:v>
       </x:c>
@@ -4863,10 +4863,10 @@
         <x:v>当前 Mac 0.3.11 应用内升级到 0.3.12</x:v>
       </x:c>
       <x:c r="G113" s="104" t="str">
-        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="114" ht="90" customHeight="1">
+        <x:v>TC-107 在线服务清单/包及隔离升级通过；用户生产 App 待自行更新验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="108.75" customHeight="1">
       <x:c r="A114" s="104" t="str">
         <x:v>REQ-023</x:v>
       </x:c>
@@ -4886,10 +4886,10 @@
         <x:v>当前 Mac 0.3.11 应用内升级到 0.3.12</x:v>
       </x:c>
       <x:c r="G114" s="104" t="str">
-        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="115" ht="90" customHeight="1">
+        <x:v>TC-107 隔离自动安装/回退通过；实际 /Applications 安装由用户手动验收，未交付。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115" ht="108.75" customHeight="1">
       <x:c r="A115" s="104" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4909,10 +4909,10 @@
         <x:v>已安装 0.3.12 缓存切页与性能</x:v>
       </x:c>
       <x:c r="G115" s="104" t="str">
-        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116" ht="90" customHeight="1">
+        <x:v>TC-108 打包 E2E 通过；性能集成命令进行中，生产新版性能待用户验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="108.75" customHeight="1">
       <x:c r="A116" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -4932,7 +4932,7 @@
         <x:v>已安装 0.3.12 缓存切页与性能</x:v>
       </x:c>
       <x:c r="G116" s="104" t="str">
-        <x:v>0.3.12 当前 Mac 实装增量已规划；独立入口、固定候选及动态结果待取得。</x:v>
+        <x:v>TC-108 缓存 E2E 通过；性能集成进行中，生产实装切页待用户确认。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5937,7 +5937,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="27" ht="266.25" customHeight="1">
+    <x:row r="27" ht="225" customHeight="1">
       <x:c r="A27" s="106" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-022</x:t>
@@ -5958,10 +5958,8 @@
           <x:t xml:space="preserve">M5（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E27" s="106" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">已编码；0.3.6 回归通过版本/摘要自动子范围，超时/空间不足等待验</x:t>
-        </x:is>
+      <x:c r="E27" s="106" t="str">
+        <x:v>0.3.12 x64 已发布到当前本机服务；TC-107 隔离升级通过，生产实装待用户验收</x:v>
       </x:c>
       <x:c r="F27" s="106" t="str">
         <x:v>DEV-024、DEV-061</x:v>
@@ -5974,10 +5972,11 @@
 docs/design.md §9–13；docs/development-plan.md §7；2026-10-03 新目标见 docs/design.md §11、docs/test-case-acceptance.md TC-034/035。旧自动通过仅覆盖版本/架构/摘要和部分停服重试；安装前坏包拒绝、空间不足与阶段状态等新增口径待验。
 2026-10-03 86a4b5b：UpdateClient 改为 downloadAndInstall，校验大小/SHA-256 后才交自动安装；文档会话在该提交复跑 TC-034 1/1、TC-035 1/1、TC-059 1/1、76 入口检查退出码 0。现有断言未单独覆盖磁盘不足、超时和真实安装失败。
 2026-10-04 / 80e7f10→0eac84b：当前候选 DMG 新 SHA-256 d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c、142591838 字节，两包 hdiutil verify VALID；原 27aae018… 为 1e70412 历史候选。此批主要验安装，TC-034/035 的原异常边界不据此提升。
-0.3.12 增量：在实际已安装 0.3.11 上，应用检查更新须从其配置的本机服务得到高于当前版本且 x64 匹配的 0.3.12 清单；“已是最新”不得掩盖无发布包、离线或鉴权错误。发现新版后才能进入下载。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="266.25" customHeight="1">
+0.3.12 增量：在实际已安装 0.3.11 上，应用检查更新须从其配置的本机服务得到高于当前版本且 x64 匹配的 0.3.12 清单；“已是最新”不得掩盖无发布包、离线或鉴权错误。发现新版后才能进入下载。
+2026-10-06 / d9b447c：TC-107 确认在线清单和下载包为 0.3.12/x64，隔离旧版升级/故障回退通过。生产 /Applications/Token.app 仍 0.3.11，由用户自行点击更新。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="225" customHeight="1">
       <x:c r="A28" s="104" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-023</x:t>
@@ -6000,10 +5999,8 @@
           <x:t xml:space="preserve">M5（计划）</x:t>
         </x:is>
       </x:c>
-      <x:c r="E28" s="104" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">部分验证；点击前可放弃、点击后下载至安装不可取消为当前决议，真实双 DMG 隔离升级与双路径五故障回退通过；全阶段无取消 UI/系统目录/生产数据待验</x:t>
-        </x:is>
+      <x:c r="E28" s="104" t="str">
+        <x:v>0.3.11→0.3.12 隔离安装自动替换/重启及故障回退通过；实际生产安装待用户手动验收</x:v>
       </x:c>
       <x:c r="F28" s="104" t="str">
         <x:v>DEV-025、DEV-061</x:v>
@@ -6023,7 +6020,8 @@
 2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
 2026-10-04 用户最新决议（覆盖前述安装前/安装中界限）：点击“开始升级”前可退出或放弃；点击后下载、校验、交接、安装直到成功或失败自动回退，均没有中断取消动作。正常成功旧版退出、原位替换、新版启动；挂载、空间、替换、启动、健康故障自动恢复旧版并清理，保留用户数据/受信状态。本轮不交付独立取消控制窗口、取消协议、按阶段取消或取消用 journal；原设计和旧测试文字只作历史备选。 当前隔离成功/五故障自动恢复证据继续有效；未知的系统目录、真实满盘/断电与目标 Mac 不升为通过。
 2026-10-04 TC-095 负责当前 Mac 真实安装/更新故障恢复与数据保留的人工发布验收；TC-076 隔离自动故障证据继续有效，不替代系统位置和现有用户数据保护。
-0.3.12 增量：先以真实 0.3.11 DMG 复制到隔离目录，在应用内发现、下载、摘要校验、原位替换及重启 0.3.12；失败保留可用旧版和测试数据。生产 /Applications/Token.app 的点击升级由用户自行执行，实际安装结果待用户手动验收，不由隔离链路代证。</x:v>
+0.3.12 增量：先以真实 0.3.11 DMG 复制到隔离目录，在应用内发现、下载、摘要校验、原位替换及重启 0.3.12；失败保留可用旧版和测试数据。生产 /Applications/Token.app 的点击升级由用户自行执行，实际安装结果待用户手动验收，不由隔离链路代证。
+2026-10-06 / d9b447c：真实 0.3.11 DMG 隔离副本升级及五种 helper 故障回退、重试通过；不触碰生产 App。当前 /Applications/Token.app 仍 0.3.11，TC-107 用户实装子范围未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="62" customHeight="1">
@@ -7195,7 +7193,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="55" ht="266.25" customHeight="1">
+    <x:row r="55" ht="225" customHeight="1">
       <x:c r="A55" s="107" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -7210,7 +7208,7 @@
         <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
       <x:c r="E55" s="107" t="str">
-        <x:v>当前 Mac 合成自动验收通过；实际安装/交付另验</x:v>
+        <x:v>0.3.12 打包 E2E 通过；最终隔离性能命令进行中，生产 App 实装待用户核验</x:v>
       </x:c>
       <x:c r="F55" s="107" t="str">
         <x:v>DEV-059、DEV-062</x:v>
@@ -7220,10 +7218,11 @@
       </x:c>
       <x:c r="H55" s="107" t="str">
         <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。
-0.3.12 增量：以最终 0.3.12 候选可执行文件的隔离安装副本及同环境无正文数据复验 1180/700px、至少 20 次冷热切换反馈 P95≤150ms、长报表 10 秒帧间隔 P95≤32ms 且无≥200ms 停顿；记录内容可交互 P50/P95。生产 /Applications 新版切页由用户升级后手动验收，不能用源码或目录包合成指标代证。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="266.25" customHeight="1">
+0.3.12 增量：以最终 0.3.12 候选可执行文件的隔离安装副本及同环境无正文数据复验 1180/700px、至少 20 次冷热切换反馈 P95≤150ms、长报表 10 秒帧间隔 P95≤32ms 且无≥200ms 停顿；记录内容可交互 P50/P95。生产 /Applications 新版切页由用户升级后手动验收，不能用源码或目录包合成指标代证。
+0.3.12 / d9b447c：完整门禁与打包 E2E 通过；TC-108 隔离性能复验进行中。性能 JSON 当前样本 35,000 事实、六方向冷热每场景 20 次，最高反馈 P95 54.3ms；10 秒滚动两宽度 P95 18.1/18.5ms、无 ≥200ms 长任务。此为仍运行批次的已写样本，尚不把 TC-108 整项标通过；生产 App 仍 0.3.11。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="225" customHeight="1">
       <x:c r="A56" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -7238,7 +7237,7 @@
         <x:v>0.3.12 当前 Mac 实装修复候选</x:v>
       </x:c>
       <x:c r="E56" s="104" t="str">
-        <x:v>已实现；当前 Mac 合成自动范围通过，实装交付待验</x:v>
+        <x:v>0.3.12 打包 E2E 对缓存切页通过；隔离性能命令进行中，用户生产实装待验</x:v>
       </x:c>
       <x:c r="F56" s="104" t="str">
         <x:v>DEV-060、DEV-062</x:v>
@@ -7248,7 +7247,8 @@
       </x:c>
       <x:c r="H56" s="104" t="str">
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：共享缓存按登录用户/角色/完整查询键复用；五分钟到期刷新，手动、筛选及数据修订即时查询；旧值失败提示、跨账号隔离、明细/CSV 同授权快照。TC-105/106 单编号和完整门禁通过；当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。
-0.3.12 增量：隔离安装副本与用户手动升级后的生产新版，在同账号、同授权及筛选下概览↔报表切回立即显示缓存结果，不反复出现首次加载、重复发查询或重置五分钟计时；手动/筛选/数据变更及失败状态沿用原合同。旧 0.3.11 实装出现每次加载的用户反馈尚待新版实测。</x:v>
+0.3.12 增量：隔离安装副本与用户手动升级后的生产新版，在同账号、同授权及筛选下概览↔报表切回立即显示缓存结果，不反复出现首次加载、重复发查询或重置五分钟计时；手动/筛选/数据变更及失败状态沿用原合同。旧 0.3.11 实装出现每次加载的用户反馈尚待新版实测。
+0.3.12 / d9b447c：完整门禁及打包 E2E 已覆盖 TC-108 缓存命中不回闪/不重复请求；TC-108 附加的性能集成正在重测，既有 2e5ee34 结果不替代最终运行。用户仍须自行升级生产 App 并手动确认同筛选切页。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9611,7 +9611,7 @@
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：缓存成功结果与待完成查询，按账号/角色/查询键隔离；五分钟边界、事实修订失效、登出清理与迟到响应代次控制；失败保留匹配旧值并提示未更新。开发侧 npm run test:gate：106 入口、107/107 单元、57/57 Electron；TC-105/106、关联 TC-079/104、性能 TC-102/103 定向通过；打包 usage-refresh 2/2。当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" ht="195" customHeight="1">
+    <x:row r="66" ht="262.5" customHeight="1">
       <x:c r="A66" s="104" t="str">
         <x:v>DEV-061</x:v>
       </x:c>
@@ -9628,13 +9628,13 @@
         <x:v>package.json；package-lock.json；本机未签名 x64 DMG；scripts/publish-update.mjs；更新服务 manifest、UpdateClient/安装 helper 及打包回归（按定位结果修改）</x:v>
       </x:c>
       <x:c r="F66" s="104" t="str">
-        <x:v>已规划；待代码、制品及实装验证</x:v>
+        <x:v>代码/候选/本机服务发布及隔离旧版升级通过；生产安装由用户手动验收</x:v>
       </x:c>
       <x:c r="G66" s="104" t="str">
-        <x:v>只读核当前 /Applications 0.3.11 与所连本机服务配置；候选版升至 0.3.12，固定代码、DMG 大小/SHA-256，发布到当前应用连接的本机更新服务并核在线清单/版本/架构/鉴权。以真实 0.3.11 DMG 复制到隔离安装目录验证应用内发现→下载→替换→重启及故障回退。开发不得替用户升级生产 /Applications/Token.app；用户自行点击更新并手动验收。不得读取或提交生产数据库/密钥。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="195" customHeight="1">
+        <x:v>d9b447cc7cf210545023f6403d2d5f009cf6699b；0.3.12 x64 DMG 142,585,554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。npm run test:gate：108 用例入口、108 单元、58 Electron；打包 Electron 58/58。TC-107 在线授权清单与完整包下载 SHA 核验、真实 0.3.11 DMG 隔离升级、五种故障回退及再次升级通过。本机服务已发布 0.3.12/x64。生产 /Applications/Token.app 仍 0.3.11，待用户自行点击更新验收。首次 helper 重试验收曾失败并撤回清单至 0.3.7；d9b447c 修复重启导航后重测通过并重新发布。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="262.5" customHeight="1">
       <x:c r="A67" s="104" t="str">
         <x:v>DEV-062</x:v>
       </x:c>
@@ -9651,10 +9651,10 @@
         <x:v>src/renderer/usage-cache.ts、overview.tsx、report.tsx、index.tsx；src/main/report.ts；独立实装性能/缓存核验脚本与按编号入口（依实际根因定稿）</x:v>
       </x:c>
       <x:c r="F67" s="104" t="str">
-        <x:v>已规划；待代码、制品及实装验证</x:v>
+        <x:v>TC-108 打包 E2E 通过；最终隔离性能集成进行中；生产新版切页由用户手动验收</x:v>
       </x:c>
       <x:c r="G67" s="104" t="str">
-        <x:v>以最终 0.3.12 可执行文件的隔离安装副本复现同筛选往返与 loading 问题；若仍触发查询/回闪，定位 actor/查询键、缓存生命周期和 IPC/渲染瓶颈并修复。以临时 userData 和无正文合成空库/35,000 事实测 1180/700px 冷热至少 20 次、10 秒长报表；生产 /Applications 新版由用户自行升级后手动确认切页表现。保留旧版本样本与失败记录，禁止测试写生产用户数据。</x:v>
+        <x:v>d9b447c 的 npm run test:gate 与 npm run test:e2e:packaged 均通过（108 入口、108 单元、58 Electron；打包 58/58）。35,000 条合成事实的 TC-108 性能复验当前文件显示最高反馈 P95 54.3ms、滚动 P95 18.1/18.5ms、≥200ms 长任务 0；开发报告该 TC-108 命令仍运行中，等待最终退出码/结果后再判通过。真实生产 App 未升级。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -16985,7 +16985,7 @@
         <x:v>当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。</x:v>
       </x:c>
     </x:row>
-    <x:row r="112" ht="225" customHeight="1">
+    <x:row r="112" ht="262.5" customHeight="1">
       <x:c r="A112" s="104" t="str">
         <x:v>TC-107</x:v>
       </x:c>
@@ -17008,25 +17008,25 @@
         <x:v>隔离旧版及用户随后操作的生产旧版均应发现 0.3.12；不把未发布/离线/拒权写成“已是最新”。隔离升级无 Finder 拖拽，替换后 0.3.12 重启，合成数据保留；故障回退旧版并清理。生产安装仅在用户自行点击后依据脱敏版本、启动、受信状态和既有用量核验，不由开发或隔离结果代替。</x:v>
       </x:c>
       <x:c r="H112" s="104" t="str">
-        <x:v>已规划；入口待注册，实际安装与动态验收未执行</x:v>
+        <x:v>TC-107 隔离更新/发布自动子范围通过；生产 /Applications 安装由用户自行点击更新，尚待手动验收</x:v>
       </x:c>
       <x:c r="I112" s="104" t="str">
-        <x:v>2026-10-06：仅核到 /Applications/Token.app 和 package.json 均为 0.3.11；用户报告旧版切页重复加载且检查更新称最新。0.3.12 尚无固定候选、在线清单、实装或动态通过证据。</x:v>
+        <x:v>固定提交 d9b447cc7cf210545023f6403d2d5f009cf6699b。开发侧报告：真实 0.3.11 DMG 隔离副本从旧版 UI 检查、下载、校验、替换、重启通过；五种 helper 故障回退、再次升级通过；当前 App 所连内置服务在线清单及完整下载大小/SHA 核验通过。本次只读核 /Applications/Token.app 仍为 0.3.11；不表示生产升级已执行。</x:v>
       </x:c>
       <x:c r="J112" s="104" t="str">
-        <x:v>npm run test:case -- TC-107（计划独立入口；隔离自动子范围与用户实装人工证据分别记录）</x:v>
+        <x:v>TOKEN_TC107_OLD_DMG=&lt;真实0.3.11 DMG&gt; TOKEN_TC107_OLD_SHA256=&lt;旧包SHA&gt; TOKEN_TC107_NEW_DMG=&lt;0.3.12 DMG&gt; TOKEN_TC107_NEW_SHA256=7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74 TOKEN_TC107_SERVER_DIR=&lt;当前 App 所连内置服务目录&gt; npm run test:case -- TC-107</x:v>
       </x:c>
       <x:c r="K112" s="104" t="str">
-        <x:v>计划在 scripts/test-cases.mjs 分配独立人工入口；实装性能脚本须使用当前已安装可执行文件，不能只跑源码构建。</x:v>
+        <x:v>scripts/test-cases.mjs 将 TC-107 绑定 scripts/verify-0312-release.mjs 与 tests/next-update.test.ts；脚本读取本机服务凭据但不输出/保存密钥，以临时 userData 和可写安装副本调用 TC-076 成功、五故障回退与重试链路。</x:v>
       </x:c>
       <x:c r="L112" s="104" t="str">
-        <x:v>当前 Mac；隔离合成测试只写临时 userData/SQLite；实际安装步骤仅留脱敏摘要、版本/制品校验与可见结果。</x:v>
+        <x:v>开发侧当前 Mac x64；固定提交 d9b447c；服务在线接口与完整安装包下载 SHA 核对；真实 0.3.11 DMG 到独立临时安装目录；不改生产 /Applications 或 userData。</x:v>
       </x:c>
       <x:c r="M112" s="104" t="str">
-        <x:v>旧 0.3.11 实装症状与 2e5ee34 源码合成通过可同时成立；不得以源码测试推断 0.3.12 实装已通过。生产数据不复制入库。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="113" ht="225" customHeight="1">
+        <x:v>隔离自动子范围通过；生产 App 仍 0.3.11，由用户自行点击更新并人工验收。生产安装/用户数据连续性未有本轮证据，签名公证与异机分发不在本用例结论内。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="262.5" customHeight="1">
       <x:c r="A113" s="104" t="str">
         <x:v>TC-108</x:v>
       </x:c>
@@ -17049,22 +17049,22 @@
         <x:v>隔离副本与用户实装新版同键切回均立即显示已授权缓存，不反复出现首次加载或重复用量查询；筛选/手动/数据变化即时更新。隔离性能每场景反馈 P95≤150ms；内容 P50/P95 留基线；双窗口长报表帧间隔 P95≤32ms、无≥200ms 停顿；旧响应与跨用户隔离、未知≠零不退化。用户实装确认前不宣称生产体验完成。</x:v>
       </x:c>
       <x:c r="H113" s="104" t="str">
-        <x:v>已规划；入口待注册，实际安装与动态验收未执行</x:v>
+        <x:v>TC-108 页面缓存打包 E2E 通过；隔离性能命令进行中；生产新版切页待用户手动验收</x:v>
       </x:c>
       <x:c r="I113" s="104" t="str">
-        <x:v>2026-10-06：仅核到 /Applications/Token.app 和 package.json 均为 0.3.11；用户报告旧版切页重复加载且检查更新称最新。0.3.12 尚无固定候选、在线清单、实装或动态通过证据。</x:v>
+        <x:v>d9b447c 的 test:gate 与打包 E2E 58/58 均通过，TC-108 页面断言覆盖切页缓存命中无加载回闪/重复请求。性能集成 JSON 当前批次：35,000 条事实、1180/700px 六方向冷/热各 20 次，反馈 P95 最高 54.3ms；内容时间作为诊断记录（最高 P95 约 871ms）；10 秒滚动 P95 18.1/18.5ms、≥200ms 长任务 0。开发报告最终 TC-108 性能命令仍运行中，待结果确认后更新整项状态。</x:v>
       </x:c>
       <x:c r="J113" s="104" t="str">
-        <x:v>npm run test:case -- TC-108（计划独立入口；隔离性能与用户实装人工证据分别记录）</x:v>
+        <x:v>TOKEN_TC108_ASAR_SHA256=3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b npm run test:case -- TC-108</x:v>
       </x:c>
       <x:c r="K113" s="104" t="str">
-        <x:v>计划在 scripts/test-cases.mjs 分配独立人工入口；实装性能脚本须使用当前已安装可执行文件，不能只跑源码构建。</x:v>
+        <x:v>scripts/test-cases.mjs 绑定 tests/e2e/usage-refresh.spec.ts 的 TC-108 与 scripts/verify-0312-navigation.mjs；后者校验 0.3.12 app.asar 哈希，复制至临时安装目录和 userData 后执行 measure-navigation。</x:v>
       </x:c>
       <x:c r="L113" s="104" t="str">
-        <x:v>当前 Mac；隔离合成测试只写临时 userData/SQLite；实际安装步骤仅留脱敏摘要、版本/制品校验与可见结果。</x:v>
+        <x:v>当前 Mac x64；隔离临时 userData；35,000 条无正文合成事实；1180/700px；冷/热各 20 次及双窗口 10 秒滚动；原始 JSON 留在 Git 忽略 test-results/，仅提交脱敏汇总。</x:v>
       </x:c>
       <x:c r="M113" s="104" t="str">
-        <x:v>旧 0.3.11 实装症状与 2e5ee34 源码合成通过可同时成立；不得以源码测试推断 0.3.12 实装已通过。生产数据不复制入库。</x:v>
+        <x:v>打包 E2E 子范围通过；性能集成结果未最终确认；实际生产 App 仍 0.3.11，待用户自行升级并人工确认。性能样本不代表生产数据；未知覆盖不写作真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17922,7 +17922,7 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="255" customHeight="1">
+    <x:row r="19" ht="277.5" customHeight="1">
       <x:c r="A19" s="104" t="str">
         <x:v>VER-014</x:v>
       </x:c>
@@ -17942,19 +17942,19 @@
         <x:v>DEV-024、DEV-025、DEV-059、DEV-060、DEV-061、DEV-062</x:v>
       </x:c>
       <x:c r="G19" s="104" t="str">
-        <x:v>TC-105/106 合成自动已有证据；新增 TC-107/108 实装/性能待注册与执行；回归 TC-034–036/076/102–104</x:v>
+        <x:v>TC-107 隔离发布/升级自动子范围通过；TC-108 打包 E2E 通过、性能复验中；生产 App 更新待用户手动验收</x:v>
       </x:c>
       <x:c r="H19" s="104" t="str">
-        <x:v>2e5ee34 缓存功能已编码且合成自动通过；当前 /Applications/Token.app 与 package.json 仍为 0.3.11。0.3.12 版本、真实 DMG、本机更新服务发布、隔离旧版 UI 升级及新版切页/性能均待实施。生产 App 由用户自行点击更新与手动验收。</x:v>
+        <x:v>0.3.12 x64 已构建并发布到当前 App 所连本机更新服务；TC-107 在线清单/完整包 SHA 核验、真实 0.3.11 DMG 隔离升级、五种 helper 故障回退和重试通过。d9b447c 上 108 用例入口、108 单元、58 Electron 完整门禁通过，打包 Electron 58/58。TC-108 页面 E2E 通过，附加隔离性能命令仍在运行。首次 TC-107 helper 重试验收失败后清单已临时撤回 0.3.7；修复重启导航后复验并重新发布 0.3.12。</x:v>
       </x:c>
       <x:c r="I19" s="104" t="str">
-        <x:v>规划中：0.3.12 尚未固定或发布；TC-107/108 隔离与用户实装均无动态通过证据。VER-014 完整交付未完成。</x:v>
+        <x:v>服务已发布，候选与隔离升级验证通过；TC-108 性能最终结果待补。生产 /Applications/Token.app 仍 0.3.11，用户尚未自行点击升级和手动验收；VER-014 未交付。</x:v>
       </x:c>
       <x:c r="J19" s="104" t="str">
-        <x:v>2026-10-06 只读核 /Applications/Token.app Info.plist 与 package.json 均为 0.3.11。用户报告旧实装切页加载/卡顿、设置称最新；2e5ee34 的 106 入口/107 单元/57 Electron 与打包定向 2/2 仅证明合成范围，不证明旧安装含该实现。0.3.12 待记录代码、DMG 大小/SHA-256、在线 manifest、TC-107/108、目标安装与性能样本。</x:v>
+        <x:v>冻结产品提交 d9b447cc7cf210545023f6403d2d5f009cf6699b，package.json 0.3.12，x64 DMG 142585554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。TC-107 已通过；test:gate 108 入口/108 单元/58 Electron，packaged 58/58。TC-108 性能命令进行中，当前样本反馈 P95≤54.3ms，滚动 18.1/18.5ms、无≥200ms 长任务。线上 latest 0.3.12/x64、包大小/SHA 与本机落盘 DMG 核一致。</x:v>
       </x:c>
       <x:c r="K19" s="104" t="str">
-        <x:v>“已是最新”也可能表示本机服务尚无新版清单，需核在线响应与鉴权后定位。开发仅发布到当前 App 所连本机服务，不替用户升级生产 /Applications。用户自行升级并手动验收前，不标实装完成；生产数据只留脱敏摘要。签名公证及异机外部分发仍属独立门槛。</x:v>
+        <x:v>生产 /Applications/Token.app 只读仍为 0.3.11；开发未替用户升级。用户需自行在应用内点击更新，并人工核新版、启动、受信状态、既有用量和切页体验后，才能更新交付状态。外部分发签名公证/异机未验；首轮 TC-107 失败及服务清单撤回历史保留。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record final TC-108 performance acceptance
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="Rcc0f0f611d124764"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Re701dbfbcaee41e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Re09c970c4cfa423f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="R22ae91b5014949b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R25a67b63f04443b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R4de58940a8ab491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rff15c95733924b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra7003df80eda41c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re0dd1a96eb96465e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R419d1a945d2b4148"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4889,7 +4889,7 @@
         <x:v>TC-107 隔离自动安装/回退通过；实际 /Applications 安装由用户手动验收，未交付。</x:v>
       </x:c>
     </x:row>
-    <x:row r="115" ht="108.75" customHeight="1">
+    <x:row r="115" ht="112.5" customHeight="1">
       <x:c r="A115" s="104" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -4909,10 +4909,10 @@
         <x:v>已安装 0.3.12 缓存切页与性能</x:v>
       </x:c>
       <x:c r="G115" s="104" t="str">
-        <x:v>TC-108 打包 E2E 通过；性能集成命令进行中，生产新版性能待用户验收。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116" ht="108.75" customHeight="1">
+        <x:v>0.3.12 TC-108 打包 E2E 与隔离性能自动范围通过；生产 App 切页待用户手动验收。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="112.5" customHeight="1">
       <x:c r="A116" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -4932,7 +4932,7 @@
         <x:v>已安装 0.3.12 缓存切页与性能</x:v>
       </x:c>
       <x:c r="G116" s="104" t="str">
-        <x:v>TC-108 缓存 E2E 通过；性能集成进行中，生产实装切页待用户确认。</x:v>
+        <x:v>0.3.12 缓存命中 E2E 与隔离性能自动范围通过；生产账号实装行为待用户手动验收。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7193,7 +7193,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="55" ht="225" customHeight="1">
+    <x:row r="55" ht="232.5" customHeight="1">
       <x:c r="A55" s="107" t="str">
         <x:v>REQ-050</x:v>
       </x:c>
@@ -7208,7 +7208,7 @@
         <x:v>0.3.11 页面性能增量（实施中）</x:v>
       </x:c>
       <x:c r="E55" s="107" t="str">
-        <x:v>0.3.12 打包 E2E 通过；最终隔离性能命令进行中，生产 App 实装待用户核验</x:v>
+        <x:v>0.3.12 隔离性能复验通过；实际生产 App 性能待用户自行升级后核验</x:v>
       </x:c>
       <x:c r="F55" s="107" t="str">
         <x:v>DEV-059、DEV-062</x:v>
@@ -7219,10 +7219,11 @@
       <x:c r="H55" s="107" t="str">
         <x:v>aa3c510 在 b8bba1d 缓存修复基础上补齐冷/热六方向、滚后操作及双用户链路。空库/35,000 无正文合成事实、1180/700px：冷/热各 24 组×20 次，反馈 P95 最高 22.1/18.7ms；10 秒滚动 P95 最高 18.6ms、最大 18.8ms。源码和打包三项定向 E2E 各 3/3；当前 Mac 合成自动验收通过。原始样本见 outputs/20261006-token-navigation-performance/README.md，真实安装另验。
 0.3.12 增量：以最终 0.3.12 候选可执行文件的隔离安装副本及同环境无正文数据复验 1180/700px、至少 20 次冷热切换反馈 P95≤150ms、长报表 10 秒帧间隔 P95≤32ms 且无≥200ms 停顿；记录内容可交互 P50/P95。生产 /Applications 新版切页由用户升级后手动验收，不能用源码或目录包合成指标代证。
-0.3.12 / d9b447c：完整门禁与打包 E2E 通过；TC-108 隔离性能复验进行中。性能 JSON 当前样本 35,000 事实、六方向冷热每场景 20 次，最高反馈 P95 54.3ms；10 秒滚动两宽度 P95 18.1/18.5ms、无 ≥200ms 长任务。此为仍运行批次的已写样本，尚不把 TC-108 整项标通过；生产 App 仍 0.3.11。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="225" customHeight="1">
+0.3.12 / d9b447c：完整门禁与打包 E2E 通过；TC-108 隔离性能复验进行中。性能 JSON 当前样本 35,000 事实、六方向冷热每场景 20 次，最高反馈 P95 54.3ms；10 秒滚动两宽度 P95 18.1/18.5ms、无 ≥200ms 长任务。此为仍运行批次的已写样本，尚不把 TC-108 整项标通过；生产 App 仍 0.3.11。
+TC-108 最终隔离性能复验已通过；样本、冷/热指标与实装边界见验收记录。生产 App 仍为 0.3.11。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="232.5" customHeight="1">
       <x:c r="A56" s="104" t="str">
         <x:v>REQ-051</x:v>
       </x:c>
@@ -7237,7 +7238,7 @@
         <x:v>0.3.12 当前 Mac 实装修复候选</x:v>
       </x:c>
       <x:c r="E56" s="104" t="str">
-        <x:v>0.3.12 打包 E2E 对缓存切页通过；隔离性能命令进行中，用户生产实装待验</x:v>
+        <x:v>0.3.12 隔离缓存切页/性能自动验收通过；实际生产新版待用户手动验收</x:v>
       </x:c>
       <x:c r="F56" s="104" t="str">
         <x:v>DEV-060、DEV-062</x:v>
@@ -7248,7 +7249,8 @@
       <x:c r="H56" s="104" t="str">
         <x:v>2e5ee34d6c77b4b1eb2d3442b231c4e54d48eced：共享缓存按登录用户/角色/完整查询键复用；五分钟到期刷新，手动、筛选及数据修订即时查询；旧值失败提示、跨账号隔离、明细/CSV 同授权快照。TC-105/106 单编号和完整门禁通过；当前 Mac 隔离无正文合成数据自动范围通过；实际系统目录安装、生产数据、正式版本号、制品哈希与外部分发未验。覆盖完整性仍未知，已确认小计 0 不等于完整真零。
 0.3.12 增量：隔离安装副本与用户手动升级后的生产新版，在同账号、同授权及筛选下概览↔报表切回立即显示缓存结果，不反复出现首次加载、重复发查询或重置五分钟计时；手动/筛选/数据变更及失败状态沿用原合同。旧 0.3.11 实装出现每次加载的用户反馈尚待新版实测。
-0.3.12 / d9b447c：完整门禁及打包 E2E 已覆盖 TC-108 缓存命中不回闪/不重复请求；TC-108 附加的性能集成正在重测，既有 2e5ee34 结果不替代最终运行。用户仍须自行升级生产 App 并手动确认同筛选切页。</x:v>
+0.3.12 / d9b447c：完整门禁及打包 E2E 已覆盖 TC-108 缓存命中不回闪/不重复请求；TC-108 附加的性能集成正在重测，既有 2e5ee34 结果不替代最终运行。用户仍须自行升级生产 App 并手动确认同筛选切页。
+TC-108 的最终 0.3.12 隔离性能通过；同版本打包 E2E 核缓存命中无加载回闪/重复请求。用户仍需自行升级生产 App 并手动确认真实筛选切页。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9634,7 +9636,7 @@
         <x:v>d9b447cc7cf210545023f6403d2d5f009cf6699b；0.3.12 x64 DMG 142,585,554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。npm run test:gate：108 用例入口、108 单元、58 Electron；打包 Electron 58/58。TC-107 在线授权清单与完整包下载 SHA 核验、真实 0.3.11 DMG 隔离升级、五种故障回退及再次升级通过。本机服务已发布 0.3.12/x64。生产 /Applications/Token.app 仍 0.3.11，待用户自行点击更新验收。首次 helper 重试验收曾失败并撤回清单至 0.3.7；d9b447c 修复重启导航后重测通过并重新发布。</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="262.5" customHeight="1">
+    <x:row r="67" ht="255" customHeight="1">
       <x:c r="A67" s="104" t="str">
         <x:v>DEV-062</x:v>
       </x:c>
@@ -9651,10 +9653,10 @@
         <x:v>src/renderer/usage-cache.ts、overview.tsx、report.tsx、index.tsx；src/main/report.ts；独立实装性能/缓存核验脚本与按编号入口（依实际根因定稿）</x:v>
       </x:c>
       <x:c r="F67" s="104" t="str">
-        <x:v>TC-108 打包 E2E 通过；最终隔离性能集成进行中；生产新版切页由用户手动验收</x:v>
+        <x:v>TC-108 打包 E2E 与隔离性能验证通过；生产新版切页由用户手动验收</x:v>
       </x:c>
       <x:c r="G67" s="104" t="str">
-        <x:v>d9b447c 的 npm run test:gate 与 npm run test:e2e:packaged 均通过（108 入口、108 单元、58 Electron；打包 58/58）。35,000 条合成事实的 TC-108 性能复验当前文件显示最高反馈 P95 54.3ms、滚动 P95 18.1/18.5ms、≥200ms 长任务 0；开发报告该 TC-108 命令仍运行中，等待最终退出码/结果后再判通过。真实生产 App 未升级。</x:v>
+        <x:v>d9b447c：test:gate 108 入口、108 单元、58 Electron 通过，packaged 58/58。2026-10-07 / d9b447c：首次 npm run test:case -- TC-108 因漏设 TOKEN_TC108_ASAR_SHA256，在输入校验处退出 1；Electron 子用例已通过，这不是产品失败。设置冻结 app.asar SHA-256 后重跑，整体退出 0。35,000 条无正文事实、1180/700px：热概览→报表反馈 P95 54.3/52.0ms、内容 P95 77.8/73.9ms；冷同向反馈 P95 47.8/46.9ms、内容 P95 59.7/56.7ms；10 秒滚动 601 帧，P95 17.5/17.5ms，最大 17.7/17.8ms，≥200ms 长任务 0。原始数值 JSON 留在开发工作树忽略的 test-results/performance-0.3.12.json，本工作簿只留脱敏汇总。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17026,7 +17028,7 @@
         <x:v>隔离自动子范围通过；生产 App 仍 0.3.11，由用户自行点击更新并人工验收。生产安装/用户数据连续性未有本轮证据，签名公证与异机分发不在本用例结论内。</x:v>
       </x:c>
     </x:row>
-    <x:row r="113" ht="262.5" customHeight="1">
+    <x:row r="113" ht="270" customHeight="1">
       <x:c r="A113" s="104" t="str">
         <x:v>TC-108</x:v>
       </x:c>
@@ -17049,22 +17051,22 @@
         <x:v>隔离副本与用户实装新版同键切回均立即显示已授权缓存，不反复出现首次加载或重复用量查询；筛选/手动/数据变化即时更新。隔离性能每场景反馈 P95≤150ms；内容 P50/P95 留基线；双窗口长报表帧间隔 P95≤32ms、无≥200ms 停顿；旧响应与跨用户隔离、未知≠零不退化。用户实装确认前不宣称生产体验完成。</x:v>
       </x:c>
       <x:c r="H113" s="104" t="str">
-        <x:v>TC-108 页面缓存打包 E2E 通过；隔离性能命令进行中；生产新版切页待用户手动验收</x:v>
+        <x:v>0.3.12 隔离打包 E2E 与性能自动范围通过；生产新版切页体验待用户手动验收</x:v>
       </x:c>
       <x:c r="I113" s="104" t="str">
-        <x:v>d9b447c 的 test:gate 与打包 E2E 58/58 均通过，TC-108 页面断言覆盖切页缓存命中无加载回闪/重复请求。性能集成 JSON 当前批次：35,000 条事实、1180/700px 六方向冷/热各 20 次，反馈 P95 最高 54.3ms；内容时间作为诊断记录（最高 P95 约 871ms）；10 秒滚动 P95 18.1/18.5ms、≥200ms 长任务 0。开发报告最终 TC-108 性能命令仍运行中，待结果确认后更新整项状态。</x:v>
+        <x:v>2026-10-07 / d9b447c：首次 npm run test:case -- TC-108 因漏设 TOKEN_TC108_ASAR_SHA256，在输入校验处退出 1；Electron 子用例已通过，这不是产品失败。设置冻结 app.asar SHA-256 后重跑，整体退出 0。35,000 条无正文事实、1180/700px：热概览→报表反馈 P95 54.3/52.0ms、内容 P95 77.8/73.9ms；冷同向反馈 P95 47.8/46.9ms、内容 P95 59.7/56.7ms；10 秒滚动 601 帧，P95 17.5/17.5ms，最大 17.7/17.8ms，≥200ms 长任务 0。原始数值 JSON 留在开发工作树忽略的 test-results/performance-0.3.12.json，本工作簿只留脱敏汇总。</x:v>
       </x:c>
       <x:c r="J113" s="104" t="str">
-        <x:v>TOKEN_TC108_ASAR_SHA256=3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b npm run test:case -- TC-108</x:v>
+        <x:v>TOKEN_TC108_ASAR_SHA256=3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b npm run test:case -- TC-108；退出码 0</x:v>
       </x:c>
       <x:c r="K113" s="104" t="str">
-        <x:v>scripts/test-cases.mjs 绑定 tests/e2e/usage-refresh.spec.ts 的 TC-108 与 scripts/verify-0312-navigation.mjs；后者校验 0.3.12 app.asar 哈希，复制至临时安装目录和 userData 后执行 measure-navigation。</x:v>
+        <x:v>scripts/test-cases.mjs 绑定 tests/e2e/usage-refresh.spec.ts 与 scripts/verify-0312-navigation.mjs；脚本核冻结 app.asar 后复制到临时安装目录，以独立 userData 运行性能脚本。</x:v>
       </x:c>
       <x:c r="L113" s="104" t="str">
         <x:v>当前 Mac x64；隔离临时 userData；35,000 条无正文合成事实；1180/700px；冷/热各 20 次及双窗口 10 秒滚动；原始 JSON 留在 Git 忽略 test-results/，仅提交脱敏汇总。</x:v>
       </x:c>
       <x:c r="M113" s="104" t="str">
-        <x:v>打包 E2E 子范围通过；性能集成结果未最终确认；实际生产 App 仍 0.3.11，待用户自行升级并人工确认。性能样本不代表生产数据；未知覆盖不写作真零。</x:v>
+        <x:v>0.3.12 隔离自动性能范围通过；实际生产 App 仍 0.3.11，用户自行升级并手动确认同筛选切页前不宣称生产体验完成。样本为合成数据；未知覆盖不写作真零。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -17922,7 +17924,7 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="277.5" customHeight="1">
+    <x:row r="19" ht="307.5" customHeight="1">
       <x:c r="A19" s="104" t="str">
         <x:v>VER-014</x:v>
       </x:c>
@@ -17942,19 +17944,19 @@
         <x:v>DEV-024、DEV-025、DEV-059、DEV-060、DEV-061、DEV-062</x:v>
       </x:c>
       <x:c r="G19" s="104" t="str">
-        <x:v>TC-107 隔离发布/升级自动子范围通过；TC-108 打包 E2E 通过、性能复验中；生产 App 更新待用户手动验收</x:v>
+        <x:v>TC-107 隔离服务/升级通过；TC-108 打包 E2E 与隔离性能通过；生产 App 更新待用户手动验收</x:v>
       </x:c>
       <x:c r="H19" s="104" t="str">
-        <x:v>0.3.12 x64 已构建并发布到当前 App 所连本机更新服务；TC-107 在线清单/完整包 SHA 核验、真实 0.3.11 DMG 隔离升级、五种 helper 故障回退和重试通过。d9b447c 上 108 用例入口、108 单元、58 Electron 完整门禁通过，打包 Electron 58/58。TC-108 页面 E2E 通过，附加隔离性能命令仍在运行。首次 TC-107 helper 重试验收失败后清单已临时撤回 0.3.7；修复重启导航后复验并重新发布 0.3.12。</x:v>
+        <x:v>固定提交 d9b447c；TC-107 服务清单/真实 0.3.11 DMG 隔离升级及故障回退通过，TC-108 打包 E2E 与隔离性能通过。完整门禁 108 入口、108 单元、58 Electron，打包 58/58。2026-10-07：TC-108 首轮漏设 app.asar 固定摘要环境变量，在输入校验退出 1，页面子用例已通过；补齐后完整命令退出 0。35,000 条合成事实热/冷反馈 P95 最高 54.3ms，滚动 P95 17.5ms、无 ≥200ms 长任务。</x:v>
       </x:c>
       <x:c r="I19" s="104" t="str">
-        <x:v>服务已发布，候选与隔离升级验证通过；TC-108 性能最终结果待补。生产 /Applications/Token.app 仍 0.3.11，用户尚未自行点击升级和手动验收；VER-014 未交付。</x:v>
+        <x:v>服务已发布，0.3.12 候选、TC-107 隔离升级及 TC-108 隔离性能自动范围通过；生产 /Applications/Token.app 仍 0.3.11，用户尚未自行点击升级和手动验收；VER-014 未交付。</x:v>
       </x:c>
       <x:c r="J19" s="104" t="str">
-        <x:v>冻结产品提交 d9b447cc7cf210545023f6403d2d5f009cf6699b，package.json 0.3.12，x64 DMG 142585554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。TC-107 已通过；test:gate 108 入口/108 单元/58 Electron，packaged 58/58。TC-108 性能命令进行中，当前样本反馈 P95≤54.3ms，滚动 18.1/18.5ms、无≥200ms 长任务。线上 latest 0.3.12/x64、包大小/SHA 与本机落盘 DMG 核一致。</x:v>
+        <x:v>冻结产品提交 d9b447cc7cf210545023f6403d2d5f009cf6699b；package.json 0.3.12；x64 DMG 142585554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。TC-107 已通过；test:gate 108 入口/108 单元/58 Electron，通过打包 E2E 58/58。TC-108 首次因漏设 TOKEN_TC108_ASAR_SHA256 在输入校验退出 1，Electron 页面子用例已通过；补齐冻结摘要后 npm run test:case -- TC-108 整体退出 0。35,000 条合成事实：热反馈 P95 54.3/52.0ms、内容 P95 77.8/73.9ms；冷反馈 P95 47.8/46.9ms、内容 P95 59.7/56.7ms；10 秒滚动 601 帧，P95 17.5/17.5ms、最大 17.7/17.8ms、≥200ms 长任务 0。首次退出属于调用参数缺失，不是产品失败。服务 latest 0.3.12/x64 与制品摘要一致。</x:v>
       </x:c>
       <x:c r="K19" s="104" t="str">
-        <x:v>生产 /Applications/Token.app 只读仍为 0.3.11；开发未替用户升级。用户需自行在应用内点击更新，并人工核新版、启动、受信状态、既有用量和切页体验后，才能更新交付状态。外部分发签名公证/异机未验；首轮 TC-107 失败及服务清单撤回历史保留。</x:v>
+        <x:v>生产 /Applications/Token.app 只读仍为 0.3.11；开发未替用户升级。用户需自行在应用内点击更新并人工核新版、启动、受信状态、既有用量和切页体验后，才能更新交付状态。外部分发签名公证/异机未验；首轮 TC-107 失败及服务清单撤回历史保留。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record 0.3.12 GitHub prerelease
</commit_message>
<xml_diff>
--- a/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
+++ b/outputs/20261002-token-docs/Token-需求开发测试追溯.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R4de58940a8ab491c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="Rff15c95733924b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="Ra7003df80eda41c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Re0dd1a96eb96465e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R419d1a945d2b4148"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯矩阵" sheetId="1" r:id="R7315fe86af444846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求" sheetId="2" r:id="R058956a3c8f84155"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="开发任务" sheetId="3" r:id="R9782e7c0e7584cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试用例" sheetId="4" r:id="Rae0091a0940f4c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本规划" sheetId="5" r:id="R627d3bb3bb654364"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -587,6 +587,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -3774,38 +3780,38 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="82" ht="337.5" customHeight="1">
-      <x:c r="A82" s="52" t="inlineStr">
+    <x:row r="82" ht="450" customHeight="1">
+      <x:c r="A82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-023</x:t>
         </x:is>
       </x:c>
-      <x:c r="B82" s="52" t="inlineStr">
+      <x:c r="B82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">应用内自动安装升级</x:t>
         </x:is>
       </x:c>
-      <x:c r="C82" s="52" t="inlineStr">
+      <x:c r="C82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-025</x:t>
         </x:is>
       </x:c>
-      <x:c r="D82" s="52" t="inlineStr">
+      <x:c r="D82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">受约束自动安装辅助进程与失败回滚</x:t>
         </x:is>
       </x:c>
-      <x:c r="E82" s="52" t="inlineStr">
+      <x:c r="E82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TC-076</x:t>
         </x:is>
       </x:c>
-      <x:c r="F82" s="52" t="inlineStr">
+      <x:c r="F82" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">实际打包 App 隔离自动升级</x:t>
         </x:is>
       </x:c>
-      <x:c r="G82" s="52" t="str">
+      <x:c r="G82" s="109" t="str">
         <x:v>真实 0.3.5→0.3.6 隔离自动成功；系统安装/故障待验
 2026-10-04 / 80e7f10→0eac84b：80e7f10 独立全命令最后状态文件竞态 exit 1；0eac84b 同包复跑 exit 0。真实 DMG 隔离成功、只读初始启动、五故障模块 hooks 回退与重试通过；真实系统目标/打包 helper/UI/安装中取消待验。
 2026-10-04 / 1961de3：TC-076 打包 helper 五故障隔离注入及最后重试独立 exit 0；系统目录、真实满盘/崩溃、安装中取消、签名公证异机仍待验。
@@ -3815,7 +3821,9 @@
 2026-10-04 用户当前决议（覆盖前述安装中取消历史目标）：安装前可放弃；开始执行应用替换/安装后不可取消；挂载、替换、重启或健康确认失败时自动恢复旧版和清理临时物，用户数据/凭证不得丢失。独立控制窗口、五阶段点击取消、替换后主动取消回滚不在本轮交付范围；下载阶段取消未核实，不声明已实现且不是本轮必需。 新包隔离升级及两层五故障回退动态子范围通过；完整系统/生产验收待补；历史取消设计保留备选。
 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2 TC-076 真实双 DMG 脚本 exit 0；范围与限制见测试用例 I/M 列。
 2026-10-04 最新用户决议：点击开始前可放弃；点击后下载/校验/交接/安装全程无取消，直到成功或失败自动恢复。独立窗口、取消协议/journal、分阶段点击取消不属本轮；旧隔离成功/五故障证据保留，系统/生产/目标 Mac 仍待验。
-46111d3：TC-076 前两次首次引导脚本假设失败、修订后第三次合成旧版链路 exit 0；真实双 DMG 故障本轮未执行，整项仍部分验证。</x:v>
+46111d3：TC-076 前两次首次引导脚本假设失败、修订后第三次合成旧版链路 exit 0；真实双 DMG 故障本轮未执行，整项仍部分验证。
+2026-10-07 / main f109abc：新 0.3.12 GitHub DMG 的真实旧/新包隔离 TC-076 成功升级、五种 helper 故障回退及重试由开发统筹报告通过；不覆盖系统目录、生产数据、真实故障或签名公证异机。
+GitHub 0.3.12 DMG 重新下载后 SHA-256 01b25b0b9fda31fd28862e612e0125c6743b84b182af0c4c2eea6fa6b34bb21a 与源资产一致。</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="135" customHeight="1">
@@ -14898,33 +14906,33 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="81" ht="200" customHeight="1">
-      <x:c r="A81" s="52" t="inlineStr">
+    <x:row r="81" ht="765" customHeight="1">
+      <x:c r="A81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TC-076</x:t>
         </x:is>
       </x:c>
-      <x:c r="B81" s="52" t="inlineStr">
+      <x:c r="B81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ-023</x:t>
         </x:is>
       </x:c>
-      <x:c r="C81" s="52" t="inlineStr">
+      <x:c r="C81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DEV-025</x:t>
         </x:is>
       </x:c>
-      <x:c r="D81" s="52" t="inlineStr">
+      <x:c r="D81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">实际打包 App 隔离自动升级</x:t>
         </x:is>
       </x:c>
-      <x:c r="E81" s="52" t="inlineStr">
+      <x:c r="E81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">打包应用/本机隔离</x:t>
         </x:is>
       </x:c>
-      <x:c r="F81" s="52" t="inlineStr">
+      <x:c r="F81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">独立临时数据库和用户数据目录中启动实际旧版 App，登录并扫描无正文合成 1280 Token；点击开始升级后从隔离更新服务检查、下载及校验新版 DMG，再由应用自动退出旧版、安装替换并启动实际新版。点击前退出或放弃，另注入磁盘不足、挂载/替换/重启失败；补测只读 DMG 按写权限自动选择 /Applications/Token.app 或 ~/Applications/Token.app，以及已有不可写系统安装。
 2026-10-04 / 80e7f10→0eac84b：当前新增只读旧 DMG 直接启动初始界面；隔离可写目录中用真实旧/新 DMG 与生产 installer 模块 hooks 注入挂载、ENOSPC、替换、启动、健康超时，逐故障核旧版实际运行/受信登录/1280 Token、备份/挂载/下载清理，再以真实 DMG 重试。
@@ -14932,7 +14940,7 @@
 2026-10-04 当前新增操作：点击开始前退出须保留旧版；点击开始后覆盖下载、校验、交接、安装直至成功/失败自动回退，不设计或点击中途取消控制。继续分别注入挂载、空间、替换、启动、健康故障核自动恢复旧版/数据、清理及重试；不新增五阶段取消正例。</x:t>
         </x:is>
       </x:c>
-      <x:c r="G81" s="52" t="inlineStr">
+      <x:c r="G81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">无需 Finder 拖拽；新版版本正确、受信登录和 1280 Token 用量延续；失败能恢复旧版/数据、清理备份/挂载/临时文件并可重试。未签名 safeStorage 如不能延续须明确重新登录恢复；只读 DMG 的 /Applications 可写/不可写两条目标选择均自动复制并重启；已有不可写系统安装须明确授权或报错，不能静默迁址。
 2026-10-04 / 80e7f10→0eac84b：每个注入故障须让 installer reject、旧版恢复且可启动、用户数据不变、临时物清理；最后 installer resolve、新版启动且受信登录/1280 Token 保留。一次性状态文件若仍存在才核 rollback/success。
@@ -14940,12 +14948,11 @@
 2026-10-04 最新预期：点击前放弃不触发升级；点击后全程没有可用中途取消，正常成功旧版退出/替换/新版启动，故障自动回退且用户数据和受信状态连续。此无取消边界仍须按真实打包 UI/服务检查；既有隔离五故障通过不代证系统目录/生产。</x:t>
         </x:is>
       </x:c>
-      <x:c r="H81" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">部分验证：当前新 DMG 隔离成功升级、installer/打包 helper 各五故障回退与重试通过；点击后全阶段无取消 UI、真实系统目录/生产数据与真实故障待验</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I81" s="68" t="str">
+      <x:c r="H81" s="109" t="str">
+        <x:v>部分验证：当前新 DMG 隔离成功升级、installer/打包 helper 各五故障回退与重试通过；点击后全阶段无取消 UI、真实系统目录/生产数据与真实故障待验
+2026-10-07：真实 0.3.11/0.3.12 DMG 的隔离 TC-076 升级与五种 helper 故障回退/重试通过；本轮只更新该隔离子范围，系统目录、生产数据库、真实故障与取消边界不因此通过。</x:v>
+      </x:c>
+      <x:c r="I81" s="109" t="str">
         <x:v>当前 1e70412：macOS 15.7.4 x86_64、Node v24.15.0；旧 DMG SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd，新候选 27aae018a895baff90c4d5de6af5a56eb62fb78db0a62342ff206f813fab1bff、142591767 字节；两包 hdiutil verify VALID。文档会话构建 0.3.6 目录包并独立运行真实模式 TC-076，退出码 0；旧 UI 下载、退出、替换/重启、受信登录、合成报表 1280 Token 通过。
 2026-10-03 仅完成计划；scripts/test-cases.mjs 尚无 TC-076，尚无新辅助进程、打包 App 自动升级执行或日志。既有 verify-local-upgrade.mjs 的外部 ditto 替换不满足本项。
 86a4b5b：文档会话在 macOS x64 独立执行 npm run test:case -- TC-076，退出码 0；pack:dir 生成 0.3.5 未签名 App，脚本复制该包并改 app.asar package.json 与 Info.plist 版本号为 0.3.4 充当旧版，合成 1280 Token/临时用户数据、隔离服务、DMG 检查下载、helper 自动退出/替换/启动、健康 success、helper 退出、受信登录和报表延续均通过。真实 0.3.4 或 0.3.0 旧二进制未作为 TC-076 旧版。
@@ -14953,33 +14960,34 @@
 508851a：TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。
 2026-10-04 用户决议：开始执行应用替换/安装后不可取消，安装前可放弃，失败自动恢复；原五阶段取消要求撤出本轮。新候选从干净 main 9af351a 构建，未签名 mac x64 DMG SHA-256 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2；需求会话报告 pack:dmg exit 0，文档会话独立重算 SHA-256 与 hdiutil verify VALID。新包成功/故障隔离动态子范围后续已测，详见本列最新证据，旧 d99d7af9 包证据不外推。
 2026-10-04 当前候选 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：需求会话在干净 main 9af351a 用真实旧 0.3.5/新 0.3.6 两个固定 SHA DMG 运行 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076，exit 0；覆盖旧 UI 自动退出、替换、新版启动、受信登录及合成 1280 Token，旧只读 DMG 首启/未确认重启；installer 模块及实际打包 helper 各自 mount/space/replace/launch/health 五故障隔离回退并重试成功。主工作区同候选 test:gate 为 94 入口、97/97 单元、43/43 Electron，打包 Electron 43/43，均 exit 0。文档会话未独立复跑动态测试；合成故障不等于真实满盘、断电、系统目录或生产数据。TC-079 日期反例此前重复 3/5、2/5 失败，仍待单独修复复测。
-2026-10-06 / 46111d3：开发会话 TC-076 前两次因旧脚本假设首次建账直达概览失败；修订 verify-auto-upgrade.mjs / verify-auto-upgrade-faults.mjs 等待并可跳过引导，第三次 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076 exit 0。隔离合成旧版（当前包改版本元数据）旧进程退出、原位替换、新版启动、受信登录及合成 1280 Token 保留，无 Finder 拖拽。文档会话只读核脚本差异，未复跑 TC-076；前两次失败保留。</x:v>
-      </x:c>
-      <x:c r="J81" s="52" t="inlineStr">
+2026-10-06 / 46111d3：开发会话 TC-076 前两次因旧脚本假设首次建账直达概览失败；修订 verify-auto-upgrade.mjs / verify-auto-upgrade-faults.mjs 等待并可跳过引导，第三次 TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076 exit 0。隔离合成旧版（当前包改版本元数据）旧进程退出、原位替换、新版启动、受信登录及合成 1280 Token 保留，无 Finder 拖拽。文档会话只读核脚本差异，未复跑 TC-076；前两次失败保留。
+2026-10-07 / main f109abc（产品代码 d9b447c）：开发统筹报告使用真实 0.3.11 与新 0.3.12 GitHub DMG 在隔离安装目录运行 TC-076；旧版 UI 自动升级通过，五种 helper 故障回退和重试通过。新 DMG 为 142585538 bytes、SHA-256 01b25b0b9fda31fd28862e612e0125c6743b84b182af0c4c2eea6fa6b34bb21a，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。执行日志和旧包摘要未随交接提供，重新下载后独立 SHA-256 回验通过；此证据仅属隔离范围。
+GitHub 资产下载回验补充：重新下载后复算 142585538 字节、SHA-256 01b25b0b9fda31fd28862e612e0125c6743b84b182af0c4c2eea6fa6b34bb21a，与发布源和远端 asset digest 一致。</x:v>
+      </x:c>
+      <x:c r="J81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">TOKEN_TC076_SKIP_BUILD=1 TOKEN_TC076_OLD_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.5.dmg TOKEN_TC076_OLD_SHA256=ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd TOKEN_TC076_NEW_DMG=/Users/lz/.codex/worktrees/m6-product/Token/Token-0.3.6.dmg TOKEN_TC076_NEW_SHA256=d99d7af9a67e35a92199335eebc5d1aaa5ece2c902a7898f4747847b3ec54a9c npm run test:case -- TC-076</x:t>
         </x:is>
       </x:c>
-      <x:c r="K81" s="52" t="inlineStr">
+      <x:c r="K81" s="109" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">scripts/test-cases.mjs：TC-076 integration 绑定 scripts/verify-auto-upgrade.mjs；给定 OLD_DMG/OLD_SHA256/NEW_DMG/NEW_SHA256 即验证真实旧/新 DMG；省略参数则为改版本元数据的合成旧版模式。
 2026-10-04 / 80e7f10→0eac84b：现另绑定 scripts/verify-auto-upgrade-faults.mjs；仅给出四个真实 DMG/摘要参数才运行真实制品故障路径；此脚本直接调用生产 installer 模块，非打包 helper 进程。
 1961de3 新增 integration scripts/verify-packaged-helper-faults.mjs；仅给定真实 OLD/NEW DMG+SHA 执行，NODE_OPTIONS 预加载限专用临时目录的打包 update-helper.cjs，五故障和最后重试逐项核。</x:t>
         </x:is>
       </x:c>
-      <x:c r="L81" s="68" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
+      <x:c r="L81" s="109" t="str">
+        <x:v>当前自动边界：真实 0.3.5 二进制从只读 DMG 复制至临时可写路径后升级；未从只读 DMG 直接启动，未安装到真实 /Applications 或 ~/Applications，未在打包态注入失败回滚；TC-036 的回滚仅合成单元。
 0.3.5 新代码的成功链路：自动退出、替换、重启、健康标记、helper 退出、受信登录与 1280 Token；真实历史旧版首次过渡、只读 DMG、不可写系统路径、取消与安装故障/真实回滚仍未在打包 App 级验收。故障注入在 TC-036 合成单元；0.3.5 DMG 另经 hdiutil verify VALID，SHA-256 ae1b8e80ec69c43f76e93d1e2312694cb4faab3521115fdaeec9e304d6e697fd。
 2026-10-04 / 80e7f10→0eac84b：当前新证据已覆盖只读旧包直接启动初始界面、隔离可写路径的五种 installer 模块 hooks 失败回退/清理和再次重试；“未确认安装”只指未点击更新。没有从只读卷触发目标选择、真实 /Applications/~/Applications、打包 helper/UI 故障闭环、安装中取消、签名或目标 Mac。前段“未直接启动”是 1e70412 历史。
 2026-10-04 当前边界：已走打包 helper/UI 的隔离注入闭环；注入并非真实磁盘满、进程崩溃或系统 /Applications/~/Applications 安装，仍未执行安装中取消、生产库或签名公证异机。上方“未在打包态注入”是 0eac84b 历史阶段。
 2026-10-04 取消正例未编码/未运行；不点击确认不算安装中取消，模块单元和现有五故障也不替代打包 UI→helper 取消路径。真实断电/满盘、系统目录、签名异机另验。
-本次并未复跑真实旧/新 DMG 与固定 SHA 的故障链；历史 1961de3 证据另列。系统安装、签名公证及安装中取消未验。
+2026-10-06 时的记录：本轮未复跑真实旧/新 DMG 与固定 SHA 的故障链；该阶段记录已由下方 2026-10-07 新制品隔离复验补充。系统安装、签名公证及安装中取消仍未验。
 2026-10-04 用户已撤出安装中取消交付要求；前文独立控制窗口/五阶段点击取消及“取消未验”属于历史阶段，不再构成当前简化目标的待验项。新包仍须按简化范围重新核安装成功、自动失败回退和数据连续性。
-2026-10-04 用户最新决议：取消交付义务的边界从“开始替换/安装”前移至点击“开始升级”；下载/校验/交接/安装均不可中断取消。上方“下载取消待核实/安装中取消待验”及阶段取消正例只属历史；本轮只验点击前放弃、正常完成与失败自动回退。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M81" s="52" t="str">
+2026-10-04 用户最新决议：取消交付义务的边界从“开始替换/安装”前移至点击“开始升级”；下载/校验/交接/安装均不可中断取消。上方“下载取消待核实/安装中取消待验”及阶段取消正例只属历史；本轮只验点击前放弃、正常完成与失败自动回退。
+2026-10-07 补充：真实旧/新 DMG 的隔离成功升级、五种打包 helper 故障回退/重试已由开发统筹报告通过；不覆盖真实 /Applications 或 ~/Applications 安装、生产用户数据、真实满盘/崩溃及其他 Mac。</x:v>
+      </x:c>
+      <x:c r="M81" s="109" t="str">
         <x:v>代码 1e70412；macOS 15.7.4 x86_64、Node v24.15.0；真实旧/新候选 DMG 哈希与大小见 I 列，TC-076 exit 0；门禁 94 入口/77 单元/38 Electron、0.3.6 目录包 E2E 38/38 均退出码 0。无生产更新服务器发布、生产用户数据操作、签名公证或异机证据。
 2026-10-04 / 80e7f10→0eac84b：固定代码 0eac84b，macOS 15.7.4 x86_64、Node 24.15.0；同真实旧/新 DMG 全命令 exit 0；独立构建 0.3.6 x64 目录包；门禁 94 入口/77 单元/38 Electron、打包版 38/38 exit 0。前次 80e7f10 exit 1 保留；详见 docs/validation.md。
 1961de3；文档会话独立 TC-076 完整命令 exit 0，真实旧/新 DMG SHA-256 分别 ae1b8e80…、d99d7af9…，两包 hdiutil verify VALID；打包 helper mount/space/replace/launch/health 各回退、受信登录/1280 Token/清理及最后重试均通过；TC-036 两单元 exit 0。
@@ -14987,7 +14995,8 @@
 508851a；macOS 15.7.4 x86_64、Node v24.15.0；TOKEN_TC076_SKIP_BUILD=1 npm run test:case -- TC-076：exit 0；当前包改版本元数据合成旧版，自动退出/替换/启动、受信登录及合成 1280 Token 延续。 2026-10-04 独立复验固定代码 508851a：test:gate 类型检查、94 注册入口、97/97 单元、43/43 Electron，exit 0；隔离临时库/无正文样本。打包全量 42/43、日期用例单项重跑 1/1；真实外部/生产验收未据此通过。
 后续新包 TC-076 隔离动态子范围已由需求会话执行通过，详见 I 列最新证据；整项仍部分验证。
 新包 8773dd3865cda61709061916723c0ff607ed126649f32edaee451a3e2d1815a2：TC-076 exit 0，打包 Electron 43/43，test:gate 97/97 单元+43/43 Electron；均由需求会话报告，文档会话未独立复跑。
-2026-10-06 本轮第三次成功只覆盖合成旧版链路，未执行真实旧/新 DMG 故障子范围、系统安装目录或生产用户数据；历史真实 DMG 证据只归属原固定候选。</x:v>
+2026-10-06 本轮第三次成功只覆盖合成旧版链路，未执行真实旧/新 DMG 故障子范围、系统安装目录或生产用户数据；历史真实 DMG 证据只归属原固定候选。
+2026-10-07：基于 main f109abc，开发统筹报告完整门禁 108 入口/108 单元/58 Electron、重新打包后 packaged 58/58；GitHub x64 未签名 DMG 及真实 0.3.11→0.3.12 隔离 TC-076/五故障回退/重试通过。GitHub DMG 重新下载后独立 SHA-256 回验通过；签名、公证、异机/外部分发和生产数据未验。</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="300" customHeight="1">
@@ -17924,7 +17933,7 @@
 主线合并是代码集成，不代替 SOP-005 目标 Mac 实际安装、制品哈希及发布/回退记录；本机未签名交付仍待独立执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="307.5" customHeight="1">
+    <x:row r="19" ht="420" customHeight="1">
       <x:c r="A19" s="104" t="str">
         <x:v>VER-014</x:v>
       </x:c>
@@ -17944,19 +17953,20 @@
         <x:v>DEV-024、DEV-025、DEV-059、DEV-060、DEV-061、DEV-062</x:v>
       </x:c>
       <x:c r="G19" s="104" t="str">
-        <x:v>TC-107 隔离服务/升级通过；TC-108 打包 E2E 与隔离性能通过；生产 App 更新待用户手动验收</x:v>
+        <x:v>TC-107/108 隔离范围通过；GitHub x64 未签名预发布已发布；VER-014 仍未完整交付，生产手动验收/外部分发待验</x:v>
       </x:c>
       <x:c r="H19" s="104" t="str">
-        <x:v>固定提交 d9b447c；TC-107 服务清单/真实 0.3.11 DMG 隔离升级及故障回退通过，TC-108 打包 E2E 与隔离性能通过。完整门禁 108 入口、108 单元、58 Electron，打包 58/58。2026-10-07：TC-108 首轮漏设 app.asar 固定摘要环境变量，在输入校验退出 1，页面子用例已通过；补齐后完整命令退出 0。35,000 条合成事实热/冷反馈 P95 最高 54.3ms，滚动 P95 17.5ms、无 ≥200ms 长任务。</x:v>
+        <x:v>本机更新服务 0.3.12 与 TC-107/108 既有证据保持原记录。2026-10-07 后续报告：GitHub https://github.com/lzhe72/Token/releases/tag/v0.3.12 从 main f109abc 重建产品代码 d9b447c 的 x64 未签名制品；当前 /Applications/Token.app 报告版本 0.3.12，app.asar 摘要匹配。该 GitHub 发布未改生产 App 或本机服务。</x:v>
       </x:c>
       <x:c r="I19" s="104" t="str">
-        <x:v>服务已发布，0.3.12 候选、TC-107 隔离升级及 TC-108 隔离性能自动范围通过；生产 /Applications/Token.app 仍 0.3.11，用户尚未自行点击升级和手动验收；VER-014 未交付。</x:v>
+        <x:v>本机更新服务仍有此前 0.3.12 x64 包（DMG SHA 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74）。GitHub v0.3.12 是独立预发布包，重新下载后独立 SHA-256 回验通过；开发报告当前安装 App 为 0.3.12。VER-014 原验收状态保持未完整交付，不能由此发布事件提升。</x:v>
       </x:c>
       <x:c r="J19" s="104" t="str">
-        <x:v>冻结产品提交 d9b447cc7cf210545023f6403d2d5f009cf6699b；package.json 0.3.12；x64 DMG 142585554 bytes，SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。TC-107 已通过；test:gate 108 入口/108 单元/58 Electron，通过打包 E2E 58/58。TC-108 首次因漏设 TOKEN_TC108_ASAR_SHA256 在输入校验退出 1，Electron 页面子用例已通过；补齐冻结摘要后 npm run test:case -- TC-108 整体退出 0。35,000 条合成事实：热反馈 P95 54.3/52.0ms、内容 P95 77.8/73.9ms；冷反馈 P95 47.8/46.9ms、内容 P95 59.7/56.7ms；10 秒滚动 601 帧，P95 17.5/17.5ms、最大 17.7/17.8ms、≥200ms 长任务 0。首次退出属于调用参数缺失，不是产品失败。服务 latest 0.3.12/x64 与制品摘要一致。</x:v>
+        <x:v>GitHub https://github.com/lzhe72/Token/releases/tag/v0.3.12：Token-0.3.12-x64.dmg，142585538 bytes，SHA-256 01b25b0b9fda31fd28862e612e0125c6743b84b182af0c4c2eea6fa6b34bb21a，hdiutil verify VALID；app.asar SHA-256 3f02efcef6be261165869d38445c6658199b53a97bbd4b8ddbb45a32d007390b。本机服务同版 DMG 142585554 bytes、SHA-256 7f431a226dd70ac8b9bbfdcc3dfdeed4edbd48103ce8dff1da8b2770d97caf74；重打包时间元数据导致文件 SHA 不同，app.asar SHA 相同。GitHub asset API 的大小/摘要与本地产物匹配为开发侧报告，重新下载后本地 SHA-256 回验通过。最新 main f109abc 上 test:gate 108 入口/108 单元/58 Electron，packaged 58/58；真实 0.3.11→GitHub 新 DMG 的隔离 TC-076 升级、五种 helper 故障回退及重试通过（开发统筹报告）。
+2026-10-07 下载回验补充：从公开 GitHub 预发布重新下载，复算 142585538 字节、SHA-256 01b25b0b9fda31fd28862e612e0125c6743b84b182af0c4c2eea6fa6b34bb21a，与源 DMG 和远端 asset digest 一致。</x:v>
       </x:c>
       <x:c r="K19" s="104" t="str">
-        <x:v>生产 /Applications/Token.app 只读仍为 0.3.11；开发未替用户升级。用户需自行在应用内点击更新并人工核新版、启动、受信状态、既有用量和切页体验后，才能更新交付状态。外部分发签名公证/异机未验；首轮 TC-107 失败及服务清单撤回历史保留。</x:v>
+        <x:v>GitHub 资产为未签名预发布测试包；无有效代码签名身份，Developer ID 签名、公证票据、其他 Mac 安装及外部分发未验。此发布不改本机更新服务/生产 App，不改变 VER-014 原未完成验收状态。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>